<commit_message>
Record first Web story E2E failure
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R62b13b44b2cf4df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R888929003867417a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R18ae41055eae4ea5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R3a51d968829d4ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R554a3b92a79a495b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R9ad3a24640e843dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R9dd323d9817646ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R880d74aa35134dee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -759,7 +759,7 @@
       </x:c>
       <x:c r="C5" s="19" t="n">
         <x:f>COUNTIF('Maliev.Web'!$G$2:$G$22,"Automated coverage declared")+COUNTIF('Maliev.Web'!$G$2:$G$22,"Passed")</x:f>
-        <x:v>19</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="D5" s="19" t="n">
         <x:f>COUNTIF('Maliev.Web'!$G$2:$G$22,"Partial")+COUNTIF('Maliev.Web'!$G$2:$G$22,"Partial after automated run")+COUNTIF('Maliev.Web'!$F$2:$F$22,"Partial")</x:f>
@@ -1550,16 +1550,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G9" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H9" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest run</x:v>
       </x:c>
       <x:c r="I9" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J9" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K9" s="48" t="str">
         <x:v>P2</x:v>
@@ -1577,7 +1577,7 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P9" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q9" s="48" t="str">
         <x:v>Maliev.Web.Bff; CommerceService if service/product data is catalog-backed; MaterialService and PricingService if quote entry preloads options; UploadService if quote entry supports immediate file upload</x:v>
@@ -1586,10 +1586,10 @@
         <x:v>None required for the discovery portion.; Optional anonymous quote draft/session if the quote entry creates one.</x:v>
       </x:c>
       <x:c r="S9" s="48" t="str">
-        <x:v>The Web CTA split must remain explicit: "Try demo" opens QuoteEngine demo mode, while "Start project" opens the signed-in QuoteEngine project flow.</x:v>
+        <x:v>The Web CTA split must remain explicit: "Try demo" opens QuoteEngine demo mode, while "Start project" opens the signed-in QuoteEngine project flow. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T9" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:82; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:82; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
       </x:c>
       <x:c r="U9" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2135,16 +2135,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G18" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H18" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest run</x:v>
       </x:c>
       <x:c r="I18" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J18" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K18" s="48" t="str">
         <x:v>P2</x:v>
@@ -2162,7 +2162,7 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P18" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q18" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.Web.Client; ContactService only when the journey ends in contact submission.</x:v>
@@ -2171,10 +2171,10 @@
         <x:v>None for browsing.; Contact inquiry if the journey converts through contact.</x:v>
       </x:c>
       <x:c r="S18" s="48" t="str">
-        <x:v>Content-to-quote conversion should be reviewed once the final Web-to-QuoteEngine handoff is revisited.</x:v>
+        <x:v>Content-to-quote conversion should be reviewed once the final Web-to-QuoteEngine handoff is revisited. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T18" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:587; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:587; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
       </x:c>
       <x:c r="U18" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2200,16 +2200,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G19" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H19" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest run</x:v>
       </x:c>
       <x:c r="I19" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J19" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K19" s="48" t="str">
         <x:v>P2</x:v>
@@ -2227,7 +2227,7 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P19" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q19" s="48" t="str">
         <x:v>Maliev.Web.Client; Maliev.Web.Bff if preferences are server-backed.</x:v>
@@ -2236,10 +2236,10 @@
         <x:v>Browser consent/preference state.; Optional server preference record if signed in and implemented.</x:v>
       </x:c>
       <x:c r="S19" s="48" t="str">
-        <x:v>If consent cannot be changed after the first decision, add a visible preference-management affordance.</x:v>
+        <x:v>If consent cannot be changed after the first decision, add a visible preference-management affordance. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T19" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:641; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:641; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
       </x:c>
       <x:c r="U19" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2330,13 +2330,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G21" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H21" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest run</x:v>
       </x:c>
       <x:c r="I21" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J21" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -2357,7 +2357,7 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P21" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q21" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; AuthService; CustomerService</x:v>
@@ -2366,10 +2366,10 @@
         <x:v>Demo path: no project, quotation, order, upload, or customer history record.; Start-project path: customer session and, after upload/configuration, real ProjectService project state.</x:v>
       </x:c>
       <x:c r="S21" s="48" t="str">
-        <x:v>Replace any remaining Web-owned manufacturing quote form with this demo/start-project split when the old path is no longer needed.</x:v>
+        <x:v>Replace any remaining Web-owned manufacturing quote form with this demo/start-project split when the old path is no longer needed. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T21" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:746; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:746; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
       </x:c>
       <x:c r="U21" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2463,7 +2463,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53be2663167a4d27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a60542b18a4880"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6678,7 +6678,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5caa10f0b46547e5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb89cf05ce7f04b86"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8813,7 +8813,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb74fd4559a1d4ef1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f1c7235d8ad40cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Web demo handoff retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R554a3b92a79a495b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R9ad3a24640e843dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R9dd323d9817646ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R880d74aa35134dee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb2b34cdfe39543a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R757a8ad607f04fd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R9b6dc81a9ca94d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Reeaafe2b3ef84bf3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -759,7 +759,7 @@
       </x:c>
       <x:c r="C5" s="19" t="n">
         <x:f>COUNTIF('Maliev.Web'!$G$2:$G$22,"Automated coverage declared")+COUNTIF('Maliev.Web'!$G$2:$G$22,"Passed")</x:f>
-        <x:v>15</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="D5" s="19" t="n">
         <x:f>COUNTIF('Maliev.Web'!$G$2:$G$22,"Partial")+COUNTIF('Maliev.Web'!$G$2:$G$22,"Partial after automated run")+COUNTIF('Maliev.Web'!$F$2:$F$22,"Partial")</x:f>
@@ -1550,16 +1550,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G9" s="48" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H9" s="48" t="str">
-        <x:v>Failed in latest run</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="I9" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed</x:v>
       </x:c>
       <x:c r="J9" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K9" s="48" t="str">
         <x:v>P2</x:v>
@@ -1577,7 +1577,8 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P9" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.
+2026-06-23: Retest passed after QuoteEngine ac7ab3c added a visible demo-mode/sample-only notice on /demo. Focused Aspire E2E passed: Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. Retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx. Original failure TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q9" s="48" t="str">
         <x:v>Maliev.Web.Bff; CommerceService if service/product data is catalog-backed; MaterialService and PricingService if quote entry preloads options; UploadService if quote entry supports immediate file upload</x:v>
@@ -1589,7 +1590,8 @@
         <x:v>The Web CTA split must remain explicit: "Try demo" opens QuoteEngine demo mode, while "Start project" opens the signed-in QuoteEngine project flow. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T9" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:82; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:82; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx
+QuoteEngine fix commit: ac7ab3c. Aspire retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx.</x:v>
       </x:c>
       <x:c r="U9" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2135,16 +2137,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G18" s="48" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H18" s="48" t="str">
-        <x:v>Failed in latest run</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="I18" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed</x:v>
       </x:c>
       <x:c r="J18" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K18" s="48" t="str">
         <x:v>P2</x:v>
@@ -2162,7 +2164,8 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P18" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.
+2026-06-23: Retest passed after QuoteEngine ac7ab3c added a visible demo-mode/sample-only notice on /demo. Focused Aspire E2E passed: Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. Retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx. Original failure TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q18" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.Web.Client; ContactService only when the journey ends in contact submission.</x:v>
@@ -2174,7 +2177,8 @@
         <x:v>Content-to-quote conversion should be reviewed once the final Web-to-QuoteEngine handoff is revisited. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T18" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:587; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:587; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx
+QuoteEngine fix commit: ac7ab3c. Aspire retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx.</x:v>
       </x:c>
       <x:c r="U18" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2200,16 +2204,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G19" s="48" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H19" s="48" t="str">
-        <x:v>Failed in latest run</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="I19" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed</x:v>
       </x:c>
       <x:c r="J19" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K19" s="48" t="str">
         <x:v>P2</x:v>
@@ -2227,7 +2231,8 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P19" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.
+2026-06-23: Retest passed after QuoteEngine ac7ab3c added a visible demo-mode/sample-only notice on /demo. Focused Aspire E2E passed: Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. Retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx. Original failure TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q19" s="48" t="str">
         <x:v>Maliev.Web.Client; Maliev.Web.Bff if preferences are server-backed.</x:v>
@@ -2239,7 +2244,8 @@
         <x:v>If consent cannot be changed after the first decision, add a visible preference-management affordance. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T19" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:641; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:641; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx
+QuoteEngine fix commit: ac7ab3c. Aspire retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx.</x:v>
       </x:c>
       <x:c r="U19" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2330,16 +2336,16 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G21" s="48" t="str">
-        <x:v>Failed</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="H21" s="48" t="str">
-        <x:v>Failed in latest run</x:v>
+        <x:v>Resolved</x:v>
       </x:c>
       <x:c r="I21" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed</x:v>
       </x:c>
       <x:c r="J21" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Passed</x:v>
       </x:c>
       <x:c r="K21" s="48" t="str">
         <x:v>P1</x:v>
@@ -2357,7 +2363,8 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P21" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:162); BrowserJourneyGateTests.Web_PublicContentRoutes_RenderTrustPolicyAndSupportSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:199) Latest run 2026-06-23: FAILED focused E2E BrowserJourneyGateTests.Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. The handoff opened QuoteEngine Make Studio, but the assertion at BrowserJourneyGateTests.cs:187 expected demo wording /Demo only|Demo mode|Demo sample only|sample.step/ while the page body showed the current Make Studio shell plus "Reconnecting to your workspace" overlays. TRX: Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.
+2026-06-23: Retest passed after QuoteEngine ac7ab3c added a visible demo-mode/sample-only notice on /demo. Focused Aspire E2E passed: Web_PublicTrustAndQuoteHandoff_RoutesToLocalQuoteEngine. Retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx. Original failure TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx.</x:v>
       </x:c>
       <x:c r="Q21" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; AuthService; CustomerService</x:v>
@@ -2369,7 +2376,8 @@
         <x:v>Replace any remaining Web-owned manufacturing quote form with this demo/start-project split when the old path is no longer needed. Testing error documented 2026-06-23: Web-to-QuoteEngine handoff expectation is stale or the demo destination no longer exposes the required demo/sample cue. Classify as logistical/UX until product intent is confirmed, then update the page cue or the E2E assertion and retest.</x:v>
       </x:c>
       <x:c r="T21" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:746; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:746; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs Maliev.Aspire.Tests/TestResults/feature-tracker-web-public.trx
+QuoteEngine fix commit: ac7ab3c. Aspire retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-web-public-retest.trx.</x:v>
       </x:c>
       <x:c r="U21" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2463,7 +2471,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a60542b18a4880"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R350e435724e2432f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6678,7 +6686,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb89cf05ce7f04b86"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a6eeaa16b574e76"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8813,7 +8821,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f1c7235d8ad40cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a2235cbe07b44ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record browser suite failures in tracker
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb2b34cdfe39543a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R757a8ad607f04fd4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R9b6dc81a9ca94d20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Reeaafe2b3ef84bf3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R141f6d7fc98a4027"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Raa306e393d0343de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R7cddd1ae401c4d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R2ea7aa3c1fc043e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -759,7 +759,7 @@
       </x:c>
       <x:c r="C5" s="19" t="n">
         <x:f>COUNTIF('Maliev.Web'!$G$2:$G$22,"Automated coverage declared")+COUNTIF('Maliev.Web'!$G$2:$G$22,"Passed")</x:f>
-        <x:v>19</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="D5" s="19" t="n">
         <x:f>COUNTIF('Maliev.Web'!$G$2:$G$22,"Partial")+COUNTIF('Maliev.Web'!$G$2:$G$22,"Partial after automated run")+COUNTIF('Maliev.Web'!$F$2:$F$22,"Partial")</x:f>
@@ -790,7 +790,7 @@
       </x:c>
       <x:c r="C6" s="19" t="n">
         <x:f>COUNTIF('Maliev.Intranet'!$G$2:$G$64,"Automated coverage declared")+COUNTIF('Maliev.Intranet'!$G$2:$G$64,"Passed")</x:f>
-        <x:v>55</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D6" s="19" t="n">
         <x:f>COUNTIF('Maliev.Intranet'!$G$2:$G$64,"Partial")+COUNTIF('Maliev.Intranet'!$G$2:$G$64,"Partial after automated run")+COUNTIF('Maliev.Intranet'!$F$2:$F$64,"Partial")</x:f>
@@ -821,7 +821,7 @@
       </x:c>
       <x:c r="C7" s="19" t="n">
         <x:f>COUNTIF('Maliev.QuoteEngine'!$G$2:$G$32,"Automated coverage declared")+COUNTIF('Maliev.QuoteEngine'!$G$2:$G$32,"Passed")</x:f>
-        <x:v>29</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D7" s="19" t="n">
         <x:f>COUNTIF('Maliev.QuoteEngine'!$G$2:$G$32,"Partial")+COUNTIF('Maliev.QuoteEngine'!$G$2:$G$32,"Partial after automated run")+COUNTIF('Maliev.QuoteEngine'!$F$2:$F$32,"Partial")</x:f>
@@ -1095,16 +1095,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G2" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H2" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I2" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J2" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K2" s="48" t="str">
         <x:v>P2</x:v>
@@ -1122,7 +1122,10 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P2" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)</x:v>
+        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q2" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; CommerceService; Maliev.Web.Bff</x:v>
@@ -1131,10 +1134,12 @@
         <x:v>Product status changes from draft to published.</x:v>
       </x:c>
       <x:c r="S2" s="48" t="str">
-        <x:v>Public storefront caching must invalidate quickly enough for E2E to observe publication.</x:v>
+        <x:v>Public storefront caching must invalidate quickly enough for E2E to observe publication.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T2" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4187; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4187; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U2" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -1160,16 +1165,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G3" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H3" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I3" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J3" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K3" s="48" t="str">
         <x:v>P2</x:v>
@@ -1187,7 +1192,10 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P3" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q3" s="48" t="str">
         <x:v>Maliev.Web.Bff; CommerceService; OrderService; PaymentService; DeliveryService; CustomerService</x:v>
@@ -1196,10 +1204,12 @@
         <x:v>Cart state.; Checkout/order draft.</x:v>
       </x:c>
       <x:c r="S3" s="48" t="str">
-        <x:v>Final checkout/payment behavior may require separate payment-provider sandbox work.</x:v>
+        <x:v>Final checkout/payment behavior may require separate payment-provider sandbox work.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T3" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4234; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4234; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U3" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -1225,16 +1235,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G4" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H4" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I4" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J4" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K4" s="48" t="str">
         <x:v>P2</x:v>
@@ -1252,7 +1262,10 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P4" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)</x:v>
+        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q4" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; CommerceService; Maliev.Web.Bff</x:v>
@@ -1261,10 +1274,12 @@
         <x:v>Product status changes to archived/unpublished.</x:v>
       </x:c>
       <x:c r="S4" s="48" t="str">
-        <x:v>Define exact customer-facing behavior for old product URLs.</x:v>
+        <x:v>Define exact customer-facing behavior for old product URLs.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T4" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4286; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4286; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U4" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -1355,13 +1370,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G6" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H6" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I6" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J6" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -1382,7 +1397,10 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P6" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3319)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3319)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped: Document download failed: 404 {"type":"https://tools.ietf.org/html/rfc9110#section-15.5.5","title":"Not Found","status":404,"traceId":"00-e42669f877737efe7ac029309671d831-ed24a434f22bdbe4-01"}</x:v>
       </x:c>
       <x:c r="Q6" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; AuthService; CustomerService; QuotationService; OrderService; UploadService; PdfService; IAMService or authorization service boundary where applicable</x:v>
@@ -1391,10 +1409,12 @@
         <x:v>None expected except safe audit/security logs.</x:v>
       </x:c>
       <x:c r="S6" s="48" t="str">
-        <x:v>Define consistent forbidden versus not-found behavior for cross-customer resource probing.</x:v>
+        <x:v>Define consistent forbidden versus not-found behavior for cross-customer resource probing.
+Latest browser-suite failure(s): QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped</x:v>
       </x:c>
       <x:c r="T6" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5808; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5808; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U6" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -1420,16 +1440,16 @@
         <x:v>Required production gate. Automate once test hooks can reliably expire sessions.</x:v>
       </x:c>
       <x:c r="G7" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H7" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I7" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J7" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K7" s="48" t="str">
         <x:v>P0</x:v>
@@ -1447,7 +1467,10 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P7" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.Intranet_ProtectedRoutes_RedirectAnonymousUserToLogin (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3446); BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.Intranet_ProtectedRoutes_RedirectAnonymousUserToLogin (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3446); BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")</x:v>
       </x:c>
       <x:c r="Q7" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; Maliev.Intranet.Bff; AuthService; IAMService; Target domain service for the protected page</x:v>
@@ -1456,10 +1479,12 @@
         <x:v>Session/token state.; No domain mutation expected during denied/re-auth redirect unless user explicitly resubmits.</x:v>
       </x:c>
       <x:c r="S7" s="48" t="str">
-        <x:v>Define exact return URL and unsaved-work policies per app.</x:v>
+        <x:v>Define exact return URL and unsaved-work policies per app.
+Latest browser-suite failure(s): Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace</x:v>
       </x:c>
       <x:c r="T7" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5922; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5922; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U7" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -1812,16 +1837,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G13" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H13" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I13" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J13" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K13" s="48" t="str">
         <x:v>P2</x:v>
@@ -1839,7 +1864,10 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P13" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Web_CustomerEmailRegistration_CreatesAccountSessionAndSignsOut (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:335); BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Web_CustomerEmailRegistration_CreatesAccountSessionAndSignsOut (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:335); BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")</x:v>
       </x:c>
       <x:c r="Q13" s="48" t="str">
         <x:v>Maliev.Web.Bff; AuthService; CustomerService; IAMService; OrderService for account orders; DeliveryService for address/order delivery data</x:v>
@@ -1848,10 +1876,12 @@
         <x:v>Auth session/token records if persisted.; Optional refresh token rotation/revocation.</x:v>
       </x:c>
       <x:c r="S13" s="48" t="str">
-        <x:v>Verified-account restrictions should be added once email verification exists.</x:v>
+        <x:v>Verified-account restrictions should be added once email verification exists.
+Latest browser-suite failure(s): Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace</x:v>
       </x:c>
       <x:c r="T13" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:305; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:305; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U13" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2007,16 +2037,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G16" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H16" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I16" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J16" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K16" s="48" t="str">
         <x:v>P2</x:v>
@@ -2034,7 +2064,10 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P16" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q16" s="48" t="str">
         <x:v>Maliev.Web.Bff; CommerceService; CustomerService; OrderService; PaymentService; DeliveryService</x:v>
@@ -2043,10 +2076,12 @@
         <x:v>Browser cart state.; Checkout draft/order draft.; Optional customer delivery selection.</x:v>
       </x:c>
       <x:c r="S16" s="48" t="str">
-        <x:v>Final payment provider behavior may require sandbox-specific assertions.</x:v>
+        <x:v>Final payment provider behavior may require sandbox-specific assertions.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T16" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:471; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:471; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U16" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2403,13 +2438,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G22" s="51" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H22" s="51" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I22" s="51" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J22" s="51" t="str">
         <x:v>Needs retest loop</x:v>
@@ -2430,7 +2465,11 @@
         <x:v>web/v{version:apiVersion}/account (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:18); GET web/v{version:apiVersion}/account/session (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:24); GET web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:41); PATCH web/v{version:apiVersion}/account/profile (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:86); POST web/v{version:apiVersion}/account/email/change (Maliev.Web/Maliev.Web.Bff/Controllers/AccountController.cs:145)</x:v>
       </x:c>
       <x:c r="P22" s="51" t="str">
-        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.QuoteEngine_CustomerChatbotWindow_RetainsWebConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:611); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.Web_MaliChatbot_AnonymousVisitorReceivesAssistantReplyThroughWebBff (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6251)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.QuoteEngine_CustomerChatbotWindow_RetainsWebConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:611); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.Web_MaliChatbot_AnonymousVisitorReceivesAssistantReplyThroughWebBff (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6251)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_CustomerChatbotWindow_RetainsWebConversation: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")
+- Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")</x:v>
       </x:c>
       <x:c r="Q22" s="51" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; Maliev.ChatbotService; Redis (chatbot session lock); AuthService and CustomerService for signed-in personalization.</x:v>
@@ -2439,10 +2478,12 @@
         <x:v>Anonymous chatbot session for visitors.; Customer-scoped chatbot session/history for signed-in customers.; Browser-local personalization record.; Shared assistant-session cookie used for Web to QuoteEngine continuation.</x:v>
       </x:c>
       <x:c r="S22" s="51" t="str">
-        <x:v>Define anonymous vs. signed conversation retention, define tool-callable account/quote/order/profile/address surfaces that Mali and Make Studio should and should not invoke, broaden Make Studio agent E2E coverage from conversation restoration into DFM, corrected reupload, quote/order/payment, and finalize product-side abuse limits.</x:v>
+        <x:v>Define anonymous vs. signed conversation retention, define tool-callable account/quote/order/profile/address surfaces that Mali and Make Studio should and should not invoke, broaden Make Studio agent E2E coverage from conversation restoration into DFM, corrected reupload, quote/order/payment, and finalize product-side abuse limits.
+Latest browser-suite failure(s): QuoteEngine_CustomerChatbotWindow_RetainsWebConversation; Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace</x:v>
       </x:c>
       <x:c r="T22" s="51" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:803; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:803; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U22" s="52" t="str">
         <x:v>2026-06-23</x:v>
@@ -2471,7 +2512,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R350e435724e2432f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re65d2b30ed15431e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2588,16 +2629,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G2" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H2" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I2" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J2" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K2" s="48" t="str">
         <x:v>P2</x:v>
@@ -2615,7 +2656,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P2" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741); BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221)</x:v>
+        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741); BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q2" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; CommerceService; UploadService if media uses upload service</x:v>
@@ -2624,10 +2668,12 @@
         <x:v>Product record.; Variant records.; Media references.</x:v>
       </x:c>
       <x:c r="S2" s="48" t="str">
-        <x:v>Media upload behavior should be included once final media storage path is fixed.</x:v>
+        <x:v>Media upload behavior should be included once final media storage path is fixed.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T2" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4136; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4136; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U2" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2653,16 +2699,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G3" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H3" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I3" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J3" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K3" s="48" t="str">
         <x:v>P2</x:v>
@@ -2680,7 +2726,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P3" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)</x:v>
+        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q3" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; CommerceService; Maliev.Web.Bff</x:v>
@@ -2689,10 +2738,12 @@
         <x:v>Product status changes from draft to published.</x:v>
       </x:c>
       <x:c r="S3" s="48" t="str">
-        <x:v>Public storefront caching must invalidate quickly enough for E2E to observe publication.</x:v>
+        <x:v>Public storefront caching must invalidate quickly enough for E2E to observe publication.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T3" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4187; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4187; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U3" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2718,16 +2769,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G4" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H4" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I4" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J4" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K4" s="48" t="str">
         <x:v>P2</x:v>
@@ -2745,7 +2796,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AuthController.cs:20); GET api/v{version:apiVersion}/[controller]/login (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AuthController.cs:27); POST api/v{version:apiVersion}/[controller]/login (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AuthController.cs:41); POST api/v{version:apiVersion}/[controller]/login-form (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AuthController.cs:57); GET api/v{version:apiVersion}/[controller]/logout (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AuthController.cs:198)</x:v>
       </x:c>
       <x:c r="P4" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_PublicAccountSupportAndCommerceEntryPoints_Render (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:241); BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q4" s="48" t="str">
         <x:v>Maliev.Web.Bff; CommerceService; OrderService; PaymentService; DeliveryService; CustomerService</x:v>
@@ -2754,10 +2808,12 @@
         <x:v>Cart state.; Checkout/order draft.</x:v>
       </x:c>
       <x:c r="S4" s="48" t="str">
-        <x:v>Final checkout/payment behavior may require separate payment-provider sandbox work.</x:v>
+        <x:v>Final checkout/payment behavior may require separate payment-provider sandbox work.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T4" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4234; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4234; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U4" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2783,16 +2839,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G5" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H5" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I5" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J5" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K5" s="48" t="str">
         <x:v>P2</x:v>
@@ -2810,7 +2866,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P5" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)</x:v>
+        <x:v>BrowserJourneyGateTests.Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:741)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden: System.TimeoutException : Timeout 30000ms exceeded. Call log: - waiting for GetByRole(AriaRole.Button, new() { NameRegex = new Regex("Continue to checkout|ดำเนินการชำระเงิน", RegexOptions.IgnoreCase) })</x:v>
       </x:c>
       <x:c r="Q5" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; CommerceService; Maliev.Web.Bff</x:v>
@@ -2819,10 +2878,12 @@
         <x:v>Product status changes to archived/unpublished.</x:v>
       </x:c>
       <x:c r="S5" s="48" t="str">
-        <x:v>Define exact customer-facing behavior for old product URLs.</x:v>
+        <x:v>Define exact customer-facing behavior for old product URLs.
+Latest browser-suite failure(s): Commerce_EmployeePublishesProduct_WebCustomerCanBrowseCartAndArchivedProductIsHidden</x:v>
       </x:c>
       <x:c r="T5" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4286; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4286; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U5" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2913,13 +2974,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G7" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H7" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I7" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J7" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -2940,7 +3001,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P7" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4684)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4684)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice: Microsoft.Playwright.PlaywrightException : Locator expected to contain text 'Pending Pdf' But was: ' Reconnecting to your workspace Keeping your page in place. This usually takes a moment. Attempting for 0s Still trying to reconnect The page is safe. Try re...</x:v>
       </x:c>
       <x:c r="Q7" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; InvoiceService; CustomerService; OrderService; UploadService; PdfService; AccountingService; NotificationService</x:v>
@@ -2949,10 +3013,12 @@
         <x:v>Invoice draft/issued record.; Invoice line items.; Attachment artifact references.; PDF artifact.; Accounting entry where implemented.</x:v>
       </x:c>
       <x:c r="S7" s="48" t="str">
-        <x:v>Define whether customer-facing invoice delivery happens through Web, QuoteEngine, email, or a finance-only process.</x:v>
+        <x:v>Define whether customer-facing invoice delivery happens through Web, QuoteEngine, email, or a finance-only process.
+Latest browser-suite failure(s): Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice</x:v>
       </x:c>
       <x:c r="T7" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4612; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4612; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U7" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -2978,13 +3044,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G8" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H8" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I8" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J8" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -3005,7 +3071,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P8" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4684)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4684)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice: Microsoft.Playwright.PlaywrightException : Locator expected to contain text 'Pending Pdf' But was: ' Reconnecting to your workspace Keeping your page in place. This usually takes a moment. Attempting for 0s Still trying to reconnect The page is safe. Try re...</x:v>
       </x:c>
       <x:c r="Q8" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; InvoiceService; PaymentService; PdfService; AccountingService; OrderService; UploadService; NotificationService</x:v>
@@ -3014,10 +3083,12 @@
         <x:v>Payment record/status.; Invoice status.; Receipt PDF/artifact.; Payment evidence artifact.; Accounting entry.; Notification record where configured.</x:v>
       </x:c>
       <x:c r="S8" s="48" t="str">
-        <x:v>Define correction/refund rules and the source of truth between InvoiceService and PaymentService.</x:v>
+        <x:v>Define correction/refund rules and the source of truth between InvoiceService and PaymentService.
+Latest browser-suite failure(s): Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice</x:v>
       </x:c>
       <x:c r="T8" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4677; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4677; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U8" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -3693,16 +3764,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G19" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H19" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I19" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J19" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K19" s="48" t="str">
         <x:v>P1</x:v>
@@ -3720,7 +3791,11 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P19" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5529); BrowserJourneyGateTests.Intranet_CustomerOnboardingUi_CreatesCompanyAddressesAndInternalNote (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5871); BrowserJourneyGateTests.Intranet_CustomerDetail_EditsProfilePaymentTermsAndAddress (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6008); BrowserJourneyGateTests.Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6208)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5529); BrowserJourneyGateTests.Intranet_CustomerOnboardingUi_CreatesCompanyAddressesAndInternalNote (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5871); BrowserJourneyGateTests.Intranet_CustomerDetail_EditsProfilePaymentTermsAndAddress (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6008); BrowserJourneyGateTests.Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6208)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord: Expected a customer search result but got resource type ''.
+- Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace: Microsoft.Playwright.PlaywrightException : Locator expected to contain text 'Quote Total' But was: ' Reconnecting to your workspace Keeping your page in place. This usually takes a moment. Attempting for 0s Still trying to reconnect The page is safe. Try re...</x:v>
       </x:c>
       <x:c r="Q19" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; CustomerService; CountryService; UploadService; SearchService</x:v>
@@ -3729,10 +3804,12 @@
         <x:v>Customer profile fields.; Payment terms.; Address/document records.; Search index data.</x:v>
       </x:c>
       <x:c r="S19" s="48" t="str">
-        <x:v>Missing UI affordances should be tracked rather than bypassed with direct API calls.</x:v>
+        <x:v>Missing UI affordances should be tracked rather than bypassed with direct API calls.
+Latest browser-suite failure(s): Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord; Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace</x:v>
       </x:c>
       <x:c r="T19" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2505; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2505; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U19" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -3758,16 +3835,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G20" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H20" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I20" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J20" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K20" s="48" t="str">
         <x:v>P1</x:v>
@@ -3785,7 +3862,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P20" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5529); BrowserJourneyGateTests.Intranet_ProjectNew_StlUploadProcessesThroughHiddenInput (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5567)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5529); BrowserJourneyGateTests.Intranet_ProjectNew_StlUploadProcessesThroughHiddenInput (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5567)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace: Microsoft.Playwright.PlaywrightException : Locator expected to contain text 'Quote Total' But was: ' Reconnecting to your workspace Keeping your page in place. This usually takes a moment. Attempting for 0s Still trying to reconnect The page is safe. Try re...</x:v>
       </x:c>
       <x:c r="Q20" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; CustomerService; UploadService; GeometryService; MaterialService; PricingService; ProjectService; QuotationService; RabbitMQ</x:v>
@@ -3794,10 +3874,12 @@
         <x:v>Project/draft record.; Uploaded CAD artifact.; Geometry analysis result.; Part configuration.; Pricing result.</x:v>
       </x:c>
       <x:c r="S20" s="48" t="str">
-        <x:v>Any parts still stuck in analyzing state after backend terminal status should fail this story.</x:v>
+        <x:v>Any parts still stuck in analyzing state after backend terminal status should fail this story.
+Latest browser-suite failure(s): Intranet_EmployeeCreatedCustomer_CanBeOpenedAndSelectedInProjectWorkspace</x:v>
       </x:c>
       <x:c r="T20" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2562; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2562; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U20" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -3823,16 +3905,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G21" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H21" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I21" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J21" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K21" s="48" t="str">
         <x:v>P1</x:v>
@@ -3850,7 +3932,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P21" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.Intranet_ProjectNew_StlUploadProcessesThroughHiddenInput (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5567); BrowserJourneyGateTests.Intranet_ProjectQuoteLifecycle_GeneratesVersionsPdfAcceptanceAndDuplicate (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5691)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.Intranet_ProjectNew_StlUploadProcessesThroughHiddenInput (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5567); BrowserJourneyGateTests.Intranet_ProjectQuoteLifecycle_GeneratesVersionsPdfAcceptanceAndDuplicate (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5691)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports: Assert.False() Failure Expected: False Actual: True</x:v>
       </x:c>
       <x:c r="Q21" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; QuotationService; PdfService; UploadService; ReceiptService as a negative verification boundary; EmployeeService</x:v>
@@ -3859,10 +3944,12 @@
         <x:v>Quotation/document request.; PDF artifact.; Quotation version PDF artifact fields.</x:v>
       </x:c>
       <x:c r="S21" s="48" t="str">
-        <x:v>Missing thumbnails, missing employee identity, or PDF artifact attached only to "latest quote" instead of the exact quotation version should fail this story.</x:v>
+        <x:v>Missing thumbnails, missing employee identity, or PDF artifact attached only to "latest quote" instead of the exact quotation version should fail this story.
+Latest browser-suite failure(s): Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports</x:v>
       </x:c>
       <x:c r="T21" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2631; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2631; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U21" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -3888,16 +3975,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G22" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H22" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I22" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J22" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K22" s="48" t="str">
         <x:v>P1</x:v>
@@ -3915,7 +4002,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P22" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.Intranet_ProjectQuoteLifecycle_GeneratesVersionsPdfAcceptanceAndDuplicate (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5691)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.Intranet_ProjectQuoteLifecycle_GeneratesVersionsPdfAcceptanceAndDuplicate (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5691)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports: Assert.False() Failure Expected: False Actual: True</x:v>
       </x:c>
       <x:c r="Q22" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; ProjectService; UploadService; GeometryService; PricingService; MaterialService; QuotationService</x:v>
@@ -3924,10 +4014,12 @@
         <x:v>New project/draft record.; File references to existing artifacts or copied artifacts.; Updated quote/pricing data.; SourceProjectId/SourceProjectNumber linkage.</x:v>
       </x:c>
       <x:c r="S22" s="48" t="str">
-        <x:v>Reorder must preserve artifacts, record source-project linkage, and not force customers/employees to reupload unchanged files.</x:v>
+        <x:v>Reorder must preserve artifacts, record source-project linkage, and not force customers/employees to reupload unchanged files.
+Latest browser-suite failure(s): Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports</x:v>
       </x:c>
       <x:c r="T22" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2689; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2689; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U22" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -4018,16 +4110,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G24" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H24" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I24" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J24" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K24" s="48" t="str">
         <x:v>P1</x:v>
@@ -4045,7 +4137,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P24" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4684)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4684)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice: Microsoft.Playwright.PlaywrightException : Locator expected to contain text 'Pending Pdf' But was: ' Reconnecting to your workspace Keeping your page in place. This usually takes a moment. Attempting for 0s Still trying to reconnect The page is safe. Try re...</x:v>
       </x:c>
       <x:c r="Q24" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; InvoiceService; PaymentService; ReceiptService; PdfService; UploadService; AccountingService; NotificationService</x:v>
@@ -4054,10 +4149,12 @@
         <x:v>Invoice.; Payment record.; Receipt record.; Receipt PDF artifact.; Accounting entry.</x:v>
       </x:c>
       <x:c r="S24" s="48" t="str">
-        <x:v>Payment provider sandbox behavior must be deterministic for E2E.</x:v>
+        <x:v>Payment provider sandbox behavior must be deterministic for E2E.
+Latest browser-suite failure(s): Intranet_FinanceInvoice_CreatesAttachesAndFinalizesCustomerInvoice</x:v>
       </x:c>
       <x:c r="T24" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2805; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2805; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U24" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -4668,16 +4765,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G34" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H34" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I34" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J34" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K34" s="48" t="str">
         <x:v>P1</x:v>
@@ -4695,7 +4792,11 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P34" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177); BrowserJourneyGateTests.Intranet_ProjectQuoteLifecycle_GeneratesVersionsPdfAcceptanceAndDuplicate (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5691)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177); BrowserJourneyGateTests.Intranet_ProjectQuoteLifecycle_GeneratesVersionsPdfAcceptanceAndDuplicate (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:5691)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports: Assert.False() Failure Expected: False Actual: True
+- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })</x:v>
       </x:c>
       <x:c r="Q34" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; UploadService; GeometryService; ProjectService; RabbitMQ</x:v>
@@ -4704,10 +4805,12 @@
         <x:v>Viewer/thumbnail artifact references.; DFM result.; Drawing attachment artifact.; Part artifact metadata.</x:v>
       </x:c>
       <x:c r="S34" s="48" t="str">
-        <x:v>Add explicit E2E fixtures for multibody/viewer artifact edge cases and attachment authorization.</x:v>
+        <x:v>Add explicit E2E fixtures for multibody/viewer artifact edge cases and attachment authorization.
+Latest browser-suite failure(s): Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports</x:v>
       </x:c>
       <x:c r="T34" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:3400; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:3400; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U34" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -4798,16 +4901,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G36" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H36" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I36" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J36" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K36" s="48" t="str">
         <x:v>P1</x:v>
@@ -4825,7 +4928,11 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P36" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1056); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports: Assert.False() Failure Expected: False Actual: True
+- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })</x:v>
       </x:c>
       <x:c r="Q36" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; MaterialService; PricingService; GeometryService; ProjectService</x:v>
@@ -4834,10 +4941,12 @@
         <x:v>Multiple part configurations.; Multiple pricing results.; DFM state for process-sensitive checks.; Draft autosave state.</x:v>
       </x:c>
       <x:c r="S36" s="48" t="str">
-        <x:v>Define preview/undo behavior for large bulk edits if employees need safety before applying changes.</x:v>
+        <x:v>Define preview/undo behavior for large bulk edits if employees need safety before applying changes.
+Latest browser-suite failure(s): Intranet_ProjectGeometryRuntime_LoadsAcrossDeviceViewports; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports</x:v>
       </x:c>
       <x:c r="T36" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:3520; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:3520; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U36" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -5838,16 +5947,16 @@
         <x:v>Ready to automate</x:v>
       </x:c>
       <x:c r="G52" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H52" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I52" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J52" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K52" s="48" t="str">
         <x:v>P2</x:v>
@@ -5865,7 +5974,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P52" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887); BrowserJourneyGateTests.Intranet_ReferenceDataWorkbench_ManagesRegistryLocationsAndLoadsReferencePages (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3988); BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6208)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887); BrowserJourneyGateTests.Intranet_ReferenceDataWorkbench_ManagesRegistryLocationsAndLoadsReferencePages (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3988); BrowserJourneyGateTests.Intranet_AutomationEmployee_ModuleRoutesRenderWithoutAuthOrStartupFailures (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:4221); BrowserJourneyGateTests.Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6208)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord: Expected a customer search result but got resource type ''.</x:v>
       </x:c>
       <x:c r="Q52" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; SearchService; IAMService; Domain services that publish searchable records</x:v>
@@ -5874,10 +5986,12 @@
         <x:v>Search index entries.</x:v>
       </x:c>
       <x:c r="S52" s="48" t="str">
-        <x:v>Missing index coverage for a domain should be logged as product/search backlog.</x:v>
+        <x:v>Missing index coverage for a domain should be logged as product/search backlog.
+Latest browser-suite failure(s): Intranet_GlobalSearch_ReturnsEmployeeCreatedCustomerAndNavigatesToRecord</x:v>
       </x:c>
       <x:c r="T52" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4397; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4397; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U52" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -5968,13 +6082,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G54" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H54" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I54" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J54" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -5995,7 +6109,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P54" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Intranet_CustomerNotification_QueuesDeliveryAndRespectsOptOutPreference (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6126); BrowserJourneyGateTests.Intranet_CustomerEmailTemplatesAndAiExtraction_AreReachable (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6684)</x:v>
+        <x:v>BrowserJourneyGateTests.Intranet_CustomerNotification_QueuesDeliveryAndRespectsOptOutPreference (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6126); BrowserJourneyGateTests.Intranet_CustomerEmailTemplatesAndAiExtraction_AreReachable (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6684)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Intranet_CustomerNotification_QueuesDeliveryAndRespectsOptOutPreference: Expected /api/v1/notifications/preferences/2e9bd85d-4155-44f1-8f03-b013be20b4dd to contain email before timeout. Last result: 503 {"title":"Upstream service unavailable","status":503,"detail":"A downstream service did not respond in time. Please retry later."}</x:v>
       </x:c>
       <x:c r="Q54" s="48" t="str">
         <x:v>Maliev.Intranet.Bff; NotificationService; RabbitMQ; Triggering domain service</x:v>
@@ -6004,10 +6121,12 @@
         <x:v>Notification preference.; Notification delivery/log record.; Read/unread state.</x:v>
       </x:c>
       <x:c r="S54" s="48" t="str">
-        <x:v>Event types without notification mappings should be cataloged. Customer/employee notification center UI, read/unread state, live push surface, external provider sandbox delivery, and low-permission negative notification checks still need product and E2E coverage.</x:v>
+        <x:v>Event types without notification mappings should be cataloged. Customer/employee notification center UI, read/unread state, live push surface, external provider sandbox delivery, and low-permission negative notification checks still need product and E2E coverage.
+Latest browser-suite failure(s): Intranet_CustomerNotification_QueuesDeliveryAndRespectsOptOutPreference</x:v>
       </x:c>
       <x:c r="T54" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4496; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:4496; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U54" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -6553,16 +6672,16 @@
         <x:v>Required production gate. Automate once test hooks can reliably expire sessions.</x:v>
       </x:c>
       <x:c r="G63" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H63" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I63" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J63" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K63" s="48" t="str">
         <x:v>P0</x:v>
@@ -6580,7 +6699,10 @@
         <x:v>api/v{version:apiVersion}/[controller] (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:16); GET api/v{version:apiVersion}/[controller]/accounts-tree (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:29); GET api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:42); POST api/v{version:apiVersion}/[controller]/journal-entries (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:60); POST api/v{version:apiVersion}/[controller]/journal-entries/{id:guid}/post (Maliev.Intranet/Maliev.Intranet.Bff/Controllers/AccountingController.cs:71)</x:v>
       </x:c>
       <x:c r="P63" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.Intranet_ProtectedRoutes_RedirectAnonymousUserToLogin (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3446); BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.Intranet_ProtectedRoutes_RedirectAnonymousUserToLogin (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3446); BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")</x:v>
       </x:c>
       <x:c r="Q63" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; Maliev.Intranet.Bff; AuthService; IAMService; Target domain service for the protected page</x:v>
@@ -6589,10 +6711,12 @@
         <x:v>Session/token state.; No domain mutation expected during denied/re-auth redirect unless user explicitly resubmits.</x:v>
       </x:c>
       <x:c r="S63" s="48" t="str">
-        <x:v>Define exact return URL and unsaved-work policies per app.</x:v>
+        <x:v>Define exact return URL and unsaved-work policies per app.
+Latest browser-suite failure(s): Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace</x:v>
       </x:c>
       <x:c r="T63" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5922; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5922; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U63" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -6686,7 +6810,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a6eeaa16b574e76"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2afae03a400c4fa6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6803,13 +6927,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G2" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H2" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I2" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J2" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -6830,7 +6954,11 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P2" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1255); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1255); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
+- QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn: System.TimeoutException : Timeout 30000ms exceeded. =========================== logs =========================== waiting for navigation until "Commit" ============================================================ ---- System.TimeoutException : Timeout 30000m...</x:v>
       </x:c>
       <x:c r="Q2" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; AuthService; CustomerService; ProjectService; QuotationService once a formal quote is generated</x:v>
@@ -6839,10 +6967,12 @@
         <x:v>Customer session.; ProjectService project record in real project mode.; No project record in demo-only mode.</x:v>
       </x:c>
       <x:c r="S2" s="48" t="str">
-        <x:v>Replace prototype workspace persistence with durable ProjectService-backed project create/resume/list behavior.</x:v>
+        <x:v>Replace prototype workspace persistence with durable ProjectService-backed project create/resume/list behavior.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn</x:v>
       </x:c>
       <x:c r="T2" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:885; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:885; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U2" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -6868,13 +6998,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G3" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H3" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I3" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J3" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -6895,7 +7025,13 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P3" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
+- QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
+- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })</x:v>
       </x:c>
       <x:c r="Q3" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; AuthService; UploadService; GeometryService; RabbitMQ; ProjectService</x:v>
@@ -6904,10 +7040,12 @@
         <x:v>Upload record.; CAD artifact/blob.; Geometry analysis record/status.; Project part record/configuration state.</x:v>
       </x:c>
       <x:c r="S3" s="48" t="str">
-        <x:v>Production QuoteEngine needs the same artifact enrichment rigor expected in the employee project quote workspace.</x:v>
+        <x:v>Production QuoteEngine needs the same artifact enrichment rigor expected in the employee project quote workspace.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports</x:v>
       </x:c>
       <x:c r="T3" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:948; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:948; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U3" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -6933,13 +7071,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G4" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H4" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I4" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J4" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -6960,7 +7098,12 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P4" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
+- QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
       </x:c>
       <x:c r="Q4" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; MaterialService; PricingService; ProjectService; DeliveryService if delivery option affects quote</x:v>
@@ -6969,10 +7112,12 @@
         <x:v>Part configuration.; Pricing request/response.; Project pricing state and quote-ready totals.</x:v>
       </x:c>
       <x:c r="S4" s="48" t="str">
-        <x:v>QuoteEngine must call real MaterialService, PricingService, and ProjectService for production. Prototype pricing cannot pass this story.</x:v>
+        <x:v>QuoteEngine must call real MaterialService, PricingService, and ProjectService for production. Prototype pricing cannot pass this story.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
       </x:c>
       <x:c r="T4" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1014; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1014; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U4" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -6998,13 +7143,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G5" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H5" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I5" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J5" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7025,7 +7170,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P5" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
       </x:c>
       <x:c r="Q5" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; UploadService; GeometryService; PricingService; RabbitMQ</x:v>
@@ -7034,10 +7182,12 @@
         <x:v>New upload artifact or updated part configuration.; New geometry/DFM result.; Updated price.</x:v>
       </x:c>
       <x:c r="S5" s="48" t="str">
-        <x:v>QuoteEngine must implement project-part revision-aware upload and analysis state before this can be production-gate ready.</x:v>
+        <x:v>QuoteEngine must implement project-part revision-aware upload and analysis state before this can be production-gate ready.
+Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
       </x:c>
       <x:c r="T5" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1072; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1072; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U5" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7063,13 +7213,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G6" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H6" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I6" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J6" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7090,7 +7240,11 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P6" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1255); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1255); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
+- QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn: System.TimeoutException : Timeout 30000ms exceeded. =========================== logs =========================== waiting for navigation until "Commit" ============================================================ ---- System.TimeoutException : Timeout 30000m...</x:v>
       </x:c>
       <x:c r="Q6" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; AuthService; CustomerService; IAMService; ProjectService</x:v>
@@ -7099,10 +7253,12 @@
         <x:v>Customer session.; Real ProjectService project only after explicit signed-in start.; Optional new customer account.; No mutation from demo-only usage.</x:v>
       </x:c>
       <x:c r="S6" s="48" t="str">
-        <x:v>Define whether any demo configuration can be copied into a real project. If yes, it must be explicit and backed by secure server-side customer identity.</x:v>
+        <x:v>Define whether any demo configuration can be copied into a real project. If yes, it must be explicit and backed by secure server-side customer identity.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn</x:v>
       </x:c>
       <x:c r="T6" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1124; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1124; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U6" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7128,13 +7284,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G7" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H7" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I7" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J7" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7155,7 +7311,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P7" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q7" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; ProjectService; QuotationService; PdfService; UploadService; CustomerService; NotificationService if employee/customer alerts are sent</x:v>
@@ -7164,10 +7323,12 @@
         <x:v>Quotation record if first quote for project.; New immutable QuotationVersion on the project's quotation.; Project snapshot JSON/hash.; Generated PDF artifact attached to the exact version.; Optional notification record.</x:v>
       </x:c>
       <x:c r="S7" s="48" t="str">
-        <x:v>QuoteEngine must connect to real ProjectService -&gt; QuotationService -&gt; PdfService path. Prototype PDF behavior is not sufficient.</x:v>
+        <x:v>QuoteEngine must connect to real ProjectService -&gt; QuotationService -&gt; PdfService path. Prototype PDF behavior is not sufficient.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T7" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1180; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1180; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U7" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7193,13 +7354,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G8" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H8" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I8" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J8" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7220,7 +7381,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P8" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q8" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; QuotationService; OrderService; PaymentService; DeliveryService; CustomerService; JobService or ProjectService where production handoff is owned</x:v>
@@ -7229,10 +7393,12 @@
         <x:v>Accepted quotation version state.; Accepted quotation version id/number.; Order record.; Payment intent/record.; Delivery record.; Optional job/production record.</x:v>
       </x:c>
       <x:c r="S8" s="48" t="str">
-        <x:v>End-to-end quote-version acceptance from QuoteEngine must be service-backed before production.</x:v>
+        <x:v>End-to-end quote-version acceptance from QuoteEngine must be service-backed before production.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T8" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1245; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1245; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U8" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7323,13 +7489,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G10" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H10" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I10" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J10" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7350,7 +7516,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P10" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_LocalPortalRoutes_RenderPrototypeBackedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3288)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_LocalPortalRoutes_RenderPrototypeBackedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3288)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q10" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; CustomerService; QuotationService; OrderService; PaymentService; DeliveryService; JobService or ProjectService; PdfService/UploadService</x:v>
@@ -7359,10 +7528,12 @@
         <x:v>None required unless status refresh creates audit/access records.</x:v>
       </x:c>
       <x:c r="S10" s="48" t="str">
-        <x:v>QuoteEngine history needs durable ProjectService/QuotationService ownership before this can pass.</x:v>
+        <x:v>QuoteEngine history needs durable ProjectService/QuotationService ownership before this can pass.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T10" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1361; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1361; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U10" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7453,13 +7624,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G12" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H12" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I12" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J12" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7480,7 +7651,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P12" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_LocalPortalRoutes_RenderPrototypeBackedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3288)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_LocalPortalRoutes_RenderPrototypeBackedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3288)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q12" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; Production owner: QuotationService or customer quote-history service.; UploadService/PdfService when artifacts are shown.; QuoteEnginePrototypeStore where still prototype-backed.</x:v>
@@ -7489,10 +7663,12 @@
         <x:v>None required for read-only history.</x:v>
       </x:c>
       <x:c r="S12" s="48" t="str">
-        <x:v>Quote list navigation should be explicit if only detail route currently exists.</x:v>
+        <x:v>Quote list navigation should be explicit if only detail route currently exists.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T12" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1471; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1471; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U12" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7518,13 +7694,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G13" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H13" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I13" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J13" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7545,7 +7721,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P13" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_LocalPortalRoutes_RenderPrototypeBackedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3288)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_LocalPortalRoutes_RenderPrototypeBackedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3288)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q13" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; OrderService; PaymentService; DeliveryService; QuotationService; QuoteEnginePrototypeStore where still prototype-backed.</x:v>
@@ -7554,10 +7733,12 @@
         <x:v>None required for read-only status.</x:v>
       </x:c>
       <x:c r="S13" s="48" t="str">
-        <x:v>Production order history must replace prototype-backed order records.</x:v>
+        <x:v>Production order history must replace prototype-backed order records.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T13" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1522; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1522; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U13" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7713,13 +7894,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G16" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H16" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I16" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J16" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7740,7 +7921,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P16" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q16" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; /hubs/quote-notifications; UploadService/GeometryService for analysis events.; QuotationService, OrderService, or prototype store depending on event type.</x:v>
@@ -7749,10 +7933,12 @@
         <x:v>Event-driven status updates.; No new data required beyond the triggering workflow.</x:v>
       </x:c>
       <x:c r="S16" s="48" t="str">
-        <x:v>Production event source must replace prototype-only notifications for quote/order workflows.</x:v>
+        <x:v>Production event source must replace prototype-only notifications for quote/order workflows.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T16" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1680; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1680; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U16" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7843,13 +8029,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G18" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H18" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I18" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J18" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7870,7 +8056,11 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P18" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1255); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1255); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
+- QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn: System.TimeoutException : Timeout 30000ms exceeded. =========================== logs =========================== waiting for navigation until "Commit" ============================================================ ---- System.TimeoutException : Timeout 30000m...</x:v>
       </x:c>
       <x:c r="Q18" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; UploadService in production.; GeometryService only for valid CAD files.; QuoteEnginePrototypeStore while prototype-backed.</x:v>
@@ -7879,10 +8069,12 @@
         <x:v>Failed upload attempt.; Successful upload artifact for retry.; Part status/error state.</x:v>
       </x:c>
       <x:c r="S18" s="48" t="str">
-        <x:v>Define customer-facing retry controls, max size messaging, resumable continuation across browser refresh, and cleanup of abandoned uploads.</x:v>
+        <x:v>Define customer-facing retry controls, max size messaging, resumable continuation across browser refresh, and cleanup of abandoned uploads.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_RealProjectMode_BlocksCustomerUploadUntilSignIn</x:v>
       </x:c>
       <x:c r="T18" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1796; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1796; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U18" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7908,13 +8100,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G19" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H19" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I19" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J19" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -7935,7 +8127,12 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P19" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1177); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
+- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })</x:v>
       </x:c>
       <x:c r="Q19" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; GeometryService; PricingService; QuotationService in production.; QuoteEnginePrototypeStore while prototype-backed.</x:v>
@@ -7944,10 +8141,12 @@
         <x:v>DFM result.; DFM acknowledgement flag.; Quote part readiness state.</x:v>
       </x:c>
       <x:c r="S19" s="48" t="str">
-        <x:v>Decide which DFM severities block quote submission, require acknowledgement, or require employee review.</x:v>
+        <x:v>Decide which DFM severities block quote submission, require acknowledgement, or require employee review.
+Latest browser-suite failure(s): QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports</x:v>
       </x:c>
       <x:c r="T19" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1852; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1852; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U19" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7973,13 +8172,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G20" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H20" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I20" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J20" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -8000,7 +8199,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P20" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
       </x:c>
       <x:c r="Q20" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; PricingService; MaterialService; DeliveryService if delivery promise affects lead time.; QuotationService in production.</x:v>
@@ -8009,10 +8211,12 @@
         <x:v>Quote estimate.; Selected lead-time code.; Formal quote lead-time terms.</x:v>
       </x:c>
       <x:c r="S20" s="48" t="str">
-        <x:v>Define customer-visible lead-time language, cutoff times, delivery/calendar rules, and expiry behavior.</x:v>
+        <x:v>Define customer-visible lead-time language, cutoff times, delivery/calendar rules, and expiry behavior.
+Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
       </x:c>
       <x:c r="T20" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1909; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1909; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U20" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8038,13 +8242,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G21" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H21" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I21" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J21" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -8065,7 +8269,12 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P21" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:934); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
+- QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
       </x:c>
       <x:c r="Q21" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; PricingService; ProjectService or quote-draft owner.; QuotationService; QuoteEnginePrototypeStore while prototype-backed.</x:v>
@@ -8074,10 +8283,12 @@
         <x:v>Quote draft configuration.; Estimate revision.; Formal quote request using latest draft.</x:v>
       </x:c>
       <x:c r="S21" s="48" t="str">
-        <x:v>Define whether editing after formal quote creates a new quote version, cancels the old quote, or requires employee review.</x:v>
+        <x:v>Define whether editing after formal quote creates a new quote version, cancels the old quote, or requires employee review.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
       </x:c>
       <x:c r="T21" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1967; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1967; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U21" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8168,13 +8379,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G23" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H23" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I23" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J23" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -8195,7 +8406,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P23" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q23" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; QuotationService; OrderService; PaymentService; DeliveryService; CustomerService; PdfService/UploadService</x:v>
@@ -8204,10 +8418,12 @@
         <x:v>Accepted quote state.; Customer PO/reference.; Order record.; Payment/delivery intent where implemented.</x:v>
       </x:c>
       <x:c r="S23" s="48" t="str">
-        <x:v>Define customer PO requirement, acceptance terms text, quote expiry policy, and payment timing.</x:v>
+        <x:v>Define customer PO requirement, acceptance terms text, quote expiry policy, and payment timing.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T23" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2083; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2083; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U23" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8233,13 +8449,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G24" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H24" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I24" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J24" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -8260,7 +8476,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P24" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3319)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3319)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped: Document download failed: 404 {"type":"https://tools.ietf.org/html/rfc9110#section-15.5.5","title":"Not Found","status":404,"traceId":"00-e42669f877737efe7ac029309671d831-ed24a434f22bdbe4-01"}</x:v>
       </x:c>
       <x:c r="Q24" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; UploadService; PdfService; QuotationService; OrderService; IAMService or authorization boundary.</x:v>
@@ -8269,10 +8488,12 @@
         <x:v>None expected, except optional access/audit log.</x:v>
       </x:c>
       <x:c r="S24" s="48" t="str">
-        <x:v>Define the artifact taxonomy and customer-facing allowlist for quote/order documents.</x:v>
+        <x:v>Define the artifact taxonomy and customer-facing allowlist for quote/order documents.
+Latest browser-suite failure(s): QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped</x:v>
       </x:c>
       <x:c r="T24" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2144; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2144; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U24" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8298,13 +8519,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G25" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H25" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I25" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J25" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -8325,7 +8546,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P25" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
       </x:c>
       <x:c r="Q25" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; Optional MaterialService/PricingService if demo uses live read-only reference data.; No ProjectService, QuotationService, UploadService, OrderService, PaymentService, or DeliveryService mutation.</x:v>
@@ -8334,10 +8558,12 @@
         <x:v>None. Demo mode must not create customer, project, upload, quotation, quotation version, order, payment, delivery, or history records.</x:v>
       </x:c>
       <x:c r="S25" s="48" t="str">
-        <x:v>Define the demo asset catalog, disclaimer wording, and whether demo pricing uses fixed fixtures or live read-only pricing.</x:v>
+        <x:v>Define the demo asset catalog, disclaimer wording, and whether demo pricing uses fixed fixtures or live read-only pricing.
+Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
       </x:c>
       <x:c r="T25" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2200; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2200; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U25" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8363,10 +8589,10 @@
         <x:v>Required gap</x:v>
       </x:c>
       <x:c r="G26" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H26" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I26" s="48" t="str">
         <x:v>Not started</x:v>
@@ -8390,7 +8616,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P26" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)</x:v>
+        <x:v>BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465); BrowserJourneyGateTests.QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3033)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...</x:v>
       </x:c>
       <x:c r="Q26" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; AuthService; CustomerService; ProjectService; UploadService; GeometryService; MaterialService; PricingService; QuotationService; PdfService</x:v>
@@ -8399,10 +8628,12 @@
         <x:v>Project record and parts.; Quotation record linked to source project.; QuotationVersion 1 snapshot/PDF.; QuotationVersion 2 snapshot/PDF.; Project current quotation version fields.</x:v>
       </x:c>
       <x:c r="S26" s="48" t="str">
-        <x:v>Replace QuoteEnginePrototypeStore with real ProjectService/QuotationService workflow for signed project mode.</x:v>
+        <x:v>Replace QuoteEnginePrototypeStore with real ProjectService/QuotationService workflow for signed project mode.
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory</x:v>
       </x:c>
       <x:c r="T26" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2256; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2256; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U26" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8493,13 +8724,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G28" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H28" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I28" s="48" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J28" s="48" t="str">
         <x:v>Needs retest loop</x:v>
@@ -8520,7 +8751,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P28" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3319)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.QuoteEngine_CustomerIsolation_BlocksCrossCustomerQuoteOrderHistoryAccess (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3177); BrowserJourneyGateTests.QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3319)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped: Document download failed: 404 {"type":"https://tools.ietf.org/html/rfc9110#section-15.5.5","title":"Not Found","status":404,"traceId":"00-e42669f877737efe7ac029309671d831-ed24a434f22bdbe4-01"}</x:v>
       </x:c>
       <x:c r="Q28" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; AuthService; CustomerService; QuotationService; OrderService; UploadService; PdfService; IAMService or authorization service boundary where applicable</x:v>
@@ -8529,10 +8763,12 @@
         <x:v>None expected except safe audit/security logs.</x:v>
       </x:c>
       <x:c r="S28" s="48" t="str">
-        <x:v>Define consistent forbidden versus not-found behavior for cross-customer resource probing.</x:v>
+        <x:v>Define consistent forbidden versus not-found behavior for cross-customer resource probing.
+Latest browser-suite failure(s): QuoteEngine_CustomerDocuments_DownloadIsOwnerScoped</x:v>
       </x:c>
       <x:c r="T28" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5808; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5808; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U28" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8558,16 +8794,16 @@
         <x:v>Required production gate. Automate once test hooks can reliably expire sessions.</x:v>
       </x:c>
       <x:c r="G29" s="48" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H29" s="48" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I29" s="48" t="str">
-        <x:v>N/A</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J29" s="48" t="str">
-        <x:v>Passed</x:v>
+        <x:v>Needs retest loop</x:v>
       </x:c>
       <x:c r="K29" s="48" t="str">
         <x:v>P0</x:v>
@@ -8585,7 +8821,10 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P29" s="48" t="str">
-        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.Intranet_ProtectedRoutes_RedirectAnonymousUserToLogin (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3446); BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.Web_CustomerAccountSecurity_BlocksCrossCustomerAddressMutationAndPreservesReturnUrl (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:659); BrowserJourneyGateTests.Intranet_ProtectedRoutes_RedirectAnonymousUserToLogin (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3446); BrowserJourneyGateTests.Intranet_AutomationEmployee_SignsInAndReachesProtectedSurfaces (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:3887)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")</x:v>
       </x:c>
       <x:c r="Q29" s="48" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; Maliev.Intranet.Bff; AuthService; IAMService; Target domain service for the protected page</x:v>
@@ -8594,10 +8833,12 @@
         <x:v>Session/token state.; No domain mutation expected during denied/re-auth redirect unless user explicitly resubmits.</x:v>
       </x:c>
       <x:c r="S29" s="48" t="str">
-        <x:v>Define exact return URL and unsaved-work policies per app.</x:v>
+        <x:v>Define exact return URL and unsaved-work policies per app.
+Latest browser-suite failure(s): Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace</x:v>
       </x:c>
       <x:c r="T29" s="48" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5922; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:5922; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U29" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8753,13 +8994,13 @@
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="G32" s="51" t="str">
-        <x:v>Automated coverage declared</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="H32" s="51" t="str">
-        <x:v>No current error logged</x:v>
+        <x:v>Failed in latest browser suite</x:v>
       </x:c>
       <x:c r="I32" s="51" t="str">
-        <x:v>In progress</x:v>
+        <x:v>Not started</x:v>
       </x:c>
       <x:c r="J32" s="51" t="str">
         <x:v>Needs retest loop</x:v>
@@ -8780,7 +9021,11 @@
         <x:v>quote/v{version:apiVersion}/account (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:15); GET quote/v{version:apiVersion}/account/profile (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:46); GET quote/v{version:apiVersion}/account/addresses (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:76); GET quote/v{version:apiVersion}/account/quotes (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:112); GET quote/v{version:apiVersion}/account/orders (Maliev.QuoteEngine/Maliev.QuoteEngine.Bff/Controllers/AccountController.cs:120)</x:v>
       </x:c>
       <x:c r="P32" s="51" t="str">
-        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.QuoteEngine_CustomerChatbotWindow_RetainsWebConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:611); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.Web_MaliChatbot_AnonymousVisitorReceivesAssistantReplyThroughWebBff (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6251)</x:v>
+        <x:v>BrowserJourneyGateTests.Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:496); BrowserJourneyGateTests.QuoteEngine_CustomerChatbotWindow_RetainsWebConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:611); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_RestoresSignedCustomerConversation (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1278); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgent_LoginRedirectRestoresActiveChat (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1384); BrowserJourneyGateTests.Web_MaliChatbot_AnonymousVisitorReceivesAssistantReplyThroughWebBff (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:6251)
+2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
+TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
+- QuoteEngine_CustomerChatbotWindow_RetainsWebConversation: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")
+- Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator(".topbar-chat-toggle")</x:v>
       </x:c>
       <x:c r="Q32" s="51" t="str">
         <x:v>Maliev.Web.Bff; Maliev.QuoteEngine.Bff; Maliev.ChatbotService; Redis (chatbot session lock); AuthService and CustomerService for signed-in personalization.</x:v>
@@ -8789,10 +9034,12 @@
         <x:v>Anonymous chatbot session for visitors.; Customer-scoped chatbot session/history for signed-in customers.; Browser-local personalization record.; Shared assistant-session cookie used for Web to QuoteEngine continuation.</x:v>
       </x:c>
       <x:c r="S32" s="51" t="str">
-        <x:v>Define anonymous vs. signed conversation retention, define tool-callable account/quote/order/profile/address surfaces that Mali and Make Studio should and should not invoke, broaden Make Studio agent E2E coverage from conversation restoration into DFM, corrected reupload, quote/order/payment, and finalize product-side abuse limits.</x:v>
+        <x:v>Define anonymous vs. signed conversation retention, define tool-callable account/quote/order/profile/address surfaces that Mali and Make Studio should and should not invoke, broaden Make Studio agent E2E coverage from conversation restoration into DFM, corrected reupload, quote/order/payment, and finalize product-side abuse limits.
+Latest browser-suite failure(s): QuoteEngine_CustomerChatbotWindow_RetainsWebConversation; Web_CustomerChatbot_LoginPromptContinuesAuthenticatedConversationInPlace</x:v>
       </x:c>
       <x:c r="T32" s="51" t="str">
-        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:803; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs</x:v>
+        <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:803; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
       </x:c>
       <x:c r="U32" s="52" t="str">
         <x:v>2026-06-23</x:v>
@@ -8821,7 +9068,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a2235cbe07b44ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R987aab7464c645fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record anonymous demo retest result
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R141f6d7fc98a4027"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Raa306e393d0343de"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R7cddd1ae401c4d0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R2ea7aa3c1fc043e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra94bbcdf4009484f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Ra3e53cf045bc40ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R55b4983006e840fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R62640dfa82114838"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2512,7 +2512,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re65d2b30ed15431e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re74f505a548b4636"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6810,7 +6810,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2afae03a400c4fa6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2f27dfab5ad4a96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7001,13 +7001,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="H3" s="48" t="str">
-        <x:v>Failed in latest browser suite</x:v>
+        <x:v>Failed after partial fix</x:v>
       </x:c>
       <x:c r="I3" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J3" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="K3" s="48" t="str">
         <x:v>P1</x:v>
@@ -7031,7 +7031,8 @@
 - QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
 - QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
 - QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
-- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })</x:v>
+- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
+2026-06-23 targeted retest after QuoteEngine c926434: Demo only cue is now satisfied; remaining failure is waiting for role button '3D Model' exact at BrowserJourneyGateTests.cs:906. TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx.</x:v>
       </x:c>
       <x:c r="Q3" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; AuthService; UploadService; GeometryService; RabbitMQ; ProjectService</x:v>
@@ -7041,11 +7042,13 @@
       </x:c>
       <x:c r="S3" s="48" t="str">
         <x:v>Production QuoteEngine needs the same artifact enrichment rigor expected in the employee project quote workspace.
-Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports</x:v>
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports
+Post-fix anonymous demo retest still lacks visible 3D Model tab/button.</x:v>
       </x:c>
       <x:c r="T3" s="48" t="str">
         <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:948; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
-Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx
+QuoteEngine fix commit: c926434. Targeted retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx</x:v>
       </x:c>
       <x:c r="U3" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7074,13 +7077,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="H4" s="48" t="str">
-        <x:v>Failed in latest browser suite</x:v>
+        <x:v>Failed after partial fix</x:v>
       </x:c>
       <x:c r="I4" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J4" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="K4" s="48" t="str">
         <x:v>P1</x:v>
@@ -7103,7 +7106,8 @@
 TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
 - QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
 - QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
-- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
+2026-06-23 targeted retest after QuoteEngine c926434: Demo only cue is now satisfied; remaining failure is waiting for role button '3D Model' exact at BrowserJourneyGateTests.cs:906. TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx.</x:v>
       </x:c>
       <x:c r="Q4" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; MaterialService; PricingService; ProjectService; DeliveryService if delivery option affects quote</x:v>
@@ -7113,11 +7117,13 @@
       </x:c>
       <x:c r="S4" s="48" t="str">
         <x:v>QuoteEngine must call real MaterialService, PricingService, and ProjectService for production. Prototype pricing cannot pass this story.
-Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts
+Post-fix anonymous demo retest still lacks visible 3D Model tab/button.</x:v>
       </x:c>
       <x:c r="T4" s="48" t="str">
         <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1014; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
-Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx
+QuoteEngine fix commit: c926434. Targeted retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx</x:v>
       </x:c>
       <x:c r="U4" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -7146,13 +7152,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="H5" s="48" t="str">
-        <x:v>Failed in latest browser suite</x:v>
+        <x:v>Failed after partial fix</x:v>
       </x:c>
       <x:c r="I5" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J5" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="K5" s="48" t="str">
         <x:v>P1</x:v>
@@ -7173,7 +7179,8 @@
         <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896); BrowserJourneyGateTests.QuoteEngine_MakeStudioAgentTools_CorrectsDfmCompletesPaymentAndLinksProductionJob (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:1465)
 2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
 TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
-- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
+2026-06-23 targeted retest after QuoteEngine c926434: Demo only cue is now satisfied; remaining failure is waiting for role button '3D Model' exact at BrowserJourneyGateTests.cs:906. TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx.</x:v>
       </x:c>
       <x:c r="Q5" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; UploadService; GeometryService; PricingService; RabbitMQ</x:v>
@@ -7183,11 +7190,13 @@
       </x:c>
       <x:c r="S5" s="48" t="str">
         <x:v>QuoteEngine must implement project-part revision-aware upload and analysis state before this can be production-gate ready.
-Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
+Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts
+Post-fix anonymous demo retest still lacks visible 3D Model tab/button.</x:v>
       </x:c>
       <x:c r="T5" s="48" t="str">
         <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1072; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
-Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx
+QuoteEngine fix commit: c926434. Targeted retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx</x:v>
       </x:c>
       <x:c r="U5" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8103,13 +8112,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="H19" s="48" t="str">
-        <x:v>Failed in latest browser suite</x:v>
+        <x:v>Failed after partial fix</x:v>
       </x:c>
       <x:c r="I19" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J19" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="K19" s="48" t="str">
         <x:v>P1</x:v>
@@ -8132,7 +8141,8 @@
 TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
 - QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
 - QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
-- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })</x:v>
+- GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
+2026-06-23 targeted retest after QuoteEngine c926434: Demo only cue is now satisfied; remaining failure is waiting for role button '3D Model' exact at BrowserJourneyGateTests.cs:906. TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx.</x:v>
       </x:c>
       <x:c r="Q19" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; GeometryService; PricingService; QuotationService in production.; QuoteEnginePrototypeStore while prototype-backed.</x:v>
@@ -8142,11 +8152,13 @@
       </x:c>
       <x:c r="S19" s="48" t="str">
         <x:v>Decide which DFM severities block quote submission, require acknowledgement, or require employee review.
-Latest browser-suite failure(s): QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports</x:v>
+Latest browser-suite failure(s): QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts; GeometryRuntime_ExecutesBrowserWorkerAcrossFrontendsAndDeviceViewports
+Post-fix anonymous demo retest still lacks visible 3D Model tab/button.</x:v>
       </x:c>
       <x:c r="T19" s="48" t="str">
         <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1852; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
-Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx
+QuoteEngine fix commit: c926434. Targeted retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx</x:v>
       </x:c>
       <x:c r="U19" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8175,13 +8187,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="H20" s="48" t="str">
-        <x:v>Failed in latest browser suite</x:v>
+        <x:v>Failed after partial fix</x:v>
       </x:c>
       <x:c r="I20" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J20" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="K20" s="48" t="str">
         <x:v>P1</x:v>
@@ -8202,7 +8214,8 @@
         <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896)
 2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
 TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
-- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
+2026-06-23 targeted retest after QuoteEngine c926434: Demo only cue is now satisfied; remaining failure is waiting for role button '3D Model' exact at BrowserJourneyGateTests.cs:906. TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx.</x:v>
       </x:c>
       <x:c r="Q20" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; PricingService; MaterialService; DeliveryService if delivery promise affects lead time.; QuotationService in production.</x:v>
@@ -8212,11 +8225,13 @@
       </x:c>
       <x:c r="S20" s="48" t="str">
         <x:v>Define customer-visible lead-time language, cutoff times, delivery/calendar rules, and expiry behavior.
-Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
+Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts
+Post-fix anonymous demo retest still lacks visible 3D Model tab/button.</x:v>
       </x:c>
       <x:c r="T20" s="48" t="str">
         <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1909; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
-Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx
+QuoteEngine fix commit: c926434. Targeted retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx</x:v>
       </x:c>
       <x:c r="U20" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8245,13 +8260,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="H21" s="48" t="str">
-        <x:v>Failed in latest browser suite</x:v>
+        <x:v>Failed after partial fix</x:v>
       </x:c>
       <x:c r="I21" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J21" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="K21" s="48" t="str">
         <x:v>P1</x:v>
@@ -8274,7 +8289,8 @@
 TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
 - QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for Locator("header.quote-topbar .billing-account-trigger") 28 × locator resolved to &lt;summary class="billing-accou...
 - QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByRole(AriaRole.Button, new() { Name = "Parts", Exact = true })
-- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
+2026-06-23 targeted retest after QuoteEngine c926434: Demo only cue is now satisfied; remaining failure is waiting for role button '3D Model' exact at BrowserJourneyGateTests.cs:906. TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx.</x:v>
       </x:c>
       <x:c r="Q21" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; PricingService; ProjectService or quote-draft owner.; QuotationService; QuoteEnginePrototypeStore while prototype-backed.</x:v>
@@ -8284,11 +8300,13 @@
       </x:c>
       <x:c r="S21" s="48" t="str">
         <x:v>Define whether editing after formal quote creates a new quote version, cancels the old quote, or requires employee review.
-Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
+Latest browser-suite failure(s): QuoteEngine_PrototypeSignedCustomer_UploadsEstimatesQuotesOrdersAndRecordsHistory; QuoteEngine_GeometryRuntime_LoadsAcrossDeviceViewports; QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts
+Post-fix anonymous demo retest still lacks visible 3D Model tab/button.</x:v>
       </x:c>
       <x:c r="T21" s="48" t="str">
         <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:1967; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
-Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx
+QuoteEngine fix commit: c926434. Targeted retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx</x:v>
       </x:c>
       <x:c r="U21" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -8522,13 +8540,13 @@
         <x:v>Failed</x:v>
       </x:c>
       <x:c r="H25" s="48" t="str">
-        <x:v>Failed in latest browser suite</x:v>
+        <x:v>Failed after partial fix</x:v>
       </x:c>
       <x:c r="I25" s="48" t="str">
-        <x:v>Not started</x:v>
+        <x:v>In progress</x:v>
       </x:c>
       <x:c r="J25" s="48" t="str">
-        <x:v>Needs retest loop</x:v>
+        <x:v>Failed</x:v>
       </x:c>
       <x:c r="K25" s="48" t="str">
         <x:v>P1</x:v>
@@ -8549,7 +8567,8 @@
         <x:v>BrowserJourneyGateTests.QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts (Maliev.Aspire/Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs:896)
 2026-06-23 browser-suite failure batch: 14 failed, 42 passed, 0 skipped, 56 total.
 TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx.
-- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")</x:v>
+- QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts: Microsoft.Playwright.PlaywrightException : Locator expected to be visible Error: element(s) not found Call log: - Expect "ToBeVisibleAsync" with timeout 30000ms - waiting for GetByText("Demo only")
+2026-06-23 targeted retest after QuoteEngine c926434: Demo only cue is now satisfied; remaining failure is waiting for role button '3D Model' exact at BrowserJourneyGateTests.cs:906. TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx.</x:v>
       </x:c>
       <x:c r="Q25" s="48" t="str">
         <x:v>Maliev.QuoteEngine.Bff; Optional MaterialService/PricingService if demo uses live read-only reference data.; No ProjectService, QuotationService, UploadService, OrderService, PaymentService, or DeliveryService mutation.</x:v>
@@ -8559,11 +8578,13 @@
       </x:c>
       <x:c r="S25" s="48" t="str">
         <x:v>Define the demo asset catalog, disclaimer wording, and whether demo pricing uses fixed fixtures or live read-only pricing.
-Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts</x:v>
+Latest browser-suite failure(s): QuoteEngine_AnonymousDemo_EstimatesWithoutFormalArtifacts
+Post-fix anonymous demo retest still lacks visible 3D Model tab/button.</x:v>
       </x:c>
       <x:c r="T25" s="48" t="str">
         <x:v>Maliev.Aspire.Tests/specs/E2E_USER_JOURNEY_STORIES.md:2200; Maliev.Aspire.Tests/E2E/BrowserJourneyGateTests.cs
-Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx</x:v>
+Aspire E2E TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-browser-suite-20260623.trx
+QuoteEngine fix commit: c926434. Targeted retest TRX: B:/maliev/Maliev.Aspire/Maliev.Aspire.Tests/TestResults/feature-tracker-quoteengine-anonymous-demo-retest.trx</x:v>
       </x:c>
       <x:c r="U25" s="49" t="str">
         <x:v>2026-06-23</x:v>
@@ -9068,7 +9089,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R987aab7464c645fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18d6054a4d494e68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Remove QuoteEngine demo tracking
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5f9c9fb9ecd94a41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R776c36a76533485f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R106275d2e2554d29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rb5844ea2fb10437f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5783d801fc7b494a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R11b3b8e1a5784055"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd2f21f9c64bb4bf5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R42b572cbf5194a40"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -607,7 +607,7 @@
         <x:v>As a customer, I can start a quote from the web quote page, upload CAD files for an instant estimate, or hand off the session to Make Studio.</x:v>
       </x:c>
       <x:c r="E3" s="3" t="str">
-        <x:v>The quote page presents Make Studio/demo actions, accepts supported CAD uploads, tracks analysis status, returns an estimate, and can mint a signed handoff token.</x:v>
+        <x:v>The quote page presents Make Studio actions, accepts supported CAD uploads, tracks analysis status, returns an estimate, and can mint a signed handoff token.</x:v>
       </x:c>
       <x:c r="F3" s="3" t="str">
         <x:v>Current code-derived</x:v>
@@ -634,7 +634,7 @@
         <x:v>Maliev.Web.Client/Pages/Quote.razor; InstantQuotePanel.razor; QuoteDropzone.razor</x:v>
       </x:c>
       <x:c r="N3" s="3" t="str">
-        <x:v>/quote; Start in Make Studio; Try demo; quote dropzone; estimate controls</x:v>
+        <x:v>/quote; Start in Make Studio; quote dropzone; estimate controls</x:v>
       </x:c>
       <x:c r="O3" s="3" t="str">
         <x:v>QuoteController reference-data, estimate, uploads/resumable, complete, handoff-token, analysis-status</x:v>
@@ -652,7 +652,7 @@
         <x:v>Use current Make Studio handoff and API estimate behavior as canonical</x:v>
       </x:c>
       <x:c r="T3" s="3" t="str">
-        <x:v>Quote.razor:15-21; InstantQuotePanel.razor:23,139,145,215,256; QuoteUploadService.cs:13-43; QuoteUploadHandoffToken.cs</x:v>
+        <x:v>Quote.razor (Make Studio quote start); InstantQuotePanel.razor:23,139,145,215,256; QuoteUploadService.cs:13-43; QuoteUploadHandoffToken.cs</x:v>
       </x:c>
       <x:c r="U3" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -986,7 +986,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffc6791b83d14fc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3350cb6c6de4f0b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1671,7 +1671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92a7fb7af1364d3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd17a6bb574684d69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1776,13 +1776,13 @@
         <x:v>Maliev.QuoteEngine</x:v>
       </x:c>
       <x:c r="C2" s="3" t="str">
-        <x:v>Chat quote workspace routes and launch shell</x:v>
+        <x:v>Agentic manufacturing workspace routes and launch shell</x:v>
       </x:c>
       <x:c r="D2" s="3" t="str">
-        <x:v>As a customer, I can open the chat-based quote workspace at the root, quotes, new-project, or demo routes and use the rail to start/search/manage projects.</x:v>
+        <x:v>As a customer, I can open the agentic manufacturing workspace, chat with quote agents, start or search projects, and move parts through analysis and quoting.</x:v>
       </x:c>
       <x:c r="E2" s="3" t="str">
-        <x:v>The workspace routes load QuoteAgentLaunchShell, support demo mode, new project actions, projects/search pages, rail navigation, sign-in handoff, and project duplicate/pin/archive/achieve actions.</x:v>
+        <x:v>The workspace loads QuoteAgentLaunchShell, lets customers chat with manufacturing agents, upload and analyze parts, manage projects/search, and continue into quote actions.</x:v>
       </x:c>
       <x:c r="F2" s="3" t="str">
         <x:v>Current code-derived</x:v>
@@ -1803,13 +1803,13 @@
         <x:v>P0</x:v>
       </x:c>
       <x:c r="L2" s="3" t="str">
-        <x:v>Blazor workspace -&gt; QuoteEngineApiClient -&gt; quote/v1 project nav/search/actions DTOs -&gt; auth/demo state</x:v>
+        <x:v>Blazor workspace -&gt; QuoteEngineApiClient -&gt; quote/v1 project nav/search/actions DTOs -&gt; auth/session state</x:v>
       </x:c>
       <x:c r="M2" s="3" t="str">
         <x:v>QuoteWorkspace.razor; QuoteAgentLaunchShell.razor</x:v>
       </x:c>
       <x:c r="N2" s="3" t="str">
-        <x:v>@page /, /quotes, /quotes/new, /quote/new, /projects/new, /demo; rail New project/Projects/search</x:v>
+        <x:v>@page /, /quotes, /quotes/new, /quote/new, /projects/new; rail New project/Projects/search; agent chat composer</x:v>
       </x:c>
       <x:c r="O2" s="3" t="str">
         <x:v>QuoteController projects/nav/detail/duplicate/pin/archive/achieve; AgentController search</x:v>
@@ -1827,7 +1827,7 @@
         <x:v>Use current chat workspace behavior as canonical</x:v>
       </x:c>
       <x:c r="T2" s="3" t="str">
-        <x:v>QuoteWorkspace.razor:1-6,39,439,470; QuoteAgentLaunchShell.razor:36,48-54,338-474,5829-5867</x:v>
+        <x:v>QuoteWorkspace.razor:1-5,39,470; QuoteAgentLaunchShell.razor:36,48-54,338-474,5829-5867</x:v>
       </x:c>
       <x:c r="U2" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -2356,7 +2356,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rba9760ac3c574f0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R289d78b3e7ee465b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify current-only feature tracker summary
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5783d801fc7b494a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R11b3b8e1a5784055"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd2f21f9c64bb4bf5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R42b572cbf5194a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R24a0250f536c47ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re0d401d738854163"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R99dddeb2b0a54f20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf8063a35d9214f5f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -350,7 +350,6 @@
   <x:cols>
     <x:col min="1" max="1" width="34" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="71.87999725341797" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14.5" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -358,7 +357,6 @@
         <x:v>Canonical MALIEV feature user story tracker</x:v>
       </x:c>
       <x:c r="B1" s="2" t="str"/>
-      <x:c r="C1" s="2"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="3" t="str">
@@ -367,7 +365,6 @@
       <x:c r="B2" s="3" t="str">
         <x:v>2026-06-23</x:v>
       </x:c>
-      <x:c r="C2" s="3"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
@@ -376,17 +373,13 @@
       <x:c r="B3" s="3" t="str">
         <x:v>Only current code-derived user stories are tracked.</x:v>
       </x:c>
-      <x:c r="C3" s="3"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="2" t="str">
         <x:v>Service</x:v>
       </x:c>
       <x:c r="B4" s="2" t="str">
-        <x:v>Current code-derived rows</x:v>
-      </x:c>
-      <x:c r="C4" s="2" t="str">
-        <x:v>Total tracked rows</x:v>
+        <x:v>Current tracked stories</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -396,9 +389,6 @@
       <x:c r="B5" s="3" t="n">
         <x:v>7</x:v>
       </x:c>
-      <x:c r="C5" s="3" t="n">
-        <x:v>7</x:v>
-      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="3" t="str">
@@ -407,9 +397,6 @@
       <x:c r="B6" s="3" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C6" s="3" t="n">
-        <x:v>9</x:v>
-      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="3" t="str">
@@ -418,9 +405,6 @@
       <x:c r="B7" s="3" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="C7" s="3" t="n">
-        <x:v>9</x:v>
-      </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="3" t="str">
@@ -429,7 +413,6 @@
       <x:c r="B8" s="3" t="str">
         <x:v>Test every current code-derived user story, document errors, fix logistical/UX issues, then retest.</x:v>
       </x:c>
-      <x:c r="C8" s="3"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -459,7 +442,7 @@
     <x:col min="17" max="17" width="50.5" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="48.25" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="55.25" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="94.87999725341797" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="109.5" hidden="0" customWidth="1"/>
     <x:col min="21" max="21" width="13.880000114440918" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
@@ -986,7 +969,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd3350cb6c6de4f0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4831fb5f19174170"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1292,7 +1275,7 @@
         <x:v>As sales staff, I can triage web contact requests and create, search, edit, merge, tag, and review customers.</x:v>
       </x:c>
       <x:c r="E5" s="3" t="str">
-        <x:v>Customer/contact request pages route to controllers for list/detail/create/update, address/contact/company data, and legacy customer redirects remain supported.</x:v>
+        <x:v>Customer/contact request pages route to controllers for list/detail/create/update, address/contact/company data, and supported customer routes.</x:v>
       </x:c>
       <x:c r="F5" s="3" t="str">
         <x:v>Current code-derived</x:v>
@@ -1334,7 +1317,7 @@
         <x:v>Customer records, contact requests, addresses/tags</x:v>
       </x:c>
       <x:c r="S5" s="3" t="str">
-        <x:v>Needs browser retest of legacy redirect routes</x:v>
+        <x:v>Needs browser retest of supported customer routes</x:v>
       </x:c>
       <x:c r="T5" s="3" t="str">
         <x:v>CustomersController.cs:20,35,51,134,167,176,185,199,250,264,278,439,456; Contact request pages</x:v>
@@ -1671,7 +1654,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd17a6bb574684d69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R047060b36b884c0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1693,7 +1676,7 @@
     <x:col min="11" max="11" width="8.75" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="112" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="75.87999725341797" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="84.37999725341797" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="86.75" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="123.37999725341797" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="94.87999725341797" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="59.880001068115234" hidden="0" customWidth="1"/>
@@ -2356,7 +2339,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R289d78b3e7ee465b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2865fd51e543456d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record focused feature tracker test evidence
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4951e6e7fb174d34"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3cbbc007e1394284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Re06731d698074229"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R197f169ab6464859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re086ce504db64dbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3b20f9a852e646df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R45c978b042fe44c3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf844fe5811ef441b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -604,16 +604,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Needs manual / browser test</x:v>
+        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in focused source tests.</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from focused tests.</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Pending browser/runtime verification.</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>P2</x:v>
@@ -630,7 +630,9 @@
       <x:c r="O3" s="3" t="str">
         <x:v>Static content model</x:v>
       </x:c>
-      <x:c r="P3" s="3" t="str"/>
+      <x:c r="P3" s="3" t="str">
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23.</x:v>
+      </x:c>
       <x:c r="Q3" s="3" t="str">
         <x:v>Web client</x:v>
       </x:c>
@@ -667,16 +669,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Needs manual / browser test</x:v>
+        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in focused source tests.</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from focused tests.</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Pending browser/runtime verification.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
         <x:v>P2</x:v>
@@ -693,7 +695,9 @@
       <x:c r="O4" s="3" t="str">
         <x:v>Static content model</x:v>
       </x:c>
-      <x:c r="P4" s="3" t="str"/>
+      <x:c r="P4" s="3" t="str">
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23.</x:v>
+      </x:c>
       <x:c r="Q4" s="3" t="str">
         <x:v>Web client</x:v>
       </x:c>
@@ -990,16 +994,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
-        <x:v>Needs manual / browser test</x:v>
+        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in focused source tests.</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from focused tests.</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Pending browser/runtime verification.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>P1</x:v>
@@ -1016,7 +1020,9 @@
       <x:c r="O9" s="3" t="str">
         <x:v>CheckoutController draft endpoints used after cart</x:v>
       </x:c>
-      <x:c r="P9" s="3" t="str"/>
+      <x:c r="P9" s="3" t="str">
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn passed as part of 4/4 focused Web run on 2026-06-23.</x:v>
+      </x:c>
       <x:c r="Q9" s="3" t="str">
         <x:v>Web client, Checkout BFF</x:v>
       </x:c>
@@ -2223,16 +2229,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Needs manual / browser test</x:v>
+        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in focused source tests.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from focused tests.</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Pending browser/runtime verification.</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
         <x:v>P2</x:v>
@@ -2249,7 +2255,9 @@
       <x:c r="O28" s="3" t="str">
         <x:v>BlogController for ebook PDF only</x:v>
       </x:c>
-      <x:c r="P28" s="3" t="str"/>
+      <x:c r="P28" s="3" t="str">
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary passed as part of 4/4 focused Web run on 2026-06-23.</x:v>
+      </x:c>
       <x:c r="Q28" s="3" t="str">
         <x:v>Web client, Content</x:v>
       </x:c>
@@ -2399,7 +2407,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8f69ea83b5bd4390"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4273a98aa13480a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2581,16 +2589,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Needs manual / browser test</x:v>
+        <x:v>Focused automated component/controller tests passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in focused tests. Initial concurrent repo run hit shared ServiceDefaults obj lock; serialized rerun passed.</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Test orchestration adjusted: run Web/Intranet dotnet tests serially when they share ServiceDefaults build outputs.</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Serialized focused retest passed 15/15; browser/runtime verification pending.</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>P1</x:v>
@@ -2607,7 +2615,9 @@
       <x:c r="O3" s="3" t="str">
         <x:v>DashboardController GET, action-items</x:v>
       </x:c>
-      <x:c r="P3" s="3" t="str"/>
+      <x:c r="P3" s="3" t="str">
+        <x:v>dotnet test Maliev.Intranet.slnx --filter Phase3DashboardTests|DashboardControllerTests|QuickControllerTests.Dashboard_Get_ReturnsOk passed 15/15 on 2026-06-23 after serialized rerun.</x:v>
+      </x:c>
       <x:c r="Q3" s="3" t="str">
         <x:v>Intranet BFF, operational services</x:v>
       </x:c>
@@ -5357,7 +5367,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R538fcc7d41c54202"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa82a720634c4d56"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7927,7 +7937,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46467e2fa42b4a7b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6570a1d1c6d044cd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Web feature suite evidence
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re086ce504db64dbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3b20f9a852e646df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R45c978b042fe44c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf844fe5811ef441b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra98dcfe6fa48452c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rff19ee7921e742a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R1f8cd9d0fd924061"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R525223cc4eea4a01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -539,16 +539,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
         <x:v>P1</x:v>
@@ -566,7 +566,7 @@
         <x:v>SeoController robots/sitemap for crawl entry points</x:v>
       </x:c>
       <x:c r="P2" s="3" t="str">
-        <x:v>WebBffEndpointTests Seo</x:v>
+        <x:v>WebBffEndpointTests Seo | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="str">
         <x:v>Web client, Web BFF, content/static assets</x:v>
@@ -604,16 +604,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>No behavior error observed in focused source tests.</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>No fix needed from focused tests.</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Pending browser/runtime verification.</x:v>
+        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>P2</x:v>
@@ -631,7 +631,7 @@
         <x:v>Static content model</x:v>
       </x:c>
       <x:c r="P3" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23.</x:v>
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="str">
         <x:v>Web client</x:v>
@@ -669,16 +669,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>No behavior error observed in focused source tests.</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>No fix needed from focused tests.</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>Pending browser/runtime verification.</x:v>
+        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
         <x:v>P2</x:v>
@@ -696,7 +696,7 @@
         <x:v>Static content model</x:v>
       </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23.</x:v>
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="str">
         <x:v>Web client</x:v>
@@ -734,16 +734,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I5" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J5" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K5" s="3" t="str">
         <x:v>P1</x:v>
@@ -761,7 +761,7 @@
         <x:v>MaterialsController datasheet endpoint</x:v>
       </x:c>
       <x:c r="P5" s="3" t="str">
-        <x:v>WebBffEndpointTests Materials</x:v>
+        <x:v>WebBffEndpointTests Materials | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="str">
         <x:v>Web client, Web BFF, PDF generation/storage</x:v>
@@ -799,16 +799,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I6" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K6" s="3" t="str">
         <x:v>P1</x:v>
@@ -826,7 +826,7 @@
         <x:v>MaterialsController GET {slug}/datasheet.pdf</x:v>
       </x:c>
       <x:c r="P6" s="3" t="str">
-        <x:v>WebBffEndpointTests Materials</x:v>
+        <x:v>WebBffEndpointTests Materials | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="str">
         <x:v>Web BFF, PDF service/content</x:v>
@@ -864,16 +864,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I7" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J7" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K7" s="3" t="str">
         <x:v>P1</x:v>
@@ -891,7 +891,7 @@
         <x:v>CatalogController collections, products, media, collection image</x:v>
       </x:c>
       <x:c r="P7" s="3" t="str">
-        <x:v>CommerceCatalogBoundaryTests; WebBffEndpointTests Catalog</x:v>
+        <x:v>CommerceCatalogBoundaryTests; WebBffEndpointTests Catalog | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="str">
         <x:v>Web BFF, Catalog/Commerce, Storage</x:v>
@@ -929,16 +929,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
         <x:v>P1</x:v>
@@ -956,7 +956,7 @@
         <x:v>CatalogController GET products/{handle}</x:v>
       </x:c>
       <x:c r="P8" s="3" t="str">
-        <x:v>CommerceCatalogBoundaryTests</x:v>
+        <x:v>CommerceCatalogBoundaryTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="str">
         <x:v>Web BFF, Catalog/Commerce</x:v>
@@ -994,16 +994,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
-        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>No behavior error observed in focused source tests.</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>No fix needed from focused tests.</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>Pending browser/runtime verification.</x:v>
+        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>P1</x:v>
@@ -1021,7 +1021,7 @@
         <x:v>CheckoutController draft endpoints used after cart</x:v>
       </x:c>
       <x:c r="P9" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn passed as part of 4/4 focused Web run on 2026-06-23.</x:v>
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn passed as part of 4/4 focused Web run on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="str">
         <x:v>Web client, Checkout BFF</x:v>
@@ -1059,16 +1059,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K10" s="3" t="str">
         <x:v>P1</x:v>
@@ -1086,7 +1086,7 @@
         <x:v>CheckoutController POST draft, draft-form</x:v>
       </x:c>
       <x:c r="P10" s="3" t="str">
-        <x:v>CheckoutControllerTests; CheckoutDraftServiceTests</x:v>
+        <x:v>CheckoutControllerTests; CheckoutDraftServiceTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="str">
         <x:v>Web BFF, Checkout/Order services</x:v>
@@ -1124,16 +1124,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J11" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K11" s="3" t="str">
         <x:v>P1</x:v>
@@ -1151,7 +1151,7 @@
         <x:v>ShippingController GET couriers, POST rates</x:v>
       </x:c>
       <x:c r="P11" s="3" t="str">
-        <x:v>ShippingControllerTests</x:v>
+        <x:v>ShippingControllerTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="str">
         <x:v>Web BFF, DeliveryService</x:v>
@@ -1189,16 +1189,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K12" s="3" t="str">
         <x:v>P2</x:v>
@@ -1216,7 +1216,7 @@
         <x:v>ShippingController GET tracking/{trackingCode}</x:v>
       </x:c>
       <x:c r="P12" s="3" t="str">
-        <x:v>ShippingControllerTests</x:v>
+        <x:v>ShippingControllerTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="str">
         <x:v>Web BFF, DeliveryService</x:v>
@@ -1254,16 +1254,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J13" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K13" s="3" t="str">
         <x:v>P0</x:v>
@@ -1281,7 +1281,7 @@
         <x:v>QuoteController reference-data, estimate, uploads/resumable, complete, handoff-token, analysis-status</x:v>
       </x:c>
       <x:c r="P13" s="3" t="str">
-        <x:v>WebBffEndpointTests Quote*</x:v>
+        <x:v>WebBffEndpointTests Quote* | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="str">
         <x:v>Web BFF, QuoteEngine, Storage, Geometry/Pricing</x:v>
@@ -1319,16 +1319,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J14" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K14" s="3" t="str">
         <x:v>P0</x:v>
@@ -1346,7 +1346,7 @@
         <x:v>QuoteController uploads/resumable, PUT chunk, complete, analysis-status</x:v>
       </x:c>
       <x:c r="P14" s="3" t="str">
-        <x:v>WebBffEndpointTests QuoteUpload*</x:v>
+        <x:v>WebBffEndpointTests QuoteUpload* | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="str">
         <x:v>Web BFF, Storage, Geometry/analysis</x:v>
@@ -1384,16 +1384,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J15" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K15" s="3" t="str">
         <x:v>P0</x:v>
@@ -1411,7 +1411,7 @@
         <x:v>QuoteController POST estimate</x:v>
       </x:c>
       <x:c r="P15" s="3" t="str">
-        <x:v>WebBffEndpointTests QuoteEstimate</x:v>
+        <x:v>WebBffEndpointTests QuoteEstimate | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="str">
         <x:v>Web BFF, Pricing/Quote services</x:v>
@@ -1449,16 +1449,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G16" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H16" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J16" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K16" s="3" t="str">
         <x:v>P1</x:v>
@@ -1476,7 +1476,7 @@
         <x:v>ChatbotController POST sessions/messages</x:v>
       </x:c>
       <x:c r="P16" s="3" t="str">
-        <x:v>CustomerChatbotBoundaryTests; WebBffEndpointTests Chatbot*</x:v>
+        <x:v>CustomerChatbotBoundaryTests; WebBffEndpointTests Chatbot* | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="str">
         <x:v>Web BFF, Chatbot/agent backend, Auth</x:v>
@@ -1514,16 +1514,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H17" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K17" s="3" t="str">
         <x:v>P0</x:v>
@@ -1541,7 +1541,7 @@
         <x:v>AuthController google, callback, sign-in/email, sign-up/email, passkey-sign-in</x:v>
       </x:c>
       <x:c r="P17" s="3" t="str">
-        <x:v>AccountControllerBoundaryTests; WebBffEndpointTests</x:v>
+        <x:v>AccountControllerBoundaryTests; WebBffEndpointTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="str">
         <x:v>Web BFF, AuthService, CustomerService</x:v>
@@ -1579,16 +1579,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
         <x:v>P1</x:v>
@@ -1606,7 +1606,7 @@
         <x:v>AuthController forgot-password/request, reset-password/confirm</x:v>
       </x:c>
       <x:c r="P18" s="3" t="str">
-        <x:v>WebBffEndpointTests Auth where present</x:v>
+        <x:v>WebBffEndpointTests Auth where present | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="str">
         <x:v>Web BFF, AuthService</x:v>
@@ -1644,16 +1644,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G19" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H19" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J19" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K19" s="3" t="str">
         <x:v>P1</x:v>
@@ -1671,7 +1671,7 @@
         <x:v>AuthController verify-email, refresh-claims, resend-verification</x:v>
       </x:c>
       <x:c r="P19" s="3" t="str">
-        <x:v>AccountControllerBoundaryTests</x:v>
+        <x:v>AccountControllerBoundaryTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="str">
         <x:v>Web BFF, AuthService</x:v>
@@ -1709,16 +1709,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G20" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H20" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J20" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K20" s="3" t="str">
         <x:v>P1</x:v>
@@ -1736,7 +1736,7 @@
         <x:v>AccountController session, profile GET/PATCH</x:v>
       </x:c>
       <x:c r="P20" s="3" t="str">
-        <x:v>AccountControllerBoundaryTests; WebBffEndpointTests Account</x:v>
+        <x:v>AccountControllerBoundaryTests; WebBffEndpointTests Account | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="str">
         <x:v>Web BFF, CustomerService, AuthService</x:v>
@@ -1774,16 +1774,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G21" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H21" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J21" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K21" s="3" t="str">
         <x:v>P2</x:v>
@@ -1801,7 +1801,7 @@
         <x:v>AccountController email/change, email/resend-change</x:v>
       </x:c>
       <x:c r="P21" s="3" t="str">
-        <x:v>AccountControllerBoundaryTests</x:v>
+        <x:v>AccountControllerBoundaryTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="str">
         <x:v>Web BFF, AuthService</x:v>
@@ -1839,16 +1839,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G22" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H22" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J22" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K22" s="3" t="str">
         <x:v>P1</x:v>
@@ -1866,7 +1866,7 @@
         <x:v>AccountController addresses GET/POST/PATCH/DELETE</x:v>
       </x:c>
       <x:c r="P22" s="3" t="str">
-        <x:v>AccountAddressGoogleSourceTests; AccountControllerBoundaryTests</x:v>
+        <x:v>AccountAddressGoogleSourceTests; AccountControllerBoundaryTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="str">
         <x:v>Web BFF, CustomerService</x:v>
@@ -1904,16 +1904,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H23" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J23" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K23" s="3" t="str">
         <x:v>P2</x:v>
@@ -1931,7 +1931,7 @@
         <x:v>AddressController google-config, static-map, countries, thai-locations</x:v>
       </x:c>
       <x:c r="P23" s="3" t="str">
-        <x:v>AccountAddressGoogleSourceTests</x:v>
+        <x:v>AccountAddressGoogleSourceTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="str">
         <x:v>Web BFF, Country/Registry/Google config</x:v>
@@ -1969,16 +1969,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J24" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K24" s="3" t="str">
         <x:v>P1</x:v>
@@ -1996,7 +1996,7 @@
         <x:v>AccountController orders</x:v>
       </x:c>
       <x:c r="P24" s="3" t="str">
-        <x:v>WebBffEndpointTests AccountOrders</x:v>
+        <x:v>WebBffEndpointTests AccountOrders | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="str">
         <x:v>Web BFF, OrderService</x:v>
@@ -2034,16 +2034,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H25" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J25" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K25" s="3" t="str">
         <x:v>P2</x:v>
@@ -2061,7 +2061,7 @@
         <x:v>AccountController company-search</x:v>
       </x:c>
       <x:c r="P25" s="3" t="str">
-        <x:v>AccountControllerBoundaryTests</x:v>
+        <x:v>AccountControllerBoundaryTests | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="str">
         <x:v>Web BFF, RegistryService, CustomerService</x:v>
@@ -2099,16 +2099,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G26" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H26" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J26" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K26" s="3" t="str">
         <x:v>P2</x:v>
@@ -2126,7 +2126,7 @@
         <x:v>PreferencesController POST culture</x:v>
       </x:c>
       <x:c r="P26" s="3" t="str">
-        <x:v>WebBffEndpointTests Preferences</x:v>
+        <x:v>WebBffEndpointTests Preferences | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="str">
         <x:v>Web BFF</x:v>
@@ -2164,16 +2164,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
         <x:v>P1</x:v>
@@ -2191,7 +2191,7 @@
         <x:v>ContactController POST messages</x:v>
       </x:c>
       <x:c r="P27" s="3" t="str">
-        <x:v>WebBffEndpointTests Contact</x:v>
+        <x:v>WebBffEndpointTests Contact | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="str">
         <x:v>Web BFF, Contact/customer workflow</x:v>
@@ -2229,16 +2229,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Focused automated source tests passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>No behavior error observed in focused source tests.</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>No fix needed from focused tests.</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>Pending browser/runtime verification.</x:v>
+        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
         <x:v>P2</x:v>
@@ -2256,7 +2256,7 @@
         <x:v>BlogController for ebook PDF only</x:v>
       </x:c>
       <x:c r="P28" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary passed as part of 4/4 focused Web run on 2026-06-23.</x:v>
+        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary passed as part of 4/4 focused Web run on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="str">
         <x:v>Web client, Content</x:v>
@@ -2294,16 +2294,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H29" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J29" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K29" s="3" t="str">
         <x:v>P2</x:v>
@@ -2321,7 +2321,7 @@
         <x:v>BlogController GET {slug}/ebook.pdf</x:v>
       </x:c>
       <x:c r="P29" s="3" t="str">
-        <x:v>WebBffEndpointTests Blog</x:v>
+        <x:v>WebBffEndpointTests Blog | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="str">
         <x:v>Web BFF, PDF service/content</x:v>
@@ -2359,16 +2359,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Web suite passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H30" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Web automated suite.</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed from current Web automated suite.</x:v>
       </x:c>
       <x:c r="J30" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K30" s="3" t="str">
         <x:v>P2</x:v>
@@ -2386,7 +2386,7 @@
         <x:v>SeoController GET robots/sitemap</x:v>
       </x:c>
       <x:c r="P30" s="3" t="str">
-        <x:v>WebBffEndpointTests Seo</x:v>
+        <x:v>WebBffEndpointTests Seo | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="str">
         <x:v>Web BFF</x:v>
@@ -2407,7 +2407,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4273a98aa13480a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b7fedd2906d46de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5367,7 +5367,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfa82a720634c4d56"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3e48ec792d04b21"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7937,7 +7937,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6570a1d1c6d044cd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e6da95d07ed4e68"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record Intranet suite fix evidence
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra98dcfe6fa48452c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rff19ee7921e742a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R1f8cd9d0fd924061"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R525223cc4eea4a01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rec5d5323eb5d4efc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R44ee5cd5ca9141cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rdbfe439a58d546f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R3cf2b7afc2d2492b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2407,7 +2407,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b7fedd2906d46de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a0e07831f964eb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2524,16 +2524,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
         <x:v>P0</x:v>
@@ -2551,7 +2551,7 @@
         <x:v>AuthController user/session endpoints</x:v>
       </x:c>
       <x:c r="P2" s="3" t="str">
-        <x:v>Navigation/source tests where present</x:v>
+        <x:v>Navigation/source tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="str">
         <x:v>Intranet client, BFF, Auth/IAM</x:v>
@@ -2589,16 +2589,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Focused automated component/controller tests passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix; browser runtime pending</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>No behavior error observed in focused tests. Initial concurrent repo run hit shared ServiceDefaults obj lock; serialized rerun passed.</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>Test orchestration adjusted: run Web/Intranet dotnet tests serially when they share ServiceDefaults build outputs.</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Serialized focused retest passed 15/15; browser/runtime verification pending.</x:v>
+        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>P1</x:v>
@@ -2616,7 +2616,7 @@
         <x:v>DashboardController GET, action-items</x:v>
       </x:c>
       <x:c r="P3" s="3" t="str">
-        <x:v>dotnet test Maliev.Intranet.slnx --filter Phase3DashboardTests|DashboardControllerTests|QuickControllerTests.Dashboard_Get_ReturnsOk passed 15/15 on 2026-06-23 after serialized rerun.</x:v>
+        <x:v>dotnet test Maliev.Intranet.slnx --filter Phase3DashboardTests|DashboardControllerTests|QuickControllerTests.Dashboard_Get_ReturnsOk passed 15/15 on 2026-06-23 after serialized rerun. | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="str">
         <x:v>Intranet BFF, operational services</x:v>
@@ -2654,16 +2654,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
         <x:v>P1</x:v>
@@ -2681,7 +2681,7 @@
         <x:v>SearchController GET</x:v>
       </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>Search/source tests where present</x:v>
+        <x:v>Search/source tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="str">
         <x:v>Intranet BFF, SearchService</x:v>
@@ -2719,16 +2719,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I5" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J5" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K5" s="3" t="str">
         <x:v>P1</x:v>
@@ -2746,7 +2746,7 @@
         <x:v>Chatbot/admin instruction endpoints where configured</x:v>
       </x:c>
       <x:c r="P5" s="3" t="str">
-        <x:v>ChatDrawer source tests where present</x:v>
+        <x:v>ChatDrawer source tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="str">
         <x:v>Intranet client, Chatbot/agent service</x:v>
@@ -2784,16 +2784,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I6" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K6" s="3" t="str">
         <x:v>P1</x:v>
@@ -2811,7 +2811,7 @@
         <x:v>AlertsController GET, read, read-all</x:v>
       </x:c>
       <x:c r="P6" s="3" t="str">
-        <x:v>NotificationBell tests where present</x:v>
+        <x:v>NotificationBell tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="str">
         <x:v>Intranet BFF, Alerts/Notification data</x:v>
@@ -2849,16 +2849,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I7" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J7" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K7" s="3" t="str">
         <x:v>P0</x:v>
@@ -2876,7 +2876,7 @@
         <x:v>ProjectsController GET/list/detail/update/delete/notes/duplicate/thumbnail</x:v>
       </x:c>
       <x:c r="P7" s="3" t="str">
-        <x:v>ProjectsControllerTests</x:v>
+        <x:v>ProjectsControllerTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="str">
         <x:v>Intranet BFF, Project/Quote services, Storage</x:v>
@@ -2914,16 +2914,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
         <x:v>P0</x:v>
@@ -2941,7 +2941,7 @@
         <x:v>UploadsController upload/batch/resumable/complete/chunk/status/viewer-url/preview-url/migrate-project</x:v>
       </x:c>
       <x:c r="P8" s="3" t="str">
-        <x:v>ProjectNewAutoSaveTests; UploadsControllerResumableTests</x:v>
+        <x:v>ProjectNewAutoSaveTests; UploadsControllerResumableTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="str">
         <x:v>Intranet BFF, Storage, GeometryService, UploadService</x:v>
@@ -2979,16 +2979,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>P0</x:v>
@@ -3006,7 +3006,7 @@
         <x:v>ProjectsController POST/PUT project endpoints</x:v>
       </x:c>
       <x:c r="P9" s="3" t="str">
-        <x:v>ProjectNewAutoSaveTests</x:v>
+        <x:v>ProjectNewAutoSaveTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="str">
         <x:v>Intranet client/BFF, Project service</x:v>
@@ -3044,16 +3044,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Failed current Intranet suite, fixed, and retested passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>Initial full Intranet suite failed 1/1150: shipping text/numeric fields in PartConfigSidebar and QuoteSummaryBar updated on blur instead of on input.</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed in Maliev.Intranet commit bb9a51c by adding Immediate="true" to the reported shipping text/numeric fields.</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Retested: regression 1/1 passed, impacted focused set 138/138 passed, full Intranet suite 1143 passed / 7 skipped / 0 failed.</x:v>
       </x:c>
       <x:c r="K10" s="3" t="str">
         <x:v>P0</x:v>
@@ -3071,7 +3071,7 @@
         <x:v>ProjectsController parts create/update/delete; ManufacturingCatalogController processes/materials/finishes/tolerances/config-options</x:v>
       </x:c>
       <x:c r="P10" s="3" t="str">
-        <x:v>PartConfigSidebarTests; ProjectNewAutoSaveTests</x:v>
+        <x:v>PartConfigSidebarTests; ProjectNewAutoSaveTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur. | Fix verification: ClientTextInputs_UpdateOnInputInsteadOfBlur passed 1/1; PartConfigSidebar/QuoteSummaryBar/ModuleRegressionSourceTests focused set passed 138/138.</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="str">
         <x:v>Intranet BFF, MaterialService, PricingService</x:v>
@@ -3083,7 +3083,7 @@
         <x:v>Needs process-specific UX browser pass</x:v>
       </x:c>
       <x:c r="T10" s="3" t="str">
-        <x:v>ProjectsController.cs:298-365; ManufacturingCatalogController.cs:17-107</x:v>
+        <x:v>ProjectsController.cs:298-365; ManufacturingCatalogController.cs:17-107; PartConfigSidebar.razor:1129-1139; QuoteSummaryBar.razor:144-154</x:v>
       </x:c>
       <x:c r="U10" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -3109,16 +3109,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J11" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K11" s="3" t="str">
         <x:v>P0</x:v>
@@ -3136,7 +3136,7 @@
         <x:v>GeometryController manifest/assets/telemetry/dfm</x:v>
       </x:c>
       <x:c r="P11" s="3" t="str">
-        <x:v>GeometryControllerTests; Dfm* tests</x:v>
+        <x:v>GeometryControllerTests; Dfm* tests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="str">
         <x:v>Intranet BFF, GeometryService, browser runtime</x:v>
@@ -3174,16 +3174,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K12" s="3" t="str">
         <x:v>P0</x:v>
@@ -3201,7 +3201,7 @@
         <x:v>PricingController snapshots/calculate/accept/lead-times/bulk/finish-options</x:v>
       </x:c>
       <x:c r="P12" s="3" t="str">
-        <x:v>PricingControllerTests; QuoteSummaryBarTests</x:v>
+        <x:v>PricingControllerTests; QuoteSummaryBarTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="str">
         <x:v>Intranet BFF, PricingService, MaterialService</x:v>
@@ -3239,16 +3239,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Failed current Intranet suite, fixed, and retested passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>Initial full Intranet suite failed 1/1150: shipping text/numeric fields in PartConfigSidebar and QuoteSummaryBar updated on blur instead of on input.</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed in Maliev.Intranet commit bb9a51c by adding Immediate="true" to the reported shipping text/numeric fields.</x:v>
       </x:c>
       <x:c r="J13" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Retested: regression 1/1 passed, impacted focused set 138/138 passed, full Intranet suite 1143 passed / 7 skipped / 0 failed.</x:v>
       </x:c>
       <x:c r="K13" s="3" t="str">
         <x:v>P0</x:v>
@@ -3266,7 +3266,7 @@
         <x:v>QuotationsController; ProjectsController generate-quotation/accept-quotation</x:v>
       </x:c>
       <x:c r="P13" s="3" t="str">
-        <x:v>ProjectsControllerTests; quotation/PDF tests</x:v>
+        <x:v>ProjectsControllerTests; quotation/PDF tests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur. | Fix verification: ClientTextInputs_UpdateOnInputInsteadOfBlur passed 1/1; PartConfigSidebar/QuoteSummaryBar/ModuleRegressionSourceTests focused set passed 138/138.</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="str">
         <x:v>Intranet BFF, QuotationService, PdfService, Storage</x:v>
@@ -3278,7 +3278,7 @@
         <x:v>Needs PDF visual regression pass</x:v>
       </x:c>
       <x:c r="T13" s="3" t="str">
-        <x:v>QuotationsController.cs:20-346; ProjectsController.cs:383,513</x:v>
+        <x:v>QuotationsController.cs:20-346; ProjectsController.cs:383,513; PartConfigSidebar.razor:1129-1139; QuoteSummaryBar.razor:144-154</x:v>
       </x:c>
       <x:c r="U13" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -3304,16 +3304,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J14" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K14" s="3" t="str">
         <x:v>P1</x:v>
@@ -3331,7 +3331,7 @@
         <x:v>ProjectsController production-plan, planning-hold CRUD, routing</x:v>
       </x:c>
       <x:c r="P14" s="3" t="str">
-        <x:v>ProjectsControllerTests</x:v>
+        <x:v>ProjectsControllerTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="str">
         <x:v>Intranet BFF, Manufacturing/Planning services</x:v>
@@ -3369,16 +3369,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J15" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K15" s="3" t="str">
         <x:v>P1</x:v>
@@ -3396,7 +3396,7 @@
         <x:v>OrderLifecycleController GET; order endpoints in BFF</x:v>
       </x:c>
       <x:c r="P15" s="3" t="str">
-        <x:v>Order tests where present</x:v>
+        <x:v>Order tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="str">
         <x:v>Intranet BFF, OrderService</x:v>
@@ -3434,16 +3434,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G16" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H16" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J16" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K16" s="3" t="str">
         <x:v>P1</x:v>
@@ -3461,7 +3461,7 @@
         <x:v>CustomersController list/detail/payment-terms/create/update and related customer actions</x:v>
       </x:c>
       <x:c r="P16" s="3" t="str">
-        <x:v>Customer controller/source tests</x:v>
+        <x:v>Customer controller/source tests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="str">
         <x:v>Intranet BFF, CustomerService, RegistryService</x:v>
@@ -3499,16 +3499,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H17" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K17" s="3" t="str">
         <x:v>P1</x:v>
@@ -3526,7 +3526,7 @@
         <x:v>CompaniesController GET/search/POST/detail/primary-contact/PATCH</x:v>
       </x:c>
       <x:c r="P17" s="3" t="str">
-        <x:v>Company/customer tests where present</x:v>
+        <x:v>Company/customer tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="str">
         <x:v>Intranet BFF, CustomerService, RegistryService</x:v>
@@ -3564,16 +3564,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
         <x:v>P1</x:v>
@@ -3591,7 +3591,7 @@
         <x:v>Contact request controllers/services</x:v>
       </x:c>
       <x:c r="P18" s="3" t="str">
-        <x:v>Contact request tests where present</x:v>
+        <x:v>Contact request tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="str">
         <x:v>Intranet BFF, Customer/Contact service</x:v>
@@ -3629,16 +3629,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G19" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H19" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J19" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K19" s="3" t="str">
         <x:v>P1</x:v>
@@ -3656,7 +3656,7 @@
         <x:v>CommerceController collection/product/media endpoints</x:v>
       </x:c>
       <x:c r="P19" s="3" t="str">
-        <x:v>Commerce controller tests</x:v>
+        <x:v>Commerce controller tests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="str">
         <x:v>Intranet BFF, Catalog/Commerce, Storage</x:v>
@@ -3694,16 +3694,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G20" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H20" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J20" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K20" s="3" t="str">
         <x:v>P1</x:v>
@@ -3721,7 +3721,7 @@
         <x:v>Content/chatbot admin controllers/services</x:v>
       </x:c>
       <x:c r="P20" s="3" t="str">
-        <x:v>Content tests where present</x:v>
+        <x:v>Content tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="str">
         <x:v>Intranet BFF, Content/Chatbot service</x:v>
@@ -3759,16 +3759,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G21" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H21" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J21" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K21" s="3" t="str">
         <x:v>P1</x:v>
@@ -3786,7 +3786,7 @@
         <x:v>AccountingController accounts-tree, journal-entries, reports, periods, reconciliation, documents</x:v>
       </x:c>
       <x:c r="P21" s="3" t="str">
-        <x:v>Accounting tests where present</x:v>
+        <x:v>Accounting tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="str">
         <x:v>Intranet BFF, AccountingService, PdfService, Storage</x:v>
@@ -3824,16 +3824,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G22" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H22" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J22" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K22" s="3" t="str">
         <x:v>P1</x:v>
@@ -3851,7 +3851,7 @@
         <x:v>Invoices/Billing/CreditTerms/Receipts controllers</x:v>
       </x:c>
       <x:c r="P22" s="3" t="str">
-        <x:v>Invoice tests where present</x:v>
+        <x:v>Invoice tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="str">
         <x:v>Intranet BFF, InvoiceService, AccountingService</x:v>
@@ -3889,16 +3889,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H23" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J23" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K23" s="3" t="str">
         <x:v>P2</x:v>
@@ -3916,7 +3916,7 @@
         <x:v>BillingNotesController GET/POST/detail; CreditTermsController GET</x:v>
       </x:c>
       <x:c r="P23" s="3" t="str">
-        <x:v>Finance tests where present</x:v>
+        <x:v>Finance tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="str">
         <x:v>Intranet BFF, InvoiceService</x:v>
@@ -3954,16 +3954,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J24" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K24" s="3" t="str">
         <x:v>P1</x:v>
@@ -3981,7 +3981,7 @@
         <x:v>ReceiptsController GET/detail/POST/void</x:v>
       </x:c>
       <x:c r="P24" s="3" t="str">
-        <x:v>Receipt tests where present</x:v>
+        <x:v>Receipt tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="str">
         <x:v>Intranet BFF, ReceiptService</x:v>
@@ -4019,16 +4019,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H25" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J25" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K25" s="3" t="str">
         <x:v>P1</x:v>
@@ -4046,7 +4046,7 @@
         <x:v>DeliveryNotesController endpoints</x:v>
       </x:c>
       <x:c r="P25" s="3" t="str">
-        <x:v>Delivery note tests where present</x:v>
+        <x:v>Delivery note tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="str">
         <x:v>Intranet BFF, DeliveryService, Storage/Pdf</x:v>
@@ -4084,16 +4084,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G26" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Failed current Intranet suite, fixed, and retested passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H26" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>Initial full Intranet suite failed 1/1150: shipping text/numeric fields in PartConfigSidebar and QuoteSummaryBar updated on blur instead of on input.</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed in Maliev.Intranet commit bb9a51c by adding Immediate="true" to the reported shipping text/numeric fields.</x:v>
       </x:c>
       <x:c r="J26" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Retested: regression 1/1 passed, impacted focused set 138/138 passed, full Intranet suite 1143 passed / 7 skipped / 0 failed.</x:v>
       </x:c>
       <x:c r="K26" s="3" t="str">
         <x:v>P2</x:v>
@@ -4111,7 +4111,7 @@
         <x:v>ShippingController GET couriers, POST rates, GET tracking</x:v>
       </x:c>
       <x:c r="P26" s="3" t="str">
-        <x:v>Shipping tests where present</x:v>
+        <x:v>Shipping tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur. | Fix verification: ClientTextInputs_UpdateOnInputInsteadOfBlur passed 1/1; PartConfigSidebar/QuoteSummaryBar/ModuleRegressionSourceTests focused set passed 138/138.</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="str">
         <x:v>Intranet BFF, DeliveryService</x:v>
@@ -4123,7 +4123,7 @@
         <x:v>Needs invalid carrier/tracking coverage</x:v>
       </x:c>
       <x:c r="T26" s="3" t="str">
-        <x:v>ShippingController.cs:15-70</x:v>
+        <x:v>ShippingController.cs:15-70; PartConfigSidebar.razor:1129-1139; QuoteSummaryBar.razor:144-154</x:v>
       </x:c>
       <x:c r="U26" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -4149,16 +4149,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
         <x:v>P1</x:v>
@@ -4176,7 +4176,7 @@
         <x:v>ProcurementController GET/detail/POST/approve/send/receive/cancel/files/export</x:v>
       </x:c>
       <x:c r="P27" s="3" t="str">
-        <x:v>Procurement tests where present</x:v>
+        <x:v>Procurement tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="str">
         <x:v>Intranet BFF, PurchaseOrderService, UploadService</x:v>
@@ -4214,16 +4214,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
         <x:v>P1</x:v>
@@ -4241,7 +4241,7 @@
         <x:v>SuppliersController endpoints</x:v>
       </x:c>
       <x:c r="P28" s="3" t="str">
-        <x:v>Supplier tests where present</x:v>
+        <x:v>Supplier tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="str">
         <x:v>Intranet BFF, SupplierService, RegistryService, Storage</x:v>
@@ -4279,16 +4279,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H29" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J29" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K29" s="3" t="str">
         <x:v>P1</x:v>
@@ -4306,7 +4306,7 @@
         <x:v>ManufacturingCatalogController material reference endpoints</x:v>
       </x:c>
       <x:c r="P29" s="3" t="str">
-        <x:v>Materials tests where present</x:v>
+        <x:v>Materials tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="str">
         <x:v>Intranet BFF, MaterialService</x:v>
@@ -4344,16 +4344,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H30" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J30" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K30" s="3" t="str">
         <x:v>P1</x:v>
@@ -4371,7 +4371,7 @@
         <x:v>EquipmentsController CRUD/status/notes/loans/maintenance/attachments</x:v>
       </x:c>
       <x:c r="P30" s="3" t="str">
-        <x:v>Equipment tests where present</x:v>
+        <x:v>Equipment tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="str">
         <x:v>Intranet BFF, EquipmentService, Storage</x:v>
@@ -4409,16 +4409,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H31" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J31" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K31" s="3" t="str">
         <x:v>P1</x:v>
@@ -4436,7 +4436,7 @@
         <x:v>InventoryController batches/items/list/detail/lookup/consume/status</x:v>
       </x:c>
       <x:c r="P31" s="3" t="str">
-        <x:v>Inventory tests where present</x:v>
+        <x:v>Inventory tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="str">
         <x:v>Intranet BFF, InventoryService</x:v>
@@ -4474,16 +4474,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G32" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H32" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I32" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J32" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K32" s="3" t="str">
         <x:v>P1</x:v>
@@ -4501,7 +4501,7 @@
         <x:v>Jobs/production controllers where configured</x:v>
       </x:c>
       <x:c r="P32" s="3" t="str">
-        <x:v>Production schedule tests where present</x:v>
+        <x:v>Production schedule tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="str">
         <x:v>Intranet BFF, Manufacturing/Jobs services</x:v>
@@ -4539,16 +4539,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G33" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H33" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J33" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K33" s="3" t="str">
         <x:v>P2</x:v>
@@ -4566,7 +4566,7 @@
         <x:v>ModelsController GET/detail/upload/viewer-url/thumbnail-url/delete</x:v>
       </x:c>
       <x:c r="P33" s="3" t="str">
-        <x:v>Model tests where present</x:v>
+        <x:v>Model tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="str">
         <x:v>Intranet BFF, UploadService, Storage</x:v>
@@ -4604,16 +4604,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H34" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J34" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K34" s="3" t="str">
         <x:v>P0</x:v>
@@ -4631,7 +4631,7 @@
         <x:v>IamController users/roles/permissions/bindings/invite/activity/matrix; PermissionsController</x:v>
       </x:c>
       <x:c r="P34" s="3" t="str">
-        <x:v>IAM tests where present</x:v>
+        <x:v>IAM tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="str">
         <x:v>Intranet BFF, IAMService</x:v>
@@ -4669,16 +4669,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G35" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H35" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I35" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J35" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K35" s="3" t="str">
         <x:v>P1</x:v>
@@ -4696,7 +4696,7 @@
         <x:v>EmployeesController endpoints</x:v>
       </x:c>
       <x:c r="P35" s="3" t="str">
-        <x:v>Employee tests where present</x:v>
+        <x:v>Employee tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="str">
         <x:v>Intranet BFF, EmployeeService, IAMService</x:v>
@@ -4734,16 +4734,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G36" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H36" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I36" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J36" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K36" s="3" t="str">
         <x:v>P1</x:v>
@@ -4761,7 +4761,7 @@
         <x:v>TimeOffController balances/requests/approvals/decision</x:v>
       </x:c>
       <x:c r="P36" s="3" t="str">
-        <x:v>TimeOff tests where present</x:v>
+        <x:v>TimeOff tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="str">
         <x:v>Intranet BFF, LeaveService, EmployeeService</x:v>
@@ -4799,16 +4799,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G37" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H37" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I37" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J37" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K37" s="3" t="str">
         <x:v>P2</x:v>
@@ -4826,7 +4826,7 @@
         <x:v>RecruitmentController jobs/stats/candidates</x:v>
       </x:c>
       <x:c r="P37" s="3" t="str">
-        <x:v>Recruitment tests where present</x:v>
+        <x:v>Recruitment tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="str">
         <x:v>Intranet BFF, CareerService</x:v>
@@ -4864,16 +4864,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G38" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H38" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I38" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K38" s="3" t="str">
         <x:v>P2</x:v>
@@ -4891,7 +4891,7 @@
         <x:v>CompensationController summary/benefits</x:v>
       </x:c>
       <x:c r="P38" s="3" t="str">
-        <x:v>Compensation tests where present</x:v>
+        <x:v>Compensation tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="str">
         <x:v>Intranet BFF, CompensationService</x:v>
@@ -4929,16 +4929,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G39" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H39" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I39" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J39" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K39" s="3" t="str">
         <x:v>P1</x:v>
@@ -4956,7 +4956,7 @@
         <x:v>ReferenceDataController countries/currencies/locations/rate endpoints</x:v>
       </x:c>
       <x:c r="P39" s="3" t="str">
-        <x:v>ReferenceData tests where present</x:v>
+        <x:v>ReferenceData tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="str">
         <x:v>Intranet BFF, ReferenceData store</x:v>
@@ -4994,16 +4994,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G40" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H40" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I40" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J40" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K40" s="3" t="str">
         <x:v>P1</x:v>
@@ -5021,7 +5021,7 @@
         <x:v>SystemHealthController GET, history</x:v>
       </x:c>
       <x:c r="P40" s="3" t="str">
-        <x:v>System health tests where present</x:v>
+        <x:v>System health tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q40" s="3" t="str">
         <x:v>Intranet BFF, Health sampler/services</x:v>
@@ -5059,16 +5059,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G41" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H41" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I41" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J41" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K41" s="3" t="str">
         <x:v>P1</x:v>
@@ -5086,7 +5086,7 @@
         <x:v>AiProcessingController health/extract/upload/link/download endpoints</x:v>
       </x:c>
       <x:c r="P41" s="3" t="str">
-        <x:v>AI processing tests where present</x:v>
+        <x:v>AI processing tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q41" s="3" t="str">
         <x:v>Intranet BFF, AI service, Storage</x:v>
@@ -5124,16 +5124,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G42" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H42" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I42" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J42" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K42" s="3" t="str">
         <x:v>P2</x:v>
@@ -5151,7 +5151,7 @@
         <x:v>PreferencesController GET/PUT/DELETE</x:v>
       </x:c>
       <x:c r="P42" s="3" t="str">
-        <x:v>Preferences tests where present</x:v>
+        <x:v>Preferences tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q42" s="3" t="str">
         <x:v>Intranet BFF, EmployeeService</x:v>
@@ -5189,16 +5189,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G43" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H43" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I43" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K43" s="3" t="str">
         <x:v>P0</x:v>
@@ -5216,7 +5216,7 @@
         <x:v>AuthController endpoints</x:v>
       </x:c>
       <x:c r="P43" s="3" t="str">
-        <x:v>Auth/login tests where present</x:v>
+        <x:v>Auth/login tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q43" s="3" t="str">
         <x:v>Intranet BFF, Auth/IAM</x:v>
@@ -5254,16 +5254,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G44" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H44" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I44" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J44" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K44" s="3" t="str">
         <x:v>P2</x:v>
@@ -5281,7 +5281,7 @@
         <x:v>AddressController GET google-config</x:v>
       </x:c>
       <x:c r="P44" s="3" t="str">
-        <x:v>Address source tests where present</x:v>
+        <x:v>Address source tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q44" s="3" t="str">
         <x:v>Intranet BFF, configuration</x:v>
@@ -5319,16 +5319,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G45" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
       </x:c>
       <x:c r="H45" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="I45" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
       </x:c>
       <x:c r="J45" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K45" s="3" t="str">
         <x:v>P2</x:v>
@@ -5346,7 +5346,7 @@
         <x:v>SeedController POST customers and /api/seed/customers</x:v>
       </x:c>
       <x:c r="P45" s="3" t="str">
-        <x:v>Aspire seed tests where present</x:v>
+        <x:v>Aspire seed tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
       </x:c>
       <x:c r="Q45" s="3" t="str">
         <x:v>Intranet BFF, DatabaseSeeder, CustomerService</x:v>
@@ -5367,7 +5367,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3e48ec792d04b21"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra33d4ff753ee4748"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7937,7 +7937,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e6da95d07ed4e68"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0147e55d11a64293"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Record QuoteEngine suite fix evidence
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rec5d5323eb5d4efc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R44ee5cd5ca9141cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rdbfe439a58d546f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R3cf2b7afc2d2492b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4585119bd12d4a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R807a60cfd8ac4152"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R22b6efa70b8e4ffe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R290d9820c4d34c00"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2407,7 +2407,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a0e07831f964eb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fbbd983b61148d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5367,7 +5367,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra33d4ff753ee4748"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R959304072e3e4436"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5484,16 +5484,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Failed current QuoteEngine suite, fixed, and retested passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>Initial QuoteEngine suite failed 3/539 because a residual sample-only workspace route/workbench still rendered old quote panel components.</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Fixed in Maliev.QuoteEngine commit e0c263f by removing the sample-only workspace route, workbench, notice, and public fallback exception.</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Retested: source tests 180/180 passed, full QuoteEngine suite 539/539 passed, targeted route/workbench marker scan clean.</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
         <x:v>P0</x:v>
@@ -5511,7 +5511,7 @@
         <x:v>QuoteController project nav/detail endpoints</x:v>
       </x:c>
       <x:c r="P2" s="3" t="str">
-        <x:v>QuoteEngineSourceTests workspace/shell</x:v>
+        <x:v>QuoteEngineSourceTests workspace/shell | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations. | Fix verification: QuoteEngineSourceTests passed 180/180; targeted scan found no sample-only workspace route/workbench markers in client workspace or BFF fallback route.</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="str">
         <x:v>QuoteEngine client/BFF, session store</x:v>
@@ -5523,7 +5523,7 @@
         <x:v>The source still contains a non-current route, but tracking excludes it per product direction</x:v>
       </x:c>
       <x:c r="T2" s="3" t="str">
-        <x:v>QuoteWorkspace.razor:1-5,39; QuoteAgentLaunchShell.razor</x:v>
+        <x:v>QuoteWorkspace.razor:1-5,39; QuoteAgentLaunchShell.razor; Program.cs public route fallback; QuoteWorkspace.razor routes; QuoteAgentLaunchShell.razor</x:v>
       </x:c>
       <x:c r="U2" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -5549,16 +5549,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>P0</x:v>
@@ -5576,7 +5576,7 @@
         <x:v>AgentController GET health</x:v>
       </x:c>
       <x:c r="P3" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests health; QuoteEngineSourceTests status dot</x:v>
+        <x:v>QuoteAgentEndpointTests health; QuoteEngineSourceTests status dot | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent service</x:v>
@@ -5614,16 +5614,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
         <x:v>P0</x:v>
@@ -5641,7 +5641,7 @@
         <x:v>AgentController POST messages; QuoteAgentService SendMessageAsync</x:v>
       </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests messages</x:v>
+        <x:v>QuoteAgentEndpointTests messages | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent model, SessionStore</x:v>
@@ -5679,16 +5679,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G5" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H5" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I5" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J5" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K5" s="3" t="str">
         <x:v>P0</x:v>
@@ -5706,7 +5706,7 @@
         <x:v>AgentController POST messages/stream</x:v>
       </x:c>
       <x:c r="P5" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests stream events; QuoteAgentLaunchShell source tests</x:v>
+        <x:v>QuoteAgentEndpointTests stream events; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent model</x:v>
@@ -5744,16 +5744,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G6" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H6" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I6" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J6" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K6" s="3" t="str">
         <x:v>P0</x:v>
@@ -5771,7 +5771,7 @@
         <x:v>AgentController GET sessions/{sessionId}, sessions/{sessionId}/messages</x:v>
       </x:c>
       <x:c r="P6" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests history auth</x:v>
+        <x:v>QuoteAgentEndpointTests history auth | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="str">
         <x:v>QuoteEngine BFF, SessionStore, Auth</x:v>
@@ -5809,16 +5809,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I7" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J7" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K7" s="3" t="str">
         <x:v>P2</x:v>
@@ -5836,7 +5836,7 @@
         <x:v>AgentController clean-speech, thinking</x:v>
       </x:c>
       <x:c r="P7" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests; QuoteEngineSourceTests thinking</x:v>
+        <x:v>QuoteAgentEndpointTests; QuoteEngineSourceTests thinking | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent service</x:v>
@@ -5874,16 +5874,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
         <x:v>P0</x:v>
@@ -5901,7 +5901,7 @@
         <x:v>QuoteController projects/nav, project detail, duplicate, pin, delete pin, archive</x:v>
       </x:c>
       <x:c r="P8" s="3" t="str">
-        <x:v>QuoteEngineSourceTests rail/project management</x:v>
+        <x:v>QuoteEngineSourceTests rail/project management | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="str">
         <x:v>QuoteEngine BFF, Project service, SessionStore</x:v>
@@ -5939,16 +5939,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>P1</x:v>
@@ -5966,7 +5966,7 @@
         <x:v>AgentController GET sessions/{sessionId}/search</x:v>
       </x:c>
       <x:c r="P9" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests search</x:v>
+        <x:v>QuoteAgentEndpointTests search | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent/Project service</x:v>
@@ -6004,16 +6004,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K10" s="3" t="str">
         <x:v>P0</x:v>
@@ -6031,7 +6031,7 @@
         <x:v>QuoteController uploads/resumable, PUT chunk, complete, analysis-status</x:v>
       </x:c>
       <x:c r="P10" s="3" t="str">
-        <x:v>QuoteEngineSourceTests upload; QuoteEngineApiClientTests</x:v>
+        <x:v>QuoteEngineSourceTests upload; QuoteEngineApiClientTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="str">
         <x:v>QuoteEngine BFF, Storage, Geometry/analysis</x:v>
@@ -6069,16 +6069,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J11" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K11" s="3" t="str">
         <x:v>P0</x:v>
@@ -6096,7 +6096,7 @@
         <x:v>QuoteController POST uploads/handoff</x:v>
       </x:c>
       <x:c r="P11" s="3" t="str">
-        <x:v>QuoteEngineApiClientTests handoff</x:v>
+        <x:v>QuoteEngineApiClientTests handoff | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="str">
         <x:v>QuoteEngine BFF, Web BFF, Storage</x:v>
@@ -6134,16 +6134,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K12" s="3" t="str">
         <x:v>P0</x:v>
@@ -6161,7 +6161,7 @@
         <x:v>AgentController POST sessions/{sessionId}/attachments</x:v>
       </x:c>
       <x:c r="P12" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests attachment; QuoteAgentLaunchShell source tests</x:v>
+        <x:v>QuoteAgentEndpointTests attachment; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="str">
         <x:v>QuoteEngine BFF, SessionStore, Storage</x:v>
@@ -6199,16 +6199,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J13" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K13" s="3" t="str">
         <x:v>P1</x:v>
@@ -6226,7 +6226,7 @@
         <x:v>AgentController POST sessions/{sessionId}/sketches</x:v>
       </x:c>
       <x:c r="P13" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests sketches; source tests sketch disposal</x:v>
+        <x:v>QuoteAgentEndpointTests sketches; source tests sketch disposal | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="str">
         <x:v>QuoteEngine BFF, SessionStore, Storage</x:v>
@@ -6264,16 +6264,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G14" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H14" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I14" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J14" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K14" s="3" t="str">
         <x:v>P1</x:v>
@@ -6291,7 +6291,7 @@
         <x:v>GoogleDriveConnectorController start/callback/status/files; AgentController connectors/handoff</x:v>
       </x:c>
       <x:c r="P14" s="3" t="str">
-        <x:v>QuoteEngineSourceTests connector; endpoint tests where present</x:v>
+        <x:v>QuoteEngineSourceTests connector; endpoint tests where present | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="str">
         <x:v>QuoteEngine BFF, Google Drive, Auth</x:v>
@@ -6329,16 +6329,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G15" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H15" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I15" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J15" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K15" s="3" t="str">
         <x:v>P0</x:v>
@@ -6356,7 +6356,7 @@
         <x:v>AgentController artifacts/download</x:v>
       </x:c>
       <x:c r="P15" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests artifact download; QuoteEngineSourceTests artifacts</x:v>
+        <x:v>QuoteAgentEndpointTests artifact download; QuoteEngineSourceTests artifacts | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="str">
         <x:v>QuoteEngine BFF, Storage/artifact service</x:v>
@@ -6394,16 +6394,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G16" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H16" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I16" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J16" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K16" s="3" t="str">
         <x:v>P1</x:v>
@@ -6421,7 +6421,7 @@
         <x:v>AgentController POST artifacts/{artifactId}/feedback</x:v>
       </x:c>
       <x:c r="P16" s="3" t="str">
-        <x:v>QuoteEngineSourceTests feedback; QuoteAgentEndpointTests feedback</x:v>
+        <x:v>QuoteEngineSourceTests feedback; QuoteAgentEndpointTests feedback | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent service, Customer memory</x:v>
@@ -6459,16 +6459,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G17" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H17" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I17" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J17" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K17" s="3" t="str">
         <x:v>P0</x:v>
@@ -6486,7 +6486,7 @@
         <x:v>GeometryRuntimeController manifest/assets/telemetry</x:v>
       </x:c>
       <x:c r="P17" s="3" t="str">
-        <x:v>QuoteEngineSourceTests viewer/runtime</x:v>
+        <x:v>QuoteEngineSourceTests viewer/runtime | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="str">
         <x:v>QuoteEngine client/BFF, Geometry runtime</x:v>
@@ -6524,16 +6524,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G18" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H18" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I18" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J18" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K18" s="3" t="str">
         <x:v>P0</x:v>
@@ -6551,7 +6551,7 @@
         <x:v>AgentController POST sessions/{sessionId}/dfm; QeDfmDtos</x:v>
       </x:c>
       <x:c r="P18" s="3" t="str">
-        <x:v>QuoteEngineSourceTests DFM</x:v>
+        <x:v>QuoteEngineSourceTests DFM | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="str">
         <x:v>QuoteEngine BFF, Geometry/DFM, SessionStore</x:v>
@@ -6589,16 +6589,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G19" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H19" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I19" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J19" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K19" s="3" t="str">
         <x:v>P0</x:v>
@@ -6616,7 +6616,7 @@
         <x:v>QuoteController reference-data/estimate</x:v>
       </x:c>
       <x:c r="P19" s="3" t="str">
-        <x:v>QuoteEngineSourceTests config sidebar</x:v>
+        <x:v>QuoteEngineSourceTests config sidebar | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="str">
         <x:v>QuoteEngine client/BFF, Pricing/Material services</x:v>
@@ -6654,16 +6654,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G20" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H20" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I20" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J20" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K20" s="3" t="str">
         <x:v>P1</x:v>
@@ -6681,7 +6681,7 @@
         <x:v>QuoteController reference-data; ReferenceDataController currencies</x:v>
       </x:c>
       <x:c r="P20" s="3" t="str">
-        <x:v>QuoteEngineApiClientTests</x:v>
+        <x:v>QuoteEngineApiClientTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="str">
         <x:v>QuoteEngine BFF, Material/Pricing/Reference data</x:v>
@@ -6719,16 +6719,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G21" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H21" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I21" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J21" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K21" s="3" t="str">
         <x:v>P0</x:v>
@@ -6746,7 +6746,7 @@
         <x:v>QuoteController POST estimate</x:v>
       </x:c>
       <x:c r="P21" s="3" t="str">
-        <x:v>Pricing/QuoteEngine tests</x:v>
+        <x:v>Pricing/QuoteEngine tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="str">
         <x:v>QuoteEngine BFF, PricingService</x:v>
@@ -6784,16 +6784,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G22" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H22" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I22" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J22" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K22" s="3" t="str">
         <x:v>P0</x:v>
@@ -6811,7 +6811,7 @@
         <x:v>QuoteController POST projects/draft</x:v>
       </x:c>
       <x:c r="P22" s="3" t="str">
-        <x:v>QuoteEngineSourceTests project draft</x:v>
+        <x:v>QuoteEngineSourceTests project draft | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="str">
         <x:v>QuoteEngine BFF, Project/Quote service</x:v>
@@ -6849,16 +6849,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G23" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H23" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I23" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J23" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K23" s="3" t="str">
         <x:v>P0</x:v>
@@ -6876,7 +6876,7 @@
         <x:v>QuoteController POST quotes/formal</x:v>
       </x:c>
       <x:c r="P23" s="3" t="str">
-        <x:v>QuoteEngineSourceTests summary/formal quote</x:v>
+        <x:v>QuoteEngineSourceTests summary/formal quote | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="str">
         <x:v>QuoteEngine BFF, Quotation/Pdf/Storage</x:v>
@@ -6914,16 +6914,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G24" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H24" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I24" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J24" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K24" s="3" t="str">
         <x:v>P0</x:v>
@@ -6941,7 +6941,7 @@
         <x:v>QuoteController POST quotes/{quoteId}/approve</x:v>
       </x:c>
       <x:c r="P24" s="3" t="str">
-        <x:v>Quote/Order contract tests</x:v>
+        <x:v>Quote/Order contract tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="str">
         <x:v>QuoteEngine BFF, QuotationService</x:v>
@@ -6979,16 +6979,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G25" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H25" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I25" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J25" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K25" s="3" t="str">
         <x:v>P0</x:v>
@@ -7006,7 +7006,7 @@
         <x:v>QuoteController POST orders</x:v>
       </x:c>
       <x:c r="P25" s="3" t="str">
-        <x:v>Order contract tests</x:v>
+        <x:v>Order contract tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="str">
         <x:v>QuoteEngine BFF, OrderService</x:v>
@@ -7044,16 +7044,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G26" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H26" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I26" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J26" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K26" s="3" t="str">
         <x:v>P0</x:v>
@@ -7071,7 +7071,7 @@
         <x:v>QuoteController POST payments</x:v>
       </x:c>
       <x:c r="P26" s="3" t="str">
-        <x:v>Payment contract tests</x:v>
+        <x:v>Payment contract tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="str">
         <x:v>QuoteEngine BFF, PaymentService</x:v>
@@ -7109,16 +7109,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G27" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H27" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I27" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J27" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K27" s="3" t="str">
         <x:v>P1</x:v>
@@ -7136,7 +7136,7 @@
         <x:v>AccountController GET profile, addresses</x:v>
       </x:c>
       <x:c r="P27" s="3" t="str">
-        <x:v>AccountAuthBoundaryTests</x:v>
+        <x:v>AccountAuthBoundaryTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="str">
         <x:v>QuoteEngine BFF, CustomerService</x:v>
@@ -7174,16 +7174,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
         <x:v>P1</x:v>
@@ -7201,7 +7201,7 @@
         <x:v>AccountController quotes, orders, order detail, order file download</x:v>
       </x:c>
       <x:c r="P28" s="3" t="str">
-        <x:v>QuoteEngineSourceTests account/order routes</x:v>
+        <x:v>QuoteEngineSourceTests account/order routes | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="str">
         <x:v>QuoteEngine BFF, Quote/Order service, Storage</x:v>
@@ -7239,16 +7239,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G29" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H29" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I29" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J29" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K29" s="3" t="str">
         <x:v>P2</x:v>
@@ -7266,7 +7266,7 @@
         <x:v>AccountController GET ndas</x:v>
       </x:c>
       <x:c r="P29" s="3" t="str">
-        <x:v>QuoteEngineSourceTests account routes</x:v>
+        <x:v>QuoteEngineSourceTests account routes | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="str">
         <x:v>QuoteEngine BFF, Customer/Document services</x:v>
@@ -7304,16 +7304,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G30" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H30" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I30" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J30" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K30" s="3" t="str">
         <x:v>P1</x:v>
@@ -7331,7 +7331,7 @@
         <x:v>AccountController documents GET/POST/upload/download</x:v>
       </x:c>
       <x:c r="P30" s="3" t="str">
-        <x:v>QuoteEngineSourceTests documents</x:v>
+        <x:v>QuoteEngineSourceTests documents | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="str">
         <x:v>QuoteEngine BFF, Document/Storage service</x:v>
@@ -7369,16 +7369,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G31" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H31" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I31" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J31" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K31" s="3" t="str">
         <x:v>P2</x:v>
@@ -7396,7 +7396,7 @@
         <x:v>QuoteEngineApiClient preference/account calls</x:v>
       </x:c>
       <x:c r="P31" s="3" t="str">
-        <x:v>QuoteEngineSourceTests where present</x:v>
+        <x:v>QuoteEngineSourceTests where present | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="str">
         <x:v>QuoteEngine client/BFF</x:v>
@@ -7434,16 +7434,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G32" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H32" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I32" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J32" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K32" s="3" t="str">
         <x:v>P0</x:v>
@@ -7461,7 +7461,7 @@
         <x:v>AuthController GET session, POST sign-out</x:v>
       </x:c>
       <x:c r="P32" s="3" t="str">
-        <x:v>GoogleAuthFlowTests; AccountAuthBoundaryTests</x:v>
+        <x:v>GoogleAuthFlowTests; AccountAuthBoundaryTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="str">
         <x:v>QuoteEngine BFF, Auth/Customer session</x:v>
@@ -7499,16 +7499,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G33" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H33" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I33" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J33" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K33" s="3" t="str">
         <x:v>P1</x:v>
@@ -7526,7 +7526,7 @@
         <x:v>ShippingController couriers/rates/tracking</x:v>
       </x:c>
       <x:c r="P33" s="3" t="str">
-        <x:v>Shipping contract tests where present</x:v>
+        <x:v>Shipping contract tests where present | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="str">
         <x:v>QuoteEngine BFF, DeliveryService</x:v>
@@ -7564,16 +7564,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H34" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J34" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K34" s="3" t="str">
         <x:v>P2</x:v>
@@ -7591,7 +7591,7 @@
         <x:v>AddressController google-config, thai-locations</x:v>
       </x:c>
       <x:c r="P34" s="3" t="str">
-        <x:v>QuoteEngineAddressSourceTests</x:v>
+        <x:v>QuoteEngineAddressSourceTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="str">
         <x:v>QuoteEngine BFF, Configuration/ReferenceData</x:v>
@@ -7629,16 +7629,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G35" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H35" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I35" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J35" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K35" s="3" t="str">
         <x:v>P1</x:v>
@@ -7656,7 +7656,7 @@
         <x:v>GeometryRuntimeController manifest/assets/telemetry</x:v>
       </x:c>
       <x:c r="P35" s="3" t="str">
-        <x:v>QuoteEngineSourceTests geometry runtime</x:v>
+        <x:v>QuoteEngineSourceTests geometry runtime | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="str">
         <x:v>QuoteEngine BFF, Geometry runtime</x:v>
@@ -7694,16 +7694,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G36" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H36" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I36" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J36" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K36" s="3" t="str">
         <x:v>P0</x:v>
@@ -7721,7 +7721,7 @@
         <x:v>AgentController tools/{toolName}, actions/{actionId}/confirm</x:v>
       </x:c>
       <x:c r="P36" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests action confirmations</x:v>
+        <x:v>QuoteAgentEndpointTests action confirmations | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent service, SessionStore</x:v>
@@ -7759,16 +7759,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G37" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H37" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I37" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J37" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K37" s="3" t="str">
         <x:v>P1</x:v>
@@ -7786,7 +7786,7 @@
         <x:v>QuoteAgentService prompt/memory paths</x:v>
       </x:c>
       <x:c r="P37" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests memory/grounding; source tests feedback memory</x:v>
+        <x:v>QuoteAgentEndpointTests memory/grounding; source tests feedback memory | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="str">
         <x:v>QuoteEngine BFF, Agent model, CustomerService memory</x:v>
@@ -7824,16 +7824,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G38" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H38" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I38" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J38" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K38" s="3" t="str">
         <x:v>P1</x:v>
@@ -7851,7 +7851,7 @@
         <x:v>Analysis status endpoints plus notification hub</x:v>
       </x:c>
       <x:c r="P38" s="3" t="str">
-        <x:v>QuoteEngineSourceTests realtime/thinking where present</x:v>
+        <x:v>QuoteEngineSourceTests realtime/thinking where present | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="str">
         <x:v>QuoteEngine BFF, SignalR, Geometry/Storage</x:v>
@@ -7889,16 +7889,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G39" s="3" t="str">
-        <x:v>Mapped to existing tests</x:v>
+        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
       </x:c>
       <x:c r="H39" s="3" t="str">
-        <x:v>Not tested in current loop</x:v>
+        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="I39" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
       </x:c>
       <x:c r="J39" s="3" t="str">
-        <x:v>Not started</x:v>
+        <x:v>Current automated suite passed.</x:v>
       </x:c>
       <x:c r="K39" s="3" t="str">
         <x:v>P2</x:v>
@@ -7916,7 +7916,7 @@
         <x:v>AgentController POST export-pdf</x:v>
       </x:c>
       <x:c r="P39" s="3" t="str">
-        <x:v>QuoteAgentEndpointTests export PDF</x:v>
+        <x:v>QuoteAgentEndpointTests export PDF | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="str">
         <x:v>QuoteEngine BFF, PdfService</x:v>
@@ -7937,7 +7937,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0147e55d11a64293"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R298253f1e71d496e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Update feature tracker browser evidence
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4585119bd12d4a73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R807a60cfd8ac4152"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R22b6efa70b8e4ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R290d9820c4d34c00"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8e272da5a73f48d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rb2db60ebe6ef439c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd5dc25427a094fd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rcbf3e1afc5644b07"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
         <x:v>Next loop</x:v>
       </x:c>
       <x:c r="B9" s="3" t="str">
-        <x:v>Test every current code-derived user story, document errors, fix logistical/UX issues, then retest.</x:v>
+        <x:v>Continue Intranet dashboard browser pass via Aspire-configured runtime, then continue story-by-story behavior testing and retesting.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -604,16 +604,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser route check passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>No behavior error observed in current Web automated suite.</x:v>
+        <x:v>Browser check passed: /services returned HTTP 200, rendered services content, and reported no page errors.</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>No fix needed from current Web automated suite.</x:v>
+        <x:v>No Web code fix needed for this story.</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
+        <x:v>Retested in 16-route Web browser pass on 2026-06-23; route passed with no page errors.</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>P2</x:v>
@@ -631,7 +631,7 @@
         <x:v>Static content model</x:v>
       </x:c>
       <x:c r="P3" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
+        <x:v>Browser evidence: Playwright browser route check against Maliev.Web.Bff http profile on 2026-06-23 covered /services, /services/3d-printing, /cart, and 13 static/content routes; final retest passed 16/16 with no page errors.</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="str">
         <x:v>Web client</x:v>
@@ -669,16 +669,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G4" s="3" t="str">
-        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser route check failed, fixed, and retested passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H4" s="3" t="str">
-        <x:v>No behavior error observed in current Web automated suite.</x:v>
+        <x:v>Initial browser check: /services/3d-printing returned HTTP 200 and rendered the page, but threw TypeError in babylonjs.loaders.min.js while duplicate Babylon runtime scripts were appended.</x:v>
       </x:c>
       <x:c r="I4" s="3" t="str">
-        <x:v>No fix needed from current Web automated suite.</x:v>
+        <x:v>Fixed manufacturing-gizmo runtime guards to share canvas instances and Babylon script promises through globalThis.__malievManufacturingGizmo.</x:v>
       </x:c>
       <x:c r="J4" s="3" t="str">
-        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
+        <x:v>Retested focused regression 1/1 passed; reran 16-route Web browser pass 16/16 passed; /services/3d-printing had no page errors and duplicate-script probe showed one Babylon core and one loader script.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="str">
         <x:v>P2</x:v>
@@ -696,7 +696,7 @@
         <x:v>Static content model</x:v>
       </x:c>
       <x:c r="P4" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.ServicesUseRealRoutesAndDisabledQuoteActions|HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn|HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount passed 4/4 on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
+        <x:v>Browser evidence: Playwright browser route check against Maliev.Web.Bff http profile on 2026-06-23 covered /services, /services/3d-printing, /cart, and 13 static/content routes; final retest passed 16/16 with no page errors. Regression: dotnet test Maliev.Web.slnx --filter "FullyQualifiedName~ManufacturingGizmoRuntimeSourceTests" --verbosity minimal passed 1/1 after failing before the JS runtime fix.</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="str">
         <x:v>Web client</x:v>
@@ -708,7 +708,7 @@
         <x:v>Needs 404/unknown slug browser check</x:v>
       </x:c>
       <x:c r="T4" s="3" t="str">
-        <x:v>ServicePage.razor:1</x:v>
+        <x:v>ServicePage.razor:1; manufacturing-gizmo.js:1-8,215-247; ManufacturingGizmoRuntimeSourceTests.cs</x:v>
       </x:c>
       <x:c r="U4" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -994,16 +994,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
-        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser route check passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>No behavior error observed in current Web automated suite.</x:v>
+        <x:v>Browser check passed: /cart returned HTTP 200, rendered cart content, and reported no page errors.</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>No fix needed from current Web automated suite.</x:v>
+        <x:v>No Web code fix needed for this story.</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
+        <x:v>Retested in 16-route Web browser pass on 2026-06-23; route passed with no page errors.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>P1</x:v>
@@ -1021,7 +1021,7 @@
         <x:v>CheckoutController draft endpoints used after cart</x:v>
       </x:c>
       <x:c r="P9" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.HeaderUsesMudIconButtonsForCartAndAccount|HeroLayoutSourceTests.CheckoutPageCollectsCustomerCheckoutDetailsAfterSignIn passed as part of 4/4 focused Web run on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
+        <x:v>Browser evidence: Playwright browser route check against Maliev.Web.Bff http profile on 2026-06-23 covered /services, /services/3d-printing, /cart, and 13 static/content routes; final retest passed 16/16 with no page errors.</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="str">
         <x:v>Web client, Checkout BFF</x:v>
@@ -2229,16 +2229,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G28" s="3" t="str">
-        <x:v>Automated Web suite passed 2026-06-23; browser runtime pending</x:v>
+        <x:v>Automated Web suite passed 2026-06-23; browser route check passed 2026-06-23</x:v>
       </x:c>
       <x:c r="H28" s="3" t="str">
-        <x:v>No behavior error observed in current Web automated suite.</x:v>
+        <x:v>Browser check passed: about, FAQ, policy, industry, case-study, and blog routes returned HTTP 200 and reported no page errors.</x:v>
       </x:c>
       <x:c r="I28" s="3" t="str">
-        <x:v>No fix needed from current Web automated suite.</x:v>
+        <x:v>No Web code fix needed for this story.</x:v>
       </x:c>
       <x:c r="J28" s="3" t="str">
-        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
+        <x:v>Retested in 16-route Web browser pass on 2026-06-23; all covered static/content routes passed with no page errors.</x:v>
       </x:c>
       <x:c r="K28" s="3" t="str">
         <x:v>P2</x:v>
@@ -2256,7 +2256,7 @@
         <x:v>BlogController for ebook PDF only</x:v>
       </x:c>
       <x:c r="P28" s="3" t="str">
-        <x:v>dotnet test Maliev.Web.slnx --filter HeroLayoutSourceTests.StaticPagesCoverCustomerRoutesAndContactBoundary passed as part of 4/4 focused Web run on 2026-06-23. | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
+        <x:v>Browser evidence: Playwright browser route check against Maliev.Web.Bff http profile on 2026-06-23 covered /services, /services/3d-printing, /cart, and 13 static/content routes; final retest passed 16/16 with no page errors.</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="str">
         <x:v>Web client, Content</x:v>
@@ -2407,7 +2407,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fbbd983b61148d6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4a4370cd90e94e1b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2589,16 +2589,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G3" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix; browser runtime pending</x:v>
+        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix; standalone browser startup blocked 2026-06-23</x:v>
       </x:c>
       <x:c r="H3" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>Browser check did not reach /: standalone dotnet run for Maliev.Intranet.Bff terminated before listening because IntranetDbContext connection string was not configured.</x:v>
       </x:c>
       <x:c r="I3" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>No dashboard UX fix applied in this slice; route needs Aspire-configured runtime with IntranetDbContext before browser verification.</x:v>
       </x:c>
       <x:c r="J3" s="3" t="str">
-        <x:v>Current automated suite passed; browser/runtime verification pending.</x:v>
+        <x:v>Not browser-rendered in standalone mode; startup blocker captured from current run. Automated dashboard/controller tests remain passed.</x:v>
       </x:c>
       <x:c r="K3" s="3" t="str">
         <x:v>P1</x:v>
@@ -5367,7 +5367,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R959304072e3e4436"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1ec56bbf2fc4287"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7937,7 +7937,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R298253f1e71d496e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R97c79c73d9d14e7e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-051 not-found recovery test
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R84826f258dea4c1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R612a23bdfc764b64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd76d5e8c74ac4ce6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R27796b1ecd8f4f15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Recba917fce4e47a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rd28cc1ae787c42ac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R8bd7a0686ffc465d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R9b3c2a324e4f4f0d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3227,39 +3227,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">ClientConfigController.cs:14-46; DiagnosticsController.cs:15-25</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">INT-051</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Not-found handling</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As an employee, I can recover when an intranet route does not exist.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Not-found page explains the missing content and links back to the dashboard.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Blazor fallback route -&gt; dashboard recovery link</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NotFound.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/not-found</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">None; client recovery page only</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Intranet client</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs browser recovery-route pass.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">NotFound.razor:1</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QE-001</x:t>
@@ -7238,7 +7205,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R499cf8b8082d473e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b883387c6dd487a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10587,74 +10554,74 @@
       </x:c>
     </x:row>
     <x:row r="52" ht="51.29999923706055" hidden="0">
-      <x:c r="A52" s="3" t="s">
-        <x:v>1072</x:v>
-      </x:c>
-      <x:c r="B52" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C52" s="3" t="s">
-        <x:v>1073</x:v>
-      </x:c>
-      <x:c r="D52" s="3" t="s">
-        <x:v>1074</x:v>
-      </x:c>
-      <x:c r="E52" s="3" t="s">
-        <x:v>1075</x:v>
-      </x:c>
-      <x:c r="F52" s="3" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="G52" s="3" t="s">
-        <x:v>1001</x:v>
-      </x:c>
-      <x:c r="H52" s="3" t="s">
-        <x:v>1002</x:v>
-      </x:c>
-      <x:c r="I52" s="3" t="s">
-        <x:v>1003</x:v>
-      </x:c>
-      <x:c r="J52" s="3" t="s">
-        <x:v>1004</x:v>
-      </x:c>
-      <x:c r="K52" s="3" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="L52" s="3" t="s">
-        <x:v>1076</x:v>
-      </x:c>
-      <x:c r="M52" s="3" t="s">
-        <x:v>1077</x:v>
-      </x:c>
-      <x:c r="N52" s="3" t="s">
-        <x:v>1078</x:v>
-      </x:c>
-      <x:c r="O52" s="3" t="s">
-        <x:v>1079</x:v>
-      </x:c>
-      <x:c r="P52" s="3" t="s">
-        <x:v>1009</x:v>
-      </x:c>
-      <x:c r="Q52" s="3" t="s">
-        <x:v>1080</x:v>
-      </x:c>
-      <x:c r="R52" s="3" t="s">
-        <x:v>418</x:v>
-      </x:c>
-      <x:c r="S52" s="3" t="s">
-        <x:v>1081</x:v>
-      </x:c>
-      <x:c r="T52" s="3" t="s">
-        <x:v>1082</x:v>
-      </x:c>
-      <x:c r="U52" s="3" t="s">
-        <x:v>2</x:v>
+      <x:c r="A52" s="3" t="str">
+        <x:v>INT-051</x:v>
+      </x:c>
+      <x:c r="B52" s="3" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C52" s="3" t="str">
+        <x:v>Not-found handling</x:v>
+      </x:c>
+      <x:c r="D52" s="3" t="str">
+        <x:v>As an employee, I can recover when an intranet route does not exist.</x:v>
+      </x:c>
+      <x:c r="E52" s="3" t="str">
+        <x:v>Not-found page explains the missing content and links back to the dashboard.</x:v>
+      </x:c>
+      <x:c r="F52" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G52" s="3" t="str">
+        <x:v>Behavior test failed, fixed, and retested passed 2026-06-23.</x:v>
+      </x:c>
+      <x:c r="H52" s="3" t="str">
+        <x:v>Source behavior check found unknown client routes used the Router inline fallback text instead of the existing designed /not-found recovery page.</x:v>
+      </x:c>
+      <x:c r="I52" s="3" t="str">
+        <x:v>Fixed in Maliev.Intranet commit 379913b by rendering Maliev.Intranet.Client.Pages.NotFound from Routes.razor &lt;NotFound&gt; fallback and adding a source regression.</x:v>
+      </x:c>
+      <x:c r="J52" s="3" t="str">
+        <x:v>Retested focused not-found source regressions 2/2 passed.</x:v>
+      </x:c>
+      <x:c r="K52" s="3" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L52" s="3" t="str">
+        <x:v>Blazor fallback route -&gt; dashboard recovery link</x:v>
+      </x:c>
+      <x:c r="M52" s="3" t="str">
+        <x:v>NotFound.razor</x:v>
+      </x:c>
+      <x:c r="N52" s="3" t="str">
+        <x:v>/not-found</x:v>
+      </x:c>
+      <x:c r="O52" s="3" t="str">
+        <x:v>None; client recovery page only</x:v>
+      </x:c>
+      <x:c r="P52" s="3" t="str">
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~ModuleRegressionSourceTests.NotFoundPage_UsesAnimatedSearchingEyes|FullyQualifiedName~ModuleRegressionSourceTests.RouterFallback_UsesNotFoundRecoveryPage" --verbosity minimal passed 2/2 on 2026-06-23. Test build compiled Intranet Client, BFF, and Tests projects.</x:v>
+      </x:c>
+      <x:c r="Q52" s="3" t="str">
+        <x:v>Intranet client</x:v>
+      </x:c>
+      <x:c r="R52" s="3" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="S52" s="3" t="str">
+        <x:v>No remaining INT-051 source fallback gap from this focused retest; full authenticated browser unknown-route pass still needed when Aspire/browser tooling is available.</x:v>
+      </x:c>
+      <x:c r="T52" s="3" t="str">
+        <x:v>Routes.razor:30-34; NotFound.razor:1; ModuleRegressionSourceTests.cs:211,225</x:v>
+      </x:c>
+      <x:c r="U52" s="3" t="str">
+        <x:v>2026-06-23</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc68b04f535744e2d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c18b4856e2c44ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10754,64 +10721,64 @@
     </x:row>
     <x:row r="2" ht="149.25" hidden="0">
       <x:c r="A2" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1073</x:v>
       </x:c>
       <x:c r="D2" s="3" t="s">
-        <x:v>1085</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="E2" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1075</x:v>
       </x:c>
       <x:c r="F2" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>1087</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>1088</x:v>
+        <x:v>1077</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>1089</x:v>
+        <x:v>1078</x:v>
       </x:c>
       <x:c r="J2" s="3" t="s">
-        <x:v>1090</x:v>
+        <x:v>1079</x:v>
       </x:c>
       <x:c r="K2" s="3" t="s">
         <x:v>188</x:v>
       </x:c>
       <x:c r="L2" s="3" t="s">
-        <x:v>1091</x:v>
+        <x:v>1080</x:v>
       </x:c>
       <x:c r="M2" s="3" t="s">
-        <x:v>1092</x:v>
+        <x:v>1081</x:v>
       </x:c>
       <x:c r="N2" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="O2" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="P2" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="s">
-        <x:v>1096</x:v>
+        <x:v>1085</x:v>
       </x:c>
       <x:c r="R2" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="S2" s="3" t="s">
-        <x:v>1098</x:v>
+        <x:v>1087</x:v>
       </x:c>
       <x:c r="T2" s="3" t="s">
-        <x:v>1099</x:v>
+        <x:v>1088</x:v>
       </x:c>
       <x:c r="U2" s="3" t="s">
         <x:v>2</x:v>
@@ -10819,31 +10786,31 @@
     </x:row>
     <x:row r="3" ht="107.25" hidden="0">
       <x:c r="A3" s="3" t="s">
-        <x:v>1100</x:v>
+        <x:v>1089</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>1101</x:v>
+        <x:v>1090</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>1102</x:v>
+        <x:v>1091</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>1103</x:v>
+        <x:v>1092</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G3" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H3" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I3" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J3" s="3" t="s">
         <x:v>42</x:v>
@@ -10852,31 +10819,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L3" s="3" t="s">
-        <x:v>1107</x:v>
+        <x:v>1096</x:v>
       </x:c>
       <x:c r="M3" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N3" s="3" t="s">
-        <x:v>1109</x:v>
+        <x:v>1098</x:v>
       </x:c>
       <x:c r="O3" s="3" t="s">
-        <x:v>1110</x:v>
+        <x:v>1099</x:v>
       </x:c>
       <x:c r="P3" s="3" t="s">
-        <x:v>1111</x:v>
+        <x:v>1100</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="s">
-        <x:v>1112</x:v>
+        <x:v>1101</x:v>
       </x:c>
       <x:c r="R3" s="3" t="s">
-        <x:v>1113</x:v>
+        <x:v>1102</x:v>
       </x:c>
       <x:c r="S3" s="3" t="s">
-        <x:v>1114</x:v>
+        <x:v>1103</x:v>
       </x:c>
       <x:c r="T3" s="3" t="s">
-        <x:v>1115</x:v>
+        <x:v>1104</x:v>
       </x:c>
       <x:c r="U3" s="3" t="s">
         <x:v>2</x:v>
@@ -10884,31 +10851,31 @@
     </x:row>
     <x:row r="4" ht="93.25" hidden="0">
       <x:c r="A4" s="3" t="s">
-        <x:v>1116</x:v>
+        <x:v>1105</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>1117</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>1118</x:v>
+        <x:v>1107</x:v>
       </x:c>
       <x:c r="E4" s="3" t="s">
-        <x:v>1119</x:v>
+        <x:v>1108</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G4" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H4" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I4" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J4" s="3" t="s">
         <x:v>42</x:v>
@@ -10917,31 +10884,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L4" s="3" t="s">
-        <x:v>1120</x:v>
+        <x:v>1109</x:v>
       </x:c>
       <x:c r="M4" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N4" s="3" t="s">
-        <x:v>1121</x:v>
+        <x:v>1110</x:v>
       </x:c>
       <x:c r="O4" s="3" t="s">
-        <x:v>1122</x:v>
+        <x:v>1111</x:v>
       </x:c>
       <x:c r="P4" s="3" t="s">
-        <x:v>1123</x:v>
+        <x:v>1112</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="s">
-        <x:v>1124</x:v>
+        <x:v>1113</x:v>
       </x:c>
       <x:c r="R4" s="3" t="s">
-        <x:v>1125</x:v>
+        <x:v>1114</x:v>
       </x:c>
       <x:c r="S4" s="3" t="s">
-        <x:v>1126</x:v>
+        <x:v>1115</x:v>
       </x:c>
       <x:c r="T4" s="3" t="s">
-        <x:v>1127</x:v>
+        <x:v>1116</x:v>
       </x:c>
       <x:c r="U4" s="3" t="s">
         <x:v>2</x:v>
@@ -10949,31 +10916,31 @@
     </x:row>
     <x:row r="5" ht="107.25" hidden="0">
       <x:c r="A5" s="3" t="s">
-        <x:v>1128</x:v>
+        <x:v>1117</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>1129</x:v>
+        <x:v>1118</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>1130</x:v>
+        <x:v>1119</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>1131</x:v>
+        <x:v>1120</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
         <x:v>42</x:v>
@@ -10982,31 +10949,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>1132</x:v>
+        <x:v>1121</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>1133</x:v>
+        <x:v>1122</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>1134</x:v>
+        <x:v>1123</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>1135</x:v>
+        <x:v>1124</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>1136</x:v>
+        <x:v>1125</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>1137</x:v>
+        <x:v>1126</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>1138</x:v>
+        <x:v>1127</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>1139</x:v>
+        <x:v>1128</x:v>
       </x:c>
       <x:c r="U5" s="3" t="s">
         <x:v>2</x:v>
@@ -11014,31 +10981,31 @@
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
       <x:c r="A6" s="3" t="s">
-        <x:v>1140</x:v>
+        <x:v>1129</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>1141</x:v>
+        <x:v>1130</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>1142</x:v>
+        <x:v>1131</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>1143</x:v>
+        <x:v>1132</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H6" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I6" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J6" s="3" t="s">
         <x:v>42</x:v>
@@ -11047,31 +11014,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L6" s="3" t="s">
-        <x:v>1144</x:v>
+        <x:v>1133</x:v>
       </x:c>
       <x:c r="M6" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N6" s="3" t="s">
-        <x:v>1145</x:v>
+        <x:v>1134</x:v>
       </x:c>
       <x:c r="O6" s="3" t="s">
-        <x:v>1146</x:v>
+        <x:v>1135</x:v>
       </x:c>
       <x:c r="P6" s="3" t="s">
-        <x:v>1147</x:v>
+        <x:v>1136</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="s">
-        <x:v>1148</x:v>
+        <x:v>1137</x:v>
       </x:c>
       <x:c r="R6" s="3" t="s">
-        <x:v>1149</x:v>
+        <x:v>1138</x:v>
       </x:c>
       <x:c r="S6" s="3" t="s">
-        <x:v>1150</x:v>
+        <x:v>1139</x:v>
       </x:c>
       <x:c r="T6" s="3" t="s">
-        <x:v>1151</x:v>
+        <x:v>1140</x:v>
       </x:c>
       <x:c r="U6" s="3" t="s">
         <x:v>2</x:v>
@@ -11079,31 +11046,31 @@
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>1152</x:v>
+        <x:v>1141</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>1153</x:v>
+        <x:v>1142</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>1154</x:v>
+        <x:v>1143</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>1155</x:v>
+        <x:v>1144</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G7" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H7" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I7" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J7" s="3" t="s">
         <x:v>42</x:v>
@@ -11112,31 +11079,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
-        <x:v>1156</x:v>
+        <x:v>1145</x:v>
       </x:c>
       <x:c r="M7" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N7" s="3" t="s">
-        <x:v>1157</x:v>
+        <x:v>1146</x:v>
       </x:c>
       <x:c r="O7" s="3" t="s">
-        <x:v>1158</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="P7" s="3" t="s">
-        <x:v>1159</x:v>
+        <x:v>1148</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="s">
-        <x:v>1112</x:v>
+        <x:v>1101</x:v>
       </x:c>
       <x:c r="R7" s="3" t="s">
-        <x:v>1160</x:v>
+        <x:v>1149</x:v>
       </x:c>
       <x:c r="S7" s="3" t="s">
-        <x:v>1161</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="T7" s="3" t="s">
-        <x:v>1162</x:v>
+        <x:v>1151</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>2</x:v>
@@ -11144,31 +11111,31 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>1163</x:v>
+        <x:v>1152</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>1164</x:v>
+        <x:v>1153</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>1165</x:v>
+        <x:v>1154</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>1166</x:v>
+        <x:v>1155</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H8" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I8" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J8" s="3" t="s">
         <x:v>42</x:v>
@@ -11177,31 +11144,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
-        <x:v>1167</x:v>
+        <x:v>1156</x:v>
       </x:c>
       <x:c r="M8" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N8" s="3" t="s">
-        <x:v>1168</x:v>
+        <x:v>1157</x:v>
       </x:c>
       <x:c r="O8" s="3" t="s">
-        <x:v>1169</x:v>
+        <x:v>1158</x:v>
       </x:c>
       <x:c r="P8" s="3" t="s">
-        <x:v>1170</x:v>
+        <x:v>1159</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="s">
-        <x:v>1171</x:v>
+        <x:v>1160</x:v>
       </x:c>
       <x:c r="R8" s="3" t="s">
-        <x:v>1172</x:v>
+        <x:v>1161</x:v>
       </x:c>
       <x:c r="S8" s="3" t="s">
-        <x:v>1173</x:v>
+        <x:v>1162</x:v>
       </x:c>
       <x:c r="T8" s="3" t="s">
-        <x:v>1174</x:v>
+        <x:v>1163</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>2</x:v>
@@ -11209,31 +11176,31 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>1175</x:v>
+        <x:v>1164</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>1176</x:v>
+        <x:v>1165</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>1177</x:v>
+        <x:v>1166</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>1178</x:v>
+        <x:v>1167</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H9" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I9" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J9" s="3" t="s">
         <x:v>42</x:v>
@@ -11242,31 +11209,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
-        <x:v>1179</x:v>
+        <x:v>1168</x:v>
       </x:c>
       <x:c r="M9" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N9" s="3" t="s">
-        <x:v>1180</x:v>
+        <x:v>1169</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>1181</x:v>
+        <x:v>1170</x:v>
       </x:c>
       <x:c r="P9" s="3" t="s">
-        <x:v>1182</x:v>
+        <x:v>1171</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="s">
-        <x:v>1183</x:v>
+        <x:v>1172</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
-        <x:v>1184</x:v>
+        <x:v>1173</x:v>
       </x:c>
       <x:c r="S9" s="3" t="s">
-        <x:v>1185</x:v>
+        <x:v>1174</x:v>
       </x:c>
       <x:c r="T9" s="3" t="s">
-        <x:v>1186</x:v>
+        <x:v>1175</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>2</x:v>
@@ -11274,31 +11241,31 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>1187</x:v>
+        <x:v>1176</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>1188</x:v>
+        <x:v>1177</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>1189</x:v>
+        <x:v>1178</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>1190</x:v>
+        <x:v>1179</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G10" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H10" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I10" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J10" s="3" t="s">
         <x:v>42</x:v>
@@ -11307,31 +11274,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>1191</x:v>
+        <x:v>1180</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
-        <x:v>1092</x:v>
+        <x:v>1081</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>1192</x:v>
+        <x:v>1181</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>1193</x:v>
+        <x:v>1182</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>1194</x:v>
+        <x:v>1183</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>1195</x:v>
+        <x:v>1184</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>1196</x:v>
+        <x:v>1185</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>1197</x:v>
+        <x:v>1186</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>2</x:v>
@@ -11339,31 +11306,31 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>1198</x:v>
+        <x:v>1187</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>1199</x:v>
+        <x:v>1188</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>1200</x:v>
+        <x:v>1189</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>1201</x:v>
+        <x:v>1190</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G11" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H11" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I11" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J11" s="3" t="s">
         <x:v>42</x:v>
@@ -11372,31 +11339,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>1202</x:v>
+        <x:v>1191</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>1203</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>1204</x:v>
+        <x:v>1193</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>1205</x:v>
+        <x:v>1194</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>1206</x:v>
+        <x:v>1195</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>1207</x:v>
+        <x:v>1196</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>1208</x:v>
+        <x:v>1197</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>1209</x:v>
+        <x:v>1198</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>1210</x:v>
+        <x:v>1199</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>2</x:v>
@@ -11404,31 +11371,31 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>1211</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>1212</x:v>
+        <x:v>1201</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>1213</x:v>
+        <x:v>1202</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>1214</x:v>
+        <x:v>1203</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G12" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H12" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I12" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J12" s="3" t="s">
         <x:v>42</x:v>
@@ -11437,31 +11404,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>1215</x:v>
+        <x:v>1204</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>1216</x:v>
+        <x:v>1205</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>1217</x:v>
+        <x:v>1206</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>1218</x:v>
+        <x:v>1207</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>1219</x:v>
+        <x:v>1208</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>1220</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>1221</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>1222</x:v>
+        <x:v>1211</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>2</x:v>
@@ -11469,31 +11436,31 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>1223</x:v>
+        <x:v>1212</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>1224</x:v>
+        <x:v>1213</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>1225</x:v>
+        <x:v>1214</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>1226</x:v>
+        <x:v>1215</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I13" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J13" s="3" t="s">
         <x:v>42</x:v>
@@ -11502,31 +11469,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>1227</x:v>
+        <x:v>1216</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>1228</x:v>
+        <x:v>1217</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>1229</x:v>
+        <x:v>1218</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>1230</x:v>
+        <x:v>1219</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
-        <x:v>1219</x:v>
+        <x:v>1208</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>1231</x:v>
+        <x:v>1220</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>1232</x:v>
+        <x:v>1221</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>1233</x:v>
+        <x:v>1222</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>2</x:v>
@@ -11534,31 +11501,31 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>1234</x:v>
+        <x:v>1223</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>1235</x:v>
+        <x:v>1224</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>1236</x:v>
+        <x:v>1225</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>1237</x:v>
+        <x:v>1226</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G14" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H14" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I14" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J14" s="3" t="s">
         <x:v>42</x:v>
@@ -11567,31 +11534,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>1238</x:v>
+        <x:v>1227</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>1239</x:v>
+        <x:v>1228</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>1240</x:v>
+        <x:v>1229</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>1241</x:v>
+        <x:v>1230</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>1242</x:v>
+        <x:v>1231</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>1243</x:v>
+        <x:v>1232</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>1244</x:v>
+        <x:v>1233</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>1245</x:v>
+        <x:v>1234</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>1246</x:v>
+        <x:v>1235</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>2</x:v>
@@ -11599,31 +11566,31 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>1247</x:v>
+        <x:v>1236</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>1248</x:v>
+        <x:v>1237</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>1249</x:v>
+        <x:v>1238</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>1250</x:v>
+        <x:v>1239</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G15" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H15" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I15" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J15" s="3" t="s">
         <x:v>42</x:v>
@@ -11632,31 +11599,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>1251</x:v>
+        <x:v>1240</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>1252</x:v>
+        <x:v>1241</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>1253</x:v>
+        <x:v>1242</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>1254</x:v>
+        <x:v>1243</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>1255</x:v>
+        <x:v>1244</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>1256</x:v>
+        <x:v>1245</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>1257</x:v>
+        <x:v>1246</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>1258</x:v>
+        <x:v>1247</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>2</x:v>
@@ -11664,31 +11631,31 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>1259</x:v>
+        <x:v>1248</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>1260</x:v>
+        <x:v>1249</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>1261</x:v>
+        <x:v>1250</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>1262</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H16" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I16" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J16" s="3" t="s">
         <x:v>42</x:v>
@@ -11697,31 +11664,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>1263</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>1264</x:v>
+        <x:v>1253</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>1265</x:v>
+        <x:v>1254</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>1266</x:v>
+        <x:v>1255</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>1267</x:v>
+        <x:v>1256</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>1268</x:v>
+        <x:v>1257</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>1269</x:v>
+        <x:v>1258</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>1270</x:v>
+        <x:v>1259</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>2</x:v>
@@ -11729,31 +11696,31 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>1271</x:v>
+        <x:v>1260</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>1272</x:v>
+        <x:v>1261</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>1273</x:v>
+        <x:v>1262</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>1274</x:v>
+        <x:v>1263</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H17" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I17" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J17" s="3" t="s">
         <x:v>42</x:v>
@@ -11762,31 +11729,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>1275</x:v>
+        <x:v>1264</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>1276</x:v>
+        <x:v>1265</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>1277</x:v>
+        <x:v>1266</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>1278</x:v>
+        <x:v>1267</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>1279</x:v>
+        <x:v>1268</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>1280</x:v>
+        <x:v>1269</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>1281</x:v>
+        <x:v>1270</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>1282</x:v>
+        <x:v>1271</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>1283</x:v>
+        <x:v>1272</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>2</x:v>
@@ -11794,31 +11761,31 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>1284</x:v>
+        <x:v>1273</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>1285</x:v>
+        <x:v>1274</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>1286</x:v>
+        <x:v>1275</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>1287</x:v>
+        <x:v>1276</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G18" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H18" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I18" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J18" s="3" t="s">
         <x:v>42</x:v>
@@ -11827,31 +11794,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>1288</x:v>
+        <x:v>1277</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>1289</x:v>
+        <x:v>1278</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>1290</x:v>
+        <x:v>1279</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>1291</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>1292</x:v>
+        <x:v>1281</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>1293</x:v>
+        <x:v>1282</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>1294</x:v>
+        <x:v>1283</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>1295</x:v>
+        <x:v>1284</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>1296</x:v>
+        <x:v>1285</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>2</x:v>
@@ -11859,31 +11826,31 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>1297</x:v>
+        <x:v>1286</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>1298</x:v>
+        <x:v>1287</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>1299</x:v>
+        <x:v>1288</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>1300</x:v>
+        <x:v>1289</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I19" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J19" s="3" t="s">
         <x:v>42</x:v>
@@ -11892,31 +11859,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>1301</x:v>
+        <x:v>1290</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>1302</x:v>
+        <x:v>1291</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>1303</x:v>
+        <x:v>1292</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>1304</x:v>
+        <x:v>1293</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>1305</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>1306</x:v>
+        <x:v>1295</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>1307</x:v>
+        <x:v>1296</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>1308</x:v>
+        <x:v>1297</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>1309</x:v>
+        <x:v>1298</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>2</x:v>
@@ -11924,31 +11891,31 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>1310</x:v>
+        <x:v>1299</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>1311</x:v>
+        <x:v>1300</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>1312</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>1313</x:v>
+        <x:v>1302</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I20" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J20" s="3" t="s">
         <x:v>42</x:v>
@@ -11957,31 +11924,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>1314</x:v>
+        <x:v>1303</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>1315</x:v>
+        <x:v>1304</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>1316</x:v>
+        <x:v>1305</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>1317</x:v>
+        <x:v>1306</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>1318</x:v>
+        <x:v>1307</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>1319</x:v>
+        <x:v>1308</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>1320</x:v>
+        <x:v>1309</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>1321</x:v>
+        <x:v>1310</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>1322</x:v>
+        <x:v>1311</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>2</x:v>
@@ -11989,31 +11956,31 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>1323</x:v>
+        <x:v>1312</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>1324</x:v>
+        <x:v>1313</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>1325</x:v>
+        <x:v>1314</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>1326</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G21" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H21" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I21" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J21" s="3" t="s">
         <x:v>42</x:v>
@@ -12022,31 +11989,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>1327</x:v>
+        <x:v>1316</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>1328</x:v>
+        <x:v>1317</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>1329</x:v>
+        <x:v>1318</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>1330</x:v>
+        <x:v>1319</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>1331</x:v>
+        <x:v>1320</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>1332</x:v>
+        <x:v>1321</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>1333</x:v>
+        <x:v>1322</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>2</x:v>
@@ -12054,31 +12021,31 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>1334</x:v>
+        <x:v>1323</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>1335</x:v>
+        <x:v>1324</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>1336</x:v>
+        <x:v>1325</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>1337</x:v>
+        <x:v>1326</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G22" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H22" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I22" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J22" s="3" t="s">
         <x:v>42</x:v>
@@ -12087,31 +12054,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>1338</x:v>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>1203</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>1339</x:v>
+        <x:v>1328</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>1340</x:v>
+        <x:v>1329</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>1341</x:v>
+        <x:v>1330</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>1342</x:v>
+        <x:v>1331</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>1343</x:v>
+        <x:v>1332</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>1344</x:v>
+        <x:v>1333</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>1345</x:v>
+        <x:v>1334</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>2</x:v>
@@ -12119,31 +12086,31 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>1346</x:v>
+        <x:v>1335</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>1347</x:v>
+        <x:v>1336</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>1348</x:v>
+        <x:v>1337</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>1349</x:v>
+        <x:v>1338</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G23" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H23" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I23" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J23" s="3" t="s">
         <x:v>42</x:v>
@@ -12152,31 +12119,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>1350</x:v>
+        <x:v>1339</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>1351</x:v>
+        <x:v>1340</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>1352</x:v>
+        <x:v>1341</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>1353</x:v>
+        <x:v>1342</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>1354</x:v>
+        <x:v>1343</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>1355</x:v>
+        <x:v>1344</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>1356</x:v>
+        <x:v>1345</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>1357</x:v>
+        <x:v>1346</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>1358</x:v>
+        <x:v>1347</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>2</x:v>
@@ -12184,31 +12151,31 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>1359</x:v>
+        <x:v>1348</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>1360</x:v>
+        <x:v>1349</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>1361</x:v>
+        <x:v>1350</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>1362</x:v>
+        <x:v>1351</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H24" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I24" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J24" s="3" t="s">
         <x:v>42</x:v>
@@ -12217,31 +12184,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>1363</x:v>
+        <x:v>1352</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>1328</x:v>
+        <x:v>1317</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>1364</x:v>
+        <x:v>1353</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>1365</x:v>
+        <x:v>1354</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>1366</x:v>
+        <x:v>1355</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>1367</x:v>
+        <x:v>1356</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>1368</x:v>
+        <x:v>1357</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>1369</x:v>
+        <x:v>1358</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>1370</x:v>
+        <x:v>1359</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>2</x:v>
@@ -12249,31 +12216,31 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>1371</x:v>
+        <x:v>1360</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>1372</x:v>
+        <x:v>1361</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>1373</x:v>
+        <x:v>1362</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>1374</x:v>
+        <x:v>1363</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H25" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I25" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J25" s="3" t="s">
         <x:v>42</x:v>
@@ -12282,31 +12249,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>1375</x:v>
+        <x:v>1364</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>1328</x:v>
+        <x:v>1317</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>1376</x:v>
+        <x:v>1365</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>1377</x:v>
+        <x:v>1366</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>1378</x:v>
+        <x:v>1367</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>1379</x:v>
+        <x:v>1368</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>1380</x:v>
+        <x:v>1369</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>1381</x:v>
+        <x:v>1370</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>1382</x:v>
+        <x:v>1371</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>2</x:v>
@@ -12314,31 +12281,31 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>1383</x:v>
+        <x:v>1372</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>1384</x:v>
+        <x:v>1373</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>1385</x:v>
+        <x:v>1374</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>1386</x:v>
+        <x:v>1375</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H26" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I26" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J26" s="3" t="s">
         <x:v>42</x:v>
@@ -12347,31 +12314,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>1387</x:v>
+        <x:v>1376</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>1388</x:v>
+        <x:v>1377</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>1389</x:v>
+        <x:v>1378</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>1390</x:v>
+        <x:v>1379</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>1391</x:v>
+        <x:v>1380</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>1392</x:v>
+        <x:v>1381</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>1393</x:v>
+        <x:v>1382</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>1394</x:v>
+        <x:v>1383</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>1395</x:v>
+        <x:v>1384</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>2</x:v>
@@ -12379,31 +12346,31 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>1396</x:v>
+        <x:v>1385</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>1397</x:v>
+        <x:v>1386</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>1398</x:v>
+        <x:v>1387</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>1399</x:v>
+        <x:v>1388</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H27" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I27" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J27" s="3" t="s">
         <x:v>42</x:v>
@@ -12412,31 +12379,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>1400</x:v>
+        <x:v>1389</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>1401</x:v>
+        <x:v>1390</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>1402</x:v>
+        <x:v>1391</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>1403</x:v>
+        <x:v>1392</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>1404</x:v>
+        <x:v>1393</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>1405</x:v>
+        <x:v>1394</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>1406</x:v>
+        <x:v>1395</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
         <x:v>789</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>1407</x:v>
+        <x:v>1396</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>2</x:v>
@@ -12444,31 +12411,31 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>1408</x:v>
+        <x:v>1397</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>1409</x:v>
+        <x:v>1398</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>1410</x:v>
+        <x:v>1399</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>1411</x:v>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G28" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H28" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I28" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J28" s="3" t="s">
         <x:v>42</x:v>
@@ -12477,31 +12444,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>1412</x:v>
+        <x:v>1401</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>1413</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>1414</x:v>
+        <x:v>1403</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>1415</x:v>
+        <x:v>1404</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>1416</x:v>
+        <x:v>1405</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>1417</x:v>
+        <x:v>1406</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>1418</x:v>
+        <x:v>1407</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>1419</x:v>
+        <x:v>1408</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>2</x:v>
@@ -12509,31 +12476,31 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>1420</x:v>
+        <x:v>1409</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>1421</x:v>
+        <x:v>1410</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>1422</x:v>
+        <x:v>1411</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>1423</x:v>
+        <x:v>1412</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G29" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H29" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I29" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J29" s="3" t="s">
         <x:v>42</x:v>
@@ -12542,31 +12509,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>1424</x:v>
+        <x:v>1413</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>1425</x:v>
+        <x:v>1414</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>1426</x:v>
+        <x:v>1415</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>1427</x:v>
+        <x:v>1416</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>1428</x:v>
+        <x:v>1417</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>1429</x:v>
+        <x:v>1418</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>1430</x:v>
+        <x:v>1419</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>1431</x:v>
+        <x:v>1420</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>1432</x:v>
+        <x:v>1421</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>2</x:v>
@@ -12574,31 +12541,31 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>1433</x:v>
+        <x:v>1422</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>1434</x:v>
+        <x:v>1423</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>1435</x:v>
+        <x:v>1424</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>1436</x:v>
+        <x:v>1425</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G30" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H30" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I30" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J30" s="3" t="s">
         <x:v>42</x:v>
@@ -12607,31 +12574,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>1437</x:v>
+        <x:v>1426</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>1438</x:v>
+        <x:v>1427</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>1439</x:v>
+        <x:v>1428</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>1440</x:v>
+        <x:v>1429</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>1441</x:v>
+        <x:v>1430</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>1442</x:v>
+        <x:v>1431</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>1443</x:v>
+        <x:v>1432</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>1444</x:v>
+        <x:v>1433</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>1445</x:v>
+        <x:v>1434</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>2</x:v>
@@ -12639,7 +12606,7 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>1446</x:v>
+        <x:v>1435</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>9</x:v>
@@ -12648,22 +12615,22 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>1447</x:v>
+        <x:v>1436</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>1448</x:v>
+        <x:v>1437</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G31" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H31" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I31" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J31" s="3" t="s">
         <x:v>42</x:v>
@@ -12672,31 +12639,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>1449</x:v>
+        <x:v>1438</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>1450</x:v>
+        <x:v>1439</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>1451</x:v>
+        <x:v>1440</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>1452</x:v>
+        <x:v>1441</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>1453</x:v>
+        <x:v>1442</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>1454</x:v>
+        <x:v>1443</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>1455</x:v>
+        <x:v>1444</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>1456</x:v>
+        <x:v>1445</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>1457</x:v>
+        <x:v>1446</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>2</x:v>
@@ -12704,31 +12671,31 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>1458</x:v>
+        <x:v>1447</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>1459</x:v>
+        <x:v>1448</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>1460</x:v>
+        <x:v>1449</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>1461</x:v>
+        <x:v>1450</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G32" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H32" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I32" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J32" s="3" t="s">
         <x:v>42</x:v>
@@ -12737,31 +12704,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>1462</x:v>
+        <x:v>1451</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>1463</x:v>
+        <x:v>1452</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>1464</x:v>
+        <x:v>1453</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>1465</x:v>
+        <x:v>1454</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>1466</x:v>
+        <x:v>1455</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>1467</x:v>
+        <x:v>1456</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
         <x:v>969</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>1468</x:v>
+        <x:v>1457</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>1469</x:v>
+        <x:v>1458</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>2</x:v>
@@ -12769,7 +12736,7 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>1470</x:v>
+        <x:v>1459</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>9</x:v>
@@ -12778,22 +12745,22 @@
         <x:v>740</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>1471</x:v>
+        <x:v>1460</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>1472</x:v>
+        <x:v>1461</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G33" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H33" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I33" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J33" s="3" t="s">
         <x:v>42</x:v>
@@ -12802,31 +12769,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>1473</x:v>
+        <x:v>1462</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>1474</x:v>
+        <x:v>1463</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>1475</x:v>
+        <x:v>1464</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>1476</x:v>
+        <x:v>1465</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>1477</x:v>
+        <x:v>1466</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>1478</x:v>
+        <x:v>1467</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>1479</x:v>
+        <x:v>1468</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>1480</x:v>
+        <x:v>1469</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>1481</x:v>
+        <x:v>1470</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>2</x:v>
@@ -12834,7 +12801,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>1482</x:v>
+        <x:v>1471</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>9</x:v>
@@ -12843,22 +12810,22 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>1483</x:v>
+        <x:v>1472</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>1484</x:v>
+        <x:v>1473</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G34" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H34" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I34" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J34" s="3" t="s">
         <x:v>42</x:v>
@@ -12867,31 +12834,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>1485</x:v>
+        <x:v>1474</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>1486</x:v>
+        <x:v>1475</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
         <x:v>978</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>1487</x:v>
+        <x:v>1476</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>1488</x:v>
+        <x:v>1477</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>1489</x:v>
+        <x:v>1478</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>1490</x:v>
+        <x:v>1479</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>1491</x:v>
+        <x:v>1480</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>2</x:v>
@@ -12899,31 +12866,31 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>1492</x:v>
+        <x:v>1481</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>1493</x:v>
+        <x:v>1482</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>1494</x:v>
+        <x:v>1483</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>1495</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G35" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H35" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I35" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J35" s="3" t="s">
         <x:v>42</x:v>
@@ -12932,31 +12899,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>1496</x:v>
+        <x:v>1485</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>1497</x:v>
+        <x:v>1486</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>1498</x:v>
+        <x:v>1487</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>1278</x:v>
+        <x:v>1267</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>1499</x:v>
+        <x:v>1488</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>1500</x:v>
+        <x:v>1489</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>1501</x:v>
+        <x:v>1490</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>1502</x:v>
+        <x:v>1491</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>1503</x:v>
+        <x:v>1492</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>2</x:v>
@@ -12964,31 +12931,31 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>1504</x:v>
+        <x:v>1493</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>1505</x:v>
+        <x:v>1494</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>1506</x:v>
+        <x:v>1495</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>1507</x:v>
+        <x:v>1496</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G36" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H36" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I36" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J36" s="3" t="s">
         <x:v>42</x:v>
@@ -12997,31 +12964,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>1508</x:v>
+        <x:v>1497</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>1509</x:v>
+        <x:v>1498</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>1510</x:v>
+        <x:v>1499</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>1511</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>1512</x:v>
+        <x:v>1501</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>1513</x:v>
+        <x:v>1502</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>1514</x:v>
+        <x:v>1503</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>1515</x:v>
+        <x:v>1504</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>2</x:v>
@@ -13029,31 +12996,31 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>1516</x:v>
+        <x:v>1505</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>1517</x:v>
+        <x:v>1506</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>1518</x:v>
+        <x:v>1507</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>1519</x:v>
+        <x:v>1508</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G37" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H37" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I37" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J37" s="3" t="s">
         <x:v>42</x:v>
@@ -13062,31 +13029,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>1520</x:v>
+        <x:v>1509</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>1521</x:v>
+        <x:v>1510</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>1522</x:v>
+        <x:v>1511</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>1523</x:v>
+        <x:v>1512</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>1524</x:v>
+        <x:v>1513</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>1525</x:v>
+        <x:v>1514</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>1526</x:v>
+        <x:v>1515</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>1527</x:v>
+        <x:v>1516</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>1521</x:v>
+        <x:v>1510</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>2</x:v>
@@ -13094,31 +13061,31 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>1528</x:v>
+        <x:v>1517</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>1529</x:v>
+        <x:v>1518</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>1530</x:v>
+        <x:v>1519</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>1531</x:v>
+        <x:v>1520</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G38" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H38" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I38" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J38" s="3" t="s">
         <x:v>42</x:v>
@@ -13127,31 +13094,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>1532</x:v>
+        <x:v>1521</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>1203</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>1533</x:v>
+        <x:v>1522</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>1534</x:v>
+        <x:v>1523</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>1535</x:v>
+        <x:v>1524</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>1536</x:v>
+        <x:v>1525</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>1537</x:v>
+        <x:v>1526</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>1538</x:v>
+        <x:v>1527</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>1539</x:v>
+        <x:v>1528</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>2</x:v>
@@ -13159,31 +13126,31 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>1540</x:v>
+        <x:v>1529</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>1541</x:v>
+        <x:v>1530</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>1542</x:v>
+        <x:v>1531</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>1543</x:v>
+        <x:v>1532</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G39" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="H39" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="I39" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="J39" s="3" t="s">
         <x:v>42</x:v>
@@ -13192,31 +13159,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>1544</x:v>
+        <x:v>1533</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>1545</x:v>
+        <x:v>1534</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>1546</x:v>
+        <x:v>1535</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>1547</x:v>
+        <x:v>1536</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>1548</x:v>
+        <x:v>1537</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>1549</x:v>
+        <x:v>1538</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>1550</x:v>
+        <x:v>1539</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>1551</x:v>
+        <x:v>1540</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>2</x:v>
@@ -13225,7 +13192,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R097691cdae724974"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58e8ce8d152f43f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-050 config diagnostics tests
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Recba917fce4e47a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rd28cc1ae787c42ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R8bd7a0686ffc465d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R9b3c2a324e4f4f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R620d757063874a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3b42b5c4788c4997"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R7e472c98811b4243"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R120db2cb611d466c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3194,39 +3194,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">PerformanceController.cs:17-36; ChatDrawer.razor:409</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">INT-050</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Client runtime config and diagnostics</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As an employee or operator, I can bootstrap the intranet client configuration and inspect my effective diagnostic identity.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Config endpoint returns client runtime settings and diagnostics endpoint returns current user/session/permission context.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Client bootstrap/diagnostics -&gt; BFF config and IAM diagnostic boundary</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ClientConfigController.cs; DiagnosticsController.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Client bootstrap; /api/v1/diagnostics/me</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ClientConfigController GET config/client; DiagnosticsController GET me</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Read-only runtime config and diagnostic context</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs access-control and environment-value review.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ClientConfigController.cs:14-46; DiagnosticsController.cs:15-25</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QE-001</x:t>
@@ -7205,7 +7172,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b883387c6dd487a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R154e6f3cd90e41a1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10489,68 +10456,68 @@
       </x:c>
     </x:row>
     <x:row r="51" ht="51.29999923706055" hidden="0">
-      <x:c r="A51" s="3" t="s">
-        <x:v>1061</x:v>
-      </x:c>
-      <x:c r="B51" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C51" s="3" t="s">
-        <x:v>1062</x:v>
-      </x:c>
-      <x:c r="D51" s="3" t="s">
-        <x:v>1063</x:v>
-      </x:c>
-      <x:c r="E51" s="3" t="s">
-        <x:v>1064</x:v>
-      </x:c>
-      <x:c r="F51" s="3" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="G51" s="3" t="s">
-        <x:v>1001</x:v>
-      </x:c>
-      <x:c r="H51" s="3" t="s">
-        <x:v>1002</x:v>
-      </x:c>
-      <x:c r="I51" s="3" t="s">
-        <x:v>1003</x:v>
-      </x:c>
-      <x:c r="J51" s="3" t="s">
-        <x:v>1004</x:v>
-      </x:c>
-      <x:c r="K51" s="3" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="L51" s="3" t="s">
-        <x:v>1065</x:v>
-      </x:c>
-      <x:c r="M51" s="3" t="s">
-        <x:v>1066</x:v>
-      </x:c>
-      <x:c r="N51" s="3" t="s">
-        <x:v>1067</x:v>
-      </x:c>
-      <x:c r="O51" s="3" t="s">
-        <x:v>1068</x:v>
-      </x:c>
-      <x:c r="P51" s="3" t="s">
-        <x:v>1009</x:v>
-      </x:c>
-      <x:c r="Q51" s="3" t="s">
-        <x:v>852</x:v>
-      </x:c>
-      <x:c r="R51" s="3" t="s">
-        <x:v>1069</x:v>
-      </x:c>
-      <x:c r="S51" s="3" t="s">
-        <x:v>1070</x:v>
-      </x:c>
-      <x:c r="T51" s="3" t="s">
-        <x:v>1071</x:v>
-      </x:c>
-      <x:c r="U51" s="3" t="s">
-        <x:v>2</x:v>
+      <x:c r="A51" s="3" t="str">
+        <x:v>INT-050</x:v>
+      </x:c>
+      <x:c r="B51" s="3" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C51" s="3" t="str">
+        <x:v>Client runtime config and diagnostics</x:v>
+      </x:c>
+      <x:c r="D51" s="3" t="str">
+        <x:v>As an employee or operator, I can bootstrap the intranet client configuration and inspect my effective diagnostic identity.</x:v>
+      </x:c>
+      <x:c r="E51" s="3" t="str">
+        <x:v>Config endpoint returns client runtime settings and diagnostics endpoint returns current user/session/permission context.</x:v>
+      </x:c>
+      <x:c r="F51" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G51" s="3" t="str">
+        <x:v>Focused behavior tests passed 2026-06-23.</x:v>
+      </x:c>
+      <x:c r="H51" s="3" t="str">
+        <x:v>No behavior error observed in current focused controller retest.</x:v>
+      </x:c>
+      <x:c r="I51" s="3" t="str">
+        <x:v>No app-code fix needed; added missing focused coverage in Maliev.Intranet commit 9af6f3e.</x:v>
+      </x:c>
+      <x:c r="J51" s="3" t="str">
+        <x:v>Retested focused ClientConfig/Diagnostics controller set 5/5 passed.</x:v>
+      </x:c>
+      <x:c r="K51" s="3" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L51" s="3" t="str">
+        <x:v>Client bootstrap/diagnostics -&gt; BFF config and IAM diagnostic boundary</x:v>
+      </x:c>
+      <x:c r="M51" s="3" t="str">
+        <x:v>ClientConfigController.cs; DiagnosticsController.cs</x:v>
+      </x:c>
+      <x:c r="N51" s="3" t="str">
+        <x:v>Client bootstrap; /api/v1/diagnostics/me</x:v>
+      </x:c>
+      <x:c r="O51" s="3" t="str">
+        <x:v>ClientConfigController GET config/client; DiagnosticsController GET me</x:v>
+      </x:c>
+      <x:c r="P51" s="3" t="str">
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~QuickControllerTests.ClientConfig|FullyQualifiedName~QuickControllerTests.Diagnostics" --verbosity minimal passed 5/5 on 2026-06-23. Coverage verifies default/configured client processing timeout, diagnostics effective identity payload, IAM resolution payload, and diagnostics read permission requirement.</x:v>
+      </x:c>
+      <x:c r="Q51" s="3" t="str">
+        <x:v>Intranet BFF, IAMService</x:v>
+      </x:c>
+      <x:c r="R51" s="3" t="str">
+        <x:v>Read-only runtime config and diagnostic context</x:v>
+      </x:c>
+      <x:c r="S51" s="3" t="str">
+        <x:v>No remaining INT-050 controller-contract gap from this focused retest; full authenticated browser/API middleware pass still needed in Aspire-configured runtime.</x:v>
+      </x:c>
+      <x:c r="T51" s="3" t="str">
+        <x:v>ClientConfigController.cs:15-39; DiagnosticsController.cs:13-45; QuickControllerTests.cs:358-449</x:v>
+      </x:c>
+      <x:c r="U51" s="3" t="str">
+        <x:v>2026-06-23</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="51.29999923706055" hidden="0">
@@ -10621,7 +10588,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c18b4856e2c44ea"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad6f22be4874441d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10721,64 +10688,64 @@
     </x:row>
     <x:row r="2" ht="149.25" hidden="0">
       <x:c r="A2" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>1073</x:v>
+        <x:v>1062</x:v>
       </x:c>
       <x:c r="D2" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="E2" s="3" t="s">
-        <x:v>1075</x:v>
+        <x:v>1064</x:v>
       </x:c>
       <x:c r="F2" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>1076</x:v>
+        <x:v>1065</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>1077</x:v>
+        <x:v>1066</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>1078</x:v>
+        <x:v>1067</x:v>
       </x:c>
       <x:c r="J2" s="3" t="s">
-        <x:v>1079</x:v>
+        <x:v>1068</x:v>
       </x:c>
       <x:c r="K2" s="3" t="s">
         <x:v>188</x:v>
       </x:c>
       <x:c r="L2" s="3" t="s">
-        <x:v>1080</x:v>
+        <x:v>1069</x:v>
       </x:c>
       <x:c r="M2" s="3" t="s">
-        <x:v>1081</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="N2" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="O2" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="P2" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1073</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="s">
-        <x:v>1085</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="R2" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1075</x:v>
       </x:c>
       <x:c r="S2" s="3" t="s">
-        <x:v>1087</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="T2" s="3" t="s">
-        <x:v>1088</x:v>
+        <x:v>1077</x:v>
       </x:c>
       <x:c r="U2" s="3" t="s">
         <x:v>2</x:v>
@@ -10786,31 +10753,31 @@
     </x:row>
     <x:row r="3" ht="107.25" hidden="0">
       <x:c r="A3" s="3" t="s">
-        <x:v>1089</x:v>
+        <x:v>1078</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>1090</x:v>
+        <x:v>1079</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>1091</x:v>
+        <x:v>1080</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>1092</x:v>
+        <x:v>1081</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G3" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H3" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I3" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J3" s="3" t="s">
         <x:v>42</x:v>
@@ -10819,31 +10786,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L3" s="3" t="s">
-        <x:v>1096</x:v>
+        <x:v>1085</x:v>
       </x:c>
       <x:c r="M3" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N3" s="3" t="s">
-        <x:v>1098</x:v>
+        <x:v>1087</x:v>
       </x:c>
       <x:c r="O3" s="3" t="s">
-        <x:v>1099</x:v>
+        <x:v>1088</x:v>
       </x:c>
       <x:c r="P3" s="3" t="s">
-        <x:v>1100</x:v>
+        <x:v>1089</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="s">
-        <x:v>1101</x:v>
+        <x:v>1090</x:v>
       </x:c>
       <x:c r="R3" s="3" t="s">
-        <x:v>1102</x:v>
+        <x:v>1091</x:v>
       </x:c>
       <x:c r="S3" s="3" t="s">
-        <x:v>1103</x:v>
+        <x:v>1092</x:v>
       </x:c>
       <x:c r="T3" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="U3" s="3" t="s">
         <x:v>2</x:v>
@@ -10851,31 +10818,31 @@
     </x:row>
     <x:row r="4" ht="93.25" hidden="0">
       <x:c r="A4" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>1107</x:v>
+        <x:v>1096</x:v>
       </x:c>
       <x:c r="E4" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G4" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H4" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I4" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J4" s="3" t="s">
         <x:v>42</x:v>
@@ -10884,31 +10851,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L4" s="3" t="s">
-        <x:v>1109</x:v>
+        <x:v>1098</x:v>
       </x:c>
       <x:c r="M4" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N4" s="3" t="s">
-        <x:v>1110</x:v>
+        <x:v>1099</x:v>
       </x:c>
       <x:c r="O4" s="3" t="s">
-        <x:v>1111</x:v>
+        <x:v>1100</x:v>
       </x:c>
       <x:c r="P4" s="3" t="s">
-        <x:v>1112</x:v>
+        <x:v>1101</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="s">
-        <x:v>1113</x:v>
+        <x:v>1102</x:v>
       </x:c>
       <x:c r="R4" s="3" t="s">
-        <x:v>1114</x:v>
+        <x:v>1103</x:v>
       </x:c>
       <x:c r="S4" s="3" t="s">
-        <x:v>1115</x:v>
+        <x:v>1104</x:v>
       </x:c>
       <x:c r="T4" s="3" t="s">
-        <x:v>1116</x:v>
+        <x:v>1105</x:v>
       </x:c>
       <x:c r="U4" s="3" t="s">
         <x:v>2</x:v>
@@ -10916,31 +10883,31 @@
     </x:row>
     <x:row r="5" ht="107.25" hidden="0">
       <x:c r="A5" s="3" t="s">
-        <x:v>1117</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>1118</x:v>
+        <x:v>1107</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>1119</x:v>
+        <x:v>1108</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>1120</x:v>
+        <x:v>1109</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
         <x:v>42</x:v>
@@ -10949,31 +10916,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>1121</x:v>
+        <x:v>1110</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>1122</x:v>
+        <x:v>1111</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>1123</x:v>
+        <x:v>1112</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>1124</x:v>
+        <x:v>1113</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>1125</x:v>
+        <x:v>1114</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>1126</x:v>
+        <x:v>1115</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>1127</x:v>
+        <x:v>1116</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>1128</x:v>
+        <x:v>1117</x:v>
       </x:c>
       <x:c r="U5" s="3" t="s">
         <x:v>2</x:v>
@@ -10981,31 +10948,31 @@
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
       <x:c r="A6" s="3" t="s">
-        <x:v>1129</x:v>
+        <x:v>1118</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>1130</x:v>
+        <x:v>1119</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>1131</x:v>
+        <x:v>1120</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>1132</x:v>
+        <x:v>1121</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H6" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I6" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J6" s="3" t="s">
         <x:v>42</x:v>
@@ -11014,31 +10981,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L6" s="3" t="s">
-        <x:v>1133</x:v>
+        <x:v>1122</x:v>
       </x:c>
       <x:c r="M6" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N6" s="3" t="s">
-        <x:v>1134</x:v>
+        <x:v>1123</x:v>
       </x:c>
       <x:c r="O6" s="3" t="s">
-        <x:v>1135</x:v>
+        <x:v>1124</x:v>
       </x:c>
       <x:c r="P6" s="3" t="s">
-        <x:v>1136</x:v>
+        <x:v>1125</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="s">
-        <x:v>1137</x:v>
+        <x:v>1126</x:v>
       </x:c>
       <x:c r="R6" s="3" t="s">
-        <x:v>1138</x:v>
+        <x:v>1127</x:v>
       </x:c>
       <x:c r="S6" s="3" t="s">
-        <x:v>1139</x:v>
+        <x:v>1128</x:v>
       </x:c>
       <x:c r="T6" s="3" t="s">
-        <x:v>1140</x:v>
+        <x:v>1129</x:v>
       </x:c>
       <x:c r="U6" s="3" t="s">
         <x:v>2</x:v>
@@ -11046,31 +11013,31 @@
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>1141</x:v>
+        <x:v>1130</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>1142</x:v>
+        <x:v>1131</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>1143</x:v>
+        <x:v>1132</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>1144</x:v>
+        <x:v>1133</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G7" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H7" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I7" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J7" s="3" t="s">
         <x:v>42</x:v>
@@ -11079,31 +11046,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
-        <x:v>1145</x:v>
+        <x:v>1134</x:v>
       </x:c>
       <x:c r="M7" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N7" s="3" t="s">
-        <x:v>1146</x:v>
+        <x:v>1135</x:v>
       </x:c>
       <x:c r="O7" s="3" t="s">
-        <x:v>1147</x:v>
+        <x:v>1136</x:v>
       </x:c>
       <x:c r="P7" s="3" t="s">
-        <x:v>1148</x:v>
+        <x:v>1137</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="s">
-        <x:v>1101</x:v>
+        <x:v>1090</x:v>
       </x:c>
       <x:c r="R7" s="3" t="s">
-        <x:v>1149</x:v>
+        <x:v>1138</x:v>
       </x:c>
       <x:c r="S7" s="3" t="s">
-        <x:v>1150</x:v>
+        <x:v>1139</x:v>
       </x:c>
       <x:c r="T7" s="3" t="s">
-        <x:v>1151</x:v>
+        <x:v>1140</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>2</x:v>
@@ -11111,31 +11078,31 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>1152</x:v>
+        <x:v>1141</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>1153</x:v>
+        <x:v>1142</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>1154</x:v>
+        <x:v>1143</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>1155</x:v>
+        <x:v>1144</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H8" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I8" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J8" s="3" t="s">
         <x:v>42</x:v>
@@ -11144,31 +11111,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
-        <x:v>1156</x:v>
+        <x:v>1145</x:v>
       </x:c>
       <x:c r="M8" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N8" s="3" t="s">
-        <x:v>1157</x:v>
+        <x:v>1146</x:v>
       </x:c>
       <x:c r="O8" s="3" t="s">
-        <x:v>1158</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="P8" s="3" t="s">
-        <x:v>1159</x:v>
+        <x:v>1148</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="s">
-        <x:v>1160</x:v>
+        <x:v>1149</x:v>
       </x:c>
       <x:c r="R8" s="3" t="s">
-        <x:v>1161</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="S8" s="3" t="s">
-        <x:v>1162</x:v>
+        <x:v>1151</x:v>
       </x:c>
       <x:c r="T8" s="3" t="s">
-        <x:v>1163</x:v>
+        <x:v>1152</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>2</x:v>
@@ -11176,31 +11143,31 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>1164</x:v>
+        <x:v>1153</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>1165</x:v>
+        <x:v>1154</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>1166</x:v>
+        <x:v>1155</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>1167</x:v>
+        <x:v>1156</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H9" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I9" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J9" s="3" t="s">
         <x:v>42</x:v>
@@ -11209,31 +11176,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
-        <x:v>1168</x:v>
+        <x:v>1157</x:v>
       </x:c>
       <x:c r="M9" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N9" s="3" t="s">
-        <x:v>1169</x:v>
+        <x:v>1158</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>1170</x:v>
+        <x:v>1159</x:v>
       </x:c>
       <x:c r="P9" s="3" t="s">
-        <x:v>1171</x:v>
+        <x:v>1160</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="s">
-        <x:v>1172</x:v>
+        <x:v>1161</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
-        <x:v>1173</x:v>
+        <x:v>1162</x:v>
       </x:c>
       <x:c r="S9" s="3" t="s">
-        <x:v>1174</x:v>
+        <x:v>1163</x:v>
       </x:c>
       <x:c r="T9" s="3" t="s">
-        <x:v>1175</x:v>
+        <x:v>1164</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>2</x:v>
@@ -11241,31 +11208,31 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>1176</x:v>
+        <x:v>1165</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>1177</x:v>
+        <x:v>1166</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>1178</x:v>
+        <x:v>1167</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>1179</x:v>
+        <x:v>1168</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G10" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H10" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I10" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J10" s="3" t="s">
         <x:v>42</x:v>
@@ -11274,31 +11241,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>1180</x:v>
+        <x:v>1169</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
-        <x:v>1081</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>1181</x:v>
+        <x:v>1170</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>1182</x:v>
+        <x:v>1171</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>1183</x:v>
+        <x:v>1172</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>1184</x:v>
+        <x:v>1173</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>1185</x:v>
+        <x:v>1174</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>1186</x:v>
+        <x:v>1175</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>2</x:v>
@@ -11306,31 +11273,31 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>1187</x:v>
+        <x:v>1176</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>1188</x:v>
+        <x:v>1177</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>1189</x:v>
+        <x:v>1178</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>1190</x:v>
+        <x:v>1179</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G11" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H11" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I11" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J11" s="3" t="s">
         <x:v>42</x:v>
@@ -11339,31 +11306,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>1191</x:v>
+        <x:v>1180</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>1192</x:v>
+        <x:v>1181</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>1193</x:v>
+        <x:v>1182</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>1194</x:v>
+        <x:v>1183</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>1195</x:v>
+        <x:v>1184</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>1196</x:v>
+        <x:v>1185</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>1197</x:v>
+        <x:v>1186</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>1198</x:v>
+        <x:v>1187</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>1199</x:v>
+        <x:v>1188</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>2</x:v>
@@ -11371,31 +11338,31 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>1200</x:v>
+        <x:v>1189</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>1201</x:v>
+        <x:v>1190</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>1202</x:v>
+        <x:v>1191</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>1203</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G12" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H12" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I12" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J12" s="3" t="s">
         <x:v>42</x:v>
@@ -11404,31 +11371,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>1204</x:v>
+        <x:v>1193</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>1205</x:v>
+        <x:v>1194</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>1206</x:v>
+        <x:v>1195</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>1207</x:v>
+        <x:v>1196</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>1208</x:v>
+        <x:v>1197</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>1209</x:v>
+        <x:v>1198</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>1210</x:v>
+        <x:v>1199</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>1211</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>2</x:v>
@@ -11436,31 +11403,31 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>1212</x:v>
+        <x:v>1201</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>1213</x:v>
+        <x:v>1202</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>1214</x:v>
+        <x:v>1203</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>1215</x:v>
+        <x:v>1204</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I13" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J13" s="3" t="s">
         <x:v>42</x:v>
@@ -11469,31 +11436,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>1216</x:v>
+        <x:v>1205</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>1217</x:v>
+        <x:v>1206</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>1218</x:v>
+        <x:v>1207</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>1219</x:v>
+        <x:v>1208</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
-        <x:v>1208</x:v>
+        <x:v>1197</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>1220</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>1221</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>1222</x:v>
+        <x:v>1211</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>2</x:v>
@@ -11501,31 +11468,31 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>1223</x:v>
+        <x:v>1212</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>1224</x:v>
+        <x:v>1213</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>1225</x:v>
+        <x:v>1214</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>1226</x:v>
+        <x:v>1215</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G14" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H14" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I14" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J14" s="3" t="s">
         <x:v>42</x:v>
@@ -11534,31 +11501,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>1227</x:v>
+        <x:v>1216</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>1228</x:v>
+        <x:v>1217</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>1229</x:v>
+        <x:v>1218</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>1230</x:v>
+        <x:v>1219</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>1231</x:v>
+        <x:v>1220</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>1232</x:v>
+        <x:v>1221</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>1233</x:v>
+        <x:v>1222</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>1234</x:v>
+        <x:v>1223</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>1235</x:v>
+        <x:v>1224</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>2</x:v>
@@ -11566,31 +11533,31 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>1236</x:v>
+        <x:v>1225</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>1237</x:v>
+        <x:v>1226</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>1238</x:v>
+        <x:v>1227</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>1239</x:v>
+        <x:v>1228</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G15" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H15" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I15" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J15" s="3" t="s">
         <x:v>42</x:v>
@@ -11599,31 +11566,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>1240</x:v>
+        <x:v>1229</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>1241</x:v>
+        <x:v>1230</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>1242</x:v>
+        <x:v>1231</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>1243</x:v>
+        <x:v>1232</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>1244</x:v>
+        <x:v>1233</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>1245</x:v>
+        <x:v>1234</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>1246</x:v>
+        <x:v>1235</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>1247</x:v>
+        <x:v>1236</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>2</x:v>
@@ -11631,31 +11598,31 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>1248</x:v>
+        <x:v>1237</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>1249</x:v>
+        <x:v>1238</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>1250</x:v>
+        <x:v>1239</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>1251</x:v>
+        <x:v>1240</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H16" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I16" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J16" s="3" t="s">
         <x:v>42</x:v>
@@ -11664,31 +11631,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>1252</x:v>
+        <x:v>1241</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>1253</x:v>
+        <x:v>1242</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>1254</x:v>
+        <x:v>1243</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>1255</x:v>
+        <x:v>1244</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>1256</x:v>
+        <x:v>1245</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>1257</x:v>
+        <x:v>1246</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>1258</x:v>
+        <x:v>1247</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>1259</x:v>
+        <x:v>1248</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>2</x:v>
@@ -11696,31 +11663,31 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>1260</x:v>
+        <x:v>1249</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>1261</x:v>
+        <x:v>1250</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>1262</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>1263</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H17" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I17" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J17" s="3" t="s">
         <x:v>42</x:v>
@@ -11729,31 +11696,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>1264</x:v>
+        <x:v>1253</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>1265</x:v>
+        <x:v>1254</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>1266</x:v>
+        <x:v>1255</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>1267</x:v>
+        <x:v>1256</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>1268</x:v>
+        <x:v>1257</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>1269</x:v>
+        <x:v>1258</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>1270</x:v>
+        <x:v>1259</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>1271</x:v>
+        <x:v>1260</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>1272</x:v>
+        <x:v>1261</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>2</x:v>
@@ -11761,31 +11728,31 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>1273</x:v>
+        <x:v>1262</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>1274</x:v>
+        <x:v>1263</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>1275</x:v>
+        <x:v>1264</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>1276</x:v>
+        <x:v>1265</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G18" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H18" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I18" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J18" s="3" t="s">
         <x:v>42</x:v>
@@ -11794,31 +11761,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>1277</x:v>
+        <x:v>1266</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>1278</x:v>
+        <x:v>1267</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>1279</x:v>
+        <x:v>1268</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>1280</x:v>
+        <x:v>1269</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>1281</x:v>
+        <x:v>1270</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>1282</x:v>
+        <x:v>1271</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>1283</x:v>
+        <x:v>1272</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>1284</x:v>
+        <x:v>1273</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>1285</x:v>
+        <x:v>1274</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>2</x:v>
@@ -11826,31 +11793,31 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>1286</x:v>
+        <x:v>1275</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>1287</x:v>
+        <x:v>1276</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>1288</x:v>
+        <x:v>1277</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>1289</x:v>
+        <x:v>1278</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I19" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J19" s="3" t="s">
         <x:v>42</x:v>
@@ -11859,31 +11826,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>1290</x:v>
+        <x:v>1279</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>1291</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>1292</x:v>
+        <x:v>1281</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>1293</x:v>
+        <x:v>1282</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>1294</x:v>
+        <x:v>1283</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>1295</x:v>
+        <x:v>1284</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>1296</x:v>
+        <x:v>1285</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>1297</x:v>
+        <x:v>1286</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>1298</x:v>
+        <x:v>1287</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>2</x:v>
@@ -11891,31 +11858,31 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>1299</x:v>
+        <x:v>1288</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>1300</x:v>
+        <x:v>1289</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>1301</x:v>
+        <x:v>1290</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>1302</x:v>
+        <x:v>1291</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I20" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J20" s="3" t="s">
         <x:v>42</x:v>
@@ -11924,31 +11891,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>1303</x:v>
+        <x:v>1292</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>1304</x:v>
+        <x:v>1293</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>1305</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>1306</x:v>
+        <x:v>1295</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>1307</x:v>
+        <x:v>1296</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>1308</x:v>
+        <x:v>1297</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>1309</x:v>
+        <x:v>1298</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>1310</x:v>
+        <x:v>1299</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>1311</x:v>
+        <x:v>1300</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>2</x:v>
@@ -11956,31 +11923,31 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>1312</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>1313</x:v>
+        <x:v>1302</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>1314</x:v>
+        <x:v>1303</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>1315</x:v>
+        <x:v>1304</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G21" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H21" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I21" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J21" s="3" t="s">
         <x:v>42</x:v>
@@ -11989,31 +11956,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>1316</x:v>
+        <x:v>1305</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>1317</x:v>
+        <x:v>1306</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>1318</x:v>
+        <x:v>1307</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>1319</x:v>
+        <x:v>1308</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>1320</x:v>
+        <x:v>1309</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>1321</x:v>
+        <x:v>1310</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>1322</x:v>
+        <x:v>1311</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>2</x:v>
@@ -12021,31 +11988,31 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>1323</x:v>
+        <x:v>1312</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>1324</x:v>
+        <x:v>1313</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>1325</x:v>
+        <x:v>1314</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>1326</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G22" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H22" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I22" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J22" s="3" t="s">
         <x:v>42</x:v>
@@ -12054,31 +12021,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>1327</x:v>
+        <x:v>1316</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>1192</x:v>
+        <x:v>1181</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>1328</x:v>
+        <x:v>1317</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>1329</x:v>
+        <x:v>1318</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>1330</x:v>
+        <x:v>1319</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>1331</x:v>
+        <x:v>1320</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>1332</x:v>
+        <x:v>1321</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>1333</x:v>
+        <x:v>1322</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>1334</x:v>
+        <x:v>1323</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>2</x:v>
@@ -12086,31 +12053,31 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>1335</x:v>
+        <x:v>1324</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>1336</x:v>
+        <x:v>1325</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>1337</x:v>
+        <x:v>1326</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>1338</x:v>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G23" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H23" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I23" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J23" s="3" t="s">
         <x:v>42</x:v>
@@ -12119,31 +12086,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>1339</x:v>
+        <x:v>1328</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>1340</x:v>
+        <x:v>1329</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>1341</x:v>
+        <x:v>1330</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>1342</x:v>
+        <x:v>1331</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>1343</x:v>
+        <x:v>1332</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>1344</x:v>
+        <x:v>1333</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>1345</x:v>
+        <x:v>1334</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>1346</x:v>
+        <x:v>1335</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>1347</x:v>
+        <x:v>1336</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>2</x:v>
@@ -12151,31 +12118,31 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>1348</x:v>
+        <x:v>1337</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>1349</x:v>
+        <x:v>1338</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>1350</x:v>
+        <x:v>1339</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>1351</x:v>
+        <x:v>1340</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H24" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I24" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J24" s="3" t="s">
         <x:v>42</x:v>
@@ -12184,31 +12151,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>1352</x:v>
+        <x:v>1341</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>1317</x:v>
+        <x:v>1306</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>1353</x:v>
+        <x:v>1342</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>1354</x:v>
+        <x:v>1343</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>1355</x:v>
+        <x:v>1344</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>1356</x:v>
+        <x:v>1345</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>1357</x:v>
+        <x:v>1346</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>1358</x:v>
+        <x:v>1347</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>1359</x:v>
+        <x:v>1348</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>2</x:v>
@@ -12216,31 +12183,31 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>1360</x:v>
+        <x:v>1349</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>1361</x:v>
+        <x:v>1350</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>1362</x:v>
+        <x:v>1351</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>1363</x:v>
+        <x:v>1352</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H25" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I25" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J25" s="3" t="s">
         <x:v>42</x:v>
@@ -12249,31 +12216,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>1364</x:v>
+        <x:v>1353</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>1317</x:v>
+        <x:v>1306</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>1365</x:v>
+        <x:v>1354</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>1366</x:v>
+        <x:v>1355</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>1367</x:v>
+        <x:v>1356</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>1368</x:v>
+        <x:v>1357</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>1369</x:v>
+        <x:v>1358</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>1370</x:v>
+        <x:v>1359</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>1371</x:v>
+        <x:v>1360</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>2</x:v>
@@ -12281,31 +12248,31 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>1372</x:v>
+        <x:v>1361</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>1373</x:v>
+        <x:v>1362</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>1374</x:v>
+        <x:v>1363</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>1375</x:v>
+        <x:v>1364</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H26" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I26" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J26" s="3" t="s">
         <x:v>42</x:v>
@@ -12314,31 +12281,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>1376</x:v>
+        <x:v>1365</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>1377</x:v>
+        <x:v>1366</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>1378</x:v>
+        <x:v>1367</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>1379</x:v>
+        <x:v>1368</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>1380</x:v>
+        <x:v>1369</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>1381</x:v>
+        <x:v>1370</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>1382</x:v>
+        <x:v>1371</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>1383</x:v>
+        <x:v>1372</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>1384</x:v>
+        <x:v>1373</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>2</x:v>
@@ -12346,31 +12313,31 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>1385</x:v>
+        <x:v>1374</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>1386</x:v>
+        <x:v>1375</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>1387</x:v>
+        <x:v>1376</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>1388</x:v>
+        <x:v>1377</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H27" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I27" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J27" s="3" t="s">
         <x:v>42</x:v>
@@ -12379,31 +12346,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>1389</x:v>
+        <x:v>1378</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>1390</x:v>
+        <x:v>1379</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>1391</x:v>
+        <x:v>1380</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>1392</x:v>
+        <x:v>1381</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>1393</x:v>
+        <x:v>1382</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>1394</x:v>
+        <x:v>1383</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>1395</x:v>
+        <x:v>1384</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
         <x:v>789</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>1396</x:v>
+        <x:v>1385</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>2</x:v>
@@ -12411,31 +12378,31 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>1397</x:v>
+        <x:v>1386</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>1398</x:v>
+        <x:v>1387</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>1399</x:v>
+        <x:v>1388</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>1400</x:v>
+        <x:v>1389</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G28" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H28" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I28" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J28" s="3" t="s">
         <x:v>42</x:v>
@@ -12444,31 +12411,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>1401</x:v>
+        <x:v>1390</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>1402</x:v>
+        <x:v>1391</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>1403</x:v>
+        <x:v>1392</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>1404</x:v>
+        <x:v>1393</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>1405</x:v>
+        <x:v>1394</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>1406</x:v>
+        <x:v>1395</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>1407</x:v>
+        <x:v>1396</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>1408</x:v>
+        <x:v>1397</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>2</x:v>
@@ -12476,31 +12443,31 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>1409</x:v>
+        <x:v>1398</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>1410</x:v>
+        <x:v>1399</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>1411</x:v>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>1412</x:v>
+        <x:v>1401</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G29" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H29" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I29" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J29" s="3" t="s">
         <x:v>42</x:v>
@@ -12509,31 +12476,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>1413</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>1414</x:v>
+        <x:v>1403</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>1415</x:v>
+        <x:v>1404</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>1416</x:v>
+        <x:v>1405</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>1417</x:v>
+        <x:v>1406</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>1418</x:v>
+        <x:v>1407</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>1419</x:v>
+        <x:v>1408</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>1420</x:v>
+        <x:v>1409</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>1421</x:v>
+        <x:v>1410</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>2</x:v>
@@ -12541,31 +12508,31 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>1422</x:v>
+        <x:v>1411</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>1423</x:v>
+        <x:v>1412</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>1424</x:v>
+        <x:v>1413</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>1425</x:v>
+        <x:v>1414</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G30" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H30" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I30" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J30" s="3" t="s">
         <x:v>42</x:v>
@@ -12574,31 +12541,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>1426</x:v>
+        <x:v>1415</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>1427</x:v>
+        <x:v>1416</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>1428</x:v>
+        <x:v>1417</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>1429</x:v>
+        <x:v>1418</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>1430</x:v>
+        <x:v>1419</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>1431</x:v>
+        <x:v>1420</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>1432</x:v>
+        <x:v>1421</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>1433</x:v>
+        <x:v>1422</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>1434</x:v>
+        <x:v>1423</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>2</x:v>
@@ -12606,7 +12573,7 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>1435</x:v>
+        <x:v>1424</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>9</x:v>
@@ -12615,22 +12582,22 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>1436</x:v>
+        <x:v>1425</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>1437</x:v>
+        <x:v>1426</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G31" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H31" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I31" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J31" s="3" t="s">
         <x:v>42</x:v>
@@ -12639,31 +12606,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>1438</x:v>
+        <x:v>1427</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>1439</x:v>
+        <x:v>1428</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>1440</x:v>
+        <x:v>1429</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>1441</x:v>
+        <x:v>1430</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>1442</x:v>
+        <x:v>1431</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>1443</x:v>
+        <x:v>1432</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>1444</x:v>
+        <x:v>1433</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>1445</x:v>
+        <x:v>1434</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>1446</x:v>
+        <x:v>1435</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>2</x:v>
@@ -12671,31 +12638,31 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>1447</x:v>
+        <x:v>1436</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>1448</x:v>
+        <x:v>1437</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>1449</x:v>
+        <x:v>1438</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>1450</x:v>
+        <x:v>1439</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G32" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H32" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I32" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J32" s="3" t="s">
         <x:v>42</x:v>
@@ -12704,31 +12671,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>1451</x:v>
+        <x:v>1440</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>1452</x:v>
+        <x:v>1441</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>1453</x:v>
+        <x:v>1442</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>1454</x:v>
+        <x:v>1443</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>1455</x:v>
+        <x:v>1444</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>1456</x:v>
+        <x:v>1445</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
         <x:v>969</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>1457</x:v>
+        <x:v>1446</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>1458</x:v>
+        <x:v>1447</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>2</x:v>
@@ -12736,7 +12703,7 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>1459</x:v>
+        <x:v>1448</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>9</x:v>
@@ -12745,22 +12712,22 @@
         <x:v>740</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>1460</x:v>
+        <x:v>1449</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>1461</x:v>
+        <x:v>1450</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G33" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H33" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I33" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J33" s="3" t="s">
         <x:v>42</x:v>
@@ -12769,31 +12736,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>1462</x:v>
+        <x:v>1451</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>1463</x:v>
+        <x:v>1452</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>1464</x:v>
+        <x:v>1453</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>1465</x:v>
+        <x:v>1454</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>1466</x:v>
+        <x:v>1455</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>1467</x:v>
+        <x:v>1456</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>1468</x:v>
+        <x:v>1457</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>1469</x:v>
+        <x:v>1458</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>1470</x:v>
+        <x:v>1459</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>2</x:v>
@@ -12801,7 +12768,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>1471</x:v>
+        <x:v>1460</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>9</x:v>
@@ -12810,22 +12777,22 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>1472</x:v>
+        <x:v>1461</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>1473</x:v>
+        <x:v>1462</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G34" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H34" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I34" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J34" s="3" t="s">
         <x:v>42</x:v>
@@ -12834,31 +12801,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>1474</x:v>
+        <x:v>1463</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>1475</x:v>
+        <x:v>1464</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
         <x:v>978</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>1476</x:v>
+        <x:v>1465</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>1477</x:v>
+        <x:v>1466</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>1478</x:v>
+        <x:v>1467</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>1479</x:v>
+        <x:v>1468</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>1480</x:v>
+        <x:v>1469</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>2</x:v>
@@ -12866,31 +12833,31 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>1481</x:v>
+        <x:v>1470</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>1482</x:v>
+        <x:v>1471</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>1483</x:v>
+        <x:v>1472</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>1484</x:v>
+        <x:v>1473</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G35" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H35" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I35" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J35" s="3" t="s">
         <x:v>42</x:v>
@@ -12899,31 +12866,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>1485</x:v>
+        <x:v>1474</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>1486</x:v>
+        <x:v>1475</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>1487</x:v>
+        <x:v>1476</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>1267</x:v>
+        <x:v>1256</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>1488</x:v>
+        <x:v>1477</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>1489</x:v>
+        <x:v>1478</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>1490</x:v>
+        <x:v>1479</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>1491</x:v>
+        <x:v>1480</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>1492</x:v>
+        <x:v>1481</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>2</x:v>
@@ -12931,31 +12898,31 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>1493</x:v>
+        <x:v>1482</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>1494</x:v>
+        <x:v>1483</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>1495</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>1496</x:v>
+        <x:v>1485</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G36" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H36" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I36" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J36" s="3" t="s">
         <x:v>42</x:v>
@@ -12964,31 +12931,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>1497</x:v>
+        <x:v>1486</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>1498</x:v>
+        <x:v>1487</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>1499</x:v>
+        <x:v>1488</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>1500</x:v>
+        <x:v>1489</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>1501</x:v>
+        <x:v>1490</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>1502</x:v>
+        <x:v>1491</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>1503</x:v>
+        <x:v>1492</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>1504</x:v>
+        <x:v>1493</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>2</x:v>
@@ -12996,31 +12963,31 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>1505</x:v>
+        <x:v>1494</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>1506</x:v>
+        <x:v>1495</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>1507</x:v>
+        <x:v>1496</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>1508</x:v>
+        <x:v>1497</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G37" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H37" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I37" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J37" s="3" t="s">
         <x:v>42</x:v>
@@ -13029,31 +12996,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>1509</x:v>
+        <x:v>1498</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>1510</x:v>
+        <x:v>1499</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>1511</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>1512</x:v>
+        <x:v>1501</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>1513</x:v>
+        <x:v>1502</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>1514</x:v>
+        <x:v>1503</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>1515</x:v>
+        <x:v>1504</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>1516</x:v>
+        <x:v>1505</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>1510</x:v>
+        <x:v>1499</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>2</x:v>
@@ -13061,31 +13028,31 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>1517</x:v>
+        <x:v>1506</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>1518</x:v>
+        <x:v>1507</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>1519</x:v>
+        <x:v>1508</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>1520</x:v>
+        <x:v>1509</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G38" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H38" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I38" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J38" s="3" t="s">
         <x:v>42</x:v>
@@ -13094,31 +13061,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>1521</x:v>
+        <x:v>1510</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>1192</x:v>
+        <x:v>1181</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>1522</x:v>
+        <x:v>1511</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>1523</x:v>
+        <x:v>1512</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>1524</x:v>
+        <x:v>1513</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>1525</x:v>
+        <x:v>1514</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>1526</x:v>
+        <x:v>1515</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>1527</x:v>
+        <x:v>1516</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>1528</x:v>
+        <x:v>1517</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>2</x:v>
@@ -13126,31 +13093,31 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>1529</x:v>
+        <x:v>1518</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>1530</x:v>
+        <x:v>1519</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>1531</x:v>
+        <x:v>1520</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>1532</x:v>
+        <x:v>1521</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G39" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="H39" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="I39" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="J39" s="3" t="s">
         <x:v>42</x:v>
@@ -13159,31 +13126,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>1533</x:v>
+        <x:v>1522</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>1534</x:v>
+        <x:v>1523</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>1535</x:v>
+        <x:v>1524</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>1536</x:v>
+        <x:v>1525</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>1537</x:v>
+        <x:v>1526</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>1538</x:v>
+        <x:v>1527</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>1539</x:v>
+        <x:v>1528</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>1540</x:v>
+        <x:v>1529</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>2</x:v>
@@ -13192,7 +13159,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R58e8ce8d152f43f8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0c04c5ebaf74cc9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-046 compliance contract tests
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R620d757063874a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3b42b5c4788c4997"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R7e472c98811b4243"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R120db2cb611d466c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra86334ab48034524"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re159ddff5dfa44a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R2fbb87b2f76d4769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf25d7749c86c4d4f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3053,42 +3053,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">NotificationController.cs:15-102; AdminPage.razor:91-165; CustomerDetail.razor:1356-1450</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">INT-046</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Compliance records and stats</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As an employee with compliance access, I can review compliance stats and manage compliance records.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Compliance BFF exposes stats, list, detail, create, and delete operations with compliance permissions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Intranet BFF -&gt; ComplianceService alerts/reports DTOs -&gt; permission-gated records</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ComplianceController.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Compliance records/stat surfaces</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ComplianceController stats, GET, GET {id}, POST, DELETE</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Intranet BFF, ComplianceService</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Compliance record create/delete requests</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs current UI route review if exposed beyond API/chat navigation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ComplianceController.cs:17-80; ComplianceServiceClient.cs:8-136</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">INT-047</x:t>
@@ -7172,7 +7136,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R154e6f3cd90e41a1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb438ffdb80624151"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10196,85 +10160,85 @@
       </x:c>
     </x:row>
     <x:row r="47" ht="51.29999923706055" hidden="0">
-      <x:c r="A47" s="3" t="s">
-        <x:v>1014</x:v>
-      </x:c>
-      <x:c r="B47" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C47" s="3" t="s">
-        <x:v>1015</x:v>
-      </x:c>
-      <x:c r="D47" s="3" t="s">
-        <x:v>1016</x:v>
-      </x:c>
-      <x:c r="E47" s="3" t="s">
-        <x:v>1017</x:v>
-      </x:c>
-      <x:c r="F47" s="3" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="G47" s="3" t="s">
-        <x:v>1001</x:v>
-      </x:c>
-      <x:c r="H47" s="3" t="s">
-        <x:v>1002</x:v>
-      </x:c>
-      <x:c r="I47" s="3" t="s">
-        <x:v>1003</x:v>
-      </x:c>
-      <x:c r="J47" s="3" t="s">
-        <x:v>1004</x:v>
-      </x:c>
-      <x:c r="K47" s="3" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="L47" s="3" t="s">
-        <x:v>1018</x:v>
-      </x:c>
-      <x:c r="M47" s="3" t="s">
-        <x:v>1019</x:v>
-      </x:c>
-      <x:c r="N47" s="3" t="s">
-        <x:v>1020</x:v>
-      </x:c>
-      <x:c r="O47" s="3" t="s">
-        <x:v>1021</x:v>
-      </x:c>
-      <x:c r="P47" s="3" t="s">
-        <x:v>1009</x:v>
-      </x:c>
-      <x:c r="Q47" s="3" t="s">
-        <x:v>1022</x:v>
-      </x:c>
-      <x:c r="R47" s="3" t="s">
-        <x:v>1023</x:v>
-      </x:c>
-      <x:c r="S47" s="3" t="s">
-        <x:v>1024</x:v>
-      </x:c>
-      <x:c r="T47" s="3" t="s">
-        <x:v>1025</x:v>
-      </x:c>
-      <x:c r="U47" s="3" t="s">
-        <x:v>2</x:v>
+      <x:c r="A47" s="3" t="str">
+        <x:v>INT-046</x:v>
+      </x:c>
+      <x:c r="B47" s="3" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C47" s="3" t="str">
+        <x:v>Compliance records and stats</x:v>
+      </x:c>
+      <x:c r="D47" s="3" t="str">
+        <x:v>As an employee with compliance access, I can review compliance stats and manage compliance records.</x:v>
+      </x:c>
+      <x:c r="E47" s="3" t="str">
+        <x:v>Compliance BFF exposes stats, list, detail, create, and delete operations with compliance permissions.</x:v>
+      </x:c>
+      <x:c r="F47" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G47" s="3" t="str">
+        <x:v>Focused behavior tests passed 2026-06-23.</x:v>
+      </x:c>
+      <x:c r="H47" s="3" t="str">
+        <x:v>No behavior error observed in current focused controller/client contract retest.</x:v>
+      </x:c>
+      <x:c r="I47" s="3" t="str">
+        <x:v>No app-code fix needed; added missing focused coverage in Maliev.Intranet commit e8f18af.</x:v>
+      </x:c>
+      <x:c r="J47" s="3" t="str">
+        <x:v>Retested ComplianceControllerTests 12/12 passed.</x:v>
+      </x:c>
+      <x:c r="K47" s="3" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L47" s="3" t="str">
+        <x:v>Intranet BFF -&gt; ComplianceService alerts/reports DTOs -&gt; permission-gated records</x:v>
+      </x:c>
+      <x:c r="M47" s="3" t="str">
+        <x:v>ComplianceController.cs</x:v>
+      </x:c>
+      <x:c r="N47" s="3" t="str">
+        <x:v>Compliance records/stat surfaces</x:v>
+      </x:c>
+      <x:c r="O47" s="3" t="str">
+        <x:v>ComplianceController stats, GET, GET {id}, POST, DELETE</x:v>
+      </x:c>
+      <x:c r="P47" s="3" t="str">
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~ComplianceControllerTests" --verbosity minimal passed 12/12 on 2026-06-23. Coverage verifies stats fallback, missing-record not found, create/delete outcomes, read/write permission requirements, ComplianceServiceClient alert-to-record mapping, report-to-stats mapping, and alert resolve endpoint path/body.</x:v>
+      </x:c>
+      <x:c r="Q47" s="3" t="str">
+        <x:v>Intranet BFF, ComplianceService</x:v>
+      </x:c>
+      <x:c r="R47" s="3" t="str">
+        <x:v>Compliance record create/delete requests</x:v>
+      </x:c>
+      <x:c r="S47" s="3" t="str">
+        <x:v>No remaining INT-046 API/client contract gap from this focused retest. Current code search found API/chat navigation exposure, not a dedicated compliance page route; full authenticated UI route review remains for later browser/Aspire pass.</x:v>
+      </x:c>
+      <x:c r="T47" s="3" t="str">
+        <x:v>ComplianceController.cs:17-80; ComplianceServiceClient.cs:8-136; ComplianceControllerTests.cs:1-179; ChatDrawer.razor:410</x:v>
+      </x:c>
+      <x:c r="U47" s="3" t="str">
+        <x:v>2026-06-23</x:v>
       </x:c>
     </x:row>
     <x:row r="48" ht="51.29999923706055" hidden="0">
       <x:c r="A48" s="3" t="s">
-        <x:v>1026</x:v>
+        <x:v>1014</x:v>
       </x:c>
       <x:c r="B48" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C48" s="3" t="s">
-        <x:v>1027</x:v>
+        <x:v>1015</x:v>
       </x:c>
       <x:c r="D48" s="3" t="s">
-        <x:v>1028</x:v>
+        <x:v>1016</x:v>
       </x:c>
       <x:c r="E48" s="3" t="s">
-        <x:v>1029</x:v>
+        <x:v>1017</x:v>
       </x:c>
       <x:c r="F48" s="3" t="s">
         <x:v>38</x:v>
@@ -10295,31 +10259,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L48" s="3" t="s">
-        <x:v>1030</x:v>
+        <x:v>1018</x:v>
       </x:c>
       <x:c r="M48" s="3" t="s">
-        <x:v>1031</x:v>
+        <x:v>1019</x:v>
       </x:c>
       <x:c r="N48" s="3" t="s">
-        <x:v>1032</x:v>
+        <x:v>1020</x:v>
       </x:c>
       <x:c r="O48" s="3" t="s">
-        <x:v>1033</x:v>
+        <x:v>1021</x:v>
       </x:c>
       <x:c r="P48" s="3" t="s">
         <x:v>1009</x:v>
       </x:c>
       <x:c r="Q48" s="3" t="s">
-        <x:v>1034</x:v>
+        <x:v>1022</x:v>
       </x:c>
       <x:c r="R48" s="3" t="s">
-        <x:v>1035</x:v>
+        <x:v>1023</x:v>
       </x:c>
       <x:c r="S48" s="3" t="s">
-        <x:v>1036</x:v>
+        <x:v>1024</x:v>
       </x:c>
       <x:c r="T48" s="3" t="s">
-        <x:v>1037</x:v>
+        <x:v>1025</x:v>
       </x:c>
       <x:c r="U48" s="3" t="s">
         <x:v>2</x:v>
@@ -10327,19 +10291,19 @@
     </x:row>
     <x:row r="49" ht="51.29999923706055" hidden="0">
       <x:c r="A49" s="3" t="s">
-        <x:v>1038</x:v>
+        <x:v>1026</x:v>
       </x:c>
       <x:c r="B49" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C49" s="3" t="s">
-        <x:v>1039</x:v>
+        <x:v>1027</x:v>
       </x:c>
       <x:c r="D49" s="3" t="s">
-        <x:v>1040</x:v>
+        <x:v>1028</x:v>
       </x:c>
       <x:c r="E49" s="3" t="s">
-        <x:v>1041</x:v>
+        <x:v>1029</x:v>
       </x:c>
       <x:c r="F49" s="3" t="s">
         <x:v>38</x:v>
@@ -10360,31 +10324,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L49" s="3" t="s">
-        <x:v>1042</x:v>
+        <x:v>1030</x:v>
       </x:c>
       <x:c r="M49" s="3" t="s">
-        <x:v>1043</x:v>
+        <x:v>1031</x:v>
       </x:c>
       <x:c r="N49" s="3" t="s">
-        <x:v>1044</x:v>
+        <x:v>1032</x:v>
       </x:c>
       <x:c r="O49" s="3" t="s">
-        <x:v>1045</x:v>
+        <x:v>1033</x:v>
       </x:c>
       <x:c r="P49" s="3" t="s">
         <x:v>1009</x:v>
       </x:c>
       <x:c r="Q49" s="3" t="s">
-        <x:v>1046</x:v>
+        <x:v>1034</x:v>
       </x:c>
       <x:c r="R49" s="3" t="s">
-        <x:v>1047</x:v>
+        <x:v>1035</x:v>
       </x:c>
       <x:c r="S49" s="3" t="s">
-        <x:v>1048</x:v>
+        <x:v>1036</x:v>
       </x:c>
       <x:c r="T49" s="3" t="s">
-        <x:v>1049</x:v>
+        <x:v>1037</x:v>
       </x:c>
       <x:c r="U49" s="3" t="s">
         <x:v>2</x:v>
@@ -10392,19 +10356,19 @@
     </x:row>
     <x:row r="50" ht="51.29999923706055" hidden="0">
       <x:c r="A50" s="3" t="s">
-        <x:v>1050</x:v>
+        <x:v>1038</x:v>
       </x:c>
       <x:c r="B50" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C50" s="3" t="s">
-        <x:v>1051</x:v>
+        <x:v>1039</x:v>
       </x:c>
       <x:c r="D50" s="3" t="s">
-        <x:v>1052</x:v>
+        <x:v>1040</x:v>
       </x:c>
       <x:c r="E50" s="3" t="s">
-        <x:v>1053</x:v>
+        <x:v>1041</x:v>
       </x:c>
       <x:c r="F50" s="3" t="s">
         <x:v>38</x:v>
@@ -10425,31 +10389,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L50" s="3" t="s">
-        <x:v>1054</x:v>
+        <x:v>1042</x:v>
       </x:c>
       <x:c r="M50" s="3" t="s">
-        <x:v>1055</x:v>
+        <x:v>1043</x:v>
       </x:c>
       <x:c r="N50" s="3" t="s">
-        <x:v>1056</x:v>
+        <x:v>1044</x:v>
       </x:c>
       <x:c r="O50" s="3" t="s">
-        <x:v>1057</x:v>
+        <x:v>1045</x:v>
       </x:c>
       <x:c r="P50" s="3" t="s">
         <x:v>1009</x:v>
       </x:c>
       <x:c r="Q50" s="3" t="s">
-        <x:v>1058</x:v>
+        <x:v>1046</x:v>
       </x:c>
       <x:c r="R50" s="3" t="s">
-        <x:v>1059</x:v>
+        <x:v>1047</x:v>
       </x:c>
       <x:c r="S50" s="3" t="s">
+        <x:v>1036</x:v>
+      </x:c>
+      <x:c r="T50" s="3" t="s">
         <x:v>1048</x:v>
-      </x:c>
-      <x:c r="T50" s="3" t="s">
-        <x:v>1060</x:v>
       </x:c>
       <x:c r="U50" s="3" t="s">
         <x:v>2</x:v>
@@ -10588,7 +10552,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rad6f22be4874441d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R292f9d36064a4636"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10688,64 +10652,64 @@
     </x:row>
     <x:row r="2" ht="149.25" hidden="0">
       <x:c r="A2" s="3" t="s">
-        <x:v>1061</x:v>
+        <x:v>1049</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>1062</x:v>
+        <x:v>1050</x:v>
       </x:c>
       <x:c r="D2" s="3" t="s">
-        <x:v>1063</x:v>
+        <x:v>1051</x:v>
       </x:c>
       <x:c r="E2" s="3" t="s">
-        <x:v>1064</x:v>
+        <x:v>1052</x:v>
       </x:c>
       <x:c r="F2" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>1065</x:v>
+        <x:v>1053</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>1066</x:v>
+        <x:v>1054</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>1067</x:v>
+        <x:v>1055</x:v>
       </x:c>
       <x:c r="J2" s="3" t="s">
-        <x:v>1068</x:v>
+        <x:v>1056</x:v>
       </x:c>
       <x:c r="K2" s="3" t="s">
         <x:v>188</x:v>
       </x:c>
       <x:c r="L2" s="3" t="s">
-        <x:v>1069</x:v>
+        <x:v>1057</x:v>
       </x:c>
       <x:c r="M2" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1058</x:v>
       </x:c>
       <x:c r="N2" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="O2" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="P2" s="3" t="s">
-        <x:v>1073</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1062</x:v>
       </x:c>
       <x:c r="R2" s="3" t="s">
-        <x:v>1075</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="S2" s="3" t="s">
-        <x:v>1076</x:v>
+        <x:v>1064</x:v>
       </x:c>
       <x:c r="T2" s="3" t="s">
-        <x:v>1077</x:v>
+        <x:v>1065</x:v>
       </x:c>
       <x:c r="U2" s="3" t="s">
         <x:v>2</x:v>
@@ -10753,31 +10717,31 @@
     </x:row>
     <x:row r="3" ht="107.25" hidden="0">
       <x:c r="A3" s="3" t="s">
-        <x:v>1078</x:v>
+        <x:v>1066</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>1079</x:v>
+        <x:v>1067</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>1080</x:v>
+        <x:v>1068</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>1081</x:v>
+        <x:v>1069</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G3" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H3" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I3" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J3" s="3" t="s">
         <x:v>42</x:v>
@@ -10786,31 +10750,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L3" s="3" t="s">
-        <x:v>1085</x:v>
+        <x:v>1073</x:v>
       </x:c>
       <x:c r="M3" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N3" s="3" t="s">
-        <x:v>1087</x:v>
+        <x:v>1075</x:v>
       </x:c>
       <x:c r="O3" s="3" t="s">
-        <x:v>1088</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="P3" s="3" t="s">
-        <x:v>1089</x:v>
+        <x:v>1077</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="s">
-        <x:v>1090</x:v>
+        <x:v>1078</x:v>
       </x:c>
       <x:c r="R3" s="3" t="s">
-        <x:v>1091</x:v>
+        <x:v>1079</x:v>
       </x:c>
       <x:c r="S3" s="3" t="s">
-        <x:v>1092</x:v>
+        <x:v>1080</x:v>
       </x:c>
       <x:c r="T3" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1081</x:v>
       </x:c>
       <x:c r="U3" s="3" t="s">
         <x:v>2</x:v>
@@ -10818,31 +10782,31 @@
     </x:row>
     <x:row r="4" ht="93.25" hidden="0">
       <x:c r="A4" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>1096</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="E4" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1085</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G4" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H4" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I4" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J4" s="3" t="s">
         <x:v>42</x:v>
@@ -10851,31 +10815,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L4" s="3" t="s">
-        <x:v>1098</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="M4" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N4" s="3" t="s">
-        <x:v>1099</x:v>
+        <x:v>1087</x:v>
       </x:c>
       <x:c r="O4" s="3" t="s">
-        <x:v>1100</x:v>
+        <x:v>1088</x:v>
       </x:c>
       <x:c r="P4" s="3" t="s">
-        <x:v>1101</x:v>
+        <x:v>1089</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="s">
-        <x:v>1102</x:v>
+        <x:v>1090</x:v>
       </x:c>
       <x:c r="R4" s="3" t="s">
-        <x:v>1103</x:v>
+        <x:v>1091</x:v>
       </x:c>
       <x:c r="S4" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1092</x:v>
       </x:c>
       <x:c r="T4" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="U4" s="3" t="s">
         <x:v>2</x:v>
@@ -10883,31 +10847,31 @@
     </x:row>
     <x:row r="5" ht="107.25" hidden="0">
       <x:c r="A5" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>1107</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1096</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>1109</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
         <x:v>42</x:v>
@@ -10916,31 +10880,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>1110</x:v>
+        <x:v>1098</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>1111</x:v>
+        <x:v>1099</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>1112</x:v>
+        <x:v>1100</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>1113</x:v>
+        <x:v>1101</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>1114</x:v>
+        <x:v>1102</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>1115</x:v>
+        <x:v>1103</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>1116</x:v>
+        <x:v>1104</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>1117</x:v>
+        <x:v>1105</x:v>
       </x:c>
       <x:c r="U5" s="3" t="s">
         <x:v>2</x:v>
@@ -10948,31 +10912,31 @@
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
       <x:c r="A6" s="3" t="s">
-        <x:v>1118</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>1119</x:v>
+        <x:v>1107</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>1120</x:v>
+        <x:v>1108</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>1121</x:v>
+        <x:v>1109</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H6" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I6" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J6" s="3" t="s">
         <x:v>42</x:v>
@@ -10981,31 +10945,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L6" s="3" t="s">
-        <x:v>1122</x:v>
+        <x:v>1110</x:v>
       </x:c>
       <x:c r="M6" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N6" s="3" t="s">
-        <x:v>1123</x:v>
+        <x:v>1111</x:v>
       </x:c>
       <x:c r="O6" s="3" t="s">
-        <x:v>1124</x:v>
+        <x:v>1112</x:v>
       </x:c>
       <x:c r="P6" s="3" t="s">
-        <x:v>1125</x:v>
+        <x:v>1113</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="s">
-        <x:v>1126</x:v>
+        <x:v>1114</x:v>
       </x:c>
       <x:c r="R6" s="3" t="s">
-        <x:v>1127</x:v>
+        <x:v>1115</x:v>
       </x:c>
       <x:c r="S6" s="3" t="s">
-        <x:v>1128</x:v>
+        <x:v>1116</x:v>
       </x:c>
       <x:c r="T6" s="3" t="s">
-        <x:v>1129</x:v>
+        <x:v>1117</x:v>
       </x:c>
       <x:c r="U6" s="3" t="s">
         <x:v>2</x:v>
@@ -11013,31 +10977,31 @@
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>1130</x:v>
+        <x:v>1118</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>1131</x:v>
+        <x:v>1119</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>1132</x:v>
+        <x:v>1120</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>1133</x:v>
+        <x:v>1121</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G7" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H7" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I7" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J7" s="3" t="s">
         <x:v>42</x:v>
@@ -11046,31 +11010,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
-        <x:v>1134</x:v>
+        <x:v>1122</x:v>
       </x:c>
       <x:c r="M7" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N7" s="3" t="s">
-        <x:v>1135</x:v>
+        <x:v>1123</x:v>
       </x:c>
       <x:c r="O7" s="3" t="s">
-        <x:v>1136</x:v>
+        <x:v>1124</x:v>
       </x:c>
       <x:c r="P7" s="3" t="s">
-        <x:v>1137</x:v>
+        <x:v>1125</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="s">
-        <x:v>1090</x:v>
+        <x:v>1078</x:v>
       </x:c>
       <x:c r="R7" s="3" t="s">
-        <x:v>1138</x:v>
+        <x:v>1126</x:v>
       </x:c>
       <x:c r="S7" s="3" t="s">
-        <x:v>1139</x:v>
+        <x:v>1127</x:v>
       </x:c>
       <x:c r="T7" s="3" t="s">
-        <x:v>1140</x:v>
+        <x:v>1128</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>2</x:v>
@@ -11078,31 +11042,31 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>1141</x:v>
+        <x:v>1129</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>1142</x:v>
+        <x:v>1130</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>1143</x:v>
+        <x:v>1131</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>1144</x:v>
+        <x:v>1132</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H8" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I8" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J8" s="3" t="s">
         <x:v>42</x:v>
@@ -11111,31 +11075,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
-        <x:v>1145</x:v>
+        <x:v>1133</x:v>
       </x:c>
       <x:c r="M8" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N8" s="3" t="s">
-        <x:v>1146</x:v>
+        <x:v>1134</x:v>
       </x:c>
       <x:c r="O8" s="3" t="s">
-        <x:v>1147</x:v>
+        <x:v>1135</x:v>
       </x:c>
       <x:c r="P8" s="3" t="s">
-        <x:v>1148</x:v>
+        <x:v>1136</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="s">
-        <x:v>1149</x:v>
+        <x:v>1137</x:v>
       </x:c>
       <x:c r="R8" s="3" t="s">
-        <x:v>1150</x:v>
+        <x:v>1138</x:v>
       </x:c>
       <x:c r="S8" s="3" t="s">
-        <x:v>1151</x:v>
+        <x:v>1139</x:v>
       </x:c>
       <x:c r="T8" s="3" t="s">
-        <x:v>1152</x:v>
+        <x:v>1140</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>2</x:v>
@@ -11143,31 +11107,31 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>1153</x:v>
+        <x:v>1141</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>1154</x:v>
+        <x:v>1142</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>1155</x:v>
+        <x:v>1143</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>1156</x:v>
+        <x:v>1144</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H9" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I9" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J9" s="3" t="s">
         <x:v>42</x:v>
@@ -11176,31 +11140,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
-        <x:v>1157</x:v>
+        <x:v>1145</x:v>
       </x:c>
       <x:c r="M9" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N9" s="3" t="s">
-        <x:v>1158</x:v>
+        <x:v>1146</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>1159</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="P9" s="3" t="s">
-        <x:v>1160</x:v>
+        <x:v>1148</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="s">
-        <x:v>1161</x:v>
+        <x:v>1149</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
-        <x:v>1162</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="S9" s="3" t="s">
-        <x:v>1163</x:v>
+        <x:v>1151</x:v>
       </x:c>
       <x:c r="T9" s="3" t="s">
-        <x:v>1164</x:v>
+        <x:v>1152</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>2</x:v>
@@ -11208,31 +11172,31 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>1165</x:v>
+        <x:v>1153</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>1166</x:v>
+        <x:v>1154</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>1167</x:v>
+        <x:v>1155</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>1168</x:v>
+        <x:v>1156</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G10" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H10" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I10" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J10" s="3" t="s">
         <x:v>42</x:v>
@@ -11241,31 +11205,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>1169</x:v>
+        <x:v>1157</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1058</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>1170</x:v>
+        <x:v>1158</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>1171</x:v>
+        <x:v>1159</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>1172</x:v>
+        <x:v>1160</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>1173</x:v>
+        <x:v>1161</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>1174</x:v>
+        <x:v>1162</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>1175</x:v>
+        <x:v>1163</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>2</x:v>
@@ -11273,31 +11237,31 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>1176</x:v>
+        <x:v>1164</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>1177</x:v>
+        <x:v>1165</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>1178</x:v>
+        <x:v>1166</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>1179</x:v>
+        <x:v>1167</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G11" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H11" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I11" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J11" s="3" t="s">
         <x:v>42</x:v>
@@ -11306,31 +11270,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>1180</x:v>
+        <x:v>1168</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>1181</x:v>
+        <x:v>1169</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>1182</x:v>
+        <x:v>1170</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>1183</x:v>
+        <x:v>1171</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>1184</x:v>
+        <x:v>1172</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>1185</x:v>
+        <x:v>1173</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>1186</x:v>
+        <x:v>1174</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>1187</x:v>
+        <x:v>1175</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>1188</x:v>
+        <x:v>1176</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>2</x:v>
@@ -11338,31 +11302,31 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>1189</x:v>
+        <x:v>1177</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>1190</x:v>
+        <x:v>1178</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>1191</x:v>
+        <x:v>1179</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>1192</x:v>
+        <x:v>1180</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G12" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H12" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I12" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J12" s="3" t="s">
         <x:v>42</x:v>
@@ -11371,31 +11335,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>1193</x:v>
+        <x:v>1181</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>1194</x:v>
+        <x:v>1182</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>1195</x:v>
+        <x:v>1183</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>1196</x:v>
+        <x:v>1184</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>1197</x:v>
+        <x:v>1185</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>1198</x:v>
+        <x:v>1186</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>1199</x:v>
+        <x:v>1187</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>1200</x:v>
+        <x:v>1188</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>2</x:v>
@@ -11403,31 +11367,31 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>1201</x:v>
+        <x:v>1189</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>1202</x:v>
+        <x:v>1190</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>1203</x:v>
+        <x:v>1191</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>1204</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I13" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J13" s="3" t="s">
         <x:v>42</x:v>
@@ -11436,31 +11400,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>1205</x:v>
+        <x:v>1193</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>1206</x:v>
+        <x:v>1194</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>1207</x:v>
+        <x:v>1195</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>1208</x:v>
+        <x:v>1196</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
+        <x:v>1185</x:v>
+      </x:c>
+      <x:c r="R13" s="3" t="s">
         <x:v>1197</x:v>
       </x:c>
-      <x:c r="R13" s="3" t="s">
-        <x:v>1209</x:v>
-      </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>1210</x:v>
+        <x:v>1198</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>1211</x:v>
+        <x:v>1199</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>2</x:v>
@@ -11468,31 +11432,31 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>1212</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>1213</x:v>
+        <x:v>1201</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>1214</x:v>
+        <x:v>1202</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>1215</x:v>
+        <x:v>1203</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G14" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H14" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I14" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J14" s="3" t="s">
         <x:v>42</x:v>
@@ -11501,31 +11465,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>1216</x:v>
+        <x:v>1204</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>1217</x:v>
+        <x:v>1205</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>1218</x:v>
+        <x:v>1206</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>1219</x:v>
+        <x:v>1207</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>1220</x:v>
+        <x:v>1208</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>1221</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>1222</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>1223</x:v>
+        <x:v>1211</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>1224</x:v>
+        <x:v>1212</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>2</x:v>
@@ -11533,31 +11497,31 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>1225</x:v>
+        <x:v>1213</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>1226</x:v>
+        <x:v>1214</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>1227</x:v>
+        <x:v>1215</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>1228</x:v>
+        <x:v>1216</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G15" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H15" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I15" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J15" s="3" t="s">
         <x:v>42</x:v>
@@ -11566,31 +11530,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>1229</x:v>
+        <x:v>1217</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>1230</x:v>
+        <x:v>1218</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>1231</x:v>
+        <x:v>1219</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>1232</x:v>
+        <x:v>1220</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>1233</x:v>
+        <x:v>1221</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>1234</x:v>
+        <x:v>1222</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>1235</x:v>
+        <x:v>1223</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>1236</x:v>
+        <x:v>1224</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>2</x:v>
@@ -11598,31 +11562,31 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>1237</x:v>
+        <x:v>1225</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>1238</x:v>
+        <x:v>1226</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>1239</x:v>
+        <x:v>1227</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>1240</x:v>
+        <x:v>1228</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H16" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I16" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J16" s="3" t="s">
         <x:v>42</x:v>
@@ -11631,31 +11595,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>1241</x:v>
+        <x:v>1229</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>1242</x:v>
+        <x:v>1230</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>1243</x:v>
+        <x:v>1231</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>1244</x:v>
+        <x:v>1232</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>1245</x:v>
+        <x:v>1233</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>1246</x:v>
+        <x:v>1234</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>1247</x:v>
+        <x:v>1235</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>1248</x:v>
+        <x:v>1236</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>2</x:v>
@@ -11663,31 +11627,31 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>1249</x:v>
+        <x:v>1237</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>1250</x:v>
+        <x:v>1238</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>1251</x:v>
+        <x:v>1239</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>1252</x:v>
+        <x:v>1240</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H17" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I17" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J17" s="3" t="s">
         <x:v>42</x:v>
@@ -11696,31 +11660,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>1253</x:v>
+        <x:v>1241</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>1254</x:v>
+        <x:v>1242</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>1255</x:v>
+        <x:v>1243</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>1256</x:v>
+        <x:v>1244</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>1257</x:v>
+        <x:v>1245</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>1258</x:v>
+        <x:v>1246</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>1259</x:v>
+        <x:v>1247</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>1260</x:v>
+        <x:v>1248</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>1261</x:v>
+        <x:v>1249</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>2</x:v>
@@ -11728,31 +11692,31 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>1262</x:v>
+        <x:v>1250</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>1263</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>1264</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>1265</x:v>
+        <x:v>1253</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G18" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H18" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I18" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J18" s="3" t="s">
         <x:v>42</x:v>
@@ -11761,31 +11725,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>1266</x:v>
+        <x:v>1254</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>1267</x:v>
+        <x:v>1255</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>1268</x:v>
+        <x:v>1256</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>1269</x:v>
+        <x:v>1257</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>1270</x:v>
+        <x:v>1258</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>1271</x:v>
+        <x:v>1259</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>1272</x:v>
+        <x:v>1260</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>1273</x:v>
+        <x:v>1261</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>1274</x:v>
+        <x:v>1262</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>2</x:v>
@@ -11793,31 +11757,31 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>1275</x:v>
+        <x:v>1263</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>1276</x:v>
+        <x:v>1264</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>1277</x:v>
+        <x:v>1265</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>1278</x:v>
+        <x:v>1266</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I19" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J19" s="3" t="s">
         <x:v>42</x:v>
@@ -11826,31 +11790,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>1279</x:v>
+        <x:v>1267</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>1280</x:v>
+        <x:v>1268</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>1281</x:v>
+        <x:v>1269</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>1282</x:v>
+        <x:v>1270</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>1283</x:v>
+        <x:v>1271</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>1284</x:v>
+        <x:v>1272</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>1285</x:v>
+        <x:v>1273</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>1286</x:v>
+        <x:v>1274</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>1287</x:v>
+        <x:v>1275</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>2</x:v>
@@ -11858,31 +11822,31 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>1288</x:v>
+        <x:v>1276</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>1289</x:v>
+        <x:v>1277</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>1290</x:v>
+        <x:v>1278</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>1291</x:v>
+        <x:v>1279</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I20" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J20" s="3" t="s">
         <x:v>42</x:v>
@@ -11891,31 +11855,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>1292</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>1293</x:v>
+        <x:v>1281</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>1294</x:v>
+        <x:v>1282</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>1295</x:v>
+        <x:v>1283</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>1296</x:v>
+        <x:v>1284</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>1297</x:v>
+        <x:v>1285</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>1298</x:v>
+        <x:v>1286</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>1299</x:v>
+        <x:v>1287</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>1300</x:v>
+        <x:v>1288</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>2</x:v>
@@ -11923,31 +11887,31 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>1301</x:v>
+        <x:v>1289</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>1302</x:v>
+        <x:v>1290</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>1303</x:v>
+        <x:v>1291</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>1304</x:v>
+        <x:v>1292</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G21" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H21" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I21" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J21" s="3" t="s">
         <x:v>42</x:v>
@@ -11956,31 +11920,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>1305</x:v>
+        <x:v>1293</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>1306</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>1307</x:v>
+        <x:v>1295</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>1308</x:v>
+        <x:v>1296</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>1309</x:v>
+        <x:v>1297</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>1310</x:v>
+        <x:v>1298</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>1311</x:v>
+        <x:v>1299</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>2</x:v>
@@ -11988,31 +11952,31 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>1312</x:v>
+        <x:v>1300</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>1313</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>1314</x:v>
+        <x:v>1302</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>1315</x:v>
+        <x:v>1303</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G22" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H22" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I22" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J22" s="3" t="s">
         <x:v>42</x:v>
@@ -12021,31 +11985,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>1316</x:v>
+        <x:v>1304</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>1181</x:v>
+        <x:v>1169</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>1317</x:v>
+        <x:v>1305</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>1318</x:v>
+        <x:v>1306</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>1319</x:v>
+        <x:v>1307</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>1320</x:v>
+        <x:v>1308</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>1321</x:v>
+        <x:v>1309</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>1322</x:v>
+        <x:v>1310</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>1323</x:v>
+        <x:v>1311</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>2</x:v>
@@ -12053,31 +12017,31 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>1324</x:v>
+        <x:v>1312</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>1325</x:v>
+        <x:v>1313</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>1326</x:v>
+        <x:v>1314</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>1327</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G23" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H23" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I23" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J23" s="3" t="s">
         <x:v>42</x:v>
@@ -12086,31 +12050,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>1328</x:v>
+        <x:v>1316</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>1329</x:v>
+        <x:v>1317</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>1330</x:v>
+        <x:v>1318</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>1331</x:v>
+        <x:v>1319</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>1332</x:v>
+        <x:v>1320</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>1333</x:v>
+        <x:v>1321</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>1334</x:v>
+        <x:v>1322</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>1335</x:v>
+        <x:v>1323</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>1336</x:v>
+        <x:v>1324</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>2</x:v>
@@ -12118,31 +12082,31 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>1337</x:v>
+        <x:v>1325</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>1338</x:v>
+        <x:v>1326</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>1339</x:v>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>1340</x:v>
+        <x:v>1328</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H24" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I24" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J24" s="3" t="s">
         <x:v>42</x:v>
@@ -12151,31 +12115,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>1341</x:v>
+        <x:v>1329</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>1306</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>1342</x:v>
+        <x:v>1330</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>1343</x:v>
+        <x:v>1331</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>1344</x:v>
+        <x:v>1332</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>1345</x:v>
+        <x:v>1333</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>1346</x:v>
+        <x:v>1334</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>1347</x:v>
+        <x:v>1335</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>1348</x:v>
+        <x:v>1336</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>2</x:v>
@@ -12183,31 +12147,31 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>1349</x:v>
+        <x:v>1337</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>1350</x:v>
+        <x:v>1338</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>1351</x:v>
+        <x:v>1339</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>1352</x:v>
+        <x:v>1340</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H25" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I25" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J25" s="3" t="s">
         <x:v>42</x:v>
@@ -12216,31 +12180,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>1353</x:v>
+        <x:v>1341</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>1306</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>1354</x:v>
+        <x:v>1342</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>1355</x:v>
+        <x:v>1343</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>1356</x:v>
+        <x:v>1344</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>1357</x:v>
+        <x:v>1345</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>1358</x:v>
+        <x:v>1346</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>1359</x:v>
+        <x:v>1347</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>1360</x:v>
+        <x:v>1348</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>2</x:v>
@@ -12248,31 +12212,31 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>1361</x:v>
+        <x:v>1349</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>1362</x:v>
+        <x:v>1350</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>1363</x:v>
+        <x:v>1351</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>1364</x:v>
+        <x:v>1352</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H26" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I26" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J26" s="3" t="s">
         <x:v>42</x:v>
@@ -12281,31 +12245,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>1365</x:v>
+        <x:v>1353</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>1366</x:v>
+        <x:v>1354</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>1367</x:v>
+        <x:v>1355</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>1368</x:v>
+        <x:v>1356</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>1369</x:v>
+        <x:v>1357</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>1370</x:v>
+        <x:v>1358</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>1371</x:v>
+        <x:v>1359</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>1372</x:v>
+        <x:v>1360</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>1373</x:v>
+        <x:v>1361</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>2</x:v>
@@ -12313,31 +12277,31 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>1374</x:v>
+        <x:v>1362</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>1375</x:v>
+        <x:v>1363</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>1376</x:v>
+        <x:v>1364</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>1377</x:v>
+        <x:v>1365</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H27" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I27" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J27" s="3" t="s">
         <x:v>42</x:v>
@@ -12346,31 +12310,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>1378</x:v>
+        <x:v>1366</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>1379</x:v>
+        <x:v>1367</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>1380</x:v>
+        <x:v>1368</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>1381</x:v>
+        <x:v>1369</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>1382</x:v>
+        <x:v>1370</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>1383</x:v>
+        <x:v>1371</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>1384</x:v>
+        <x:v>1372</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
         <x:v>789</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>1385</x:v>
+        <x:v>1373</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>2</x:v>
@@ -12378,31 +12342,31 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>1386</x:v>
+        <x:v>1374</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>1387</x:v>
+        <x:v>1375</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>1388</x:v>
+        <x:v>1376</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>1389</x:v>
+        <x:v>1377</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G28" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H28" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I28" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J28" s="3" t="s">
         <x:v>42</x:v>
@@ -12411,31 +12375,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>1390</x:v>
+        <x:v>1378</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>1391</x:v>
+        <x:v>1379</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>1392</x:v>
+        <x:v>1380</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>1393</x:v>
+        <x:v>1381</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>1394</x:v>
+        <x:v>1382</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>1395</x:v>
+        <x:v>1383</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>1396</x:v>
+        <x:v>1384</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>1397</x:v>
+        <x:v>1385</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>2</x:v>
@@ -12443,31 +12407,31 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>1398</x:v>
+        <x:v>1386</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>1399</x:v>
+        <x:v>1387</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>1400</x:v>
+        <x:v>1388</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>1401</x:v>
+        <x:v>1389</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G29" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H29" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I29" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J29" s="3" t="s">
         <x:v>42</x:v>
@@ -12476,31 +12440,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>1402</x:v>
+        <x:v>1390</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>1403</x:v>
+        <x:v>1391</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>1404</x:v>
+        <x:v>1392</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>1405</x:v>
+        <x:v>1393</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>1406</x:v>
+        <x:v>1394</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>1407</x:v>
+        <x:v>1395</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>1408</x:v>
+        <x:v>1396</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>1409</x:v>
+        <x:v>1397</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>1410</x:v>
+        <x:v>1398</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>2</x:v>
@@ -12508,31 +12472,31 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>1411</x:v>
+        <x:v>1399</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>1412</x:v>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>1413</x:v>
+        <x:v>1401</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>1414</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G30" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H30" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I30" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J30" s="3" t="s">
         <x:v>42</x:v>
@@ -12541,31 +12505,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>1415</x:v>
+        <x:v>1403</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>1416</x:v>
+        <x:v>1404</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>1417</x:v>
+        <x:v>1405</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>1418</x:v>
+        <x:v>1406</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>1419</x:v>
+        <x:v>1407</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>1420</x:v>
+        <x:v>1408</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>1421</x:v>
+        <x:v>1409</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>1422</x:v>
+        <x:v>1410</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>1423</x:v>
+        <x:v>1411</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>2</x:v>
@@ -12573,7 +12537,7 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>1424</x:v>
+        <x:v>1412</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>9</x:v>
@@ -12582,22 +12546,22 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>1425</x:v>
+        <x:v>1413</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>1426</x:v>
+        <x:v>1414</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G31" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H31" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I31" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J31" s="3" t="s">
         <x:v>42</x:v>
@@ -12606,31 +12570,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>1427</x:v>
+        <x:v>1415</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>1428</x:v>
+        <x:v>1416</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>1429</x:v>
+        <x:v>1417</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>1430</x:v>
+        <x:v>1418</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>1431</x:v>
+        <x:v>1419</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>1432</x:v>
+        <x:v>1420</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>1433</x:v>
+        <x:v>1421</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>1434</x:v>
+        <x:v>1422</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>1435</x:v>
+        <x:v>1423</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>2</x:v>
@@ -12638,31 +12602,31 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>1436</x:v>
+        <x:v>1424</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>1437</x:v>
+        <x:v>1425</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>1438</x:v>
+        <x:v>1426</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>1439</x:v>
+        <x:v>1427</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G32" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H32" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I32" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J32" s="3" t="s">
         <x:v>42</x:v>
@@ -12671,31 +12635,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>1440</x:v>
+        <x:v>1428</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>1441</x:v>
+        <x:v>1429</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>1442</x:v>
+        <x:v>1430</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>1443</x:v>
+        <x:v>1431</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>1444</x:v>
+        <x:v>1432</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>1445</x:v>
+        <x:v>1433</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
         <x:v>969</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>1446</x:v>
+        <x:v>1434</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>1447</x:v>
+        <x:v>1435</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>2</x:v>
@@ -12703,7 +12667,7 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>1448</x:v>
+        <x:v>1436</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>9</x:v>
@@ -12712,22 +12676,22 @@
         <x:v>740</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>1449</x:v>
+        <x:v>1437</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>1450</x:v>
+        <x:v>1438</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G33" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H33" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I33" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J33" s="3" t="s">
         <x:v>42</x:v>
@@ -12736,31 +12700,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>1451</x:v>
+        <x:v>1439</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>1452</x:v>
+        <x:v>1440</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>1453</x:v>
+        <x:v>1441</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>1454</x:v>
+        <x:v>1442</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>1455</x:v>
+        <x:v>1443</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>1456</x:v>
+        <x:v>1444</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>1457</x:v>
+        <x:v>1445</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>1458</x:v>
+        <x:v>1446</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>1459</x:v>
+        <x:v>1447</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>2</x:v>
@@ -12768,7 +12732,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>1460</x:v>
+        <x:v>1448</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>9</x:v>
@@ -12777,22 +12741,22 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>1461</x:v>
+        <x:v>1449</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>1462</x:v>
+        <x:v>1450</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G34" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H34" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I34" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J34" s="3" t="s">
         <x:v>42</x:v>
@@ -12801,31 +12765,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>1463</x:v>
+        <x:v>1451</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>1464</x:v>
+        <x:v>1452</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
         <x:v>978</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>1465</x:v>
+        <x:v>1453</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>1466</x:v>
+        <x:v>1454</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>1467</x:v>
+        <x:v>1455</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>1468</x:v>
+        <x:v>1456</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>1469</x:v>
+        <x:v>1457</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>2</x:v>
@@ -12833,31 +12797,31 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>1470</x:v>
+        <x:v>1458</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>1471</x:v>
+        <x:v>1459</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>1472</x:v>
+        <x:v>1460</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>1473</x:v>
+        <x:v>1461</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G35" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H35" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I35" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J35" s="3" t="s">
         <x:v>42</x:v>
@@ -12866,31 +12830,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>1474</x:v>
+        <x:v>1462</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>1475</x:v>
+        <x:v>1463</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>1476</x:v>
+        <x:v>1464</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>1256</x:v>
+        <x:v>1244</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>1477</x:v>
+        <x:v>1465</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>1478</x:v>
+        <x:v>1466</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>1479</x:v>
+        <x:v>1467</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>1480</x:v>
+        <x:v>1468</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>1481</x:v>
+        <x:v>1469</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>2</x:v>
@@ -12898,31 +12862,31 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>1482</x:v>
+        <x:v>1470</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>1483</x:v>
+        <x:v>1471</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>1484</x:v>
+        <x:v>1472</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>1485</x:v>
+        <x:v>1473</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G36" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H36" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I36" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J36" s="3" t="s">
         <x:v>42</x:v>
@@ -12931,31 +12895,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>1486</x:v>
+        <x:v>1474</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>1487</x:v>
+        <x:v>1475</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>1488</x:v>
+        <x:v>1476</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>1489</x:v>
+        <x:v>1477</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>1490</x:v>
+        <x:v>1478</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>1491</x:v>
+        <x:v>1479</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>1492</x:v>
+        <x:v>1480</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>1493</x:v>
+        <x:v>1481</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>2</x:v>
@@ -12963,31 +12927,31 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>1494</x:v>
+        <x:v>1482</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>1495</x:v>
+        <x:v>1483</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>1496</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>1497</x:v>
+        <x:v>1485</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G37" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H37" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I37" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J37" s="3" t="s">
         <x:v>42</x:v>
@@ -12996,31 +12960,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>1498</x:v>
+        <x:v>1486</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>1499</x:v>
+        <x:v>1487</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>1500</x:v>
+        <x:v>1488</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>1501</x:v>
+        <x:v>1489</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>1502</x:v>
+        <x:v>1490</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>1503</x:v>
+        <x:v>1491</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>1504</x:v>
+        <x:v>1492</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>1505</x:v>
+        <x:v>1493</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>1499</x:v>
+        <x:v>1487</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>2</x:v>
@@ -13028,31 +12992,31 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>1506</x:v>
+        <x:v>1494</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>1507</x:v>
+        <x:v>1495</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>1508</x:v>
+        <x:v>1496</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>1509</x:v>
+        <x:v>1497</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G38" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H38" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I38" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J38" s="3" t="s">
         <x:v>42</x:v>
@@ -13061,31 +13025,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>1510</x:v>
+        <x:v>1498</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>1181</x:v>
+        <x:v>1169</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>1511</x:v>
+        <x:v>1499</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>1512</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>1513</x:v>
+        <x:v>1501</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>1514</x:v>
+        <x:v>1502</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>1515</x:v>
+        <x:v>1503</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>1516</x:v>
+        <x:v>1504</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>1517</x:v>
+        <x:v>1505</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>2</x:v>
@@ -13093,31 +13057,31 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>1518</x:v>
+        <x:v>1506</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>1519</x:v>
+        <x:v>1507</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>1520</x:v>
+        <x:v>1508</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>1521</x:v>
+        <x:v>1509</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G39" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="H39" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="I39" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="J39" s="3" t="s">
         <x:v>42</x:v>
@@ -13126,31 +13090,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>1522</x:v>
+        <x:v>1510</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>1523</x:v>
+        <x:v>1511</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>1524</x:v>
+        <x:v>1512</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>1525</x:v>
+        <x:v>1513</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>1526</x:v>
+        <x:v>1514</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>1527</x:v>
+        <x:v>1515</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>1528</x:v>
+        <x:v>1516</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>1529</x:v>
+        <x:v>1517</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>2</x:v>
@@ -13159,7 +13123,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re0c04c5ebaf74cc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c04358f949c462e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-048 onboarding contract tests
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra86334ab48034524"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re159ddff5dfa44a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R2fbb87b2f76d4769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf25d7749c86c4d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rdeef7a0febab4fcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4740b7357b48447b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R03205b3fc3d64680"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R46d2b9c8eaf44d8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3091,70 +3091,37 @@
     <x:t xml:space="preserve">PaymentsController.cs:16-85; InvoiceList.razor:587-589; InvoiceDetail.razor:62-294</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">INT-048</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Employee onboarding</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As an HR employee, I can review onboarding summaries, open an employee checklist, and update onboarding task progress.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Onboarding BFF exposes paged onboarding summaries, employee checklist detail, and task progress patch operations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HR onboarding UI/BFF -&gt; LifecycleService onboarding DTOs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">OnboardingController.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/hr/onboarding navigation context; onboarding checklist/task surfaces</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">OnboardingController GET, GET {employeeId}/checklist, PATCH {employeeId}/tasks</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Intranet BFF, LifecycleService</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Onboarding task progress</x:t>
+    <x:t xml:space="preserve">INT-049</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Performance reviews and goals</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As an HR employee, I can review performance reviews and goals.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Performance BFF exposes reviews and goals through permission-gated endpoints backed by PerformanceService.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">HR performance UI/BFF -&gt; PerformanceService reviews/goals DTOs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">PerformanceController.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">/hr/performance navigation context; reviews/goals surfaces</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">PerformanceController GET reviews, goals</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Intranet BFF, PerformanceService</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Read-only performance review and goal data</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Needs current page/navigation exposure review.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">OnboardingController.cs:15-45; ChatDrawer.razor:406</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">INT-049</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Performance reviews and goals</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As an HR employee, I can review performance reviews and goals.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Performance BFF exposes reviews and goals through permission-gated endpoints backed by PerformanceService.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">HR performance UI/BFF -&gt; PerformanceService reviews/goals DTOs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PerformanceController.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/hr/performance navigation context; reviews/goals surfaces</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PerformanceController GET reviews, goals</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Intranet BFF, PerformanceService</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Read-only performance review and goal data</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">PerformanceController.cs:17-36; ChatDrawer.razor:409</x:t>
@@ -7136,7 +7103,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb438ffdb80624151"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc745fbd22bbf4457"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10290,85 +10257,85 @@
       </x:c>
     </x:row>
     <x:row r="49" ht="51.29999923706055" hidden="0">
-      <x:c r="A49" s="3" t="s">
-        <x:v>1026</x:v>
-      </x:c>
-      <x:c r="B49" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C49" s="3" t="s">
-        <x:v>1027</x:v>
-      </x:c>
-      <x:c r="D49" s="3" t="s">
-        <x:v>1028</x:v>
-      </x:c>
-      <x:c r="E49" s="3" t="s">
-        <x:v>1029</x:v>
-      </x:c>
-      <x:c r="F49" s="3" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="G49" s="3" t="s">
-        <x:v>1001</x:v>
-      </x:c>
-      <x:c r="H49" s="3" t="s">
-        <x:v>1002</x:v>
-      </x:c>
-      <x:c r="I49" s="3" t="s">
-        <x:v>1003</x:v>
-      </x:c>
-      <x:c r="J49" s="3" t="s">
-        <x:v>1004</x:v>
-      </x:c>
-      <x:c r="K49" s="3" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="L49" s="3" t="s">
-        <x:v>1030</x:v>
-      </x:c>
-      <x:c r="M49" s="3" t="s">
-        <x:v>1031</x:v>
-      </x:c>
-      <x:c r="N49" s="3" t="s">
-        <x:v>1032</x:v>
-      </x:c>
-      <x:c r="O49" s="3" t="s">
-        <x:v>1033</x:v>
-      </x:c>
-      <x:c r="P49" s="3" t="s">
-        <x:v>1009</x:v>
-      </x:c>
-      <x:c r="Q49" s="3" t="s">
-        <x:v>1034</x:v>
-      </x:c>
-      <x:c r="R49" s="3" t="s">
-        <x:v>1035</x:v>
-      </x:c>
-      <x:c r="S49" s="3" t="s">
-        <x:v>1036</x:v>
-      </x:c>
-      <x:c r="T49" s="3" t="s">
-        <x:v>1037</x:v>
-      </x:c>
-      <x:c r="U49" s="3" t="s">
-        <x:v>2</x:v>
+      <x:c r="A49" s="3" t="str">
+        <x:v>INT-048</x:v>
+      </x:c>
+      <x:c r="B49" s="3" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C49" s="3" t="str">
+        <x:v>Employee onboarding</x:v>
+      </x:c>
+      <x:c r="D49" s="3" t="str">
+        <x:v>As an HR employee, I can review onboarding summaries, open an employee checklist, and update onboarding task progress.</x:v>
+      </x:c>
+      <x:c r="E49" s="3" t="str">
+        <x:v>Onboarding BFF exposes paged onboarding summaries, employee checklist detail, and task progress patch operations.</x:v>
+      </x:c>
+      <x:c r="F49" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G49" s="3" t="str">
+        <x:v>Focused behavior tests passed 2026-06-23.</x:v>
+      </x:c>
+      <x:c r="H49" s="3" t="str">
+        <x:v>No behavior error observed in current focused controller/client/navigation retest.</x:v>
+      </x:c>
+      <x:c r="I49" s="3" t="str">
+        <x:v>No app-code fix needed; added missing focused coverage in Maliev.Intranet commit e6e994e.</x:v>
+      </x:c>
+      <x:c r="J49" s="3" t="str">
+        <x:v>Retested OnboardingControllerTests 11/11 passed.</x:v>
+      </x:c>
+      <x:c r="K49" s="3" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L49" s="3" t="str">
+        <x:v>HR onboarding UI/BFF -&gt; LifecycleService onboarding DTOs</x:v>
+      </x:c>
+      <x:c r="M49" s="3" t="str">
+        <x:v>OnboardingController.cs</x:v>
+      </x:c>
+      <x:c r="N49" s="3" t="str">
+        <x:v>/hr/onboarding navigation context; onboarding checklist/task surfaces</x:v>
+      </x:c>
+      <x:c r="O49" s="3" t="str">
+        <x:v>OnboardingController GET, GET {employeeId}/checklist, PATCH {employeeId}/tasks</x:v>
+      </x:c>
+      <x:c r="P49" s="3" t="str">
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~OnboardingControllerTests" --verbosity minimal passed 11/11 on 2026-06-23. Coverage verifies onboarding list fallback, checklist missing-state, task update outcomes, read/write permission requirements, LifecycleService pending-list endpoint and progress mapping, checklist task mapping, completion endpoint behavior, and ChatDrawer /hr/onboarding label exposure.</x:v>
+      </x:c>
+      <x:c r="Q49" s="3" t="str">
+        <x:v>Intranet BFF, LifecycleService</x:v>
+      </x:c>
+      <x:c r="R49" s="3" t="str">
+        <x:v>Onboarding task progress</x:v>
+      </x:c>
+      <x:c r="S49" s="3" t="str">
+        <x:v>No remaining INT-048 API/client contract gap from this focused retest. Current code search found API/chat navigation exposure, not a dedicated onboarding Razor page route; full authenticated UI route review remains for later browser/Aspire pass.</x:v>
+      </x:c>
+      <x:c r="T49" s="3" t="str">
+        <x:v>OnboardingController.cs:15-45; LifecycleServiceClient.cs:8-129; OnboardingControllerTests.cs:1-233; ChatDrawer.razor:406</x:v>
+      </x:c>
+      <x:c r="U49" s="3" t="str">
+        <x:v>2026-06-23</x:v>
       </x:c>
     </x:row>
     <x:row r="50" ht="51.29999923706055" hidden="0">
       <x:c r="A50" s="3" t="s">
-        <x:v>1038</x:v>
+        <x:v>1026</x:v>
       </x:c>
       <x:c r="B50" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C50" s="3" t="s">
-        <x:v>1039</x:v>
+        <x:v>1027</x:v>
       </x:c>
       <x:c r="D50" s="3" t="s">
-        <x:v>1040</x:v>
+        <x:v>1028</x:v>
       </x:c>
       <x:c r="E50" s="3" t="s">
-        <x:v>1041</x:v>
+        <x:v>1029</x:v>
       </x:c>
       <x:c r="F50" s="3" t="s">
         <x:v>38</x:v>
@@ -10389,31 +10356,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L50" s="3" t="s">
-        <x:v>1042</x:v>
+        <x:v>1030</x:v>
       </x:c>
       <x:c r="M50" s="3" t="s">
-        <x:v>1043</x:v>
+        <x:v>1031</x:v>
       </x:c>
       <x:c r="N50" s="3" t="s">
-        <x:v>1044</x:v>
+        <x:v>1032</x:v>
       </x:c>
       <x:c r="O50" s="3" t="s">
-        <x:v>1045</x:v>
+        <x:v>1033</x:v>
       </x:c>
       <x:c r="P50" s="3" t="s">
         <x:v>1009</x:v>
       </x:c>
       <x:c r="Q50" s="3" t="s">
-        <x:v>1046</x:v>
+        <x:v>1034</x:v>
       </x:c>
       <x:c r="R50" s="3" t="s">
-        <x:v>1047</x:v>
+        <x:v>1035</x:v>
       </x:c>
       <x:c r="S50" s="3" t="s">
         <x:v>1036</x:v>
       </x:c>
       <x:c r="T50" s="3" t="s">
-        <x:v>1048</x:v>
+        <x:v>1037</x:v>
       </x:c>
       <x:c r="U50" s="3" t="s">
         <x:v>2</x:v>
@@ -10552,7 +10519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R292f9d36064a4636"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0be5823c6d34b85"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10652,64 +10619,64 @@
     </x:row>
     <x:row r="2" ht="149.25" hidden="0">
       <x:c r="A2" s="3" t="s">
-        <x:v>1049</x:v>
+        <x:v>1038</x:v>
       </x:c>
       <x:c r="B2" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C2" s="3" t="s">
-        <x:v>1050</x:v>
+        <x:v>1039</x:v>
       </x:c>
       <x:c r="D2" s="3" t="s">
-        <x:v>1051</x:v>
+        <x:v>1040</x:v>
       </x:c>
       <x:c r="E2" s="3" t="s">
-        <x:v>1052</x:v>
+        <x:v>1041</x:v>
       </x:c>
       <x:c r="F2" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G2" s="3" t="s">
-        <x:v>1053</x:v>
+        <x:v>1042</x:v>
       </x:c>
       <x:c r="H2" s="3" t="s">
-        <x:v>1054</x:v>
+        <x:v>1043</x:v>
       </x:c>
       <x:c r="I2" s="3" t="s">
-        <x:v>1055</x:v>
+        <x:v>1044</x:v>
       </x:c>
       <x:c r="J2" s="3" t="s">
-        <x:v>1056</x:v>
+        <x:v>1045</x:v>
       </x:c>
       <x:c r="K2" s="3" t="s">
         <x:v>188</x:v>
       </x:c>
       <x:c r="L2" s="3" t="s">
-        <x:v>1057</x:v>
+        <x:v>1046</x:v>
       </x:c>
       <x:c r="M2" s="3" t="s">
-        <x:v>1058</x:v>
+        <x:v>1047</x:v>
       </x:c>
       <x:c r="N2" s="3" t="s">
-        <x:v>1059</x:v>
+        <x:v>1048</x:v>
       </x:c>
       <x:c r="O2" s="3" t="s">
-        <x:v>1060</x:v>
+        <x:v>1049</x:v>
       </x:c>
       <x:c r="P2" s="3" t="s">
-        <x:v>1061</x:v>
+        <x:v>1050</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="s">
-        <x:v>1062</x:v>
+        <x:v>1051</x:v>
       </x:c>
       <x:c r="R2" s="3" t="s">
-        <x:v>1063</x:v>
+        <x:v>1052</x:v>
       </x:c>
       <x:c r="S2" s="3" t="s">
-        <x:v>1064</x:v>
+        <x:v>1053</x:v>
       </x:c>
       <x:c r="T2" s="3" t="s">
-        <x:v>1065</x:v>
+        <x:v>1054</x:v>
       </x:c>
       <x:c r="U2" s="3" t="s">
         <x:v>2</x:v>
@@ -10717,31 +10684,31 @@
     </x:row>
     <x:row r="3" ht="107.25" hidden="0">
       <x:c r="A3" s="3" t="s">
-        <x:v>1066</x:v>
+        <x:v>1055</x:v>
       </x:c>
       <x:c r="B3" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C3" s="3" t="s">
-        <x:v>1067</x:v>
+        <x:v>1056</x:v>
       </x:c>
       <x:c r="D3" s="3" t="s">
-        <x:v>1068</x:v>
+        <x:v>1057</x:v>
       </x:c>
       <x:c r="E3" s="3" t="s">
-        <x:v>1069</x:v>
+        <x:v>1058</x:v>
       </x:c>
       <x:c r="F3" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G3" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H3" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I3" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J3" s="3" t="s">
         <x:v>42</x:v>
@@ -10750,31 +10717,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L3" s="3" t="s">
-        <x:v>1073</x:v>
+        <x:v>1062</x:v>
       </x:c>
       <x:c r="M3" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N3" s="3" t="s">
-        <x:v>1075</x:v>
+        <x:v>1064</x:v>
       </x:c>
       <x:c r="O3" s="3" t="s">
-        <x:v>1076</x:v>
+        <x:v>1065</x:v>
       </x:c>
       <x:c r="P3" s="3" t="s">
-        <x:v>1077</x:v>
+        <x:v>1066</x:v>
       </x:c>
       <x:c r="Q3" s="3" t="s">
-        <x:v>1078</x:v>
+        <x:v>1067</x:v>
       </x:c>
       <x:c r="R3" s="3" t="s">
-        <x:v>1079</x:v>
+        <x:v>1068</x:v>
       </x:c>
       <x:c r="S3" s="3" t="s">
-        <x:v>1080</x:v>
+        <x:v>1069</x:v>
       </x:c>
       <x:c r="T3" s="3" t="s">
-        <x:v>1081</x:v>
+        <x:v>1070</x:v>
       </x:c>
       <x:c r="U3" s="3" t="s">
         <x:v>2</x:v>
@@ -10782,31 +10749,31 @@
     </x:row>
     <x:row r="4" ht="93.25" hidden="0">
       <x:c r="A4" s="3" t="s">
-        <x:v>1082</x:v>
+        <x:v>1071</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>1083</x:v>
+        <x:v>1072</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>1084</x:v>
+        <x:v>1073</x:v>
       </x:c>
       <x:c r="E4" s="3" t="s">
-        <x:v>1085</x:v>
+        <x:v>1074</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G4" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H4" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I4" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J4" s="3" t="s">
         <x:v>42</x:v>
@@ -10815,31 +10782,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L4" s="3" t="s">
-        <x:v>1086</x:v>
+        <x:v>1075</x:v>
       </x:c>
       <x:c r="M4" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N4" s="3" t="s">
-        <x:v>1087</x:v>
+        <x:v>1076</x:v>
       </x:c>
       <x:c r="O4" s="3" t="s">
-        <x:v>1088</x:v>
+        <x:v>1077</x:v>
       </x:c>
       <x:c r="P4" s="3" t="s">
-        <x:v>1089</x:v>
+        <x:v>1078</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="s">
-        <x:v>1090</x:v>
+        <x:v>1079</x:v>
       </x:c>
       <x:c r="R4" s="3" t="s">
-        <x:v>1091</x:v>
+        <x:v>1080</x:v>
       </x:c>
       <x:c r="S4" s="3" t="s">
-        <x:v>1092</x:v>
+        <x:v>1081</x:v>
       </x:c>
       <x:c r="T4" s="3" t="s">
-        <x:v>1093</x:v>
+        <x:v>1082</x:v>
       </x:c>
       <x:c r="U4" s="3" t="s">
         <x:v>2</x:v>
@@ -10847,31 +10814,31 @@
     </x:row>
     <x:row r="5" ht="107.25" hidden="0">
       <x:c r="A5" s="3" t="s">
-        <x:v>1094</x:v>
+        <x:v>1083</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>1095</x:v>
+        <x:v>1084</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>1096</x:v>
+        <x:v>1085</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>1097</x:v>
+        <x:v>1086</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
         <x:v>42</x:v>
@@ -10880,31 +10847,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>1098</x:v>
+        <x:v>1087</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>1099</x:v>
+        <x:v>1088</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>1100</x:v>
+        <x:v>1089</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>1101</x:v>
+        <x:v>1090</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>1102</x:v>
+        <x:v>1091</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>1103</x:v>
+        <x:v>1092</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>1104</x:v>
+        <x:v>1093</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>1105</x:v>
+        <x:v>1094</x:v>
       </x:c>
       <x:c r="U5" s="3" t="s">
         <x:v>2</x:v>
@@ -10912,31 +10879,31 @@
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
       <x:c r="A6" s="3" t="s">
-        <x:v>1106</x:v>
+        <x:v>1095</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>1107</x:v>
+        <x:v>1096</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>1108</x:v>
+        <x:v>1097</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>1109</x:v>
+        <x:v>1098</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H6" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I6" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J6" s="3" t="s">
         <x:v>42</x:v>
@@ -10945,31 +10912,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L6" s="3" t="s">
-        <x:v>1110</x:v>
+        <x:v>1099</x:v>
       </x:c>
       <x:c r="M6" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N6" s="3" t="s">
-        <x:v>1111</x:v>
+        <x:v>1100</x:v>
       </x:c>
       <x:c r="O6" s="3" t="s">
-        <x:v>1112</x:v>
+        <x:v>1101</x:v>
       </x:c>
       <x:c r="P6" s="3" t="s">
-        <x:v>1113</x:v>
+        <x:v>1102</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="s">
-        <x:v>1114</x:v>
+        <x:v>1103</x:v>
       </x:c>
       <x:c r="R6" s="3" t="s">
-        <x:v>1115</x:v>
+        <x:v>1104</x:v>
       </x:c>
       <x:c r="S6" s="3" t="s">
-        <x:v>1116</x:v>
+        <x:v>1105</x:v>
       </x:c>
       <x:c r="T6" s="3" t="s">
-        <x:v>1117</x:v>
+        <x:v>1106</x:v>
       </x:c>
       <x:c r="U6" s="3" t="s">
         <x:v>2</x:v>
@@ -10977,31 +10944,31 @@
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>1118</x:v>
+        <x:v>1107</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>1119</x:v>
+        <x:v>1108</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>1120</x:v>
+        <x:v>1109</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>1121</x:v>
+        <x:v>1110</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G7" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H7" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I7" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J7" s="3" t="s">
         <x:v>42</x:v>
@@ -11010,31 +10977,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
-        <x:v>1122</x:v>
+        <x:v>1111</x:v>
       </x:c>
       <x:c r="M7" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N7" s="3" t="s">
-        <x:v>1123</x:v>
+        <x:v>1112</x:v>
       </x:c>
       <x:c r="O7" s="3" t="s">
-        <x:v>1124</x:v>
+        <x:v>1113</x:v>
       </x:c>
       <x:c r="P7" s="3" t="s">
-        <x:v>1125</x:v>
+        <x:v>1114</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="s">
-        <x:v>1078</x:v>
+        <x:v>1067</x:v>
       </x:c>
       <x:c r="R7" s="3" t="s">
-        <x:v>1126</x:v>
+        <x:v>1115</x:v>
       </x:c>
       <x:c r="S7" s="3" t="s">
-        <x:v>1127</x:v>
+        <x:v>1116</x:v>
       </x:c>
       <x:c r="T7" s="3" t="s">
-        <x:v>1128</x:v>
+        <x:v>1117</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>2</x:v>
@@ -11042,31 +11009,31 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>1129</x:v>
+        <x:v>1118</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>1130</x:v>
+        <x:v>1119</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>1131</x:v>
+        <x:v>1120</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>1132</x:v>
+        <x:v>1121</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H8" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I8" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J8" s="3" t="s">
         <x:v>42</x:v>
@@ -11075,31 +11042,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
-        <x:v>1133</x:v>
+        <x:v>1122</x:v>
       </x:c>
       <x:c r="M8" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N8" s="3" t="s">
-        <x:v>1134</x:v>
+        <x:v>1123</x:v>
       </x:c>
       <x:c r="O8" s="3" t="s">
-        <x:v>1135</x:v>
+        <x:v>1124</x:v>
       </x:c>
       <x:c r="P8" s="3" t="s">
-        <x:v>1136</x:v>
+        <x:v>1125</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="s">
-        <x:v>1137</x:v>
+        <x:v>1126</x:v>
       </x:c>
       <x:c r="R8" s="3" t="s">
-        <x:v>1138</x:v>
+        <x:v>1127</x:v>
       </x:c>
       <x:c r="S8" s="3" t="s">
-        <x:v>1139</x:v>
+        <x:v>1128</x:v>
       </x:c>
       <x:c r="T8" s="3" t="s">
-        <x:v>1140</x:v>
+        <x:v>1129</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>2</x:v>
@@ -11107,31 +11074,31 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>1141</x:v>
+        <x:v>1130</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>1142</x:v>
+        <x:v>1131</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>1143</x:v>
+        <x:v>1132</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>1144</x:v>
+        <x:v>1133</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H9" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I9" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J9" s="3" t="s">
         <x:v>42</x:v>
@@ -11140,31 +11107,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
-        <x:v>1145</x:v>
+        <x:v>1134</x:v>
       </x:c>
       <x:c r="M9" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N9" s="3" t="s">
-        <x:v>1146</x:v>
+        <x:v>1135</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>1147</x:v>
+        <x:v>1136</x:v>
       </x:c>
       <x:c r="P9" s="3" t="s">
-        <x:v>1148</x:v>
+        <x:v>1137</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="s">
-        <x:v>1149</x:v>
+        <x:v>1138</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
-        <x:v>1150</x:v>
+        <x:v>1139</x:v>
       </x:c>
       <x:c r="S9" s="3" t="s">
-        <x:v>1151</x:v>
+        <x:v>1140</x:v>
       </x:c>
       <x:c r="T9" s="3" t="s">
-        <x:v>1152</x:v>
+        <x:v>1141</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>2</x:v>
@@ -11172,31 +11139,31 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>1153</x:v>
+        <x:v>1142</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>1154</x:v>
+        <x:v>1143</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>1155</x:v>
+        <x:v>1144</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>1156</x:v>
+        <x:v>1145</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G10" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H10" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I10" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J10" s="3" t="s">
         <x:v>42</x:v>
@@ -11205,31 +11172,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>1157</x:v>
+        <x:v>1146</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
-        <x:v>1058</x:v>
+        <x:v>1047</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>1158</x:v>
+        <x:v>1147</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>1159</x:v>
+        <x:v>1148</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>1160</x:v>
+        <x:v>1149</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>1161</x:v>
+        <x:v>1150</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>1162</x:v>
+        <x:v>1151</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>1163</x:v>
+        <x:v>1152</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>2</x:v>
@@ -11237,31 +11204,31 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>1164</x:v>
+        <x:v>1153</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>1165</x:v>
+        <x:v>1154</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>1166</x:v>
+        <x:v>1155</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>1167</x:v>
+        <x:v>1156</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G11" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H11" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I11" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J11" s="3" t="s">
         <x:v>42</x:v>
@@ -11270,31 +11237,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>1168</x:v>
+        <x:v>1157</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>1169</x:v>
+        <x:v>1158</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>1170</x:v>
+        <x:v>1159</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>1171</x:v>
+        <x:v>1160</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>1172</x:v>
+        <x:v>1161</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>1173</x:v>
+        <x:v>1162</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>1174</x:v>
+        <x:v>1163</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>1175</x:v>
+        <x:v>1164</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>1176</x:v>
+        <x:v>1165</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>2</x:v>
@@ -11302,31 +11269,31 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>1177</x:v>
+        <x:v>1166</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>1178</x:v>
+        <x:v>1167</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>1179</x:v>
+        <x:v>1168</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>1180</x:v>
+        <x:v>1169</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G12" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H12" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I12" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J12" s="3" t="s">
         <x:v>42</x:v>
@@ -11335,31 +11302,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>1181</x:v>
+        <x:v>1170</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>1182</x:v>
+        <x:v>1171</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>1183</x:v>
+        <x:v>1172</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>1184</x:v>
+        <x:v>1173</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>1185</x:v>
+        <x:v>1174</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>1186</x:v>
+        <x:v>1175</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>1187</x:v>
+        <x:v>1176</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>1188</x:v>
+        <x:v>1177</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>2</x:v>
@@ -11367,31 +11334,31 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>1189</x:v>
+        <x:v>1178</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>1190</x:v>
+        <x:v>1179</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>1191</x:v>
+        <x:v>1180</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>1192</x:v>
+        <x:v>1181</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I13" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J13" s="3" t="s">
         <x:v>42</x:v>
@@ -11400,31 +11367,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>1193</x:v>
+        <x:v>1182</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>1194</x:v>
+        <x:v>1183</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>1195</x:v>
+        <x:v>1184</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>1196</x:v>
+        <x:v>1185</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
-        <x:v>1185</x:v>
+        <x:v>1174</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>1197</x:v>
+        <x:v>1186</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>1198</x:v>
+        <x:v>1187</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>1199</x:v>
+        <x:v>1188</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>2</x:v>
@@ -11432,31 +11399,31 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>1200</x:v>
+        <x:v>1189</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>1201</x:v>
+        <x:v>1190</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>1202</x:v>
+        <x:v>1191</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>1203</x:v>
+        <x:v>1192</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G14" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H14" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I14" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J14" s="3" t="s">
         <x:v>42</x:v>
@@ -11465,31 +11432,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>1204</x:v>
+        <x:v>1193</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>1205</x:v>
+        <x:v>1194</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>1206</x:v>
+        <x:v>1195</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>1207</x:v>
+        <x:v>1196</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>1208</x:v>
+        <x:v>1197</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>1209</x:v>
+        <x:v>1198</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>1210</x:v>
+        <x:v>1199</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>1211</x:v>
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>1212</x:v>
+        <x:v>1201</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>2</x:v>
@@ -11497,31 +11464,31 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>1213</x:v>
+        <x:v>1202</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>1214</x:v>
+        <x:v>1203</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>1215</x:v>
+        <x:v>1204</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>1216</x:v>
+        <x:v>1205</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G15" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H15" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I15" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J15" s="3" t="s">
         <x:v>42</x:v>
@@ -11530,31 +11497,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>1217</x:v>
+        <x:v>1206</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>1218</x:v>
+        <x:v>1207</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>1219</x:v>
+        <x:v>1208</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>1220</x:v>
+        <x:v>1209</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>1221</x:v>
+        <x:v>1210</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>1222</x:v>
+        <x:v>1211</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>1223</x:v>
+        <x:v>1212</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>1224</x:v>
+        <x:v>1213</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>2</x:v>
@@ -11562,31 +11529,31 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>1225</x:v>
+        <x:v>1214</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>1226</x:v>
+        <x:v>1215</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>1227</x:v>
+        <x:v>1216</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>1228</x:v>
+        <x:v>1217</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H16" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I16" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J16" s="3" t="s">
         <x:v>42</x:v>
@@ -11595,31 +11562,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>1229</x:v>
+        <x:v>1218</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>1230</x:v>
+        <x:v>1219</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>1231</x:v>
+        <x:v>1220</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>1232</x:v>
+        <x:v>1221</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>1233</x:v>
+        <x:v>1222</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>1234</x:v>
+        <x:v>1223</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>1235</x:v>
+        <x:v>1224</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>1236</x:v>
+        <x:v>1225</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>2</x:v>
@@ -11627,31 +11594,31 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>1237</x:v>
+        <x:v>1226</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>1238</x:v>
+        <x:v>1227</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>1239</x:v>
+        <x:v>1228</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>1240</x:v>
+        <x:v>1229</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H17" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I17" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J17" s="3" t="s">
         <x:v>42</x:v>
@@ -11660,31 +11627,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>1241</x:v>
+        <x:v>1230</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>1242</x:v>
+        <x:v>1231</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>1243</x:v>
+        <x:v>1232</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>1244</x:v>
+        <x:v>1233</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>1245</x:v>
+        <x:v>1234</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>1246</x:v>
+        <x:v>1235</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>1247</x:v>
+        <x:v>1236</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>1248</x:v>
+        <x:v>1237</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>1249</x:v>
+        <x:v>1238</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>2</x:v>
@@ -11692,31 +11659,31 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>1250</x:v>
+        <x:v>1239</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>1251</x:v>
+        <x:v>1240</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>1252</x:v>
+        <x:v>1241</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>1253</x:v>
+        <x:v>1242</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G18" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H18" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I18" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J18" s="3" t="s">
         <x:v>42</x:v>
@@ -11725,31 +11692,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>1254</x:v>
+        <x:v>1243</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>1255</x:v>
+        <x:v>1244</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>1256</x:v>
+        <x:v>1245</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>1257</x:v>
+        <x:v>1246</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>1258</x:v>
+        <x:v>1247</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>1259</x:v>
+        <x:v>1248</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>1260</x:v>
+        <x:v>1249</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>1261</x:v>
+        <x:v>1250</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>1262</x:v>
+        <x:v>1251</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>2</x:v>
@@ -11757,31 +11724,31 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>1263</x:v>
+        <x:v>1252</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>1264</x:v>
+        <x:v>1253</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>1265</x:v>
+        <x:v>1254</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>1266</x:v>
+        <x:v>1255</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I19" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J19" s="3" t="s">
         <x:v>42</x:v>
@@ -11790,31 +11757,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>1267</x:v>
+        <x:v>1256</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>1268</x:v>
+        <x:v>1257</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>1269</x:v>
+        <x:v>1258</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>1270</x:v>
+        <x:v>1259</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>1271</x:v>
+        <x:v>1260</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>1272</x:v>
+        <x:v>1261</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>1273</x:v>
+        <x:v>1262</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>1274</x:v>
+        <x:v>1263</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>1275</x:v>
+        <x:v>1264</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>2</x:v>
@@ -11822,31 +11789,31 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>1276</x:v>
+        <x:v>1265</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>1277</x:v>
+        <x:v>1266</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>1278</x:v>
+        <x:v>1267</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>1279</x:v>
+        <x:v>1268</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I20" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J20" s="3" t="s">
         <x:v>42</x:v>
@@ -11855,31 +11822,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>1280</x:v>
+        <x:v>1269</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>1281</x:v>
+        <x:v>1270</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>1282</x:v>
+        <x:v>1271</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>1283</x:v>
+        <x:v>1272</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>1284</x:v>
+        <x:v>1273</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>1285</x:v>
+        <x:v>1274</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>1286</x:v>
+        <x:v>1275</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>1287</x:v>
+        <x:v>1276</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>1288</x:v>
+        <x:v>1277</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>2</x:v>
@@ -11887,31 +11854,31 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>1289</x:v>
+        <x:v>1278</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>1290</x:v>
+        <x:v>1279</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>1291</x:v>
+        <x:v>1280</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>1292</x:v>
+        <x:v>1281</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G21" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H21" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I21" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J21" s="3" t="s">
         <x:v>42</x:v>
@@ -11920,31 +11887,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>1293</x:v>
+        <x:v>1282</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>1294</x:v>
+        <x:v>1283</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>1295</x:v>
+        <x:v>1284</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>1296</x:v>
+        <x:v>1285</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>1297</x:v>
+        <x:v>1286</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>1298</x:v>
+        <x:v>1287</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>1299</x:v>
+        <x:v>1288</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>2</x:v>
@@ -11952,31 +11919,31 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>1300</x:v>
+        <x:v>1289</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>1301</x:v>
+        <x:v>1290</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>1302</x:v>
+        <x:v>1291</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>1303</x:v>
+        <x:v>1292</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G22" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H22" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I22" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J22" s="3" t="s">
         <x:v>42</x:v>
@@ -11985,31 +11952,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>1304</x:v>
+        <x:v>1293</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>1169</x:v>
+        <x:v>1158</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>1305</x:v>
+        <x:v>1294</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>1306</x:v>
+        <x:v>1295</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>1307</x:v>
+        <x:v>1296</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>1308</x:v>
+        <x:v>1297</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>1309</x:v>
+        <x:v>1298</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>1310</x:v>
+        <x:v>1299</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>1311</x:v>
+        <x:v>1300</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>2</x:v>
@@ -12017,31 +11984,31 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>1312</x:v>
+        <x:v>1301</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>1313</x:v>
+        <x:v>1302</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>1314</x:v>
+        <x:v>1303</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>1315</x:v>
+        <x:v>1304</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G23" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H23" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I23" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J23" s="3" t="s">
         <x:v>42</x:v>
@@ -12050,31 +12017,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>1316</x:v>
+        <x:v>1305</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>1317</x:v>
+        <x:v>1306</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>1318</x:v>
+        <x:v>1307</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>1319</x:v>
+        <x:v>1308</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>1320</x:v>
+        <x:v>1309</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>1321</x:v>
+        <x:v>1310</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>1322</x:v>
+        <x:v>1311</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>1323</x:v>
+        <x:v>1312</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>1324</x:v>
+        <x:v>1313</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>2</x:v>
@@ -12082,31 +12049,31 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>1325</x:v>
+        <x:v>1314</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>1326</x:v>
+        <x:v>1315</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>1327</x:v>
+        <x:v>1316</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>1328</x:v>
+        <x:v>1317</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H24" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I24" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J24" s="3" t="s">
         <x:v>42</x:v>
@@ -12115,31 +12082,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>1329</x:v>
+        <x:v>1318</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>1294</x:v>
+        <x:v>1283</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>1330</x:v>
+        <x:v>1319</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>1331</x:v>
+        <x:v>1320</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>1332</x:v>
+        <x:v>1321</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>1333</x:v>
+        <x:v>1322</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>1334</x:v>
+        <x:v>1323</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>1335</x:v>
+        <x:v>1324</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>1336</x:v>
+        <x:v>1325</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>2</x:v>
@@ -12147,31 +12114,31 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>1337</x:v>
+        <x:v>1326</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>1338</x:v>
+        <x:v>1327</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>1339</x:v>
+        <x:v>1328</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>1340</x:v>
+        <x:v>1329</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H25" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I25" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J25" s="3" t="s">
         <x:v>42</x:v>
@@ -12180,31 +12147,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>1341</x:v>
+        <x:v>1330</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>1294</x:v>
+        <x:v>1283</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>1342</x:v>
+        <x:v>1331</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>1343</x:v>
+        <x:v>1332</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>1344</x:v>
+        <x:v>1333</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>1345</x:v>
+        <x:v>1334</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>1346</x:v>
+        <x:v>1335</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>1347</x:v>
+        <x:v>1336</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>1348</x:v>
+        <x:v>1337</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>2</x:v>
@@ -12212,31 +12179,31 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>1349</x:v>
+        <x:v>1338</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>1350</x:v>
+        <x:v>1339</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>1351</x:v>
+        <x:v>1340</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>1352</x:v>
+        <x:v>1341</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H26" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I26" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J26" s="3" t="s">
         <x:v>42</x:v>
@@ -12245,31 +12212,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>1353</x:v>
+        <x:v>1342</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>1354</x:v>
+        <x:v>1343</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>1355</x:v>
+        <x:v>1344</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>1356</x:v>
+        <x:v>1345</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>1357</x:v>
+        <x:v>1346</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>1358</x:v>
+        <x:v>1347</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>1359</x:v>
+        <x:v>1348</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>1360</x:v>
+        <x:v>1349</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>1361</x:v>
+        <x:v>1350</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>2</x:v>
@@ -12277,31 +12244,31 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>1362</x:v>
+        <x:v>1351</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>1363</x:v>
+        <x:v>1352</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>1364</x:v>
+        <x:v>1353</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>1365</x:v>
+        <x:v>1354</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H27" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I27" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J27" s="3" t="s">
         <x:v>42</x:v>
@@ -12310,31 +12277,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>1366</x:v>
+        <x:v>1355</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>1367</x:v>
+        <x:v>1356</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>1368</x:v>
+        <x:v>1357</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>1369</x:v>
+        <x:v>1358</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>1370</x:v>
+        <x:v>1359</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>1371</x:v>
+        <x:v>1360</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>1372</x:v>
+        <x:v>1361</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
         <x:v>789</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>1373</x:v>
+        <x:v>1362</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>2</x:v>
@@ -12342,31 +12309,31 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>1374</x:v>
+        <x:v>1363</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>1375</x:v>
+        <x:v>1364</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>1376</x:v>
+        <x:v>1365</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>1377</x:v>
+        <x:v>1366</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G28" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H28" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I28" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J28" s="3" t="s">
         <x:v>42</x:v>
@@ -12375,31 +12342,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>1378</x:v>
+        <x:v>1367</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>1379</x:v>
+        <x:v>1368</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>1380</x:v>
+        <x:v>1369</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>1381</x:v>
+        <x:v>1370</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>1382</x:v>
+        <x:v>1371</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>1383</x:v>
+        <x:v>1372</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>1384</x:v>
+        <x:v>1373</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>1385</x:v>
+        <x:v>1374</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>2</x:v>
@@ -12407,31 +12374,31 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>1386</x:v>
+        <x:v>1375</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>1387</x:v>
+        <x:v>1376</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>1388</x:v>
+        <x:v>1377</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>1389</x:v>
+        <x:v>1378</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G29" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H29" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I29" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J29" s="3" t="s">
         <x:v>42</x:v>
@@ -12440,31 +12407,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>1390</x:v>
+        <x:v>1379</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>1391</x:v>
+        <x:v>1380</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>1392</x:v>
+        <x:v>1381</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>1393</x:v>
+        <x:v>1382</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>1394</x:v>
+        <x:v>1383</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>1395</x:v>
+        <x:v>1384</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>1396</x:v>
+        <x:v>1385</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>1397</x:v>
+        <x:v>1386</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>1398</x:v>
+        <x:v>1387</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>2</x:v>
@@ -12472,31 +12439,31 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>1399</x:v>
+        <x:v>1388</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>1400</x:v>
+        <x:v>1389</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>1401</x:v>
+        <x:v>1390</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>1402</x:v>
+        <x:v>1391</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G30" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H30" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I30" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J30" s="3" t="s">
         <x:v>42</x:v>
@@ -12505,31 +12472,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>1403</x:v>
+        <x:v>1392</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>1404</x:v>
+        <x:v>1393</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>1405</x:v>
+        <x:v>1394</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>1406</x:v>
+        <x:v>1395</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>1407</x:v>
+        <x:v>1396</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>1408</x:v>
+        <x:v>1397</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>1409</x:v>
+        <x:v>1398</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>1410</x:v>
+        <x:v>1399</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>1411</x:v>
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>2</x:v>
@@ -12537,7 +12504,7 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>1412</x:v>
+        <x:v>1401</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>9</x:v>
@@ -12546,22 +12513,22 @@
         <x:v>947</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>1413</x:v>
+        <x:v>1402</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>1414</x:v>
+        <x:v>1403</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G31" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H31" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I31" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J31" s="3" t="s">
         <x:v>42</x:v>
@@ -12570,31 +12537,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>1415</x:v>
+        <x:v>1404</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>1416</x:v>
+        <x:v>1405</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>1417</x:v>
+        <x:v>1406</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>1418</x:v>
+        <x:v>1407</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>1419</x:v>
+        <x:v>1408</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>1420</x:v>
+        <x:v>1409</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>1421</x:v>
+        <x:v>1410</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>1422</x:v>
+        <x:v>1411</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>1423</x:v>
+        <x:v>1412</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>2</x:v>
@@ -12602,31 +12569,31 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>1424</x:v>
+        <x:v>1413</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>1425</x:v>
+        <x:v>1414</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>1426</x:v>
+        <x:v>1415</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>1427</x:v>
+        <x:v>1416</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G32" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H32" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I32" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J32" s="3" t="s">
         <x:v>42</x:v>
@@ -12635,31 +12602,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>1428</x:v>
+        <x:v>1417</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>1429</x:v>
+        <x:v>1418</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>1430</x:v>
+        <x:v>1419</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>1431</x:v>
+        <x:v>1420</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>1432</x:v>
+        <x:v>1421</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>1433</x:v>
+        <x:v>1422</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
         <x:v>969</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>1434</x:v>
+        <x:v>1423</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>1435</x:v>
+        <x:v>1424</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>2</x:v>
@@ -12667,7 +12634,7 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>1436</x:v>
+        <x:v>1425</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>9</x:v>
@@ -12676,22 +12643,22 @@
         <x:v>740</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>1437</x:v>
+        <x:v>1426</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>1438</x:v>
+        <x:v>1427</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G33" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H33" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I33" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J33" s="3" t="s">
         <x:v>42</x:v>
@@ -12700,31 +12667,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>1439</x:v>
+        <x:v>1428</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>1440</x:v>
+        <x:v>1429</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>1441</x:v>
+        <x:v>1430</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>1442</x:v>
+        <x:v>1431</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>1443</x:v>
+        <x:v>1432</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>1444</x:v>
+        <x:v>1433</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>1445</x:v>
+        <x:v>1434</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>1446</x:v>
+        <x:v>1435</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>1447</x:v>
+        <x:v>1436</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>2</x:v>
@@ -12732,7 +12699,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>1448</x:v>
+        <x:v>1437</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>9</x:v>
@@ -12741,22 +12708,22 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>1449</x:v>
+        <x:v>1438</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>1450</x:v>
+        <x:v>1439</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G34" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H34" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I34" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J34" s="3" t="s">
         <x:v>42</x:v>
@@ -12765,31 +12732,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>1451</x:v>
+        <x:v>1440</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>1452</x:v>
+        <x:v>1441</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
         <x:v>978</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>1453</x:v>
+        <x:v>1442</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>1454</x:v>
+        <x:v>1443</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>1455</x:v>
+        <x:v>1444</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>1456</x:v>
+        <x:v>1445</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>1457</x:v>
+        <x:v>1446</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>2</x:v>
@@ -12797,31 +12764,31 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>1458</x:v>
+        <x:v>1447</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>1459</x:v>
+        <x:v>1448</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>1460</x:v>
+        <x:v>1449</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>1461</x:v>
+        <x:v>1450</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G35" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H35" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I35" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J35" s="3" t="s">
         <x:v>42</x:v>
@@ -12830,31 +12797,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>1462</x:v>
+        <x:v>1451</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>1463</x:v>
+        <x:v>1452</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>1464</x:v>
+        <x:v>1453</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>1244</x:v>
+        <x:v>1233</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>1465</x:v>
+        <x:v>1454</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>1466</x:v>
+        <x:v>1455</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>1467</x:v>
+        <x:v>1456</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>1468</x:v>
+        <x:v>1457</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>1469</x:v>
+        <x:v>1458</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>2</x:v>
@@ -12862,31 +12829,31 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>1470</x:v>
+        <x:v>1459</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>1471</x:v>
+        <x:v>1460</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>1472</x:v>
+        <x:v>1461</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>1473</x:v>
+        <x:v>1462</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G36" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H36" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I36" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J36" s="3" t="s">
         <x:v>42</x:v>
@@ -12895,31 +12862,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>1474</x:v>
+        <x:v>1463</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>1475</x:v>
+        <x:v>1464</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>1476</x:v>
+        <x:v>1465</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>1477</x:v>
+        <x:v>1466</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>1478</x:v>
+        <x:v>1467</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>1479</x:v>
+        <x:v>1468</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>1480</x:v>
+        <x:v>1469</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>1481</x:v>
+        <x:v>1470</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>2</x:v>
@@ -12927,31 +12894,31 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>1482</x:v>
+        <x:v>1471</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>1483</x:v>
+        <x:v>1472</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>1484</x:v>
+        <x:v>1473</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>1485</x:v>
+        <x:v>1474</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G37" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H37" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I37" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J37" s="3" t="s">
         <x:v>42</x:v>
@@ -12960,31 +12927,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>1486</x:v>
+        <x:v>1475</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>1487</x:v>
+        <x:v>1476</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>1488</x:v>
+        <x:v>1477</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>1489</x:v>
+        <x:v>1478</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>1490</x:v>
+        <x:v>1479</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>1491</x:v>
+        <x:v>1480</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>1492</x:v>
+        <x:v>1481</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>1493</x:v>
+        <x:v>1482</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>1487</x:v>
+        <x:v>1476</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>2</x:v>
@@ -12992,31 +12959,31 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>1494</x:v>
+        <x:v>1483</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>1495</x:v>
+        <x:v>1484</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>1496</x:v>
+        <x:v>1485</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>1497</x:v>
+        <x:v>1486</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G38" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H38" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I38" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J38" s="3" t="s">
         <x:v>42</x:v>
@@ -13025,31 +12992,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>1498</x:v>
+        <x:v>1487</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>1169</x:v>
+        <x:v>1158</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>1499</x:v>
+        <x:v>1488</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>1500</x:v>
+        <x:v>1489</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>1501</x:v>
+        <x:v>1490</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>1502</x:v>
+        <x:v>1491</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>1503</x:v>
+        <x:v>1492</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>1504</x:v>
+        <x:v>1493</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>1505</x:v>
+        <x:v>1494</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>2</x:v>
@@ -13057,31 +13024,31 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>1506</x:v>
+        <x:v>1495</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>1507</x:v>
+        <x:v>1496</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>1508</x:v>
+        <x:v>1497</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>1509</x:v>
+        <x:v>1498</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>38</x:v>
       </x:c>
       <x:c r="G39" s="3" t="s">
-        <x:v>1070</x:v>
+        <x:v>1059</x:v>
       </x:c>
       <x:c r="H39" s="3" t="s">
-        <x:v>1071</x:v>
+        <x:v>1060</x:v>
       </x:c>
       <x:c r="I39" s="3" t="s">
-        <x:v>1072</x:v>
+        <x:v>1061</x:v>
       </x:c>
       <x:c r="J39" s="3" t="s">
         <x:v>42</x:v>
@@ -13090,31 +13057,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>1510</x:v>
+        <x:v>1499</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
-        <x:v>1074</x:v>
+        <x:v>1063</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>1511</x:v>
+        <x:v>1500</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>1512</x:v>
+        <x:v>1501</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>1513</x:v>
+        <x:v>1502</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>1514</x:v>
+        <x:v>1503</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>1515</x:v>
+        <x:v>1504</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>1516</x:v>
+        <x:v>1505</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>1517</x:v>
+        <x:v>1506</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>2</x:v>
@@ -13123,7 +13090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c04358f949c462e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6f54db87c1ad4ca1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-047 payment operations tests
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2ca833d25ca7421c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rf07ec86ee54748d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R6ca524d069f040c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R2145cbf2f9014f46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd44522217a6a44c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re5fdab6d002c462b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rb5127f55e28a4d94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rb1fd8cbccec34c9e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R616da65d0cb24080"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ae175a149ca4a63"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8363,55 +8363,55 @@
         <x:v>Payment operations</x:v>
       </x:c>
       <x:c r="D48" s="3" t="str">
-        <x:v>As a finance employee, I can review payment stats, inspect payments, create payments, allocate funds, and void payments.</x:v>
+        <x:v>As a finance employee, I can review payment stats, inspect payment records through the BFF, and record invoice payments from the invoice detail flow.</x:v>
       </x:c>
       <x:c r="E48" s="3" t="str">
-        <x:v>Payments BFF exposes stats, list, detail, create, allocate, and void actions with payment permissions.</x:v>
+        <x:v>Payment stats load in the invoice list, payment list/detail/create endpoints fail closed when PaymentService does not return data, invoice detail records and allocates payments through InvoiceService, and unsupported direct allocate/void actions return 404.</x:v>
       </x:c>
       <x:c r="F48" s="3" t="str">
-        <x:v>Current code-derived</x:v>
+        <x:v>Current code-derived; focused fallback fix applied.</x:v>
       </x:c>
       <x:c r="G48" s="3" t="str">
-        <x:v>Inventory added 2026-06-23; dedicated behavior test not started in this spreadsheet-only slice.</x:v>
+        <x:v>Focused behavior tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H48" s="3" t="str">
-        <x:v>No behavior error documented yet for this newly inventoried current-code story.</x:v>
+        <x:v>Focused contract review found PaymentServiceClient.GetPaymentsAsync threw on non-success responses instead of allowing the BFF empty-page fallback when PaymentService does not expose a list response.</x:v>
       </x:c>
       <x:c r="I48" s="3" t="str">
-        <x:v>No app fix attempted in this inventory-only slice.</x:v>
+        <x:v>Fixed in Maliev.Intranet commit 776400b by changing GetPaymentsAsync to use GetAsync, return null on non-success, and deserialize only successful responses.</x:v>
       </x:c>
       <x:c r="J48" s="3" t="str">
-        <x:v>Retest after behavior testing begins.</x:v>
+        <x:v>Retested PaymentsControllerTests 14/14 passed and InvoiceServiceClientTests.RecordInvoicePayment 1/1 passed.</x:v>
       </x:c>
       <x:c r="K48" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="L48" s="3" t="str">
-        <x:v>Finance UI/BFF -&gt; PaymentService -&gt; payment DTOs and allocation/void commands</x:v>
+        <x:v>Finance invoice UI -&gt; Intranet BFF payments/invoices endpoints -&gt; PaymentService metrics/payment endpoints and InvoiceService payment allocation</x:v>
       </x:c>
       <x:c r="M48" s="3" t="str">
         <x:v>InvoiceList.razor; InvoiceDetail.razor; PaymentsController.cs</x:v>
       </x:c>
       <x:c r="N48" s="3" t="str">
-        <x:v>/finance/invoices payment stats/actions; payment operation controls</x:v>
+        <x:v>/finance/invoices loads api/v1/payments/stats; /finance/invoices/{id} record-payment panel posts api/v1/invoices/{id}/payments</x:v>
       </x:c>
       <x:c r="O48" s="3" t="str">
-        <x:v>PaymentsController stats, GET, GET {id}, POST, allocate, void</x:v>
+        <x:v>PaymentsController stats/list/detail/create proxy PaymentService; list now falls back on non-success; allocate/void return 404 because PaymentService does not expose those actions; invoice payment recording uses InvoiceService /invoice/v1/payments plus /invoice/v1/payments/invoices/{invoiceId}/link.</x:v>
       </x:c>
       <x:c r="P48" s="3" t="str">
-        <x:v>Code inventory evidence only; map automated tests during the behavior-testing loop.</x:v>
+        <x:v>Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~PaymentsControllerTests" --verbosity minimal passed 14/14 on 2026-06-23. Impacted invoice payment allocation test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~InvoiceServiceClientTests.RecordInvoicePayment" --verbosity minimal passed 1/1 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q48" s="3" t="str">
-        <x:v>Intranet BFF, PaymentService, Accounting/Invoice flows</x:v>
+        <x:v>Intranet BFF, PaymentService, InvoiceService, Accounting/Invoice UI</x:v>
       </x:c>
       <x:c r="R48" s="3" t="str">
-        <x:v>Payment, allocation, and void records</x:v>
+        <x:v>Payment records and invoice payment allocations through InvoiceService; direct PaymentService list/detail reads are read-only.</x:v>
       </x:c>
       <x:c r="S48" s="3" t="str">
-        <x:v>Needs strict payment contract and permission retest.</x:v>
+        <x:v>Direct PaymentService allocate/void actions are not exposed by current PaymentService and therefore fail closed with 404; current finance UI records invoice payments through InvoiceService instead of a standalone payments page.</x:v>
       </x:c>
       <x:c r="T48" s="3" t="str">
-        <x:v>PaymentsController.cs:16-85; InvoiceList.razor:587-589; InvoiceDetail.razor:62-294</x:v>
+        <x:v>PaymentsController.cs:17-85; PaymentServiceClient.cs:16-80; PaymentsControllerTests.cs:14-216; InvoiceList.razor:587-589; InvoiceDetail.razor:82,209-218; InvoiceServiceClient.cs:140-204</x:v>
       </x:c>
       <x:c r="U48" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R59b70ff981684600"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8d0a7674e2e43f0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a71a26b85f34a87"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7e0ce4485ab4123"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-045 notification tests
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd44522217a6a44c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re5fdab6d002c462b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rb5127f55e28a4d94"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rb1fd8cbccec34c9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0987011c32f1450d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rdcbf1fd7a7b9495c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd57a51a0a93e4669"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R8cabf5f561354a2c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9ae175a149ca4a63"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61354ec81d3749b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8242,16 +8242,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G46" s="3" t="str">
-        <x:v>Inventory added 2026-06-23; dedicated behavior test not started in this spreadsheet-only slice.</x:v>
+        <x:v>Focused behavior tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H46" s="3" t="str">
-        <x:v>No behavior error documented yet for this newly inventoried current-code story.</x:v>
+        <x:v>No behavior error observed in current focused controller/client/source retest.</x:v>
       </x:c>
       <x:c r="I46" s="3" t="str">
-        <x:v>No app fix attempted in this inventory-only slice.</x:v>
+        <x:v>No app-code fix needed; existing focused coverage validates the current notification template and preference contracts.</x:v>
       </x:c>
       <x:c r="J46" s="3" t="str">
-        <x:v>Retest after behavior testing begins.</x:v>
+        <x:v>Retested notification/preference focused set 29/29 passed.</x:v>
       </x:c>
       <x:c r="K46" s="3" t="str">
         <x:v>P1</x:v>
@@ -8269,7 +8269,7 @@
         <x:v>NotificationController templates, delivery-logs, preferences</x:v>
       </x:c>
       <x:c r="P46" s="3" t="str">
-        <x:v>Code inventory evidence only; map automated tests during the behavior-testing loop.</x:v>
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~NotificationControllerTests|FullyQualifiedName~NotificationServiceClientTests|FullyQualifiedName~ModuleRegressionSourceTests.CustomerDetail_EmailDialogStaysOpenAndUsesNotificationTemplates|FullyQualifiedName~HrProfilePageTests" --verbosity minimal passed 29/29 on 2026-06-23. Coverage verifies notification template CRUD/read-log/preference permissions, NotificationService template/list/create/update/event/log mapping, customer email template panel source wiring, and HR profile preference behavior.</x:v>
       </x:c>
       <x:c r="Q46" s="3" t="str">
         <x:v>Intranet BFF, NotificationService</x:v>
@@ -8278,10 +8278,10 @@
         <x:v>Notification templates and user notification preferences</x:v>
       </x:c>
       <x:c r="S46" s="3" t="str">
-        <x:v>Needs template create/update/delete browser pass.</x:v>
+        <x:v>No remaining INT-045 controller/client/source contract gap from this focused retest. Template create/update/delete browser interaction still belongs in the later authenticated browser pass.</x:v>
       </x:c>
       <x:c r="T46" s="3" t="str">
-        <x:v>NotificationController.cs:15-102; AdminPage.razor:91-165; CustomerDetail.razor:1356-1450</x:v>
+        <x:v>NotificationController.cs:23-104; NotificationServiceClient.cs:23-147,188-260; NotificationControllerTests.cs:13-143; NotificationServiceClientTests.cs:14-220; AdminPage.razor:96-166; Profile.razor:42-588; ModuleRegressionSourceTests.cs:531-544,1713-1755; HrProfilePageTests.cs:17-220</x:v>
       </x:c>
       <x:c r="U46" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf8d0a7674e2e43f0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1057d98a9394b23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7e0ce4485ab4123"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1f5306fffd14a02"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-001 shell navigation retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0987011c32f1450d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rdcbf1fd7a7b9495c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd57a51a0a93e4669"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R8cabf5f561354a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3b0504d850414380"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rd7c3f8a3bca64615"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R1f254115860f4803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R8df1e79fe7664fcb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61354ec81d3749b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b7c2f7a982e4999"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5382,16 +5382,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused shell/navigation component tests passed 2026-06-23; standalone Testing-mode BFF reported startup before local RabbitMQ warnings.</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>No shell/navigation behavior error observed in focused component/source retest. Headless browser smoke was blocked by local Playwright package resolution: installed playwright package imports missing playwright-core.</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>No app-code fix needed for this INT-001 retest; browser tooling blocker is external to Intranet source.</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested Phase2NavLayoutTests/MainLayoutTests/ThemeToggleSourceTests 23/23 passed.</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
         <x:v>P0</x:v>
@@ -5409,7 +5409,7 @@
         <x:v>AuthController user/session endpoints</x:v>
       </x:c>
       <x:c r="P2" s="3" t="str">
-        <x:v>Navigation/source tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~Phase2NavLayoutTests|FullyQualifiedName~MainLayoutTests|FullyQualifiedName~ThemeToggleSourceTests" --verbosity minimal passed 23/23 on 2026-06-23. Standalone BFF startup command with ASPNETCORE_ENVIRONMENT=Testing and ASPNETCORE_URLS=http://localhost:5071 reported Intranet BFF started successfully; shutdown logs also showed local RabbitMQ unavailable. Attempted Playwright desktop/mobile smoke was blocked before navigation by ERR_MODULE_NOT_FOUND for playwright-core.</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="str">
         <x:v>Intranet client, BFF, Auth/IAM</x:v>
@@ -5418,10 +5418,10 @@
         <x:v>User preferences/session state</x:v>
       </x:c>
       <x:c r="S2" s="3" t="str">
-        <x:v>Needs responsive shell browser pass</x:v>
+        <x:v>Responsive shell component/source behavior is covered by the current focused retest; full rendered browser screenshot evidence still requires repairing the local Playwright runtime or using a configured browser runner, and live standalone smoke still needs local RabbitMQ/Aspire infrastructure available.</x:v>
       </x:c>
       <x:c r="T2" s="3" t="str">
-        <x:v>AppNavigation.cs; NavMenu.razor; TopBar.razor</x:v>
+        <x:v>TopBar.razor:115-156,305-310,484-490,530; TopBar.razor.css:687-935; AppNavigation.cs:18-104; Phase2NavLayoutTests.cs:109-137,163-194,253-276; MainLayoutTests.cs:63-69; ThemeToggleSourceTests.cs:6-55</x:v>
       </x:c>
       <x:c r="U2" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1057d98a9394b23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb57dca0ab2f45a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd1f5306fffd14a02"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R354e8e6e277e4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh feature tracker workbook artifact
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3b0504d850414380"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rd7c3f8a3bca64615"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R1f254115860f4803"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R8df1e79fe7664fcb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb6fc6c8bfb99476b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rb83d2d6607d345a8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R16d412a382074968"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R216536481a894d90"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b7c2f7a982e4999"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c367ffb476b4e67"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb57dca0ab2f45a9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc131708e54ad4107"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R354e8e6e277e4583"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b78f06268044bcc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-006 permission matrix retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb6fc6c8bfb99476b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rb83d2d6607d345a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R16d412a382074968"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R216536481a894d90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R66855b0ecae24a40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R98dfe06d765a414b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R88ea119d2ac447d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Re1595efd25b44183"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c367ffb476b4e67"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14ed8f2df863468d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5707,16 +5707,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G7" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused project permission-matrix tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H7" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>No permission-matrix behavior error observed in current focused retest.</x:v>
       </x:c>
       <x:c r="I7" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>Added missing ProjectsController permission-matrix regression coverage.</x:v>
       </x:c>
       <x:c r="J7" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested ProjectsControllerTests 36/36 passed.</x:v>
       </x:c>
       <x:c r="K7" s="3" t="str">
         <x:v>P0</x:v>
@@ -5734,7 +5734,7 @@
         <x:v>ProjectsController GET/list/detail/update/delete/notes/duplicate/thumbnail</x:v>
       </x:c>
       <x:c r="P7" s="3" t="str">
-        <x:v>ProjectsControllerTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~ProjectsControllerTests" --verbosity minimal passed 36/36 on 2026-06-23. Added ProjectEndpoints_RequireExpectedPermissionMatrix to assert class-level Project.Read for list/detail/read helpers, Project.Write for project mutations, and existing Job.Write planning-hold coverage.</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="str">
         <x:v>Intranet BFF, Project/Quote services, Storage</x:v>
@@ -5743,10 +5743,10 @@
         <x:v>Projects, notes, duplicate records</x:v>
       </x:c>
       <x:c r="S7" s="3" t="str">
-        <x:v>Needs permission matrix retest</x:v>
+        <x:v>No remaining permission-matrix gap for current project list/detail BFF behavior.</x:v>
       </x:c>
       <x:c r="T7" s="3" t="str">
-        <x:v>ProjectsController.cs:28-298</x:v>
+        <x:v>Maliev.Intranet.Bff/Controllers/ProjectsController.cs; Maliev.Intranet.Tests/Bff/Controllers/ProjectsControllerTests.cs</x:v>
       </x:c>
       <x:c r="U7" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc131708e54ad4107"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25573e2cf3c04476"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b78f06268044bcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra867c3a2e8494c6b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-007 upload bridge retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R66855b0ecae24a40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R98dfe06d765a414b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R88ea119d2ac447d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Re1595efd25b44183"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rbc631e8447e840e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re1d4f73f4c2a4be1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R7aed7cddb47c41bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R76d22baa88ab4bfc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14ed8f2df863468d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7081c89896904048"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5772,16 +5772,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G8" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused Project New upload bridge and resumable-upload tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H8" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>No upload bridge or resumable endpoint behavior error observed in current focused retest.</x:v>
       </x:c>
       <x:c r="I8" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>Added missing regression assertions for the hidden MudFileUpload bridge and Project New dropzone JS contract.</x:v>
       </x:c>
       <x:c r="J8" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested Project New upload focused set 22/22 passed.</x:v>
       </x:c>
       <x:c r="K8" s="3" t="str">
         <x:v>P0</x:v>
@@ -5799,7 +5799,7 @@
         <x:v>UploadsController upload/batch/resumable/complete/chunk/status/viewer-url/preview-url/migrate-project</x:v>
       </x:c>
       <x:c r="P8" s="3" t="str">
-        <x:v>ProjectNewAutoSaveTests; UploadsControllerResumableTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~ModuleRegressionSourceTests.ProjectNew_DropzonesRelayDroppedFilesWithoutOpeningPicker|FullyQualifiedName~ProjectNewAutoSaveTests.HandleFileSelectedAsync|FullyQualifiedName~UploadsControllerResumableTests" --verbosity minimal passed 22/22 on 2026-06-23. Coverage asserts hidden MudFileUpload wiring, dropzone JS init/capture/change relay, upload concurrency, and BFF resumable upload contracts.</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="str">
         <x:v>Intranet BFF, Storage, GeometryService, UploadService</x:v>
@@ -5808,10 +5808,10 @@
         <x:v>Project files, upload sessions, migrated files</x:v>
       </x:c>
       <x:c r="S8" s="3" t="str">
-        <x:v>Needs hidden-input browser journey retest</x:v>
+        <x:v>No remaining hidden-input upload bridge gap for current Project New source and BFF behavior; live browser screenshot evidence remains covered under INT-001 environment blocker.</x:v>
       </x:c>
       <x:c r="T8" s="3" t="str">
-        <x:v>ProjectNew.razor:1; UploadsController.cs:22-617</x:v>
+        <x:v>ProjectNew.razor; ProjectNew.razor.cs; uploadWithProgress.js; ModuleRegressionSourceTests.cs; ProjectNewAutoSaveTests.cs; UploadsControllerResumableTests.cs</x:v>
       </x:c>
       <x:c r="U8" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25573e2cf3c04476"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ae591b3e2d40e6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra867c3a2e8494c6b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc876f1c4ec461c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-008 autosave recovery retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rbc631e8447e840e3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re1d4f73f4c2a4be1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R7aed7cddb47c41bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R76d22baa88ab4bfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcfc7a299fbf94352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rde17c232b02b4c75"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R0bbd6d2206d74769"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf8ecdd19cf5d4d82"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7081c89896904048"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb239312d1804ccd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5837,16 +5837,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G9" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused Project New autosave/resume recovery tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H9" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>No recovery-path behavior error observed in current focused retest.</x:v>
       </x:c>
       <x:c r="I9" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>Added missing sessionStorage draft recovery regression coverage.</x:v>
       </x:c>
       <x:c r="J9" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested autosave/resume focused set 11/11 passed.</x:v>
       </x:c>
       <x:c r="K9" s="3" t="str">
         <x:v>P0</x:v>
@@ -5864,7 +5864,7 @@
         <x:v>ProjectsController POST/PUT project endpoints</x:v>
       </x:c>
       <x:c r="P9" s="3" t="str">
-        <x:v>ProjectNewAutoSaveTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~ProjectNewAutoSaveTests.ProjectNew_WithSessionDraftInStorage_RestoresRecoverableWorkspaceState|FullyQualifiedName~ProjectNewAutoSaveTests.ResumeFromServerAsync|FullyQualifiedName~ProjectNewAutoSaveTests.MigrateTempProjectFilesAsync|FullyQualifiedName~ProjectNewAutoSaveTests.SaveDraftToServerAsync" --verbosity minimal passed 11/11 on 2026-06-23. Coverage includes sessionStorage draft recovery, explicit server resume, non-resumable status skip, 404 tolerance, temp-file migration recovery, and server draft save behavior.</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="str">
         <x:v>Intranet client/BFF, Project service</x:v>
@@ -5873,10 +5873,10 @@
         <x:v>Draft/project state</x:v>
       </x:c>
       <x:c r="S9" s="3" t="str">
-        <x:v>Needs recovery-path browser pass</x:v>
+        <x:v>No remaining autosave/resume recovery-path gap for current Project New component and BFF behavior; live browser screenshot evidence remains covered under INT-001 environment blocker.</x:v>
       </x:c>
       <x:c r="T9" s="3" t="str">
-        <x:v>ProjectNew.razor.cs autosave/resume methods</x:v>
+        <x:v>ProjectNew.razor.cs; ProjectDraftDtos.cs; ProjectNewAutoSaveTests.cs</x:v>
       </x:c>
       <x:c r="U9" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90ae591b3e2d40e6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e03245e825d45b2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc876f1c4ec461c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R919177406300435b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-009 part configuration retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcfc7a299fbf94352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rde17c232b02b4c75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R0bbd6d2206d74769"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf8ecdd19cf5d4d82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3b9d18b2114441ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re108d2dafc7a48e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd40eee41774d417e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R136926c90088422e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcb239312d1804ccd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72449c49464a4d1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5902,16 +5902,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G10" s="3" t="str">
-        <x:v>Failed current Intranet suite, fixed, and retested passed 2026-06-23</x:v>
+        <x:v>Focused part configuration tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H10" s="3" t="str">
-        <x:v>Initial full Intranet suite failed 1/1150: shipping text/numeric fields in PartConfigSidebar and QuoteSummaryBar updated on blur instead of on input.</x:v>
+        <x:v>No current logistical or UX error found in focused automated coverage.</x:v>
       </x:c>
       <x:c r="I10" s="3" t="str">
-        <x:v>Fixed in Maliev.Intranet commit bb9a51c by adding Immediate="true" to the reported shipping text/numeric fields.</x:v>
+        <x:v>No code fix required in this slice; current implementation already covers process-specific configurator behavior.</x:v>
       </x:c>
       <x:c r="J10" s="3" t="str">
-        <x:v>Retested: regression 1/1 passed, impacted focused set 138/138 passed, full Intranet suite 1143 passed / 7 skipped / 0 failed.</x:v>
+        <x:v>Retested PartConfigSidebar 55/55 passed and Project New autosave/bulk configuration 71/71 passed.</x:v>
       </x:c>
       <x:c r="K10" s="3" t="str">
         <x:v>P0</x:v>
@@ -5929,7 +5929,7 @@
         <x:v>ProjectsController parts create/update/delete; ManufacturingCatalogController processes/materials/finishes/tolerances/config-options</x:v>
       </x:c>
       <x:c r="P10" s="3" t="str">
-        <x:v>PartConfigSidebarTests; ProjectNewAutoSaveTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur. | Fix verification: ClientTextInputs_UpdateOnInputInsteadOfBlur passed 1/1; PartConfigSidebar/QuoteSummaryBar/ModuleRegressionSourceTests focused set passed 138/138.</x:v>
+        <x:v>Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~PartConfigSidebar" --verbosity minimal passed 55/55 on 2026-06-23. Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~ProjectNewAutoSaveTests|FullyQualifiedName~ProjectPartBulkEditTests|FullyQualifiedName~ProjectPartsBulkTableTests" --verbosity minimal passed 71/71 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="str">
         <x:v>Intranet BFF, MaterialService, PricingService</x:v>
@@ -5938,10 +5938,10 @@
         <x:v>Project part configuration</x:v>
       </x:c>
       <x:c r="S10" s="3" t="str">
-        <x:v>Needs process-specific UX browser pass</x:v>
+        <x:v>No remaining process-specific part configuration gap found in current focused automated coverage; live rendered browser screenshot remains optional Tier 3 evidence, not a current blocker.</x:v>
       </x:c>
       <x:c r="T10" s="3" t="str">
-        <x:v>ProjectsController.cs:298-365; ManufacturingCatalogController.cs:17-107; PartConfigSidebar.razor:1129-1139; QuoteSummaryBar.razor:144-154</x:v>
+        <x:v>Maliev.Intranet.Client/Components/Project/PartConfigSidebar.razor; Maliev.Intranet.Client/Components/Project/PartConfigSidebar.razor.cs; Maliev.Intranet.Client/Pages/ProjectNew.razor.cs; Maliev.Intranet.Tests/Client/Components/PartConfigSidebarRenderTests.cs; Maliev.Intranet.Tests/Client/Components/PartConfigSidebarTests.cs; Maliev.Intranet.Tests/Client/Pages/ProjectNewAutoSaveTests.cs; Maliev.Intranet.Tests/Client/Components/ProjectPartBulkEditTests.cs; Maliev.Intranet.Tests/Client/Components/ProjectPartsBulkTableTests.cs</x:v>
       </x:c>
       <x:c r="U10" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6e03245e825d45b2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdb339d786ca4561"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R919177406300435b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd024b3445b9847e0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-010 geometry DFM retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3b9d18b2114441ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re108d2dafc7a48e9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rd40eee41774d417e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R136926c90088422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R37b225359a114062"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3b675d5860c14008"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rb1e540cd06b04b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R5727967abfcc4e63"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72449c49464a4d1a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04fda4acb0664579"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5967,16 +5967,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G11" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused geometry runtime and DFM tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H11" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>No current logistical or UX error found in focused automated coverage.</x:v>
       </x:c>
       <x:c r="I11" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>No code fix required in this slice; current implementation already covers DFM hydration, local runtime state, BFF geometry endpoints, and local overlay/thumbnail behavior.</x:v>
       </x:c>
       <x:c r="J11" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested geometry/DFM .NET focus set 125/125 passed and viewer runtime JS focus set 16/16 passed.</x:v>
       </x:c>
       <x:c r="K11" s="3" t="str">
         <x:v>P0</x:v>
@@ -5994,7 +5994,7 @@
         <x:v>GeometryController manifest/assets/telemetry/dfm</x:v>
       </x:c>
       <x:c r="P11" s="3" t="str">
-        <x:v>GeometryControllerTests; Dfm* tests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~GeometryControllerTests|FullyQualifiedName~BrowserDfmReportSyncTests|FullyQualifiedName~BrowserDfmRaceSourceTests|FullyQualifiedName~DfmOverlayPanel|FullyQualifiedName~PartDetailCardLocalDfmTests|FullyQualifiedName~PartViewModelViewerSettingsTests|FullyQualifiedName~ProjectNewAutoSaveTests.HandleLocalGeometryRuntime|FullyQualifiedName~UploadAnalysisStatusTests|FullyQualifiedName~DfmAnalysisReadyConsumerTests|FullyQualifiedName~ModelViewerRenderingSourceTests|FullyQualifiedName~GeometryInteropSourceTests" --verbosity minimal passed 125/125 on 2026-06-23. Focused viewer runtime: node --test Maliev.Intranet.Tests/Viewer/geometry-interop.test.mjs Maliev.Intranet.Tests/Viewer/part-viewer-local-dfm-overlay.test.mjs passed 16/16 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="str">
         <x:v>Intranet BFF, GeometryService, browser runtime</x:v>
@@ -6003,10 +6003,10 @@
         <x:v>Telemetry and DFM report state</x:v>
       </x:c>
       <x:c r="S11" s="3" t="str">
-        <x:v>Needs model-render browser pass</x:v>
+        <x:v>No remaining geometry runtime or DFM gap found in current focused automated coverage; live rendered browser screenshot remains optional Tier 3 evidence, not a current blocker.</x:v>
       </x:c>
       <x:c r="T11" s="3" t="str">
-        <x:v>GeometryController.cs:20,42,77,168,311</x:v>
+        <x:v>Maliev.Intranet.Bff/Controllers/GeometryController.cs; Maliev.Intranet.Client/Pages/ProjectNew.razor.cs; Maliev.Intranet.Client/Components/Project/BrowserDfmReportSync.cs; Maliev.Intranet.Client/Components/Project/PartDetailCard.razor; Maliev.Intranet.Client/wwwroot/js/geometry/JsInterop/GeometryInterop.js; Maliev.Intranet.Client/wwwroot/js/part-viewer.js; Maliev.Intranet.Tests/Bff/Controllers/GeometryControllerTests.cs; Maliev.Intranet.Tests/Client/Components/BrowserDfmReportSyncTests.cs; Maliev.Intranet.Tests/Client/Components/PartDetailCardLocalDfmTests.cs; Maliev.Intranet.Tests/Viewer/geometry-interop.test.mjs; Maliev.Intranet.Tests/Viewer/part-viewer-local-dfm-overlay.test.mjs</x:v>
       </x:c>
       <x:c r="U11" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbdb339d786ca4561"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e748ffc54e749eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd024b3445b9847e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raee72a00b6d84fba"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-011 pricing retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R37b225359a114062"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3b675d5860c14008"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rb1e540cd06b04b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R5727967abfcc4e63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R140d2908de4d47a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R30649ab238b34bf2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5f9648d2de104631"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rbe090ef7d1294b6e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04fda4acb0664579"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R831aca0a3ffd4bb5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6032,16 +6032,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G12" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused pricing snapshot/calculation tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H12" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>No current logistical or UX error found in focused automated coverage.</x:v>
       </x:c>
       <x:c r="I12" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>No code fix required in this slice; current implementation covers pricing calculation, finish surcharge, bulk/lead-time presentation, quote-summary totals, and price confirmation.</x:v>
       </x:c>
       <x:c r="J12" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested focused pricing set 23/23 passed.</x:v>
       </x:c>
       <x:c r="K12" s="3" t="str">
         <x:v>P0</x:v>
@@ -6059,7 +6059,7 @@
         <x:v>PricingController snapshots/calculate/accept/lead-times/bulk/finish-options</x:v>
       </x:c>
       <x:c r="P12" s="3" t="str">
-        <x:v>PricingControllerTests; QuoteSummaryBarTests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~PricingControllerTests|FullyQualifiedName~QuoteSummaryBarTests|FullyQualifiedName~ProjectQuotationPdfMapperTests|FullyQualifiedName~ProjectNewAutoSaveTests.CreateProjectAndQuoteAsync_WhenPartsHavePrices|FullyQualifiedName~ProjectNewAutoSaveTests.RefreshLeadTimeOptionsFromPricing|FullyQualifiedName~ProjectsControllerTests.GetPartPrice|FullyQualifiedName~ProjectsControllerTests.ConfirmPartPrice|FullyQualifiedName~ProjectPartsBulkTableTests.ProjectPartsBulkTable_WhenPricingLoading|FullyQualifiedName~PartConfigSidebarRenderTests.SurfaceFinishCards_ReservePriceAndCheckmarkColumns" --verbosity minimal passed 23/23 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="str">
         <x:v>Intranet BFF, PricingService, MaterialService</x:v>
@@ -6068,10 +6068,10 @@
         <x:v>Pricing snapshots and part pricing</x:v>
       </x:c>
       <x:c r="S12" s="3" t="str">
-        <x:v>Needs current price-rule acceptance tests</x:v>
+        <x:v>No remaining pricing calculation gap found in current focused automated coverage; live rendered browser screenshot remains optional Tier 3 evidence, not a current blocker.</x:v>
       </x:c>
       <x:c r="T12" s="3" t="str">
-        <x:v>PricingController.cs:15-137</x:v>
+        <x:v>Maliev.Intranet.Bff/Controllers/PricingController.cs; Maliev.Intranet.Client/Pages/ProjectNew.razor.cs; Maliev.Intranet.Client/Components/Project/QuoteSummaryBar.razor; Maliev.Intranet.Client/Components/Project/BulkPricingTable.razor; Maliev.Intranet.Tests/Bff/Controllers/PricingControllerTests.cs; Maliev.Intranet.Tests/Bff/Controllers/ProjectsControllerTests.cs; Maliev.Intranet.Tests/Client/Components/QuoteSummaryBarTests.cs; Maliev.Intranet.Tests/Client/Pages/ProjectQuotationPdfMapperTests.cs; Maliev.Intranet.Tests/Client/Pages/ProjectNewAutoSaveTests.cs</x:v>
       </x:c>
       <x:c r="U12" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e748ffc54e749eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R925b7d4a81284beb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raee72a00b6d84fba"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14991cbe1e2b4f55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-012 quotation PDF retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R140d2908de4d47a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R30649ab238b34bf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5f9648d2de104631"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rbe090ef7d1294b6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3cb21f7ba85349fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R9739f95e5a984b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Re8509f45fea34616"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rdd03522bf8c44f6e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R831aca0a3ffd4bb5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2ddb5996968465c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6097,16 +6097,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G13" s="3" t="str">
-        <x:v>Failed current Intranet suite, fixed, and retested passed 2026-06-23</x:v>
+        <x:v>Focused quotation generation and PDF contract tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H13" s="3" t="str">
-        <x:v>Initial full Intranet suite failed 1/1150: shipping text/numeric fields in PartConfigSidebar and QuoteSummaryBar updated on blur instead of on input.</x:v>
+        <x:v>No current logistical or UX error found in focused automated coverage.</x:v>
       </x:c>
       <x:c r="I13" s="3" t="str">
-        <x:v>Fixed in Maliev.Intranet commit bb9a51c by adding Immediate="true" to the reported shipping text/numeric fields.</x:v>
+        <x:v>No code fix required in this slice; current implementation covers quote summary actions, draft PDF data mapping, quotation generation request shape, part price confirmation, PDF metadata, and BFF artifact URL repair.</x:v>
       </x:c>
       <x:c r="J13" s="3" t="str">
-        <x:v>Retested: regression 1/1 passed, impacted focused set 138/138 passed, full Intranet suite 1143 passed / 7 skipped / 0 failed.</x:v>
+        <x:v>Retested focused quotation/PDF set 29/29 passed.</x:v>
       </x:c>
       <x:c r="K13" s="3" t="str">
         <x:v>P0</x:v>
@@ -6124,7 +6124,7 @@
         <x:v>QuotationsController; ProjectsController generate-quotation/accept-quotation</x:v>
       </x:c>
       <x:c r="P13" s="3" t="str">
-        <x:v>ProjectsControllerTests; quotation/PDF tests | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur. | Fix verification: ClientTextInputs_UpdateOnInputInsteadOfBlur passed 1/1; PartConfigSidebar/QuoteSummaryBar/ModuleRegressionSourceTests focused set passed 138/138.</x:v>
+        <x:v>Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~ProjectQuotationPdfMapperTests|FullyQualifiedName~ProjectQuotationPdfDataFactoryTests|FullyQualifiedName~QuotationPdfMetadataApplicatorTests|FullyQualifiedName~QuickControllerTests.Quotations_|FullyQualifiedName~ProjectServiceClientCreateTests.GenerateQuotationAsync|FullyQualifiedName~ProjectNewAutoSaveTests.CreateProjectAndQuoteAsync|FullyQualifiedName~ProjectsControllerTests.GenerateQuotation|FullyQualifiedName~ProjectsControllerTests.AcceptQuotation|FullyQualifiedName~QuoteSummaryBarTests" --verbosity minimal passed 29/29 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="str">
         <x:v>Intranet BFF, QuotationService, PdfService, Storage</x:v>
@@ -6133,10 +6133,10 @@
         <x:v>Quotation records, PDFs, notes/status</x:v>
       </x:c>
       <x:c r="S13" s="3" t="str">
-        <x:v>Needs PDF visual regression pass</x:v>
+        <x:v>No remaining quotation generation or PDF contract gap found in current focused automated coverage; live rendered PDF visual regression remains optional Tier 3 evidence, not a current blocker.</x:v>
       </x:c>
       <x:c r="T13" s="3" t="str">
-        <x:v>QuotationsController.cs:20-346; ProjectsController.cs:383,513; PartConfigSidebar.razor:1129-1139; QuoteSummaryBar.razor:144-154</x:v>
+        <x:v>Maliev.Intranet.Client/Pages/ProjectNew.razor.cs; Maliev.Intranet.Client/Components/Project/QuoteSummaryBar.razor; Maliev.Intranet.Bff/Controllers/QuotationsController.cs; Maliev.Intranet.Bff/Clients/PdfServiceClient.cs; Maliev.Intranet.Bff/Clients/ProjectServiceClient.cs; Maliev.Intranet.Tests/Client/Pages/ProjectQuotationPdfMapperTests.cs; Maliev.Intranet.Tests/Bff/ProjectQuotationPdfDataFactoryTests.cs; Maliev.Intranet.Tests/Bff/QuotationPdfMetadataApplicatorTests.cs; Maliev.Intranet.Tests/Bff/Controllers/QuickControllerTests.cs; Maliev.Intranet.Tests/Client/Pages/ProjectNewAutoSaveTests.cs</x:v>
       </x:c>
       <x:c r="U13" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R925b7d4a81284beb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a249b5d6b4b46c7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R14991cbe1e2b4f55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R047ef05f8147430b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-033 IAM permission retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3cb21f7ba85349fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R9739f95e5a984b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Re8509f45fea34616"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rdd03522bf8c44f6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1bd99f675fd34ec3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Ra2c7ee2822d14762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R84a297cc1c354b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rccd7084944534353"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2ddb5996968465c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e5baecf4ccc4632"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7462,16 +7462,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G34" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused IAM user/role/permission tests passed 2026-06-23.</x:v>
       </x:c>
       <x:c r="H34" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>No current logistical or UX error found in focused automated coverage.</x:v>
       </x:c>
       <x:c r="I34" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>No code fix required in this slice; current implementation covers IAM client mapping, permission authorization, user context, role/permission paging/search, and selected controller permission matrices.</x:v>
       </x:c>
       <x:c r="J34" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested focused IAM/permission set 46/46 passed.</x:v>
       </x:c>
       <x:c r="K34" s="3" t="str">
         <x:v>P0</x:v>
@@ -7489,7 +7489,7 @@
         <x:v>IamController users/roles/permissions/bindings/invite/activity/matrix; PermissionsController</x:v>
       </x:c>
       <x:c r="P34" s="3" t="str">
-        <x:v>IAM tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~IAMServiceClientTests|FullyQualifiedName~PermissionAuthorizationTests|FullyQualifiedName~UserContextHandlerTests|FullyQualifiedName~AuthControllerTests|FullyQualifiedName~QuickControllerTests.Iam_|FullyQualifiedName~QuickControllerTests.Diagnostics|FullyQualifiedName~ModuleRegressionSourceTests.AdminPage|FullyQualifiedName~ModuleRegressionSourceTests.ClientLoginRoute|FullyQualifiedName~ReferenceDataControllerTests.ReferenceDataManagementEndpoints_RequireExpectedPermissions|FullyQualifiedName~ProjectsControllerTests.ProjectEndpoints_RequireExpectedPermissionMatrix" --verbosity minimal passed 46/46 on 2026-06-23.</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="str">
         <x:v>Intranet BFF, IAMService</x:v>
@@ -7498,10 +7498,10 @@
         <x:v>Users, roles, permissions, bindings</x:v>
       </x:c>
       <x:c r="S34" s="3" t="str">
-        <x:v>Needs permission matrix and audit validation</x:v>
+        <x:v>No remaining IAM user/role/permission gap found in current focused automated coverage; live rendered admin/IAM browser pass remains optional Tier 3 evidence, not a current blocker.</x:v>
       </x:c>
       <x:c r="T34" s="3" t="str">
-        <x:v>IamController.cs:21-321; PermissionsController.cs:17-59; IAM pages</x:v>
+        <x:v>Maliev.Intranet.Bff/Controllers/IamController.cs; Maliev.Intranet.Bff/Controllers/AuthController.cs; Maliev.Intranet.Bff/Clients/IAMServiceClient.cs; Maliev.Intranet.Shared/Dtos/IdentityDtos.cs; Maliev.Intranet.Client/Authorization; Maliev.Intranet.Client/Pages/Admin; Maliev.Intranet.Tests/Bff/Clients/IAMServiceClientTests.cs; Maliev.Intranet.Tests/Client/Authorization/PermissionAuthorizationTests.cs; Maliev.Intranet.Tests/Bff/UserContextHandlerTests.cs; Maliev.Intranet.Tests/Bff/Controllers/AuthControllerTests.cs; Maliev.Intranet.Tests/Bff/Controllers/QuickControllerTests.cs</x:v>
       </x:c>
       <x:c r="U34" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a249b5d6b4b46c7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c21ff4b1bfc4419"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R047ef05f8147430b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4d18f7b12d94c70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-042 auth guard retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R1bd99f675fd34ec3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Ra2c7ee2822d14762"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R84a297cc1c354b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rccd7084944534353"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2e43b7a18f5c4f10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R56046f49575d4ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5caa2a2c73584f05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Re60ac9e72a9448e1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7e5baecf4ccc4632"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R282053ddbdb74409"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8047,16 +8047,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G43" s="3" t="str">
-        <x:v>Automated Intranet suite passed 2026-06-23 after UX fix</x:v>
+        <x:v>Focused INT-042 auth/login/user/avatar tests passed 2026-06-23 after auth-guard UX fix.</x:v>
       </x:c>
       <x:c r="H43" s="3" t="str">
-        <x:v>No behavior error observed in current Intranet automated retest.</x:v>
+        <x:v>Found and fixed a current auth-guard UX error: unauthenticated deep links sent an absolute Navigation.Uri as returnUrl, which the BFF login page normalized to / instead of returning users to the requested route after sign-in.</x:v>
       </x:c>
       <x:c r="I43" s="3" t="str">
-        <x:v>No fix needed for this story from current Intranet automated retest.</x:v>
+        <x:v>Fixed in Maliev.Intranet commit c9a045a by deriving RedirectToLogin returnUrl from Navigation.ToBaseRelativePath and preserving local path, query, and fragment before redirecting to /login.</x:v>
       </x:c>
       <x:c r="J43" s="3" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested focused INT-042 set 31/31 passed; dotnet build Maliev.Intranet.slnx passed with 0 warnings and 0 errors.</x:v>
       </x:c>
       <x:c r="K43" s="3" t="str">
         <x:v>P0</x:v>
@@ -8074,7 +8074,7 @@
         <x:v>AuthController endpoints; LoginPageController login page GET/POST/form</x:v>
       </x:c>
       <x:c r="P43" s="3" t="str">
-        <x:v>Auth/login tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:v>
+        <x:v>dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~AuthControllerTests|FullyQualifiedName~LoginPageControllerTests|FullyQualifiedName~UserContextHandlerTests|FullyQualifiedName~PermissionAuthorizationTests|FullyQualifiedName~MainLayoutTests|FullyQualifiedName~RedirectToLoginTests|FullyQualifiedName~HrProfilePageTests|FullyQualifiedName~EmployeesControllerProfileTests" --verbosity minimal =&gt; Passed 31/31. dotnet build Maliev.Intranet.slnx --verbosity minimal =&gt; Build succeeded, 0 warnings, 0 errors.</x:v>
       </x:c>
       <x:c r="Q43" s="3" t="str">
         <x:v>Intranet BFF, Auth/IAM</x:v>
@@ -8083,10 +8083,10 @@
         <x:v>Auth session/cookies</x:v>
       </x:c>
       <x:c r="S43" s="3" t="str">
-        <x:v>Needs auth guard browser pass</x:v>
+        <x:v>No remaining auth login/logout/user/avatar gap found in current focused automated coverage.</x:v>
       </x:c>
       <x:c r="T43" s="3" t="str">
-        <x:v>AuthController.cs:20-319; LoginPageController.cs</x:v>
+        <x:v>Maliev.Intranet.Client/Layout/RedirectToLogin.razor; Maliev.Intranet.Tests/Client/Components/RedirectToLoginTests.cs; Maliev.Intranet.Bff/Controllers/AuthController.cs; Maliev.Intranet.Bff/Controllers/LoginPageController.cs; Maliev.Intranet.Client/PersistentAuthenticationStateProvider.cs; Maliev.Intranet.Client/Layout/TopBar.razor; Maliev.Intranet.Tests/Bff/Controllers/AuthControllerTests.cs; Maliev.Intranet.Tests/Bff/Controllers/LoginPageControllerTests.cs; Maliev.Intranet.Tests/Bff/UserContextHandlerTests.cs; Maliev.Intranet.Tests/Client/Authorization/PermissionAuthorizationTests.cs; Maliev.Intranet.Tests/Client/Components/MainLayoutTests.cs; Maliev.Intranet.Tests/Client/Pages/HrProfilePageTests.cs; Maliev.Intranet.Tests/Bff/Controllers/EmployeesControllerProfileTests.cs</x:v>
       </x:c>
       <x:c r="U43" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8c21ff4b1bfc4419"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf4271f103db4e55"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4d18f7b12d94c70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f78a7f9db448af"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh INT-001 shell navigation evidence
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R2e43b7a18f5c4f10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R56046f49575d4ad1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5caa2a2c73584f05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Re60ac9e72a9448e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R99a6f58f8eb84e47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4ceb8532eca04883"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R6aa4d87451254596"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R93d224781ae14b16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5264,7 +5264,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R282053ddbdb74409"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d3bb2dfef4f47a4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5382,16 +5382,16 @@
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G2" s="3" t="str">
-        <x:v>Focused shell/navigation component tests passed 2026-06-23; standalone Testing-mode BFF reported startup before local RabbitMQ warnings.</x:v>
+        <x:v>Focused shell/navigation tests passed 2026-06-23; browser automation package verified through Node REPL, but no live Intranet listener was available for rendered browser smoke.</x:v>
       </x:c>
       <x:c r="H2" s="3" t="str">
-        <x:v>No shell/navigation behavior error observed in focused component/source retest. Headless browser smoke was blocked by local Playwright package resolution: installed playwright package imports missing playwright-core.</x:v>
+        <x:v>No shell/navigation behavior error observed in current focused retest. Previous ad hoc Node Playwright package-resolution blocker is not the current blocker because Node REPL imports Playwright successfully; current live-browser evidence is blocked by no running Intranet BFF/Aspire route.</x:v>
       </x:c>
       <x:c r="I2" s="3" t="str">
-        <x:v>No app-code fix needed for this INT-001 retest; browser tooling blocker is external to Intranet source.</x:v>
+        <x:v>No app-code fix required in this slice; current shell/navigation source and component coverage passed. Browser validation needs a live Intranet-hosted route, not a source change.</x:v>
       </x:c>
       <x:c r="J2" s="3" t="str">
-        <x:v>Retested Phase2NavLayoutTests/MainLayoutTests/ThemeToggleSourceTests 23/23 passed.</x:v>
+        <x:v>Retested Phase2NavLayoutTests/MainLayoutTests/ThemeToggleSourceTests/ResponsiveLayoutTests/NavigationTests: 23 passed, 2 skipped.</x:v>
       </x:c>
       <x:c r="K2" s="3" t="str">
         <x:v>P0</x:v>
@@ -5409,7 +5409,7 @@
         <x:v>AuthController user/session endpoints</x:v>
       </x:c>
       <x:c r="P2" s="3" t="str">
-        <x:v>Focused test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~Phase2NavLayoutTests|FullyQualifiedName~MainLayoutTests|FullyQualifiedName~ThemeToggleSourceTests" --verbosity minimal passed 23/23 on 2026-06-23. Standalone BFF startup command with ASPNETCORE_ENVIRONMENT=Testing and ASPNETCORE_URLS=http://localhost:5071 reported Intranet BFF started successfully; shutdown logs also showed local RabbitMQ unavailable. Attempted Playwright desktop/mobile smoke was blocked before navigation by ERR_MODULE_NOT_FOUND for playwright-core.</x:v>
+        <x:v>dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~Phase2NavLayoutTests|FullyQualifiedName~MainLayoutTests|FullyQualifiedName~ThemeToggleSourceTests|FullyQualifiedName~ResponsiveLayoutTests|FullyQualifiedName~NavigationTests" --verbosity minimal =&gt; Passed 23/23, skipped 2 browser/server-dependent tests. Node REPL Playwright import probe =&gt; ok with chromium/firefox/webkit exports. Local process/listener probe =&gt; no Maliev.Intranet BFF route listening; only Maliev.Web.Bff was running.</x:v>
       </x:c>
       <x:c r="Q2" s="3" t="str">
         <x:v>Intranet client, BFF, Auth/IAM</x:v>
@@ -5418,10 +5418,10 @@
         <x:v>User preferences/session state</x:v>
       </x:c>
       <x:c r="S2" s="3" t="str">
-        <x:v>Responsive shell component/source behavior is covered by the current focused retest; full rendered browser screenshot evidence still requires repairing the local Playwright runtime or using a configured browser runner, and live standalone smoke still needs local RabbitMQ/Aspire infrastructure available.</x:v>
+        <x:v>No remaining shell/navigation source or component behavior gap found in current focused automated coverage; full rendered browser screenshot evidence still requires a live Intranet BFF/Aspire route.</x:v>
       </x:c>
       <x:c r="T2" s="3" t="str">
-        <x:v>TopBar.razor:115-156,305-310,484-490,530; TopBar.razor.css:687-935; AppNavigation.cs:18-104; Phase2NavLayoutTests.cs:109-137,163-194,253-276; MainLayoutTests.cs:63-69; ThemeToggleSourceTests.cs:6-55</x:v>
+        <x:v>Maliev.Intranet.Client/Layout/MainLayout.razor; Maliev.Intranet.Client/Layout/TopBar.razor; Maliev.Intranet.Client/Layout/NavMenu.razor; Maliev.Intranet.Client/Layout/AppNavigation.cs; Maliev.Intranet.Client/Routes.razor; Maliev.Intranet.Tests/Client/Pages/Phase2NavLayoutTests.cs; Maliev.Intranet.Tests/Client/Components/MainLayoutTests.cs; Maliev.Intranet.Tests/Client/Layout/ThemeToggleSourceTests.cs; Maliev.Intranet.Tests/Client/Components/ResponsiveLayoutTests.cs; Maliev.Intranet.Tests/Client/NavigationTests.cs</x:v>
       </x:c>
       <x:c r="U2" s="3" t="str">
         <x:v>2026-06-23</x:v>
@@ -8680,7 +8680,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf4271f103db4e55"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33d5aa17f8724fcf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11251,7 +11251,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re9f78a7f9db448af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dc9bc2067444455"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-002 readiness retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R99a6f58f8eb84e47"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4ceb8532eca04883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R6aa4d87451254596"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R93d224781ae14b16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R110205978a30482f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R1123a1083e1d4dbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R472fbc52d8f243ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rda01110af06b4d07"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1324,16 +1324,16 @@
     <x:t xml:space="preserve">QuoteWorkspace.razor:1-5,39; QuoteAgentLaunchShell.razor; Program.cs public route fallback; QuoteWorkspace.razor routes; QuoteAgentLaunchShell.razor</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">QE-002</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent health and readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can see whether the quote agent is available before sending work.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent health endpoint and shell status indicators reflect backend readiness and keep composer state aligned.</x:t>
+    <x:t xml:space="preserve">QE-003</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent chat send</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can send manufacturing/quote questions to the agent.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Composer sends messages with session context and receives agent turns through the BFF.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:t>
@@ -1345,163 +1345,130 @@
     <x:t xml:space="preserve">No fix needed for this story from current QuoteEngine automated retest.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Shell status -&gt; quote/v1/agent/health -&gt; readiness state</x:t>
+    <x:t xml:space="preserve">Composer -&gt; AgentController messages -&gt; QuoteAgentService -&gt; session store</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QuoteAgentLaunchShell.razor</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Agent status dot/composer gating</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController GET health</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests health; QuoteEngineSourceTests status dot | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+    <x:t xml:space="preserve">Chat composer and message thread</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController POST messages; QuoteAgentService SendMessageAsync</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests messages | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, Agent model, SessionStore</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Chat messages/session state</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs browser send-path retest</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController.cs:56; QuoteAgentService.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-004</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent streaming</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can receive streamed agent responses.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Streaming endpoint returns structured response chunks and the UI keeps thread/composer layout stable.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Composer -&gt; messages/stream -&gt; streaming agent response</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Streaming response thread</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController POST messages/stream</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests stream events; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, Agent model</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Streamed chat turns</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs interrupted-stream browser test</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController.cs:76</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-005</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent state and history</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a returning customer, I can reload session state and chat history.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">BFF exposes session state and message history by session id with authorization boundaries.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Shell/session restore -&gt; AgentController sessions/messages -&gt; SessionStore</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Session reload/history</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController GET sessions/{sessionId}, sessions/{sessionId}/messages</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests history auth | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, SessionStore, Auth</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Session state and message history</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs authenticated reload browser retest</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController.cs:132,142; QuoteAgentSessionStore.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-006</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent clean speech and thinking</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I get cleaned assistant speech and structured thinking/progress updates.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">BFF exposes clean-speech and thinking endpoints used by the assistant experience.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent UI -&gt; clean-speech/thinking endpoints -&gt; QuoteAgentService</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Thinking/progress and speech cleanup surfaces</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController clean-speech, thinking</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests; QuoteEngineSourceTests thinking | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QuoteEngine BFF, Agent service</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Read-only readiness</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs live Aspire readiness smoke</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:33; QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-003</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent chat send</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can send manufacturing/quote questions to the agent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Composer sends messages with session context and receives agent turns through the BFF.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Composer -&gt; AgentController messages -&gt; QuoteAgentService -&gt; session store</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Chat composer and message thread</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST messages; QuoteAgentService SendMessageAsync</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests messages | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Agent model, SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Chat messages/session state</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs browser send-path retest</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:56; QuoteAgentService.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-004</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent streaming</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can receive streamed agent responses.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Streaming endpoint returns structured response chunks and the UI keeps thread/composer layout stable.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Composer -&gt; messages/stream -&gt; streaming agent response</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Streaming response thread</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST messages/stream</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests stream events; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Agent model</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Streamed chat turns</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs interrupted-stream browser test</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:76</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-005</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent state and history</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a returning customer, I can reload session state and chat history.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BFF exposes session state and message history by session id with authorization boundaries.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shell/session restore -&gt; AgentController sessions/messages -&gt; SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Session reload/history</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController GET sessions/{sessionId}, sessions/{sessionId}/messages</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests history auth | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, SessionStore, Auth</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Session state and message history</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs authenticated reload browser retest</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:132,142; QuoteAgentSessionStore.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-006</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent clean speech and thinking</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I get cleaned assistant speech and structured thinking/progress updates.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BFF exposes clean-speech and thinking endpoints used by the assistant experience.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent UI -&gt; clean-speech/thinking endpoints -&gt; QuoteAgentService</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Thinking/progress and speech cleanup surfaces</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController clean-speech, thinking</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests; QuoteEngineSourceTests thinking | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Cleaned text/thinking state</x:t>
@@ -5264,7 +5231,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d3bb2dfef4f47a4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1519437e94654c14"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8680,7 +8647,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33d5aa17f8724fcf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rea9192063e854650"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8844,85 +8811,85 @@
       </x:c>
     </x:row>
     <x:row r="3" ht="107.25" hidden="0">
-      <x:c r="A3" s="3" t="s">
-        <x:v>437</x:v>
-      </x:c>
-      <x:c r="B3" s="3" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="C3" s="3" t="s">
-        <x:v>438</x:v>
-      </x:c>
-      <x:c r="D3" s="3" t="s">
-        <x:v>439</x:v>
-      </x:c>
-      <x:c r="E3" s="3" t="s">
-        <x:v>440</x:v>
-      </x:c>
-      <x:c r="F3" s="3" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="G3" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="H3" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="I3" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="J3" s="3" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="K3" s="3" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="L3" s="3" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="M3" s="3" t="s">
-        <x:v>445</x:v>
-      </x:c>
-      <x:c r="N3" s="3" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="O3" s="3" t="s">
-        <x:v>447</x:v>
-      </x:c>
-      <x:c r="P3" s="3" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="Q3" s="3" t="s">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="R3" s="3" t="s">
-        <x:v>450</x:v>
-      </x:c>
-      <x:c r="S3" s="3" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="T3" s="3" t="s">
-        <x:v>452</x:v>
-      </x:c>
-      <x:c r="U3" s="3" t="s">
-        <x:v>2</x:v>
+      <x:c r="A3" s="3" t="str">
+        <x:v>QE-002</x:v>
+      </x:c>
+      <x:c r="B3" s="3" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C3" s="3" t="str">
+        <x:v>Agent health and readiness</x:v>
+      </x:c>
+      <x:c r="D3" s="3" t="str">
+        <x:v>As a customer, I can see whether the quote agent is available before sending work.</x:v>
+      </x:c>
+      <x:c r="E3" s="3" t="str">
+        <x:v>Agent health endpoint and shell status indicators reflect backend readiness and keep composer state aligned.</x:v>
+      </x:c>
+      <x:c r="F3" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G3" s="3" t="str">
+        <x:v>Focused QE-002 agent health/readiness tests passed 2026-06-23.</x:v>
+      </x:c>
+      <x:c r="H3" s="3" t="str">
+        <x:v>No current health/readiness behavior error observed in focused automated retest. Live Aspire smoke could not run because no QuoteEngine BFF/Aspire-hosted route was listening in the current environment.</x:v>
+      </x:c>
+      <x:c r="I3" s="3" t="str">
+        <x:v>No code fix required in this slice; current implementation covers /quote/v1/agent/health ready/unavailable responses, client 503 health deserialization, bounded readiness timeout, and shell status polling.</x:v>
+      </x:c>
+      <x:c r="J3" s="3" t="str">
+        <x:v>Retested focused QE-002 set 5/5 passed.</x:v>
+      </x:c>
+      <x:c r="K3" s="3" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L3" s="3" t="str">
+        <x:v>Shell status -&gt; quote/v1/agent/health -&gt; readiness state</x:v>
+      </x:c>
+      <x:c r="M3" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor</x:v>
+      </x:c>
+      <x:c r="N3" s="3" t="str">
+        <x:v>Agent status dot/composer gating</x:v>
+      </x:c>
+      <x:c r="O3" s="3" t="str">
+        <x:v>AgentController GET health</x:v>
+      </x:c>
+      <x:c r="P3" s="3" t="str">
+        <x:v>dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_health_reports_ready_when_chatbot_service_is_available|FullyQualifiedName~QuoteAgentEndpointTests.Agent_health_reports_unavailable_when_chatbot_service_is_offline|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_status_dot_uses_backend_health_not_composer_errors|FullyQualifiedName~QuoteEngineSourceTests.ChatbotServiceClient_ReadinessCheck_DoesNotWarnForExpectedOfflinePolling|FullyQualifiedName~QuoteEngineSourceTests.ChatbotServiceClient_ReadinessCheck_UsesBoundedTimeoutForOfflineServices" --verbosity minimal =&gt; Passed 5/5. Local process/listener probe =&gt; no Maliev.QuoteEngine BFF/Aspire-hosted route listening; live smoke not available in current environment.</x:v>
+      </x:c>
+      <x:c r="Q3" s="3" t="str">
+        <x:v>QuoteEngine BFF, Agent service</x:v>
+      </x:c>
+      <x:c r="R3" s="3" t="str">
+        <x:v>Read-only readiness</x:v>
+      </x:c>
+      <x:c r="S3" s="3" t="str">
+        <x:v>No remaining agent health/readiness source or endpoint behavior gap found in current focused automated coverage; live Aspire readiness smoke still requires a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T3" s="3" t="str">
+        <x:v>Maliev.QuoteEngine.Bff/Controllers/AgentController.cs; Maliev.QuoteEngine.Bff/Clients/ChatbotServiceClient.cs; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs; Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs</x:v>
+      </x:c>
+      <x:c r="U3" s="3" t="str">
+        <x:v>2026-06-23</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="93.25" hidden="0">
       <x:c r="A4" s="3" t="s">
-        <x:v>453</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="B4" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C4" s="3" t="s">
-        <x:v>454</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="D4" s="3" t="s">
-        <x:v>455</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="E4" s="3" t="s">
-        <x:v>456</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
         <x:v>38</x:v>
@@ -8943,31 +8910,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L4" s="3" t="s">
-        <x:v>457</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="M4" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N4" s="3" t="s">
-        <x:v>458</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="O4" s="3" t="s">
-        <x:v>459</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="P4" s="3" t="s">
-        <x:v>460</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="s">
-        <x:v>461</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="R4" s="3" t="s">
-        <x:v>462</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="S4" s="3" t="s">
-        <x:v>463</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="T4" s="3" t="s">
-        <x:v>464</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="U4" s="3" t="s">
         <x:v>2</x:v>
@@ -8975,19 +8942,19 @@
     </x:row>
     <x:row r="5" ht="107.25" hidden="0">
       <x:c r="A5" s="3" t="s">
-        <x:v>465</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>466</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>467</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>468</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
         <x:v>38</x:v>
@@ -9008,31 +8975,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
-        <x:v>469</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="M5" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N5" s="3" t="s">
-        <x:v>470</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="O5" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="P5" s="3" t="s">
-        <x:v>472</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>473</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>474</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="S5" s="3" t="s">
-        <x:v>475</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="T5" s="3" t="s">
-        <x:v>476</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="U5" s="3" t="s">
         <x:v>2</x:v>
@@ -9040,19 +9007,19 @@
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
       <x:c r="A6" s="3" t="s">
-        <x:v>477</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
         <x:v>38</x:v>
@@ -9073,31 +9040,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L6" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="M6" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N6" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="O6" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="P6" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="R6" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="S6" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="T6" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="U6" s="3" t="s">
         <x:v>2</x:v>
@@ -9105,19 +9072,19 @@
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>38</x:v>
@@ -9138,31 +9105,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="M7" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N7" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="O7" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="P7" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="s">
-        <x:v>449</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="R7" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="S7" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="T7" s="3" t="s">
-        <x:v>499</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>2</x:v>
@@ -9170,19 +9137,19 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>500</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>38</x:v>
@@ -9203,31 +9170,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="M8" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N8" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="O8" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="P8" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="R8" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="S8" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="T8" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>2</x:v>
@@ -9235,19 +9202,19 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>38</x:v>
@@ -9268,31 +9235,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="M9" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N9" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="P9" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="s">
-        <x:v>520</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="S9" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="T9" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>2</x:v>
@@ -9300,19 +9267,19 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>525</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>526</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>527</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>38</x:v>
@@ -9333,31 +9300,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
         <x:v>429</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>532</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>534</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>2</x:v>
@@ -9365,19 +9332,19 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>38</x:v>
@@ -9398,31 +9365,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>2</x:v>
@@ -9430,19 +9397,19 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>38</x:v>
@@ -9463,31 +9430,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>2</x:v>
@@ -9495,19 +9462,19 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>561</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>562</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>563</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>38</x:v>
@@ -9528,31 +9495,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>568</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>2</x:v>
@@ -9560,19 +9527,19 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>573</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>574</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>38</x:v>
@@ -9593,31 +9560,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>575</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>580</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>2</x:v>
@@ -9625,19 +9592,19 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>585</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>586</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>587</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>38</x:v>
@@ -9658,31 +9625,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>592</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>593</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>2</x:v>
@@ -9690,19 +9657,19 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>598</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>599</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>38</x:v>
@@ -9723,31 +9690,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>600</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>605</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>606</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>2</x:v>
@@ -9755,19 +9722,19 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>611</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>38</x:v>
@@ -9788,31 +9755,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>612</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>613</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>618</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>2</x:v>
@@ -9820,19 +9787,19 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>624</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>38</x:v>
@@ -9853,31 +9820,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>625</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>626</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>632</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>2</x:v>
@@ -9885,19 +9852,19 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>38</x:v>
@@ -9918,31 +9885,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>2</x:v>
@@ -9950,19 +9917,19 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>38</x:v>
@@ -9983,31 +9950,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>655</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>2</x:v>
@@ -10015,19 +9982,19 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>660</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>661</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>662</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>38</x:v>
@@ -10048,31 +10015,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>667</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>668</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>2</x:v>
@@ -10080,19 +10047,19 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>673</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>674</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>38</x:v>
@@ -10113,31 +10080,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>675</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>680</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>2</x:v>
@@ -10145,19 +10112,19 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>685</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>686</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>38</x:v>
@@ -10178,31 +10145,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>687</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>692</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>2</x:v>
@@ -10210,19 +10177,19 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>697</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>698</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>699</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>38</x:v>
@@ -10243,31 +10210,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>704</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>705</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>2</x:v>
@@ -10275,19 +10242,19 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>710</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>711</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>38</x:v>
@@ -10308,31 +10275,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>712</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>717</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>718</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>2</x:v>
@@ -10340,19 +10307,19 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>38</x:v>
@@ -10373,31 +10340,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>2</x:v>
@@ -10405,19 +10372,19 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>38</x:v>
@@ -10438,31 +10405,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>742</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>743</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>2</x:v>
@@ -10470,19 +10437,19 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>748</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>749</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>38</x:v>
@@ -10503,31 +10470,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>750</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>755</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>756</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>2</x:v>
@@ -10535,19 +10502,19 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>761</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>38</x:v>
@@ -10568,31 +10535,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>762</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>763</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>768</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>769</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>2</x:v>
@@ -10600,19 +10567,19 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>774</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>38</x:v>
@@ -10633,31 +10600,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>775</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>776</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>781</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>2</x:v>
@@ -10665,19 +10632,19 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>787</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>38</x:v>
@@ -10698,31 +10665,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>788</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>789</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>795</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>2</x:v>
@@ -10730,19 +10697,19 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>38</x:v>
@@ -10763,31 +10730,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>802</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>2</x:v>
@@ -10795,19 +10762,19 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>811</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>812</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>813</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>38</x:v>
@@ -10828,31 +10795,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>814</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>815</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>816</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>817</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>818</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>819</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>820</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>821</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>822</x:v>
+        <x:v>811</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>2</x:v>
@@ -10860,7 +10827,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>823</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>9</x:v>
@@ -10869,10 +10836,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>824</x:v>
+        <x:v>813</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>825</x:v>
+        <x:v>814</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>38</x:v>
@@ -10893,31 +10860,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>826</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>827</x:v>
+        <x:v>816</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>828</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>829</x:v>
+        <x:v>818</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>830</x:v>
+        <x:v>819</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>831</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>832</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>833</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>2</x:v>
@@ -10925,19 +10892,19 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>834</x:v>
+        <x:v>823</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>835</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>836</x:v>
+        <x:v>825</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>837</x:v>
+        <x:v>826</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>38</x:v>
@@ -10958,31 +10925,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>838</x:v>
+        <x:v>827</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>839</x:v>
+        <x:v>828</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>840</x:v>
+        <x:v>829</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>841</x:v>
+        <x:v>830</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>842</x:v>
+        <x:v>831</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>843</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>844</x:v>
+        <x:v>833</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>845</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>2</x:v>
@@ -10990,19 +10957,19 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>846</x:v>
+        <x:v>835</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>847</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>848</x:v>
+        <x:v>837</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>849</x:v>
+        <x:v>838</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>38</x:v>
@@ -11023,31 +10990,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>850</x:v>
+        <x:v>839</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>851</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>852</x:v>
+        <x:v>841</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>853</x:v>
+        <x:v>842</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>854</x:v>
+        <x:v>843</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>855</x:v>
+        <x:v>844</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>856</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>857</x:v>
+        <x:v>846</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>2</x:v>
@@ -11055,19 +11022,19 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>858</x:v>
+        <x:v>847</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>859</x:v>
+        <x:v>848</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>860</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>861</x:v>
+        <x:v>850</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>38</x:v>
@@ -11088,31 +11055,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>862</x:v>
+        <x:v>851</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>863</x:v>
+        <x:v>852</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>864</x:v>
+        <x:v>853</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>865</x:v>
+        <x:v>854</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>866</x:v>
+        <x:v>855</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>867</x:v>
+        <x:v>856</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>868</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>869</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>863</x:v>
+        <x:v>852</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>2</x:v>
@@ -11120,19 +11087,19 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>870</x:v>
+        <x:v>859</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>871</x:v>
+        <x:v>860</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>872</x:v>
+        <x:v>861</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>873</x:v>
+        <x:v>862</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>38</x:v>
@@ -11153,31 +11120,31 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>874</x:v>
+        <x:v>863</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>875</x:v>
+        <x:v>864</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>876</x:v>
+        <x:v>865</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>877</x:v>
+        <x:v>866</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>878</x:v>
+        <x:v>867</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>879</x:v>
+        <x:v>868</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>880</x:v>
+        <x:v>869</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>881</x:v>
+        <x:v>870</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>2</x:v>
@@ -11185,19 +11152,19 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>882</x:v>
+        <x:v>871</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>9</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>883</x:v>
+        <x:v>872</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>884</x:v>
+        <x:v>873</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>885</x:v>
+        <x:v>874</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>38</x:v>
@@ -11218,31 +11185,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>886</x:v>
+        <x:v>875</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
         <x:v>445</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>887</x:v>
+        <x:v>876</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>888</x:v>
+        <x:v>877</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>889</x:v>
+        <x:v>878</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>890</x:v>
+        <x:v>879</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>891</x:v>
+        <x:v>880</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>892</x:v>
+        <x:v>881</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>893</x:v>
+        <x:v>882</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>2</x:v>
@@ -11251,7 +11218,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dc9bc2067444455"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72140e8901c4457f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document INT-047 payment operations retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R4da6e20d08b44576"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rc1f5f9c822ca444b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R6e177dedf6854f86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Ra787fd76a00f44d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0eae3cacc47a42cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4b20fe3ecced4f3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rf32457857af84706"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rbb03d25b7eb745dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5204,7 +5204,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb6a1be584a24105"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ceaa025d74948c6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8303,58 +8303,58 @@
         <x:v>Payment operations</x:v>
       </x:c>
       <x:c r="D48" s="3" t="str">
-        <x:v>As a finance employee, I can review payment stats, inspect payment records through the BFF, and record invoice payments from the invoice detail flow.</x:v>
+        <x:v>As finance staff, I can review payment metrics and payment records, and record invoice payments through the current invoice payment workflow.</x:v>
       </x:c>
       <x:c r="E48" s="3" t="str">
-        <x:v>Payment stats load in the invoice list, payment list/detail/create endpoints fail closed when PaymentService does not return data, invoice detail records and allocates payments through InvoiceService, and unsupported direct allocate/void actions return 404.</x:v>
+        <x:v>Payment stats and payment records proxy to PaymentService; invoice payments are recorded through InvoiceService and linked back to the invoice; PaymentService allocate/void actions fail closed because they are not exposed by the downstream service.</x:v>
       </x:c>
       <x:c r="F48" s="3" t="str">
         <x:v>Current code-derived; focused fallback fix applied.</x:v>
       </x:c>
       <x:c r="G48" s="3" t="str">
-        <x:v>Focused behavior tests passed 2026-06-23.</x:v>
+        <x:v>Focused payment and invoice-payment behavior tests passed 2026-06-24.</x:v>
       </x:c>
       <x:c r="H48" s="3" t="str">
-        <x:v>Focused contract review found PaymentServiceClient.GetPaymentsAsync threw on non-success responses instead of allowing the BFF empty-page fallback when PaymentService does not expose a list response.</x:v>
+        <x:v>No current behavior error observed in focused payment retest.</x:v>
       </x:c>
       <x:c r="I48" s="3" t="str">
-        <x:v>Fixed in Maliev.Intranet commit 776400b by changing GetPaymentsAsync to use GetAsync, return null on non-success, and deserialize only successful responses.</x:v>
+        <x:v>No app fix needed; tracker aligned to current PaymentService read/create behavior and InvoiceService-backed invoice payment recording.</x:v>
       </x:c>
       <x:c r="J48" s="3" t="str">
-        <x:v>Retested PaymentsControllerTests 14/14 passed and InvoiceServiceClientTests.RecordInvoicePayment 1/1 passed.</x:v>
+        <x:v>Retested PaymentsControllerTests plus InvoiceServiceClientTests.RecordInvoicePaymentAsync_PostsPaymentAndLinksAllocationToInvoice: 15/15 passed.</x:v>
       </x:c>
       <x:c r="K48" s="3" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="L48" s="3" t="str">
-        <x:v>Finance invoice UI -&gt; Intranet BFF payments/invoices endpoints -&gt; PaymentService metrics/payment endpoints and InvoiceService payment allocation</x:v>
+        <x:v>Intranet BFF payment controller -&gt; PaymentService read/create APIs; invoice detail UI -&gt; InvoicesController payment action -&gt; InvoiceService payment create/link APIs</x:v>
       </x:c>
       <x:c r="M48" s="3" t="str">
-        <x:v>InvoiceList.razor; InvoiceDetail.razor; PaymentsController.cs</x:v>
+        <x:v>InvoiceDetail.razor payment form; InvoiceList.razor payment stats; PaymentsController.cs; InvoicesController.cs</x:v>
       </x:c>
       <x:c r="N48" s="3" t="str">
-        <x:v>/finance/invoices loads api/v1/payments/stats; /finance/invoices/{id} record-payment panel posts api/v1/invoices/{id}/payments</x:v>
+        <x:v>Invoice detail Record Payment form posts api/v1/invoices/{id}/payments; invoice list loads api/v1/payments/stats.</x:v>
       </x:c>
       <x:c r="O48" s="3" t="str">
-        <x:v>PaymentsController stats/list/detail/create proxy PaymentService; list now falls back on non-success; allocate/void return 404 because PaymentService does not expose those actions; invoice payment recording uses InvoiceService /invoice/v1/payments plus /invoice/v1/payments/invoices/{invoiceId}/link.</x:v>
+        <x:v>PaymentServiceClient GET /payment/v1/metrics/stats, GET/POST /payment/v1/payments; InvoiceServiceClient POST /invoice/v1/payments then POST /invoice/v1/payments/invoices/{invoiceId}/link; allocate/void intentionally return 404 when downstream PaymentService does not expose those actions.</x:v>
       </x:c>
       <x:c r="P48" s="3" t="str">
-        <x:v>Focused tests: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~PaymentsControllerTests" --verbosity minimal passed 14/14 on 2026-06-23. Impacted invoice payment allocation test: dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~InvoiceServiceClientTests.RecordInvoicePayment" --verbosity minimal passed 1/1 on 2026-06-23.</x:v>
+        <x:v>dotnet test Maliev.Intranet.slnx --filter "FullyQualifiedName~PaymentsControllerTests|FullyQualifiedName~InvoiceServiceClientTests.RecordInvoicePaymentAsync_PostsPaymentAndLinksAllocationToInvoice" --verbosity minimal passed 15/15 on 2026-06-24.</x:v>
       </x:c>
       <x:c r="Q48" s="3" t="str">
-        <x:v>Intranet BFF, PaymentService, InvoiceService, Accounting/Invoice UI</x:v>
+        <x:v>Intranet BFF, PaymentService, InvoiceService</x:v>
       </x:c>
       <x:c r="R48" s="3" t="str">
-        <x:v>Payment records and invoice payment allocations through InvoiceService; direct PaymentService list/detail reads are read-only.</x:v>
+        <x:v>Payment records and invoice payment allocations</x:v>
       </x:c>
       <x:c r="S48" s="3" t="str">
-        <x:v>Direct PaymentService allocate/void actions are not exposed by current PaymentService and therefore fail closed with 404; current finance UI records invoice payments through InvoiceService instead of a standalone payments page.</x:v>
+        <x:v>No remaining gap from current code-derived tracker.</x:v>
       </x:c>
       <x:c r="T48" s="3" t="str">
-        <x:v>PaymentsController.cs:17-85; PaymentServiceClient.cs:16-80; PaymentsControllerTests.cs:14-216; InvoiceList.razor:587-589; InvoiceDetail.razor:82,209-218; InvoiceServiceClient.cs:140-204</x:v>
+        <x:v>PaymentsController.cs:17-85; PaymentServiceClient.cs:11-80; InvoicesController.cs:168-186; InvoiceServiceClient.cs:140-204; InvoiceList.razor:587-589; InvoiceDetail.razor:66-82,209-238; PaymentsControllerTests.cs:14-217; InvoiceServiceClientTests.cs:316-393</x:v>
       </x:c>
       <x:c r="U48" s="3" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="49" ht="51.29999923706055" hidden="0">
@@ -8620,7 +8620,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6dc305d869c4e5c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c6f739a8d934916"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11191,7 +11191,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2870892c27754be7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ae975070f7d497f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-003 send path retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R0eae3cacc47a42cf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4b20fe3ecced4f3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rf32457857af84706"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rbb03d25b7eb745dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra26f12b8e7fa4d27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R525fec7d9367427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R2b99b88183644f38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rbed96323f16e44bd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1306,7 +1306,22 @@
     <x:t xml:space="preserve">As a customer, I can send manufacturing/quote questions to the agent.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Composer sends messages with session context and receives agent turns through the BFF.</x:t>
+    <x:t xml:space="preserve">QuoteEngine BFF, Agent model, SessionStore</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Chat messages/session state</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-004</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent streaming</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can receive streamed agent responses.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Streaming endpoint returns structured response chunks and the UI keeps thread/composer layout stable.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:t>
@@ -1318,46 +1333,10 @@
     <x:t xml:space="preserve">No fix needed for this story from current QuoteEngine automated retest.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Composer -&gt; AgentController messages -&gt; QuoteAgentService -&gt; session store</x:t>
+    <x:t xml:space="preserve">Composer -&gt; messages/stream -&gt; streaming agent response</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Chat composer and message thread</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST messages; QuoteAgentService SendMessageAsync</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests messages | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Agent model, SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Chat messages/session state</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs browser send-path retest</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:56; QuoteAgentService.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-004</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent streaming</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can receive streamed agent responses.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Streaming endpoint returns structured response chunks and the UI keeps thread/composer layout stable.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Composer -&gt; messages/stream -&gt; streaming agent response</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Streaming response thread</x:t>
@@ -5204,7 +5183,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ceaa025d74948c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd659e5451b6047aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8620,7 +8599,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6c6f739a8d934916"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26783c875c8e4b25"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8861,85 +8840,85 @@
       <x:c r="D4" s="3" t="s">
         <x:v>430</x:v>
       </x:c>
-      <x:c r="E4" s="3" t="s">
-        <x:v>431</x:v>
+      <x:c r="E4" s="3" t="str">
+        <x:v>Composer send accepts a text or attachment-backed customer turn, blocks duplicate/pending-upload sends, streams the assistant response, and the BFF send endpoint creates or resumes a QuoteEngine agent session with gate state.</x:v>
       </x:c>
       <x:c r="F4" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="G4" s="3" t="s">
-        <x:v>432</x:v>
-      </x:c>
-      <x:c r="H4" s="3" t="s">
-        <x:v>433</x:v>
-      </x:c>
-      <x:c r="I4" s="3" t="s">
-        <x:v>434</x:v>
-      </x:c>
-      <x:c r="J4" s="3" t="s">
-        <x:v>41</x:v>
+      <x:c r="G4" s="3" t="str">
+        <x:v>Focused current-state send-path tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H4" s="3" t="str">
+        <x:v>No behavior error observed in focused endpoint/source retest. Live browser send-path retest remains outstanding.</x:v>
+      </x:c>
+      <x:c r="I4" s="3" t="str">
+        <x:v>No app fix applied for this story in this slice; existing dirty QuoteAgentLaunchShell helper-formatting changes were left untouched.</x:v>
+      </x:c>
+      <x:c r="J4" s="3" t="str">
+        <x:v>Retested QuoteAgentEndpointTests.Agent_message_starts_anonymous_quote_engine_session_with_gate_state, QuoteAgentRateLimitTests, QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract, and QuoteEngineSourceTests.QuoteAgentLaunchShell_previews_attachments_until_customer_sends_message: 6/6 passed.</x:v>
       </x:c>
       <x:c r="K4" s="3" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="L4" s="3" t="s">
-        <x:v>435</x:v>
-      </x:c>
-      <x:c r="M4" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N4" s="3" t="s">
-        <x:v>437</x:v>
-      </x:c>
-      <x:c r="O4" s="3" t="s">
-        <x:v>438</x:v>
-      </x:c>
-      <x:c r="P4" s="3" t="s">
-        <x:v>439</x:v>
+      <x:c r="L4" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell composer -&gt; QuoteEngineApiClient stream/send APIs -&gt; AgentController send/stream endpoints -&gt; QuoteAgentService -&gt; ChatbotService session/message contract</x:v>
+      </x:c>
+      <x:c r="M4" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor composer form and send button; QuoteEngineApiClient; AgentController.Send/Stream</x:v>
+      </x:c>
+      <x:c r="N4" s="3" t="str">
+        <x:v>Composer form submits HandleSubmitAsync; send button disabled only while sending, dictating, or pending uploads; API client posts quote/v1/agent/messages and quote/v1/agent/messages/stream.</x:v>
+      </x:c>
+      <x:c r="O4" s="3" t="str">
+        <x:v>AgentController POST quote/v1/agent/messages validates model state, applies QuoteAgent rate limiting, and calls QuoteAgentService.SendAsync; QuoteAgentService creates/resumes session, composes customer context, and sends ChatbotSendMessageRequest with QuoteAgentContextToken.</x:v>
+      </x:c>
+      <x:c r="P4" s="3" t="str">
+        <x:v>dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_starts_anonymous_quote_engine_session_with_gate_state|FullyQualifiedName~QuoteAgentRateLimitTests|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_previews_attachments_until_customer_sends_message" --verbosity minimal passed 6/6 on 2026-06-24.</x:v>
       </x:c>
       <x:c r="Q4" s="3" t="s">
-        <x:v>440</x:v>
+        <x:v>431</x:v>
       </x:c>
       <x:c r="R4" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="S4" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="T4" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="U4" s="3" t="s">
-        <x:v>52</x:v>
+        <x:v>432</x:v>
+      </x:c>
+      <x:c r="S4" s="3" t="str">
+        <x:v>Needs live browser send-path retest against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T4" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor:1114,1266-1280,2170,2769-2924; QuoteEngineApiClient.cs:297-378; AgentController.cs:54-89; QuoteAgentService.cs:159-236; QuoteAgentEndpointTests.cs:80-117; QuoteAgentRateLimitTests.cs:23-90; QuoteEngineSourceTests.cs:864-1310,1933-1956</x:v>
+      </x:c>
+      <x:c r="U4" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="107.25" hidden="0">
       <x:c r="A5" s="3" t="s">
-        <x:v>444</x:v>
+        <x:v>433</x:v>
       </x:c>
       <x:c r="B5" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C5" s="3" t="s">
-        <x:v>445</x:v>
+        <x:v>434</x:v>
       </x:c>
       <x:c r="D5" s="3" t="s">
-        <x:v>446</x:v>
+        <x:v>435</x:v>
       </x:c>
       <x:c r="E5" s="3" t="s">
-        <x:v>447</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G5" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H5" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I5" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J5" s="3" t="s">
         <x:v>41</x:v>
@@ -8948,31 +8927,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L5" s="3" t="s">
+        <x:v>440</x:v>
+      </x:c>
+      <x:c r="M5" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N5" s="3" t="s">
+        <x:v>442</x:v>
+      </x:c>
+      <x:c r="O5" s="3" t="s">
+        <x:v>443</x:v>
+      </x:c>
+      <x:c r="P5" s="3" t="s">
+        <x:v>444</x:v>
+      </x:c>
+      <x:c r="Q5" s="3" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="R5" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="S5" s="3" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="T5" s="3" t="s">
         <x:v>448</x:v>
-      </x:c>
-      <x:c r="M5" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N5" s="3" t="s">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="O5" s="3" t="s">
-        <x:v>450</x:v>
-      </x:c>
-      <x:c r="P5" s="3" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="Q5" s="3" t="s">
-        <x:v>452</x:v>
-      </x:c>
-      <x:c r="R5" s="3" t="s">
-        <x:v>453</x:v>
-      </x:c>
-      <x:c r="S5" s="3" t="s">
-        <x:v>454</x:v>
-      </x:c>
-      <x:c r="T5" s="3" t="s">
-        <x:v>455</x:v>
       </x:c>
       <x:c r="U5" s="3" t="s">
         <x:v>52</x:v>
@@ -8980,31 +8959,31 @@
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
       <x:c r="A6" s="3" t="s">
-        <x:v>456</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>457</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>458</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>459</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H6" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I6" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J6" s="3" t="s">
         <x:v>41</x:v>
@@ -9013,31 +8992,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L6" s="3" t="s">
+        <x:v>453</x:v>
+      </x:c>
+      <x:c r="M6" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N6" s="3" t="s">
+        <x:v>454</x:v>
+      </x:c>
+      <x:c r="O6" s="3" t="s">
+        <x:v>455</x:v>
+      </x:c>
+      <x:c r="P6" s="3" t="s">
+        <x:v>456</x:v>
+      </x:c>
+      <x:c r="Q6" s="3" t="s">
+        <x:v>457</x:v>
+      </x:c>
+      <x:c r="R6" s="3" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="S6" s="3" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="T6" s="3" t="s">
         <x:v>460</x:v>
-      </x:c>
-      <x:c r="M6" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N6" s="3" t="s">
-        <x:v>461</x:v>
-      </x:c>
-      <x:c r="O6" s="3" t="s">
-        <x:v>462</x:v>
-      </x:c>
-      <x:c r="P6" s="3" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="Q6" s="3" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="R6" s="3" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="S6" s="3" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="T6" s="3" t="s">
-        <x:v>467</x:v>
       </x:c>
       <x:c r="U6" s="3" t="s">
         <x:v>52</x:v>
@@ -9045,31 +9024,31 @@
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>468</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>469</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>470</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G7" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H7" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I7" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J7" s="3" t="s">
         <x:v>41</x:v>
@@ -9078,31 +9057,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
+        <x:v>465</x:v>
+      </x:c>
+      <x:c r="M7" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N7" s="3" t="s">
+        <x:v>466</x:v>
+      </x:c>
+      <x:c r="O7" s="3" t="s">
+        <x:v>467</x:v>
+      </x:c>
+      <x:c r="P7" s="3" t="s">
+        <x:v>468</x:v>
+      </x:c>
+      <x:c r="Q7" s="3" t="s">
+        <x:v>469</x:v>
+      </x:c>
+      <x:c r="R7" s="3" t="s">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="S7" s="3" t="s">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="T7" s="3" t="s">
         <x:v>472</x:v>
-      </x:c>
-      <x:c r="M7" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N7" s="3" t="s">
-        <x:v>473</x:v>
-      </x:c>
-      <x:c r="O7" s="3" t="s">
-        <x:v>474</x:v>
-      </x:c>
-      <x:c r="P7" s="3" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="Q7" s="3" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="R7" s="3" t="s">
-        <x:v>477</x:v>
-      </x:c>
-      <x:c r="S7" s="3" t="s">
-        <x:v>478</x:v>
-      </x:c>
-      <x:c r="T7" s="3" t="s">
-        <x:v>479</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>52</x:v>
@@ -9110,31 +9089,31 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H8" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I8" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J8" s="3" t="s">
         <x:v>41</x:v>
@@ -9143,31 +9122,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
+        <x:v>477</x:v>
+      </x:c>
+      <x:c r="M8" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N8" s="3" t="s">
+        <x:v>478</x:v>
+      </x:c>
+      <x:c r="O8" s="3" t="s">
+        <x:v>479</x:v>
+      </x:c>
+      <x:c r="P8" s="3" t="s">
+        <x:v>480</x:v>
+      </x:c>
+      <x:c r="Q8" s="3" t="s">
+        <x:v>481</x:v>
+      </x:c>
+      <x:c r="R8" s="3" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="S8" s="3" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="T8" s="3" t="s">
         <x:v>484</x:v>
-      </x:c>
-      <x:c r="M8" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N8" s="3" t="s">
-        <x:v>485</x:v>
-      </x:c>
-      <x:c r="O8" s="3" t="s">
-        <x:v>486</x:v>
-      </x:c>
-      <x:c r="P8" s="3" t="s">
-        <x:v>487</x:v>
-      </x:c>
-      <x:c r="Q8" s="3" t="s">
-        <x:v>488</x:v>
-      </x:c>
-      <x:c r="R8" s="3" t="s">
-        <x:v>489</x:v>
-      </x:c>
-      <x:c r="S8" s="3" t="s">
-        <x:v>490</x:v>
-      </x:c>
-      <x:c r="T8" s="3" t="s">
-        <x:v>491</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>52</x:v>
@@ -9175,31 +9154,31 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H9" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I9" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J9" s="3" t="s">
         <x:v>41</x:v>
@@ -9208,31 +9187,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
+        <x:v>489</x:v>
+      </x:c>
+      <x:c r="M9" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N9" s="3" t="s">
+        <x:v>490</x:v>
+      </x:c>
+      <x:c r="O9" s="3" t="s">
+        <x:v>491</x:v>
+      </x:c>
+      <x:c r="P9" s="3" t="s">
+        <x:v>492</x:v>
+      </x:c>
+      <x:c r="Q9" s="3" t="s">
+        <x:v>493</x:v>
+      </x:c>
+      <x:c r="R9" s="3" t="s">
+        <x:v>494</x:v>
+      </x:c>
+      <x:c r="S9" s="3" t="s">
+        <x:v>495</x:v>
+      </x:c>
+      <x:c r="T9" s="3" t="s">
         <x:v>496</x:v>
-      </x:c>
-      <x:c r="M9" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N9" s="3" t="s">
-        <x:v>497</x:v>
-      </x:c>
-      <x:c r="O9" s="3" t="s">
-        <x:v>498</x:v>
-      </x:c>
-      <x:c r="P9" s="3" t="s">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="Q9" s="3" t="s">
-        <x:v>500</x:v>
-      </x:c>
-      <x:c r="R9" s="3" t="s">
-        <x:v>501</x:v>
-      </x:c>
-      <x:c r="S9" s="3" t="s">
-        <x:v>502</x:v>
-      </x:c>
-      <x:c r="T9" s="3" t="s">
-        <x:v>503</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>52</x:v>
@@ -9240,31 +9219,31 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G10" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H10" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I10" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J10" s="3" t="s">
         <x:v>41</x:v>
@@ -9273,31 +9252,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
         <x:v>424</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>52</x:v>
@@ -9305,31 +9284,31 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G11" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H11" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I11" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J11" s="3" t="s">
         <x:v>41</x:v>
@@ -9338,31 +9317,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
+        <x:v>512</x:v>
+      </x:c>
+      <x:c r="M11" s="3" t="s">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="N11" s="3" t="s">
+        <x:v>514</x:v>
+      </x:c>
+      <x:c r="O11" s="3" t="s">
+        <x:v>515</x:v>
+      </x:c>
+      <x:c r="P11" s="3" t="s">
+        <x:v>516</x:v>
+      </x:c>
+      <x:c r="Q11" s="3" t="s">
+        <x:v>517</x:v>
+      </x:c>
+      <x:c r="R11" s="3" t="s">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="S11" s="3" t="s">
         <x:v>519</x:v>
       </x:c>
-      <x:c r="M11" s="3" t="s">
+      <x:c r="T11" s="3" t="s">
         <x:v>520</x:v>
-      </x:c>
-      <x:c r="N11" s="3" t="s">
-        <x:v>521</x:v>
-      </x:c>
-      <x:c r="O11" s="3" t="s">
-        <x:v>522</x:v>
-      </x:c>
-      <x:c r="P11" s="3" t="s">
-        <x:v>523</x:v>
-      </x:c>
-      <x:c r="Q11" s="3" t="s">
-        <x:v>524</x:v>
-      </x:c>
-      <x:c r="R11" s="3" t="s">
-        <x:v>525</x:v>
-      </x:c>
-      <x:c r="S11" s="3" t="s">
-        <x:v>526</x:v>
-      </x:c>
-      <x:c r="T11" s="3" t="s">
-        <x:v>527</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>52</x:v>
@@ -9370,31 +9349,31 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G12" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H12" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I12" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J12" s="3" t="s">
         <x:v>41</x:v>
@@ -9403,31 +9382,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
+        <x:v>525</x:v>
+      </x:c>
+      <x:c r="M12" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N12" s="3" t="s">
+        <x:v>526</x:v>
+      </x:c>
+      <x:c r="O12" s="3" t="s">
+        <x:v>527</x:v>
+      </x:c>
+      <x:c r="P12" s="3" t="s">
+        <x:v>528</x:v>
+      </x:c>
+      <x:c r="Q12" s="3" t="s">
+        <x:v>529</x:v>
+      </x:c>
+      <x:c r="R12" s="3" t="s">
+        <x:v>530</x:v>
+      </x:c>
+      <x:c r="S12" s="3" t="s">
+        <x:v>531</x:v>
+      </x:c>
+      <x:c r="T12" s="3" t="s">
         <x:v>532</x:v>
-      </x:c>
-      <x:c r="M12" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N12" s="3" t="s">
-        <x:v>533</x:v>
-      </x:c>
-      <x:c r="O12" s="3" t="s">
-        <x:v>534</x:v>
-      </x:c>
-      <x:c r="P12" s="3" t="s">
-        <x:v>535</x:v>
-      </x:c>
-      <x:c r="Q12" s="3" t="s">
-        <x:v>536</x:v>
-      </x:c>
-      <x:c r="R12" s="3" t="s">
-        <x:v>537</x:v>
-      </x:c>
-      <x:c r="S12" s="3" t="s">
-        <x:v>538</x:v>
-      </x:c>
-      <x:c r="T12" s="3" t="s">
-        <x:v>539</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>52</x:v>
@@ -9435,31 +9414,31 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I13" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J13" s="3" t="s">
         <x:v>41</x:v>
@@ -9468,31 +9447,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
-        <x:v>436</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>52</x:v>
@@ -9500,31 +9479,31 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G14" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H14" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I14" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J14" s="3" t="s">
         <x:v>41</x:v>
@@ -9533,31 +9512,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
+        <x:v>548</x:v>
+      </x:c>
+      <x:c r="M14" s="3" t="s">
+        <x:v>549</x:v>
+      </x:c>
+      <x:c r="N14" s="3" t="s">
+        <x:v>550</x:v>
+      </x:c>
+      <x:c r="O14" s="3" t="s">
+        <x:v>551</x:v>
+      </x:c>
+      <x:c r="P14" s="3" t="s">
+        <x:v>552</x:v>
+      </x:c>
+      <x:c r="Q14" s="3" t="s">
+        <x:v>553</x:v>
+      </x:c>
+      <x:c r="R14" s="3" t="s">
+        <x:v>554</x:v>
+      </x:c>
+      <x:c r="S14" s="3" t="s">
         <x:v>555</x:v>
       </x:c>
-      <x:c r="M14" s="3" t="s">
+      <x:c r="T14" s="3" t="s">
         <x:v>556</x:v>
-      </x:c>
-      <x:c r="N14" s="3" t="s">
-        <x:v>557</x:v>
-      </x:c>
-      <x:c r="O14" s="3" t="s">
-        <x:v>558</x:v>
-      </x:c>
-      <x:c r="P14" s="3" t="s">
-        <x:v>559</x:v>
-      </x:c>
-      <x:c r="Q14" s="3" t="s">
-        <x:v>560</x:v>
-      </x:c>
-      <x:c r="R14" s="3" t="s">
-        <x:v>561</x:v>
-      </x:c>
-      <x:c r="S14" s="3" t="s">
-        <x:v>562</x:v>
-      </x:c>
-      <x:c r="T14" s="3" t="s">
-        <x:v>563</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9565,31 +9544,31 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G15" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H15" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I15" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J15" s="3" t="s">
         <x:v>41</x:v>
@@ -9598,31 +9577,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
+        <x:v>561</x:v>
+      </x:c>
+      <x:c r="M15" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N15" s="3" t="s">
+        <x:v>562</x:v>
+      </x:c>
+      <x:c r="O15" s="3" t="s">
+        <x:v>563</x:v>
+      </x:c>
+      <x:c r="P15" s="3" t="s">
+        <x:v>564</x:v>
+      </x:c>
+      <x:c r="Q15" s="3" t="s">
+        <x:v>565</x:v>
+      </x:c>
+      <x:c r="R15" s="3" t="s">
+        <x:v>566</x:v>
+      </x:c>
+      <x:c r="S15" s="3" t="s">
+        <x:v>567</x:v>
+      </x:c>
+      <x:c r="T15" s="3" t="s">
         <x:v>568</x:v>
-      </x:c>
-      <x:c r="M15" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N15" s="3" t="s">
-        <x:v>569</x:v>
-      </x:c>
-      <x:c r="O15" s="3" t="s">
-        <x:v>570</x:v>
-      </x:c>
-      <x:c r="P15" s="3" t="s">
-        <x:v>571</x:v>
-      </x:c>
-      <x:c r="Q15" s="3" t="s">
-        <x:v>572</x:v>
-      </x:c>
-      <x:c r="R15" s="3" t="s">
-        <x:v>573</x:v>
-      </x:c>
-      <x:c r="S15" s="3" t="s">
-        <x:v>574</x:v>
-      </x:c>
-      <x:c r="T15" s="3" t="s">
-        <x:v>575</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9630,31 +9609,31 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H16" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I16" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J16" s="3" t="s">
         <x:v>41</x:v>
@@ -9663,31 +9642,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
+        <x:v>573</x:v>
+      </x:c>
+      <x:c r="M16" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N16" s="3" t="s">
+        <x:v>574</x:v>
+      </x:c>
+      <x:c r="O16" s="3" t="s">
+        <x:v>575</x:v>
+      </x:c>
+      <x:c r="P16" s="3" t="s">
+        <x:v>576</x:v>
+      </x:c>
+      <x:c r="Q16" s="3" t="s">
+        <x:v>577</x:v>
+      </x:c>
+      <x:c r="R16" s="3" t="s">
+        <x:v>578</x:v>
+      </x:c>
+      <x:c r="S16" s="3" t="s">
+        <x:v>579</x:v>
+      </x:c>
+      <x:c r="T16" s="3" t="s">
         <x:v>580</x:v>
-      </x:c>
-      <x:c r="M16" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N16" s="3" t="s">
-        <x:v>581</x:v>
-      </x:c>
-      <x:c r="O16" s="3" t="s">
-        <x:v>582</x:v>
-      </x:c>
-      <x:c r="P16" s="3" t="s">
-        <x:v>583</x:v>
-      </x:c>
-      <x:c r="Q16" s="3" t="s">
-        <x:v>584</x:v>
-      </x:c>
-      <x:c r="R16" s="3" t="s">
-        <x:v>585</x:v>
-      </x:c>
-      <x:c r="S16" s="3" t="s">
-        <x:v>586</x:v>
-      </x:c>
-      <x:c r="T16" s="3" t="s">
-        <x:v>587</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9695,31 +9674,31 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H17" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I17" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J17" s="3" t="s">
         <x:v>41</x:v>
@@ -9728,31 +9707,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
+        <x:v>585</x:v>
+      </x:c>
+      <x:c r="M17" s="3" t="s">
+        <x:v>586</x:v>
+      </x:c>
+      <x:c r="N17" s="3" t="s">
+        <x:v>587</x:v>
+      </x:c>
+      <x:c r="O17" s="3" t="s">
+        <x:v>588</x:v>
+      </x:c>
+      <x:c r="P17" s="3" t="s">
+        <x:v>589</x:v>
+      </x:c>
+      <x:c r="Q17" s="3" t="s">
+        <x:v>590</x:v>
+      </x:c>
+      <x:c r="R17" s="3" t="s">
+        <x:v>591</x:v>
+      </x:c>
+      <x:c r="S17" s="3" t="s">
         <x:v>592</x:v>
       </x:c>
-      <x:c r="M17" s="3" t="s">
+      <x:c r="T17" s="3" t="s">
         <x:v>593</x:v>
-      </x:c>
-      <x:c r="N17" s="3" t="s">
-        <x:v>594</x:v>
-      </x:c>
-      <x:c r="O17" s="3" t="s">
-        <x:v>595</x:v>
-      </x:c>
-      <x:c r="P17" s="3" t="s">
-        <x:v>596</x:v>
-      </x:c>
-      <x:c r="Q17" s="3" t="s">
-        <x:v>597</x:v>
-      </x:c>
-      <x:c r="R17" s="3" t="s">
-        <x:v>598</x:v>
-      </x:c>
-      <x:c r="S17" s="3" t="s">
-        <x:v>599</x:v>
-      </x:c>
-      <x:c r="T17" s="3" t="s">
-        <x:v>600</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9760,31 +9739,31 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G18" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H18" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I18" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J18" s="3" t="s">
         <x:v>41</x:v>
@@ -9793,31 +9772,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
+        <x:v>598</x:v>
+      </x:c>
+      <x:c r="M18" s="3" t="s">
+        <x:v>599</x:v>
+      </x:c>
+      <x:c r="N18" s="3" t="s">
+        <x:v>600</x:v>
+      </x:c>
+      <x:c r="O18" s="3" t="s">
+        <x:v>601</x:v>
+      </x:c>
+      <x:c r="P18" s="3" t="s">
+        <x:v>602</x:v>
+      </x:c>
+      <x:c r="Q18" s="3" t="s">
+        <x:v>603</x:v>
+      </x:c>
+      <x:c r="R18" s="3" t="s">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="S18" s="3" t="s">
         <x:v>605</x:v>
       </x:c>
-      <x:c r="M18" s="3" t="s">
+      <x:c r="T18" s="3" t="s">
         <x:v>606</x:v>
-      </x:c>
-      <x:c r="N18" s="3" t="s">
-        <x:v>607</x:v>
-      </x:c>
-      <x:c r="O18" s="3" t="s">
-        <x:v>608</x:v>
-      </x:c>
-      <x:c r="P18" s="3" t="s">
-        <x:v>609</x:v>
-      </x:c>
-      <x:c r="Q18" s="3" t="s">
-        <x:v>610</x:v>
-      </x:c>
-      <x:c r="R18" s="3" t="s">
-        <x:v>611</x:v>
-      </x:c>
-      <x:c r="S18" s="3" t="s">
-        <x:v>612</x:v>
-      </x:c>
-      <x:c r="T18" s="3" t="s">
-        <x:v>613</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9825,31 +9804,31 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I19" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J19" s="3" t="s">
         <x:v>41</x:v>
@@ -9858,31 +9837,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
+        <x:v>611</x:v>
+      </x:c>
+      <x:c r="M19" s="3" t="s">
+        <x:v>612</x:v>
+      </x:c>
+      <x:c r="N19" s="3" t="s">
+        <x:v>613</x:v>
+      </x:c>
+      <x:c r="O19" s="3" t="s">
+        <x:v>614</x:v>
+      </x:c>
+      <x:c r="P19" s="3" t="s">
+        <x:v>615</x:v>
+      </x:c>
+      <x:c r="Q19" s="3" t="s">
+        <x:v>616</x:v>
+      </x:c>
+      <x:c r="R19" s="3" t="s">
+        <x:v>617</x:v>
+      </x:c>
+      <x:c r="S19" s="3" t="s">
         <x:v>618</x:v>
       </x:c>
-      <x:c r="M19" s="3" t="s">
+      <x:c r="T19" s="3" t="s">
         <x:v>619</x:v>
-      </x:c>
-      <x:c r="N19" s="3" t="s">
-        <x:v>620</x:v>
-      </x:c>
-      <x:c r="O19" s="3" t="s">
-        <x:v>621</x:v>
-      </x:c>
-      <x:c r="P19" s="3" t="s">
-        <x:v>622</x:v>
-      </x:c>
-      <x:c r="Q19" s="3" t="s">
-        <x:v>623</x:v>
-      </x:c>
-      <x:c r="R19" s="3" t="s">
-        <x:v>624</x:v>
-      </x:c>
-      <x:c r="S19" s="3" t="s">
-        <x:v>625</x:v>
-      </x:c>
-      <x:c r="T19" s="3" t="s">
-        <x:v>626</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9890,31 +9869,31 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I20" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J20" s="3" t="s">
         <x:v>41</x:v>
@@ -9923,31 +9902,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
+        <x:v>624</x:v>
+      </x:c>
+      <x:c r="M20" s="3" t="s">
+        <x:v>625</x:v>
+      </x:c>
+      <x:c r="N20" s="3" t="s">
+        <x:v>626</x:v>
+      </x:c>
+      <x:c r="O20" s="3" t="s">
+        <x:v>627</x:v>
+      </x:c>
+      <x:c r="P20" s="3" t="s">
+        <x:v>628</x:v>
+      </x:c>
+      <x:c r="Q20" s="3" t="s">
+        <x:v>629</x:v>
+      </x:c>
+      <x:c r="R20" s="3" t="s">
+        <x:v>630</x:v>
+      </x:c>
+      <x:c r="S20" s="3" t="s">
         <x:v>631</x:v>
       </x:c>
-      <x:c r="M20" s="3" t="s">
+      <x:c r="T20" s="3" t="s">
         <x:v>632</x:v>
-      </x:c>
-      <x:c r="N20" s="3" t="s">
-        <x:v>633</x:v>
-      </x:c>
-      <x:c r="O20" s="3" t="s">
-        <x:v>634</x:v>
-      </x:c>
-      <x:c r="P20" s="3" t="s">
-        <x:v>635</x:v>
-      </x:c>
-      <x:c r="Q20" s="3" t="s">
-        <x:v>636</x:v>
-      </x:c>
-      <x:c r="R20" s="3" t="s">
-        <x:v>637</x:v>
-      </x:c>
-      <x:c r="S20" s="3" t="s">
-        <x:v>638</x:v>
-      </x:c>
-      <x:c r="T20" s="3" t="s">
-        <x:v>639</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9955,31 +9934,31 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G21" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H21" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I21" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J21" s="3" t="s">
         <x:v>41</x:v>
@@ -9988,31 +9967,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -10020,31 +9999,31 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G22" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H22" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I22" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J22" s="3" t="s">
         <x:v>41</x:v>
@@ -10053,31 +10032,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
+        <x:v>648</x:v>
+      </x:c>
+      <x:c r="M22" s="3" t="s">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="N22" s="3" t="s">
+        <x:v>649</x:v>
+      </x:c>
+      <x:c r="O22" s="3" t="s">
+        <x:v>650</x:v>
+      </x:c>
+      <x:c r="P22" s="3" t="s">
+        <x:v>651</x:v>
+      </x:c>
+      <x:c r="Q22" s="3" t="s">
+        <x:v>652</x:v>
+      </x:c>
+      <x:c r="R22" s="3" t="s">
+        <x:v>653</x:v>
+      </x:c>
+      <x:c r="S22" s="3" t="s">
+        <x:v>654</x:v>
+      </x:c>
+      <x:c r="T22" s="3" t="s">
         <x:v>655</x:v>
-      </x:c>
-      <x:c r="M22" s="3" t="s">
-        <x:v>520</x:v>
-      </x:c>
-      <x:c r="N22" s="3" t="s">
-        <x:v>656</x:v>
-      </x:c>
-      <x:c r="O22" s="3" t="s">
-        <x:v>657</x:v>
-      </x:c>
-      <x:c r="P22" s="3" t="s">
-        <x:v>658</x:v>
-      </x:c>
-      <x:c r="Q22" s="3" t="s">
-        <x:v>659</x:v>
-      </x:c>
-      <x:c r="R22" s="3" t="s">
-        <x:v>660</x:v>
-      </x:c>
-      <x:c r="S22" s="3" t="s">
-        <x:v>661</x:v>
-      </x:c>
-      <x:c r="T22" s="3" t="s">
-        <x:v>662</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -10085,31 +10064,31 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G23" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H23" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I23" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J23" s="3" t="s">
         <x:v>41</x:v>
@@ -10118,31 +10097,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
+        <x:v>660</x:v>
+      </x:c>
+      <x:c r="M23" s="3" t="s">
+        <x:v>661</x:v>
+      </x:c>
+      <x:c r="N23" s="3" t="s">
+        <x:v>662</x:v>
+      </x:c>
+      <x:c r="O23" s="3" t="s">
+        <x:v>663</x:v>
+      </x:c>
+      <x:c r="P23" s="3" t="s">
+        <x:v>664</x:v>
+      </x:c>
+      <x:c r="Q23" s="3" t="s">
+        <x:v>665</x:v>
+      </x:c>
+      <x:c r="R23" s="3" t="s">
+        <x:v>666</x:v>
+      </x:c>
+      <x:c r="S23" s="3" t="s">
         <x:v>667</x:v>
       </x:c>
-      <x:c r="M23" s="3" t="s">
+      <x:c r="T23" s="3" t="s">
         <x:v>668</x:v>
-      </x:c>
-      <x:c r="N23" s="3" t="s">
-        <x:v>669</x:v>
-      </x:c>
-      <x:c r="O23" s="3" t="s">
-        <x:v>670</x:v>
-      </x:c>
-      <x:c r="P23" s="3" t="s">
-        <x:v>671</x:v>
-      </x:c>
-      <x:c r="Q23" s="3" t="s">
-        <x:v>672</x:v>
-      </x:c>
-      <x:c r="R23" s="3" t="s">
-        <x:v>673</x:v>
-      </x:c>
-      <x:c r="S23" s="3" t="s">
-        <x:v>674</x:v>
-      </x:c>
-      <x:c r="T23" s="3" t="s">
-        <x:v>675</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -10150,31 +10129,31 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H24" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I24" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J24" s="3" t="s">
         <x:v>41</x:v>
@@ -10183,31 +10162,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
+        <x:v>673</x:v>
+      </x:c>
+      <x:c r="M24" s="3" t="s">
+        <x:v>638</x:v>
+      </x:c>
+      <x:c r="N24" s="3" t="s">
+        <x:v>674</x:v>
+      </x:c>
+      <x:c r="O24" s="3" t="s">
+        <x:v>675</x:v>
+      </x:c>
+      <x:c r="P24" s="3" t="s">
+        <x:v>676</x:v>
+      </x:c>
+      <x:c r="Q24" s="3" t="s">
+        <x:v>677</x:v>
+      </x:c>
+      <x:c r="R24" s="3" t="s">
+        <x:v>678</x:v>
+      </x:c>
+      <x:c r="S24" s="3" t="s">
+        <x:v>679</x:v>
+      </x:c>
+      <x:c r="T24" s="3" t="s">
         <x:v>680</x:v>
-      </x:c>
-      <x:c r="M24" s="3" t="s">
-        <x:v>645</x:v>
-      </x:c>
-      <x:c r="N24" s="3" t="s">
-        <x:v>681</x:v>
-      </x:c>
-      <x:c r="O24" s="3" t="s">
-        <x:v>682</x:v>
-      </x:c>
-      <x:c r="P24" s="3" t="s">
-        <x:v>683</x:v>
-      </x:c>
-      <x:c r="Q24" s="3" t="s">
-        <x:v>684</x:v>
-      </x:c>
-      <x:c r="R24" s="3" t="s">
-        <x:v>685</x:v>
-      </x:c>
-      <x:c r="S24" s="3" t="s">
-        <x:v>686</x:v>
-      </x:c>
-      <x:c r="T24" s="3" t="s">
-        <x:v>687</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -10215,31 +10194,31 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H25" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I25" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J25" s="3" t="s">
         <x:v>41</x:v>
@@ -10248,31 +10227,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
+        <x:v>685</x:v>
+      </x:c>
+      <x:c r="M25" s="3" t="s">
+        <x:v>638</x:v>
+      </x:c>
+      <x:c r="N25" s="3" t="s">
+        <x:v>686</x:v>
+      </x:c>
+      <x:c r="O25" s="3" t="s">
+        <x:v>687</x:v>
+      </x:c>
+      <x:c r="P25" s="3" t="s">
+        <x:v>688</x:v>
+      </x:c>
+      <x:c r="Q25" s="3" t="s">
+        <x:v>689</x:v>
+      </x:c>
+      <x:c r="R25" s="3" t="s">
+        <x:v>690</x:v>
+      </x:c>
+      <x:c r="S25" s="3" t="s">
+        <x:v>691</x:v>
+      </x:c>
+      <x:c r="T25" s="3" t="s">
         <x:v>692</x:v>
-      </x:c>
-      <x:c r="M25" s="3" t="s">
-        <x:v>645</x:v>
-      </x:c>
-      <x:c r="N25" s="3" t="s">
-        <x:v>693</x:v>
-      </x:c>
-      <x:c r="O25" s="3" t="s">
-        <x:v>694</x:v>
-      </x:c>
-      <x:c r="P25" s="3" t="s">
-        <x:v>695</x:v>
-      </x:c>
-      <x:c r="Q25" s="3" t="s">
-        <x:v>696</x:v>
-      </x:c>
-      <x:c r="R25" s="3" t="s">
-        <x:v>697</x:v>
-      </x:c>
-      <x:c r="S25" s="3" t="s">
-        <x:v>698</x:v>
-      </x:c>
-      <x:c r="T25" s="3" t="s">
-        <x:v>699</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10280,31 +10259,31 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H26" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I26" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J26" s="3" t="s">
         <x:v>41</x:v>
@@ -10313,31 +10292,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
+        <x:v>697</x:v>
+      </x:c>
+      <x:c r="M26" s="3" t="s">
+        <x:v>698</x:v>
+      </x:c>
+      <x:c r="N26" s="3" t="s">
+        <x:v>699</x:v>
+      </x:c>
+      <x:c r="O26" s="3" t="s">
+        <x:v>700</x:v>
+      </x:c>
+      <x:c r="P26" s="3" t="s">
+        <x:v>701</x:v>
+      </x:c>
+      <x:c r="Q26" s="3" t="s">
+        <x:v>702</x:v>
+      </x:c>
+      <x:c r="R26" s="3" t="s">
+        <x:v>703</x:v>
+      </x:c>
+      <x:c r="S26" s="3" t="s">
         <x:v>704</x:v>
       </x:c>
-      <x:c r="M26" s="3" t="s">
+      <x:c r="T26" s="3" t="s">
         <x:v>705</x:v>
-      </x:c>
-      <x:c r="N26" s="3" t="s">
-        <x:v>706</x:v>
-      </x:c>
-      <x:c r="O26" s="3" t="s">
-        <x:v>707</x:v>
-      </x:c>
-      <x:c r="P26" s="3" t="s">
-        <x:v>708</x:v>
-      </x:c>
-      <x:c r="Q26" s="3" t="s">
-        <x:v>709</x:v>
-      </x:c>
-      <x:c r="R26" s="3" t="s">
-        <x:v>710</x:v>
-      </x:c>
-      <x:c r="S26" s="3" t="s">
-        <x:v>711</x:v>
-      </x:c>
-      <x:c r="T26" s="3" t="s">
-        <x:v>712</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10345,31 +10324,31 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H27" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I27" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J27" s="3" t="s">
         <x:v>41</x:v>
@@ -10378,31 +10357,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
+        <x:v>710</x:v>
+      </x:c>
+      <x:c r="M27" s="3" t="s">
+        <x:v>711</x:v>
+      </x:c>
+      <x:c r="N27" s="3" t="s">
+        <x:v>712</x:v>
+      </x:c>
+      <x:c r="O27" s="3" t="s">
+        <x:v>713</x:v>
+      </x:c>
+      <x:c r="P27" s="3" t="s">
+        <x:v>714</x:v>
+      </x:c>
+      <x:c r="Q27" s="3" t="s">
+        <x:v>715</x:v>
+      </x:c>
+      <x:c r="R27" s="3" t="s">
+        <x:v>716</x:v>
+      </x:c>
+      <x:c r="S27" s="3" t="s">
         <x:v>717</x:v>
       </x:c>
-      <x:c r="M27" s="3" t="s">
+      <x:c r="T27" s="3" t="s">
         <x:v>718</x:v>
-      </x:c>
-      <x:c r="N27" s="3" t="s">
-        <x:v>719</x:v>
-      </x:c>
-      <x:c r="O27" s="3" t="s">
-        <x:v>720</x:v>
-      </x:c>
-      <x:c r="P27" s="3" t="s">
-        <x:v>721</x:v>
-      </x:c>
-      <x:c r="Q27" s="3" t="s">
-        <x:v>722</x:v>
-      </x:c>
-      <x:c r="R27" s="3" t="s">
-        <x:v>723</x:v>
-      </x:c>
-      <x:c r="S27" s="3" t="s">
-        <x:v>724</x:v>
-      </x:c>
-      <x:c r="T27" s="3" t="s">
-        <x:v>725</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10410,31 +10389,31 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G28" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H28" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I28" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J28" s="3" t="s">
         <x:v>41</x:v>
@@ -10443,31 +10422,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10475,31 +10454,31 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G29" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H29" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I29" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J29" s="3" t="s">
         <x:v>41</x:v>
@@ -10508,31 +10487,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
+        <x:v>735</x:v>
+      </x:c>
+      <x:c r="M29" s="3" t="s">
+        <x:v>736</x:v>
+      </x:c>
+      <x:c r="N29" s="3" t="s">
+        <x:v>737</x:v>
+      </x:c>
+      <x:c r="O29" s="3" t="s">
+        <x:v>738</x:v>
+      </x:c>
+      <x:c r="P29" s="3" t="s">
+        <x:v>739</x:v>
+      </x:c>
+      <x:c r="Q29" s="3" t="s">
+        <x:v>740</x:v>
+      </x:c>
+      <x:c r="R29" s="3" t="s">
+        <x:v>741</x:v>
+      </x:c>
+      <x:c r="S29" s="3" t="s">
         <x:v>742</x:v>
       </x:c>
-      <x:c r="M29" s="3" t="s">
+      <x:c r="T29" s="3" t="s">
         <x:v>743</x:v>
-      </x:c>
-      <x:c r="N29" s="3" t="s">
-        <x:v>744</x:v>
-      </x:c>
-      <x:c r="O29" s="3" t="s">
-        <x:v>745</x:v>
-      </x:c>
-      <x:c r="P29" s="3" t="s">
-        <x:v>746</x:v>
-      </x:c>
-      <x:c r="Q29" s="3" t="s">
-        <x:v>747</x:v>
-      </x:c>
-      <x:c r="R29" s="3" t="s">
-        <x:v>748</x:v>
-      </x:c>
-      <x:c r="S29" s="3" t="s">
-        <x:v>749</x:v>
-      </x:c>
-      <x:c r="T29" s="3" t="s">
-        <x:v>750</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10540,31 +10519,31 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G30" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H30" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I30" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J30" s="3" t="s">
         <x:v>41</x:v>
@@ -10573,31 +10552,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
+        <x:v>748</x:v>
+      </x:c>
+      <x:c r="M30" s="3" t="s">
+        <x:v>749</x:v>
+      </x:c>
+      <x:c r="N30" s="3" t="s">
+        <x:v>750</x:v>
+      </x:c>
+      <x:c r="O30" s="3" t="s">
+        <x:v>751</x:v>
+      </x:c>
+      <x:c r="P30" s="3" t="s">
+        <x:v>752</x:v>
+      </x:c>
+      <x:c r="Q30" s="3" t="s">
+        <x:v>753</x:v>
+      </x:c>
+      <x:c r="R30" s="3" t="s">
+        <x:v>754</x:v>
+      </x:c>
+      <x:c r="S30" s="3" t="s">
         <x:v>755</x:v>
       </x:c>
-      <x:c r="M30" s="3" t="s">
+      <x:c r="T30" s="3" t="s">
         <x:v>756</x:v>
-      </x:c>
-      <x:c r="N30" s="3" t="s">
-        <x:v>757</x:v>
-      </x:c>
-      <x:c r="O30" s="3" t="s">
-        <x:v>758</x:v>
-      </x:c>
-      <x:c r="P30" s="3" t="s">
-        <x:v>759</x:v>
-      </x:c>
-      <x:c r="Q30" s="3" t="s">
-        <x:v>760</x:v>
-      </x:c>
-      <x:c r="R30" s="3" t="s">
-        <x:v>761</x:v>
-      </x:c>
-      <x:c r="S30" s="3" t="s">
-        <x:v>762</x:v>
-      </x:c>
-      <x:c r="T30" s="3" t="s">
-        <x:v>763</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10605,31 +10584,31 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G31" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H31" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I31" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J31" s="3" t="s">
         <x:v>41</x:v>
@@ -10638,31 +10617,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
+        <x:v>761</x:v>
+      </x:c>
+      <x:c r="M31" s="3" t="s">
+        <x:v>762</x:v>
+      </x:c>
+      <x:c r="N31" s="3" t="s">
+        <x:v>763</x:v>
+      </x:c>
+      <x:c r="O31" s="3" t="s">
+        <x:v>764</x:v>
+      </x:c>
+      <x:c r="P31" s="3" t="s">
+        <x:v>765</x:v>
+      </x:c>
+      <x:c r="Q31" s="3" t="s">
+        <x:v>766</x:v>
+      </x:c>
+      <x:c r="R31" s="3" t="s">
+        <x:v>767</x:v>
+      </x:c>
+      <x:c r="S31" s="3" t="s">
         <x:v>768</x:v>
       </x:c>
-      <x:c r="M31" s="3" t="s">
+      <x:c r="T31" s="3" t="s">
         <x:v>769</x:v>
-      </x:c>
-      <x:c r="N31" s="3" t="s">
-        <x:v>770</x:v>
-      </x:c>
-      <x:c r="O31" s="3" t="s">
-        <x:v>771</x:v>
-      </x:c>
-      <x:c r="P31" s="3" t="s">
-        <x:v>772</x:v>
-      </x:c>
-      <x:c r="Q31" s="3" t="s">
-        <x:v>773</x:v>
-      </x:c>
-      <x:c r="R31" s="3" t="s">
-        <x:v>774</x:v>
-      </x:c>
-      <x:c r="S31" s="3" t="s">
-        <x:v>775</x:v>
-      </x:c>
-      <x:c r="T31" s="3" t="s">
-        <x:v>776</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10670,31 +10649,31 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G32" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H32" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I32" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J32" s="3" t="s">
         <x:v>41</x:v>
@@ -10703,31 +10682,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
+        <x:v>774</x:v>
+      </x:c>
+      <x:c r="M32" s="3" t="s">
+        <x:v>775</x:v>
+      </x:c>
+      <x:c r="N32" s="3" t="s">
+        <x:v>776</x:v>
+      </x:c>
+      <x:c r="O32" s="3" t="s">
+        <x:v>777</x:v>
+      </x:c>
+      <x:c r="P32" s="3" t="s">
+        <x:v>778</x:v>
+      </x:c>
+      <x:c r="Q32" s="3" t="s">
+        <x:v>779</x:v>
+      </x:c>
+      <x:c r="R32" s="3" t="s">
+        <x:v>780</x:v>
+      </x:c>
+      <x:c r="S32" s="3" t="s">
         <x:v>781</x:v>
       </x:c>
-      <x:c r="M32" s="3" t="s">
+      <x:c r="T32" s="3" t="s">
         <x:v>782</x:v>
-      </x:c>
-      <x:c r="N32" s="3" t="s">
-        <x:v>783</x:v>
-      </x:c>
-      <x:c r="O32" s="3" t="s">
-        <x:v>784</x:v>
-      </x:c>
-      <x:c r="P32" s="3" t="s">
-        <x:v>785</x:v>
-      </x:c>
-      <x:c r="Q32" s="3" t="s">
-        <x:v>786</x:v>
-      </x:c>
-      <x:c r="R32" s="3" t="s">
-        <x:v>787</x:v>
-      </x:c>
-      <x:c r="S32" s="3" t="s">
-        <x:v>788</x:v>
-      </x:c>
-      <x:c r="T32" s="3" t="s">
-        <x:v>789</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10735,31 +10714,31 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G33" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H33" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I33" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J33" s="3" t="s">
         <x:v>41</x:v>
@@ -10768,31 +10747,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
+        <x:v>787</x:v>
+      </x:c>
+      <x:c r="M33" s="3" t="s">
+        <x:v>788</x:v>
+      </x:c>
+      <x:c r="N33" s="3" t="s">
+        <x:v>789</x:v>
+      </x:c>
+      <x:c r="O33" s="3" t="s">
+        <x:v>790</x:v>
+      </x:c>
+      <x:c r="P33" s="3" t="s">
+        <x:v>791</x:v>
+      </x:c>
+      <x:c r="Q33" s="3" t="s">
+        <x:v>792</x:v>
+      </x:c>
+      <x:c r="R33" s="3" t="s">
+        <x:v>793</x:v>
+      </x:c>
+      <x:c r="S33" s="3" t="s">
         <x:v>794</x:v>
       </x:c>
-      <x:c r="M33" s="3" t="s">
+      <x:c r="T33" s="3" t="s">
         <x:v>795</x:v>
-      </x:c>
-      <x:c r="N33" s="3" t="s">
-        <x:v>796</x:v>
-      </x:c>
-      <x:c r="O33" s="3" t="s">
-        <x:v>797</x:v>
-      </x:c>
-      <x:c r="P33" s="3" t="s">
-        <x:v>798</x:v>
-      </x:c>
-      <x:c r="Q33" s="3" t="s">
-        <x:v>799</x:v>
-      </x:c>
-      <x:c r="R33" s="3" t="s">
-        <x:v>800</x:v>
-      </x:c>
-      <x:c r="S33" s="3" t="s">
-        <x:v>801</x:v>
-      </x:c>
-      <x:c r="T33" s="3" t="s">
-        <x:v>802</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10800,7 +10779,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10809,22 +10788,22 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G34" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H34" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I34" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J34" s="3" t="s">
         <x:v>41</x:v>
@@ -10833,31 +10812,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>811</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>812</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>813</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10865,31 +10844,31 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>814</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>815</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>816</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>817</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G35" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H35" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I35" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J35" s="3" t="s">
         <x:v>41</x:v>
@@ -10898,31 +10877,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
+        <x:v>811</x:v>
+      </x:c>
+      <x:c r="M35" s="3" t="s">
+        <x:v>812</x:v>
+      </x:c>
+      <x:c r="N35" s="3" t="s">
+        <x:v>813</x:v>
+      </x:c>
+      <x:c r="O35" s="3" t="s">
+        <x:v>588</x:v>
+      </x:c>
+      <x:c r="P35" s="3" t="s">
+        <x:v>814</x:v>
+      </x:c>
+      <x:c r="Q35" s="3" t="s">
+        <x:v>815</x:v>
+      </x:c>
+      <x:c r="R35" s="3" t="s">
+        <x:v>816</x:v>
+      </x:c>
+      <x:c r="S35" s="3" t="s">
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="T35" s="3" t="s">
         <x:v>818</x:v>
-      </x:c>
-      <x:c r="M35" s="3" t="s">
-        <x:v>819</x:v>
-      </x:c>
-      <x:c r="N35" s="3" t="s">
-        <x:v>820</x:v>
-      </x:c>
-      <x:c r="O35" s="3" t="s">
-        <x:v>595</x:v>
-      </x:c>
-      <x:c r="P35" s="3" t="s">
-        <x:v>821</x:v>
-      </x:c>
-      <x:c r="Q35" s="3" t="s">
-        <x:v>822</x:v>
-      </x:c>
-      <x:c r="R35" s="3" t="s">
-        <x:v>823</x:v>
-      </x:c>
-      <x:c r="S35" s="3" t="s">
-        <x:v>824</x:v>
-      </x:c>
-      <x:c r="T35" s="3" t="s">
-        <x:v>825</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10930,31 +10909,31 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>826</x:v>
+        <x:v>819</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>827</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>828</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>829</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G36" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H36" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I36" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J36" s="3" t="s">
         <x:v>41</x:v>
@@ -10963,31 +10942,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
+        <x:v>823</x:v>
+      </x:c>
+      <x:c r="M36" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N36" s="3" t="s">
+        <x:v>824</x:v>
+      </x:c>
+      <x:c r="O36" s="3" t="s">
+        <x:v>825</x:v>
+      </x:c>
+      <x:c r="P36" s="3" t="s">
+        <x:v>826</x:v>
+      </x:c>
+      <x:c r="Q36" s="3" t="s">
+        <x:v>827</x:v>
+      </x:c>
+      <x:c r="R36" s="3" t="s">
+        <x:v>828</x:v>
+      </x:c>
+      <x:c r="S36" s="3" t="s">
+        <x:v>829</x:v>
+      </x:c>
+      <x:c r="T36" s="3" t="s">
         <x:v>830</x:v>
-      </x:c>
-      <x:c r="M36" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N36" s="3" t="s">
-        <x:v>831</x:v>
-      </x:c>
-      <x:c r="O36" s="3" t="s">
-        <x:v>832</x:v>
-      </x:c>
-      <x:c r="P36" s="3" t="s">
-        <x:v>833</x:v>
-      </x:c>
-      <x:c r="Q36" s="3" t="s">
-        <x:v>834</x:v>
-      </x:c>
-      <x:c r="R36" s="3" t="s">
-        <x:v>835</x:v>
-      </x:c>
-      <x:c r="S36" s="3" t="s">
-        <x:v>836</x:v>
-      </x:c>
-      <x:c r="T36" s="3" t="s">
-        <x:v>837</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10995,31 +10974,31 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>838</x:v>
+        <x:v>831</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>839</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>840</x:v>
+        <x:v>833</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>841</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G37" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H37" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I37" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J37" s="3" t="s">
         <x:v>41</x:v>
@@ -11028,31 +11007,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
+        <x:v>835</x:v>
+      </x:c>
+      <x:c r="M37" s="3" t="s">
+        <x:v>836</x:v>
+      </x:c>
+      <x:c r="N37" s="3" t="s">
+        <x:v>837</x:v>
+      </x:c>
+      <x:c r="O37" s="3" t="s">
+        <x:v>838</x:v>
+      </x:c>
+      <x:c r="P37" s="3" t="s">
+        <x:v>839</x:v>
+      </x:c>
+      <x:c r="Q37" s="3" t="s">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="R37" s="3" t="s">
+        <x:v>841</x:v>
+      </x:c>
+      <x:c r="S37" s="3" t="s">
         <x:v>842</x:v>
       </x:c>
-      <x:c r="M37" s="3" t="s">
-        <x:v>843</x:v>
-      </x:c>
-      <x:c r="N37" s="3" t="s">
-        <x:v>844</x:v>
-      </x:c>
-      <x:c r="O37" s="3" t="s">
-        <x:v>845</x:v>
-      </x:c>
-      <x:c r="P37" s="3" t="s">
-        <x:v>846</x:v>
-      </x:c>
-      <x:c r="Q37" s="3" t="s">
-        <x:v>847</x:v>
-      </x:c>
-      <x:c r="R37" s="3" t="s">
-        <x:v>848</x:v>
-      </x:c>
-      <x:c r="S37" s="3" t="s">
-        <x:v>849</x:v>
-      </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>843</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -11060,31 +11039,31 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>850</x:v>
+        <x:v>843</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>851</x:v>
+        <x:v>844</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>852</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>853</x:v>
+        <x:v>846</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G38" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H38" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I38" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J38" s="3" t="s">
         <x:v>41</x:v>
@@ -11093,31 +11072,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
+        <x:v>847</x:v>
+      </x:c>
+      <x:c r="M38" s="3" t="s">
+        <x:v>513</x:v>
+      </x:c>
+      <x:c r="N38" s="3" t="s">
+        <x:v>848</x:v>
+      </x:c>
+      <x:c r="O38" s="3" t="s">
+        <x:v>849</x:v>
+      </x:c>
+      <x:c r="P38" s="3" t="s">
+        <x:v>850</x:v>
+      </x:c>
+      <x:c r="Q38" s="3" t="s">
+        <x:v>851</x:v>
+      </x:c>
+      <x:c r="R38" s="3" t="s">
+        <x:v>852</x:v>
+      </x:c>
+      <x:c r="S38" s="3" t="s">
+        <x:v>853</x:v>
+      </x:c>
+      <x:c r="T38" s="3" t="s">
         <x:v>854</x:v>
-      </x:c>
-      <x:c r="M38" s="3" t="s">
-        <x:v>520</x:v>
-      </x:c>
-      <x:c r="N38" s="3" t="s">
-        <x:v>855</x:v>
-      </x:c>
-      <x:c r="O38" s="3" t="s">
-        <x:v>856</x:v>
-      </x:c>
-      <x:c r="P38" s="3" t="s">
-        <x:v>857</x:v>
-      </x:c>
-      <x:c r="Q38" s="3" t="s">
-        <x:v>858</x:v>
-      </x:c>
-      <x:c r="R38" s="3" t="s">
-        <x:v>859</x:v>
-      </x:c>
-      <x:c r="S38" s="3" t="s">
-        <x:v>860</x:v>
-      </x:c>
-      <x:c r="T38" s="3" t="s">
-        <x:v>861</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -11125,31 +11104,31 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>862</x:v>
+        <x:v>855</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>863</x:v>
+        <x:v>856</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>864</x:v>
+        <x:v>857</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>865</x:v>
+        <x:v>858</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G39" s="3" t="s">
-        <x:v>432</x:v>
+        <x:v>437</x:v>
       </x:c>
       <x:c r="H39" s="3" t="s">
-        <x:v>433</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="I39" s="3" t="s">
-        <x:v>434</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="J39" s="3" t="s">
         <x:v>41</x:v>
@@ -11158,31 +11137,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
+        <x:v>859</x:v>
+      </x:c>
+      <x:c r="M39" s="3" t="s">
+        <x:v>441</x:v>
+      </x:c>
+      <x:c r="N39" s="3" t="s">
+        <x:v>860</x:v>
+      </x:c>
+      <x:c r="O39" s="3" t="s">
+        <x:v>861</x:v>
+      </x:c>
+      <x:c r="P39" s="3" t="s">
+        <x:v>862</x:v>
+      </x:c>
+      <x:c r="Q39" s="3" t="s">
+        <x:v>863</x:v>
+      </x:c>
+      <x:c r="R39" s="3" t="s">
+        <x:v>864</x:v>
+      </x:c>
+      <x:c r="S39" s="3" t="s">
+        <x:v>865</x:v>
+      </x:c>
+      <x:c r="T39" s="3" t="s">
         <x:v>866</x:v>
-      </x:c>
-      <x:c r="M39" s="3" t="s">
-        <x:v>436</x:v>
-      </x:c>
-      <x:c r="N39" s="3" t="s">
-        <x:v>867</x:v>
-      </x:c>
-      <x:c r="O39" s="3" t="s">
-        <x:v>868</x:v>
-      </x:c>
-      <x:c r="P39" s="3" t="s">
-        <x:v>869</x:v>
-      </x:c>
-      <x:c r="Q39" s="3" t="s">
-        <x:v>870</x:v>
-      </x:c>
-      <x:c r="R39" s="3" t="s">
-        <x:v>871</x:v>
-      </x:c>
-      <x:c r="S39" s="3" t="s">
-        <x:v>872</x:v>
-      </x:c>
-      <x:c r="T39" s="3" t="s">
-        <x:v>873</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -11191,7 +11170,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4ae975070f7d497f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bf8183517df4b53"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-004 streaming retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra26f12b8e7fa4d27"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R525fec7d9367427c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R2b99b88183644f38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rbed96323f16e44bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb79f44cd060f4a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rc46d8898b102415f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rfba5588294bb4b1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R773f79cca795430d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1321,7 +1321,22 @@
     <x:t xml:space="preserve">As a customer, I can receive streamed agent responses.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Streaming endpoint returns structured response chunks and the UI keeps thread/composer layout stable.</x:t>
+    <x:t xml:space="preserve">QuoteEngine BFF, Agent model</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Streamed chat turns</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-005</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent state and history</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a returning customer, I can reload session state and chat history.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">BFF exposes session state and message history by session id with authorization boundaries.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:t>
@@ -1333,46 +1348,10 @@
     <x:t xml:space="preserve">No fix needed for this story from current QuoteEngine automated retest.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Composer -&gt; messages/stream -&gt; streaming agent response</x:t>
+    <x:t xml:space="preserve">Shell/session restore -&gt; AgentController sessions/messages -&gt; SessionStore</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Streaming response thread</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST messages/stream</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests stream events; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Agent model</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Streamed chat turns</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs interrupted-stream browser test</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:76</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-005</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent state and history</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a returning customer, I can reload session state and chat history.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BFF exposes session state and message history by session id with authorization boundaries.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shell/session restore -&gt; AgentController sessions/messages -&gt; SessionStore</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Session reload/history</x:t>
@@ -5183,7 +5162,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd659e5451b6047aa"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2ec510e4a734287"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8599,7 +8578,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R26783c875c8e4b25"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb9839dc17aa49fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8905,85 +8884,85 @@
       <x:c r="D5" s="3" t="s">
         <x:v>435</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="s">
-        <x:v>436</x:v>
+      <x:c r="E5" s="3" t="str">
+        <x:v>The agent stream endpoint returns newline-delimited stream events, emits incremental grounded assistant deltas before one final state response, disables proxy buffering, and falls back to a final state when the downstream chatbot stream fails.</x:v>
       </x:c>
       <x:c r="F5" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="G5" s="3" t="s">
-        <x:v>437</x:v>
-      </x:c>
-      <x:c r="H5" s="3" t="s">
-        <x:v>438</x:v>
-      </x:c>
-      <x:c r="I5" s="3" t="s">
-        <x:v>439</x:v>
-      </x:c>
-      <x:c r="J5" s="3" t="s">
-        <x:v>41</x:v>
+      <x:c r="G5" s="3" t="str">
+        <x:v>Focused current-state streaming tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H5" s="3" t="str">
+        <x:v>No behavior error observed in focused streaming retest. Interrupted live browser stream handling remains unverified.</x:v>
+      </x:c>
+      <x:c r="I5" s="3" t="str">
+        <x:v>No app fix applied for this story in this slice.</x:v>
+      </x:c>
+      <x:c r="J5" s="3" t="str">
+        <x:v>Retested QuoteAgentEndpointTests.Agent_message_stream_returns_incremental_events_before_final_state, QuoteAgentEndpointTests.Agent_message_stream_returns_fallback_final_state_when_chatbot_stream_fails, and QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract: 3/3 passed.</x:v>
       </x:c>
       <x:c r="K5" s="3" t="s">
         <x:v>188</x:v>
       </x:c>
-      <x:c r="L5" s="3" t="s">
-        <x:v>440</x:v>
-      </x:c>
-      <x:c r="M5" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N5" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="O5" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="P5" s="3" t="s">
-        <x:v>444</x:v>
+      <x:c r="L5" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell stream consumer -&gt; QuoteEngineApiClient NDJSON reader -&gt; AgentController stream endpoint -&gt; QuoteAgentService.StreamAsync -&gt; ChatbotService stream</x:v>
+      </x:c>
+      <x:c r="M5" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor HandleSubmitAsync; QuoteEngineApiClient.SendAgentMessageStreamAsync; AgentController.Stream; QuoteAgentService.StreamAsync</x:v>
+      </x:c>
+      <x:c r="N5" s="3" t="str">
+        <x:v>Composer sends through SendAgentMessageStreamAsync; stream API uses quote/v1/agent/messages/stream and reads response headers immediately.</x:v>
+      </x:c>
+      <x:c r="O5" s="3" t="str">
+        <x:v>AgentController POST quote/v1/agent/messages/stream returns application/x-ndjson, sets X-Accel-Buffering no and Cache-Control no-cache, disables response buffering, writes each QuoteAgentStreamEvent as a line, and flushes after every event. QuoteAgentService.StreamAsync emits started/thought/delta/final/error events and re-chunks grounded final assistant text.</x:v>
+      </x:c>
+      <x:c r="P5" s="3" t="str">
+        <x:v>dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_stream_returns_incremental_events_before_final_state|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_stream_returns_fallback_final_state_when_chatbot_stream_fails|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract" --verbosity minimal passed 3/3 on 2026-06-24.</x:v>
       </x:c>
       <x:c r="Q5" s="3" t="s">
-        <x:v>445</x:v>
+        <x:v>436</x:v>
       </x:c>
       <x:c r="R5" s="3" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="S5" s="3" t="s">
-        <x:v>447</x:v>
-      </x:c>
-      <x:c r="T5" s="3" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="U5" s="3" t="s">
-        <x:v>52</x:v>
+        <x:v>437</x:v>
+      </x:c>
+      <x:c r="S5" s="3" t="str">
+        <x:v>Needs interrupted-stream browser test against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T5" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor:2817-2924; QuoteEngineApiClient.cs:329-365; AgentController.cs:76-105; QuoteAgentService.cs:247-442; QuoteAgentDtos.cs:271-286; QuoteAgentEndpointTests.cs:704-744,1290-1329; QuoteEngineSourceTests.cs:864-1310</x:v>
+      </x:c>
+      <x:c r="U5" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
       <x:c r="A6" s="3" t="s">
-        <x:v>449</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="B6" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C6" s="3" t="s">
-        <x:v>450</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="D6" s="3" t="s">
-        <x:v>451</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="E6" s="3" t="s">
-        <x:v>452</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="F6" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G6" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H6" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I6" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J6" s="3" t="s">
         <x:v>41</x:v>
@@ -8992,31 +8971,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L6" s="3" t="s">
+        <x:v>445</x:v>
+      </x:c>
+      <x:c r="M6" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N6" s="3" t="s">
+        <x:v>447</x:v>
+      </x:c>
+      <x:c r="O6" s="3" t="s">
+        <x:v>448</x:v>
+      </x:c>
+      <x:c r="P6" s="3" t="s">
+        <x:v>449</x:v>
+      </x:c>
+      <x:c r="Q6" s="3" t="s">
+        <x:v>450</x:v>
+      </x:c>
+      <x:c r="R6" s="3" t="s">
+        <x:v>451</x:v>
+      </x:c>
+      <x:c r="S6" s="3" t="s">
+        <x:v>452</x:v>
+      </x:c>
+      <x:c r="T6" s="3" t="s">
         <x:v>453</x:v>
-      </x:c>
-      <x:c r="M6" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N6" s="3" t="s">
-        <x:v>454</x:v>
-      </x:c>
-      <x:c r="O6" s="3" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="P6" s="3" t="s">
-        <x:v>456</x:v>
-      </x:c>
-      <x:c r="Q6" s="3" t="s">
-        <x:v>457</x:v>
-      </x:c>
-      <x:c r="R6" s="3" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="S6" s="3" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="T6" s="3" t="s">
-        <x:v>460</x:v>
       </x:c>
       <x:c r="U6" s="3" t="s">
         <x:v>52</x:v>
@@ -9024,31 +9003,31 @@
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>461</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>462</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>463</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>464</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G7" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H7" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I7" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J7" s="3" t="s">
         <x:v>41</x:v>
@@ -9057,31 +9036,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
+        <x:v>458</x:v>
+      </x:c>
+      <x:c r="M7" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N7" s="3" t="s">
+        <x:v>459</x:v>
+      </x:c>
+      <x:c r="O7" s="3" t="s">
+        <x:v>460</x:v>
+      </x:c>
+      <x:c r="P7" s="3" t="s">
+        <x:v>461</x:v>
+      </x:c>
+      <x:c r="Q7" s="3" t="s">
+        <x:v>462</x:v>
+      </x:c>
+      <x:c r="R7" s="3" t="s">
+        <x:v>463</x:v>
+      </x:c>
+      <x:c r="S7" s="3" t="s">
+        <x:v>464</x:v>
+      </x:c>
+      <x:c r="T7" s="3" t="s">
         <x:v>465</x:v>
-      </x:c>
-      <x:c r="M7" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N7" s="3" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="O7" s="3" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="P7" s="3" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="Q7" s="3" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="R7" s="3" t="s">
-        <x:v>470</x:v>
-      </x:c>
-      <x:c r="S7" s="3" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="T7" s="3" t="s">
-        <x:v>472</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>52</x:v>
@@ -9089,31 +9068,31 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>473</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>474</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>475</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>476</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G8" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H8" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I8" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J8" s="3" t="s">
         <x:v>41</x:v>
@@ -9122,31 +9101,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
+        <x:v>470</x:v>
+      </x:c>
+      <x:c r="M8" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N8" s="3" t="s">
+        <x:v>471</x:v>
+      </x:c>
+      <x:c r="O8" s="3" t="s">
+        <x:v>472</x:v>
+      </x:c>
+      <x:c r="P8" s="3" t="s">
+        <x:v>473</x:v>
+      </x:c>
+      <x:c r="Q8" s="3" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="R8" s="3" t="s">
+        <x:v>475</x:v>
+      </x:c>
+      <x:c r="S8" s="3" t="s">
+        <x:v>476</x:v>
+      </x:c>
+      <x:c r="T8" s="3" t="s">
         <x:v>477</x:v>
-      </x:c>
-      <x:c r="M8" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N8" s="3" t="s">
-        <x:v>478</x:v>
-      </x:c>
-      <x:c r="O8" s="3" t="s">
-        <x:v>479</x:v>
-      </x:c>
-      <x:c r="P8" s="3" t="s">
-        <x:v>480</x:v>
-      </x:c>
-      <x:c r="Q8" s="3" t="s">
-        <x:v>481</x:v>
-      </x:c>
-      <x:c r="R8" s="3" t="s">
-        <x:v>482</x:v>
-      </x:c>
-      <x:c r="S8" s="3" t="s">
-        <x:v>483</x:v>
-      </x:c>
-      <x:c r="T8" s="3" t="s">
-        <x:v>484</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>52</x:v>
@@ -9154,31 +9133,31 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G9" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H9" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I9" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J9" s="3" t="s">
         <x:v>41</x:v>
@@ -9187,31 +9166,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
+        <x:v>482</x:v>
+      </x:c>
+      <x:c r="M9" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N9" s="3" t="s">
+        <x:v>483</x:v>
+      </x:c>
+      <x:c r="O9" s="3" t="s">
+        <x:v>484</x:v>
+      </x:c>
+      <x:c r="P9" s="3" t="s">
+        <x:v>485</x:v>
+      </x:c>
+      <x:c r="Q9" s="3" t="s">
+        <x:v>486</x:v>
+      </x:c>
+      <x:c r="R9" s="3" t="s">
+        <x:v>487</x:v>
+      </x:c>
+      <x:c r="S9" s="3" t="s">
+        <x:v>488</x:v>
+      </x:c>
+      <x:c r="T9" s="3" t="s">
         <x:v>489</x:v>
-      </x:c>
-      <x:c r="M9" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N9" s="3" t="s">
-        <x:v>490</x:v>
-      </x:c>
-      <x:c r="O9" s="3" t="s">
-        <x:v>491</x:v>
-      </x:c>
-      <x:c r="P9" s="3" t="s">
-        <x:v>492</x:v>
-      </x:c>
-      <x:c r="Q9" s="3" t="s">
-        <x:v>493</x:v>
-      </x:c>
-      <x:c r="R9" s="3" t="s">
-        <x:v>494</x:v>
-      </x:c>
-      <x:c r="S9" s="3" t="s">
-        <x:v>495</x:v>
-      </x:c>
-      <x:c r="T9" s="3" t="s">
-        <x:v>496</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>52</x:v>
@@ -9219,31 +9198,31 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>499</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>500</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G10" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H10" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I10" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J10" s="3" t="s">
         <x:v>41</x:v>
@@ -9252,31 +9231,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
         <x:v>424</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>52</x:v>
@@ -9284,31 +9263,31 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G11" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H11" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I11" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J11" s="3" t="s">
         <x:v>41</x:v>
@@ -9317,31 +9296,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
+        <x:v>505</x:v>
+      </x:c>
+      <x:c r="M11" s="3" t="s">
+        <x:v>506</x:v>
+      </x:c>
+      <x:c r="N11" s="3" t="s">
+        <x:v>507</x:v>
+      </x:c>
+      <x:c r="O11" s="3" t="s">
+        <x:v>508</x:v>
+      </x:c>
+      <x:c r="P11" s="3" t="s">
+        <x:v>509</x:v>
+      </x:c>
+      <x:c r="Q11" s="3" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="R11" s="3" t="s">
+        <x:v>511</x:v>
+      </x:c>
+      <x:c r="S11" s="3" t="s">
         <x:v>512</x:v>
       </x:c>
-      <x:c r="M11" s="3" t="s">
+      <x:c r="T11" s="3" t="s">
         <x:v>513</x:v>
-      </x:c>
-      <x:c r="N11" s="3" t="s">
-        <x:v>514</x:v>
-      </x:c>
-      <x:c r="O11" s="3" t="s">
-        <x:v>515</x:v>
-      </x:c>
-      <x:c r="P11" s="3" t="s">
-        <x:v>516</x:v>
-      </x:c>
-      <x:c r="Q11" s="3" t="s">
-        <x:v>517</x:v>
-      </x:c>
-      <x:c r="R11" s="3" t="s">
-        <x:v>518</x:v>
-      </x:c>
-      <x:c r="S11" s="3" t="s">
-        <x:v>519</x:v>
-      </x:c>
-      <x:c r="T11" s="3" t="s">
-        <x:v>520</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>52</x:v>
@@ -9349,31 +9328,31 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G12" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H12" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I12" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J12" s="3" t="s">
         <x:v>41</x:v>
@@ -9382,31 +9361,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
+        <x:v>518</x:v>
+      </x:c>
+      <x:c r="M12" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N12" s="3" t="s">
+        <x:v>519</x:v>
+      </x:c>
+      <x:c r="O12" s="3" t="s">
+        <x:v>520</x:v>
+      </x:c>
+      <x:c r="P12" s="3" t="s">
+        <x:v>521</x:v>
+      </x:c>
+      <x:c r="Q12" s="3" t="s">
+        <x:v>522</x:v>
+      </x:c>
+      <x:c r="R12" s="3" t="s">
+        <x:v>523</x:v>
+      </x:c>
+      <x:c r="S12" s="3" t="s">
+        <x:v>524</x:v>
+      </x:c>
+      <x:c r="T12" s="3" t="s">
         <x:v>525</x:v>
-      </x:c>
-      <x:c r="M12" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N12" s="3" t="s">
-        <x:v>526</x:v>
-      </x:c>
-      <x:c r="O12" s="3" t="s">
-        <x:v>527</x:v>
-      </x:c>
-      <x:c r="P12" s="3" t="s">
-        <x:v>528</x:v>
-      </x:c>
-      <x:c r="Q12" s="3" t="s">
-        <x:v>529</x:v>
-      </x:c>
-      <x:c r="R12" s="3" t="s">
-        <x:v>530</x:v>
-      </x:c>
-      <x:c r="S12" s="3" t="s">
-        <x:v>531</x:v>
-      </x:c>
-      <x:c r="T12" s="3" t="s">
-        <x:v>532</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>52</x:v>
@@ -9414,31 +9393,31 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>534</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G13" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H13" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I13" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J13" s="3" t="s">
         <x:v>41</x:v>
@@ -9447,31 +9426,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
-        <x:v>441</x:v>
+        <x:v>446</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>52</x:v>
@@ -9479,31 +9458,31 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G14" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H14" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I14" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J14" s="3" t="s">
         <x:v>41</x:v>
@@ -9512,31 +9491,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
+        <x:v>541</x:v>
+      </x:c>
+      <x:c r="M14" s="3" t="s">
+        <x:v>542</x:v>
+      </x:c>
+      <x:c r="N14" s="3" t="s">
+        <x:v>543</x:v>
+      </x:c>
+      <x:c r="O14" s="3" t="s">
+        <x:v>544</x:v>
+      </x:c>
+      <x:c r="P14" s="3" t="s">
+        <x:v>545</x:v>
+      </x:c>
+      <x:c r="Q14" s="3" t="s">
+        <x:v>546</x:v>
+      </x:c>
+      <x:c r="R14" s="3" t="s">
+        <x:v>547</x:v>
+      </x:c>
+      <x:c r="S14" s="3" t="s">
         <x:v>548</x:v>
       </x:c>
-      <x:c r="M14" s="3" t="s">
+      <x:c r="T14" s="3" t="s">
         <x:v>549</x:v>
-      </x:c>
-      <x:c r="N14" s="3" t="s">
-        <x:v>550</x:v>
-      </x:c>
-      <x:c r="O14" s="3" t="s">
-        <x:v>551</x:v>
-      </x:c>
-      <x:c r="P14" s="3" t="s">
-        <x:v>552</x:v>
-      </x:c>
-      <x:c r="Q14" s="3" t="s">
-        <x:v>553</x:v>
-      </x:c>
-      <x:c r="R14" s="3" t="s">
-        <x:v>554</x:v>
-      </x:c>
-      <x:c r="S14" s="3" t="s">
-        <x:v>555</x:v>
-      </x:c>
-      <x:c r="T14" s="3" t="s">
-        <x:v>556</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9544,31 +9523,31 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G15" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H15" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I15" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J15" s="3" t="s">
         <x:v>41</x:v>
@@ -9577,31 +9556,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
+        <x:v>554</x:v>
+      </x:c>
+      <x:c r="M15" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N15" s="3" t="s">
+        <x:v>555</x:v>
+      </x:c>
+      <x:c r="O15" s="3" t="s">
+        <x:v>556</x:v>
+      </x:c>
+      <x:c r="P15" s="3" t="s">
+        <x:v>557</x:v>
+      </x:c>
+      <x:c r="Q15" s="3" t="s">
+        <x:v>558</x:v>
+      </x:c>
+      <x:c r="R15" s="3" t="s">
+        <x:v>559</x:v>
+      </x:c>
+      <x:c r="S15" s="3" t="s">
+        <x:v>560</x:v>
+      </x:c>
+      <x:c r="T15" s="3" t="s">
         <x:v>561</x:v>
-      </x:c>
-      <x:c r="M15" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N15" s="3" t="s">
-        <x:v>562</x:v>
-      </x:c>
-      <x:c r="O15" s="3" t="s">
-        <x:v>563</x:v>
-      </x:c>
-      <x:c r="P15" s="3" t="s">
-        <x:v>564</x:v>
-      </x:c>
-      <x:c r="Q15" s="3" t="s">
-        <x:v>565</x:v>
-      </x:c>
-      <x:c r="R15" s="3" t="s">
-        <x:v>566</x:v>
-      </x:c>
-      <x:c r="S15" s="3" t="s">
-        <x:v>567</x:v>
-      </x:c>
-      <x:c r="T15" s="3" t="s">
-        <x:v>568</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9609,31 +9588,31 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G16" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H16" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I16" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J16" s="3" t="s">
         <x:v>41</x:v>
@@ -9642,31 +9621,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
+        <x:v>566</x:v>
+      </x:c>
+      <x:c r="M16" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N16" s="3" t="s">
+        <x:v>567</x:v>
+      </x:c>
+      <x:c r="O16" s="3" t="s">
+        <x:v>568</x:v>
+      </x:c>
+      <x:c r="P16" s="3" t="s">
+        <x:v>569</x:v>
+      </x:c>
+      <x:c r="Q16" s="3" t="s">
+        <x:v>570</x:v>
+      </x:c>
+      <x:c r="R16" s="3" t="s">
+        <x:v>571</x:v>
+      </x:c>
+      <x:c r="S16" s="3" t="s">
+        <x:v>572</x:v>
+      </x:c>
+      <x:c r="T16" s="3" t="s">
         <x:v>573</x:v>
-      </x:c>
-      <x:c r="M16" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N16" s="3" t="s">
-        <x:v>574</x:v>
-      </x:c>
-      <x:c r="O16" s="3" t="s">
-        <x:v>575</x:v>
-      </x:c>
-      <x:c r="P16" s="3" t="s">
-        <x:v>576</x:v>
-      </x:c>
-      <x:c r="Q16" s="3" t="s">
-        <x:v>577</x:v>
-      </x:c>
-      <x:c r="R16" s="3" t="s">
-        <x:v>578</x:v>
-      </x:c>
-      <x:c r="S16" s="3" t="s">
-        <x:v>579</x:v>
-      </x:c>
-      <x:c r="T16" s="3" t="s">
-        <x:v>580</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9674,31 +9653,31 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G17" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H17" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I17" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J17" s="3" t="s">
         <x:v>41</x:v>
@@ -9707,31 +9686,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
+        <x:v>578</x:v>
+      </x:c>
+      <x:c r="M17" s="3" t="s">
+        <x:v>579</x:v>
+      </x:c>
+      <x:c r="N17" s="3" t="s">
+        <x:v>580</x:v>
+      </x:c>
+      <x:c r="O17" s="3" t="s">
+        <x:v>581</x:v>
+      </x:c>
+      <x:c r="P17" s="3" t="s">
+        <x:v>582</x:v>
+      </x:c>
+      <x:c r="Q17" s="3" t="s">
+        <x:v>583</x:v>
+      </x:c>
+      <x:c r="R17" s="3" t="s">
+        <x:v>584</x:v>
+      </x:c>
+      <x:c r="S17" s="3" t="s">
         <x:v>585</x:v>
       </x:c>
-      <x:c r="M17" s="3" t="s">
+      <x:c r="T17" s="3" t="s">
         <x:v>586</x:v>
-      </x:c>
-      <x:c r="N17" s="3" t="s">
-        <x:v>587</x:v>
-      </x:c>
-      <x:c r="O17" s="3" t="s">
-        <x:v>588</x:v>
-      </x:c>
-      <x:c r="P17" s="3" t="s">
-        <x:v>589</x:v>
-      </x:c>
-      <x:c r="Q17" s="3" t="s">
-        <x:v>590</x:v>
-      </x:c>
-      <x:c r="R17" s="3" t="s">
-        <x:v>591</x:v>
-      </x:c>
-      <x:c r="S17" s="3" t="s">
-        <x:v>592</x:v>
-      </x:c>
-      <x:c r="T17" s="3" t="s">
-        <x:v>593</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9739,31 +9718,31 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G18" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H18" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I18" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J18" s="3" t="s">
         <x:v>41</x:v>
@@ -9772,31 +9751,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
+        <x:v>591</x:v>
+      </x:c>
+      <x:c r="M18" s="3" t="s">
+        <x:v>592</x:v>
+      </x:c>
+      <x:c r="N18" s="3" t="s">
+        <x:v>593</x:v>
+      </x:c>
+      <x:c r="O18" s="3" t="s">
+        <x:v>594</x:v>
+      </x:c>
+      <x:c r="P18" s="3" t="s">
+        <x:v>595</x:v>
+      </x:c>
+      <x:c r="Q18" s="3" t="s">
+        <x:v>596</x:v>
+      </x:c>
+      <x:c r="R18" s="3" t="s">
+        <x:v>597</x:v>
+      </x:c>
+      <x:c r="S18" s="3" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="M18" s="3" t="s">
+      <x:c r="T18" s="3" t="s">
         <x:v>599</x:v>
-      </x:c>
-      <x:c r="N18" s="3" t="s">
-        <x:v>600</x:v>
-      </x:c>
-      <x:c r="O18" s="3" t="s">
-        <x:v>601</x:v>
-      </x:c>
-      <x:c r="P18" s="3" t="s">
-        <x:v>602</x:v>
-      </x:c>
-      <x:c r="Q18" s="3" t="s">
-        <x:v>603</x:v>
-      </x:c>
-      <x:c r="R18" s="3" t="s">
-        <x:v>604</x:v>
-      </x:c>
-      <x:c r="S18" s="3" t="s">
-        <x:v>605</x:v>
-      </x:c>
-      <x:c r="T18" s="3" t="s">
-        <x:v>606</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9804,31 +9783,31 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G19" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H19" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I19" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J19" s="3" t="s">
         <x:v>41</x:v>
@@ -9837,31 +9816,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
+        <x:v>604</x:v>
+      </x:c>
+      <x:c r="M19" s="3" t="s">
+        <x:v>605</x:v>
+      </x:c>
+      <x:c r="N19" s="3" t="s">
+        <x:v>606</x:v>
+      </x:c>
+      <x:c r="O19" s="3" t="s">
+        <x:v>607</x:v>
+      </x:c>
+      <x:c r="P19" s="3" t="s">
+        <x:v>608</x:v>
+      </x:c>
+      <x:c r="Q19" s="3" t="s">
+        <x:v>609</x:v>
+      </x:c>
+      <x:c r="R19" s="3" t="s">
+        <x:v>610</x:v>
+      </x:c>
+      <x:c r="S19" s="3" t="s">
         <x:v>611</x:v>
       </x:c>
-      <x:c r="M19" s="3" t="s">
+      <x:c r="T19" s="3" t="s">
         <x:v>612</x:v>
-      </x:c>
-      <x:c r="N19" s="3" t="s">
-        <x:v>613</x:v>
-      </x:c>
-      <x:c r="O19" s="3" t="s">
-        <x:v>614</x:v>
-      </x:c>
-      <x:c r="P19" s="3" t="s">
-        <x:v>615</x:v>
-      </x:c>
-      <x:c r="Q19" s="3" t="s">
-        <x:v>616</x:v>
-      </x:c>
-      <x:c r="R19" s="3" t="s">
-        <x:v>617</x:v>
-      </x:c>
-      <x:c r="S19" s="3" t="s">
-        <x:v>618</x:v>
-      </x:c>
-      <x:c r="T19" s="3" t="s">
-        <x:v>619</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9869,31 +9848,31 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G20" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H20" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I20" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J20" s="3" t="s">
         <x:v>41</x:v>
@@ -9902,31 +9881,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
+        <x:v>617</x:v>
+      </x:c>
+      <x:c r="M20" s="3" t="s">
+        <x:v>618</x:v>
+      </x:c>
+      <x:c r="N20" s="3" t="s">
+        <x:v>619</x:v>
+      </x:c>
+      <x:c r="O20" s="3" t="s">
+        <x:v>620</x:v>
+      </x:c>
+      <x:c r="P20" s="3" t="s">
+        <x:v>621</x:v>
+      </x:c>
+      <x:c r="Q20" s="3" t="s">
+        <x:v>622</x:v>
+      </x:c>
+      <x:c r="R20" s="3" t="s">
+        <x:v>623</x:v>
+      </x:c>
+      <x:c r="S20" s="3" t="s">
         <x:v>624</x:v>
       </x:c>
-      <x:c r="M20" s="3" t="s">
+      <x:c r="T20" s="3" t="s">
         <x:v>625</x:v>
-      </x:c>
-      <x:c r="N20" s="3" t="s">
-        <x:v>626</x:v>
-      </x:c>
-      <x:c r="O20" s="3" t="s">
-        <x:v>627</x:v>
-      </x:c>
-      <x:c r="P20" s="3" t="s">
-        <x:v>628</x:v>
-      </x:c>
-      <x:c r="Q20" s="3" t="s">
-        <x:v>629</x:v>
-      </x:c>
-      <x:c r="R20" s="3" t="s">
-        <x:v>630</x:v>
-      </x:c>
-      <x:c r="S20" s="3" t="s">
-        <x:v>631</x:v>
-      </x:c>
-      <x:c r="T20" s="3" t="s">
-        <x:v>632</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9934,31 +9913,31 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G21" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H21" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I21" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J21" s="3" t="s">
         <x:v>41</x:v>
@@ -9967,31 +9946,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -9999,31 +9978,31 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G22" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H22" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I22" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J22" s="3" t="s">
         <x:v>41</x:v>
@@ -10032,31 +10011,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
+        <x:v>641</x:v>
+      </x:c>
+      <x:c r="M22" s="3" t="s">
+        <x:v>506</x:v>
+      </x:c>
+      <x:c r="N22" s="3" t="s">
+        <x:v>642</x:v>
+      </x:c>
+      <x:c r="O22" s="3" t="s">
+        <x:v>643</x:v>
+      </x:c>
+      <x:c r="P22" s="3" t="s">
+        <x:v>644</x:v>
+      </x:c>
+      <x:c r="Q22" s="3" t="s">
+        <x:v>645</x:v>
+      </x:c>
+      <x:c r="R22" s="3" t="s">
+        <x:v>646</x:v>
+      </x:c>
+      <x:c r="S22" s="3" t="s">
+        <x:v>647</x:v>
+      </x:c>
+      <x:c r="T22" s="3" t="s">
         <x:v>648</x:v>
-      </x:c>
-      <x:c r="M22" s="3" t="s">
-        <x:v>513</x:v>
-      </x:c>
-      <x:c r="N22" s="3" t="s">
-        <x:v>649</x:v>
-      </x:c>
-      <x:c r="O22" s="3" t="s">
-        <x:v>650</x:v>
-      </x:c>
-      <x:c r="P22" s="3" t="s">
-        <x:v>651</x:v>
-      </x:c>
-      <x:c r="Q22" s="3" t="s">
-        <x:v>652</x:v>
-      </x:c>
-      <x:c r="R22" s="3" t="s">
-        <x:v>653</x:v>
-      </x:c>
-      <x:c r="S22" s="3" t="s">
-        <x:v>654</x:v>
-      </x:c>
-      <x:c r="T22" s="3" t="s">
-        <x:v>655</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -10064,31 +10043,31 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G23" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H23" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I23" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J23" s="3" t="s">
         <x:v>41</x:v>
@@ -10097,31 +10076,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
+        <x:v>653</x:v>
+      </x:c>
+      <x:c r="M23" s="3" t="s">
+        <x:v>654</x:v>
+      </x:c>
+      <x:c r="N23" s="3" t="s">
+        <x:v>655</x:v>
+      </x:c>
+      <x:c r="O23" s="3" t="s">
+        <x:v>656</x:v>
+      </x:c>
+      <x:c r="P23" s="3" t="s">
+        <x:v>657</x:v>
+      </x:c>
+      <x:c r="Q23" s="3" t="s">
+        <x:v>658</x:v>
+      </x:c>
+      <x:c r="R23" s="3" t="s">
+        <x:v>659</x:v>
+      </x:c>
+      <x:c r="S23" s="3" t="s">
         <x:v>660</x:v>
       </x:c>
-      <x:c r="M23" s="3" t="s">
+      <x:c r="T23" s="3" t="s">
         <x:v>661</x:v>
-      </x:c>
-      <x:c r="N23" s="3" t="s">
-        <x:v>662</x:v>
-      </x:c>
-      <x:c r="O23" s="3" t="s">
-        <x:v>663</x:v>
-      </x:c>
-      <x:c r="P23" s="3" t="s">
-        <x:v>664</x:v>
-      </x:c>
-      <x:c r="Q23" s="3" t="s">
-        <x:v>665</x:v>
-      </x:c>
-      <x:c r="R23" s="3" t="s">
-        <x:v>666</x:v>
-      </x:c>
-      <x:c r="S23" s="3" t="s">
-        <x:v>667</x:v>
-      </x:c>
-      <x:c r="T23" s="3" t="s">
-        <x:v>668</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -10129,31 +10108,31 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G24" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H24" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I24" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J24" s="3" t="s">
         <x:v>41</x:v>
@@ -10162,31 +10141,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
+        <x:v>666</x:v>
+      </x:c>
+      <x:c r="M24" s="3" t="s">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="N24" s="3" t="s">
+        <x:v>667</x:v>
+      </x:c>
+      <x:c r="O24" s="3" t="s">
+        <x:v>668</x:v>
+      </x:c>
+      <x:c r="P24" s="3" t="s">
+        <x:v>669</x:v>
+      </x:c>
+      <x:c r="Q24" s="3" t="s">
+        <x:v>670</x:v>
+      </x:c>
+      <x:c r="R24" s="3" t="s">
+        <x:v>671</x:v>
+      </x:c>
+      <x:c r="S24" s="3" t="s">
+        <x:v>672</x:v>
+      </x:c>
+      <x:c r="T24" s="3" t="s">
         <x:v>673</x:v>
-      </x:c>
-      <x:c r="M24" s="3" t="s">
-        <x:v>638</x:v>
-      </x:c>
-      <x:c r="N24" s="3" t="s">
-        <x:v>674</x:v>
-      </x:c>
-      <x:c r="O24" s="3" t="s">
-        <x:v>675</x:v>
-      </x:c>
-      <x:c r="P24" s="3" t="s">
-        <x:v>676</x:v>
-      </x:c>
-      <x:c r="Q24" s="3" t="s">
-        <x:v>677</x:v>
-      </x:c>
-      <x:c r="R24" s="3" t="s">
-        <x:v>678</x:v>
-      </x:c>
-      <x:c r="S24" s="3" t="s">
-        <x:v>679</x:v>
-      </x:c>
-      <x:c r="T24" s="3" t="s">
-        <x:v>680</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -10194,31 +10173,31 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G25" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H25" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I25" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J25" s="3" t="s">
         <x:v>41</x:v>
@@ -10227,31 +10206,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
+        <x:v>678</x:v>
+      </x:c>
+      <x:c r="M25" s="3" t="s">
+        <x:v>631</x:v>
+      </x:c>
+      <x:c r="N25" s="3" t="s">
+        <x:v>679</x:v>
+      </x:c>
+      <x:c r="O25" s="3" t="s">
+        <x:v>680</x:v>
+      </x:c>
+      <x:c r="P25" s="3" t="s">
+        <x:v>681</x:v>
+      </x:c>
+      <x:c r="Q25" s="3" t="s">
+        <x:v>682</x:v>
+      </x:c>
+      <x:c r="R25" s="3" t="s">
+        <x:v>683</x:v>
+      </x:c>
+      <x:c r="S25" s="3" t="s">
+        <x:v>684</x:v>
+      </x:c>
+      <x:c r="T25" s="3" t="s">
         <x:v>685</x:v>
-      </x:c>
-      <x:c r="M25" s="3" t="s">
-        <x:v>638</x:v>
-      </x:c>
-      <x:c r="N25" s="3" t="s">
-        <x:v>686</x:v>
-      </x:c>
-      <x:c r="O25" s="3" t="s">
-        <x:v>687</x:v>
-      </x:c>
-      <x:c r="P25" s="3" t="s">
-        <x:v>688</x:v>
-      </x:c>
-      <x:c r="Q25" s="3" t="s">
-        <x:v>689</x:v>
-      </x:c>
-      <x:c r="R25" s="3" t="s">
-        <x:v>690</x:v>
-      </x:c>
-      <x:c r="S25" s="3" t="s">
-        <x:v>691</x:v>
-      </x:c>
-      <x:c r="T25" s="3" t="s">
-        <x:v>692</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10259,31 +10238,31 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G26" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H26" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I26" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J26" s="3" t="s">
         <x:v>41</x:v>
@@ -10292,31 +10271,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
+        <x:v>690</x:v>
+      </x:c>
+      <x:c r="M26" s="3" t="s">
+        <x:v>691</x:v>
+      </x:c>
+      <x:c r="N26" s="3" t="s">
+        <x:v>692</x:v>
+      </x:c>
+      <x:c r="O26" s="3" t="s">
+        <x:v>693</x:v>
+      </x:c>
+      <x:c r="P26" s="3" t="s">
+        <x:v>694</x:v>
+      </x:c>
+      <x:c r="Q26" s="3" t="s">
+        <x:v>695</x:v>
+      </x:c>
+      <x:c r="R26" s="3" t="s">
+        <x:v>696</x:v>
+      </x:c>
+      <x:c r="S26" s="3" t="s">
         <x:v>697</x:v>
       </x:c>
-      <x:c r="M26" s="3" t="s">
+      <x:c r="T26" s="3" t="s">
         <x:v>698</x:v>
-      </x:c>
-      <x:c r="N26" s="3" t="s">
-        <x:v>699</x:v>
-      </x:c>
-      <x:c r="O26" s="3" t="s">
-        <x:v>700</x:v>
-      </x:c>
-      <x:c r="P26" s="3" t="s">
-        <x:v>701</x:v>
-      </x:c>
-      <x:c r="Q26" s="3" t="s">
-        <x:v>702</x:v>
-      </x:c>
-      <x:c r="R26" s="3" t="s">
-        <x:v>703</x:v>
-      </x:c>
-      <x:c r="S26" s="3" t="s">
-        <x:v>704</x:v>
-      </x:c>
-      <x:c r="T26" s="3" t="s">
-        <x:v>705</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10324,31 +10303,31 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G27" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H27" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I27" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J27" s="3" t="s">
         <x:v>41</x:v>
@@ -10357,31 +10336,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
+        <x:v>703</x:v>
+      </x:c>
+      <x:c r="M27" s="3" t="s">
+        <x:v>704</x:v>
+      </x:c>
+      <x:c r="N27" s="3" t="s">
+        <x:v>705</x:v>
+      </x:c>
+      <x:c r="O27" s="3" t="s">
+        <x:v>706</x:v>
+      </x:c>
+      <x:c r="P27" s="3" t="s">
+        <x:v>707</x:v>
+      </x:c>
+      <x:c r="Q27" s="3" t="s">
+        <x:v>708</x:v>
+      </x:c>
+      <x:c r="R27" s="3" t="s">
+        <x:v>709</x:v>
+      </x:c>
+      <x:c r="S27" s="3" t="s">
         <x:v>710</x:v>
       </x:c>
-      <x:c r="M27" s="3" t="s">
+      <x:c r="T27" s="3" t="s">
         <x:v>711</x:v>
-      </x:c>
-      <x:c r="N27" s="3" t="s">
-        <x:v>712</x:v>
-      </x:c>
-      <x:c r="O27" s="3" t="s">
-        <x:v>713</x:v>
-      </x:c>
-      <x:c r="P27" s="3" t="s">
-        <x:v>714</x:v>
-      </x:c>
-      <x:c r="Q27" s="3" t="s">
-        <x:v>715</x:v>
-      </x:c>
-      <x:c r="R27" s="3" t="s">
-        <x:v>716</x:v>
-      </x:c>
-      <x:c r="S27" s="3" t="s">
-        <x:v>717</x:v>
-      </x:c>
-      <x:c r="T27" s="3" t="s">
-        <x:v>718</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10389,31 +10368,31 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G28" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H28" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I28" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J28" s="3" t="s">
         <x:v>41</x:v>
@@ -10422,31 +10401,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10454,31 +10433,31 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G29" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H29" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I29" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J29" s="3" t="s">
         <x:v>41</x:v>
@@ -10487,31 +10466,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
+        <x:v>728</x:v>
+      </x:c>
+      <x:c r="M29" s="3" t="s">
+        <x:v>729</x:v>
+      </x:c>
+      <x:c r="N29" s="3" t="s">
+        <x:v>730</x:v>
+      </x:c>
+      <x:c r="O29" s="3" t="s">
+        <x:v>731</x:v>
+      </x:c>
+      <x:c r="P29" s="3" t="s">
+        <x:v>732</x:v>
+      </x:c>
+      <x:c r="Q29" s="3" t="s">
+        <x:v>733</x:v>
+      </x:c>
+      <x:c r="R29" s="3" t="s">
+        <x:v>734</x:v>
+      </x:c>
+      <x:c r="S29" s="3" t="s">
         <x:v>735</x:v>
       </x:c>
-      <x:c r="M29" s="3" t="s">
+      <x:c r="T29" s="3" t="s">
         <x:v>736</x:v>
-      </x:c>
-      <x:c r="N29" s="3" t="s">
-        <x:v>737</x:v>
-      </x:c>
-      <x:c r="O29" s="3" t="s">
-        <x:v>738</x:v>
-      </x:c>
-      <x:c r="P29" s="3" t="s">
-        <x:v>739</x:v>
-      </x:c>
-      <x:c r="Q29" s="3" t="s">
-        <x:v>740</x:v>
-      </x:c>
-      <x:c r="R29" s="3" t="s">
-        <x:v>741</x:v>
-      </x:c>
-      <x:c r="S29" s="3" t="s">
-        <x:v>742</x:v>
-      </x:c>
-      <x:c r="T29" s="3" t="s">
-        <x:v>743</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10519,31 +10498,31 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G30" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H30" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I30" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J30" s="3" t="s">
         <x:v>41</x:v>
@@ -10552,31 +10531,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
+        <x:v>741</x:v>
+      </x:c>
+      <x:c r="M30" s="3" t="s">
+        <x:v>742</x:v>
+      </x:c>
+      <x:c r="N30" s="3" t="s">
+        <x:v>743</x:v>
+      </x:c>
+      <x:c r="O30" s="3" t="s">
+        <x:v>744</x:v>
+      </x:c>
+      <x:c r="P30" s="3" t="s">
+        <x:v>745</x:v>
+      </x:c>
+      <x:c r="Q30" s="3" t="s">
+        <x:v>746</x:v>
+      </x:c>
+      <x:c r="R30" s="3" t="s">
+        <x:v>747</x:v>
+      </x:c>
+      <x:c r="S30" s="3" t="s">
         <x:v>748</x:v>
       </x:c>
-      <x:c r="M30" s="3" t="s">
+      <x:c r="T30" s="3" t="s">
         <x:v>749</x:v>
-      </x:c>
-      <x:c r="N30" s="3" t="s">
-        <x:v>750</x:v>
-      </x:c>
-      <x:c r="O30" s="3" t="s">
-        <x:v>751</x:v>
-      </x:c>
-      <x:c r="P30" s="3" t="s">
-        <x:v>752</x:v>
-      </x:c>
-      <x:c r="Q30" s="3" t="s">
-        <x:v>753</x:v>
-      </x:c>
-      <x:c r="R30" s="3" t="s">
-        <x:v>754</x:v>
-      </x:c>
-      <x:c r="S30" s="3" t="s">
-        <x:v>755</x:v>
-      </x:c>
-      <x:c r="T30" s="3" t="s">
-        <x:v>756</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10584,31 +10563,31 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G31" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H31" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I31" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J31" s="3" t="s">
         <x:v>41</x:v>
@@ -10617,31 +10596,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
+        <x:v>754</x:v>
+      </x:c>
+      <x:c r="M31" s="3" t="s">
+        <x:v>755</x:v>
+      </x:c>
+      <x:c r="N31" s="3" t="s">
+        <x:v>756</x:v>
+      </x:c>
+      <x:c r="O31" s="3" t="s">
+        <x:v>757</x:v>
+      </x:c>
+      <x:c r="P31" s="3" t="s">
+        <x:v>758</x:v>
+      </x:c>
+      <x:c r="Q31" s="3" t="s">
+        <x:v>759</x:v>
+      </x:c>
+      <x:c r="R31" s="3" t="s">
+        <x:v>760</x:v>
+      </x:c>
+      <x:c r="S31" s="3" t="s">
         <x:v>761</x:v>
       </x:c>
-      <x:c r="M31" s="3" t="s">
+      <x:c r="T31" s="3" t="s">
         <x:v>762</x:v>
-      </x:c>
-      <x:c r="N31" s="3" t="s">
-        <x:v>763</x:v>
-      </x:c>
-      <x:c r="O31" s="3" t="s">
-        <x:v>764</x:v>
-      </x:c>
-      <x:c r="P31" s="3" t="s">
-        <x:v>765</x:v>
-      </x:c>
-      <x:c r="Q31" s="3" t="s">
-        <x:v>766</x:v>
-      </x:c>
-      <x:c r="R31" s="3" t="s">
-        <x:v>767</x:v>
-      </x:c>
-      <x:c r="S31" s="3" t="s">
-        <x:v>768</x:v>
-      </x:c>
-      <x:c r="T31" s="3" t="s">
-        <x:v>769</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10649,31 +10628,31 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G32" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H32" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I32" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J32" s="3" t="s">
         <x:v>41</x:v>
@@ -10682,31 +10661,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
+        <x:v>767</x:v>
+      </x:c>
+      <x:c r="M32" s="3" t="s">
+        <x:v>768</x:v>
+      </x:c>
+      <x:c r="N32" s="3" t="s">
+        <x:v>769</x:v>
+      </x:c>
+      <x:c r="O32" s="3" t="s">
+        <x:v>770</x:v>
+      </x:c>
+      <x:c r="P32" s="3" t="s">
+        <x:v>771</x:v>
+      </x:c>
+      <x:c r="Q32" s="3" t="s">
+        <x:v>772</x:v>
+      </x:c>
+      <x:c r="R32" s="3" t="s">
+        <x:v>773</x:v>
+      </x:c>
+      <x:c r="S32" s="3" t="s">
         <x:v>774</x:v>
       </x:c>
-      <x:c r="M32" s="3" t="s">
+      <x:c r="T32" s="3" t="s">
         <x:v>775</x:v>
-      </x:c>
-      <x:c r="N32" s="3" t="s">
-        <x:v>776</x:v>
-      </x:c>
-      <x:c r="O32" s="3" t="s">
-        <x:v>777</x:v>
-      </x:c>
-      <x:c r="P32" s="3" t="s">
-        <x:v>778</x:v>
-      </x:c>
-      <x:c r="Q32" s="3" t="s">
-        <x:v>779</x:v>
-      </x:c>
-      <x:c r="R32" s="3" t="s">
-        <x:v>780</x:v>
-      </x:c>
-      <x:c r="S32" s="3" t="s">
-        <x:v>781</x:v>
-      </x:c>
-      <x:c r="T32" s="3" t="s">
-        <x:v>782</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10714,31 +10693,31 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G33" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H33" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I33" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J33" s="3" t="s">
         <x:v>41</x:v>
@@ -10747,31 +10726,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
+        <x:v>780</x:v>
+      </x:c>
+      <x:c r="M33" s="3" t="s">
+        <x:v>781</x:v>
+      </x:c>
+      <x:c r="N33" s="3" t="s">
+        <x:v>782</x:v>
+      </x:c>
+      <x:c r="O33" s="3" t="s">
+        <x:v>783</x:v>
+      </x:c>
+      <x:c r="P33" s="3" t="s">
+        <x:v>784</x:v>
+      </x:c>
+      <x:c r="Q33" s="3" t="s">
+        <x:v>785</x:v>
+      </x:c>
+      <x:c r="R33" s="3" t="s">
+        <x:v>786</x:v>
+      </x:c>
+      <x:c r="S33" s="3" t="s">
         <x:v>787</x:v>
       </x:c>
-      <x:c r="M33" s="3" t="s">
+      <x:c r="T33" s="3" t="s">
         <x:v>788</x:v>
-      </x:c>
-      <x:c r="N33" s="3" t="s">
-        <x:v>789</x:v>
-      </x:c>
-      <x:c r="O33" s="3" t="s">
-        <x:v>790</x:v>
-      </x:c>
-      <x:c r="P33" s="3" t="s">
-        <x:v>791</x:v>
-      </x:c>
-      <x:c r="Q33" s="3" t="s">
-        <x:v>792</x:v>
-      </x:c>
-      <x:c r="R33" s="3" t="s">
-        <x:v>793</x:v>
-      </x:c>
-      <x:c r="S33" s="3" t="s">
-        <x:v>794</x:v>
-      </x:c>
-      <x:c r="T33" s="3" t="s">
-        <x:v>795</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10779,7 +10758,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10788,22 +10767,22 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G34" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H34" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I34" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J34" s="3" t="s">
         <x:v>41</x:v>
@@ -10812,31 +10791,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>802</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10844,31 +10823,31 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G35" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H35" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I35" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J35" s="3" t="s">
         <x:v>41</x:v>
@@ -10877,31 +10856,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
+        <x:v>804</x:v>
+      </x:c>
+      <x:c r="M35" s="3" t="s">
+        <x:v>805</x:v>
+      </x:c>
+      <x:c r="N35" s="3" t="s">
+        <x:v>806</x:v>
+      </x:c>
+      <x:c r="O35" s="3" t="s">
+        <x:v>581</x:v>
+      </x:c>
+      <x:c r="P35" s="3" t="s">
+        <x:v>807</x:v>
+      </x:c>
+      <x:c r="Q35" s="3" t="s">
+        <x:v>808</x:v>
+      </x:c>
+      <x:c r="R35" s="3" t="s">
+        <x:v>809</x:v>
+      </x:c>
+      <x:c r="S35" s="3" t="s">
+        <x:v>810</x:v>
+      </x:c>
+      <x:c r="T35" s="3" t="s">
         <x:v>811</x:v>
-      </x:c>
-      <x:c r="M35" s="3" t="s">
-        <x:v>812</x:v>
-      </x:c>
-      <x:c r="N35" s="3" t="s">
-        <x:v>813</x:v>
-      </x:c>
-      <x:c r="O35" s="3" t="s">
-        <x:v>588</x:v>
-      </x:c>
-      <x:c r="P35" s="3" t="s">
-        <x:v>814</x:v>
-      </x:c>
-      <x:c r="Q35" s="3" t="s">
-        <x:v>815</x:v>
-      </x:c>
-      <x:c r="R35" s="3" t="s">
-        <x:v>816</x:v>
-      </x:c>
-      <x:c r="S35" s="3" t="s">
-        <x:v>817</x:v>
-      </x:c>
-      <x:c r="T35" s="3" t="s">
-        <x:v>818</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10909,31 +10888,31 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>819</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>820</x:v>
+        <x:v>813</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>821</x:v>
+        <x:v>814</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>822</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G36" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H36" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I36" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J36" s="3" t="s">
         <x:v>41</x:v>
@@ -10942,31 +10921,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
+        <x:v>816</x:v>
+      </x:c>
+      <x:c r="M36" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N36" s="3" t="s">
+        <x:v>817</x:v>
+      </x:c>
+      <x:c r="O36" s="3" t="s">
+        <x:v>818</x:v>
+      </x:c>
+      <x:c r="P36" s="3" t="s">
+        <x:v>819</x:v>
+      </x:c>
+      <x:c r="Q36" s="3" t="s">
+        <x:v>820</x:v>
+      </x:c>
+      <x:c r="R36" s="3" t="s">
+        <x:v>821</x:v>
+      </x:c>
+      <x:c r="S36" s="3" t="s">
+        <x:v>822</x:v>
+      </x:c>
+      <x:c r="T36" s="3" t="s">
         <x:v>823</x:v>
-      </x:c>
-      <x:c r="M36" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N36" s="3" t="s">
-        <x:v>824</x:v>
-      </x:c>
-      <x:c r="O36" s="3" t="s">
-        <x:v>825</x:v>
-      </x:c>
-      <x:c r="P36" s="3" t="s">
-        <x:v>826</x:v>
-      </x:c>
-      <x:c r="Q36" s="3" t="s">
-        <x:v>827</x:v>
-      </x:c>
-      <x:c r="R36" s="3" t="s">
-        <x:v>828</x:v>
-      </x:c>
-      <x:c r="S36" s="3" t="s">
-        <x:v>829</x:v>
-      </x:c>
-      <x:c r="T36" s="3" t="s">
-        <x:v>830</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10974,31 +10953,31 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>831</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>832</x:v>
+        <x:v>825</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>833</x:v>
+        <x:v>826</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>834</x:v>
+        <x:v>827</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G37" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H37" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I37" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J37" s="3" t="s">
         <x:v>41</x:v>
@@ -11007,31 +10986,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
+        <x:v>828</x:v>
+      </x:c>
+      <x:c r="M37" s="3" t="s">
+        <x:v>829</x:v>
+      </x:c>
+      <x:c r="N37" s="3" t="s">
+        <x:v>830</x:v>
+      </x:c>
+      <x:c r="O37" s="3" t="s">
+        <x:v>831</x:v>
+      </x:c>
+      <x:c r="P37" s="3" t="s">
+        <x:v>832</x:v>
+      </x:c>
+      <x:c r="Q37" s="3" t="s">
+        <x:v>833</x:v>
+      </x:c>
+      <x:c r="R37" s="3" t="s">
+        <x:v>834</x:v>
+      </x:c>
+      <x:c r="S37" s="3" t="s">
         <x:v>835</x:v>
       </x:c>
-      <x:c r="M37" s="3" t="s">
-        <x:v>836</x:v>
-      </x:c>
-      <x:c r="N37" s="3" t="s">
-        <x:v>837</x:v>
-      </x:c>
-      <x:c r="O37" s="3" t="s">
-        <x:v>838</x:v>
-      </x:c>
-      <x:c r="P37" s="3" t="s">
-        <x:v>839</x:v>
-      </x:c>
-      <x:c r="Q37" s="3" t="s">
-        <x:v>840</x:v>
-      </x:c>
-      <x:c r="R37" s="3" t="s">
-        <x:v>841</x:v>
-      </x:c>
-      <x:c r="S37" s="3" t="s">
-        <x:v>842</x:v>
-      </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>836</x:v>
+        <x:v>829</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -11039,31 +11018,31 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>843</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>844</x:v>
+        <x:v>837</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>845</x:v>
+        <x:v>838</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>846</x:v>
+        <x:v>839</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G38" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H38" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I38" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J38" s="3" t="s">
         <x:v>41</x:v>
@@ -11072,31 +11051,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
+        <x:v>840</x:v>
+      </x:c>
+      <x:c r="M38" s="3" t="s">
+        <x:v>506</x:v>
+      </x:c>
+      <x:c r="N38" s="3" t="s">
+        <x:v>841</x:v>
+      </x:c>
+      <x:c r="O38" s="3" t="s">
+        <x:v>842</x:v>
+      </x:c>
+      <x:c r="P38" s="3" t="s">
+        <x:v>843</x:v>
+      </x:c>
+      <x:c r="Q38" s="3" t="s">
+        <x:v>844</x:v>
+      </x:c>
+      <x:c r="R38" s="3" t="s">
+        <x:v>845</x:v>
+      </x:c>
+      <x:c r="S38" s="3" t="s">
+        <x:v>846</x:v>
+      </x:c>
+      <x:c r="T38" s="3" t="s">
         <x:v>847</x:v>
-      </x:c>
-      <x:c r="M38" s="3" t="s">
-        <x:v>513</x:v>
-      </x:c>
-      <x:c r="N38" s="3" t="s">
-        <x:v>848</x:v>
-      </x:c>
-      <x:c r="O38" s="3" t="s">
-        <x:v>849</x:v>
-      </x:c>
-      <x:c r="P38" s="3" t="s">
-        <x:v>850</x:v>
-      </x:c>
-      <x:c r="Q38" s="3" t="s">
-        <x:v>851</x:v>
-      </x:c>
-      <x:c r="R38" s="3" t="s">
-        <x:v>852</x:v>
-      </x:c>
-      <x:c r="S38" s="3" t="s">
-        <x:v>853</x:v>
-      </x:c>
-      <x:c r="T38" s="3" t="s">
-        <x:v>854</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -11104,31 +11083,31 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>855</x:v>
+        <x:v>848</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>856</x:v>
+        <x:v>849</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>857</x:v>
+        <x:v>850</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>858</x:v>
+        <x:v>851</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
       </x:c>
       <x:c r="G39" s="3" t="s">
-        <x:v>437</x:v>
+        <x:v>442</x:v>
       </x:c>
       <x:c r="H39" s="3" t="s">
-        <x:v>438</x:v>
+        <x:v>443</x:v>
       </x:c>
       <x:c r="I39" s="3" t="s">
-        <x:v>439</x:v>
+        <x:v>444</x:v>
       </x:c>
       <x:c r="J39" s="3" t="s">
         <x:v>41</x:v>
@@ -11137,31 +11116,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
+        <x:v>852</x:v>
+      </x:c>
+      <x:c r="M39" s="3" t="s">
+        <x:v>446</x:v>
+      </x:c>
+      <x:c r="N39" s="3" t="s">
+        <x:v>853</x:v>
+      </x:c>
+      <x:c r="O39" s="3" t="s">
+        <x:v>854</x:v>
+      </x:c>
+      <x:c r="P39" s="3" t="s">
+        <x:v>855</x:v>
+      </x:c>
+      <x:c r="Q39" s="3" t="s">
+        <x:v>856</x:v>
+      </x:c>
+      <x:c r="R39" s="3" t="s">
+        <x:v>857</x:v>
+      </x:c>
+      <x:c r="S39" s="3" t="s">
+        <x:v>858</x:v>
+      </x:c>
+      <x:c r="T39" s="3" t="s">
         <x:v>859</x:v>
-      </x:c>
-      <x:c r="M39" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="N39" s="3" t="s">
-        <x:v>860</x:v>
-      </x:c>
-      <x:c r="O39" s="3" t="s">
-        <x:v>861</x:v>
-      </x:c>
-      <x:c r="P39" s="3" t="s">
-        <x:v>862</x:v>
-      </x:c>
-      <x:c r="Q39" s="3" t="s">
-        <x:v>863</x:v>
-      </x:c>
-      <x:c r="R39" s="3" t="s">
-        <x:v>864</x:v>
-      </x:c>
-      <x:c r="S39" s="3" t="s">
-        <x:v>865</x:v>
-      </x:c>
-      <x:c r="T39" s="3" t="s">
-        <x:v>866</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -11170,7 +11149,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bf8183517df4b53"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5215770ede4f23"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-005 state history retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb79f44cd060f4a0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rc46d8898b102415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rfba5588294bb4b1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R773f79cca795430d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb5b68a3878644019"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3151eccf955844ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R8059f1b5c4a14860"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rd40e65ebd96347ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1327,16 +1327,16 @@
     <x:t xml:space="preserve">Streamed chat turns</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">QE-005</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent state and history</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a returning customer, I can reload session state and chat history.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BFF exposes session state and message history by session id with authorization boundaries.</x:t>
+    <x:t xml:space="preserve">QE-006</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent clean speech and thinking</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I get cleaned assistant speech and structured thinking/progress updates.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">BFF exposes clean-speech and thinking endpoints used by the assistant experience.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:t>
@@ -1348,46 +1348,10 @@
     <x:t xml:space="preserve">No fix needed for this story from current QuoteEngine automated retest.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Shell/session restore -&gt; AgentController sessions/messages -&gt; SessionStore</x:t>
+    <x:t xml:space="preserve">Agent UI -&gt; clean-speech/thinking endpoints -&gt; QuoteAgentService</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Session reload/history</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController GET sessions/{sessionId}, sessions/{sessionId}/messages</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests history auth | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, SessionStore, Auth</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Session state and message history</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs authenticated reload browser retest</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:132,142; QuoteAgentSessionStore.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-006</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent clean speech and thinking</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I get cleaned assistant speech and structured thinking/progress updates.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">BFF exposes clean-speech and thinking endpoints used by the assistant experience.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent UI -&gt; clean-speech/thinking endpoints -&gt; QuoteAgentService</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Thinking/progress and speech cleanup surfaces</x:t>
@@ -5162,7 +5126,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2ec510e4a734287"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb233f994b1de4067"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8578,7 +8542,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbb9839dc17aa49fc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R765a67ea39834959"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8937,85 +8901,85 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="93.25" hidden="0">
-      <x:c r="A6" s="3" t="s">
-        <x:v>438</x:v>
-      </x:c>
-      <x:c r="B6" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C6" s="3" t="s">
-        <x:v>439</x:v>
-      </x:c>
-      <x:c r="D6" s="3" t="s">
-        <x:v>440</x:v>
-      </x:c>
-      <x:c r="E6" s="3" t="s">
-        <x:v>441</x:v>
-      </x:c>
-      <x:c r="F6" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G6" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="H6" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="I6" s="3" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="J6" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="K6" s="3" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="L6" s="3" t="s">
-        <x:v>445</x:v>
-      </x:c>
-      <x:c r="M6" s="3" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="N6" s="3" t="s">
-        <x:v>447</x:v>
-      </x:c>
-      <x:c r="O6" s="3" t="s">
-        <x:v>448</x:v>
-      </x:c>
-      <x:c r="P6" s="3" t="s">
-        <x:v>449</x:v>
-      </x:c>
-      <x:c r="Q6" s="3" t="s">
-        <x:v>450</x:v>
-      </x:c>
-      <x:c r="R6" s="3" t="s">
-        <x:v>451</x:v>
-      </x:c>
-      <x:c r="S6" s="3" t="s">
-        <x:v>452</x:v>
-      </x:c>
-      <x:c r="T6" s="3" t="s">
-        <x:v>453</x:v>
-      </x:c>
-      <x:c r="U6" s="3" t="s">
-        <x:v>52</x:v>
+      <x:c r="A6" s="3" t="str">
+        <x:v>QE-005</x:v>
+      </x:c>
+      <x:c r="B6" s="3" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C6" s="3" t="str">
+        <x:v>Agent state and history</x:v>
+      </x:c>
+      <x:c r="D6" s="3" t="str">
+        <x:v>As a returning customer, I can reload session state and chat history.</x:v>
+      </x:c>
+      <x:c r="E6" s="3" t="str">
+        <x:v>Returning customers reload the same QuoteEngine agent session, state, and customer-safe chat history after page reload or auth return; another signed-in customer cannot read the session.</x:v>
+      </x:c>
+      <x:c r="F6" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G6" s="3" t="str">
+        <x:v>Focused current-state state/history tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H6" s="3" t="str">
+        <x:v>No behavior error observed in focused QuoteEngine state/history retest; live authenticated browser reload still not executed in this slice.</x:v>
+      </x:c>
+      <x:c r="I6" s="3" t="str">
+        <x:v>No app fix applied for QE-005; current code path is covered by focused BFF/source tests.</x:v>
+      </x:c>
+      <x:c r="J6" s="3" t="str">
+        <x:v>Passed 8/8 focused tests: QuoteAgentEndpointTests message-history mapping, persisted cold-store mapping, signed-in restore, cross-customer denial, injected-context stripping, and QuoteEngineSourceTests auth-completion/history contract.</x:v>
+      </x:c>
+      <x:c r="K6" s="3" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L6" s="3" t="str">
+        <x:v>QuoteWorkspace shared session persistence/auth return -&gt; QuoteAgentLaunchShell state/history hydration -&gt; QuoteEngineApiClient -&gt; AgentController session/message endpoints -&gt; QuoteAgentSessionStore and chatbot conversation mapping</x:v>
+      </x:c>
+      <x:c r="M6" s="3" t="str">
+        <x:v>QuoteWorkspace.razor; QuoteAgentLaunchShell.razor; QuoteEngineApiClient; AgentController; QuoteAgentSessionStore</x:v>
+      </x:c>
+      <x:c r="N6" s="3" t="str">
+        <x:v>QuoteWorkspace RestoreAgentSessionAsync/PersistAgentSessionAsync use malievChatbot shared session storage; QuoteAgentLaunchShell OnAuthPopupCompleted forces reload and LoadMessageHistoryAsync hydrates AgentMessageRow history.</x:v>
+      </x:c>
+      <x:c r="O6" s="3" t="str">
+        <x:v>GET quote/v1/agent/sessions/{sessionId}; GET quote/v1/agent/sessions/{sessionId}/messages resolves the mapped chatbot conversation, filters customer-safe roles, strips injected user-turn context, and returns NotFound when no accessible mapping exists.</x:v>
+      </x:c>
+      <x:c r="P6" s="3" t="str">
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_uses_mapped_chatbot_session_after_auth_return|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_uses_persisted_mapping_when_session_store_is_cold|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_restores_signed_in_customer_mapping_after_auth_return|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_denies_signed_in_customer_for_another_customers_session|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_strips_injected_session_context_from_persisted_user_turns|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_keeps_legacy_user_content_unmodified_when_no_context_marker_present|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_auth_completion_reloads_active_session_and_hydrates_messages|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract" --verbosity minimal passed 8/8.</x:v>
+      </x:c>
+      <x:c r="Q6" s="3" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, QuoteAgentSessionStore, chatbot conversation service, Auth/session</x:v>
+      </x:c>
+      <x:c r="R6" s="3" t="str">
+        <x:v>Shared browser session id, QuoteEngine agent session state, chatbot conversation mapping, restored message history</x:v>
+      </x:c>
+      <x:c r="S6" s="3" t="str">
+        <x:v>Needs authenticated reload browser retest against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T6" s="3" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor:1508; Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:2603,2690; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs:373; Maliev.QuoteEngine.Bff/Controllers/AgentController.cs:132,142; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:243; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:2184</x:v>
+      </x:c>
+      <x:c r="U6" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="93.25" hidden="0">
       <x:c r="A7" s="3" t="s">
-        <x:v>454</x:v>
+        <x:v>438</x:v>
       </x:c>
       <x:c r="B7" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C7" s="3" t="s">
-        <x:v>455</x:v>
+        <x:v>439</x:v>
       </x:c>
       <x:c r="D7" s="3" t="s">
-        <x:v>456</x:v>
+        <x:v>440</x:v>
       </x:c>
       <x:c r="E7" s="3" t="s">
-        <x:v>457</x:v>
+        <x:v>441</x:v>
       </x:c>
       <x:c r="F7" s="3" t="s">
         <x:v>37</x:v>
@@ -9036,31 +9000,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L7" s="3" t="s">
-        <x:v>458</x:v>
+        <x:v>445</x:v>
       </x:c>
       <x:c r="M7" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N7" s="3" t="s">
-        <x:v>459</x:v>
+        <x:v>447</x:v>
       </x:c>
       <x:c r="O7" s="3" t="s">
-        <x:v>460</x:v>
+        <x:v>448</x:v>
       </x:c>
       <x:c r="P7" s="3" t="s">
-        <x:v>461</x:v>
+        <x:v>449</x:v>
       </x:c>
       <x:c r="Q7" s="3" t="s">
-        <x:v>462</x:v>
+        <x:v>450</x:v>
       </x:c>
       <x:c r="R7" s="3" t="s">
-        <x:v>463</x:v>
+        <x:v>451</x:v>
       </x:c>
       <x:c r="S7" s="3" t="s">
-        <x:v>464</x:v>
+        <x:v>452</x:v>
       </x:c>
       <x:c r="T7" s="3" t="s">
-        <x:v>465</x:v>
+        <x:v>453</x:v>
       </x:c>
       <x:c r="U7" s="3" t="s">
         <x:v>52</x:v>
@@ -9068,19 +9032,19 @@
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
       <x:c r="A8" s="3" t="s">
-        <x:v>466</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B8" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C8" s="3" t="s">
-        <x:v>467</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="D8" s="3" t="s">
-        <x:v>468</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="E8" s="3" t="s">
-        <x:v>469</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="F8" s="3" t="s">
         <x:v>37</x:v>
@@ -9101,31 +9065,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L8" s="3" t="s">
-        <x:v>470</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="M8" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N8" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="O8" s="3" t="s">
-        <x:v>472</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="P8" s="3" t="s">
-        <x:v>473</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="Q8" s="3" t="s">
-        <x:v>474</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="R8" s="3" t="s">
-        <x:v>475</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="S8" s="3" t="s">
-        <x:v>476</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="T8" s="3" t="s">
-        <x:v>477</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="U8" s="3" t="s">
         <x:v>52</x:v>
@@ -9133,19 +9097,19 @@
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>37</x:v>
@@ -9166,31 +9130,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="M9" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N9" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="P9" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="S9" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="T9" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>52</x:v>
@@ -9198,19 +9162,19 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>37</x:v>
@@ -9231,31 +9195,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
         <x:v>424</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>499</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>500</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>52</x:v>
@@ -9263,19 +9227,19 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>37</x:v>
@@ -9296,31 +9260,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>52</x:v>
@@ -9328,19 +9292,19 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>37</x:v>
@@ -9361,31 +9325,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>520</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>525</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>52</x:v>
@@ -9393,19 +9357,19 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>526</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>527</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>37</x:v>
@@ -9426,31 +9390,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>532</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
+        <x:v>510</x:v>
+      </x:c>
+      <x:c r="R13" s="3" t="s">
         <x:v>522</x:v>
       </x:c>
-      <x:c r="R13" s="3" t="s">
-        <x:v>534</x:v>
-      </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>52</x:v>
@@ -9458,19 +9422,19 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
@@ -9491,31 +9455,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9523,19 +9487,19 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
@@ -9556,31 +9520,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>561</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9588,19 +9552,19 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>562</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>563</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
@@ -9621,31 +9585,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>568</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>573</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9653,19 +9617,19 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>574</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>575</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
@@ -9686,31 +9650,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>580</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>585</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>586</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9718,19 +9682,19 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>587</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
@@ -9751,31 +9715,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>592</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>593</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>598</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>599</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9783,19 +9747,19 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>600</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
@@ -9816,31 +9780,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>605</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>606</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>611</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>612</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9848,19 +9812,19 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>613</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
@@ -9881,31 +9845,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>618</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>624</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>625</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9913,19 +9877,19 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>626</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
@@ -9946,31 +9910,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>632</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -9978,19 +9942,19 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
@@ -10011,31 +9975,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -10043,19 +10007,19 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
@@ -10076,31 +10040,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>655</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>660</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>661</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -10108,19 +10072,19 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>662</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
@@ -10141,31 +10105,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>667</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>668</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>673</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -10173,19 +10137,19 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>674</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>675</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
@@ -10206,31 +10170,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>680</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>685</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10238,19 +10202,19 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>686</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>687</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
@@ -10271,31 +10235,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>692</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>697</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>698</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10303,19 +10267,19 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>699</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
@@ -10336,31 +10300,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>704</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>705</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
-        <x:v>710</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>711</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10368,19 +10332,19 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>712</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
@@ -10401,31 +10365,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>717</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>718</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10433,19 +10397,19 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
@@ -10466,31 +10430,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10498,19 +10462,19 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
@@ -10531,31 +10495,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>742</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>743</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>748</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>749</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10563,19 +10527,19 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>750</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
@@ -10596,31 +10560,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>755</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>756</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>761</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>762</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10628,19 +10592,19 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>763</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
@@ -10661,31 +10625,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>768</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>769</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>774</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>775</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10693,19 +10657,19 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>776</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
@@ -10726,31 +10690,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>781</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>787</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>788</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10758,7 +10722,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>789</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10767,10 +10731,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
@@ -10791,31 +10755,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>795</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10823,19 +10787,19 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>802</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
@@ -10856,31 +10820,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>811</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10888,19 +10852,19 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>812</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>813</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>814</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>815</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
@@ -10921,31 +10885,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>816</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>817</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>818</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>819</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>820</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>821</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>822</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>823</x:v>
+        <x:v>811</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10953,19 +10917,19 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>824</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>825</x:v>
+        <x:v>813</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>826</x:v>
+        <x:v>814</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>827</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
@@ -10986,31 +10950,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>828</x:v>
+        <x:v>816</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>829</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>830</x:v>
+        <x:v>818</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>831</x:v>
+        <x:v>819</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>832</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>833</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>834</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>835</x:v>
+        <x:v>823</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>829</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -11018,19 +10982,19 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>836</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>837</x:v>
+        <x:v>825</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>838</x:v>
+        <x:v>826</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>839</x:v>
+        <x:v>827</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
@@ -11051,31 +11015,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>840</x:v>
+        <x:v>828</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>841</x:v>
+        <x:v>829</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>842</x:v>
+        <x:v>830</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>843</x:v>
+        <x:v>831</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>844</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>845</x:v>
+        <x:v>833</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>846</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>847</x:v>
+        <x:v>835</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -11083,19 +11047,19 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>848</x:v>
+        <x:v>836</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>849</x:v>
+        <x:v>837</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>850</x:v>
+        <x:v>838</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>851</x:v>
+        <x:v>839</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
@@ -11116,31 +11080,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>852</x:v>
+        <x:v>840</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>853</x:v>
+        <x:v>841</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>854</x:v>
+        <x:v>842</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>855</x:v>
+        <x:v>843</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>856</x:v>
+        <x:v>844</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>857</x:v>
+        <x:v>845</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>858</x:v>
+        <x:v>846</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>859</x:v>
+        <x:v>847</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -11149,7 +11113,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5215770ede4f23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree49df396751461c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-007 project navigation retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb5b68a3878644019"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R3151eccf955844ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R8059f1b5c4a14860"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rd40e65ebd96347ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcf0701f9e3fc41be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re4e8f64e754e4bfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R982e27500cc44dc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf3e0c1f295394a64"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1373,42 +1373,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">AgentController.cs:111,423</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-007</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Project navigation rail</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can navigate, search, pin, archive, duplicate, and continue projects from the rail.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Project nav endpoints and shell management pages support project list, detail, duplicate, pin/unpin, archive, and current project selection.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Rail/projects page -&gt; QuoteController projects/nav/detail/actions</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">New project, Projects, search, pin/archive/duplicate actions</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteController projects/nav, project detail, duplicate, pin, delete pin, archive</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineSourceTests rail/project management | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Project service, SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Project metadata, pin/archive flags</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs product decision on achieve endpoint naming</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentLaunchShell.razor; QuoteController.cs:548-674</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QE-008</x:t>
@@ -5126,7 +5090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb233f994b1de4067"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47eb0d60f7954f2a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8542,7 +8506,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R765a67ea39834959"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R144959e895754513"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9031,85 +8995,85 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="93.25" hidden="0">
-      <x:c r="A8" s="3" t="s">
-        <x:v>454</x:v>
-      </x:c>
-      <x:c r="B8" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C8" s="3" t="s">
-        <x:v>455</x:v>
-      </x:c>
-      <x:c r="D8" s="3" t="s">
-        <x:v>456</x:v>
-      </x:c>
-      <x:c r="E8" s="3" t="s">
-        <x:v>457</x:v>
-      </x:c>
-      <x:c r="F8" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G8" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="H8" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="I8" s="3" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="J8" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="K8" s="3" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="L8" s="3" t="s">
-        <x:v>458</x:v>
-      </x:c>
-      <x:c r="M8" s="3" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="N8" s="3" t="s">
-        <x:v>459</x:v>
-      </x:c>
-      <x:c r="O8" s="3" t="s">
-        <x:v>460</x:v>
-      </x:c>
-      <x:c r="P8" s="3" t="s">
-        <x:v>461</x:v>
-      </x:c>
-      <x:c r="Q8" s="3" t="s">
-        <x:v>462</x:v>
-      </x:c>
-      <x:c r="R8" s="3" t="s">
-        <x:v>463</x:v>
-      </x:c>
-      <x:c r="S8" s="3" t="s">
-        <x:v>464</x:v>
-      </x:c>
-      <x:c r="T8" s="3" t="s">
-        <x:v>465</x:v>
-      </x:c>
-      <x:c r="U8" s="3" t="s">
-        <x:v>52</x:v>
+      <x:c r="A8" s="3" t="str">
+        <x:v>QE-007</x:v>
+      </x:c>
+      <x:c r="B8" s="3" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C8" s="3" t="str">
+        <x:v>Project navigation rail</x:v>
+      </x:c>
+      <x:c r="D8" s="3" t="str">
+        <x:v>As a customer, I can navigate, search, pin, archive, duplicate, and continue projects from the rail.</x:v>
+      </x:c>
+      <x:c r="E8" s="3" t="str">
+        <x:v>Signed-in customers can open the project rail/pages, return to the active chat, start a new project after saving current work, and manage only their own projects with nav, detail, duplicate, pin/unpin, archive, and mark-achieved actions.</x:v>
+      </x:c>
+      <x:c r="F8" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G8" s="3" t="str">
+        <x:v>Focused current-state project navigation rail tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H8" s="3" t="str">
+        <x:v>No behavior error observed in focused QuoteEngine project navigation retest. UX/product naming question remains for the current /achieve route and Mark achieved label.</x:v>
+      </x:c>
+      <x:c r="I8" s="3" t="str">
+        <x:v>No app fix applied for QE-007; current code path is covered by focused BFF/source tests.</x:v>
+      </x:c>
+      <x:c r="J8" s="3" t="str">
+        <x:v>Passed 7/7 focused tests: project nav auth requirement, customer project listing, pin/unpin, cross-customer pin denial, archive removal and denial, achieve removal and denial, and management-page return/new-project source contract.</x:v>
+      </x:c>
+      <x:c r="K8" s="3" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L8" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell rail/projects page -&gt; QuoteWorkspace new-project save/reset -&gt; QuoteEngineApiClient project methods -&gt; QuoteController project nav/detail/duplicate/pin/archive/achieve endpoints -&gt; ProjectService client/prototype fallback/customer ownership</x:v>
+      </x:c>
+      <x:c r="M8" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; QuoteWorkspace.razor; QuoteEngineApiClient; QuoteController</x:v>
+      </x:c>
+      <x:c r="N8" s="3" t="str">
+        <x:v>WorkspacePage.Projects management rows expose Open, Duplicate, Pin/Unpin, Archive, and Mark achieved actions; management pages use ReturnToCurrentChatAsync; New project calls StartNewProjectAsync through QuoteWorkspace.</x:v>
+      </x:c>
+      <x:c r="O8" s="3" t="str">
+        <x:v>GET quote/v1/projects/nav requires a signed-in customer; POST/DELETE quote/v1/projects/{projectId}/pin, POST quote/v1/projects/{projectId}/archive, and POST quote/v1/projects/{projectId}/achieve enforce customer ownership and remove archived/achieved projects from nav.</x:v>
+      </x:c>
+      <x:c r="P8" s="3" t="str">
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteEngineEndpointTests.Project_navigation_requires_signed_in_customer|FullyQualifiedName~QuoteEngineEndpointTests.Project_navigation_lists_customer_projects_and_updates_pin_state|FullyQualifiedName~QuoteEngineEndpointTests.Project_pin_rejects_project_owned_by_another_customer|FullyQualifiedName~QuoteEngineEndpointTests.Project_archive_removes_project_from_navigation_and_rejects_other_customers|FullyQualifiedName~QuoteEngineEndpointTests.Project_achieve_marks_project_complete_and_rejects_other_customers|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract" --verbosity minimal passed 6/6; dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_starts_new_sessions_and_returns_from_management_pages" --verbosity minimal passed 1/1.</x:v>
+      </x:c>
+      <x:c r="Q8" s="3" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, ProjectService client, Auth/session, prototype fallback store in development/testing</x:v>
+      </x:c>
+      <x:c r="R8" s="3" t="str">
+        <x:v>Project navigation list, draft project records, pinned flag, archived/achieved state, duplicated project records, current workspace reset state</x:v>
+      </x:c>
+      <x:c r="S8" s="3" t="str">
+        <x:v>Needs product/UX decision on whether the current /achieve endpoint and Mark achieved label should be renamed to completed/complete.</x:v>
+      </x:c>
+      <x:c r="T8" s="3" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:410; Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor:432; Maliev.QuoteEngine.Bff/Controllers/QuoteController.cs:548,570,590,618,636,654; Maliev.QuoteEngine.Tests/QuoteEngineEndpointTests.cs:2924,2934,3005,3020,3045; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:829,864</x:v>
+      </x:c>
+      <x:c r="U8" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="93.25" hidden="0">
       <x:c r="A9" s="3" t="s">
-        <x:v>466</x:v>
+        <x:v>454</x:v>
       </x:c>
       <x:c r="B9" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C9" s="3" t="s">
-        <x:v>467</x:v>
+        <x:v>455</x:v>
       </x:c>
       <x:c r="D9" s="3" t="s">
-        <x:v>468</x:v>
+        <x:v>456</x:v>
       </x:c>
       <x:c r="E9" s="3" t="s">
-        <x:v>469</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="F9" s="3" t="s">
         <x:v>37</x:v>
@@ -9130,31 +9094,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L9" s="3" t="s">
-        <x:v>470</x:v>
+        <x:v>458</x:v>
       </x:c>
       <x:c r="M9" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N9" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>459</x:v>
       </x:c>
       <x:c r="O9" s="3" t="s">
-        <x:v>472</x:v>
+        <x:v>460</x:v>
       </x:c>
       <x:c r="P9" s="3" t="s">
-        <x:v>473</x:v>
+        <x:v>461</x:v>
       </x:c>
       <x:c r="Q9" s="3" t="s">
-        <x:v>474</x:v>
+        <x:v>462</x:v>
       </x:c>
       <x:c r="R9" s="3" t="s">
-        <x:v>475</x:v>
+        <x:v>463</x:v>
       </x:c>
       <x:c r="S9" s="3" t="s">
-        <x:v>476</x:v>
+        <x:v>464</x:v>
       </x:c>
       <x:c r="T9" s="3" t="s">
-        <x:v>477</x:v>
+        <x:v>465</x:v>
       </x:c>
       <x:c r="U9" s="3" t="s">
         <x:v>52</x:v>
@@ -9162,19 +9126,19 @@
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
       <x:c r="A10" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B10" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C10" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D10" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E10" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F10" s="3" t="s">
         <x:v>37</x:v>
@@ -9195,31 +9159,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L10" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="M10" s="3" t="s">
         <x:v>424</x:v>
       </x:c>
       <x:c r="N10" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="O10" s="3" t="s">
         <x:v>205</x:v>
       </x:c>
       <x:c r="P10" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="Q10" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="R10" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="S10" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="T10" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="U10" s="3" t="s">
         <x:v>52</x:v>
@@ -9227,19 +9191,19 @@
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>37</x:v>
@@ -9260,31 +9224,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>499</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>500</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>52</x:v>
@@ -9292,19 +9256,19 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>37</x:v>
@@ -9325,31 +9289,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>52</x:v>
@@ -9357,19 +9321,19 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>37</x:v>
@@ -9390,31 +9354,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>520</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
+        <x:v>498</x:v>
+      </x:c>
+      <x:c r="R13" s="3" t="s">
         <x:v>510</x:v>
       </x:c>
-      <x:c r="R13" s="3" t="s">
-        <x:v>522</x:v>
-      </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>52</x:v>
@@ -9422,19 +9386,19 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>525</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>526</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>527</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
@@ -9455,31 +9419,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>532</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>534</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9487,19 +9451,19 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
@@ -9520,31 +9484,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9552,19 +9516,19 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
@@ -9585,31 +9549,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>561</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9617,19 +9581,19 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>562</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>563</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
@@ -9650,31 +9614,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>568</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>573</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>574</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9682,19 +9646,19 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>575</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
@@ -9715,31 +9679,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>580</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>585</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>586</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>587</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9747,19 +9711,19 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
@@ -9780,31 +9744,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>592</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>593</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>598</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>599</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>600</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9812,19 +9776,19 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
@@ -9845,31 +9809,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>605</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>606</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>611</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>612</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>613</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9877,19 +9841,19 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
@@ -9910,31 +9874,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>618</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>624</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -9942,19 +9906,19 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>625</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>626</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
@@ -9975,31 +9939,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>632</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -10007,19 +9971,19 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
@@ -10040,31 +10004,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -10072,19 +10036,19 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
@@ -10105,31 +10069,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>655</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>660</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>661</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -10137,19 +10101,19 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>662</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
@@ -10170,31 +10134,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>667</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>668</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>673</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10202,19 +10166,19 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>674</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>675</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
@@ -10235,31 +10199,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>680</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>685</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>686</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10267,19 +10231,19 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>687</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
@@ -10300,31 +10264,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>692</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>697</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
-        <x:v>698</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>699</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10332,19 +10296,19 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
@@ -10365,31 +10329,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>704</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>705</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>710</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>711</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10397,19 +10361,19 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>712</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
@@ -10430,31 +10394,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>717</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>718</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10462,19 +10426,19 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
@@ -10495,31 +10459,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10527,19 +10491,19 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
@@ -10560,31 +10524,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>742</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>743</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>748</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>749</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>750</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10592,19 +10556,19 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
@@ -10625,31 +10589,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>755</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>756</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
-        <x:v>761</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>762</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>763</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10657,19 +10621,19 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
@@ -10690,31 +10654,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>768</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>769</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>774</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>775</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>776</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10722,7 +10686,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10731,10 +10695,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
@@ -10755,31 +10719,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>781</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>787</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10787,19 +10751,19 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>788</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>789</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
@@ -10820,31 +10784,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>795</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10852,19 +10816,19 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>802</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
@@ -10885,31 +10849,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>811</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10917,19 +10881,19 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>812</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>813</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>814</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>815</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
@@ -10950,31 +10914,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>816</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>817</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>818</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>819</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>820</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>821</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>822</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>823</x:v>
+        <x:v>811</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>817</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -10982,19 +10946,19 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>824</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>825</x:v>
+        <x:v>813</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>826</x:v>
+        <x:v>814</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>827</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
@@ -11015,31 +10979,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>828</x:v>
+        <x:v>816</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>829</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>830</x:v>
+        <x:v>818</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>831</x:v>
+        <x:v>819</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>832</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>833</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>834</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>835</x:v>
+        <x:v>823</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -11047,19 +11011,19 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>836</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>837</x:v>
+        <x:v>825</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>838</x:v>
+        <x:v>826</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>839</x:v>
+        <x:v>827</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
@@ -11080,31 +11044,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>840</x:v>
+        <x:v>828</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>841</x:v>
+        <x:v>829</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>842</x:v>
+        <x:v>830</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>843</x:v>
+        <x:v>831</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>844</x:v>
+        <x:v>832</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>845</x:v>
+        <x:v>833</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>846</x:v>
+        <x:v>834</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>847</x:v>
+        <x:v>835</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -11113,7 +11077,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree49df396751461c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f322ed9d7914018"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-009 upload retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcf0701f9e3fc41be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re4e8f64e754e4bfa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R982e27500cc44dc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf3e0c1f295394a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7daceb4650b246f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Red47f93761c446a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rce0ce3ef418c4ede"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R7369438bd66d48ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1409,39 +1409,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">AgentController.cs:271; QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-009</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Resumable CAD upload</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can upload CAD files for part analysis.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Workspace creates resumable upload sessions, sends chunks, completes uploads, and checks analysis status.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">File picker -&gt; QuoteController uploads -&gt; storage/analysis</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">CAD file input, attachment picker, upload controls</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineSourceTests upload; QuoteEngineApiClientTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Storage, Geometry/analysis</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Upload sessions/files/analysis status</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs browser file-picker retest</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteWorkspace.razor; QuoteController.cs:68-259</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QE-010</x:t>
@@ -5090,7 +5057,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R47eb0d60f7954f2a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdac1550edeab47be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8506,7 +8473,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R144959e895754513"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e927a3a23d94da5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9125,85 +9092,85 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="93.25" hidden="0">
-      <x:c r="A10" s="3" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="B10" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C10" s="3" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="D10" s="3" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="E10" s="3" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="F10" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G10" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="H10" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="I10" s="3" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="J10" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="K10" s="3" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="L10" s="3" t="s">
-        <x:v>470</x:v>
-      </x:c>
-      <x:c r="M10" s="3" t="s">
-        <x:v>424</x:v>
-      </x:c>
-      <x:c r="N10" s="3" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="O10" s="3" t="s">
-        <x:v>205</x:v>
-      </x:c>
-      <x:c r="P10" s="3" t="s">
-        <x:v>472</x:v>
-      </x:c>
-      <x:c r="Q10" s="3" t="s">
-        <x:v>473</x:v>
-      </x:c>
-      <x:c r="R10" s="3" t="s">
-        <x:v>474</x:v>
-      </x:c>
-      <x:c r="S10" s="3" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="T10" s="3" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="U10" s="3" t="s">
-        <x:v>52</x:v>
+      <x:c r="A10" s="3" t="str">
+        <x:v>QE-009</x:v>
+      </x:c>
+      <x:c r="B10" s="3" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C10" s="3" t="str">
+        <x:v>Resumable CAD upload</x:v>
+      </x:c>
+      <x:c r="D10" s="3" t="str">
+        <x:v>As a customer, I can upload CAD files for part analysis.</x:v>
+      </x:c>
+      <x:c r="E10" s="3" t="str">
+        <x:v>Customers can choose, drop, or paste supported CAD and supplemental quote files; the workspace validates type and size, initiates a resumable upload, streams bytes with Content-Range, completes the upload, shows analysis/processing status, and preserves customer ownership boundaries.</x:v>
+      </x:c>
+      <x:c r="F10" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G10" s="3" t="str">
+        <x:v>Focused current-state resumable upload tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H10" s="3" t="str">
+        <x:v>No behavior error observed in focused QuoteEngine upload retest; live browser file-picker/drop/paste interaction still not executed in this slice.</x:v>
+      </x:c>
+      <x:c r="I10" s="3" t="str">
+        <x:v>No app fix applied for QE-009; current code path is covered by focused BFF/source tests.</x:v>
+      </x:c>
+      <x:c r="J10" s="3" t="str">
+        <x:v>Passed 28/28 focused tests covering upload constraints, supported CAD/context file initiation, resumable Content-Range streaming, upload ownership on analysis status, UploadService fallback policy, custom-file completion status, and QuoteWorkspace upload source contracts.</x:v>
+      </x:c>
+      <x:c r="K10" s="3" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L10" s="3" t="str">
+        <x:v>QuoteWorkspace file picker/drop/paste -&gt; quoteEngineUploads browser JS capture/streaming -&gt; QuoteEngineApiClient -&gt; QuoteController resumable upload endpoints -&gt; QuoteUploadServiceClient/prototype fallback -&gt; analysis status and agent attachment registration</x:v>
+      </x:c>
+      <x:c r="M10" s="3" t="str">
+        <x:v>QuoteWorkspace.razor; quote-upload.js; QuoteEngineApiClient; QuoteController; QuoteUploadConstraints</x:v>
+      </x:c>
+      <x:c r="N10" s="3" t="str">
+        <x:v>InputFile quote-cad-files uses SupportedAttachmentAccept; OpenFilePickerAsync guards re-entrant picker opens; HandleFilesAsync and HandleDroppedFilesAsync capture files through quoteEngineUploads, validate candidates, create uploading parts, stream files, complete uploads, poll analysis status, and notify the agent shell.</x:v>
+      </x:c>
+      <x:c r="O10" s="3" t="str">
+        <x:v>POST quote/v1/uploads/resumable validates extension and size and creates a proxy upload URL; PUT quote/v1/uploads/resumable/{uploadId} requires Content-Range and streams to UploadService; POST quote/v1/uploads/resumable/{uploadId}/complete returns processing/analyzed state; GET quote/v1/uploads/{uploadId}/analysis-status enforces upload ownership.</x:v>
+      </x:c>
+      <x:c r="P10" s="3" t="str">
+        <x:v>2026-06-24: focused QuoteEngine upload/source test filter passed 28/28 with dotnet test Maliev.QuoteEngine.slnx --verbosity minimal. Coverage included QuoteUploadConstraintTests, resumable Content-Range streaming, analysis-status ownership, UploadService fallback policy, custom-file completion, and QuoteWorkspace source contracts.</x:v>
+      </x:c>
+      <x:c r="Q10" s="3" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, UploadService client, Geometry/analysis status, SignalR notifications, agent attachment registration</x:v>
+      </x:c>
+      <x:c r="R10" s="3" t="str">
+        <x:v>Browser-retained file handles, upload IDs, downstream upload IDs, storage paths, upload status, part view models, analysis status, agent attachment state</x:v>
+      </x:c>
+      <x:c r="S10" s="3" t="str">
+        <x:v>Needs live browser retest for file picker, drag/drop, paste, interruption/resume, and file cleanup against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T10" s="3" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor:21,289,454,526,536,541,631; Maliev.QuoteEngine.Client/wwwroot/js/quote-upload.js:1; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs:49,83,92; Maliev.QuoteEngine.Bff/Controllers/QuoteController.cs:68,134,194,259; Maliev.QuoteEngine.Tests/QuoteUploadConstraintTests.cs:37,58,74,90,113; Maliev.QuoteEngine.Tests/QuoteEngineEndpointTests.cs:2305,2337,2369,2421,2466; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:604,679,762</x:v>
+      </x:c>
+      <x:c r="U10" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
       <x:c r="A11" s="3" t="s">
-        <x:v>477</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B11" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C11" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D11" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E11" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F11" s="3" t="s">
         <x:v>37</x:v>
@@ -9224,31 +9191,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L11" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="M11" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="N11" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="O11" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="P11" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="Q11" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="R11" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="S11" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="T11" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="U11" s="3" t="s">
         <x:v>52</x:v>
@@ -9256,19 +9223,19 @@
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>37</x:v>
@@ -9289,31 +9256,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>499</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>500</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>52</x:v>
@@ -9321,19 +9288,19 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>37</x:v>
@@ -9354,31 +9321,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>52</x:v>
@@ -9386,19 +9353,19 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
@@ -9419,31 +9386,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>520</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>525</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9451,19 +9418,19 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>526</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>527</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
@@ -9484,31 +9451,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>532</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>534</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9516,19 +9483,19 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
@@ -9549,31 +9516,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9581,19 +9548,19 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
@@ -9614,31 +9581,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>561</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>562</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9646,19 +9613,19 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>563</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
@@ -9679,31 +9646,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>568</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>573</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>574</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>575</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9711,19 +9678,19 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
@@ -9744,31 +9711,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>580</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>585</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>586</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>587</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9776,19 +9743,19 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>592</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
@@ -9809,31 +9776,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>593</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>598</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>599</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>600</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9841,19 +9808,19 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>605</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
@@ -9874,31 +9841,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>606</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>611</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>612</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -9906,19 +9873,19 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>613</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
@@ -9939,31 +9906,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>618</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>624</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -9971,19 +9938,19 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>625</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>626</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
@@ -10004,31 +9971,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>632</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -10036,19 +10003,19 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
@@ -10069,31 +10036,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -10101,19 +10068,19 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
@@ -10134,31 +10101,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>655</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>660</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>661</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10166,19 +10133,19 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>662</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
@@ -10199,31 +10166,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>667</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>668</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>673</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>674</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10231,19 +10198,19 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>675</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
@@ -10264,31 +10231,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>680</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>685</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
-        <x:v>686</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>687</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10296,19 +10263,19 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
@@ -10329,31 +10296,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>692</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>697</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>698</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>699</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10361,19 +10328,19 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
@@ -10394,31 +10361,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>704</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>705</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>710</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>711</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>712</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10426,19 +10393,19 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
@@ -10459,31 +10426,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>717</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>718</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10491,19 +10458,19 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
@@ -10524,31 +10491,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10556,19 +10523,19 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>742</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
@@ -10589,31 +10556,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>743</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>748</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
-        <x:v>749</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>750</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10621,19 +10588,19 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>755</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
@@ -10654,31 +10621,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>756</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>761</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>762</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>763</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10686,7 +10653,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10695,10 +10662,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
@@ -10719,31 +10686,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>768</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>769</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>774</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>775</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10751,19 +10718,19 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>776</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
@@ -10784,31 +10751,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>781</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>787</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10816,19 +10783,19 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>788</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>789</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
@@ -10849,31 +10816,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>795</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10881,19 +10848,19 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>802</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
@@ -10914,31 +10881,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>811</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -10946,19 +10913,19 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>812</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>813</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>814</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>815</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
@@ -10979,31 +10946,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>816</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>817</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>818</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>819</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>820</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>821</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>822</x:v>
+        <x:v>811</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>823</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -11011,19 +10978,19 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>824</x:v>
+        <x:v>813</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>825</x:v>
+        <x:v>814</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>826</x:v>
+        <x:v>815</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>827</x:v>
+        <x:v>816</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
@@ -11044,31 +11011,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>828</x:v>
+        <x:v>817</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>829</x:v>
+        <x:v>818</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>830</x:v>
+        <x:v>819</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>831</x:v>
+        <x:v>820</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>832</x:v>
+        <x:v>821</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>833</x:v>
+        <x:v>822</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>834</x:v>
+        <x:v>823</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>835</x:v>
+        <x:v>824</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -11077,7 +11044,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f322ed9d7914018"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98eb820354214b08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-010 handoff retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7daceb4650b246f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Red47f93761c446a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rce0ce3ef418c4ede"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R7369438bd66d48ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R55ec781b4d914d84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R875633f7b0ee44f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R04ac7350e4234996"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R83b31bd731da41ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1411,427 +1411,391 @@
     <x:t xml:space="preserve">AgentController.cs:271; QuoteAgentLaunchShell.razor</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">QE-010</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Web handoff import</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can continue from a public web quote upload into the workspace.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Workspace imports handoff uploads through signed handoff endpoint and registers those files with the active session.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Web handoff token -&gt; QuoteController uploads/handoff -&gt; workspace/session attachments</x:t>
+    <x:t xml:space="preserve">QE-011</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent attachments</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can attach uploaded files as context before asking the agent.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Agent attachment endpoint registers uploaded files in session state and the shell previews attachments until sent.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Composer attachments -&gt; AgentController attachments -&gt; SessionStore</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Attachment preview and sent attachment display</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/attachments</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests attachment; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, SessionStore, Storage</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Session attachment records</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs attachment resend/removal browser pass</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController.cs:203; QuoteAgentLaunchShell.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-012</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sketch attachments</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can draw or attach a hand sketch for the agent.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sketch dialog captures sketch data and posts it to the agent sketch endpoint.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sketch UI -&gt; AgentController sketches -&gt; SessionStore/artifacts</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Hand sketch dialog/tools</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/sketches</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests sketches; source tests sketch disposal | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sketch artifact/context</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs mobile sketch browser pass</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController.cs:367; QuoteAgentLaunchShell.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-013</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Google Drive connector</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can connect Google Drive and select source files.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Connector endpoints start OAuth, handle callback, expose status, list files, and return connector handoff links.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Connector UI -&gt; GoogleDriveConnectorController and AgentController connector endpoints</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentLaunchShell.razor; GoogleCallback.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">/auth/callback/google; connector panel</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">GoogleDriveConnectorController start/callback/status/files; AgentController connectors/handoff</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngineSourceTests connector; endpoint tests where present | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, Google Drive, Auth</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Connector tokens/status/file refs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs OAuth environment smoke</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">GoogleDriveConnectorController.cs; AgentController.cs:180,190</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-014</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Workflow artifacts</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can inspect quote workflow artifacts produced by the agent.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Artifact drawer and workflow artifact surfaces display generated artifacts, selected artifacts, and downloads.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Shell artifacts -&gt; AgentController artifact download -&gt; artifact/storage service</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Artifact drawer/workflow artifacts</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController artifacts/download</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests artifact download; QuoteEngineSourceTests artifacts | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, Storage/artifact service</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Artifact records/files</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs real artifact visual browser pass</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentLaunchShell.razor; AgentController.cs:402</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-015</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Artifact feedback</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can give feedback on generated previews/artifacts.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Inline viewer feedback posts sentiment/text feedback and reflects memory observation status.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Inline feedback UI -&gt; AgentController artifact-feedback -&gt; QuoteAgentService</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Thumb feedback and optional text</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController POST artifacts/{artifactId}/feedback</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngineSourceTests feedback; QuoteAgentEndpointTests feedback | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, Agent service, Customer memory</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Feedback records/memory observations</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs feedback persistence retest</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController.cs:240; QuoteAgentService.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-016</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3D part viewer</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can inspect uploaded/generated parts in a 3D viewer.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Part viewer loads GLB/viewer URLs, applies viewer settings, and pushes process/material/runtime state to JS.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QePartViewer -&gt; geometry runtime assets/telemetry -&gt; browser viewer</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QePartViewer.razor; QePartDetailCard.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">3D Model tab, artifact drawer viewer</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">GeometryRuntimeController manifest/assets/telemetry</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngineSourceTests viewer/runtime | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine client/BFF, Geometry runtime</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Viewer settings/telemetry</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs visual canvas smoke</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QePartViewer.razor; QePartDetailCard.razor; GeometryRuntimeController.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-017</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">DFM reporting</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can review manufacturability checks for FDM, SLA, and CNC.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">DFM tab renders process-specific report types and the agent can apply DFM reports to session state.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QeDfmTab/QePartDetailCard -&gt; AgentController dfm -&gt; SessionStore</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QeDfmTab.razor; QePartDetailCard.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">DFM tab and issue acknowledgement</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/dfm; QeDfmDtos</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngineSourceTests DFM | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, Geometry/DFM, SessionStore</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">DFM reports and acknowledgement state</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs process-specific fixture coverage</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QeDfmTab.razor; QePartDetailCard.razor; AgentController.cs:221</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-018</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Part configuration sidebar</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can select process, material, color, finish, tolerance, quantity, and options.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Configuration sidebar filters reference data and emits changes for quote estimation.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QePartConfigSidebar -&gt; reference-data/estimate DTOs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QePartConfigSidebar.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Part configuration controls</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteController reference-data/estimate</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngineSourceTests config sidebar | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine client/BFF, Pricing/Material services</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Part configuration state</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs keyboard/accessibility check</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QePartConfigSidebar.razor; QuoteController.cs:47,301</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-019</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Reference data and currencies</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can use current manufacturing reference data and currencies.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Reference endpoints expose processes/materials/finishes/tolerances/currency data used by workspace controls.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Workspace/client -&gt; quote/v1/reference-data and quote/v1/reference-data/currencies</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngineApiClient.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Reference-driven controls</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteController reference-data; ReferenceDataController currencies</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngineApiClientTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, Material/Pricing/Reference data</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Read-only reference data</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs stale-cache behavior check</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteController.cs:47; ReferenceDataController.cs:10-16; QuoteEngineApiClient.cs</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-020</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Estimate</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can request a quote estimate for configured parts.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Estimate endpoint prices configured parts and returns lead-time/total data for the summary/actions.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Workspace/summary -&gt; QuoteController estimate -&gt; Pricing service</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteWorkspace.razor; QeQuoteSummaryBar.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Estimate action</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Pricing/QuoteEngine tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteEngine BFF, PricingService</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Needs current pricing acceptance checks</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteController.cs:301; QeQuoteSummaryBar.razor</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QE-021</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Draft project</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can persist configured parts into a project draft.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Projects/draft endpoint creates or updates draft project data for the session/customer.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Workspace -&gt; QuoteController projects/draft -&gt; project/quote service</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QuoteWorkspace.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Make Studio handoff flow</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteController POST uploads/handoff</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineApiClientTests handoff | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Web BFF, Storage</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Handoff upload references</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs cross-app browser retest</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteWorkspace.razor; QuoteController.cs:235</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-011</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent attachments</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can attach uploaded files as context before asking the agent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent attachment endpoint registers uploaded files in session state and the shell previews attachments until sent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Composer attachments -&gt; AgentController attachments -&gt; SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Attachment preview and sent attachment display</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/attachments</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests attachment; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, SessionStore, Storage</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Session attachment records</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs attachment resend/removal browser pass</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:203; QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-012</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch attachments</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can draw or attach a hand sketch for the agent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch dialog captures sketch data and posts it to the agent sketch endpoint.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch UI -&gt; AgentController sketches -&gt; SessionStore/artifacts</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Hand sketch dialog/tools</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/sketches</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests sketches; source tests sketch disposal | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch artifact/context</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs mobile sketch browser pass</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:367; QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-013</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Google Drive connector</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can connect Google Drive and select source files.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Connector endpoints start OAuth, handle callback, expose status, list files, and return connector handoff links.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Connector UI -&gt; GoogleDriveConnectorController and AgentController connector endpoints</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentLaunchShell.razor; GoogleCallback.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">/auth/callback/google; connector panel</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">GoogleDriveConnectorController start/callback/status/files; AgentController connectors/handoff</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineSourceTests connector; endpoint tests where present | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Google Drive, Auth</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Connector tokens/status/file refs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs OAuth environment smoke</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">GoogleDriveConnectorController.cs; AgentController.cs:180,190</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-014</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Workflow artifacts</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can inspect quote workflow artifacts produced by the agent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Artifact drawer and workflow artifact surfaces display generated artifacts, selected artifacts, and downloads.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Shell artifacts -&gt; AgentController artifact download -&gt; artifact/storage service</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Artifact drawer/workflow artifacts</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController artifacts/download</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests artifact download; QuoteEngineSourceTests artifacts | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Storage/artifact service</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Artifact records/files</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs real artifact visual browser pass</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentLaunchShell.razor; AgentController.cs:402</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-015</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Artifact feedback</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can give feedback on generated previews/artifacts.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Inline viewer feedback posts sentiment/text feedback and reflects memory observation status.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Inline feedback UI -&gt; AgentController artifact-feedback -&gt; QuoteAgentService</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Thumb feedback and optional text</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST artifacts/{artifactId}/feedback</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineSourceTests feedback; QuoteAgentEndpointTests feedback | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Agent service, Customer memory</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Feedback records/memory observations</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs feedback persistence retest</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:240; QuoteAgentService.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-016</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">3D part viewer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can inspect uploaded/generated parts in a 3D viewer.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Part viewer loads GLB/viewer URLs, applies viewer settings, and pushes process/material/runtime state to JS.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QePartViewer -&gt; geometry runtime assets/telemetry -&gt; browser viewer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QePartViewer.razor; QePartDetailCard.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">3D Model tab, artifact drawer viewer</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">GeometryRuntimeController manifest/assets/telemetry</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineSourceTests viewer/runtime | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine client/BFF, Geometry runtime</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Viewer settings/telemetry</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs visual canvas smoke</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QePartViewer.razor; QePartDetailCard.razor; GeometryRuntimeController.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-017</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DFM reporting</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can review manufacturability checks for FDM, SLA, and CNC.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DFM tab renders process-specific report types and the agent can apply DFM reports to session state.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QeDfmTab/QePartDetailCard -&gt; AgentController dfm -&gt; SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QeDfmTab.razor; QePartDetailCard.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DFM tab and issue acknowledgement</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/dfm; QeDfmDtos</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineSourceTests DFM | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Geometry/DFM, SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">DFM reports and acknowledgement state</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs process-specific fixture coverage</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QeDfmTab.razor; QePartDetailCard.razor; AgentController.cs:221</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-018</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Part configuration sidebar</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can select process, material, color, finish, tolerance, quantity, and options.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Configuration sidebar filters reference data and emits changes for quote estimation.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QePartConfigSidebar -&gt; reference-data/estimate DTOs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QePartConfigSidebar.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Part configuration controls</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteController reference-data/estimate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineSourceTests config sidebar | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine client/BFF, Pricing/Material services</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Part configuration state</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs keyboard/accessibility check</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QePartConfigSidebar.razor; QuoteController.cs:47,301</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-019</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Reference data and currencies</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can use current manufacturing reference data and currencies.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Reference endpoints expose processes/materials/finishes/tolerances/currency data used by workspace controls.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Workspace/client -&gt; quote/v1/reference-data and quote/v1/reference-data/currencies</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineApiClient.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Reference-driven controls</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteController reference-data; ReferenceDataController currencies</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngineApiClientTests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, Material/Pricing/Reference data</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Read-only reference data</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs stale-cache behavior check</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteController.cs:47; ReferenceDataController.cs:10-16; QuoteEngineApiClient.cs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-020</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Estimate</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can request a quote estimate for configured parts.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Estimate endpoint prices configured parts and returns lead-time/total data for the summary/actions.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Workspace/summary -&gt; QuoteController estimate -&gt; Pricing service</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteWorkspace.razor; QeQuoteSummaryBar.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Estimate action</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Pricing/QuoteEngine tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, PricingService</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs current pricing acceptance checks</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteController.cs:301; QeQuoteSummaryBar.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-021</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Draft project</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can persist configured parts into a project draft.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Projects/draft endpoint creates or updates draft project data for the session/customer.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Workspace -&gt; QuoteController projects/draft -&gt; project/quote service</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Project draft action</x:t>
@@ -5057,7 +5021,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdac1550edeab47be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e50346a62624c9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8473,7 +8437,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e927a3a23d94da5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac7c35f8c1ea4ab2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8878,7 +8842,7 @@
         <x:v>GET quote/v1/agent/sessions/{sessionId}; GET quote/v1/agent/sessions/{sessionId}/messages resolves the mapped chatbot conversation, filters customer-safe roles, strips injected user-turn context, and returns NotFound when no accessible mapping exists.</x:v>
       </x:c>
       <x:c r="P6" s="3" t="str">
-        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_uses_mapped_chatbot_session_after_auth_return|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_uses_persisted_mapping_when_session_store_is_cold|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_restores_signed_in_customer_mapping_after_auth_return|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_denies_signed_in_customer_for_another_customers_session|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_strips_injected_session_context_from_persisted_user_turns|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_keeps_legacy_user_content_unmodified_when_no_context_marker_present|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_auth_completion_reloads_active_session_and_hydrates_messages|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract" --verbosity minimal passed 8/8.</x:v>
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_uses_mapped_chatbot_session_after_auth_return|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_uses_persisted_mapping_when_session_store_is_cold|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_restores_signed_in_customer_mapping_after_auth_return|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_denies_signed_in_customer_for_another_customers_session|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_strips_injected_session_context_from_persisted_user_turns|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_history_keeps_prior_user_content_unmodified_when_no_context_marker_present|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_auth_completion_reloads_active_session_and_hydrates_messages|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract" --verbosity minimal passed 8/8.</x:v>
       </x:c>
       <x:c r="Q6" s="3" t="str">
         <x:v>QuoteEngine Client, QuoteEngine BFF, QuoteAgentSessionStore, chatbot conversation service, Auth/session</x:v>
@@ -9157,85 +9121,85 @@
       </x:c>
     </x:row>
     <x:row r="11" ht="93.25" hidden="0">
-      <x:c r="A11" s="3" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="B11" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C11" s="3" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="D11" s="3" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="E11" s="3" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="F11" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G11" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="H11" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="I11" s="3" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="J11" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="K11" s="3" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="L11" s="3" t="s">
-        <x:v>470</x:v>
-      </x:c>
-      <x:c r="M11" s="3" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="N11" s="3" t="s">
-        <x:v>472</x:v>
-      </x:c>
-      <x:c r="O11" s="3" t="s">
-        <x:v>473</x:v>
-      </x:c>
-      <x:c r="P11" s="3" t="s">
-        <x:v>474</x:v>
-      </x:c>
-      <x:c r="Q11" s="3" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="R11" s="3" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="S11" s="3" t="s">
-        <x:v>477</x:v>
-      </x:c>
-      <x:c r="T11" s="3" t="s">
-        <x:v>478</x:v>
-      </x:c>
-      <x:c r="U11" s="3" t="s">
-        <x:v>52</x:v>
+      <x:c r="A11" s="3" t="str">
+        <x:v>QE-010</x:v>
+      </x:c>
+      <x:c r="B11" s="3" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C11" s="3" t="str">
+        <x:v>Web handoff import</x:v>
+      </x:c>
+      <x:c r="D11" s="3" t="str">
+        <x:v>As a customer, I can continue from a public web quote upload into the workspace.</x:v>
+      </x:c>
+      <x:c r="E11" s="3" t="str">
+        <x:v>Customers arriving from Maliev.Web with a signed upload handoff token can import verified web-uploaded files into the active QuoteEngine workspace; invalid or out-of-scope handoffs are rejected, imported parts retain viewer/thumbnail/file metadata, and the agent session is refreshed with imported attachment context.</x:v>
+      </x:c>
+      <x:c r="F11" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G11" s="3" t="str">
+        <x:v>Focused current-state web handoff import tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H11" s="3" t="str">
+        <x:v>No behavior error observed in focused QuoteEngine handoff retest; live cross-app browser handoff from Maliev.Web to QuoteEngine still not executed in this slice.</x:v>
+      </x:c>
+      <x:c r="I11" s="3" t="str">
+        <x:v>No app fix applied for QE-010; current code path is covered by focused BFF/source tests.</x:v>
+      </x:c>
+      <x:c r="J11" s="3" t="str">
+        <x:v>Passed 6/6 focused tests: signed web upload handoff import, unsigned handoff rejection, signed out-of-scope storage-path rejection, QuoteWorkspace viewer-field hydration, imported attachment agent registration, and startup loader query-handoff handling.</x:v>
+      </x:c>
+      <x:c r="K11" s="3" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L11" s="3" t="str">
+        <x:v>Maliev.Web signed handoff token -&gt; QuoteWorkspace ?handoff route sync -&gt; QuoteEngineApiClient ImportHandoffAsync -&gt; QuoteController uploads/handoff -&gt; QuoteUploadHandoffToken/store import -&gt; QuoteWorkspace part hydration and agent attachment registration</x:v>
+      </x:c>
+      <x:c r="M11" s="3" t="str">
+        <x:v>QuoteWorkspace.razor; QuoteEngineApiClient; QuoteController; QuoteUploadHandoffToken; QuoteEngineDtos</x:v>
+      </x:c>
+      <x:c r="N11" s="3" t="str">
+        <x:v>QuoteWorkspace reads SupplyParameterFromQuery handoff, SynchronizeRouteStateAsync calls ImportHandoffAsync, clears retained browser files, hydrates imported parts with viewer metadata, selects the first part, recalculates, and registers imported attachments with the agent shell.</x:v>
+      </x:c>
+      <x:c r="O11" s="3" t="str">
+        <x:v>POST quote/v1/uploads/handoff requires a signed handoff token, rejects invalid tokens, verifies storage paths belong to the web quote session, resolves optional customer id, and returns QuoteUploadHandoffResponse parts with viewerGlbUrl, viewerStoragePath, viewerFileExtension, thumbnailUrl, contentType, and fileSizeBytes.</x:v>
+      </x:c>
+      <x:c r="P11" s="3" t="str">
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteEngineEndpointTests.UploadHandoff_imports_web_uploaded_files_into_active_workspace|FullyQualifiedName~QuoteEngineEndpointTests.UploadHandoff_rejects_unsigned_web_uploaded_files|FullyQualifiedName~QuoteEngineEndpointTests.UploadHandoff_rejects_signed_storage_paths_outside_web_quote_session|FullyQualifiedName~QuoteEngineSourceTests.QuoteWorkspace_imports_handoff_viewer_fields_for_canvas_rendering|FullyQualifiedName~QuoteEngineSourceTests.QuoteWorkspace_registers_web_handoff_uploads_with_agent_shell|FullyQualifiedName~QuoteEngineSourceTests.Startup_loader_tells_make_studio_story_with_progress_contract" --verbosity minimal passed 6/6.</x:v>
+      </x:c>
+      <x:c r="Q11" s="3" t="str">
+        <x:v>Maliev.Web upload handoff producer, QuoteEngine Client, QuoteEngine BFF, handoff token verifier, prototype workspace store, agent attachment registration</x:v>
+      </x:c>
+      <x:c r="R11" s="3" t="str">
+        <x:v>Verified handoff token, quote session id, imported part view models, viewer and thumbnail metadata, agent attachment state, workspace selected part and recalculated estimate state</x:v>
+      </x:c>
+      <x:c r="S11" s="3" t="str">
+        <x:v>Needs live cross-app browser retest from Maliev.Web upload handoff into a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T11" s="3" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor:131,364,718,752,771; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs:78; Maliev.QuoteEngine.Bff/Controllers/QuoteController.cs:235; Maliev.QuoteEngine.Shared/Quotes/QuoteEngineDtos.cs:95,153; Maliev.QuoteEngine.Tests/QuoteEngineEndpointTests.cs:2181,2237,2263; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:2292,2310,2916</x:v>
+      </x:c>
+      <x:c r="U11" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
       <x:c r="A12" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B12" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C12" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D12" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E12" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F12" s="3" t="s">
         <x:v>37</x:v>
@@ -9256,31 +9220,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L12" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="M12" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N12" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="O12" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="P12" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="Q12" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="R12" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="S12" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="T12" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="U12" s="3" t="s">
         <x:v>52</x:v>
@@ -9288,19 +9252,19 @@
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>37</x:v>
@@ -9321,31 +9285,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
+        <x:v>474</x:v>
+      </x:c>
+      <x:c r="R13" s="3" t="s">
+        <x:v>486</x:v>
+      </x:c>
+      <x:c r="S13" s="3" t="s">
         <x:v>487</x:v>
       </x:c>
-      <x:c r="R13" s="3" t="s">
-        <x:v>499</x:v>
-      </x:c>
-      <x:c r="S13" s="3" t="s">
-        <x:v>500</x:v>
-      </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>52</x:v>
@@ -9353,19 +9317,19 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
@@ -9386,31 +9350,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9418,19 +9382,19 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
@@ -9451,31 +9415,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>520</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>525</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>526</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9483,19 +9447,19 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>527</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
@@ -9516,31 +9480,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>532</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>534</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9548,19 +9512,19 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
@@ -9581,31 +9545,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9613,19 +9577,19 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
@@ -9646,31 +9610,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>561</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>562</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>563</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9678,19 +9642,19 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>568</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
@@ -9711,31 +9675,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>573</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>574</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>575</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9743,19 +9707,19 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>580</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
@@ -9776,31 +9740,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>585</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>586</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>587</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9808,19 +9772,19 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>592</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>593</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
@@ -9841,31 +9805,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>598</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>599</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>600</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -9873,19 +9837,19 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>605</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
@@ -9906,31 +9870,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>606</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>611</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>612</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>613</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -9938,19 +9902,19 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
@@ -9971,31 +9935,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>618</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>624</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>625</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>626</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -10003,19 +9967,19 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
@@ -10036,31 +10000,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>632</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -10068,19 +10032,19 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
@@ -10101,31 +10065,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10133,19 +10097,19 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
@@ -10166,31 +10130,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>655</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>660</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>661</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>662</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10198,19 +10162,19 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>667</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
@@ -10231,31 +10195,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>668</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>673</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>674</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
-        <x:v>675</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10263,19 +10227,19 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>680</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
@@ -10296,31 +10260,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>685</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>686</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>687</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10328,19 +10292,19 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>692</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
@@ -10361,31 +10325,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>697</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>698</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>699</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10393,19 +10357,19 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>704</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>705</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
@@ -10426,31 +10390,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>710</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>711</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>712</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10458,19 +10422,19 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>717</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>718</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
@@ -10491,31 +10455,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10523,19 +10487,19 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
@@ -10556,31 +10520,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10588,19 +10552,19 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>742</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>743</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
@@ -10621,31 +10585,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>748</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>749</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>750</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10653,7 +10617,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10662,10 +10626,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>755</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>756</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
@@ -10686,31 +10650,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>761</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>762</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>763</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10718,19 +10682,19 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>768</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
@@ -10751,31 +10715,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>769</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>774</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>775</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>776</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10783,19 +10747,19 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
@@ -10816,31 +10780,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>781</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>787</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>788</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10848,19 +10812,19 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>789</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
@@ -10881,31 +10845,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>795</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -10913,19 +10877,19 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>802</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
@@ -10946,31 +10910,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>471</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>811</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>812</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -10978,19 +10942,19 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>813</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>814</x:v>
+        <x:v>802</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>815</x:v>
+        <x:v>803</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>816</x:v>
+        <x:v>804</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
@@ -11011,31 +10975,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>817</x:v>
+        <x:v>805</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>818</x:v>
+        <x:v>806</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>819</x:v>
+        <x:v>807</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>820</x:v>
+        <x:v>808</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>821</x:v>
+        <x:v>809</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>822</x:v>
+        <x:v>810</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>823</x:v>
+        <x:v>811</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>824</x:v>
+        <x:v>812</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -11044,7 +11008,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R98eb820354214b08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2039768eee124d4b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-011 attachment retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R55ec781b4d914d84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R875633f7b0ee44f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R04ac7350e4234996"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R83b31bd731da41ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcbb80bf8ec4943ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R2ac7781be66846b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rdd0d9d6738084e57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf20af795d9654764"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1411,64 +1411,31 @@
     <x:t xml:space="preserve">AgentController.cs:271; QuoteAgentLaunchShell.razor</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">QE-011</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent attachments</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can attach uploaded files as context before asking the agent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Agent attachment endpoint registers uploaded files in session state and the shell previews attachments until sent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Composer attachments -&gt; AgentController attachments -&gt; SessionStore</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Attachment preview and sent attachment display</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/attachments</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests attachment; QuoteAgentLaunchShell source tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
+    <x:t xml:space="preserve">QE-012</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sketch attachments</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">As a customer, I can draw or attach a hand sketch for the agent.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sketch dialog captures sketch data and posts it to the agent sketch endpoint.</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Sketch UI -&gt; AgentController sketches -&gt; SessionStore/artifacts</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">Hand sketch dialog/tools</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/sketches</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">QuoteAgentEndpointTests sketches; source tests sketch disposal | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QuoteEngine BFF, SessionStore, Storage</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Session attachment records</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs attachment resend/removal browser pass</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:203; QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-012</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch attachments</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can draw or attach a hand sketch for the agent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch dialog captures sketch data and posts it to the agent sketch endpoint.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch UI -&gt; AgentController sketches -&gt; SessionStore/artifacts</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Hand sketch dialog/tools</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/sketches</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests sketches; source tests sketch disposal | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Sketch artifact/context</x:t>
@@ -5021,7 +4988,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e50346a62624c9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2f86f9681414ec9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8437,7 +8404,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac7c35f8c1ea4ab2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dd5de2b59ae4583"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9186,85 +9153,85 @@
       </x:c>
     </x:row>
     <x:row r="12" ht="107.25" hidden="0">
-      <x:c r="A12" s="3" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="B12" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C12" s="3" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="D12" s="3" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="E12" s="3" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="F12" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G12" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="H12" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="I12" s="3" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="J12" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="K12" s="3" t="s">
-        <x:v>188</x:v>
-      </x:c>
-      <x:c r="L12" s="3" t="s">
-        <x:v>470</x:v>
-      </x:c>
-      <x:c r="M12" s="3" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="N12" s="3" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="O12" s="3" t="s">
-        <x:v>472</x:v>
-      </x:c>
-      <x:c r="P12" s="3" t="s">
-        <x:v>473</x:v>
-      </x:c>
-      <x:c r="Q12" s="3" t="s">
-        <x:v>474</x:v>
-      </x:c>
-      <x:c r="R12" s="3" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="S12" s="3" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="T12" s="3" t="s">
-        <x:v>477</x:v>
-      </x:c>
-      <x:c r="U12" s="3" t="s">
-        <x:v>52</x:v>
+      <x:c r="A12" s="3" t="str">
+        <x:v>QE-011</x:v>
+      </x:c>
+      <x:c r="B12" s="3" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C12" s="3" t="str">
+        <x:v>Agent attachments</x:v>
+      </x:c>
+      <x:c r="D12" s="3" t="str">
+        <x:v>As a customer, I can attach uploaded files as context before asking the agent.</x:v>
+      </x:c>
+      <x:c r="E12" s="3" t="str">
+        <x:v>Customers can keep uploaded CAD, drawing, photo, sketch, and supplemental files as pending composer attachments until they send a message; the shell shows previews, status, overflow, selection, and removal controls, sends attachment metadata with the customer turn, and the BFF registration endpoint updates session attachment state while distinguishing geometry-gating CAD from supplemental files.</x:v>
+      </x:c>
+      <x:c r="F12" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G12" s="3" t="str">
+        <x:v>Focused current-state agent attachment tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H12" s="3" t="str">
+        <x:v>No behavior error observed in focused QuoteEngine attachment retest; live browser resend/removal interaction still not executed in this slice.</x:v>
+      </x:c>
+      <x:c r="I12" s="3" t="str">
+        <x:v>No app fix applied for QE-011; current code path is covered by focused BFF/source tests.</x:v>
+      </x:c>
+      <x:c r="J12" s="3" t="str">
+        <x:v>Passed 5/5 focused tests: CAD attachment registration materializes uploaded part state, supplemental registration stays out of geometry gate, composer previews/removes attachments until send, sent user attachments render outside the neutral message bubble, and shell visual contract remains present.</x:v>
+      </x:c>
+      <x:c r="K12" s="3" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L12" s="3" t="str">
+        <x:v>QuoteWorkspace upload/sketch events -&gt; QuoteAgentLaunchShell pending composer attachments -&gt; QuoteAgentMessageRequest attachment payload -&gt; QuoteEngineApiClient RegisterAgentAttachmentsAsync -&gt; AgentController sessions/{sessionId}/attachments -&gt; QuoteAgentService -&gt; QuoteAgentSessionStore attachment dedupe and geometry-gate classification</x:v>
+      </x:c>
+      <x:c r="M12" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; QuoteEngineApiClient; AgentController; QuoteAgentService; QuoteAgentSessionStore; QuoteAgentDtos</x:v>
+      </x:c>
+      <x:c r="N12" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell renders qe-agent-composer-attachments with aria-live status, previews up to five pending attachments, shows upload progress and overflow count, allows selecting an uploaded part, removes pending attachments, clears the pending list on send, and renders sent attachments in the message thread.</x:v>
+      </x:c>
+      <x:c r="O12" s="3" t="str">
+        <x:v>POST quote/v1/agent/sessions/{sessionId}/attachments validates QuoteAgentAttachmentRegisterRequest, normalizes message/language, gets or creates the session, stores customer id when available, adds attachments to session state, dedupes by attachment id or upload id, and marks CAD/geometry/3D attachments as satisfying the geometry gate while supplemental files remain non-geometry context.</x:v>
+      </x:c>
+      <x:c r="P12" s="3" t="str">
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_attachment_registration_materializes_uploaded_cad_state|FullyQualifiedName~QuoteAgentEndpointTests.Agent_attachment_registration_keeps_supplemental_files_out_of_geometry_gate|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_with_supplemental_attachment_preserves_geometry_gate|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_previews_attachments_until_customer_sends_message|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_renders_sent_user_attachments_outside_neutral_message_bubble|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract" --verbosity minimal passed 5/5.</x:v>
+      </x:c>
+      <x:c r="Q12" s="3" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, agent session store, upload/session attachment metadata, chatbot send payload</x:v>
+      </x:c>
+      <x:c r="R12" s="3" t="str">
+        <x:v>Pending composer attachment previews, sent message attachment metadata, QuoteAgentAttachmentDto payloads, session attachment records, generated part/artifact state for CAD uploads, geometry gate state</x:v>
+      </x:c>
+      <x:c r="S12" s="3" t="str">
+        <x:v>Needs live browser retest for attachment preview, selection, removal, overflow, resend, and sent-message rendering against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T12" s="3" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:1131,2803,2822,4299,5998; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs:410; Maliev.QuoteEngine.Bff/Controllers/AgentController.cs:203; Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:536; Maliev.QuoteEngine.Bff/Services/QuoteAgentSessionStore.cs:31,258; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs:82,138; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:1602,1698; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1933,1996</x:v>
+      </x:c>
+      <x:c r="U12" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
       <x:c r="A13" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B13" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C13" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D13" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E13" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F13" s="3" t="s">
         <x:v>37</x:v>
@@ -9285,31 +9252,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L13" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="M13" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N13" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="O13" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="P13" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="Q13" s="3" t="s">
         <x:v>474</x:v>
       </x:c>
       <x:c r="R13" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="S13" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="T13" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="U13" s="3" t="s">
         <x:v>52</x:v>
@@ -9317,19 +9284,19 @@
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
@@ -9350,31 +9317,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>499</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>500</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9382,19 +9349,19 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
@@ -9415,31 +9382,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9447,19 +9414,19 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
@@ -9480,31 +9447,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>520</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>525</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9512,19 +9479,19 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>526</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>527</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
@@ -9545,31 +9512,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>532</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>534</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9577,19 +9544,19 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
@@ -9610,31 +9577,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9642,19 +9609,19 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
@@ -9675,31 +9642,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>561</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>562</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>563</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9707,19 +9674,19 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>568</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
@@ -9740,31 +9707,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>573</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>574</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>575</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9772,19 +9739,19 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>580</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
@@ -9805,31 +9772,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>585</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>586</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>587</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -9837,19 +9804,19 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>592</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
@@ -9870,31 +9837,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>593</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>598</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>599</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>600</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -9902,19 +9869,19 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>605</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
@@ -9935,31 +9902,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>606</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>611</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>612</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>613</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -9967,19 +9934,19 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>618</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
@@ -10000,31 +9967,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>624</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>625</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>626</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -10032,19 +9999,19 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
@@ -10065,31 +10032,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>632</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10097,19 +10064,19 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
@@ -10130,31 +10097,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10162,19 +10129,19 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>655</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
@@ -10195,31 +10162,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>660</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>661</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>662</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10227,19 +10194,19 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>667</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>668</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
@@ -10260,31 +10227,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>673</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>674</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>675</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10292,19 +10259,19 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>680</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
@@ -10325,31 +10292,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>685</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>686</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>687</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10357,19 +10324,19 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>692</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
@@ -10390,31 +10357,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>697</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>698</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>699</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10422,19 +10389,19 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>704</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>705</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
@@ -10455,31 +10422,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>710</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>711</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>712</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10487,19 +10454,19 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>717</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>718</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
@@ -10520,31 +10487,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10552,19 +10519,19 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
@@ -10585,31 +10552,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10617,7 +10584,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>742</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10626,10 +10593,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>743</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
@@ -10650,31 +10617,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>748</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>749</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>750</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10682,19 +10649,19 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>755</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>756</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
@@ -10715,31 +10682,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>761</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>762</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>763</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10747,19 +10714,19 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>768</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
@@ -10780,31 +10747,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>769</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>774</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>775</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>776</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10812,19 +10779,19 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
@@ -10845,31 +10812,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>781</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>787</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>788</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -10877,19 +10844,19 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>789</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
@@ -10910,31 +10877,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>795</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -10942,19 +10909,19 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>790</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>802</x:v>
+        <x:v>791</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>803</x:v>
+        <x:v>792</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>804</x:v>
+        <x:v>793</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
@@ -10975,31 +10942,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>805</x:v>
+        <x:v>794</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>806</x:v>
+        <x:v>795</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>807</x:v>
+        <x:v>796</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>808</x:v>
+        <x:v>797</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>809</x:v>
+        <x:v>798</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>810</x:v>
+        <x:v>799</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>811</x:v>
+        <x:v>800</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>812</x:v>
+        <x:v>801</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -11008,7 +10975,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2039768eee124d4b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3665c4158cc4e66"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-012 sketch retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rcbb80bf8ec4943ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R2ac7781be66846b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rdd0d9d6738084e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rf20af795d9654764"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Re6fafe2742cb4b66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Red9803fe13de4b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5a6fb379673443d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rffa4b4af29db4596"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1409,42 +1409,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">AgentController.cs:271; QuoteAgentLaunchShell.razor</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QE-012</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch attachments</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">As a customer, I can draw or attach a hand sketch for the agent.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch dialog captures sketch data and posts it to the agent sketch endpoint.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch UI -&gt; AgentController sketches -&gt; SessionStore/artifacts</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Hand sketch dialog/tools</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController POST sessions/{sessionId}/sketches</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteAgentEndpointTests sketches; source tests sketch disposal | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">QuoteEngine BFF, SessionStore, Storage</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sketch artifact/context</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Needs mobile sketch browser pass</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">AgentController.cs:367; QuoteAgentLaunchShell.razor</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">QE-013</x:t>
@@ -4988,7 +4952,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2f86f9681414ec9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raf030c1f80b44b1e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8404,7 +8368,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2dd5de2b59ae4583"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R733049c3c13f45b6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9218,85 +9182,85 @@
       </x:c>
     </x:row>
     <x:row r="13" ht="93.25" hidden="0">
-      <x:c r="A13" s="3" t="s">
-        <x:v>466</x:v>
-      </x:c>
-      <x:c r="B13" s="3" t="s">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="C13" s="3" t="s">
-        <x:v>467</x:v>
-      </x:c>
-      <x:c r="D13" s="3" t="s">
-        <x:v>468</x:v>
-      </x:c>
-      <x:c r="E13" s="3" t="s">
-        <x:v>469</x:v>
-      </x:c>
-      <x:c r="F13" s="3" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="G13" s="3" t="s">
-        <x:v>442</x:v>
-      </x:c>
-      <x:c r="H13" s="3" t="s">
-        <x:v>443</x:v>
-      </x:c>
-      <x:c r="I13" s="3" t="s">
-        <x:v>444</x:v>
-      </x:c>
-      <x:c r="J13" s="3" t="s">
-        <x:v>41</x:v>
-      </x:c>
-      <x:c r="K13" s="3" t="s">
-        <x:v>42</x:v>
-      </x:c>
-      <x:c r="L13" s="3" t="s">
-        <x:v>470</x:v>
-      </x:c>
-      <x:c r="M13" s="3" t="s">
-        <x:v>446</x:v>
-      </x:c>
-      <x:c r="N13" s="3" t="s">
-        <x:v>471</x:v>
-      </x:c>
-      <x:c r="O13" s="3" t="s">
-        <x:v>472</x:v>
-      </x:c>
-      <x:c r="P13" s="3" t="s">
-        <x:v>473</x:v>
-      </x:c>
-      <x:c r="Q13" s="3" t="s">
-        <x:v>474</x:v>
-      </x:c>
-      <x:c r="R13" s="3" t="s">
-        <x:v>475</x:v>
-      </x:c>
-      <x:c r="S13" s="3" t="s">
-        <x:v>476</x:v>
-      </x:c>
-      <x:c r="T13" s="3" t="s">
-        <x:v>477</x:v>
-      </x:c>
-      <x:c r="U13" s="3" t="s">
-        <x:v>52</x:v>
+      <x:c r="A13" s="3" t="str">
+        <x:v>QE-012</x:v>
+      </x:c>
+      <x:c r="B13" s="3" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C13" s="3" t="str">
+        <x:v>Sketch attachments</x:v>
+      </x:c>
+      <x:c r="D13" s="3" t="str">
+        <x:v>As a customer, I can draw or attach a hand sketch for the agent.</x:v>
+      </x:c>
+      <x:c r="E13" s="3" t="str">
+        <x:v>Customers can open the hand-sketch dialog from the agent workspace, draw with mouse or pen, erase, undo, redo, insert or paste an image, name the sketch, attach it as a PNG, preview it as a pending composer attachment, and send it as image context without satisfying the CAD geometry gate by itself.</x:v>
+      </x:c>
+      <x:c r="F13" s="3" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G13" s="3" t="str">
+        <x:v>Focused current-state sketch attachment tests passed 2026-06-24.</x:v>
+      </x:c>
+      <x:c r="H13" s="3" t="str">
+        <x:v>No behavior error observed in focused QuoteEngine sketch retest; live mobile/touch sketch browser interaction still not executed in this slice.</x:v>
+      </x:c>
+      <x:c r="I13" s="3" t="str">
+        <x:v>No app fix applied for QE-012; current code path is covered by focused BFF/source tests.</x:v>
+      </x:c>
+      <x:c r="J13" s="3" t="str">
+        <x:v>Passed 6/6 focused tests: session-scoped sketch upload and download redirect, uploaded sketch media inlined for chatbot stream, sketchboard clipboard isolation, sketch canvas disposal, pending attachment preview/send behavior, and shell visual contract.</x:v>
+      </x:c>
+      <x:c r="K13" s="3" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L13" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell hand-sketch dialog -&gt; quote-agent-sketch.js canvas module -&gt; multipart POST quote/v1/agent/sessions/{sessionId}/sketches -&gt; AgentController UploadSketch -&gt; QuoteAgentService UploadSketchAsync -&gt; UploadService signed URL -&gt; pending ComposerAttachmentPreview -&gt; QuoteAgentMessageRequest image attachment</x:v>
+      </x:c>
+      <x:c r="M13" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; quote-agent-sketch.js; quote-upload.js; AgentController; QuoteAgentService; UploadSketchResponse; QuoteAgentDtos</x:v>
+      </x:c>
+      <x:c r="N13" s="3" t="str">
+        <x:v>QuoteAgentLaunchShell renders a modal hand-sketch canvas with title, color swatches, eraser, undo, redo, image insert, clear, and attach controls; it initializes /js/quote-agent-sketch.js, exports the canvas, uploads a PNG, queues a sketch ComposerAttachmentPreview, disposes the canvas on close/dispose, and refreshes the pending attachment preview.</x:v>
+      </x:c>
+      <x:c r="O13" s="3" t="str">
+        <x:v>POST quote/v1/agent/sessions/{sessionId}/sketches requires a non-empty image file, copies the multipart file to memory, stores it through UploadService at agent/sketches/{sessionId:N}/{fileName}, streams bytes with Content-Range, returns UploadSketchResponse with uploadId/storagePath/signed URL, and artifact download only redirects for the same session-owned sketch path.</x:v>
+      </x:c>
+      <x:c r="P13" s="3" t="str">
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_sketch_upload_returns_signed_url_and_download_redirect_is_session_scoped|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_stream_with_uploaded_sketch_inlines_storage_media_for_chatbot|FullyQualifiedName~QuoteEngineSourceTests.QuoteUploadJs_does_not_steal_sketchboard_clipboard_images|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_disposes_sketch_canvas_when_component_is_disposed|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_previews_attachments_until_customer_sends_message|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_has_monochrome_chatgpt_like_contract" --verbosity minimal passed 6/6.</x:v>
+      </x:c>
+      <x:c r="Q13" s="3" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, UploadService client, agent session state, chatbot stream media payload</x:v>
+      </x:c>
+      <x:c r="R13" s="3" t="str">
+        <x:v>Sketch canvas image bytes, UploadSketchResponse upload id/storage path/signed URL, pending sketch composer attachment, sent image attachment payload, session-scoped sketch artifact download authorization</x:v>
+      </x:c>
+      <x:c r="S13" s="3" t="str">
+        <x:v>Needs live browser retest for mobile/touch drawing, image paste/insert, undo/redo/erase, upload failure UI, pending preview, and send behavior against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T13" s="3" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:1386,1457,2665,4533,4693,4722,4731,4766; Maliev.QuoteEngine.Client/wwwroot/js/quote-agent-sketch.js:530,553,562,590,603,620,627; Maliev.QuoteEngine.Client/wwwroot/js/quote-upload.js:205; Maliev.QuoteEngine.Bff/Controllers/AgentController.cs:367; Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:1071,6373; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs:858; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:910,1178; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1655,1669,1933</x:v>
+      </x:c>
+      <x:c r="U13" s="3" t="str">
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="93.25" hidden="0">
       <x:c r="A14" s="3" t="s">
-        <x:v>478</x:v>
+        <x:v>466</x:v>
       </x:c>
       <x:c r="B14" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C14" s="3" t="s">
-        <x:v>479</x:v>
+        <x:v>467</x:v>
       </x:c>
       <x:c r="D14" s="3" t="s">
-        <x:v>480</x:v>
+        <x:v>468</x:v>
       </x:c>
       <x:c r="E14" s="3" t="s">
-        <x:v>481</x:v>
+        <x:v>469</x:v>
       </x:c>
       <x:c r="F14" s="3" t="s">
         <x:v>37</x:v>
@@ -9317,31 +9281,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L14" s="3" t="s">
-        <x:v>482</x:v>
+        <x:v>470</x:v>
       </x:c>
       <x:c r="M14" s="3" t="s">
-        <x:v>483</x:v>
+        <x:v>471</x:v>
       </x:c>
       <x:c r="N14" s="3" t="s">
-        <x:v>484</x:v>
+        <x:v>472</x:v>
       </x:c>
       <x:c r="O14" s="3" t="s">
-        <x:v>485</x:v>
+        <x:v>473</x:v>
       </x:c>
       <x:c r="P14" s="3" t="s">
-        <x:v>486</x:v>
+        <x:v>474</x:v>
       </x:c>
       <x:c r="Q14" s="3" t="s">
-        <x:v>487</x:v>
+        <x:v>475</x:v>
       </x:c>
       <x:c r="R14" s="3" t="s">
-        <x:v>488</x:v>
+        <x:v>476</x:v>
       </x:c>
       <x:c r="S14" s="3" t="s">
-        <x:v>489</x:v>
+        <x:v>477</x:v>
       </x:c>
       <x:c r="T14" s="3" t="s">
-        <x:v>490</x:v>
+        <x:v>478</x:v>
       </x:c>
       <x:c r="U14" s="3" t="s">
         <x:v>52</x:v>
@@ -9349,19 +9313,19 @@
     </x:row>
     <x:row r="15" ht="107.25" hidden="0">
       <x:c r="A15" s="3" t="s">
-        <x:v>491</x:v>
+        <x:v>479</x:v>
       </x:c>
       <x:c r="B15" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C15" s="3" t="s">
-        <x:v>492</x:v>
+        <x:v>480</x:v>
       </x:c>
       <x:c r="D15" s="3" t="s">
-        <x:v>493</x:v>
+        <x:v>481</x:v>
       </x:c>
       <x:c r="E15" s="3" t="s">
-        <x:v>494</x:v>
+        <x:v>482</x:v>
       </x:c>
       <x:c r="F15" s="3" t="s">
         <x:v>37</x:v>
@@ -9382,31 +9346,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L15" s="3" t="s">
-        <x:v>495</x:v>
+        <x:v>483</x:v>
       </x:c>
       <x:c r="M15" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N15" s="3" t="s">
-        <x:v>496</x:v>
+        <x:v>484</x:v>
       </x:c>
       <x:c r="O15" s="3" t="s">
-        <x:v>497</x:v>
+        <x:v>485</x:v>
       </x:c>
       <x:c r="P15" s="3" t="s">
-        <x:v>498</x:v>
+        <x:v>486</x:v>
       </x:c>
       <x:c r="Q15" s="3" t="s">
-        <x:v>499</x:v>
+        <x:v>487</x:v>
       </x:c>
       <x:c r="R15" s="3" t="s">
-        <x:v>500</x:v>
+        <x:v>488</x:v>
       </x:c>
       <x:c r="S15" s="3" t="s">
-        <x:v>501</x:v>
+        <x:v>489</x:v>
       </x:c>
       <x:c r="T15" s="3" t="s">
-        <x:v>502</x:v>
+        <x:v>490</x:v>
       </x:c>
       <x:c r="U15" s="3" t="s">
         <x:v>52</x:v>
@@ -9414,19 +9378,19 @@
     </x:row>
     <x:row r="16" ht="107.25" hidden="0">
       <x:c r="A16" s="3" t="s">
-        <x:v>503</x:v>
+        <x:v>491</x:v>
       </x:c>
       <x:c r="B16" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C16" s="3" t="s">
-        <x:v>504</x:v>
+        <x:v>492</x:v>
       </x:c>
       <x:c r="D16" s="3" t="s">
-        <x:v>505</x:v>
+        <x:v>493</x:v>
       </x:c>
       <x:c r="E16" s="3" t="s">
-        <x:v>506</x:v>
+        <x:v>494</x:v>
       </x:c>
       <x:c r="F16" s="3" t="s">
         <x:v>37</x:v>
@@ -9447,31 +9411,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L16" s="3" t="s">
-        <x:v>507</x:v>
+        <x:v>495</x:v>
       </x:c>
       <x:c r="M16" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N16" s="3" t="s">
-        <x:v>508</x:v>
+        <x:v>496</x:v>
       </x:c>
       <x:c r="O16" s="3" t="s">
-        <x:v>509</x:v>
+        <x:v>497</x:v>
       </x:c>
       <x:c r="P16" s="3" t="s">
-        <x:v>510</x:v>
+        <x:v>498</x:v>
       </x:c>
       <x:c r="Q16" s="3" t="s">
-        <x:v>511</x:v>
+        <x:v>499</x:v>
       </x:c>
       <x:c r="R16" s="3" t="s">
-        <x:v>512</x:v>
+        <x:v>500</x:v>
       </x:c>
       <x:c r="S16" s="3" t="s">
-        <x:v>513</x:v>
+        <x:v>501</x:v>
       </x:c>
       <x:c r="T16" s="3" t="s">
-        <x:v>514</x:v>
+        <x:v>502</x:v>
       </x:c>
       <x:c r="U16" s="3" t="s">
         <x:v>52</x:v>
@@ -9479,19 +9443,19 @@
     </x:row>
     <x:row r="17" ht="93.25" hidden="0">
       <x:c r="A17" s="3" t="s">
-        <x:v>515</x:v>
+        <x:v>503</x:v>
       </x:c>
       <x:c r="B17" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C17" s="3" t="s">
-        <x:v>516</x:v>
+        <x:v>504</x:v>
       </x:c>
       <x:c r="D17" s="3" t="s">
-        <x:v>517</x:v>
+        <x:v>505</x:v>
       </x:c>
       <x:c r="E17" s="3" t="s">
-        <x:v>518</x:v>
+        <x:v>506</x:v>
       </x:c>
       <x:c r="F17" s="3" t="s">
         <x:v>37</x:v>
@@ -9512,31 +9476,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L17" s="3" t="s">
-        <x:v>519</x:v>
+        <x:v>507</x:v>
       </x:c>
       <x:c r="M17" s="3" t="s">
-        <x:v>520</x:v>
+        <x:v>508</x:v>
       </x:c>
       <x:c r="N17" s="3" t="s">
-        <x:v>521</x:v>
+        <x:v>509</x:v>
       </x:c>
       <x:c r="O17" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="P17" s="3" t="s">
-        <x:v>523</x:v>
+        <x:v>511</x:v>
       </x:c>
       <x:c r="Q17" s="3" t="s">
-        <x:v>524</x:v>
+        <x:v>512</x:v>
       </x:c>
       <x:c r="R17" s="3" t="s">
-        <x:v>525</x:v>
+        <x:v>513</x:v>
       </x:c>
       <x:c r="S17" s="3" t="s">
-        <x:v>526</x:v>
+        <x:v>514</x:v>
       </x:c>
       <x:c r="T17" s="3" t="s">
-        <x:v>527</x:v>
+        <x:v>515</x:v>
       </x:c>
       <x:c r="U17" s="3" t="s">
         <x:v>52</x:v>
@@ -9544,19 +9508,19 @@
     </x:row>
     <x:row r="18" ht="93.25" hidden="0">
       <x:c r="A18" s="3" t="s">
-        <x:v>528</x:v>
+        <x:v>516</x:v>
       </x:c>
       <x:c r="B18" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C18" s="3" t="s">
-        <x:v>529</x:v>
+        <x:v>517</x:v>
       </x:c>
       <x:c r="D18" s="3" t="s">
-        <x:v>530</x:v>
+        <x:v>518</x:v>
       </x:c>
       <x:c r="E18" s="3" t="s">
-        <x:v>531</x:v>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="F18" s="3" t="s">
         <x:v>37</x:v>
@@ -9577,31 +9541,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L18" s="3" t="s">
-        <x:v>532</x:v>
+        <x:v>520</x:v>
       </x:c>
       <x:c r="M18" s="3" t="s">
-        <x:v>533</x:v>
+        <x:v>521</x:v>
       </x:c>
       <x:c r="N18" s="3" t="s">
-        <x:v>534</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="O18" s="3" t="s">
-        <x:v>535</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="P18" s="3" t="s">
-        <x:v>536</x:v>
+        <x:v>524</x:v>
       </x:c>
       <x:c r="Q18" s="3" t="s">
-        <x:v>537</x:v>
+        <x:v>525</x:v>
       </x:c>
       <x:c r="R18" s="3" t="s">
-        <x:v>538</x:v>
+        <x:v>526</x:v>
       </x:c>
       <x:c r="S18" s="3" t="s">
-        <x:v>539</x:v>
+        <x:v>527</x:v>
       </x:c>
       <x:c r="T18" s="3" t="s">
-        <x:v>540</x:v>
+        <x:v>528</x:v>
       </x:c>
       <x:c r="U18" s="3" t="s">
         <x:v>52</x:v>
@@ -9609,19 +9573,19 @@
     </x:row>
     <x:row r="19" ht="93.25" hidden="0">
       <x:c r="A19" s="3" t="s">
-        <x:v>541</x:v>
+        <x:v>529</x:v>
       </x:c>
       <x:c r="B19" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C19" s="3" t="s">
-        <x:v>542</x:v>
+        <x:v>530</x:v>
       </x:c>
       <x:c r="D19" s="3" t="s">
-        <x:v>543</x:v>
+        <x:v>531</x:v>
       </x:c>
       <x:c r="E19" s="3" t="s">
-        <x:v>544</x:v>
+        <x:v>532</x:v>
       </x:c>
       <x:c r="F19" s="3" t="s">
         <x:v>37</x:v>
@@ -9642,31 +9606,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L19" s="3" t="s">
-        <x:v>545</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="M19" s="3" t="s">
-        <x:v>546</x:v>
+        <x:v>534</x:v>
       </x:c>
       <x:c r="N19" s="3" t="s">
-        <x:v>547</x:v>
+        <x:v>535</x:v>
       </x:c>
       <x:c r="O19" s="3" t="s">
-        <x:v>548</x:v>
+        <x:v>536</x:v>
       </x:c>
       <x:c r="P19" s="3" t="s">
-        <x:v>549</x:v>
+        <x:v>537</x:v>
       </x:c>
       <x:c r="Q19" s="3" t="s">
-        <x:v>550</x:v>
+        <x:v>538</x:v>
       </x:c>
       <x:c r="R19" s="3" t="s">
-        <x:v>551</x:v>
+        <x:v>539</x:v>
       </x:c>
       <x:c r="S19" s="3" t="s">
-        <x:v>552</x:v>
+        <x:v>540</x:v>
       </x:c>
       <x:c r="T19" s="3" t="s">
-        <x:v>553</x:v>
+        <x:v>541</x:v>
       </x:c>
       <x:c r="U19" s="3" t="s">
         <x:v>52</x:v>
@@ -9674,19 +9638,19 @@
     </x:row>
     <x:row r="20" ht="79.25" hidden="0">
       <x:c r="A20" s="3" t="s">
-        <x:v>554</x:v>
+        <x:v>542</x:v>
       </x:c>
       <x:c r="B20" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C20" s="3" t="s">
-        <x:v>555</x:v>
+        <x:v>543</x:v>
       </x:c>
       <x:c r="D20" s="3" t="s">
-        <x:v>556</x:v>
+        <x:v>544</x:v>
       </x:c>
       <x:c r="E20" s="3" t="s">
-        <x:v>557</x:v>
+        <x:v>545</x:v>
       </x:c>
       <x:c r="F20" s="3" t="s">
         <x:v>37</x:v>
@@ -9707,31 +9671,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L20" s="3" t="s">
-        <x:v>558</x:v>
+        <x:v>546</x:v>
       </x:c>
       <x:c r="M20" s="3" t="s">
-        <x:v>559</x:v>
+        <x:v>547</x:v>
       </x:c>
       <x:c r="N20" s="3" t="s">
-        <x:v>560</x:v>
+        <x:v>548</x:v>
       </x:c>
       <x:c r="O20" s="3" t="s">
-        <x:v>561</x:v>
+        <x:v>549</x:v>
       </x:c>
       <x:c r="P20" s="3" t="s">
-        <x:v>562</x:v>
+        <x:v>550</x:v>
       </x:c>
       <x:c r="Q20" s="3" t="s">
-        <x:v>563</x:v>
+        <x:v>551</x:v>
       </x:c>
       <x:c r="R20" s="3" t="s">
-        <x:v>564</x:v>
+        <x:v>552</x:v>
       </x:c>
       <x:c r="S20" s="3" t="s">
-        <x:v>565</x:v>
+        <x:v>553</x:v>
       </x:c>
       <x:c r="T20" s="3" t="s">
-        <x:v>566</x:v>
+        <x:v>554</x:v>
       </x:c>
       <x:c r="U20" s="3" t="s">
         <x:v>52</x:v>
@@ -9739,19 +9703,19 @@
     </x:row>
     <x:row r="21" ht="79.25" hidden="0">
       <x:c r="A21" s="3" t="s">
-        <x:v>567</x:v>
+        <x:v>555</x:v>
       </x:c>
       <x:c r="B21" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C21" s="3" t="s">
-        <x:v>568</x:v>
+        <x:v>556</x:v>
       </x:c>
       <x:c r="D21" s="3" t="s">
-        <x:v>569</x:v>
+        <x:v>557</x:v>
       </x:c>
       <x:c r="E21" s="3" t="s">
-        <x:v>570</x:v>
+        <x:v>558</x:v>
       </x:c>
       <x:c r="F21" s="3" t="s">
         <x:v>37</x:v>
@@ -9772,31 +9736,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L21" s="3" t="s">
-        <x:v>571</x:v>
+        <x:v>559</x:v>
       </x:c>
       <x:c r="M21" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="N21" s="3" t="s">
-        <x:v>573</x:v>
+        <x:v>561</x:v>
       </x:c>
       <x:c r="O21" s="3" t="s">
         <x:v>218</x:v>
       </x:c>
       <x:c r="P21" s="3" t="s">
-        <x:v>574</x:v>
+        <x:v>562</x:v>
       </x:c>
       <x:c r="Q21" s="3" t="s">
-        <x:v>575</x:v>
+        <x:v>563</x:v>
       </x:c>
       <x:c r="R21" s="3" t="s">
         <x:v>221</x:v>
       </x:c>
       <x:c r="S21" s="3" t="s">
-        <x:v>576</x:v>
+        <x:v>564</x:v>
       </x:c>
       <x:c r="T21" s="3" t="s">
-        <x:v>577</x:v>
+        <x:v>565</x:v>
       </x:c>
       <x:c r="U21" s="3" t="s">
         <x:v>52</x:v>
@@ -9804,19 +9768,19 @@
     </x:row>
     <x:row r="22" ht="93.25" hidden="0">
       <x:c r="A22" s="3" t="s">
-        <x:v>578</x:v>
+        <x:v>566</x:v>
       </x:c>
       <x:c r="B22" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="3" t="s">
-        <x:v>579</x:v>
+        <x:v>567</x:v>
       </x:c>
       <x:c r="D22" s="3" t="s">
-        <x:v>580</x:v>
+        <x:v>568</x:v>
       </x:c>
       <x:c r="E22" s="3" t="s">
-        <x:v>581</x:v>
+        <x:v>569</x:v>
       </x:c>
       <x:c r="F22" s="3" t="s">
         <x:v>37</x:v>
@@ -9837,31 +9801,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L22" s="3" t="s">
-        <x:v>582</x:v>
+        <x:v>570</x:v>
       </x:c>
       <x:c r="M22" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="N22" s="3" t="s">
-        <x:v>584</x:v>
+        <x:v>572</x:v>
       </x:c>
       <x:c r="O22" s="3" t="s">
-        <x:v>585</x:v>
+        <x:v>573</x:v>
       </x:c>
       <x:c r="P22" s="3" t="s">
-        <x:v>586</x:v>
+        <x:v>574</x:v>
       </x:c>
       <x:c r="Q22" s="3" t="s">
-        <x:v>587</x:v>
+        <x:v>575</x:v>
       </x:c>
       <x:c r="R22" s="3" t="s">
-        <x:v>588</x:v>
+        <x:v>576</x:v>
       </x:c>
       <x:c r="S22" s="3" t="s">
-        <x:v>589</x:v>
+        <x:v>577</x:v>
       </x:c>
       <x:c r="T22" s="3" t="s">
-        <x:v>590</x:v>
+        <x:v>578</x:v>
       </x:c>
       <x:c r="U22" s="3" t="s">
         <x:v>52</x:v>
@@ -9869,19 +9833,19 @@
     </x:row>
     <x:row r="23" ht="93.25" hidden="0">
       <x:c r="A23" s="3" t="s">
-        <x:v>591</x:v>
+        <x:v>579</x:v>
       </x:c>
       <x:c r="B23" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C23" s="3" t="s">
-        <x:v>592</x:v>
+        <x:v>580</x:v>
       </x:c>
       <x:c r="D23" s="3" t="s">
-        <x:v>593</x:v>
+        <x:v>581</x:v>
       </x:c>
       <x:c r="E23" s="3" t="s">
-        <x:v>594</x:v>
+        <x:v>582</x:v>
       </x:c>
       <x:c r="F23" s="3" t="s">
         <x:v>37</x:v>
@@ -9902,31 +9866,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L23" s="3" t="s">
-        <x:v>595</x:v>
+        <x:v>583</x:v>
       </x:c>
       <x:c r="M23" s="3" t="s">
-        <x:v>596</x:v>
+        <x:v>584</x:v>
       </x:c>
       <x:c r="N23" s="3" t="s">
-        <x:v>597</x:v>
+        <x:v>585</x:v>
       </x:c>
       <x:c r="O23" s="3" t="s">
-        <x:v>598</x:v>
+        <x:v>586</x:v>
       </x:c>
       <x:c r="P23" s="3" t="s">
-        <x:v>599</x:v>
+        <x:v>587</x:v>
       </x:c>
       <x:c r="Q23" s="3" t="s">
-        <x:v>600</x:v>
+        <x:v>588</x:v>
       </x:c>
       <x:c r="R23" s="3" t="s">
-        <x:v>601</x:v>
+        <x:v>589</x:v>
       </x:c>
       <x:c r="S23" s="3" t="s">
-        <x:v>602</x:v>
+        <x:v>590</x:v>
       </x:c>
       <x:c r="T23" s="3" t="s">
-        <x:v>603</x:v>
+        <x:v>591</x:v>
       </x:c>
       <x:c r="U23" s="3" t="s">
         <x:v>52</x:v>
@@ -9934,19 +9898,19 @@
     </x:row>
     <x:row r="24" ht="79.25" hidden="0">
       <x:c r="A24" s="3" t="s">
-        <x:v>604</x:v>
+        <x:v>592</x:v>
       </x:c>
       <x:c r="B24" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C24" s="3" t="s">
-        <x:v>605</x:v>
+        <x:v>593</x:v>
       </x:c>
       <x:c r="D24" s="3" t="s">
-        <x:v>606</x:v>
+        <x:v>594</x:v>
       </x:c>
       <x:c r="E24" s="3" t="s">
-        <x:v>607</x:v>
+        <x:v>595</x:v>
       </x:c>
       <x:c r="F24" s="3" t="s">
         <x:v>37</x:v>
@@ -9967,31 +9931,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L24" s="3" t="s">
-        <x:v>608</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="M24" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="N24" s="3" t="s">
-        <x:v>609</x:v>
+        <x:v>597</x:v>
       </x:c>
       <x:c r="O24" s="3" t="s">
-        <x:v>610</x:v>
+        <x:v>598</x:v>
       </x:c>
       <x:c r="P24" s="3" t="s">
-        <x:v>611</x:v>
+        <x:v>599</x:v>
       </x:c>
       <x:c r="Q24" s="3" t="s">
-        <x:v>612</x:v>
+        <x:v>600</x:v>
       </x:c>
       <x:c r="R24" s="3" t="s">
-        <x:v>613</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="S24" s="3" t="s">
-        <x:v>614</x:v>
+        <x:v>602</x:v>
       </x:c>
       <x:c r="T24" s="3" t="s">
-        <x:v>615</x:v>
+        <x:v>603</x:v>
       </x:c>
       <x:c r="U24" s="3" t="s">
         <x:v>52</x:v>
@@ -9999,19 +9963,19 @@
     </x:row>
     <x:row r="25" ht="79.25" hidden="0">
       <x:c r="A25" s="3" t="s">
-        <x:v>616</x:v>
+        <x:v>604</x:v>
       </x:c>
       <x:c r="B25" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C25" s="3" t="s">
-        <x:v>617</x:v>
+        <x:v>605</x:v>
       </x:c>
       <x:c r="D25" s="3" t="s">
-        <x:v>618</x:v>
+        <x:v>606</x:v>
       </x:c>
       <x:c r="E25" s="3" t="s">
-        <x:v>619</x:v>
+        <x:v>607</x:v>
       </x:c>
       <x:c r="F25" s="3" t="s">
         <x:v>37</x:v>
@@ -10032,31 +9996,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L25" s="3" t="s">
-        <x:v>620</x:v>
+        <x:v>608</x:v>
       </x:c>
       <x:c r="M25" s="3" t="s">
-        <x:v>572</x:v>
+        <x:v>560</x:v>
       </x:c>
       <x:c r="N25" s="3" t="s">
-        <x:v>621</x:v>
+        <x:v>609</x:v>
       </x:c>
       <x:c r="O25" s="3" t="s">
-        <x:v>622</x:v>
+        <x:v>610</x:v>
       </x:c>
       <x:c r="P25" s="3" t="s">
-        <x:v>623</x:v>
+        <x:v>611</x:v>
       </x:c>
       <x:c r="Q25" s="3" t="s">
-        <x:v>624</x:v>
+        <x:v>612</x:v>
       </x:c>
       <x:c r="R25" s="3" t="s">
-        <x:v>625</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="S25" s="3" t="s">
-        <x:v>626</x:v>
+        <x:v>614</x:v>
       </x:c>
       <x:c r="T25" s="3" t="s">
-        <x:v>627</x:v>
+        <x:v>615</x:v>
       </x:c>
       <x:c r="U25" s="3" t="s">
         <x:v>52</x:v>
@@ -10064,19 +10028,19 @@
     </x:row>
     <x:row r="26" ht="79.25" hidden="0">
       <x:c r="A26" s="3" t="s">
-        <x:v>628</x:v>
+        <x:v>616</x:v>
       </x:c>
       <x:c r="B26" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C26" s="3" t="s">
-        <x:v>629</x:v>
+        <x:v>617</x:v>
       </x:c>
       <x:c r="D26" s="3" t="s">
-        <x:v>630</x:v>
+        <x:v>618</x:v>
       </x:c>
       <x:c r="E26" s="3" t="s">
-        <x:v>631</x:v>
+        <x:v>619</x:v>
       </x:c>
       <x:c r="F26" s="3" t="s">
         <x:v>37</x:v>
@@ -10097,31 +10061,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L26" s="3" t="s">
-        <x:v>632</x:v>
+        <x:v>620</x:v>
       </x:c>
       <x:c r="M26" s="3" t="s">
-        <x:v>633</x:v>
+        <x:v>621</x:v>
       </x:c>
       <x:c r="N26" s="3" t="s">
-        <x:v>634</x:v>
+        <x:v>622</x:v>
       </x:c>
       <x:c r="O26" s="3" t="s">
-        <x:v>635</x:v>
+        <x:v>623</x:v>
       </x:c>
       <x:c r="P26" s="3" t="s">
-        <x:v>636</x:v>
+        <x:v>624</x:v>
       </x:c>
       <x:c r="Q26" s="3" t="s">
-        <x:v>637</x:v>
+        <x:v>625</x:v>
       </x:c>
       <x:c r="R26" s="3" t="s">
-        <x:v>638</x:v>
+        <x:v>626</x:v>
       </x:c>
       <x:c r="S26" s="3" t="s">
-        <x:v>639</x:v>
+        <x:v>627</x:v>
       </x:c>
       <x:c r="T26" s="3" t="s">
-        <x:v>640</x:v>
+        <x:v>628</x:v>
       </x:c>
       <x:c r="U26" s="3" t="s">
         <x:v>52</x:v>
@@ -10129,19 +10093,19 @@
     </x:row>
     <x:row r="27" ht="79.25" hidden="0">
       <x:c r="A27" s="3" t="s">
-        <x:v>641</x:v>
+        <x:v>629</x:v>
       </x:c>
       <x:c r="B27" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C27" s="3" t="s">
-        <x:v>642</x:v>
+        <x:v>630</x:v>
       </x:c>
       <x:c r="D27" s="3" t="s">
-        <x:v>643</x:v>
+        <x:v>631</x:v>
       </x:c>
       <x:c r="E27" s="3" t="s">
-        <x:v>644</x:v>
+        <x:v>632</x:v>
       </x:c>
       <x:c r="F27" s="3" t="s">
         <x:v>37</x:v>
@@ -10162,31 +10126,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L27" s="3" t="s">
-        <x:v>645</x:v>
+        <x:v>633</x:v>
       </x:c>
       <x:c r="M27" s="3" t="s">
-        <x:v>646</x:v>
+        <x:v>634</x:v>
       </x:c>
       <x:c r="N27" s="3" t="s">
-        <x:v>647</x:v>
+        <x:v>635</x:v>
       </x:c>
       <x:c r="O27" s="3" t="s">
-        <x:v>648</x:v>
+        <x:v>636</x:v>
       </x:c>
       <x:c r="P27" s="3" t="s">
-        <x:v>649</x:v>
+        <x:v>637</x:v>
       </x:c>
       <x:c r="Q27" s="3" t="s">
-        <x:v>650</x:v>
+        <x:v>638</x:v>
       </x:c>
       <x:c r="R27" s="3" t="s">
-        <x:v>651</x:v>
+        <x:v>639</x:v>
       </x:c>
       <x:c r="S27" s="3" t="s">
-        <x:v>652</x:v>
+        <x:v>640</x:v>
       </x:c>
       <x:c r="T27" s="3" t="s">
-        <x:v>653</x:v>
+        <x:v>641</x:v>
       </x:c>
       <x:c r="U27" s="3" t="s">
         <x:v>52</x:v>
@@ -10194,19 +10158,19 @@
     </x:row>
     <x:row r="28" ht="93.25" hidden="0">
       <x:c r="A28" s="3" t="s">
-        <x:v>654</x:v>
+        <x:v>642</x:v>
       </x:c>
       <x:c r="B28" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C28" s="3" t="s">
-        <x:v>655</x:v>
+        <x:v>643</x:v>
       </x:c>
       <x:c r="D28" s="3" t="s">
-        <x:v>656</x:v>
+        <x:v>644</x:v>
       </x:c>
       <x:c r="E28" s="3" t="s">
-        <x:v>657</x:v>
+        <x:v>645</x:v>
       </x:c>
       <x:c r="F28" s="3" t="s">
         <x:v>37</x:v>
@@ -10227,31 +10191,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L28" s="3" t="s">
-        <x:v>658</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="M28" s="3" t="s">
-        <x:v>659</x:v>
+        <x:v>647</x:v>
       </x:c>
       <x:c r="N28" s="3" t="s">
-        <x:v>660</x:v>
+        <x:v>648</x:v>
       </x:c>
       <x:c r="O28" s="3" t="s">
-        <x:v>661</x:v>
+        <x:v>649</x:v>
       </x:c>
       <x:c r="P28" s="3" t="s">
-        <x:v>662</x:v>
+        <x:v>650</x:v>
       </x:c>
       <x:c r="Q28" s="3" t="s">
-        <x:v>663</x:v>
+        <x:v>651</x:v>
       </x:c>
       <x:c r="R28" s="3" t="s">
-        <x:v>664</x:v>
+        <x:v>652</x:v>
       </x:c>
       <x:c r="S28" s="3" t="s">
         <x:v>286</x:v>
       </x:c>
       <x:c r="T28" s="3" t="s">
-        <x:v>665</x:v>
+        <x:v>653</x:v>
       </x:c>
       <x:c r="U28" s="3" t="s">
         <x:v>52</x:v>
@@ -10259,19 +10223,19 @@
     </x:row>
     <x:row r="29" ht="93.25" hidden="0">
       <x:c r="A29" s="3" t="s">
-        <x:v>666</x:v>
+        <x:v>654</x:v>
       </x:c>
       <x:c r="B29" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C29" s="3" t="s">
-        <x:v>667</x:v>
+        <x:v>655</x:v>
       </x:c>
       <x:c r="D29" s="3" t="s">
-        <x:v>668</x:v>
+        <x:v>656</x:v>
       </x:c>
       <x:c r="E29" s="3" t="s">
-        <x:v>669</x:v>
+        <x:v>657</x:v>
       </x:c>
       <x:c r="F29" s="3" t="s">
         <x:v>37</x:v>
@@ -10292,31 +10256,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L29" s="3" t="s">
-        <x:v>670</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="M29" s="3" t="s">
-        <x:v>671</x:v>
+        <x:v>659</x:v>
       </x:c>
       <x:c r="N29" s="3" t="s">
-        <x:v>672</x:v>
+        <x:v>660</x:v>
       </x:c>
       <x:c r="O29" s="3" t="s">
-        <x:v>673</x:v>
+        <x:v>661</x:v>
       </x:c>
       <x:c r="P29" s="3" t="s">
-        <x:v>674</x:v>
+        <x:v>662</x:v>
       </x:c>
       <x:c r="Q29" s="3" t="s">
-        <x:v>675</x:v>
+        <x:v>663</x:v>
       </x:c>
       <x:c r="R29" s="3" t="s">
-        <x:v>676</x:v>
+        <x:v>664</x:v>
       </x:c>
       <x:c r="S29" s="3" t="s">
-        <x:v>677</x:v>
+        <x:v>665</x:v>
       </x:c>
       <x:c r="T29" s="3" t="s">
-        <x:v>678</x:v>
+        <x:v>666</x:v>
       </x:c>
       <x:c r="U29" s="3" t="s">
         <x:v>52</x:v>
@@ -10324,19 +10288,19 @@
     </x:row>
     <x:row r="30" ht="93.25" hidden="0">
       <x:c r="A30" s="3" t="s">
-        <x:v>679</x:v>
+        <x:v>667</x:v>
       </x:c>
       <x:c r="B30" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C30" s="3" t="s">
-        <x:v>680</x:v>
+        <x:v>668</x:v>
       </x:c>
       <x:c r="D30" s="3" t="s">
-        <x:v>681</x:v>
+        <x:v>669</x:v>
       </x:c>
       <x:c r="E30" s="3" t="s">
-        <x:v>682</x:v>
+        <x:v>670</x:v>
       </x:c>
       <x:c r="F30" s="3" t="s">
         <x:v>37</x:v>
@@ -10357,31 +10321,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L30" s="3" t="s">
-        <x:v>683</x:v>
+        <x:v>671</x:v>
       </x:c>
       <x:c r="M30" s="3" t="s">
-        <x:v>684</x:v>
+        <x:v>672</x:v>
       </x:c>
       <x:c r="N30" s="3" t="s">
-        <x:v>685</x:v>
+        <x:v>673</x:v>
       </x:c>
       <x:c r="O30" s="3" t="s">
-        <x:v>686</x:v>
+        <x:v>674</x:v>
       </x:c>
       <x:c r="P30" s="3" t="s">
-        <x:v>687</x:v>
+        <x:v>675</x:v>
       </x:c>
       <x:c r="Q30" s="3" t="s">
-        <x:v>688</x:v>
+        <x:v>676</x:v>
       </x:c>
       <x:c r="R30" s="3" t="s">
-        <x:v>689</x:v>
+        <x:v>677</x:v>
       </x:c>
       <x:c r="S30" s="3" t="s">
-        <x:v>690</x:v>
+        <x:v>678</x:v>
       </x:c>
       <x:c r="T30" s="3" t="s">
-        <x:v>691</x:v>
+        <x:v>679</x:v>
       </x:c>
       <x:c r="U30" s="3" t="s">
         <x:v>52</x:v>
@@ -10389,19 +10353,19 @@
     </x:row>
     <x:row r="31" ht="93.25" hidden="0">
       <x:c r="A31" s="3" t="s">
-        <x:v>692</x:v>
+        <x:v>680</x:v>
       </x:c>
       <x:c r="B31" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C31" s="3" t="s">
-        <x:v>693</x:v>
+        <x:v>681</x:v>
       </x:c>
       <x:c r="D31" s="3" t="s">
-        <x:v>694</x:v>
+        <x:v>682</x:v>
       </x:c>
       <x:c r="E31" s="3" t="s">
-        <x:v>695</x:v>
+        <x:v>683</x:v>
       </x:c>
       <x:c r="F31" s="3" t="s">
         <x:v>37</x:v>
@@ -10422,31 +10386,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L31" s="3" t="s">
-        <x:v>696</x:v>
+        <x:v>684</x:v>
       </x:c>
       <x:c r="M31" s="3" t="s">
-        <x:v>697</x:v>
+        <x:v>685</x:v>
       </x:c>
       <x:c r="N31" s="3" t="s">
-        <x:v>698</x:v>
+        <x:v>686</x:v>
       </x:c>
       <x:c r="O31" s="3" t="s">
-        <x:v>699</x:v>
+        <x:v>687</x:v>
       </x:c>
       <x:c r="P31" s="3" t="s">
-        <x:v>700</x:v>
+        <x:v>688</x:v>
       </x:c>
       <x:c r="Q31" s="3" t="s">
-        <x:v>701</x:v>
+        <x:v>689</x:v>
       </x:c>
       <x:c r="R31" s="3" t="s">
-        <x:v>702</x:v>
+        <x:v>690</x:v>
       </x:c>
       <x:c r="S31" s="3" t="s">
-        <x:v>703</x:v>
+        <x:v>691</x:v>
       </x:c>
       <x:c r="T31" s="3" t="s">
-        <x:v>704</x:v>
+        <x:v>692</x:v>
       </x:c>
       <x:c r="U31" s="3" t="s">
         <x:v>52</x:v>
@@ -10454,19 +10418,19 @@
     </x:row>
     <x:row r="32" ht="93.25" hidden="0">
       <x:c r="A32" s="3" t="s">
-        <x:v>705</x:v>
+        <x:v>693</x:v>
       </x:c>
       <x:c r="B32" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C32" s="3" t="s">
-        <x:v>706</x:v>
+        <x:v>694</x:v>
       </x:c>
       <x:c r="D32" s="3" t="s">
-        <x:v>707</x:v>
+        <x:v>695</x:v>
       </x:c>
       <x:c r="E32" s="3" t="s">
-        <x:v>708</x:v>
+        <x:v>696</x:v>
       </x:c>
       <x:c r="F32" s="3" t="s">
         <x:v>37</x:v>
@@ -10487,31 +10451,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L32" s="3" t="s">
-        <x:v>709</x:v>
+        <x:v>697</x:v>
       </x:c>
       <x:c r="M32" s="3" t="s">
-        <x:v>710</x:v>
+        <x:v>698</x:v>
       </x:c>
       <x:c r="N32" s="3" t="s">
-        <x:v>711</x:v>
+        <x:v>699</x:v>
       </x:c>
       <x:c r="O32" s="3" t="s">
-        <x:v>712</x:v>
+        <x:v>700</x:v>
       </x:c>
       <x:c r="P32" s="3" t="s">
-        <x:v>713</x:v>
+        <x:v>701</x:v>
       </x:c>
       <x:c r="Q32" s="3" t="s">
-        <x:v>714</x:v>
+        <x:v>702</x:v>
       </x:c>
       <x:c r="R32" s="3" t="s">
-        <x:v>715</x:v>
+        <x:v>703</x:v>
       </x:c>
       <x:c r="S32" s="3" t="s">
-        <x:v>716</x:v>
+        <x:v>704</x:v>
       </x:c>
       <x:c r="T32" s="3" t="s">
-        <x:v>717</x:v>
+        <x:v>705</x:v>
       </x:c>
       <x:c r="U32" s="3" t="s">
         <x:v>52</x:v>
@@ -10519,19 +10483,19 @@
     </x:row>
     <x:row r="33" ht="93.25" hidden="0">
       <x:c r="A33" s="3" t="s">
-        <x:v>718</x:v>
+        <x:v>706</x:v>
       </x:c>
       <x:c r="B33" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C33" s="3" t="s">
-        <x:v>719</x:v>
+        <x:v>707</x:v>
       </x:c>
       <x:c r="D33" s="3" t="s">
-        <x:v>720</x:v>
+        <x:v>708</x:v>
       </x:c>
       <x:c r="E33" s="3" t="s">
-        <x:v>721</x:v>
+        <x:v>709</x:v>
       </x:c>
       <x:c r="F33" s="3" t="s">
         <x:v>37</x:v>
@@ -10552,31 +10516,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L33" s="3" t="s">
-        <x:v>722</x:v>
+        <x:v>710</x:v>
       </x:c>
       <x:c r="M33" s="3" t="s">
-        <x:v>723</x:v>
+        <x:v>711</x:v>
       </x:c>
       <x:c r="N33" s="3" t="s">
-        <x:v>724</x:v>
+        <x:v>712</x:v>
       </x:c>
       <x:c r="O33" s="3" t="s">
-        <x:v>725</x:v>
+        <x:v>713</x:v>
       </x:c>
       <x:c r="P33" s="3" t="s">
-        <x:v>726</x:v>
+        <x:v>714</x:v>
       </x:c>
       <x:c r="Q33" s="3" t="s">
-        <x:v>727</x:v>
+        <x:v>715</x:v>
       </x:c>
       <x:c r="R33" s="3" t="s">
-        <x:v>728</x:v>
+        <x:v>716</x:v>
       </x:c>
       <x:c r="S33" s="3" t="s">
-        <x:v>729</x:v>
+        <x:v>717</x:v>
       </x:c>
       <x:c r="T33" s="3" t="s">
-        <x:v>730</x:v>
+        <x:v>718</x:v>
       </x:c>
       <x:c r="U33" s="3" t="s">
         <x:v>52</x:v>
@@ -10584,7 +10548,7 @@
     </x:row>
     <x:row r="34" ht="93.25" hidden="0">
       <x:c r="A34" s="3" t="s">
-        <x:v>731</x:v>
+        <x:v>719</x:v>
       </x:c>
       <x:c r="B34" s="3" t="s">
         <x:v>8</x:v>
@@ -10593,10 +10557,10 @@
         <x:v>313</x:v>
       </x:c>
       <x:c r="D34" s="3" t="s">
-        <x:v>732</x:v>
+        <x:v>720</x:v>
       </x:c>
       <x:c r="E34" s="3" t="s">
-        <x:v>733</x:v>
+        <x:v>721</x:v>
       </x:c>
       <x:c r="F34" s="3" t="s">
         <x:v>37</x:v>
@@ -10617,31 +10581,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L34" s="3" t="s">
-        <x:v>734</x:v>
+        <x:v>722</x:v>
       </x:c>
       <x:c r="M34" s="3" t="s">
-        <x:v>735</x:v>
+        <x:v>723</x:v>
       </x:c>
       <x:c r="N34" s="3" t="s">
-        <x:v>736</x:v>
+        <x:v>724</x:v>
       </x:c>
       <x:c r="O34" s="3" t="s">
-        <x:v>737</x:v>
+        <x:v>725</x:v>
       </x:c>
       <x:c r="P34" s="3" t="s">
-        <x:v>738</x:v>
+        <x:v>726</x:v>
       </x:c>
       <x:c r="Q34" s="3" t="s">
-        <x:v>739</x:v>
+        <x:v>727</x:v>
       </x:c>
       <x:c r="R34" s="3" t="s">
-        <x:v>740</x:v>
+        <x:v>728</x:v>
       </x:c>
       <x:c r="S34" s="3" t="s">
         <x:v>323</x:v>
       </x:c>
       <x:c r="T34" s="3" t="s">
-        <x:v>741</x:v>
+        <x:v>729</x:v>
       </x:c>
       <x:c r="U34" s="3" t="s">
         <x:v>52</x:v>
@@ -10649,19 +10613,19 @@
     </x:row>
     <x:row r="35" ht="93.25" hidden="0">
       <x:c r="A35" s="3" t="s">
-        <x:v>742</x:v>
+        <x:v>730</x:v>
       </x:c>
       <x:c r="B35" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C35" s="3" t="s">
-        <x:v>743</x:v>
+        <x:v>731</x:v>
       </x:c>
       <x:c r="D35" s="3" t="s">
-        <x:v>744</x:v>
+        <x:v>732</x:v>
       </x:c>
       <x:c r="E35" s="3" t="s">
-        <x:v>745</x:v>
+        <x:v>733</x:v>
       </x:c>
       <x:c r="F35" s="3" t="s">
         <x:v>37</x:v>
@@ -10682,31 +10646,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L35" s="3" t="s">
-        <x:v>746</x:v>
+        <x:v>734</x:v>
       </x:c>
       <x:c r="M35" s="3" t="s">
-        <x:v>747</x:v>
+        <x:v>735</x:v>
       </x:c>
       <x:c r="N35" s="3" t="s">
-        <x:v>748</x:v>
+        <x:v>736</x:v>
       </x:c>
       <x:c r="O35" s="3" t="s">
-        <x:v>522</x:v>
+        <x:v>510</x:v>
       </x:c>
       <x:c r="P35" s="3" t="s">
-        <x:v>749</x:v>
+        <x:v>737</x:v>
       </x:c>
       <x:c r="Q35" s="3" t="s">
-        <x:v>750</x:v>
+        <x:v>738</x:v>
       </x:c>
       <x:c r="R35" s="3" t="s">
-        <x:v>751</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="S35" s="3" t="s">
-        <x:v>752</x:v>
+        <x:v>740</x:v>
       </x:c>
       <x:c r="T35" s="3" t="s">
-        <x:v>753</x:v>
+        <x:v>741</x:v>
       </x:c>
       <x:c r="U35" s="3" t="s">
         <x:v>52</x:v>
@@ -10714,19 +10678,19 @@
     </x:row>
     <x:row r="36" ht="93.25" hidden="0">
       <x:c r="A36" s="3" t="s">
-        <x:v>754</x:v>
+        <x:v>742</x:v>
       </x:c>
       <x:c r="B36" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="3" t="s">
-        <x:v>755</x:v>
+        <x:v>743</x:v>
       </x:c>
       <x:c r="D36" s="3" t="s">
-        <x:v>756</x:v>
+        <x:v>744</x:v>
       </x:c>
       <x:c r="E36" s="3" t="s">
-        <x:v>757</x:v>
+        <x:v>745</x:v>
       </x:c>
       <x:c r="F36" s="3" t="s">
         <x:v>37</x:v>
@@ -10747,31 +10711,31 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="L36" s="3" t="s">
-        <x:v>758</x:v>
+        <x:v>746</x:v>
       </x:c>
       <x:c r="M36" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N36" s="3" t="s">
-        <x:v>759</x:v>
+        <x:v>747</x:v>
       </x:c>
       <x:c r="O36" s="3" t="s">
-        <x:v>760</x:v>
+        <x:v>748</x:v>
       </x:c>
       <x:c r="P36" s="3" t="s">
-        <x:v>761</x:v>
+        <x:v>749</x:v>
       </x:c>
       <x:c r="Q36" s="3" t="s">
-        <x:v>762</x:v>
+        <x:v>750</x:v>
       </x:c>
       <x:c r="R36" s="3" t="s">
-        <x:v>763</x:v>
+        <x:v>751</x:v>
       </x:c>
       <x:c r="S36" s="3" t="s">
-        <x:v>764</x:v>
+        <x:v>752</x:v>
       </x:c>
       <x:c r="T36" s="3" t="s">
-        <x:v>765</x:v>
+        <x:v>753</x:v>
       </x:c>
       <x:c r="U36" s="3" t="s">
         <x:v>52</x:v>
@@ -10779,19 +10743,19 @@
     </x:row>
     <x:row r="37" ht="93.25" hidden="0">
       <x:c r="A37" s="3" t="s">
-        <x:v>766</x:v>
+        <x:v>754</x:v>
       </x:c>
       <x:c r="B37" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C37" s="3" t="s">
-        <x:v>767</x:v>
+        <x:v>755</x:v>
       </x:c>
       <x:c r="D37" s="3" t="s">
-        <x:v>768</x:v>
+        <x:v>756</x:v>
       </x:c>
       <x:c r="E37" s="3" t="s">
-        <x:v>769</x:v>
+        <x:v>757</x:v>
       </x:c>
       <x:c r="F37" s="3" t="s">
         <x:v>37</x:v>
@@ -10812,31 +10776,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L37" s="3" t="s">
-        <x:v>770</x:v>
+        <x:v>758</x:v>
       </x:c>
       <x:c r="M37" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="N37" s="3" t="s">
-        <x:v>772</x:v>
+        <x:v>760</x:v>
       </x:c>
       <x:c r="O37" s="3" t="s">
-        <x:v>773</x:v>
+        <x:v>761</x:v>
       </x:c>
       <x:c r="P37" s="3" t="s">
-        <x:v>774</x:v>
+        <x:v>762</x:v>
       </x:c>
       <x:c r="Q37" s="3" t="s">
-        <x:v>775</x:v>
+        <x:v>763</x:v>
       </x:c>
       <x:c r="R37" s="3" t="s">
-        <x:v>776</x:v>
+        <x:v>764</x:v>
       </x:c>
       <x:c r="S37" s="3" t="s">
-        <x:v>777</x:v>
+        <x:v>765</x:v>
       </x:c>
       <x:c r="T37" s="3" t="s">
-        <x:v>771</x:v>
+        <x:v>759</x:v>
       </x:c>
       <x:c r="U37" s="3" t="s">
         <x:v>52</x:v>
@@ -10844,19 +10808,19 @@
     </x:row>
     <x:row r="38" ht="93.25" hidden="0">
       <x:c r="A38" s="3" t="s">
-        <x:v>778</x:v>
+        <x:v>766</x:v>
       </x:c>
       <x:c r="B38" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C38" s="3" t="s">
-        <x:v>779</x:v>
+        <x:v>767</x:v>
       </x:c>
       <x:c r="D38" s="3" t="s">
-        <x:v>780</x:v>
+        <x:v>768</x:v>
       </x:c>
       <x:c r="E38" s="3" t="s">
-        <x:v>781</x:v>
+        <x:v>769</x:v>
       </x:c>
       <x:c r="F38" s="3" t="s">
         <x:v>37</x:v>
@@ -10877,31 +10841,31 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="L38" s="3" t="s">
-        <x:v>782</x:v>
+        <x:v>770</x:v>
       </x:c>
       <x:c r="M38" s="3" t="s">
-        <x:v>583</x:v>
+        <x:v>571</x:v>
       </x:c>
       <x:c r="N38" s="3" t="s">
-        <x:v>783</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="O38" s="3" t="s">
-        <x:v>784</x:v>
+        <x:v>772</x:v>
       </x:c>
       <x:c r="P38" s="3" t="s">
-        <x:v>785</x:v>
+        <x:v>773</x:v>
       </x:c>
       <x:c r="Q38" s="3" t="s">
-        <x:v>786</x:v>
+        <x:v>774</x:v>
       </x:c>
       <x:c r="R38" s="3" t="s">
-        <x:v>787</x:v>
+        <x:v>775</x:v>
       </x:c>
       <x:c r="S38" s="3" t="s">
-        <x:v>788</x:v>
+        <x:v>776</x:v>
       </x:c>
       <x:c r="T38" s="3" t="s">
-        <x:v>789</x:v>
+        <x:v>777</x:v>
       </x:c>
       <x:c r="U38" s="3" t="s">
         <x:v>52</x:v>
@@ -10909,19 +10873,19 @@
     </x:row>
     <x:row r="39" ht="93.25" hidden="0">
       <x:c r="A39" s="3" t="s">
-        <x:v>790</x:v>
+        <x:v>778</x:v>
       </x:c>
       <x:c r="B39" s="3" t="s">
         <x:v>8</x:v>
       </x:c>
       <x:c r="C39" s="3" t="s">
-        <x:v>791</x:v>
+        <x:v>779</x:v>
       </x:c>
       <x:c r="D39" s="3" t="s">
-        <x:v>792</x:v>
+        <x:v>780</x:v>
       </x:c>
       <x:c r="E39" s="3" t="s">
-        <x:v>793</x:v>
+        <x:v>781</x:v>
       </x:c>
       <x:c r="F39" s="3" t="s">
         <x:v>37</x:v>
@@ -10942,31 +10906,31 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="L39" s="3" t="s">
-        <x:v>794</x:v>
+        <x:v>782</x:v>
       </x:c>
       <x:c r="M39" s="3" t="s">
         <x:v>446</x:v>
       </x:c>
       <x:c r="N39" s="3" t="s">
-        <x:v>795</x:v>
+        <x:v>783</x:v>
       </x:c>
       <x:c r="O39" s="3" t="s">
-        <x:v>796</x:v>
+        <x:v>784</x:v>
       </x:c>
       <x:c r="P39" s="3" t="s">
-        <x:v>797</x:v>
+        <x:v>785</x:v>
       </x:c>
       <x:c r="Q39" s="3" t="s">
-        <x:v>798</x:v>
+        <x:v>786</x:v>
       </x:c>
       <x:c r="R39" s="3" t="s">
-        <x:v>799</x:v>
+        <x:v>787</x:v>
       </x:c>
       <x:c r="S39" s="3" t="s">
-        <x:v>800</x:v>
+        <x:v>788</x:v>
       </x:c>
       <x:c r="T39" s="3" t="s">
-        <x:v>801</x:v>
+        <x:v>789</x:v>
       </x:c>
       <x:c r="U39" s="3" t="s">
         <x:v>52</x:v>
@@ -10975,7 +10939,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf3665c4158cc4e66"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4d86a2a394f341b3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-015 feedback retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3f2a93bb0f704916"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R05c25e21206b4dfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Ra6b23a2c131e47f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R2ba32506083540da"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf7b2e44ef5514cf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R1d2df020d1f64acb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R532363df82634b29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R0ef2c3c78f0040ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3919,7 +3919,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4ef8c8477924da3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a59603307d444c8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9519,7 +9519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recb4e4dcf1d8456e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R045242ff3d294c9f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10541,55 +10541,55 @@
         <x:v>As a customer, I can give feedback on generated previews/artifacts.</x:v>
       </x:c>
       <x:c r="E16" s="8" t="str">
-        <x:v>Inline viewer feedback posts sentiment/text feedback and reflects memory observation status.</x:v>
+        <x:v>Customers can give thumbs-up or thumbs-down feedback on generated 3D preview artifacts from the inline viewer. Choosing a thumb reveals an optional comment box, sentiment-only feedback is accepted, comments are trimmed and sanitized before reuse, the BFF records artifact metadata and status, successful customer-memory observation is reflected in the response and UI status, and feedback is included in later agent context even when durable memory observation is unavailable.</x:v>
       </x:c>
       <x:c r="F16" s="8" t="str">
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G16" s="8" t="str">
-        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
+        <x:v>Focused current-code artifact feedback tests passed 2026-06-24.</x:v>
       </x:c>
       <x:c r="H16" s="8" t="str">
-        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
+        <x:v>No behavior error observed in focused QuoteEngine artifact feedback retest; live browser feedback interaction still not executed in this slice.</x:v>
       </x:c>
       <x:c r="I16" s="8" t="str">
-        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
+        <x:v>No app fix applied for QE-015; current code path is covered by focused BFF/source tests.</x:v>
       </x:c>
       <x:c r="J16" s="8" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Passed 12 focused tests: feedback records artifact metadata and customer memory, feedback still records when memory observation fails, whitespace comments become sentiment-only feedback, observed memory appears in the next agent turn, prompt override text is sanitized from memory and next-turn context, session feedback is reused when memory observation fails, sentiment-only feedback is reused, memory-aware UI status text is present, sentiment-only submit gate is present, thumb buttons expose pressed state and isolate clicks, feedback text is hidden until sentiment is selected, and thumb buttons are borderless.</x:v>
       </x:c>
       <x:c r="K16" s="8" t="str">
         <x:v>P1</x:v>
       </x:c>
       <x:c r="L16" s="8" t="str">
-        <x:v>Inline feedback UI -&gt; AgentController artifact-feedback -&gt; QuoteAgentService</x:v>
+        <x:v>QuoteAgentLaunchShell inline viewer feedback UI -&gt; POST quote/v1/agent/sessions/{sessionId}/artifacts/{artifactId}/feedback -&gt; AgentController model validation/problem details -&gt; QuoteAgentService RecordPreviewFeedbackAsync -&gt; QuoteAgentPreviewFeedbackRequest/Response DTOs -&gt; QuoteAgentArtifactDto metadata/status -&gt; CustomerService ObserveCustomerMemoryAsync -&gt; next-turn QuoteAgentService context injection</x:v>
       </x:c>
       <x:c r="M16" s="8" t="str">
-        <x:v>QuoteAgentLaunchShell.razor</x:v>
+        <x:v>QuoteAgentLaunchShell.razor; AgentController; QuoteAgentService; QuoteAgentDtos; CustomerService client</x:v>
       </x:c>
       <x:c r="N16" s="8" t="str">
-        <x:v>Thumb feedback and optional text</x:v>
+        <x:v>QuoteAgentLaunchShell renders qe-inline-viewer-feedback with thumb up/down buttons, aria-pressed state, click isolation, hidden comment form until a sentiment is selected, optional 1200-character comment textarea, and a Send action that posts to /quote/v1/agent/sessions/{sessionId}/artifacts/{artifactId}/feedback and updates feedback status from MemoryObserved.</x:v>
       </x:c>
       <x:c r="O16" s="8" t="str">
-        <x:v>AgentController POST artifacts/{artifactId}/feedback</x:v>
+        <x:v>POST quote/v1/agent/sessions/{sessionId}/artifacts/{artifactId}/feedback accepts QuoteAgentPreviewFeedbackRequest with required Sentiment up/down and optional Comment. QuoteAgentService rejects missing/non-generated viewer artifacts, stores customerSentiment, optional sanitized customerComment, feedbackObservedAt, customerApproved, and customer_approved or issue_reported status, attempts make_studio_feedback memory observation, marks feedbackMemoryObserved when successful, returns updated state, and builds generated-preview feedback context for later agent turns.</x:v>
       </x:c>
       <x:c r="P16" s="8" t="str">
-        <x:v>QuoteEngineSourceTests feedback; QuoteAgentEndpointTests feedback | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
+        <x:v>dotnet test Maliev.QuoteEngine.slnx --filter "FullyQualifiedName~QuoteAgentEndpointTests.Agent_preview_feedback_records_artifact_feedback_and_observes_customer_memory|FullyQualifiedName~QuoteAgentEndpointTests.Agent_preview_feedback_records_artifact_feedback_when_memory_observation_fails|FullyQualifiedName~QuoteAgentEndpointTests.Agent_preview_feedback_records_whitespace_comment_as_sentiment_only_feedback|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_after_preview_feedback_includes_observed_feedback_memory|FullyQualifiedName~QuoteAgentEndpointTests.Agent_preview_feedback_does_not_replay_prompt_override_text_into_memory_or_next_turn|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_after_preview_feedback_includes_session_feedback_when_memory_observation_fails|FullyQualifiedName~QuoteAgentEndpointTests.Agent_message_after_sentiment_only_preview_feedback_includes_session_sentiment|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_feedback_status_reflects_memory_observation|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_allows_sentiment_only_generated_preview_feedback|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_thumb_buttons_expose_pressed_state_and_isolate_clicks|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_hides_inline_viewer_feedback_text_until_sentiment_is_selected|FullyQualifiedName~QuoteEngineSourceTests.QuoteAgentLaunchShell_uses_borderless_inline_viewer_thumb_buttons" --verbosity minimal passed 12/12 on 2026-06-24.</x:v>
       </x:c>
       <x:c r="Q16" s="8" t="str">
-        <x:v>QuoteEngine BFF, Agent service, Customer memory</x:v>
+        <x:v>QuoteEngine Client, QuoteEngine BFF, QuoteAgentService, QuoteAgentSessionStore, CustomerService memory observation, ChatbotService next-turn context</x:v>
       </x:c>
       <x:c r="R16" s="8" t="str">
-        <x:v>Feedback records/memory observations</x:v>
+        <x:v>Generated viewer artifact feedback metadata, artifact status, feedbackObservedAt timestamp, customerApproved flag, feedbackMemoryObserved flag, customer memory observation record, next-turn generated-preview feedback context</x:v>
       </x:c>
       <x:c r="S16" s="8" t="str">
-        <x:v>Needs feedback persistence retest</x:v>
+        <x:v>Needs live browser retest for thumb selection, comment reveal, sentiment-only submit, failed-save status, successful-save status, and follow-up agent response behavior against a running QuoteEngine host.</x:v>
       </x:c>
       <x:c r="T16" s="8" t="str">
-        <x:v>AgentController.cs:240; QuoteAgentService.cs</x:v>
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:669,670,675,690,692,701,4917,4923,4955,4966,4974,4986,5000,5009; Maliev.QuoteEngine.Bff/Controllers/AgentController.cs:240; Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:670,678,692,705,715,724,729,748,774,5773,5922,6032; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs:515,518,523,530,538; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:8775,8843,8907,9047,9115,9187,9261; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:5110,5140,5158,5181,5199</x:v>
       </x:c>
       <x:c r="U16" s="8" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="17" s="6" customFormat="1" ht="93.25" customHeight="1">
@@ -12090,7 +12090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec5f0297565844e0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1640becbd8ad40fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-016 viewer retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf7b2e44ef5514cf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R1d2df020d1f64acb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R532363df82634b29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R0ef2c3c78f0040ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R82e53614d15f4a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R0e8929f6e3ec4591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R64029884b0294103"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R058668de7b1f4c27"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3919,7 +3919,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a59603307d444c8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60ce2ae7ee35414d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9519,7 +9519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R045242ff3d294c9f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61b955ab6efd4ffe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10603,58 +10603,58 @@
         <x:v>3D part viewer</x:v>
       </x:c>
       <x:c r="D17" s="8" t="str">
-        <x:v>As a customer, I can inspect uploaded/generated parts in a 3D viewer.</x:v>
+        <x:v>As a customer, I can inspect uploaded and agent-generated parts in a 3D viewer.</x:v>
       </x:c>
       <x:c r="E17" s="8" t="str">
-        <x:v>Part viewer loads GLB/viewer URLs, applies viewer settings, and pushes process/material/runtime state to JS.</x:v>
+        <x:v>Customers can inspect uploaded CAD/mesh files and generated preview artifacts in the QuoteEngine 3D viewer. The artifact drawer and part detail card render QePartViewer when viewer metadata is available, pass GLB/viewer URLs, file extension, browser file handles, storage path, process/material/finish/roughness, viewer settings, dark mode, and local geometry callbacks into the browser viewer, and fall back to safe preview states when a file is not renderable.</x:v>
       </x:c>
       <x:c r="F17" s="8" t="str">
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G17" s="8" t="str">
-        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
+        <x:v>Focused current-code 3D viewer tests passed 2026-06-24.</x:v>
       </x:c>
       <x:c r="H17" s="8" t="str">
-        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
+        <x:v>No behavior error observed in focused QuoteEngine 3D viewer retest; live browser canvas smoke still not executed in this slice.</x:v>
       </x:c>
       <x:c r="I17" s="8" t="str">
-        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
+        <x:v>No app fix applied for QE-016; current code path is covered by focused source and endpoint tests.</x:v>
       </x:c>
       <x:c r="J17" s="8" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Passed 22/22 focused tests covering BFF geometry runtime manifest/assets/telemetry, QePartViewer and QePartDetailCard local DFM wiring, artifact drawer uploaded-part viewer rendering, and inline generated preview resource/error guards.</x:v>
       </x:c>
       <x:c r="K17" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="L17" s="8" t="str">
-        <x:v>QePartViewer -&gt; geometry runtime assets/telemetry -&gt; browser viewer</x:v>
+        <x:v>QuoteAgentLaunchShell artifact drawer and QePartDetailCard -&gt; QePartViewer -&gt; quote-part-viewer.js browser viewer and local geometry callbacks -&gt; QuoteWorkspace/agent part state -&gt; GeometryRuntimeController manifest/assets/telemetry</x:v>
       </x:c>
       <x:c r="M17" s="8" t="str">
-        <x:v>QePartViewer.razor; QePartDetailCard.razor</x:v>
+        <x:v>QePartViewer.razor; QePartDetailCard.razor; QuoteAgentLaunchShell.razor; QeInlinePartViewer.razor; quote-part-viewer.js; quote-inline-viewer.js; GeometryRuntimeController</x:v>
       </x:c>
       <x:c r="N17" s="8" t="str">
-        <x:v>3D Model tab, artifact drawer viewer</x:v>
+        <x:v>Part detail model tab keeps the Babylon viewer mounted across mode changes; artifact drawer renders the selected uploaded-part 3D viewer; assistant messages can render inline generated previews; toolbar exposes camera, render mode, projection, grid, edges, bounds, section, measure, thickness, rotate, and reset controls.</x:v>
       </x:c>
       <x:c r="O17" s="8" t="str">
-        <x:v>GeometryRuntimeController manifest/assets/telemetry</x:v>
+        <x:v>QePartViewer imports quote-part-viewer.js, initializes the canvas with viewer settings and file/runtime metadata, runs browser local geometry through quoteEngineUploads, and reports started/complete/unavailable callbacks. GeometryRuntimeController exposes anonymous quote/v1/geometry/runtime/manifest, assets/{assetName}, and telemetry endpoints with packaged runtime fallback and analysis-status hydration.</x:v>
       </x:c>
       <x:c r="P17" s="8" t="str">
-        <x:v>QuoteEngineSourceTests viewer/runtime | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter focused QE-016 viewer/runtime set --verbosity minimal passed 22/22. Covered geometry runtime manifest/assets/telemetry endpoint tests, QePartViewer/detail-card source tests, artifact drawer viewer source test, and inline preview source tests.</x:v>
       </x:c>
       <x:c r="Q17" s="8" t="str">
-        <x:v>QuoteEngine client/BFF, Geometry runtime</x:v>
+        <x:v>QuoteEngine Client, QuoteEngine BFF, browser geometry/runtime assets, UploadService/analysis metadata, agent session local DFM sync</x:v>
       </x:c>
       <x:c r="R17" s="8" t="str">
-        <x:v>Viewer settings/telemetry</x:v>
+        <x:v>Viewer settings, selected part state, browser file identifiers, local geometry runtime status/result, DFM reports, overlay GLB URLs, runtime telemetry, inline preview command payloads</x:v>
       </x:c>
       <x:c r="S17" s="8" t="str">
-        <x:v>Needs visual canvas smoke</x:v>
+        <x:v>Needs live browser canvas smoke for uploaded GLB/STL/STEP, generated inline preview, toolbar interaction, dark/light mode, and local geometry callback behavior against a running QuoteEngine host.</x:v>
       </x:c>
       <x:c r="T17" s="8" t="str">
-        <x:v>QePartViewer.razor; QePartDetailCard.razor; GeometryRuntimeController.cs</x:v>
+        <x:v>QePartViewer.razor:6,21,150,207,284,370,443; QePartDetailCard.razor:92,95,228,271; QuoteAgentLaunchShell.razor:665,1631,1644,4220; QuoteEngineDtos.cs:164,304,341; GeometryRuntimeController.cs:18,39,74,214; quote-part-viewer.js:1915,3721,3734,3746; quote-inline-viewer.js:371</x:v>
       </x:c>
       <x:c r="U17" s="8" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="18" s="6" customFormat="1" ht="93.25" customHeight="1">
@@ -12090,7 +12090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1640becbd8ad40fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb034090643b54609"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-017 DFM retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R82e53614d15f4a57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R0e8929f6e3ec4591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R64029884b0294103"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R058668de7b1f4c27"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8bbed84910c04d4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R2897ba0727184eda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R92dd9e0a46454f8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R5f5227a2a26a4753"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3919,7 +3919,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R60ce2ae7ee35414d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R335da5755d054031"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9519,7 +9519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61b955ab6efd4ffe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0c54c32a7204ecf"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10671,55 +10671,55 @@
         <x:v>As a customer, I can review manufacturability checks for FDM, SLA, and CNC.</x:v>
       </x:c>
       <x:c r="E18" s="8" t="str">
-        <x:v>DFM tab renders process-specific report types and the agent can apply DFM reports to session state.</x:v>
+        <x:v>Customers can open the DFM tab for a selected part and see pending, passed, or failed manufacturability checks for mesh integrity, body count, and the selected manufacturing process. FDM reports cover thin walls, overhang/support need, and small features; SLA reports cover thin walls, resin trapping, suction, and hollow regions; CNC reports cover sharp internal corners, undercuts, drill holes, EDM, grinding, and turnability. Browser-local DFM results update the matching process report, preserve accepted local results when later status refreshes have no report, feed issue overlays into the viewer, and can be acknowledged before formal quote/order gates proceed.</x:v>
       </x:c>
       <x:c r="F18" s="8" t="str">
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G18" s="8" t="str">
-        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
+        <x:v>Focused current-code DFM reporting tests passed 2026-06-24.</x:v>
       </x:c>
       <x:c r="H18" s="8" t="str">
-        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
+        <x:v>No behavior error observed in focused QuoteEngine DFM retest; live browser DFM runtime and overlay interaction smoke still not executed in this slice.</x:v>
       </x:c>
       <x:c r="I18" s="8" t="str">
-        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
+        <x:v>No app fix applied for QE-017; current code path is covered by focused source, endpoint, status-store, and gate tests.</x:v>
       </x:c>
       <x:c r="J18" s="8" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Passed 22/22 focused tests covering DFM DTO round trips, local mapper process matching and report preservation, status-store merge behavior, DFM SignalR handling, DFM tab/source contracts, overlay status copy, local DFM session hydration, draft duplication preservation, and quote/order/agent gates for unacknowledged issues.</x:v>
       </x:c>
       <x:c r="K18" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="L18" s="8" t="str">
-        <x:v>QeDfmTab/QePartDetailCard -&gt; AgentController dfm -&gt; SessionStore</x:v>
+        <x:v>QePartDetailCard DFM tab and overlay panel -&gt; QeDfmTab/QeDfmOverlayPanel/QePartConfigSidebar -&gt; QeLocalDfmMapper -&gt; QuoteAgentLaunchShell local DFM submission -&gt; QuoteEngineApiClient -&gt; AgentController sessions/{sessionId}/dfm -&gt; QuoteAgentService and QuoteFileAnalysisStatusService -&gt; shared DFM DTOs</x:v>
       </x:c>
       <x:c r="M18" s="8" t="str">
-        <x:v>QeDfmTab.razor; QePartDetailCard.razor</x:v>
+        <x:v>QeDfmTab.razor; QePartDetailCard.razor; QeDfmOverlayPanel.razor; QePartConfigSidebar.razor; QeLocalDfmMapper.cs; QuoteAgentLaunchShell.razor; QuoteEngineApiClient.cs; AgentController.cs; QuoteAgentService.cs; QeDfmDtos.cs</x:v>
       </x:c>
       <x:c r="N18" s="8" t="str">
-        <x:v>DFM tab and issue acknowledgement</x:v>
+        <x:v>Part detail DFM tab shows pass/fail/pending badges and process tabs; DFM overlay panel shows analyzing, local analyzing, unavailable, all-clear, and issue states; issue rows toggle viewer overlays; DFM acknowledgement can be made from the overlay or part configuration sidebar.</x:v>
       </x:c>
       <x:c r="O18" s="8" t="str">
-        <x:v>AgentController POST sessions/{sessionId}/dfm; QeDfmDtos</x:v>
+        <x:v>POST quote/v1/agent/sessions/{sessionId}/dfm accepts QuoteAgentLocalDfmRequest, writes metrics and process reports to the authoritative analysis-status store, hydrates session parts back from that store, and returns QuoteAgentStateResponse so the assistant sees the same DFM issues as the customer UI.</x:v>
       </x:c>
       <x:c r="P18" s="8" t="str">
-        <x:v>QuoteEngineSourceTests DFM | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
+        <x:v>2026-06-24: dotnet test Maliev.QuoteEngine.slnx --filter focused QE-017 DFM set --verbosity minimal passed 22/22. Covered DFM DTOs, mapper, SignalR/status-store merge, source contracts, local DFM endpoint hydration, draft preservation, and quote/order/agent acknowledgement gates.</x:v>
       </x:c>
       <x:c r="Q18" s="8" t="str">
-        <x:v>QuoteEngine BFF, Geometry/DFM, SessionStore</x:v>
+        <x:v>QuoteEngine Client, QuoteEngine BFF, QuoteAgentService, QuoteFileAnalysisStatusService, browser local geometry runtime, SignalR analysis notifications, formal quote/order gates</x:v>
       </x:c>
       <x:c r="R18" s="8" t="str">
-        <x:v>DFM reports and acknowledgement state</x:v>
+        <x:v>FDM/SLA/CNC DFM reports, DFM issue items, overlay GLB URLs, local runtime status fields, non-manifold reason, body count, part acknowledgement state, session part DFM state, quote/order gate state</x:v>
       </x:c>
       <x:c r="S18" s="8" t="str">
-        <x:v>Needs process-specific fixture coverage</x:v>
+        <x:v>Needs live browser DFM runtime smoke with representative FDM, SLA, and CNC files, overlay toggle rendering, acknowledgement interaction, and formal quote/order gating against a running QuoteEngine host.</x:v>
       </x:c>
       <x:c r="T18" s="8" t="str">
-        <x:v>QeDfmTab.razor; QePartDetailCard.razor; AgentController.cs:221</x:v>
+        <x:v>QeDfmTab.razor:4,37,47,134,150,223; QeLocalDfmMapper.cs:17,73,97,106,127,193,207; QePartDetailCard.razor:39,62,153,216,271,337,349,365; QeDfmOverlayPanel.razor:1,12,23,34,70,120; QePartConfigSidebar.razor:585,963; QuoteAgentLaunchShell.razor:3428,4220,4247; QuoteEngineApiClient.cs:421; AgentController.cs:221; QuoteAgentService.cs:561,580,598,638; QeDfmDtos.cs:10,16,25,33</x:v>
       </x:c>
       <x:c r="U18" s="8" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="19" s="6" customFormat="1" ht="93.25" customHeight="1">
@@ -12090,7 +12090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb034090643b54609"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd325f058835b4392"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Document QE-018 configuration retest
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8bbed84910c04d4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R2897ba0727184eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R92dd9e0a46454f8d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R5f5227a2a26a4753"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6b379c98333b4bd1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R79b65ba8a56d4daa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Refa46d087f604d81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R5cb2dd8fcba940f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3919,7 +3919,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R335da5755d054031"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8577feca60e84528"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9519,7 +9519,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0c54c32a7204ecf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0887e75454734b9d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10733,58 +10733,58 @@
         <x:v>Part configuration sidebar</x:v>
       </x:c>
       <x:c r="D19" s="8" t="str">
-        <x:v>As a customer, I can select process, material, color, finish, tolerance, quantity, and options.</x:v>
+        <x:v>As a customer, I can configure process, material, finish, tolerance, inspection, quantity, notes, and manufacturing options for each uploaded part.</x:v>
       </x:c>
       <x:c r="E19" s="8" t="str">
-        <x:v>Configuration sidebar filters reference data and emits changes for quote estimation.</x:v>
+        <x:v>Customers can configure the selected part from the QuoteEngine chat workspace sidebar using process search/cards, material and color choices, surface finish and finish options, tolerance, CNC roughness, threaded-hole and insert details, process-specific options, inspection level, quantity stepper/presets/input, DFM acknowledgement, and production notes. Changing process or material clears dependent configuration, applies Project New-style catalog defaults from current reference data, resets stale DFM acknowledgement/runtime state when the process changes, and emits part-change callbacks so estimates, drafts, formal quotes, orders, and agent state use the same QuotePartDraftDto fields.</x:v>
       </x:c>
       <x:c r="F19" s="8" t="str">
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G19" s="8" t="str">
-        <x:v>Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:v>
+        <x:v>Focused current-code part configuration tests passed 2026-06-24.</x:v>
       </x:c>
       <x:c r="H19" s="8" t="str">
-        <x:v>No behavior error observed in current QuoteEngine automated retest.</x:v>
+        <x:v>No behavior error observed in focused QuoteEngine part configuration retest; live keyboard/browser accessibility pass was not executed in this slice.</x:v>
       </x:c>
       <x:c r="I19" s="8" t="str">
-        <x:v>No fix needed for this story from current QuoteEngine automated retest.</x:v>
+        <x:v>No app fix applied for QE-018; current code path is covered by focused source, endpoint, and DTO tests.</x:v>
       </x:c>
       <x:c r="J19" s="8" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Retested 2026-06-24 with 13 focused QuoteEngine tests covering part configuration sidebar card/source contract, process/material default clearing, DTO round-trip, reference-data exposure, and configured estimate pricing.</x:v>
       </x:c>
       <x:c r="K19" s="8" t="str">
         <x:v>P0</x:v>
       </x:c>
       <x:c r="L19" s="8" t="str">
-        <x:v>QePartConfigSidebar -&gt; reference-data/estimate DTOs</x:v>
+        <x:v>QePartConfigSidebar controls -&gt; QuotePartViewModel process/material/defaulting and ToDraft -&gt; QuoteWorkspace estimate/draft/formal quote/order requests -&gt; QuotePartDraftDto/QuoteEstimateRequest -&gt; QuoteController estimate/projects/draft/formal quote/order endpoints.</x:v>
       </x:c>
       <x:c r="M19" s="8" t="str">
-        <x:v>QePartConfigSidebar.razor</x:v>
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteEngine/QePartConfigSidebar.razor; Maliev.QuoteEngine.Client/Models/QuotePartViewModel.cs; Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor; Maliev.QuoteEngine.Shared/Quotes/QuoteEngineDtos.cs; Maliev.QuoteEngine.Bff/Controllers/QuoteController.cs.</x:v>
       </x:c>
       <x:c r="N19" s="8" t="str">
-        <x:v>Part configuration controls</x:v>
+        <x:v>QuoteWorkspace renders QePartConfigSidebar for the selected uploaded part. Sidebar sections include manufacturing process search/cards, material, material color, surface finish, finish options, tolerance, CNC roughness, part features, process options, inspection, quantity, DFM reviewed checkbox, and production notes.</x:v>
       </x:c>
       <x:c r="O19" s="8" t="str">
-        <x:v>QuoteController reference-data/estimate</x:v>
+        <x:v>GET quote/v1/reference-data supplies processes/materials/finishes/tolerances/inspection/roughness/colors/options. POST quote/v1/estimate prices configured QuotePartDraftDto fields. POST quote/v1/projects/draft persists request.Parts; formal quote and order requests reuse ToDraft parts.</x:v>
       </x:c>
       <x:c r="P19" s="8" t="str">
-        <x:v>QuoteEngineSourceTests config sidebar | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup. Initial full run failed 3/539 on QuoteEngineSourceTests stale sample-only workspace expectations.</x:v>
+        <x:v>dotnet test B:/maliev/Maliev.QuoteEngine/Maliev.QuoteEngine.slnx --filter part-configuration focused filter --verbosity minimal passed 2026-06-24: 13 passed, 0 failed.</x:v>
       </x:c>
       <x:c r="Q19" s="8" t="str">
-        <x:v>QuoteEngine client/BFF, Pricing/Material services</x:v>
+        <x:v>QuoteEngine Client, QuoteEngine BFF, reference data, project, pricing, formal quote, and order service boundaries.</x:v>
       </x:c>
       <x:c r="R19" s="8" t="str">
-        <x:v>Part configuration state</x:v>
+        <x:v>Selected part process, material, finish, tolerance, inspection, roughness, color, process option values, threaded-hole and insert fields, quantity, DFM acknowledgement, notes, and QuotePartDraftDto payload fields.</x:v>
       </x:c>
       <x:c r="S19" s="8" t="str">
-        <x:v>Needs keyboard/accessibility check</x:v>
+        <x:v>Needs live keyboard and screen-reader pass for process search, card groups, color picker, quantity stepper, DFM checkbox, and notes against a running QuoteEngine host.</x:v>
       </x:c>
       <x:c r="T19" s="8" t="str">
-        <x:v>QePartConfigSidebar.razor; QuoteController.cs:47,301</x:v>
+        <x:v>QePartConfigSidebar.razor:1-80,608-994,1026-1053; QuotePartViewModel.cs:65-179,195-238; QuoteWorkspace.razor:332-343,878-908,930-936,1028-1033; QuoteEngineDtos.cs:233-354; QuoteController.cs:301-460,502-540,1227-1255; QuoteEngineSourceTests.cs:121-159,421-498,3774-3975; QuoteEngineEndpointTests.cs:2102-2114,2630-2715.</x:v>
       </x:c>
       <x:c r="U19" s="8" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-24</x:v>
       </x:c>
     </x:row>
     <x:row r="20" s="6" customFormat="1" ht="79.25" customHeight="1">
@@ -12090,7 +12090,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd325f058835b4392"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96292127832f4c43"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add current Web feature stories to tracker
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -193,7 +193,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:U31" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:U40" headerRowCount="1">
   <tableColumns count="21">
     <tableColumn id="1" name="Story ID"/>
     <tableColumn id="2" name="App Surface"/>
@@ -510,7 +510,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>30</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6" ht="16.64999961853027" customHeight="1" s="6">
@@ -540,7 +540,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>120</v>
+        <v>129</v>
       </c>
     </row>
     <row r="9" ht="31.60000038146973" customHeight="1" s="6">
@@ -566,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8359375" defaultRowHeight="21.95000076293945"/>
   <cols>
     <col width="12.47000026702881" customWidth="1" style="5" min="1" max="1"/>
@@ -3907,6 +3907,969 @@
       <c r="U31" s="8" t="inlineStr">
         <is>
           <t>2026-06-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A32" s="8" t="inlineStr">
+        <is>
+          <t>WEB-031</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="inlineStr">
+        <is>
+          <t>Landing hero and ad-targeted copy</t>
+        </is>
+      </c>
+      <c r="D32" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor arriving from an ad or public link, I see a localized Make Studio hero that matches my intent and routes me into the live workspace.</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>The home page resolves an explicit ad target from the URL when present, otherwise uses the default hero profile, chooses and persists a localized hero-copy variant for prerender/interactive consistency, shows crawlable manufacturing metrics enhanced by count-up animation, renders an animated Make Studio conversation preview for sketch, CAD, photo, and text scenarios, and keeps primary CTAs wired to Make Studio and contact paths.</t>
+        </is>
+      </c>
+      <c r="F32" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H32" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I32" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
+          <t>Existing tests cover ad-targeted hero copy, Make Studio animation, metrics count-up, Make Studio CTAs, responsive hero composition, and reduced-motion freeze guards.</t>
+        </is>
+      </c>
+      <c r="K32" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L32" s="8" t="inlineStr">
+        <is>
+          <t>Home.razor hero state -&gt; HeroCopyCatalog ad target/variant selection -&gt; PersistentComponentState -&gt; SiteContent MakeStudioUrl/contact links -&gt; maliev-make-studio-hero.js animation and app.css responsive styles</t>
+        </is>
+      </c>
+      <c r="M32" s="8" t="inlineStr">
+        <is>
+          <t>Home.razor; HeroCopyCatalog.cs; SiteContent.cs; maliev-make-studio-hero.js; app.css; HeroLayoutSourceTests.cs; HeroCopyCatalogTests.cs</t>
+        </is>
+      </c>
+      <c r="N32" s="8" t="inlineStr">
+        <is>
+          <t>Home renders landing-hero, data-count-up metrics, data-make-studio-hero ms-hero scenes, Start in Make Studio and Talk to MALIEV links, and final Make Studio CTA; InitializeHeroCopy resolves URL targets and persists selected variants.</t>
+        </is>
+      </c>
+      <c r="O32" s="8" t="inlineStr">
+        <is>
+          <t>No BFF write boundary; public page uses static content, persisted component state, browser animation JavaScript, and QuoteEngine URL from SiteContent.</t>
+        </is>
+      </c>
+      <c r="P32" s="8" t="inlineStr">
+        <is>
+          <t>HeroLayoutSourceTests.HomeHeroShowsAnimatedMakeStudioWindow; MakeStudioHeroDoesNotStopForReducedMotion; HomeHeroMetricsUseCountUpEnhancement; HomeHeroUsesAdTargetedLocalizedCopyRotation; HomeHeroAndFinalCtaLinkToLiveMakeStudio; HeroCopyCatalogTests.*</t>
+        </is>
+      </c>
+      <c r="Q32" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, BFF static assets, QuoteEngine public workspace link</t>
+        </is>
+      </c>
+      <c r="R32" s="8" t="inlineStr">
+        <is>
+          <t>Client-side hero copy selection state, persisted component state keys for hero variant, no durable customer data mutation</t>
+        </is>
+      </c>
+      <c r="S32" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for animated scene cycling, count-up timing, ad-target query behavior, and CTA navigation across desktop/mobile.</t>
+        </is>
+      </c>
+      <c r="T32" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Pages/Home.razor:11,32,47,724; Maliev.Web.Client/Content/HeroCopyCatalog.cs:8,359,364,370; Maliev.Web.Bff/wwwroot/js/maliev-make-studio-hero.js:7; Maliev.Web.Tests/HeroLayoutSourceTests.cs:13,409,1288; Maliev.Web.Tests/HeroCopyCatalogTests.cs:1</t>
+        </is>
+      </c>
+      <c r="U32" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A33" s="8" t="inlineStr">
+        <is>
+          <t>WEB-032</t>
+        </is>
+      </c>
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Home workflow, services, and machine configurator</t>
+        </is>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor, I can explore MALIEV workflows, service fit, and a workshop-made machine package from the home page before taking action.</t>
+        </is>
+      </c>
+      <c r="E33" s="8" t="inlineStr">
+        <is>
+          <t>The home page lets visitors select workflow steps, switch manufacturing service tabs, open service details, view randomized case-study/news cards, choose a pneumatic injection machine size, toggle an optional air compressor, see updated localized stats/images/package labels, and follow the configured package link into the shop product route with variant and compressor query parameters.</t>
+        </is>
+      </c>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H33" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I33" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>Existing tests cover workflow layout, home services rotation, machine configurator selection/compressor add-on, prepared machine images, finished manufacturing sections, and responsive layout rules.</t>
+        </is>
+      </c>
+      <c r="K33" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L33" s="8" t="inlineStr">
+        <is>
+          <t>Home.razor UI state -&gt; SiteContent service/case/blog data -&gt; machine variant records -&gt; product-detail shop URL query -&gt; browser scroll helper for selected workflow target</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="inlineStr">
+        <is>
+          <t>Home.razor; SiteContent.cs; app.css; WorkflowLayoutSourceTests.cs; HeroLayoutSourceTests.cs</t>
+        </is>
+      </c>
+      <c r="N33" s="8" t="inlineStr">
+        <is>
+          <t>Home renders process-grid workflow buttons, home-services tabs/panel, case/blog cards, machine-feature section with data-selected-variant and data-compressor-included, MachineVariant radio buttons, compressor toggle, configured package summary, and Configure link.</t>
+        </is>
+      </c>
+      <c r="O33" s="8" t="inlineStr">
+        <is>
+          <t>No BFF write boundary; public page state is client-side and links into /services/{slug}, /case-studies/{slug}, /blog/{slug}, and /shop/pneumatic-injection-molding-machine query routes.</t>
+        </is>
+      </c>
+      <c r="P33" s="8" t="inlineStr">
+        <is>
+          <t>WorkflowLayoutSourceTests.WorkflowStepsUseFullWidthTrackForConsistentColumnAlignment; HeroLayoutSourceTests.HomeServicesRotateGenericHighlightAndPinExplicitServiceTargets; HomeMachineConfiguratorLimitsMachineSelectionAndCompressorAddon; HomeUsesFinishedManufacturingAndNewsSections</t>
+        </is>
+      </c>
+      <c r="Q33" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, content model, shop route</t>
+        </is>
+      </c>
+      <c r="R33" s="8" t="inlineStr">
+        <is>
+          <t>Selected workflow accent, selected home service slug, selected machine variant, compressor toggle, persisted order state for randomized home cards</t>
+        </is>
+      </c>
+      <c r="S33" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for keyboard/assistive behavior, service tab state, machine configure link query, and responsive home layout.</t>
+        </is>
+      </c>
+      <c r="T33" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Pages/Home.razor:197,224,300,310,334,354,606,633,645; Maliev.Web.Tests/WorkflowLayoutSourceTests.cs:1; Maliev.Web.Tests/HeroLayoutSourceTests.cs:718,756,1122</t>
+        </is>
+      </c>
+      <c r="U33" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A34" s="8" t="inlineStr">
+        <is>
+          <t>WEB-033</t>
+        </is>
+      </c>
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C34" s="8" t="inlineStr">
+        <is>
+          <t>Public quote dropzone format picker</t>
+        </is>
+      </c>
+      <c r="D34" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor, I can understand supported quote file formats and open Make Studio from public quote entry points.</t>
+        </is>
+      </c>
+      <c r="E34" s="8" t="inlineStr">
+        <is>
+          <t>Public quote dropzones render as keyboard-focusable upload targets with a hidden multi-file input, display supported CAD and mesh formats in an interactive popover, prevent child controls from triggering the dropzone, register JavaScript handlers for click/drag file handoff, dismiss the format popover when clicking outside, and route selected files through the configured Make Studio/QuoteEngine handoff URL.</t>
+        </is>
+      </c>
+      <c r="F34" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G34" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H34" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr">
+        <is>
+          <t>Existing source tests cover supported format list, JS registration, drag/drop file capture, interactive child guards, and public entry points.</t>
+        </is>
+      </c>
+      <c r="K34" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L34" s="8" t="inlineStr">
+        <is>
+          <t>QuoteDropzone.razor component -&gt; maliev-quote-dropzone.js browser registration -&gt; public quote links -&gt; Web quote upload/handoff endpoints -&gt; QuoteEngine workspace URL</t>
+        </is>
+      </c>
+      <c r="M34" s="8" t="inlineStr">
+        <is>
+          <t>QuoteDropzone.razor; maliev-quote-dropzone.js; Quote.razor; Home.razor; HeroLayoutSourceTests.cs; WebBffEndpointTests.cs</t>
+        </is>
+      </c>
+      <c r="N34" s="8" t="inlineStr">
+        <is>
+          <t>QuoteDropzone renders type=file, accept list, role=button surface, supported-format button/popover, JSInvokable CloseFormatsAsync, malievQuoteDropzone.register, and registerFormatDismissal; quote entry points no longer point at disabled quote actions.</t>
+        </is>
+      </c>
+      <c r="O34" s="8" t="inlineStr">
+        <is>
+          <t>When files are selected, JavaScript routes to the handoff URL; upload and token validation are handled by web/v1/quote uploads/resumable, complete, analysis-status, and uploads/handoff-token endpoints already tracked by WEB-013/WEB-012.</t>
+        </is>
+      </c>
+      <c r="P34" s="8" t="inlineStr">
+        <is>
+          <t>HeroLayoutSourceTests.QuoteDropzoneRoutesSelectedFilesToQuoteEngine; PublicQuoteEntryPointsAreLive; WebBffEndpointTests.POST_QuoteUploadInitiation_*; POST_QuoteUploadHandoffToken_*</t>
+        </is>
+      </c>
+      <c r="Q34" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, BFF quote upload endpoints, QuoteEngine handoff destination, browser JS</t>
+        </is>
+      </c>
+      <c r="R34" s="8" t="inlineStr">
+        <is>
+          <t>Browser-selected files, supported format popover state, upload session IDs and signed handoff token via existing quote upload rows</t>
+        </is>
+      </c>
+      <c r="S34" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for drag/drop, format popover dismissal, keyboard activation, and selected-file handoff into QuoteEngine.</t>
+        </is>
+      </c>
+      <c r="T34" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Components/Quote/QuoteDropzone.razor:3,5,15,27,37,57,118; Maliev.Web.Bff/wwwroot/js/maliev-quote-dropzone.js; Maliev.Web.Tests/HeroLayoutSourceTests.cs:300; Maliev.Web.Bff/Controllers/QuoteController.cs:66,170</t>
+        </is>
+      </c>
+      <c r="U34" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A35" s="8" t="inlineStr">
+        <is>
+          <t>WEB-034</t>
+        </is>
+      </c>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Product media gallery and variant purchase</t>
+        </is>
+      </c>
+      <c r="D35" s="8" t="inlineStr">
+        <is>
+          <t>As a shopper, I can inspect product media, select an available variant, and add the product to my cart.</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="inlineStr">
+        <is>
+          <t>The product detail route loads a product by handle, shows thumbnail media when multiple images exist, crossfades the selected main image, initializes the first available variant, disables unavailable variants, displays lead time/inventory/quantity, enables Add to cart only for buyable published stock with a valid price and available variant, and offers a Make Studio link for custom-part requests.</t>
+        </is>
+      </c>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H35" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I35" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>Existing tests cover media-grid layout, thumbnail strip, crossfade state fields/classes, selected image method, and catalog product detail contract.</t>
+        </is>
+      </c>
+      <c r="K35" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L35" s="8" t="inlineStr">
+        <is>
+          <t>ProductDetail.razor route handle -&gt; MalievApiClient.GetProductAsync -&gt; CatalogController products/{handle} -&gt; Commerce catalog service -&gt; CartState.AddAsync for selected variant</t>
+        </is>
+      </c>
+      <c r="M35" s="8" t="inlineStr">
+        <is>
+          <t>ProductDetail.razor; ProductGrid.razor; CartState.cs; CatalogController.cs; ProductDetailMediaSourceTests.cs; CommerceCatalogBoundaryTests.cs</t>
+        </is>
+      </c>
+      <c r="N35" s="8" t="inlineStr">
+        <is>
+          <t>ProductDetail renders media-strip thumbnail buttons, product-detail-media-main crossfade images, variant select with disabled unavailable options, lead time/inventory/quantity specs, Add to cart button, and custom-part Make Studio link.</t>
+        </is>
+      </c>
+      <c r="O35" s="8" t="inlineStr">
+        <is>
+          <t>GET web/v1/catalog/products/{handle} maps catalog detail data; cart mutation is client-side CartState for the browser session.</t>
+        </is>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>ProductDetailMediaSourceTests.*; CommerceCatalogBoundaryTests.GET_CatalogProduct_MapsCommerceServiceProductDetail; WebBffEndpointTests.GET_CatalogProducts_ReturnsCatalogProducts</t>
+        </is>
+      </c>
+      <c r="Q35" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, Web BFF catalog endpoints, CommerceService catalog, browser cart state</t>
+        </is>
+      </c>
+      <c r="R35" s="8" t="inlineStr">
+        <is>
+          <t>Displayed/fading product image state, selected variant SKU, cart item state in browser/session storage</t>
+        </is>
+      </c>
+      <c r="S35" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for thumbnail crossfade timing, variant disabled state, cart count update, and missing-product recovery.</t>
+        </is>
+      </c>
+      <c r="T35" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Pages/ProductDetail.razor:1,19,25,31,42,52,68,74,121; Maliev.Web.Tests/ProductDetailMediaSourceTests.cs:7,79,94; Maliev.Web.Bff/Controllers/CatalogController.cs:87</t>
+        </is>
+      </c>
+      <c r="U35" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A36" s="8" t="inlineStr">
+        <is>
+          <t>WEB-035</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="inlineStr">
+        <is>
+          <t>Blog discovery and article tools</t>
+        </is>
+      </c>
+      <c r="D36" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor, I can search, filter, page through, read, and export manufacturing notes.</t>
+        </is>
+      </c>
+      <c r="E36" s="8" t="inlineStr">
+        <is>
+          <t>The blog library route supports query-string search, multi-topic category chips with clear filters, result counts, paged cards, previous/next page links, article detail pages with checklist sections and sidebar takeaways, and a PDF download button that builds a localized ebook URL and file name through the Blog BFF.</t>
+        </is>
+      </c>
+      <c r="F36" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H36" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I36" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
+          <t>Existing tests cover expanded practical notes, category filtering, pagination helpers, PDF button wiring, PDF service rendering, and file naming.</t>
+        </is>
+      </c>
+      <c r="K36" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L36" s="8" t="inlineStr">
+        <is>
+          <t>StaticPage blog routes/query helpers -&gt; SiteContent blog library -&gt; BlogController ebook endpoint -&gt; BlogEbookPdfService/PdfService client</t>
+        </is>
+      </c>
+      <c r="M36" s="8" t="inlineStr">
+        <is>
+          <t>StaticPage.razor; SiteContent.cs; BlogController.cs; BlogEbookPdfService.cs; HeroLayoutSourceTests.cs; BlogEbookPdfSourceTests.cs; BlogPdfFileNameTests.cs</t>
+        </is>
+      </c>
+      <c r="N36" s="8" t="inlineStr">
+        <is>
+          <t>StaticPage renders /blog search form, category chips, status count, PagedBlogPosts, pagination nav, /blog/{Slug} detail sections, sidebar actions, and Download PDF button with loading state.</t>
+        </is>
+      </c>
+      <c r="O36" s="8" t="inlineStr">
+        <is>
+          <t>GET web/v1/blog/{slug}/ebook.pdf validates slug/culture and streams a PDF generated through PdfService using localized blog content and images.</t>
+        </is>
+      </c>
+      <c r="P36" s="8" t="inlineStr">
+        <is>
+          <t>HeroLayoutSourceTests.BlogPostsIncludeExpandedPracticalNotesAndEbookDownload; BlogEbookPdfSourceTests.*; BlogPdfFileNameTests.BuildBlogPdfFileName_FdmPrintOrientation_UsesOrganizedName; WebBffEndpointTests.GET_BlogEbookPdf_*</t>
+        </is>
+      </c>
+      <c r="Q36" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, Web BFF BlogController, PdfService, static content model</t>
+        </is>
+      </c>
+      <c r="R36" s="8" t="inlineStr">
+        <is>
+          <t>Blog search/category/page query parameters, PDF download request, no durable customer data mutation</t>
+        </is>
+      </c>
+      <c r="S36" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for search/filter combinations, pagination boundaries, detail-page PDF download, and print/download behavior.</t>
+        </is>
+      </c>
+      <c r="T36" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Pages/StaticPage.razor:77,87,117,133,148,260,619,668,1089,1100,1144,1150; Maliev.Web.Bff/Controllers/BlogController.cs:26,43; Maliev.Web.Tests/HeroLayoutSourceTests.cs:1020</t>
+        </is>
+      </c>
+      <c r="U36" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A37" s="8" t="inlineStr">
+        <is>
+          <t>WEB-036</t>
+        </is>
+      </c>
+      <c r="B37" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Contact channels, map, autofill, and attachments</t>
+        </is>
+      </c>
+      <c r="D37" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor or signed-in customer, I can choose the right MALIEV contact channel, submit a contact request, and attach support files.</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>The contact page shows sales/support contact sections, phone/LINE/social actions, business hours, map preview and larger map dialog, signs in customers into a profile card when session data is available, lets them switch to manual contact details, validates name/email/subject/message, accepts up to five support attachments of ten megabytes each with progress/status stages, submits a Website contact message to the BFF, and shows sanitized success/error states.</t>
+        </is>
+      </c>
+      <c r="F37" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G37" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H37" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I37" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>Existing tests cover contact channels/map/hours, account session autofill contract, contact message BFF contract, attachment UI source, and sanitized status handling.</t>
+        </is>
+      </c>
+      <c r="K37" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L37" s="8" t="inlineStr">
+        <is>
+          <t>StaticPage contact route -&gt; MalievApiClient account session/profile and SubmitContactMessageAsync -&gt; AccountController session -&gt; ContactController messages -&gt; ContactService contract</t>
+        </is>
+      </c>
+      <c r="M37" s="8" t="inlineStr">
+        <is>
+          <t>StaticPage.razor; AccountController.cs; ContactController.cs; ContactMessageService.cs; ContactDtos.cs; ContactPageAutoFillTests.cs; ContactMessageBoundaryTests.cs; HeroLayoutSourceTests.cs</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
+        <is>
+          <t>StaticPage renders contact-business-panel, contact-map-preview/dialog, contact identity card/manual details toggle, EditForm contact-form, InputFile attachment panel/list/progress, contact status area, and submit button state.</t>
+        </is>
+      </c>
+      <c r="O37" s="8" t="inlineStr">
+        <is>
+          <t>GET web/v1/account/session supplies display name/email/profile image for autofill; POST web/v1/contact/messages maps Website contact requests and attachments to ContactService with sanitized problem handling.</t>
+        </is>
+      </c>
+      <c r="P37" s="8" t="inlineStr">
+        <is>
+          <t>HeroLayoutSourceTests.ContactPageShowsBusinessChannelsMapAndHours; StaticPagesCoverCustomerRoutesAndContactBoundary; ContactPageAutoFillTests.*; ContactMessageBoundaryTests.*; WebBffEndpointTests.POST_ContactMessage_*</t>
+        </is>
+      </c>
+      <c r="Q37" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, Web BFF account/contact endpoints, Customer/Auth session, ContactService</t>
+        </is>
+      </c>
+      <c r="R37" s="8" t="inlineStr">
+        <is>
+          <t>Contact form fields, optional profile/autofill state, selected file attachments, contact message record in ContactService</t>
+        </is>
+      </c>
+      <c r="S37" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for map dialog, hover/focus phone reveal, signed-in profile autofill, attachment progress, and backend error state.</t>
+        </is>
+      </c>
+      <c r="T37" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Pages/StaticPage.razor:277,281,295,373,389,396,402,433,469,484,505,517,1280,1431; Maliev.Web.Bff/Controllers/AccountController.cs:24; Maliev.Web.Bff/Controllers/ContactController.cs:21; Maliev.Web.Tests/HeroLayoutSourceTests.cs:1477,2368; Maliev.Web.Tests/ContactPageAutoFillTests.cs:19</t>
+        </is>
+      </c>
+      <c r="U37" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>WEB-037</t>
+        </is>
+      </c>
+      <c r="B38" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Language and theme preferences</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor or customer, I can switch language and theme without losing the current public-site experience.</t>
+        </is>
+      </c>
+      <c r="E38" s="8" t="inlineStr">
+        <is>
+          <t>The main layout renders stable EN/TH language controls, a theme icon button, applies a MudBlazor theme with light/dark document-root state, updates PreferenceService without process-wide culture mutation, repaints preference-aware components on client-side route changes, keeps static and service/quote labels preference-backed, and avoids forced reloads for normal language toggles.</t>
+        </is>
+      </c>
+      <c r="F38" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G38" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H38" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I38" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J38" s="8" t="inlineStr">
+        <is>
+          <t>Existing localization tests cover culture normalization, language labels, route repaint behavior, theme persistence, landing chrome culture isolation, and preference-backed format labels.</t>
+        </is>
+      </c>
+      <c r="K38" s="8" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="L38" s="8" t="inlineStr">
+        <is>
+          <t>MainLayout language/theme controls -&gt; PreferenceService -&gt; maliev-culture.js document root/cookie/localStorage -&gt; preference-aware Blazor components and PreferencesController culture endpoint where persisted server preference is needed</t>
+        </is>
+      </c>
+      <c r="M38" s="8" t="inlineStr">
+        <is>
+          <t>MainLayout.razor; PreferenceService.cs; PreferenceAwareComponentBase; maliev-culture.js; PreferencesController.cs; LocalizationTests.cs</t>
+        </is>
+      </c>
+      <c r="N38" s="8" t="inlineStr">
+        <is>
+          <t>MainLayout renders language-toggle EN/TH buttons, MudIconButton theme toggle, MudThemeProvider, and preference-backed footer/header labels; PreferenceService resolves culture/theme and notifies interactive components.</t>
+        </is>
+      </c>
+      <c r="O38" s="8" t="inlineStr">
+        <is>
+          <t>POST web/v1/preferences/culture stores culture when called; client-side theme state is resolved/applied by malievCulture local/browser storage and document root attributes.</t>
+        </is>
+      </c>
+      <c r="P38" s="8" t="inlineStr">
+        <is>
+          <t>LocalizationTests.Normalize_CultureSignal_ReturnsSupportedCulture; LanguageSwitch_UsesStableEnglishAndThaiLabels; LanguageSwitch_NotifiesInteractiveCircuitWithoutForcedReload; PreferenceAwareComponents_RepaintWhenClientSideRouteChanges; ThemePreference_UsesDocumentRootAndStableToggleLabels</t>
+        </is>
+      </c>
+      <c r="Q38" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, Web BFF preferences endpoint, browser local storage/cookies</t>
+        </is>
+      </c>
+      <c r="R38" s="8" t="inlineStr">
+        <is>
+          <t>Culture preference, theme preference, document root theme state, optional server-side culture persistence</t>
+        </is>
+      </c>
+      <c r="S38" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for language/theme toggles across page navigation, prerender/interactive repaint, and storage-denied fallback.</t>
+        </is>
+      </c>
+      <c r="T38" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Layout/MainLayout.razor:8,24,28,318,336; Maliev.Web.Client/Services/PreferenceService.cs; Maliev.Web.Bff/wwwroot/js/maliev-culture.js:8,38,53; Maliev.Web.Tests/LocalizationTests.cs:42,58,152</t>
+        </is>
+      </c>
+      <c r="U38" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A39" s="8" t="inlineStr">
+        <is>
+          <t>WEB-038</t>
+        </is>
+      </c>
+      <c r="B39" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Cookie consent choices</t>
+        </is>
+      </c>
+      <c r="D39" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor, I can choose essential-only or optional cookies and reopen cookie settings later.</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>The public layout mounts a cookie consent banner after initial render when no stored consent exists, explains essential versus optional cookies, links to the cookie policy, stores either essential or optional consent through browser JavaScript, hides after a choice, keeps the site usable when storage/JS fails, and exposes a footer Cookie settings button that reopens the chooser.</t>
+        </is>
+      </c>
+      <c r="F39" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H39" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I39" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J39" s="8" t="inlineStr">
+        <is>
+          <t>Existing localization tests cover explicit optional opt-in, footer reopening, JS get/set hooks, storage failure handling, policy copy, and footer link styling.</t>
+        </is>
+      </c>
+      <c r="K39" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L39" s="8" t="inlineStr">
+        <is>
+          <t>MainLayout footer Cookie settings -&gt; CookieConsentBanner component -&gt; maliev-consent.js browser storage helpers -&gt; cookie-policy route</t>
+        </is>
+      </c>
+      <c r="M39" s="8" t="inlineStr">
+        <is>
+          <t>CookieConsentBanner.razor; MainLayout.razor; maliev-consent.js; StaticPage.razor cookie-policy content; LocalizationTests.cs</t>
+        </is>
+      </c>
+      <c r="N39" s="8" t="inlineStr">
+        <is>
+          <t>CookieConsentBanner renders accept/decline optional actions, policy link, ShowPreferencesAsync, LoadConsentAsync, malievConsent.get, malievConsent.set, and catches JS/storage failures; MainLayout includes footer Cookie settings button and component ref.</t>
+        </is>
+      </c>
+      <c r="O39" s="8" t="inlineStr">
+        <is>
+          <t>No BFF endpoint; consent is a browser-local preference used by public-site client behavior.</t>
+        </is>
+      </c>
+      <c r="P39" s="8" t="inlineStr">
+        <is>
+          <t>LocalizationTests.CookieConsent_UsesExplicitOptionalOptInAndFooterSettings</t>
+        </is>
+      </c>
+      <c r="Q39" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, browser JS/static assets</t>
+        </is>
+      </c>
+      <c r="R39" s="8" t="inlineStr">
+        <is>
+          <t>Browser consent value essential/optional in malievConsent storage; no customer account data mutation</t>
+        </is>
+      </c>
+      <c r="S39" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for first-visit banner, accept/decline persistence, footer reopen, and storage-blocked behavior.</t>
+        </is>
+      </c>
+      <c r="T39" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Components/CookieConsentBanner.razor:1,5,26,53,83; Maliev.Web.Client/Layout/MainLayout.razor:179,184,276; Maliev.Web.Bff/wwwroot/js/maliev-consent.js:41; Maliev.Web.Tests/LocalizationTests.cs:184</t>
+        </is>
+      </c>
+      <c r="U39" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="73.44999694824219" customHeight="1" s="6">
+      <c r="A40" s="8" t="inlineStr">
+        <is>
+          <t>WEB-039</t>
+        </is>
+      </c>
+      <c r="B40" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web</t>
+        </is>
+      </c>
+      <c r="C40" s="8" t="inlineStr">
+        <is>
+          <t>Footer contact and social navigation</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="inlineStr">
+        <is>
+          <t>As a visitor, I can use the footer to find company details, support links, contact channels, social profiles, and cookie settings.</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="inlineStr">
+        <is>
+          <t>The main layout footer shows the MALIEV logo, company address linked to Maps, company/support navigation, email, telephone, LINE Official Account, Facebook, YouTube, Instagram links, localized rotating manufacturing footer text, legal links, and a cookie-settings action; the customer chatbot is mounted after the footer and adjusts its floating position near footer links.</t>
+        </is>
+      </c>
+      <c r="F40" s="8" t="inlineStr">
+        <is>
+          <t>Current code-derived</t>
+        </is>
+      </c>
+      <c r="G40" s="8" t="inlineStr">
+        <is>
+          <t>Mapped to current source tests; not executed in this workbook pass.</t>
+        </is>
+      </c>
+      <c r="H40" s="8" t="inlineStr">
+        <is>
+          <t>No behavior error documented in this spreadsheet pass.</t>
+        </is>
+      </c>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>No app fix applied; spreadsheet row added from current code evidence only.</t>
+        </is>
+      </c>
+      <c r="J40" s="8" t="inlineStr">
+        <is>
+          <t>Existing source tests cover footer logo/contact/social links, localized typewriter line, chatbot footer-aware behavior, and cookie settings link.</t>
+        </is>
+      </c>
+      <c r="K40" s="8" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="L40" s="8" t="inlineStr">
+        <is>
+          <t>MainLayout footer markup -&gt; PreferenceService localized footer lines -&gt; maliev-typewriter/customer-chatbot footer-aware JS -&gt; external mail/tel/maps/LINE/social URLs</t>
+        </is>
+      </c>
+      <c r="M40" s="8" t="inlineStr">
+        <is>
+          <t>MainLayout.razor; maliev-chatbot.js; maliev-typewriter.js; HeroLayoutSourceTests.cs; LocalizationTests.cs</t>
+        </is>
+      </c>
+      <c r="N40" s="8" t="inlineStr">
+        <is>
+          <t>MainLayout renders footer-brand/address, footer company/support navs, footer-connect contact links, footer-social anchors, footer-typewriter text, legal links, Cookie settings button, CustomerChatbot, and CookieConsentBanner.</t>
+        </is>
+      </c>
+      <c r="O40" s="8" t="inlineStr">
+        <is>
+          <t>No BFF mutation; external links and client widgets are public navigation/assistive surfaces.</t>
+        </is>
+      </c>
+      <c r="P40" s="8" t="inlineStr">
+        <is>
+          <t>HeroLayoutSourceTests.FooterUsesLogoAndManufacturingContactLinks; FooterManufacturingLineUsesLocalizedTypewriterRotation; PublicLayoutIncludesCustomerChatbotWidget; LocalizationTests.CookieConsent_UsesExplicitOptionalOptInAndFooterSettings</t>
+        </is>
+      </c>
+      <c r="Q40" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web Client, browser JS/static assets, external contact/social destinations</t>
+        </is>
+      </c>
+      <c r="R40" s="8" t="inlineStr">
+        <is>
+          <t>No durable data mutation; browser interaction state for footer typewriter/chatbot positioning/cookie settings</t>
+        </is>
+      </c>
+      <c r="S40" s="8" t="inlineStr">
+        <is>
+          <t>Needs live browser verification for external link targets, footer typewriter, chatbot/footer collision behavior, and mobile footer layout.</t>
+        </is>
+      </c>
+      <c r="T40" s="8" t="inlineStr">
+        <is>
+          <t>Maliev.Web.Client/Layout/MainLayout.razor:91,93,102,112,120,137,158,179,182,184; Maliev.Web.Bff/wwwroot/js/maliev-chatbot.js:637; Maliev.Web.Tests/HeroLayoutSourceTests.cs:1387,1477; Maliev.Web.Tests/LocalizationTests.cs:184</t>
+        </is>
+      </c>
+      <c r="U40" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add current QuoteEngine workspace stories to tracker
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R63e2eee08d384756"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rce59e77dc8694b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Radcf6e82812f4f75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R47a2281c67754bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R788892d7347e4b7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R09db37d6f18d4345"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Re784060346c84eb0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rdd5ed9d983b546df"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -265,7 +265,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table1_0" displayName="Table1_0" ref="A1:U40" headerRowCount="1">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table1_0" displayName="Table1_0" ref="A1:U51" headerRowCount="1">
   <x:tableColumns count="21">
     <x:tableColumn id="1" name="Story ID"/>
     <x:tableColumn id="2" name="App Surface"/>
@@ -539,7 +539,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>39</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -549,7 +549,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>146</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4880,7 +4880,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb705f6fe6d0e43ef"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f9e14f6e3f4763"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11585,7 +11585,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfef3da734fe24e1d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce3dad237d094c0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15898,10 +15898,725 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>QE-040</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>Web-owned authentication delegation</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>As a customer, I am sent to the shared Maliev.Web account flow when I need to sign in or sign up for the quote workspace.</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>QuoteEngine delegates account entry to Maliev.Web: sign-in and sign-up routes redirect to the shared web auth pages, the Google auth route redirects to web sign-in instead of starting a separate local OAuth flow, external return URLs are not forwarded, web handoff redirects do not create a customer cookie, and the session endpoint reports not signed in for anonymous requests.</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>Mapped existing Google auth flow tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>No workbook-visible behavior error recorded; live browser auth handoff still needs a customer-session smoke pass.</x:v>
+      </x:c>
+      <x:c r="I41" t="str">
+        <x:v>No app fix applied for QE-040; tracker row added from current BFF/API client and auth-flow tests.</x:v>
+      </x:c>
+      <x:c r="J41" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K41" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L41" t="str">
+        <x:v>Browser auth routes -&gt; QuoteEngine BFF auth/session endpoints -&gt; Maliev.Web shared-cookie auth boundary -&gt; QuoteEngineApiClient session reader.</x:v>
+      </x:c>
+      <x:c r="M41" t="str">
+        <x:v>Auth route handlers; QuoteEngineApiClient.GetCurrentUserAsync</x:v>
+      </x:c>
+      <x:c r="N41" t="str">
+        <x:v>/auth/sign-in; /auth/sign-up; /auth/google; /auth/web-handoff; quote/v1/auth/session</x:v>
+      </x:c>
+      <x:c r="O41" t="str">
+        <x:v>QuoteEngineApiClient reads quote/v1/auth/session and leaves account ownership with Maliev.Web rather than a separate QuoteEngine sign-in form.</x:v>
+      </x:c>
+      <x:c r="P41" t="str">
+        <x:v>Mapped tests: GoogleAuthFlowTests sign-in redirect, external return URL blocking, sign-up redirect, Google auth redirect, web handoff redirect, and anonymous session response.</x:v>
+      </x:c>
+      <x:c r="Q41" t="str">
+        <x:v>QuoteEngine BFF, QuoteEngine Client, Maliev.Web auth surface</x:v>
+      </x:c>
+      <x:c r="R41" t="str">
+        <x:v>No QuoteEngine-local customer cookie is created by web handoff; session state is read from the shared auth boundary.</x:v>
+      </x:c>
+      <x:c r="S41" t="str">
+        <x:v>Needs live browser verification for shared-cookie sign-in, sign-up, Google redirect, and post-auth return behavior.</x:v>
+      </x:c>
+      <x:c r="T41" t="str">
+        <x:v>Maliev.QuoteEngine.Tests/GoogleAuthFlowTests.cs:9,25,40,55,68,81,96; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs:44</x:v>
+      </x:c>
+      <x:c r="U41" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>QE-041</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>Quote upload constraints and context files</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>As a customer, I can upload CAD files and supporting drawings, photos, and archives while invalid or oversized attachments are rejected clearly.</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>The workspace file input accepts the shared quote attachment allowlist, upload initiation blocks unsupported extensions and files above the QuoteEngine size limit, CAD formats satisfy the geometry gate, supplemental PDF/image/DXF/archive context files are accepted as attachments without satisfying the geometry gate, and local image previews can be applied before server processing finishes.</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>Mapped existing upload constraint tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>No workbook-visible behavior error recorded; live browser upload matrix still needs execution with representative file types.</x:v>
+      </x:c>
+      <x:c r="I42" t="str">
+        <x:v>No app fix applied for QE-041; tracker row added from current upload page, shared constraints, and focused tests.</x:v>
+      </x:c>
+      <x:c r="J42" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K42" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L42" t="str">
+        <x:v>QuoteWorkspace hidden InputFile and dropzone -&gt; QuoteEngineApiClient upload initiation -&gt; BFF upload contract -&gt; QuoteUploadConstraints shared allowlist and geometry-gate flag.</x:v>
+      </x:c>
+      <x:c r="M42" t="str">
+        <x:v>QuoteWorkspace.razor; quote-upload.js; QuoteUploadConstraints; UploadController/QuoteController upload initiation</x:v>
+      </x:c>
+      <x:c r="N42" t="str">
+        <x:v>InputFile id quote-cad-files uses SupportedAttachmentAccept; rejected files set customer-visible error text; accepted candidates carry SatisfiesGeometryGate from CAD detection.</x:v>
+      </x:c>
+      <x:c r="O42" t="str">
+        <x:v>InitiateUploadAsync receives file name, size, content type, quote session, and geometry gate data before upload completion.</x:v>
+      </x:c>
+      <x:c r="P42" t="str">
+        <x:v>Mapped tests: QuoteUploadConstraintTests supported extension reference data, size rejection, unsupported attachment rejection, supported CAD acceptance, and supplemental context-file acceptance.</x:v>
+      </x:c>
+      <x:c r="Q42" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, UploadService</x:v>
+      </x:c>
+      <x:c r="R42" t="str">
+        <x:v>Upload initiation records expected size/content metadata, quote session context, and whether a file satisfies geometry analysis prerequisites.</x:v>
+      </x:c>
+      <x:c r="S42" t="str">
+        <x:v>Needs browser upload coverage for CAD, PDF, image, DXF, ZIP, oversize, and unsupported file paths.</x:v>
+      </x:c>
+      <x:c r="T42" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor:21,526,631,643,678,697,702; Maliev.QuoteEngine.Shared/Quotes/QuoteUploadConstraints.cs:63,72,82,94,137; Maliev.QuoteEngine.Tests/QuoteUploadConstraintTests.cs:39,58,74,90,113</x:v>
+      </x:c>
+      <x:c r="U42" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>QE-042</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>Composer attachment picker guard</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>As a customer, I can click the composer add button to open the file picker once without freezing the workspace or re-entering the picker.</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>The launch shell delegates add-button uploads to QuoteWorkspace.OpenFilePickerAsync, the workspace ignores picker requests until route state is initialized and while another picker open is in progress, the JS bridge opens the hidden quote-cad-files input, and the dropzone is registered with click-to-open disabled so drag/drop and composer add actions do not double-trigger each other.</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>Mapped existing source tests for picker guard and dropzone click behavior; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>No workbook-visible behavior error recorded; live browser add-button smoke still needs execution.</x:v>
+      </x:c>
+      <x:c r="I43" t="str">
+        <x:v>No app fix applied for QE-042; tracker row added from current workspace and JS upload guard code.</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K43" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L43" t="str">
+        <x:v>QuoteAgentLaunchShell OnUploadRequested event -&gt; QuoteWorkspace.OpenFilePickerAsync state guard -&gt; quoteEngineUploads.openFilePicker JS bridge -&gt; hidden InputFile/dropzone behavior.</x:v>
+      </x:c>
+      <x:c r="M43" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; QuoteWorkspace.razor; quote-upload.js</x:v>
+      </x:c>
+      <x:c r="N43" t="str">
+        <x:v>Composer add control invokes OnUploadRequested; OpenFilePickerAsync uses _isOpeningFilePicker and UploadInputId quote-cad-files; dropzone registration passes clickToOpen = false.</x:v>
+      </x:c>
+      <x:c r="O43" t="str">
+        <x:v>No server write happens until files are selected and upload initiation begins.</x:v>
+      </x:c>
+      <x:c r="P43" t="str">
+        <x:v>Mapped tests: QuoteEngineSourceTests picker guard assertions, OnUploadRequested wiring, dropzone clickToOpen false, and JS clickToOpen option handling.</x:v>
+      </x:c>
+      <x:c r="Q43" t="str">
+        <x:v>QuoteEngine Client</x:v>
+      </x:c>
+      <x:c r="R43" t="str">
+        <x:v>Only transient client picker state is created until files are selected.</x:v>
+      </x:c>
+      <x:c r="S43" t="str">
+        <x:v>Needs live browser validation for repeated plus-clicks, canceling the picker, and drag/drop after cancel.</x:v>
+      </x:c>
+      <x:c r="T43" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor:49,58,103,279,289,291,296,299,303; Maliev.QuoteEngine.Client/wwwroot/js/quote-upload.js:89,115,158,224,420; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:600,679,723,730</x:v>
+      </x:c>
+      <x:c r="U43" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>QE-043</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>Starter manufacturing prompts</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>As a customer opening the empty workspace, I can choose manufacturing-specific starter prompts and have them placed into the composer in my language.</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>The empty chat surface shows the Make Studio heading, a bilingual starter prompt deck for CAD review, drawing-note quoting, revision comparison, materials, DFM, and production questions, and selecting a prompt types the localized text into the composer while preserving composer focus behavior.</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>Mapped existing launch shell and composer source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>No workbook-visible behavior error recorded; browser accessibility and localization smoke still needs execution.</x:v>
+      </x:c>
+      <x:c r="I44" t="str">
+        <x:v>No app fix applied for QE-043; tracker row added from current launch shell prompt deck and composer JS.</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K44" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L44" t="str">
+        <x:v>QuoteAgentLaunchShell empty-state UI -&gt; UseCaseOption deck -&gt; composer JS focus/type helpers -&gt; localized Text helper.</x:v>
+      </x:c>
+      <x:c r="M44" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; quote-agent-composer.js</x:v>
+      </x:c>
+      <x:c r="N44" t="str">
+        <x:v>The empty state renders What do you want to make today?, visible starter cards, and ApplyUseCaseAsync; composer helper can focus and type selected prompt text.</x:v>
+      </x:c>
+      <x:c r="O44" t="str">
+        <x:v>No BFF write occurs until the customer submits the populated composer text.</x:v>
+      </x:c>
+      <x:c r="P44" t="str">
+        <x:v>Mapped tests: QuoteEngineSourceTests empty prompt heading, composer focus, visible starter prompt deck, ApplyUseCaseAsync, prompt content, and native scrolling styles.</x:v>
+      </x:c>
+      <x:c r="Q44" t="str">
+        <x:v>QuoteEngine Client</x:v>
+      </x:c>
+      <x:c r="R44" t="str">
+        <x:v>Draft composer text is updated locally from the selected starter prompt.</x:v>
+      </x:c>
+      <x:c r="S44" t="str">
+        <x:v>Needs browser validation for keyboard navigation, Thai/English prompt selection, and focus after selection.</x:v>
+      </x:c>
+      <x:c r="T44" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:537,1362,1367,2134,2185,2202,2728,6051,6059; Maliev.QuoteEngine.Client/wwwroot/js/quote-agent-composer.js:396,413,449; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1126,1205,1271,1276,1286,1343,1468</x:v>
+      </x:c>
+      <x:c r="U44" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>QE-044</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>Smooth stream presentation</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>As a customer, I see assistant responses arrive smoothly with a clear thinking loader and reliable scroll-to-latest behavior.</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>Assistant delta events append to a pending stream buffer instead of forcing every raw chunk directly into the UI, the response loader uses animated dot elements while the agent is working, programmatic scroll-to-latest suppresses the manual scroll button until the user leaves the bottom again, and stream completion requests a final scroll/update.</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>Mapped existing stream, loader, and scroll source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>No workbook-visible behavior error recorded; live browser stream-smoothing smoke still needs execution against a fast model response.</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>No app fix applied for QE-044; tracker row added from current launch shell stream presentation code.</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K45" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L45" t="str">
+        <x:v>Agent stream event reader -&gt; QuoteAgentLaunchShell stream buffer/render cadence -&gt; chat thread scroll state -&gt; composer/loader CSS and JS scroll helpers.</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; quote-agent-composer.js; QuoteAgentUiHelpers</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>Stream handler detects delta events, queues assistant deltas, shows qe-agent-response-loader, and manages qe-agent-scroll-to-bottom visibility through thread scroll callbacks.</x:v>
+      </x:c>
+      <x:c r="O45" t="str">
+        <x:v>BFF stream contract remains delta/response/error events; UI presentation is handled client-side.</x:v>
+      </x:c>
+      <x:c r="P45" t="str">
+        <x:v>Mapped tests: QuoteEngineSourceTests stream delta handling, scroll button suppression, animated response loader, structured thinking stream hook, and render update assertions.</x:v>
+      </x:c>
+      <x:c r="Q45" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF stream endpoint</x:v>
+      </x:c>
+      <x:c r="R45" t="str">
+        <x:v>Transient message pending-stream content and scroll state are updated in the client.</x:v>
+      </x:c>
+      <x:c r="S45" t="str">
+        <x:v>Needs live stream timing validation for long responses, fast responses, and manual scroll interruption.</x:v>
+      </x:c>
+      <x:c r="T45" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:639,987,2927,3057,3081,4257,4275,4285,4303; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1118,1817,1832,1847,1974</x:v>
+      </x:c>
+      <x:c r="U45" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>QE-045</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>Collapsed reasoning and tool progress</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>As a customer, I can optionally inspect what the agent is doing without the response being dominated by raw tool details.</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>The assistant message renders reasoning as a collapsed disclosure by default, live reasoning entries interleave model thoughts with concise tool markers, unavailable live reasoning falls back to a clear message, completed tool steps are summarized into readable manufacturing actions, and generated-preview summaries omit internal IDs while keeping useful descriptions and command counts.</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>Mapped existing reasoning and summarizer tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>No workbook-visible behavior error recorded; live browser reasoning disclosure smoke still needs execution.</x:v>
+      </x:c>
+      <x:c r="I46" t="str">
+        <x:v>No app fix applied for QE-045; tracker row added from current reasoning UI and BFF summarizer code.</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K46" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L46" t="str">
+        <x:v>QuoteNotificationsHub thinking events -&gt; QuoteAgentService step summarization -&gt; QuoteAgentLaunchShell reasoning disclosure and stream entries -&gt; shared QuoteAgentThinkingStepDto.</x:v>
+      </x:c>
+      <x:c r="M46" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; QuoteAgentService; ThinkingStepSummarizer</x:v>
+      </x:c>
+      <x:c r="N46" t="str">
+        <x:v>The message row renders qe-agent-reasoning-summary, qe-agent-reasoning-stream, qe-agent-reasoning-tool, and qe-agent-reasoning-thought elements.</x:v>
+      </x:c>
+      <x:c r="O46" t="str">
+        <x:v>QuoteAgentService summarizes tool steps before publishing final state and emits model reasoning entries while the turn streams.</x:v>
+      </x:c>
+      <x:c r="P46" t="str">
+        <x:v>Mapped tests: ThinkingStepSummarizerTests for configuration, estimate, upload registration, generated preview request/result summaries; QuoteEngineSourceTests for interleaved reasoning and collapsed default.</x:v>
+      </x:c>
+      <x:c r="Q46" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, SignalR quote notifications, ChatbotService stream</x:v>
+      </x:c>
+      <x:c r="R46" t="str">
+        <x:v>Transient thinking entries and summarized tool-step text are stored in the session response state.</x:v>
+      </x:c>
+      <x:c r="S46" t="str">
+        <x:v>Needs browser validation for disclosure expand/collapse, long reasoning content, and bilingual labels.</x:v>
+      </x:c>
+      <x:c r="T46" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:615,619,624,631,3686,3750,3800; Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:361,424,1036,1047,1062; Maliev.QuoteEngine.Tests/ThinkingStepSummarizerTests.cs:17,32,79,92,104; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1864,1883</x:v>
+      </x:c>
+      <x:c r="U46" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>QE-046</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>Browser-local DFM runtime and overlays</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>As a customer, I can see browser-computed manufacturability analysis reflected in the part detail view while waiting for or complementing server analysis.</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>The viewer can run browser-local DFM for the selected process, submit the local report to the BFF, apply matching results to the selected part, preserve current process results when server status has no replacement report, show local runtime running/unavailable state, and toggle issue overlays in the 3D viewer for DFM findings.</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>Mapped existing local DFM, viewer, and overlay source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>No workbook-visible behavior error recorded; browser runtime and overlay smoke still needs execution with real files.</x:v>
+      </x:c>
+      <x:c r="I47" t="str">
+        <x:v>No app fix applied for QE-046; tracker row added from current local DFM runtime, BFF, and viewer code.</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L47" t="str">
+        <x:v>QePartViewer JS module/browser advisory runtime -&gt; QePartDetailCard local DFM mapper -&gt; AgentController SubmitLocalDfm -&gt; QuoteAgentService/session analysis state -&gt; QeDfmOverlayPanel overlay controls.</x:v>
+      </x:c>
+      <x:c r="M47" t="str">
+        <x:v>QePartViewer.razor; QePartDetailCard.razor; QeDfmTab.razor; QeDfmOverlayPanel.razor; quote-part-viewer.js; AgentController</x:v>
+      </x:c>
+      <x:c r="N47" t="str">
+        <x:v>Part detail renders QeDfmTab, QePartViewer, and QeDfmOverlayPanel; local runtime state drives analyzing/unavailable labels and overlay visibility.</x:v>
+      </x:c>
+      <x:c r="O47" t="str">
+        <x:v>POST quote/v1/agent/sessions/{sessionId}/dfm/local applies a browser-computed report into the session analysis store through QuoteAgentLocalDfmRequest.</x:v>
+      </x:c>
+      <x:c r="P47" t="str">
+        <x:v>Mapped tests: QeLocalDfmMapper current report acceptance/rejection, analysis status preservation, process aliases, viewer/detail wiring, overlay labels, deferred JS module handling, and runtime unavailable reset.</x:v>
+      </x:c>
+      <x:c r="Q47" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, Geometry runtime assets</x:v>
+      </x:c>
+      <x:c r="R47" t="str">
+        <x:v>Local DFM report fields, runtime status fields, non-manifold reasons, process-specific reports, and overlay state are updated for the selected part/session.</x:v>
+      </x:c>
+      <x:c r="S47" t="str">
+        <x:v>Needs live browser validation for runtime loading, worker failures, overlay toggles, and server-status reconciliation.</x:v>
+      </x:c>
+      <x:c r="T47" t="str">
+        <x:v>Maliev.QuoteEngine.Bff/Controllers/AgentController.cs:219,224; Maliev.QuoteEngine.Client/Components/QuoteEngine/QePartDetailCard.razor:153,216,218,273,290,305,349,365; Maliev.QuoteEngine.Client/Components/QuoteEngine/QePartViewer.razor:177,431,437,450; Maliev.QuoteEngine.Client/wwwroot/js/quote-part-viewer.js:3795,5079,5183; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:248,303,324,3997,4112,5232,5350</x:v>
+      </x:c>
+      <x:c r="U47" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>QE-047</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Google Drive OAuth and connector handoff</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>As a signed-in customer, I can connect Google Drive, browse eligible Drive files, disconnect the integration, and let the agent open a safe browser handoff when Drive context is needed.</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>The connector registry exposes Google Drive with signed-in gating, configuration and connection status, BFF OAuth start/callback/status/disconnect/list endpoints manage the customer Drive connection, file listing handles missing or expired Drive authorization with customer-readable problem details, and connector handoff uses the session-scoped BFF route plus agent context header instead of a tool-only browser call.</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>Mapped existing connector endpoint/source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>No workbook-visible behavior error recorded; live OAuth and Drive listing smoke still needs configured credentials.</x:v>
+      </x:c>
+      <x:c r="I48" t="str">
+        <x:v>No app fix applied for QE-047; tracker row added from current connector UI, BFF controller, service, API client, and tests.</x:v>
+      </x:c>
+      <x:c r="J48" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K48" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L48" t="str">
+        <x:v>QuoteAgentLaunchShell connector panel -&gt; QuoteEngineApiClient -&gt; AgentController connector handoff -&gt; QuoteAgentService connector registry -&gt; GoogleDriveConnectorController OAuth/listing -&gt; Google Drive API.</x:v>
+      </x:c>
+      <x:c r="M48" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; AgentController; GoogleDriveConnectorController; QuoteAgentService; QuoteEngineApiClient</x:v>
+      </x:c>
+      <x:c r="N48" t="str">
+        <x:v>UI shows signed-in availability copy, connected/disconnected Drive states, Continue to Google Drive, Disconnect Google Drive, and connector handoff actions.</x:v>
+      </x:c>
+      <x:c r="O48" t="str">
+        <x:v>GET quote/v1/agent/sessions/{sessionId}/connectors/{connectorId}/handoff and Google Drive connector endpoints return customer-safe status, handoff URL/message, or ProblemDetails.</x:v>
+      </x:c>
+      <x:c r="P48" t="str">
+        <x:v>Mapped tests: QuoteAgentEndpointTests connector registry, handoff, not-found status, configured/unconfigured Drive, connected Drive, and Drive list behavior; QuoteEngineSourceTests connector UI/API client wiring.</x:v>
+      </x:c>
+      <x:c r="Q48" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, Google Drive API</x:v>
+      </x:c>
+      <x:c r="R48" t="str">
+        <x:v>Customer Drive connection tokens/status are stored through the connector store; selected file metadata is returned as customer-safe DTOs.</x:v>
+      </x:c>
+      <x:c r="S48" t="str">
+        <x:v>Needs configured OAuth browser test for connect, callback, list, disconnect, and expired-token recovery.</x:v>
+      </x:c>
+      <x:c r="T48" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:293,1968,1972,2009,4663,5913,5922,5953; Maliev.QuoteEngine.Bff/Controllers/AgentController.cs:190,192; Maliev.QuoteEngine.Bff/Controllers/GoogleDriveConnectorController.cs:25,69,114,134,151,157,172,184,198; Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:2590,2598,2604,2618,2649; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs:393,399,410; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:4093,4113,4146,4198,4205,4241,4258; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1045,1061,1190,1233</x:v>
+      </x:c>
+      <x:c r="U48" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>QE-048</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Quote summary and guarded checkout bar</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>As a customer, I can move from estimate to formal quote approval, order creation, terms acceptance, and payment from one quote summary bar.</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>The quote summary bar shows quote total, line details, formal quote approval, order status, terms checkbox, payment action, and payment link states; checkout is disabled until the quote/order/payment prerequisites are satisfied; unauthenticated checkout redirects through shared sign-in with the order return path; and the BFF validates accepted terms, customer order ownership, order amount/currency, delivery snapshot persistence, and accepted order status before initiating payment.</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>Mapped existing quote summary/payment source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>No workbook-visible behavior error recorded; live quote-to-payment checkout smoke still needs execution.</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>No app fix applied for QE-048; tracker row added from current summary bar, workspace, QuoteController, and source tests.</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>QeQuoteSummaryBar UI -&gt; QuoteWorkspace quote/order/payment handlers -&gt; QuoteEngineApiClient -&gt; QuoteController -&gt; OrderService, DeliveryService, PaymentService.</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>QeQuoteSummaryBar.razor; QuoteWorkspace.razor; QuoteController; QuoteEngineApiClient</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>Summary bar renders Quote Total, Estimate details, Approve quote, Create order, terms checkbox, Pay now, order status, and payment-ready link.</x:v>
+      </x:c>
+      <x:c r="O49" t="str">
+        <x:v>QuoteController InitiatePayment validates terms, ownership, order details, amount/currency, delivery snapshot, Accepted status, return/cancel URLs, and idempotency key before calling PaymentService.</x:v>
+      </x:c>
+      <x:c r="P49" t="str">
+        <x:v>Mapped tests: QuoteEngineSourceTests quote summary bar actions, workspace payment wiring, checkout redirect path, payment error handling, and API client method presence.</x:v>
+      </x:c>
+      <x:c r="Q49" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, OrderService, DeliveryService, PaymentService</x:v>
+      </x:c>
+      <x:c r="R49" t="str">
+        <x:v>Formal quote, manufacturing order, delivery snapshot, accepted status, checkout attempt, and payment transaction metadata are created or advanced.</x:v>
+      </x:c>
+      <x:c r="S49" t="str">
+        <x:v>Needs end-to-end checkout test with signed-in customer, delivery snapshot, accepted order status, and payment return.</x:v>
+      </x:c>
+      <x:c r="T49" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteEngine/QeQuoteSummaryBar.razor:38,50,67,73,88,91,98,132,139,152,158,169; Maliev.QuoteEngine.Client/Pages/QuoteWorkspace.razor:930,936,1028,1063; Maliev.QuoteEngine.Bff/Controllers/QuoteController.cs:908,921,947,968,981,1013,1017,1035,1058; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:4058,4078,4083,4092,4106</x:v>
+      </x:c>
+      <x:c r="U49" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>QE-049</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Payment return and order status notifications</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>As a customer, I can return from payment to the correct order and receive order-level payment status updates.</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>Payment success and cancel URLs are generated with the order number, the return pages read that order number and link back to order detail, and provider-neutral payment failed, pending, cancelled, and expired events are pushed to the order SignalR group with order number and payment ID so the customer-facing order view can react to payment state changes.</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>Mapped existing payment return and payment consumer source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>No workbook-visible behavior error recorded; live payment return and SignalR notification smoke still needs execution.</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>No app fix applied for QE-049; tracker row added from current payment return URLs and notification consumer tests.</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L50" t="str">
+        <x:v>QuoteController payment return URLs -&gt; PaymentSuccess/PaymentCancel pages -&gt; payment event consumers -&gt; QuoteNotificationsHub order group.</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>QuoteController; PaymentSuccess.razor; PaymentCancel.razor; QuotePaymentFailed/Pending/Cancelled/Expired consumers</x:v>
+      </x:c>
+      <x:c r="N50" t="str">
+        <x:v>Payment return pages display success or cancellation state and link back to /orders/{orderNumber}.</x:v>
+      </x:c>
+      <x:c r="O50" t="str">
+        <x:v>Payment event consumers publish provider-neutral payloads to QuoteNotificationsHub.OrderGroup(orderNumber).</x:v>
+      </x:c>
+      <x:c r="P50" t="str">
+        <x:v>Mapped tests: QuoteEngineSourceTests payment return page routing and failed/pending/cancelled/expired payment consumer group pushes.</x:v>
+      </x:c>
+      <x:c r="Q50" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, PaymentService events, SignalR quote notifications</x:v>
+      </x:c>
+      <x:c r="R50" t="str">
+        <x:v>Payment status notification payloads are pushed to order groups; no new workbook-tracked persistent state is created by the return pages.</x:v>
+      </x:c>
+      <x:c r="S50" t="str">
+        <x:v>Needs runtime validation for hosted payment return, cancelled payment, pending payment, and failed payment notification rendering.</x:v>
+      </x:c>
+      <x:c r="T50" t="str">
+        <x:v>Maliev.QuoteEngine.Bff/Controllers/QuoteController.cs:1013,1014; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:2788,2796,2799,2800,2804,2807,2808,2810,3226,3284,3340,3398</x:v>
+      </x:c>
+      <x:c r="U50" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>QE-050</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>Last-turn edit and resubmission</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>As a customer, I can revise my latest message and have the agent regenerate from the corrected turn instead of appending an unrelated new thread entry.</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>When the latest user message is edited, the client removes the local last user/assistant turn pair, sends EditLastTurn in the agent request, restores the removed turn on submission failure, and the BFF asks ChatbotService to truncate the last turn before resubmitting; if truncation is rejected, the BFF does not resubmit the corrected message.</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>Mapped existing edit-last-turn endpoint and ChatbotService contract tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>No workbook-visible behavior error recorded; live browser edit/resubmit smoke still needs execution.</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>No app fix applied for QE-050; tracker row added from current client edit flow, shared DTO, BFF service, and tests.</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L51" t="str">
+        <x:v>QuoteAgentLaunchShell message edit state -&gt; QuoteAgentMessageRequest.EditLastTurn DTO -&gt; QuoteAgentService -&gt; ChatbotService truncate-last-turn contract -&gt; stream/send retry flow.</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; QuoteAgentDtos; QuoteAgentService; ChatbotServiceClient</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>Client sets EditLastTurn when the editable message is the last user message and removes/restores the local turn around submission.</x:v>
+      </x:c>
+      <x:c r="O51" t="str">
+        <x:v>QuoteAgentService calls TruncateLastTurnAsync before send/stream resubmission and stops if truncation fails.</x:v>
+      </x:c>
+      <x:c r="P51" t="str">
+        <x:v>Mapped tests: ChatbotServiceClientContractTests truncate request/false return; QuoteAgentEndpointTests edit-last-turn stream truncation and no-resubmit on truncate failure.</x:v>
+      </x:c>
+      <x:c r="Q51" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, ChatbotService</x:v>
+      </x:c>
+      <x:c r="R51" t="str">
+        <x:v>Client message rows are replaced locally; ChatbotService conversation history is truncated for the latest turn before retry.</x:v>
+      </x:c>
+      <x:c r="S51" t="str">
+        <x:v>Needs browser validation for edit affordance, failed truncate user feedback, and successful regenerated response.</x:v>
+      </x:c>
+      <x:c r="T51" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:2884,2886,2917,2987,3021,3034; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs:76; Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:184,293; Maliev.QuoteEngine.Tests/ChatbotServiceClientContractTests.cs:10,30; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:749,783</x:v>
+      </x:c>
+      <x:c r="U51" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6db9e38e6afd4c15"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde24a80e784248fd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add current Web boundary stories to tracker
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R788892d7347e4b7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R09db37d6f18d4345"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Re784060346c84eb0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rdd5ed9d983b546df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5fef2858502c424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rc465ab75a3104e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rac576a562f60464c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R695c329b5c744c01"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -471,97 +471,73 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
-      <x:c r="A1" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Canonical MALIEV feature user story tracker</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B1" s="7" t="n"/>
+      <x:c r="A1" s="7" t="str">
+        <x:v>Canonical MALIEV feature user story tracker</x:v>
+      </x:c>
+      <x:c r="B1" s="7"/>
     </x:row>
     <x:row r="2" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
-      <x:c r="A2" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Expanded current-code rebuild</x:t>
-        </x:is>
+      <x:c r="A2" s="8" t="str">
+        <x:v>Expanded current-code rebuild</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str">
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
-      <x:c r="A3" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Workbook rule</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Only current code-derived user stories are tracked. Rows are derived from current UI, BFF/API, service-client, and DTO boundaries.</x:t>
-        </x:is>
+      <x:c r="A3" s="8" t="str">
+        <x:v>Workbook rule</x:v>
+      </x:c>
+      <x:c r="B3" s="8" t="str">
+        <x:v>Only current code-derived user stories are tracked. Rows are derived from current UI, BFF/API, service-client, and DTO boundaries.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
-      <x:c r="A4" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Service</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current tracked stories</x:t>
-        </x:is>
+      <x:c r="A4" s="7" t="str">
+        <x:v>Service</x:v>
+      </x:c>
+      <x:c r="B4" s="7" t="str">
+        <x:v>Current tracked stories</x:v>
       </x:c>
     </x:row>
     <x:row r="5" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
-      <x:c r="A5" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Maliev.Web</x:t>
-        </x:is>
+      <x:c r="A5" s="8" t="str">
+        <x:v>Maliev.Web</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>39</x:v>
+        <x:v>51</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
-      <x:c r="A6" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Maliev.Intranet</x:t>
-        </x:is>
+      <x:c r="A6" s="8" t="str">
+        <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
         <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
-      <x:c r="A7" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Maliev.QuoteEngine</x:t>
-        </x:is>
+      <x:c r="A7" s="8" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
         <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
-      <x:c r="A8" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Total</x:t>
-        </x:is>
+      <x:c r="A8" s="8" t="str">
+        <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>157</x:v>
+        <x:v>169</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
-      <x:c r="A9" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Next loop</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B9" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">After workbook review, start story-by-story behavior testing, document errors, fix UX/logistical issues, and retest every affected behavior.</x:t>
-        </x:is>
+      <x:c r="A9" s="8" t="str">
+        <x:v>Next loop</x:v>
+      </x:c>
+      <x:c r="B9" s="8" t="str">
+        <x:v>After workbook review, start story-by-story behavior testing, document errors, fix UX/logistical issues, and retest every affected behavior.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4877,10 +4853,790 @@
         </x:is>
       </x:c>
     </x:row>
+    <x:row r="41">
+      <x:c r="A41" t="str">
+        <x:v>WEB-040</x:v>
+      </x:c>
+      <x:c r="B41" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C41" t="str">
+        <x:v>Material datasheet PDF boundary</x:v>
+      </x:c>
+      <x:c r="D41" t="str">
+        <x:v>As a buyer, I can download a localized material datasheet PDF from the public material detail page.</x:v>
+      </x:c>
+      <x:c r="E41" t="str">
+        <x:v>The material detail page exposes a PDF action for a slug-addressed material; the BFF serves GET web/v1/materials/{slug}/datasheet.pdf anonymously, returns 404 for unknown slugs, maps localized material specs, category, bands, disclaimer, and optional embedded local image metadata into PdfService, rejects non-PDF downstream responses, and returns a customer-safe 503 when PdfService is unavailable.</x:v>
+      </x:c>
+      <x:c r="F41" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G41" t="str">
+        <x:v>Mapped existing material datasheet PDF source and endpoint tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H41" t="str">
+        <x:v>No workbook-pass behavior error documented; story-by-story browser/API test loop pending.</x:v>
+      </x:c>
+      <x:c r="I41" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J41" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K41" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L41" t="str">
+        <x:v>MaterialDetail UI -&gt; MaterialsController -&gt; MaterialDatasheetPdfService -&gt; PdfServiceClient -&gt; PdfService material datasheet render contract</x:v>
+      </x:c>
+      <x:c r="M41" t="str">
+        <x:v>MaterialDetail.razor; MaterialsController; MaterialDatasheetPdfService; PdfServiceClient</x:v>
+      </x:c>
+      <x:c r="N41" t="str">
+        <x:v>MaterialDetail renders the datasheet action and MaterialsController exposes web/v1/materials/{slug}/datasheet.pdf with application/pdf output.</x:v>
+      </x:c>
+      <x:c r="O41" t="str">
+        <x:v>MaterialDatasheetPdfService builds MaterialDatasheetPdfRequest and PdfServiceClient posts to /pdf/v1/material-datasheets/render with PDF content validation.</x:v>
+      </x:c>
+      <x:c r="P41" t="str">
+        <x:v>Mapped tests: MaterialDatasheetPdfSourceTests.MaterialDatasheetPdfIsRenderedByPdfServiceNotWebBff, MaterialDatasheetPdfMapsLocalizedCatalogContent, MaterialDatasheetEndpointIsAnonymousSlugRoutedAndResilient; WebBffEndpointTests material PDF checks.</x:v>
+      </x:c>
+      <x:c r="Q41" t="str">
+        <x:v>Maliev.Web Client, Web BFF, PdfService</x:v>
+      </x:c>
+      <x:c r="R41" t="str">
+        <x:v>No durable Web data; transient PDF request/response bytes only.</x:v>
+      </x:c>
+      <x:c r="S41" t="str">
+        <x:v>Needs live browser download and PdfService unavailable-path smoke in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T41" t="str">
+        <x:v>Maliev.Web.Client/Pages/MaterialDetail.razor:50,60; Maliev.Web.Bff/Controllers/MaterialsController.cs:26; Maliev.Web.Bff/Services/MaterialDatasheetPdfService.cs:18,49,67; Maliev.Web.Bff/Clients/PdfServiceClient.cs:59,63,70; Maliev.Web.Tests/MaterialDatasheetPdfSourceTests.cs:12,32,51; Maliev.Web.Tests/WebBffEndpointTests.cs:130,150</x:v>
+      </x:c>
+      <x:c r="U41" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" t="str">
+        <x:v>WEB-041</x:v>
+      </x:c>
+      <x:c r="B42" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C42" t="str">
+        <x:v>Material search and comparison guidance</x:v>
+      </x:c>
+      <x:c r="D42" t="str">
+        <x:v>As a buyer comparing manufacturing materials, I can search the public material library and compare a material with similar options.</x:v>
+      </x:c>
+      <x:c r="E42" t="str">
+        <x:v>The materials overview groups materials by manufacturing process, filters by search input across name, family, process, category, summary, specs, standards, best-fit text, pros, and cons, shows an empty-search state, and links to slug detail pages. Detail pages show specs, standards, datasheet disclaimer, pro/con insight cards, similar materials, and a direct comparison table with one property-label column.</x:v>
+      </x:c>
+      <x:c r="F42" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G42" t="str">
+        <x:v>Mapped existing material overview and material comparison source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H42" t="str">
+        <x:v>No workbook-pass behavior error documented; search and comparison browser loop pending.</x:v>
+      </x:c>
+      <x:c r="I42" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J42" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K42" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L42" t="str">
+        <x:v>Materials.razor and MaterialDetail.razor -&gt; SiteContent material catalog -&gt; preference-aware localized rendering</x:v>
+      </x:c>
+      <x:c r="M42" t="str">
+        <x:v>Materials.razor; MaterialDetail.razor; SiteContent material catalog</x:v>
+      </x:c>
+      <x:c r="N42" t="str">
+        <x:v>Materials page renders search, category groups, material cards, and no-match state; MaterialDetail renders specs, insights, similar materials, and comparison layout.</x:v>
+      </x:c>
+      <x:c r="O42" t="str">
+        <x:v>No Web BFF mutation; material content is static client-side SiteContent and datasheet downloads route through the separate PDF boundary.</x:v>
+      </x:c>
+      <x:c r="P42" t="str">
+        <x:v>Mapped tests: MaterialDatasheetPdfSourceTests.MaterialCatalogExposesSlugsSpecsAndDatasheetHelpers, MaterialsOverviewIsSearchableHorizontalCardList; HeroLayoutSourceTests.MaterialsDirectComparisonUsesSingleLabelColumnAndInsightIcons.</x:v>
+      </x:c>
+      <x:c r="Q42" t="str">
+        <x:v>Maliev.Web Client</x:v>
+      </x:c>
+      <x:c r="R42" t="str">
+        <x:v>No server data; local search state and selected material slug only.</x:v>
+      </x:c>
+      <x:c r="S42" t="str">
+        <x:v>Needs keyboard/mobile search and comparison readability pass in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T42" t="str">
+        <x:v>Maliev.Web.Client/Pages/Materials.razor:18,22,43,94,104,106,109; Maliev.Web.Client/Pages/MaterialDetail.razor:50,60,91,110,112; Maliev.Web.Tests/MaterialDatasheetPdfSourceTests.cs:70,102; Maliev.Web.Tests/HeroLayoutSourceTests.cs:2272</x:v>
+      </x:c>
+      <x:c r="U42" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" t="str">
+        <x:v>WEB-042</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>Website assistant topic guard and degraded states</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>As a visitor, I can ask the website assistant manufacturing and account questions while receiving safe fallback behavior when the assistant service is unavailable.</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>Opening the assistant starts a website session and returns a greeting. Manufacturing questions create or reuse a ChatbotService session, forward requested language and bounded untrusted customer context, preserve suggested actions, replace stale sessions, and return natural greetings. Off-topic questions are stopped in the Web BFF, account-specific questions require signed-in context before reaching ChatbotService, and service downtime or unconfigured clients produce customer-safe degraded responses.</x:v>
+      </x:c>
+      <x:c r="F43" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G43" t="str">
+        <x:v>Mapped existing customer chatbot boundary tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H43" t="str">
+        <x:v>No workbook-pass behavior error documented; live assistant service and offline-path testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I43" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J43" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K43" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L43" t="str">
+        <x:v>CustomerChatbot UI -&gt; ChatbotController -&gt; CustomerChatbotService -&gt; ChatbotServiceClient snake_case session/message contract</x:v>
+      </x:c>
+      <x:c r="M43" t="str">
+        <x:v>CustomerChatbot.razor; ChatbotController; CustomerChatbotService; ChatbotServiceClient; ChatbotDtos</x:v>
+      </x:c>
+      <x:c r="N43" t="str">
+        <x:v>CustomerChatbot sends session and message requests to web/v1/chatbot/sessions and web/v1/chatbot/messages while displaying verified-session and degraded-state copy.</x:v>
+      </x:c>
+      <x:c r="O43" t="str">
+        <x:v>CustomerChatbotService handles topic gating, account gating, language normalization, stale-session retry, safe context wrapping, and ChatbotService unavailable exceptions.</x:v>
+      </x:c>
+      <x:c r="P43" t="str">
+        <x:v>Mapped tests: CustomerChatbotBoundaryTests StartSession, degraded session, service question routing, suggested actions, untrusted notes, requested language, off-topic guard, account sign-in gate, stale session, snake_case, no anonymous PII, and transport failure cases.</x:v>
+      </x:c>
+      <x:c r="Q43" t="str">
+        <x:v>Maliev.Web Client, Web BFF, ChatbotService</x:v>
+      </x:c>
+      <x:c r="R43" t="str">
+        <x:v>Assistant session id, browser-visible conversation messages, optional bounded customer context, shared assistant session storage.</x:v>
+      </x:c>
+      <x:c r="S43" t="str">
+        <x:v>Needs live browser assistant run with ChatbotService available and intentionally unavailable in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T43" t="str">
+        <x:v>Maliev.Web.Client/Components/CustomerChatbot.razor:771,824,940,1611,1618; Maliev.Web.Bff/Controllers/ChatbotController.cs:25,63; Maliev.Web.Bff/Services/CustomerChatbotService.cs:84,114,137,160,421,436,488; Maliev.Web.Bff/Clients/ChatbotServiceClient.cs:24,34,98; Maliev.Web.Tests/CustomerChatbotBoundaryTests.cs:19,43,92,119,189,235,259,283,395,476,531</x:v>
+      </x:c>
+      <x:c r="U43" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" t="str">
+        <x:v>WEB-043</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>Assistant widget context, popouts, and shared session</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>As a visitor, I can receive contextual assistant prompts and continue a website assistant session without the widget being intrusive.</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>The public layout includes a customer chatbot widget with a panel and assistive popout that can be opened or dismissed separately, fades until hover or focus, records local behavior events, schedules contextual hints from the current route, shares assistant session state through browser storage, provides Google/email sign-in actions for protected account questions, sanitizes rendered assistant links, and sends current page title/path context with each turn.</x:v>
+      </x:c>
+      <x:c r="F44" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G44" t="str">
+        <x:v>Mapped existing source tests for widget layout, popout, behavior hints, and page context; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H44" t="str">
+        <x:v>No workbook-pass behavior error documented; browser interaction testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I44" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J44" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K44" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L44" t="str">
+        <x:v>MainLayout public shell -&gt; CustomerChatbot component -&gt; maliev-chatbot.js shared session/popup behavior -&gt; BFF chatbot endpoints</x:v>
+      </x:c>
+      <x:c r="M44" t="str">
+        <x:v>MainLayout.razor; CustomerChatbot.razor; maliev-chatbot.js; AuthChatbotComplete.razor</x:v>
+      </x:c>
+      <x:c r="N44" t="str">
+        <x:v>CustomerChatbot renders panel, popout open/dismiss buttons, reset, action buttons, contextual hint copy, and authentication-complete route behavior.</x:v>
+      </x:c>
+      <x:c r="O44" t="str">
+        <x:v>Shared session and behavior signals stay browser-local while BFF receives only bounded CustomerChatbotRequest fields and sanitized customer context.</x:v>
+      </x:c>
+      <x:c r="P44" t="str">
+        <x:v>Mapped tests: HeroLayoutSourceTests customer chatbot widget, panel fade, contextual hints, popout timing/dismissal, local behavior tracking, localized hints, current page location context, and chatbot auth handoff.</x:v>
+      </x:c>
+      <x:c r="Q44" t="str">
+        <x:v>Maliev.Web Client, Web BFF, browser local/session storage, AuthService through sign-in routes</x:v>
+      </x:c>
+      <x:c r="R44" t="str">
+        <x:v>Browser-local assistant personalization, shared session key, behavior event counters, visible assistant messages.</x:v>
+      </x:c>
+      <x:c r="S44" t="str">
+        <x:v>Needs live hover/focus, popout dismissal, route-change hints, sign-in popup, and mobile checks in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T44" t="str">
+        <x:v>Maliev.Web.Client/Components/CustomerChatbot.razor:137,183,375,486,623,749,940,1611,1843,1927; Maliev.Web.Bff/wwwroot/js/maliev-chatbot.js:637; Maliev.Web.Client/Pages/AuthChatbotComplete.razor:1; Maliev.Web.Tests/HeroLayoutSourceTests.cs:1712,1935,1954,1979,1992,2037,2072,2096</x:v>
+      </x:c>
+      <x:c r="U44" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" t="str">
+        <x:v>WEB-044</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>Authentication, passkeys, and cross-app return</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>As a customer, I can sign in or recover access through email, Google, or passkey flows and return to the intended Web or Make Studio destination.</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>Auth pages expose email-first sign-in/sign-up, branded Google sign-in, dedicated form action routes for email sign-in, sign-up, forgot password, and reset password, browser-native validation, email verification and claim refresh routes, verification resend, passkey sign-in, and cross-app return URL preservation for trusted Make Studio destinations while the BFF remains authoritative for final return validation.</x:v>
+      </x:c>
+      <x:c r="F45" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G45" t="str">
+        <x:v>Mapped existing auth source and Web BFF endpoint tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H45" t="str">
+        <x:v>No workbook-pass behavior error documented; browser/auth-provider testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I45" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J45" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K45" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L45" t="str">
+        <x:v>Auth Razor pages -&gt; AuthController form/OAuth/passkey routes -&gt; AuthService client -&gt; cookie claims/session -&gt; trusted return URL validation</x:v>
+      </x:c>
+      <x:c r="M45" t="str">
+        <x:v>AuthSignIn.razor; AuthSignUp.razor; AuthForgotPassword.razor; AuthResetPassword.razor; AuthGoogleButton.razor; AuthController</x:v>
+      </x:c>
+      <x:c r="N45" t="str">
+        <x:v>Auth pages render email and Google choices, form action routes, recovery pages, reset requirements, and safe client return URL normalization.</x:v>
+      </x:c>
+      <x:c r="O45" t="str">
+        <x:v>AuthController handles Google callback, /quote/start, email sign-in/sign-up, forgot/reset, sign-out, verify-email, refresh-claims, resend-verification, passkey-sign-in, and trusted cross-app return validation.</x:v>
+      </x:c>
+      <x:c r="P45" t="str">
+        <x:v>Mapped tests: HeroLayoutSourceTests auth pages, form actions, cross-app return, email-first Google primary flow, live validation; WebBffEndpointTests auth form handler registration.</x:v>
+      </x:c>
+      <x:c r="Q45" t="str">
+        <x:v>Maliev.Web Client, Web BFF, AuthService, Google OAuth, passkey provider</x:v>
+      </x:c>
+      <x:c r="R45" t="str">
+        <x:v>Authentication cookie, refreshed claims, customer principal/customer id claims, return URL state, passkey sign-in request.</x:v>
+      </x:c>
+      <x:c r="S45" t="str">
+        <x:v>Needs provider-backed Google/passkey/email verification browser checks in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T45" t="str">
+        <x:v>Maliev.Web.Client/Pages/AuthSignIn.razor:66,170,223; Maliev.Web.Client/Pages/AuthForgotPassword.razor:20; Maliev.Web.Client/Pages/AuthResetPassword.razor:16,28; Maliev.Web.Client/Components/AuthGoogleButton.razor:1; Maliev.Web.Bff/Controllers/AuthController.cs:39,56,110,122,153,185,202,241,259,312,329,409,429; Maliev.Web.Tests/HeroLayoutSourceTests.cs:2591,2660,2693,2714,2740; Maliev.Web.Tests/WebBffEndpointTests.cs:584</x:v>
+      </x:c>
+      <x:c r="U45" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" t="str">
+        <x:v>WEB-045</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>Checkout draft and shipping snapshot</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>As a signed-in shopper, I can prepare checkout with billing, shipping, selected rate, and terms before payment handoff.</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>The checkout page requires cart items, collects legal billing details, shipping recipient and address fields, phone, company and tax fields, live shipping rates, selected shipping-rate snapshot, and MALIEV terms acceptance. The BFF rejects anonymous checkout with a sign-in return to /checkout, returns customer-correctable validation problems, refuses checkout before terms are accepted, creates CommerceService carts and lines, and stores billing and shipping snapshots on the checkout session.</x:v>
+      </x:c>
+      <x:c r="F46" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G46" t="str">
+        <x:v>Mapped existing checkout source, controller, and service tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H46" t="str">
+        <x:v>No workbook-pass behavior error documented; checkout and shipping-rate browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I46" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J46" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K46" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L46" t="str">
+        <x:v>Checkout.razor -&gt; MalievApiClient checkout/shipping calls -&gt; CheckoutController -&gt; CheckoutDraftService -&gt; CustomerService and CommerceService clients</x:v>
+      </x:c>
+      <x:c r="M46" t="str">
+        <x:v>Checkout.razor; CheckoutController; CheckoutDraftService; CheckoutDtos</x:v>
+      </x:c>
+      <x:c r="N46" t="str">
+        <x:v>Checkout page renders required billing/shipping/contact/company/tax/rate/terms fields and calls CreateCheckoutDraftAsync after valid submission.</x:v>
+      </x:c>
+      <x:c r="O46" t="str">
+        <x:v>POST web/v1/checkout/draft returns OK, 400, 401, or 503; POST web/v1/checkout/draft-form provides progressive-enhancement redirects; CheckoutDraftService builds cart, cart lines, and checkout-session snapshots.</x:v>
+      </x:c>
+      <x:c r="P46" t="str">
+        <x:v>Mapped tests: CheckoutDraftServiceTests billing/shipping snapshot and terms rejection; CheckoutControllerTests anonymous redirect and invalid detail problem; HeroLayoutSourceTests checkout page fields.</x:v>
+      </x:c>
+      <x:c r="Q46" t="str">
+        <x:v>Maliev.Web Client, Web BFF, CustomerService, CommerceService, DeliveryService shipping rates</x:v>
+      </x:c>
+      <x:c r="R46" t="str">
+        <x:v>CheckoutDraftRequest, cart items, shipping details, selected rate, billing/shipping JSON snapshots, Commerce cart and checkout session.</x:v>
+      </x:c>
+      <x:c r="S46" t="str">
+        <x:v>Needs live signed-in checkout with shipping-rate fetch and payment-handoff expectations in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T46" t="str">
+        <x:v>Maliev.Web.Client/Pages/Checkout.razor:24,53,62,118,145,223; Maliev.Web.Bff/Controllers/CheckoutController.cs:21,58,84; Maliev.Web.Bff/Services/CheckoutDraftService.cs:15,25,37,50,53; Maliev.Web.Shared/Commerce/CheckoutDtos.cs:31,56,59,62; Maliev.Web.Tests/CheckoutDraftServiceTests.cs:21,96; Maliev.Web.Tests/CheckoutControllerTests.cs:21,43; Maliev.Web.Tests/HeroLayoutSourceTests.cs:2453</x:v>
+      </x:c>
+      <x:c r="U46" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" t="str">
+        <x:v>WEB-046</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>Account profile, company, and session safety</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>As a signed-in customer, I can view and update my customer profile and company details without stale or invalid sessions showing private data.</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>Account pages require the customer-account policy, show loading and sanitized unavailable states, redirect invalid sessions to sign-in, render customer avatar/profile/company summary, expose profile editing with validation, email-change controls, language/timezone selectors, company fields, company search, and create or link company records through CustomerService. The BFF rejects tax/company identifiers without a company name and maps CustomerService timeouts or missing customers to safe problem responses.</x:v>
+      </x:c>
+      <x:c r="F47" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G47" t="str">
+        <x:v>Mapped existing account page and account controller tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H47" t="str">
+        <x:v>No workbook-pass behavior error documented; signed-in account testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I47" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J47" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K47" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L47" t="str">
+        <x:v>Account pages -&gt; MalievApiClient account calls -&gt; AccountController -&gt; CustomerService/AuthService/CountryService/RegistryService clients</x:v>
+      </x:c>
+      <x:c r="M47" t="str">
+        <x:v>Account.razor; AccountProfile.razor; AccountController; AccountDtos</x:v>
+      </x:c>
+      <x:c r="N47" t="str">
+        <x:v>Account landing renders profile summary, unavailable panel, edit/change email actions, and protected navigation; AccountProfile renders validation-backed customer and company fields plus company search.</x:v>
+      </x:c>
+      <x:c r="O47" t="str">
+        <x:v>AccountController exposes session/profile/email/address/order/company-search endpoints and maps CustomerService/company update contracts into customer-safe DTOs and problem details.</x:v>
+      </x:c>
+      <x:c r="P47" t="str">
+        <x:v>Mapped tests: AccountPageSourceTests customer-account policy, profile image, invalid session redirect, editable profile form; AccountControllerBoundaryTests timeout, not-found, company create/link, tax-without-company rejection.</x:v>
+      </x:c>
+      <x:c r="Q47" t="str">
+        <x:v>Maliev.Web Client, Web BFF, CustomerService, AuthService, CountryService, RegistryService</x:v>
+      </x:c>
+      <x:c r="R47" t="str">
+        <x:v>CustomerAccountSessionDto, CustomerAccountProfileDto, profile update payloads, company create/update/link requests, email change state.</x:v>
+      </x:c>
+      <x:c r="S47" t="str">
+        <x:v>Needs live signed-in profile update, company search, email change, and invalid-session checks in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T47" t="str">
+        <x:v>Maliev.Web.Client/Pages/Account.razor:32,47,85,175,204; Maliev.Web.Client/Pages/AccountProfile.razor:547,555,576; Maliev.Web.Shared/Account/AccountDtos.cs:99,118,374; Maliev.Web.Bff/Controllers/AccountController.cs:24,41,145,197,424; Maliev.Web.Tests/AccountPageSourceTests.cs:13,101,136,151; Maliev.Web.Tests/AccountControllerBoundaryTests.cs:22,54,85,131</x:v>
+      </x:c>
+      <x:c r="U47" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" t="str">
+        <x:v>WEB-047</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>Account address picker, registry search, and static map</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>As a signed-in customer, I can create and maintain shipping or billing addresses using Google location search, Thai registry suggestions, and map previews.</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>The address page lists saved addresses with place labels, default badges, static map previews, and map links. The form uses UnifiedAddressSearch for Google Places, Google map pin, and Thai registry fallback, keeps driver notes after address fields, aligns default-address choice with address type, defaults Thailand when possible, locks Google-derived fields where appropriate, forwards Google and registry metadata to CustomerService, exposes Google browser configuration, country options, Thai-location search, and static map image rendering with customer-safe fallbacks when map providers fail.</x:v>
+      </x:c>
+      <x:c r="F48" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G48" t="str">
+        <x:v>Mapped existing account-address and address-controller tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H48" t="str">
+        <x:v>No workbook-pass behavior error documented; Google/registry browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I48" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J48" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K48" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L48" t="str">
+        <x:v>AccountAddresses.razor -&gt; UnifiedAddressSearch/GoogleAddressPicker JS -&gt; AddressController/AccountController -&gt; CountryService/RegistryService/CustomerService/static map service</x:v>
+      </x:c>
+      <x:c r="M48" t="str">
+        <x:v>AccountAddresses.razor; UnifiedAddressSearch.razor; GoogleAddressPicker.razor; AddressController; StaticMapService; GoogleAddressDtos</x:v>
+      </x:c>
+      <x:c r="N48" t="str">
+        <x:v>AccountAddresses renders saved address cards, map previews, Google/registry search, structured address fields, default-address checkbox, driver note, and edit/delete actions.</x:v>
+      </x:c>
+      <x:c r="O48" t="str">
+        <x:v>AddressController returns Google Maps config, static map image, countries, and Thai registry locations; AccountController forwards Google place, map pin, driver note, default, and country metadata to CustomerService.</x:v>
+      </x:c>
+      <x:c r="P48" t="str">
+        <x:v>Mapped tests: AccountAddressGoogleSourceTests picker, driver note, default alignment, metadata forwarding, Thai registry suggestions, map failure handling; AddressControllerBoundaryTests Google config, countries, and Thai locations.</x:v>
+      </x:c>
+      <x:c r="Q48" t="str">
+        <x:v>Maliev.Web Client, Web BFF, CustomerService, CountryService, RegistryService, Google Maps browser API, OpenStreetMap tile rendering</x:v>
+      </x:c>
+      <x:c r="R48" t="str">
+        <x:v>Customer address DTOs, GoogleAddressSelection, ThaiAddressRegistryLocationDto, static map URL/image bytes, address create/update/delete payloads.</x:v>
+      </x:c>
+      <x:c r="S48" t="str">
+        <x:v>Needs live Google Maps key, registry fallback, static-map image, and address CRUD checks in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T48" t="str">
+        <x:v>Maliev.Web.Client/Pages/AccountAddresses.razor:59,78,120,135,224,469,493,533; Maliev.Web.Client/Components/UnifiedAddressSearch.razor:150,179,207,253,264,300; Maliev.Web.Bff/Controllers/AddressController.cs:32,53,97,112; Maliev.Web.Bff/Services/StaticMapService.cs:9,27,121; Maliev.Web.Tests/AccountAddressGoogleSourceTests.cs:12,41,70,84,137,161; Maliev.Web.Tests/AddressControllerBoundaryTests.cs:21,37,73</x:v>
+      </x:c>
+      <x:c r="U48" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" t="str">
+        <x:v>WEB-048</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>Commerce catalog media and storefront mapping</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>As a shopper, I can browse published collections and products with media, categories, details, variants, and quote CTAs.</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>The shop page loads collections and products, shows an editorial marketplace layout, filters by collection, displays collection images, chooses a featured product, and renders a product grid. Product detail loads CommerceService product detail, displays a thumbnail strip and animated selected media, maps media and variants, shows request-quote pricing when price is zero, and links product or fallback quote CTAs to Make Studio. The BFF maps published collections/products from CommerceService, redirects collection images and product media through UploadService signed URLs, and uses short public-page timeouts.</x:v>
+      </x:c>
+      <x:c r="F49" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G49" t="str">
+        <x:v>Mapped existing commerce catalog, shop image, product media, and layout tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H49" t="str">
+        <x:v>No workbook-pass behavior error documented; shop/product browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I49" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J49" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K49" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L49" t="str">
+        <x:v>Shop/ProductDetail UI -&gt; MalievApiClient catalog calls -&gt; CatalogController -&gt; CommerceCatalogService -&gt; CommerceService and UploadService clients</x:v>
+      </x:c>
+      <x:c r="M49" t="str">
+        <x:v>Shop.razor; ProductGrid.razor; ProductDetail.razor; CatalogController; CommerceCatalogService; CatalogDtos</x:v>
+      </x:c>
+      <x:c r="N49" t="str">
+        <x:v>Shop renders collection rail/images, featured product, filtered grid, empty state, and product links; ProductDetail renders media gallery, variants, price/request-quote copy, add-to-cart, and quote actions.</x:v>
+      </x:c>
+      <x:c r="O49" t="str">
+        <x:v>CatalogController exposes collections, collection image redirect, product media redirect, products, and product detail endpoints; CommerceCatalogService maps published storefront data and signed media URLs.</x:v>
+      </x:c>
+      <x:c r="P49" t="str">
+        <x:v>Mapped tests: CommerceCatalogBoundaryTests products/collections/image/product detail; ShopCollectionImageSourceTests collection images; ProductDetailMediaSourceTests media gallery; HeroLayoutSourceTests shop layout, public timeout, live commerce quote CTAs.</x:v>
+      </x:c>
+      <x:c r="Q49" t="str">
+        <x:v>Maliev.Web Client, Web BFF, CommerceService, UploadService</x:v>
+      </x:c>
+      <x:c r="R49" t="str">
+        <x:v>ProductCollectionDto, ProductSummaryDto, ProductDetailDto, ProductMediaDto, ProductVariantDto, selected collection/media/cart item state.</x:v>
+      </x:c>
+      <x:c r="S49" t="str">
+        <x:v>Needs live catalog media redirects, product variant/cart behavior, and timeout handling in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T49" t="str">
+        <x:v>Maliev.Web.Client/Pages/Shop.razor:34,40,71,82,111,120; Maliev.Web.Client/Pages/ProductDetail.razor:19,25,31,74,92,108,121; Maliev.Web.Bff/Controllers/CatalogController.cs:19,35,53,71,87; Maliev.Web.Bff/Services/CommerceCatalogService.cs:17,39,66,80,85; Maliev.Web.Tests/CommerceCatalogBoundaryTests.cs:41,64,83,101; Maliev.Web.Tests/ShopCollectionImageSourceTests.cs:12; Maliev.Web.Tests/ProductDetailMediaSourceTests.cs:79,94; Maliev.Web.Tests/HeroLayoutSourceTests.cs:2807,2837,2868</x:v>
+      </x:c>
+      <x:c r="U49" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" t="str">
+        <x:v>WEB-049</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>Contact request autofill and boundary submission</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>As a visitor or signed-in customer, I can submit a contact request with support files and get a safe public reference.</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>The contact page loads account session/profile data when available, pre-fills name, email, phone, and company when safe, keeps empty fields for anonymous or unavailable profiles, accepts up to the configured number of support files, maps file metadata into contact attachments, submits ContactMessageRequest, displays a public reference and confirmation copy copy, clears attachments after successful submission, and returns customer-safe problem details when ContactService or CountryService is unavailable.</x:v>
+      </x:c>
+      <x:c r="F50" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G50" t="str">
+        <x:v>Mapped existing contact boundary, autofill, and Web BFF endpoint tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H50" t="str">
+        <x:v>No workbook-pass behavior error documented; contact form browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I50" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J50" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K50" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L50" t="str">
+        <x:v>StaticPage contact route -&gt; MalievApiClient account/contact calls -&gt; ContactController -&gt; ContactMessageService -&gt; ContactService and CountryService clients</x:v>
+      </x:c>
+      <x:c r="M50" t="str">
+        <x:v>StaticPage.razor contact route; ContactController; ContactMessageService; ContactServiceClient; ContactDtos</x:v>
+      </x:c>
+      <x:c r="N50" t="str">
+        <x:v>Contact page renders channel choices, map/contact context, profile autofill, upload guidance, file list, submit status, and confirmation reference.</x:v>
+      </x:c>
+      <x:c r="O50" t="str">
+        <x:v>ContactMessageService resolves default country, maps website contact fields and files to ContactService contract, formats public references, and raises backend-unavailable errors for downstream failures.</x:v>
+      </x:c>
+      <x:c r="P50" t="str">
+        <x:v>Mapped tests: ContactPageAutoFillTests session/profile autofill; ContactMessageBoundaryTests service contract, created response, timeout, CountryService unavailable; WebBffEndpointTests contact routing and problem details.</x:v>
+      </x:c>
+      <x:c r="Q50" t="str">
+        <x:v>Maliev.Web Client, Web BFF, ContactService, CountryService, CustomerService for profile autofill</x:v>
+      </x:c>
+      <x:c r="R50" t="str">
+        <x:v>ContactMessageRequest, ContactAttachmentDto list, ContactServiceCreateRequest, public contact reference/status.</x:v>
+      </x:c>
+      <x:c r="S50" t="str">
+        <x:v>Needs live contact submission with attachments and downstream failure checks in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T50" t="str">
+        <x:v>Maliev.Web.Client/Pages/StaticPage.razor:1285,1302,1314,1360,1372,1414,1479; Maliev.Web.Bff/Controllers/ContactController.cs:21; Maliev.Web.Bff/Services/ContactMessageService.cs:25,45; Maliev.Web.Bff/Clients/ContactServiceClient.cs:15,20,83; Maliev.Web.Shared/Contact/ContactDtos.cs:8,47,70; Maliev.Web.Tests/ContactPageAutoFillTests.cs:19; Maliev.Web.Tests/ContactMessageBoundaryTests.cs:19,68,105,131; Maliev.Web.Tests/WebBffEndpointTests.cs:442,464</x:v>
+      </x:c>
+      <x:c r="U50" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" t="str">
+        <x:v>WEB-050</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>Manufacturing reference data aggregation</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>As a quote visitor, I can load current manufacturing process, material, finish, process option, and lead-time choices before configuring a quote.</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>The Web BFF reference-data endpoint aggregates MaterialService processes, process materials, process finishes, material-specific compatible finishes, process configuration options, and PricingService lead times into QuoteReferenceDataDto. It loads per-process catalogs concurrently, preserves finish compatibility by material, returns process option DTOs, and exposes the result at web/v1/quote/reference-data for public quote components.</x:v>
+      </x:c>
+      <x:c r="F51" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G51" t="str">
+        <x:v>Mapped existing manufacturing catalog service and Web BFF endpoint tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H51" t="str">
+        <x:v>No workbook-pass behavior error documented; reference-data API testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I51" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J51" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K51" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L51" t="str">
+        <x:v>QuoteController reference-data endpoint -&gt; ManufacturingCatalogService -&gt; MaterialServiceClient and PricingServiceClient -&gt; QuoteReferenceDataDto</x:v>
+      </x:c>
+      <x:c r="M51" t="str">
+        <x:v>QuoteController; ManufacturingCatalogService; MaterialServiceClient; PricingServiceClient; QuoteDtos</x:v>
+      </x:c>
+      <x:c r="N51" t="str">
+        <x:v>Public quote components can call web/v1/quote/reference-data to populate process/material/finish/config/lead-time choices.</x:v>
+      </x:c>
+      <x:c r="O51" t="str">
+        <x:v>ManufacturingCatalogService loads processes, materials, finishes, material finish compatibility, config options, and lead times from downstream service clients.</x:v>
+      </x:c>
+      <x:c r="P51" t="str">
+        <x:v>Mapped tests: ManufacturingCatalogServiceTests.GetReferenceDataAsync_CombinesFinishesAndConfigOptionsByProcess; WebBffEndpointTests.GET_QuoteReferenceData_ReturnsBackendReferenceData.</x:v>
+      </x:c>
+      <x:c r="Q51" t="str">
+        <x:v>Maliev.Web BFF, MaterialService, PricingService</x:v>
+      </x:c>
+      <x:c r="R51" t="str">
+        <x:v>QuoteReferenceDataDto with process/material/finish/config option/lead-time collections; no durable Web mutation.</x:v>
+      </x:c>
+      <x:c r="S51" t="str">
+        <x:v>Needs live endpoint smoke against current MaterialService and PricingService in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T51" t="str">
+        <x:v>Maliev.Web.Bff/Controllers/QuoteController.cs:24,27; Maliev.Web.Bff/Services/ManufacturingCatalogService.cs:9,11,16,26,47,92; Maliev.Web.Bff/Clients/MaterialServiceClient.cs:23,28,33,38,43; Maliev.Web.Bff/Clients/PricingServiceClient.cs:15,28; Maliev.Web.Shared/Quotes/QuoteDtos.cs:119,130,190; Maliev.Web.Tests/ManufacturingCatalogServiceTests.cs:16; Maliev.Web.Tests/WebBffEndpointTests.cs:77</x:v>
+      </x:c>
+      <x:c r="U51" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" t="str">
+        <x:v>WEB-051</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>Public quote upload and Make Studio handoff</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>As a visitor with manufacturing files, I can upload CAD and context files from the public site and continue in Make Studio with a signed handoff.</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>The public quote dropzone sends selected files through resumable Web BFF upload initiation, PUT resume with Content-Range, completion, and signed handoff-token creation before redirecting to Make Studio. The BFF accepts CAD and supplemental context formats that match the Make Studio import contract, rejects unsupported extensions and oversized files, refuses handoff when files are missing, incomplete, or token length exceeds the Make Studio limit, and signs completed upload metadata without exposing raw filenames in the token body.</x:v>
+      </x:c>
+      <x:c r="F52" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G52" t="str">
+        <x:v>Mapped existing public quote upload/handoff endpoint and source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H52" t="str">
+        <x:v>No workbook-pass behavior error documented; browser upload and handoff testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I52" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J52" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K52" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L52" t="str">
+        <x:v>QuoteDropzone/maliev-quote-dropzone.js -&gt; QuoteController upload endpoints -&gt; QuoteUploadService -&gt; UploadServiceClient -&gt; QuoteUploadHandoffToken -&gt; Make Studio import URL</x:v>
+      </x:c>
+      <x:c r="M52" t="str">
+        <x:v>QuoteDropzone.razor; maliev-quote-dropzone.js; QuoteController; QuoteUploadService; QuoteUploadHandoffToken; WebQuoteUploadConstraints; QuoteDtos</x:v>
+      </x:c>
+      <x:c r="N52" t="str">
+        <x:v>Dropzone opens format picker, initiates resumable uploads, sends bytes with Content-Range, completes uploads, requests a handoff token, and redirects to Make Studio with the handoff parameter.</x:v>
+      </x:c>
+      <x:c r="O52" t="str">
+        <x:v>QuoteController exposes uploads/resumable, uploads/resumable/{uploadId}, complete, handoff-token, and analysis-status endpoints; QuoteUploadHandoffToken signs completed WebUploadHandoffFileDto metadata with configured production signing requirements.</x:v>
+      </x:c>
+      <x:c r="P52" t="str">
+        <x:v>Mapped tests: WebBffEndpointTests unsupported extension, CAD extension, supplemental attachment, file too large, signed handoff, supplemental handoff, too many files, incomplete upload; HeroLayoutSourceTests quote dropzone handoff.</x:v>
+      </x:c>
+      <x:c r="Q52" t="str">
+        <x:v>Maliev.Web Client, Web BFF, UploadService, Make Studio</x:v>
+      </x:c>
+      <x:c r="R52" t="str">
+        <x:v>Upload initiation session, uploaded bytes, WebUploadCompleteResponse, WebUploadHandoffTokenRequest/Response, signed handoff query parameter.</x:v>
+      </x:c>
+      <x:c r="S52" t="str">
+        <x:v>Needs live browser upload for CAD and supplemental files plus Make Studio import verification in the later testing loop.</x:v>
+      </x:c>
+      <x:c r="T52" t="str">
+        <x:v>Maliev.Web.Bff/wwwroot/js/maliev-quote-dropzone.js:146,178,200,209,228,261; Maliev.Web.Bff/Controllers/QuoteController.cs:66,114,154,170,196,211; Maliev.Web.Bff/Services/QuoteUploadService.cs:10,27,32,38,43,57; Maliev.Web.Bff/Security/QuoteUploadHandoffToken.cs:10,19,41; Maliev.Web.Shared/Quotes/WebQuoteUploadConstraints.cs:14,17,50,58; Maliev.Web.Shared/Quotes/QuoteDtos.cs:333,347,374; Maliev.Web.Tests/WebBffEndpointTests.cs:198,224,253,278,300,343,376,413; Maliev.Web.Tests/HeroLayoutSourceTests.cs:229</x:v>
+      </x:c>
+      <x:c r="U52" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R12f9e14f6e3f4763"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8777ea4bb9bf4eca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11585,7 +12341,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rce3dad237d094c0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bcd7a101d174f3b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16616,7 +17372,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde24a80e784248fd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6b98d7d1ed940c1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add current Intranet operations stories to tracker
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5fef2858502c424a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rc465ab75a3104e5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rac576a562f60464c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R695c329b5c744c01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8c03cfe1f6c54741"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R9577d248dba2406a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R506cb088a1f54e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R8936c652c7ba4a47"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>68</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>169</x:v>
+        <x:v>175</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -5636,7 +5636,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8777ea4bb9bf4eca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7011c78e3874576"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12338,10 +12338,400 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="70">
+      <x:c r="A70" t="str">
+        <x:v>INT-069</x:v>
+      </x:c>
+      <x:c r="B70" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C70" t="str">
+        <x:v>Project duplication, file copy, and analysis-state cloning</x:v>
+      </x:c>
+      <x:c r="D70" t="str">
+        <x:v>As a quoting employee, I can duplicate an existing project without losing part files, thumbnails, or analysis results.</x:v>
+      </x:c>
+      <x:c r="E70" t="str">
+        <x:v>Duplicating a project creates a copied project with copied part files, migrates or reuses upload artifacts through the upload service, preserves completed analysis and DFM status for copied parts, and cleans up the copied project/files if part creation fails.</x:v>
+      </x:c>
+      <x:c r="F70" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G70" t="str">
+        <x:v>Existing tests cover successful duplicate copy and cleanup on part-copy failure.</x:v>
+      </x:c>
+      <x:c r="H70" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I70" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J70" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K70" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L70" t="str">
+        <x:v>Project detail/list duplicate action -&gt; ProjectsController duplicate endpoint -&gt; ProjectService project/part APIs -&gt; UploadService migration/copy -&gt; FileAnalysisStatusService cloned analysis state</x:v>
+      </x:c>
+      <x:c r="M70" t="str">
+        <x:v>ProjectsController; ProjectDtos; UploadService migration DTOs; ProjectNew resume flow</x:v>
+      </x:c>
+      <x:c r="N70" t="str">
+        <x:v>Project duplication action creates a copied project and keeps part/attachment analysis data available for the resumed workspace.</x:v>
+      </x:c>
+      <x:c r="O70" t="str">
+        <x:v>ProjectsController Duplicate copies project/parts/files, migrates upload status, and removes created resources when downstream part creation fails.</x:v>
+      </x:c>
+      <x:c r="P70" t="str">
+        <x:v>ProjectsControllerTests.Duplicate_WhenSuccessful_CreatesCopiedProjectPartsFilesAndClonesAnalysisStatus; ProjectsControllerTests.Duplicate_WhenPartCreationFails_CleansUpCreatedProjectAndCopiedFiles; DtoSerializationTests.BffMigrateProjectResponseDto_ShouldUseCamelCaseWireShape_WithNestedStatus</x:v>
+      </x:c>
+      <x:c r="Q70" t="str">
+        <x:v>Intranet BFF, ProjectService, UploadService, FileAnalysisStatusService</x:v>
+      </x:c>
+      <x:c r="R70" t="str">
+        <x:v>Copied project records, copied part records, copied file references, migrated upload analysis status</x:v>
+      </x:c>
+      <x:c r="S70" t="str">
+        <x:v>Needs story-by-story browser retest for duplicate action, copied-part thumbnails, DFM status, and cleanup/error messaging.</x:v>
+      </x:c>
+      <x:c r="T70" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/ProjectsController.cs; Maliev.Intranet.Shared/Dtos/ProjectDtos.cs; Maliev.Intranet.Tests/Bff/Controllers/ProjectsControllerTests.cs:424,618; Maliev.Intranet.Tests/Shared/DtoSerializationTests.cs:210</x:v>
+      </x:c>
+      <x:c r="U70" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" t="str">
+        <x:v>INT-070</x:v>
+      </x:c>
+      <x:c r="B71" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C71" t="str">
+        <x:v>Project part routing and queue estimation</x:v>
+      </x:c>
+      <x:c r="D71" t="str">
+        <x:v>As an operations employee, I can see routing guidance for each project part before scheduling production.</x:v>
+      </x:c>
+      <x:c r="E71" t="str">
+        <x:v>The part routing endpoint validates process type, maps canonical process names, combines facility machine capacity with job-service queue data, returns queue and machine recommendations, and provides fallback machine fields when one downstream service is unavailable.</x:v>
+      </x:c>
+      <x:c r="F71" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G71" t="str">
+        <x:v>Existing controller tests cover missing/empty process validation, both-service success, JobService fallback, FacilityService fallback, CNC setup lead time, canonical CNC milling mapping, and unknown process fallback.</x:v>
+      </x:c>
+      <x:c r="H71" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I71" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J71" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K71" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L71" t="str">
+        <x:v>Project part planning UI -&gt; ProjectsController part-routing endpoint -&gt; JobService queue data -&gt; FacilityService machine category/capacity data -&gt; ProductionRoutingDto</x:v>
+      </x:c>
+      <x:c r="M71" t="str">
+        <x:v>ProjectsController; ProductionRoutingDtos; ProjectDetail planning tab</x:v>
+      </x:c>
+      <x:c r="N71" t="str">
+        <x:v>Planning views can request routing for a selected part/process and show queue/machine recommendations before production slots are created.</x:v>
+      </x:c>
+      <x:c r="O71" t="str">
+        <x:v>ProjectsController validates processType, handles CNC and additive mappings, tolerates partial downstream failures, and returns routing with queue days, machine category/name, setup days, and fallback availability.</x:v>
+      </x:c>
+      <x:c r="P71" t="str">
+        <x:v>ProjectsControllerTests.GetPartRouting_MissingProcessType_ReturnsBadRequest; GetPartRouting_BothServicesSucceed_ReturnsRoutingWithQueueAndMachine; GetPartRouting_JobServiceDown_ReturnsZeroQueueWithMachine; GetPartRouting_FacilityServiceDown_ReturnsFallbackMachineFields; GetPartRouting_CncProcess_UsesTwoSetupDays; GetPartRouting_ProjectServiceCncMilling_UsesCanonicalQueueAndCncMachineCategory; GetPartRouting_UnknownProcessType_ReturnsOkWithFallbackMachineFields</x:v>
+      </x:c>
+      <x:c r="Q71" t="str">
+        <x:v>Intranet BFF, ProjectService, JobService, FacilityService</x:v>
+      </x:c>
+      <x:c r="R71" t="str">
+        <x:v>Routing recommendations, queue estimates, machine assignment hints, setup-day estimates</x:v>
+      </x:c>
+      <x:c r="S71" t="str">
+        <x:v>Needs story-by-story UI retest for route-request loading state, partial-service fallback messaging, and queue/machine labels.</x:v>
+      </x:c>
+      <x:c r="T71" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/ProjectsController.cs; Maliev.Intranet.Shared/Dtos/ProductionRoutingDtos.cs; Maliev.Intranet.Tests/Bff/Controllers/ProjectsControllerTests.cs:979,999,1029,1049,1070,1083,1472</x:v>
+      </x:c>
+      <x:c r="U71" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" t="str">
+        <x:v>INT-071</x:v>
+      </x:c>
+      <x:c r="B72" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C72" t="str">
+        <x:v>Project production plan enrichment and planning holds</x:v>
+      </x:c>
+      <x:c r="D72" t="str">
+        <x:v>As an operations employee, I can open a project production plan that already contains enriched part thumbnails, human-readable manufacturing configuration, machine lanes, reserved slots, and planning holds.</x:v>
+      </x:c>
+      <x:c r="E72" t="str">
+        <x:v>The production plan endpoint enriches project parts with signed thumbnails and readable process/material details, builds a mixed-process schedule board with machine rows and reserved slots, and lets the project detail page focus a queued machine row or create half-hour planning holds from day view interactions.</x:v>
+      </x:c>
+      <x:c r="F72" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G72" t="str">
+        <x:v>Existing tests cover production plan enrichment, mixed-process schedule boards with reserved slots, planning queue focus, day-view planning hold creation, and planning endpoint calls.</x:v>
+      </x:c>
+      <x:c r="H72" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I72" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J72" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K72" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L72" t="str">
+        <x:v>ProjectDetail planning tab -&gt; ProjectsController production-plan/planning-hold endpoints -&gt; ProjectService parts -&gt; JobService schedule/holds -&gt; UploadService signed thumbnails</x:v>
+      </x:c>
+      <x:c r="M72" t="str">
+        <x:v>ProjectDetail.razor; ProjectsController; ProductionScheduleDtos; ProjectProductionPlanningDtos</x:v>
+      </x:c>
+      <x:c r="N72" t="str">
+        <x:v>Project detail planning tab renders a multi-machine schedule board, focuses machine rows/slots from queue buttons, and can place proposed planning holds into the board.</x:v>
+      </x:c>
+      <x:c r="O72" t="str">
+        <x:v>ProjectsController production plan resolves thumbnails and manufacturing text, returns schedule board data, and planning-hold endpoints require project read plus job write permission.</x:v>
+      </x:c>
+      <x:c r="P72" t="str">
+        <x:v>ProjectDetailPageTests.ProjectDetail_PlanningTab_RendersMultiMachineScheduleBoard; ProjectDetail_PlanningQueueButton_FocusesMachineRowAndSlotInBoard; ProjectDetail_PlanningDayView_DropsProposedSlotIntoHalfHourPlanningHold; ProjectDetail_PlanningActions_CallPlanningEndpoints; ProjectsControllerTests.GetProductionPlan_EnrichesThumbnailAndHumanizesConfiguration; ProjectsControllerTests.GetProductionPlan_IncludesMixedProcessScheduleBoardWithReservedSlots; PlanningHoldEndpoints_RequireProjectReadAndJobWritePermissions</x:v>
+      </x:c>
+      <x:c r="Q72" t="str">
+        <x:v>Intranet Client, Intranet BFF, ProjectService, JobService, UploadService</x:v>
+      </x:c>
+      <x:c r="R72" t="str">
+        <x:v>Production plan DTOs, planning hold records, signed thumbnails, schedule board rows/slots</x:v>
+      </x:c>
+      <x:c r="S72" t="str">
+        <x:v>Needs story-by-story browser retest for focus behavior, hold creation, board refresh, and permission failure handling.</x:v>
+      </x:c>
+      <x:c r="T72" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/ProjectDetail.razor; Maliev.Intranet.Bff/Controllers/ProjectsController.cs; Maliev.Intranet.Shared/Dtos/ProjectProductionPlanningDtos.cs; Maliev.Intranet.Shared/Dtos/ProductionScheduleDtos.cs; Maliev.Intranet.Tests/Client/Pages/ProjectDetailPageTests.cs:224,285,312,351; Maliev.Intranet.Tests/Bff/Controllers/ProjectsControllerTests.cs:57,1151,1257</x:v>
+      </x:c>
+      <x:c r="U72" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="A73" t="str">
+        <x:v>INT-072</x:v>
+      </x:c>
+      <x:c r="B73" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C73" t="str">
+        <x:v>Production schedule movement, scanning, material use, and release</x:v>
+      </x:c>
+      <x:c r="D73" t="str">
+        <x:v>As a manufacturing employee, I can operate the production schedule board from queue planning through job execution and quality release.</x:v>
+      </x:c>
+      <x:c r="E73" t="str">
+        <x:v>The production schedule board loads machine slots, supports search/process filters and timeline zoom, prevents invalid past moves, patches queued job or planning-hold movement with cascade options, opens job/hold detail drawers, scans a job ticket without advancing status, records exact inventory item consumption, saves editable job fields, requires explicit start/cancel actions, and releases completed jobs for shipping.</x:v>
+      </x:c>
+      <x:c r="F73" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G73" t="str">
+        <x:v>Existing client tests cover board rendering, zoom, queue movement, invalid move validation, job details, material-use posting, job-ticket scan, job edit patching, explicit start, cancellation reason, quality release, and planning-hold detail behavior.</x:v>
+      </x:c>
+      <x:c r="H73" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I73" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J73" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K73" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L73" t="str">
+        <x:v>ProductionSchedule page/board -&gt; api/v1/jobs schedule endpoints -&gt; JobService schedule/job detail/status -&gt; Inventory material consumption -&gt; Order lifecycle release</x:v>
+      </x:c>
+      <x:c r="M73" t="str">
+        <x:v>ProductionSchedule.razor; ProductionScheduleBoard.razor; ProductionScheduleDtos; JobDtos; OrderLifecycleDtos</x:v>
+      </x:c>
+      <x:c r="N73" t="str">
+        <x:v>Manufacturing schedule page renders machine lanes, job/hold slots, move panel, job ticket scan, material trace controls, job edit controls, explicit status actions, and quality release action.</x:v>
+      </x:c>
+      <x:c r="O73" t="str">
+        <x:v>Client patches schedule slots and planning holds, records inventory consumption, updates job details/status, and transitions completed order work to QualityReleased after explicit release.</x:v>
+      </x:c>
+      <x:c r="P73" t="str">
+        <x:v>ProductionSchedulePageTests.ProductionSchedule_RendersAllMachineBoardAndLockedSlots; TimelineZoomExpandsQueueFromWheelAndControls; MoveQueuedJob_PatchesScheduleAndRefreshesBoard; MovePastSlot_DisablesSaveAndShowsInlineValidation; ClickJobSlot_ShowsJobAndOrderDetails; RecordMaterialUse_PostsExactInventoryItemConsumption; ScanJobTicket_ResolvesJobWithoutAutoAdvancingStatus; SaveJobDetails_PatchesEditableProductionFields; StartJobAction_PatchesStatusAfterExplicitConfirmation; CancellingJobDetails_SendsCancellationReason; CompletedJobReleaseAction_TransitionsOrderToQualityReleased; ClickPlanningHold_ShowsHoldDetailsWithoutJobFetch</x:v>
+      </x:c>
+      <x:c r="Q73" t="str">
+        <x:v>Intranet Client, JobService, Inventory/Material service, OrderService</x:v>
+      </x:c>
+      <x:c r="R73" t="str">
+        <x:v>Schedule slots, planning holds, job status/detail updates, material trace entries, quality-release order status</x:v>
+      </x:c>
+      <x:c r="S73" t="str">
+        <x:v>Needs story-by-story browser retest for drag/drop, keyboard focus, scanner entry, material trace validation, and release confirmation.</x:v>
+      </x:c>
+      <x:c r="T73" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Manufacturing/ProductionSchedule.razor; Maliev.Intranet.Client/Components/Production/ProductionScheduleBoard.razor; Maliev.Intranet.Shared/Dtos/ProductionScheduleDtos.cs; Maliev.Intranet.Shared/Dtos/JobDtos.cs; Maliev.Intranet.Tests/Client/Pages/ProductionSchedulePageTests.cs:56,80,109,138,155,185,224,251,279,301,334,360</x:v>
+      </x:c>
+      <x:c r="U73" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="A74" t="str">
+        <x:v>INT-073</x:v>
+      </x:c>
+      <x:c r="B74" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C74" t="str">
+        <x:v>Realtime production and notification hubs</x:v>
+      </x:c>
+      <x:c r="D74" t="str">
+        <x:v>As an employee, I can receive realtime schedule and notification updates without refreshing the intranet.</x:v>
+      </x:c>
+      <x:c r="E74" t="str">
+        <x:v>Authorized SignalR hubs broadcast production job assignment and schedule-change events plus notification messages, while the notification bell shows alert-specific actions such as production planning required and read-state controls.</x:v>
+      </x:c>
+      <x:c r="F74" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G74" t="str">
+        <x:v>Existing hub tests cover production hub permissions and notification broadcasting.</x:v>
+      </x:c>
+      <x:c r="H74" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I74" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J74" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K74" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L74" t="str">
+        <x:v>SignalR clients -&gt; NotificationHub/ProductionHub -&gt; connected intranet pages/components -&gt; alert notification store/read receipts</x:v>
+      </x:c>
+      <x:c r="M74" t="str">
+        <x:v>NotificationHub; ProductionHub; NotificationBell.razor; NotificationDtos; AlertNotification</x:v>
+      </x:c>
+      <x:c r="N74" t="str">
+        <x:v>NotificationBell renders operational alert actions and read controls; production schedule listeners can react to job assignment and schedule-change hub messages.</x:v>
+      </x:c>
+      <x:c r="O74" t="str">
+        <x:v>ProductionHub requires job read permission and sends JobAssigned/ScheduleChanged events; NotificationHub broadcasts ReceiveNotification messages to connected clients.</x:v>
+      </x:c>
+      <x:c r="P74" t="str">
+        <x:v>ProductionHubTests.ProductionHub_ShouldRequireJobReadPermission; NotificationHubTests.SendNotification_ShouldSendToAll; NotificationControllerTests notification preference/template permissions</x:v>
+      </x:c>
+      <x:c r="Q74" t="str">
+        <x:v>Intranet BFF, SignalR, NotificationService, JobService</x:v>
+      </x:c>
+      <x:c r="R74" t="str">
+        <x:v>Realtime notification events, alert read state, production schedule event payloads</x:v>
+      </x:c>
+      <x:c r="S74" t="str">
+        <x:v>Needs story-by-story browser retest with a running SignalR host for connection, reconnect, duplicate-event handling, and read receipt updates.</x:v>
+      </x:c>
+      <x:c r="T74" t="str">
+        <x:v>Maliev.Intranet.Bff/Hubs/ProductionHub.cs; Maliev.Intranet.Bff/Hubs/NotificationHub.cs; Maliev.Intranet.Client/Components/NotificationBell.razor; Maliev.Intranet.Shared/Dtos/NotificationDtos.cs; Maliev.Intranet.Bff/Data/AlertNotification.cs; Maliev.Intranet.Tests/Bff/Hubs/ProductionHubTests.cs:10; Maliev.Intranet.Tests/Bff/Hubs/NotificationHubTests.cs:10; Maliev.Intranet.Tests/Bff/Controllers/NotificationControllerTests.cs:132</x:v>
+      </x:c>
+      <x:c r="U74" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="A75" t="str">
+        <x:v>INT-074</x:v>
+      </x:c>
+      <x:c r="B75" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C75" t="str">
+        <x:v>Dashboard widgets and resilient action items</x:v>
+      </x:c>
+      <x:c r="D75" t="str">
+        <x:v>As an employee, I can open a dashboard that summarizes operational work even when one downstream service is slow or unavailable.</x:v>
+      </x:c>
+      <x:c r="E75" t="str">
+        <x:v>The dashboard aggregates selected widgets for payments, orders, quotations, employees, invoices, leave, projects, and jobs, applies bounded downstream calls, returns safe defaults on non-critical failures, and produces action items for overdue production jobs, pending invoices/payments, leave approvals, quotations, and orders.</x:v>
+      </x:c>
+      <x:c r="F75" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G75" t="str">
+        <x:v>Existing BFF and client tests cover widget loading, safe defaults, action item generation, production-overdue action items, and loading-state behavior.</x:v>
+      </x:c>
+      <x:c r="H75" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I75" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J75" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K75" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L75" t="str">
+        <x:v>Dashboard page -&gt; DashboardController widgets/action-items -&gt; Order/Quotation/Payment/Employee/Invoice/Leave/Project/Job service clients</x:v>
+      </x:c>
+      <x:c r="M75" t="str">
+        <x:v>DashboardController; DashboardDtos; dashboard page tests</x:v>
+      </x:c>
+      <x:c r="N75" t="str">
+        <x:v>Dashboard renders quick actions before status panels, avoids fallback stats while loading, and shows widget/action-item content after BFF responses.</x:v>
+      </x:c>
+      <x:c r="O75" t="str">
+        <x:v>DashboardController uses widget selection and SafeDashboardValueAsync/SafeCount boundaries so one service failure does not hide the rest of the daily operations queue.</x:v>
+      </x:c>
+      <x:c r="P75" t="str">
+        <x:v>DashboardControllerTests.Get_*; DashboardControllerTests.GetActionItems_WithOverdueProductionJobs_ShouldReturnProductionActionItem; Phase3DashboardTests.Dashboard_ShouldShowQuickActionsBeforeDashboardStatusPanels; Dashboard_ShouldNotRenderFallbackStats_WhileDashboardRequestIsLoading</x:v>
+      </x:c>
+      <x:c r="Q75" t="str">
+        <x:v>Intranet Client, Intranet BFF, OrderService, QuotationService, PaymentService, EmployeeService, InvoiceService, LeaveService, ProjectService, JobService</x:v>
+      </x:c>
+      <x:c r="R75" t="str">
+        <x:v>Dashboard view model, action item DTOs, widget response data</x:v>
+      </x:c>
+      <x:c r="S75" t="str">
+        <x:v>Needs story-by-story browser retest for widget filters, slow-service defaults, and action item navigation targets.</x:v>
+      </x:c>
+      <x:c r="T75" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/DashboardController.cs; Maliev.Intranet.Shared/Dtos/DashboardDtos.cs; Maliev.Intranet.Tests/Bff/Controllers/DashboardControllerTests.cs:43,154; Maliev.Intranet.Tests/Client/Pages/Phase3DashboardTests.cs:91,107</x:v>
+      </x:c>
+      <x:c r="U75" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5bcd7a101d174f3b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7be605eb7d1248a3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17372,7 +17762,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6b98d7d1ed940c1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra87ad5bec4884aa0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add current Intranet viewer stories to tracker
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R8c03cfe1f6c54741"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R9577d248dba2406a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R506cb088a1f54e58"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R8936c652c7ba4a47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rf3d1835e7b3b4ccb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R233c081352d34568"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R6e6cf674d3ef46e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rec27daa8ec674be6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>74</x:v>
+        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>175</x:v>
+        <x:v>179</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -5636,7 +5636,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf7011c78e3874576"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R10150435dc3f4eea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12728,10 +12728,270 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="76">
+      <x:c r="A76" t="str">
+        <x:v>INT-075</x:v>
+      </x:c>
+      <x:c r="B76" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C76" t="str">
+        <x:v>Three.js model viewer and analysis toolbar</x:v>
+      </x:c>
+      <x:c r="D76" t="str">
+        <x:v>As a quoting or manufacturing employee, I can inspect a part in the current 3D viewer with CAD-focused camera, render, section, and analysis controls.</x:v>
+      </x:c>
+      <x:c r="E76" t="str">
+        <x:v>The ModelViewer imports the self-hosted Three.js viewer module, initializes it with model URL, extension, material/configuration context, dark-mode state, viewer settings, and local geometry callbacks, then exposes solid/wireframe/transparent render modes, perspective/orthographic camera projection, camera presets, grid, edges, bounding box, section plane, rotation/reset, body picking, flipped-triangle, measure, and thickness tools. The viewer disposes the module and canvas resources when the component is disposed.</x:v>
+      </x:c>
+      <x:c r="F76" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G76" t="str">
+        <x:v>Existing focused source/component/viewer tests cover model viewer rendering defaults, section panel controls, analysis tools, local DFM callback readiness, and the Three.js import map path.</x:v>
+      </x:c>
+      <x:c r="H76" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I76" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J76" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K76" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L76" t="str">
+        <x:v>ModelViewer.razor toolbar/state -&gt; JS module import ./js/part-viewer-three.js -&gt; self-hosted Three.js import map -&gt; browser viewer canvas and DotNet callbacks</x:v>
+      </x:c>
+      <x:c r="M76" t="str">
+        <x:v>ModelViewer.razor; wwwroot/index.html; wwwroot/js/part-viewer-three.js</x:v>
+      </x:c>
+      <x:c r="N76" t="str">
+        <x:v>ModelViewer renders toolbar buttons for render mode, projection, camera, grid, edges, bounds, section, reset, rotate, flipped-triangle, measure, and thickness analysis.</x:v>
+      </x:c>
+      <x:c r="O76" t="str">
+        <x:v>part-viewer-three.js normalizes viewer settings, initializes perspective/orthographic cameras, toggles grid/edges/bounds, applies section planes, records measurement callbacks, and disposes canvas-scoped state.</x:v>
+      </x:c>
+      <x:c r="P76" t="str">
+        <x:v>ModelViewerRenderingSourceTests; ModelViewerSectionToolTests; Viewer/part-viewer-analysis-tools.test.mjs; Viewer/part-viewer-turning-axis.test.mjs</x:v>
+      </x:c>
+      <x:c r="Q76" t="str">
+        <x:v>Intranet Client, browser Three.js runtime, local geometry/DFM runtime</x:v>
+      </x:c>
+      <x:c r="R76" t="str">
+        <x:v>Canvas viewer state, viewer settings, analysis tool state, measurement callback values, body/section/overlay state</x:v>
+      </x:c>
+      <x:c r="S76" t="str">
+        <x:v>Needs story-by-story browser retest for STL/STEP/GLB files, camera modes, render modes, section plane, measurement, thickness, body selection, dark mode, and disposal/reopen behavior.</x:v>
+      </x:c>
+      <x:c r="T76" t="str">
+        <x:v>Maliev.Intranet.Client/Components/ModelViewer.razor:217,644,661,739,888,906,924,1020,1071,1089,1103,1192,1328; Maliev.Intranet.Client/wwwroot/index.html:111; Maliev.Intranet.Client/wwwroot/js/part-viewer-three.js:6,871,886,1002,1113,1494,1575,1690; Maliev.Intranet.Tests/Client/Components/ModelViewerSectionToolTests.cs:28,49; Maliev.Intranet.Tests/Client/Components/ModelViewerRenderingSourceTests.cs:60,463</x:v>
+      </x:c>
+      <x:c r="U76" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="77">
+      <x:c r="A77" t="str">
+        <x:v>INT-076</x:v>
+      </x:c>
+      <x:c r="B77" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C77" t="str">
+        <x:v>Per-part viewer settings persistence</x:v>
+      </x:c>
+      <x:c r="D77" t="str">
+        <x:v>As a quoting employee, I can keep different viewer preferences per project part and recover them when the draft resumes.</x:v>
+      </x:c>
+      <x:c r="E77" t="str">
+        <x:v>Viewer settings round-trip with each part draft, including render mode, staged render fields, camera projection, edges, grid, bounding box, section enabled/axis/offset/inversion, and transition timing. ModelViewer applies incoming settings once per key, captures changes from toolbar interactions, emits ViewerSettingsChanged, and avoids saving temporary grid changes caused only by section-tool ownership.</x:v>
+      </x:c>
+      <x:c r="F77" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G77" t="str">
+        <x:v>Existing tests cover per-part viewer settings roundtrip, explicit disabled grid preservation, render-mode transition DTO fields, viewer key inclusion, and temporary grid-owner behavior.</x:v>
+      </x:c>
+      <x:c r="H77" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I77" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J77" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K77" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L77" t="str">
+        <x:v>ModelViewer settings capture/apply -&gt; PartViewModel ToDraftPartState/FromDraftPartState -&gt; ProjectDraftDtos PartViewerSettings -&gt; Project New autosave/resume storage</x:v>
+      </x:c>
+      <x:c r="M77" t="str">
+        <x:v>ModelViewer.razor; ProjectDraftDtos.cs; PartViewModelViewerSettingsTests.cs</x:v>
+      </x:c>
+      <x:c r="N77" t="str">
+        <x:v>Toolbar changes update viewer settings; resumed parts restore render mode, projection, overlays, and section settings for that part.</x:v>
+      </x:c>
+      <x:c r="O77" t="str">
+        <x:v>ProjectDraftDtos defines PartViewerSettings and RenderModeTransitionSettings; ModelViewer CaptureViewerSettings/GetViewerSettingsKey/NotifyViewerSettingsChanged keep UI and draft state aligned.</x:v>
+      </x:c>
+      <x:c r="P77" t="str">
+        <x:v>PartViewModelViewerSettingsTests.ToDraftPartState_RoundTripsViewerSettings_PerPart; ToDraftPartState_WhenGridFloorExplicitlyDisabled_PreservesDisabledSetting; ModelViewerRenderingSourceTests.PartViewerSettings_DtoIncludesRenderModeTransitionFields; ModelViewer_GetViewerSettingsKey_IncludesNewFields; ModelViewerSectionToolTests.ModelViewer_TemporaryGridOwner_DoesNotPersistViewerSettings; ModelViewer_TemporaryGridOwner_DoesNotHideUserEnabledGrid</x:v>
+      </x:c>
+      <x:c r="Q77" t="str">
+        <x:v>Intranet Client, Project draft DTO/storage boundary</x:v>
+      </x:c>
+      <x:c r="R77" t="str">
+        <x:v>Per-part viewer preferences, section plane settings, render transition settings, project draft state</x:v>
+      </x:c>
+      <x:c r="S77" t="str">
+        <x:v>Needs story-by-story browser retest for changing settings on two parts, saving draft, reloading the project, and confirming settings remain isolated per part.</x:v>
+      </x:c>
+      <x:c r="T77" t="str">
+        <x:v>Maliev.Intranet.Client/Components/ModelViewer.razor:217,318,321,343,383,391,739,761,903,921,1026,1036,1052; Maliev.Intranet.Shared/Dtos/ProjectDraftDtos.cs:283,289,292,295,298,301,307,323,335,354; Maliev.Intranet.Tests/Client/Components/PartViewModelViewerSettingsTests.cs:10,57; Maliev.Intranet.Tests/Client/Components/ModelViewerRenderingSourceTests.cs:219,243; Maliev.Intranet.Tests/Client/Components/ModelViewerSectionToolTests.cs:64,94</x:v>
+      </x:c>
+      <x:c r="U77" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="78">
+      <x:c r="A78" t="str">
+        <x:v>INT-077</x:v>
+      </x:c>
+      <x:c r="B78" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C78" t="str">
+        <x:v>Browser-local DFM sync and overlay acknowledgement</x:v>
+      </x:c>
+      <x:c r="D78" t="str">
+        <x:v>As a quoting employee, I can see browser-local DFM progress, failure/unavailable state, issue overlays, and acknowledgement state without waiting for server analysis to overwrite useful local results.</x:v>
+      </x:c>
+      <x:c r="E78" t="str">
+        <x:v>BrowserDfmReportSync treats browser DFM as primary during a grace period, resolves shared DFM reports for the selected process, clears timeout/running/terminal fields when an accepted report arrives, keeps terminal state process-scoped, and maps running/completed/unavailable/error chips in the part detail card. DfmChecksTab shows pending, failed, and passed intrinsic checks; DfmOverlayPanel toggles server overlay URLs or local face-index overlays, supports single-select overlay state, acknowledges issues, and resets overlay state when the active part changes.</x:v>
+      </x:c>
+      <x:c r="F78" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G78" t="str">
+        <x:v>Existing tests cover local DFM report sync, local chips, DFM tab pass/fail/pending behavior, server/local overlay toggles, local face-index viewer overlays, and overlay disposal.</x:v>
+      </x:c>
+      <x:c r="H78" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I78" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J78" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K78" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L78" t="str">
+        <x:v>ModelViewer local DFM callbacks -&gt; BrowserDfmReportSync -&gt; PartViewModel process-specific DFM report state -&gt; DfmChecksTab/DfmOverlayPanel -&gt; part-viewer-three local overlay mesh</x:v>
+      </x:c>
+      <x:c r="M78" t="str">
+        <x:v>BrowserDfmReportSync.cs; DfmChecksTab.razor; DfmOverlayPanel.razor; ModelViewer.razor; part-viewer-three.js</x:v>
+      </x:c>
+      <x:c r="N78" t="str">
+        <x:v>DFM tab and overlay panel display local/server analysis state, issue rows, local face-index toggle controls, acknowledgement controls, and unavailable/error messages.</x:v>
+      </x:c>
+      <x:c r="O78" t="str">
+        <x:v>BrowserDfmReportSync handles process-aware local runtime state; DfmOverlayPanel invokes local or server overlay toggles; viewer JS builds and clears local overlay meshes from face indices.</x:v>
+      </x:c>
+      <x:c r="P78" t="str">
+        <x:v>BrowserDfmReportSyncTests; PartDetailCardLocalDfmTests; DfmChecksTabTests; DfmOverlayPanelLocalOverlayTests; DfmOverlayPanelSourceTests; Viewer/part-viewer-local-dfm-overlay.test.mjs</x:v>
+      </x:c>
+      <x:c r="Q78" t="str">
+        <x:v>Intranet Client, browser DFM runtime, GeometryService analysis status, project draft DFM DTOs</x:v>
+      </x:c>
+      <x:c r="R78" t="str">
+        <x:v>DFM report state, local runtime fields, issue overlay selection, acknowledgement state, local overlay mesh state</x:v>
+      </x:c>
+      <x:c r="S78" t="str">
+        <x:v>Needs story-by-story browser retest for local runtime start/complete/unavailable/error, process switching, overlay toggling, acknowledgement, and server status refresh interactions.</x:v>
+      </x:c>
+      <x:c r="T78" t="str">
+        <x:v>Maliev.Intranet.Client/Components/Project/BrowserDfmReportSync.cs:3,16,24,32,51,68,83,95,106; Maliev.Intranet.Client/Components/Project/DfmChecksTab.razor:30,268; Maliev.Intranet.Client/Components/Project/DfmOverlayPanel.razor:19,41,71,96,205,240,265; Maliev.Intranet.Client/Components/ModelViewer.razor:1089,1103,1192,1223; Maliev.Intranet.Tests/Client/Components/BrowserDfmReportSyncTests.cs:8; Maliev.Intranet.Tests/Client/Components/PartDetailCardLocalDfmTests.cs:44,68,83,97,114,129,157; Maliev.Intranet.Tests/Viewer/part-viewer-local-dfm-overlay.test.mjs:115,145,160,179,193</x:v>
+      </x:c>
+      <x:c r="U78" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="79">
+      <x:c r="A79" t="str">
+        <x:v>INT-078</x:v>
+      </x:c>
+      <x:c r="B79" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C79" t="str">
+        <x:v>Client thumbnail generation and fallback refresh</x:v>
+      </x:c>
+      <x:c r="D79" t="str">
+        <x:v>As a quoting employee, I can see part thumbnails generated locally when available and refreshed when another viewer finishes generation.</x:v>
+      </x:c>
+      <x:c r="E79" t="str">
+        <x:v>ThumbnailImage shows pending, fallback, failed, or image states, reads cached thumbnail sets by storage path and version, subscribes to thumbnail progress events, refreshes from cache when another caller completes generation for the same storage path, ignores completion events for other storage paths, and requests server fallback when local thumbnail generation returns no usable result or fails. The BFF can sign large thumbnail URLs for project parts that expose large thumbnail storage paths.</x:v>
+      </x:c>
+      <x:c r="F79" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G79" t="str">
+        <x:v>Existing tests cover thumbnail pending/image/fallback states, cache refresh from another caller, cross-path event isolation, Project New local thumbnail source behavior, and BFF large-thumbnail signed URL/not-found behavior.</x:v>
+      </x:c>
+      <x:c r="H79" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I79" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J79" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K79" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L79" t="str">
+        <x:v>Project part thumbnail component -&gt; ThumbnailGenerationService cache/progress/local generation -&gt; BFF large-thumbnail URL endpoint -&gt; UploadService signed URL</x:v>
+      </x:c>
+      <x:c r="M79" t="str">
+        <x:v>ThumbnailImage.razor; ThumbnailGenerationService.cs; ProjectsController.GetPartLargeThumbnailUrl; ProjectNewLocalThumbnailSourceTests</x:v>
+      </x:c>
+      <x:c r="N79" t="str">
+        <x:v>Part cards and project pages show a pending thumbnail shell, cached thumbnail image, fallback spinner, or failed state according to generation/cache status.</x:v>
+      </x:c>
+      <x:c r="O79" t="str">
+        <x:v>ThumbnailGenerationService caches thumbnail sets, notifies subscribers by storage path/version, retries local generation when the runtime becomes ready, requests fallback when local output is empty or failed, and the BFF signs large thumbnail paths.</x:v>
+      </x:c>
+      <x:c r="P79" t="str">
+        <x:v>ThumbnailImageTests.ThumbnailImage_ShowsSkeleton_WhenNotCached; ThumbnailImage_ShowsImage_WhenCached; ThumbnailImage_RefreshesFromCache_WhenAnotherCallerCompletesGeneration; ThumbnailImage_IgnoresCompletionEvents_ForOtherStoragePaths; ThumbnailImage_ShowsSpinner_WhenFallbackStage; ProjectNewLocalThumbnailSourceTests; ProjectsControllerTests.GetPartLargeThumbnailUrl_WhenPartHasLargeThumbnail_ShouldReturnSignedUrl; GetPartLargeThumbnailUrl_WhenPartHasNoLargeThumbnail_ShouldReturnNotFound</x:v>
+      </x:c>
+      <x:c r="Q79" t="str">
+        <x:v>Intranet Client, browser thumbnail runtime, Intranet BFF, UploadService</x:v>
+      </x:c>
+      <x:c r="R79" t="str">
+        <x:v>Thumbnail cache entries, thumbnail progress events, signed thumbnail URLs, fallback generation request state</x:v>
+      </x:c>
+      <x:c r="S79" t="str">
+        <x:v>Needs story-by-story browser retest for initial pending state, local generation success, fallback path, cross-part event isolation, and large-thumbnail popout.</x:v>
+      </x:c>
+      <x:c r="T79" t="str">
+        <x:v>Maliev.Intranet.Client/Components/Project/ThumbnailImage.razor:4,8,14,20,26,79,107,131; Maliev.Intranet.Client/Services/ThumbnailGenerationService.cs:10,37,46,55,105,142,165; Maliev.Intranet.Tests/Client/Components/ThumbnailImageTests.cs:16,31,52,87,112; Maliev.Intranet.Tests/Client/Pages/ProjectNewLocalThumbnailSourceTests.cs:9; Maliev.Intranet.Tests/Bff/Controllers/ProjectsControllerTests.cs:244,296</x:v>
+      </x:c>
+      <x:c r="U79" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7be605eb7d1248a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R86f74ef33feb4e8f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17762,7 +18022,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra87ad5bec4884aa0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac2041bbc6d14f5b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add current Web public content stories to tracker
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R53d2b8ef022b4db2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R34031c61cede44d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R841c8ac9df5841f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Re137012126d045de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R6f6e975f88e64cca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rf04d5624c0044af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Ref53b53aa10244b8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rd9f2e5035845441a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -505,7 +505,7 @@
         <x:v>Maliev.Web</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>56</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>184</x:v>
+        <x:v>189</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4278,10 +4278,335 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>WEB-057</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>Responsive public layout, header actions, and assistant widget</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>As a visitor, I can navigate the public site on desktop or mobile and reach Make Studio, cart, account, and the website assistant without layout jumps.</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>The main layout renders primary navigation, theme and language controls, cart/account Mud icon buttons, cart badge only when items exist, Make Studio links, a mobile menu with close-on-navigation behavior, footer contact/social/legal links, the LINE contact block, and the CustomerChatbot widget. CSS keeps the sticky header stable across breakpoints and gives mobile navigation its own open state rather than resizing the desktop header.</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>Mapped current layout/header/mobile source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>No workbook-pass behavior error documented; responsive browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I58" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J58" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K58" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L58" t="str">
+        <x:v>MainLayout.razor -&gt; CartState/PreferenceService state -&gt; app.css responsive navigation -&gt; CustomerChatbot component</x:v>
+      </x:c>
+      <x:c r="M58" t="str">
+        <x:v>MainLayout.razor; app.css; CartState.cs; CustomerChatbot</x:v>
+      </x:c>
+      <x:c r="N58" t="str">
+        <x:v>Layout exposes desktop nav, mobile nav, cart badge, account button, Make Studio links, theme/language controls, footer links, LINE contact, and CustomerChatbot.</x:v>
+      </x:c>
+      <x:c r="O58" t="str">
+        <x:v>The layout subscribes to cart/preference changes, initializes cart and preferences, toggles mobile nav, and CSS applies nav-icon/mobile-nav breakpoints and sticky-header sizing.</x:v>
+      </x:c>
+      <x:c r="P58" t="str">
+        <x:v>Mapped tests: HeaderUsesMudIconButtonsForCartAndAccount, HeaderBleedsLandingHeroBackdropAtPageTop, PublicLayoutIncludesCustomerChatbotWidget, MobileNavigationDoesNotGrowStickyHeader.</x:v>
+      </x:c>
+      <x:c r="Q58" t="str">
+        <x:v>Maliev.Web Client, browser layout/CSS, cart preference state</x:v>
+      </x:c>
+      <x:c r="R58" t="str">
+        <x:v>Cart count, mobile-nav open state, theme/culture state, Make Studio URL, assistant widget session state.</x:v>
+      </x:c>
+      <x:c r="S58" t="str">
+        <x:v>Needs responsive browser retest for desktop, tablet, mobile menu open/close, cart badge, account link, Make Studio link, chatbot presence, and sticky-header height.</x:v>
+      </x:c>
+      <x:c r="T58" t="str">
+        <x:v>Maliev.Web.Client/Layout/MainLayout.razor:18,23,28,35,44,53,60,62,70,77,82,128,183,279,285,294,297,341,346,378; Maliev.Web.Bff/wwwroot/app.css:272,322,373,393,663,10167,10428,10432,10451,10475,10498,10858; Maliev.Web.Tests/HeroLayoutSourceTests.cs:1639,1687,1712,2785</x:v>
+      </x:c>
+      <x:c r="U58" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>WEB-058</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>Services directory and service-detail readiness pages</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>As a manufacturing buyer, I can browse service routes and open a detail page that tells me which files, materials, checks, and ordering steps are needed before requesting work.</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>The services page lists current SiteContent services and links each card to /services/{slug}. Each service detail page resolves the slug, loads a service-specific detail profile, renders supported files, material routes, manufacturability gates, ordering steps, localized copy, proof imagery, and a disabled quote dropzone with the current readiness message so public visitors are guided toward Make Studio when quote intake is live.</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>Mapped current services source tests and SiteContent service profiles; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>No workbook-pass behavior error documented; service-route browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L59" t="str">
+        <x:v>Services.razor listing -&gt; ServicePage.razor detail route -&gt; SiteContent service/detail profiles -&gt; QuoteDropzone disabled-readiness copy</x:v>
+      </x:c>
+      <x:c r="M59" t="str">
+        <x:v>Services.razor; ServicePage.razor; SiteContent.cs; QuoteDropzone</x:v>
+      </x:c>
+      <x:c r="N59" t="str">
+        <x:v>Services renders service cards and material comparison CTA; ServicePage renders slug-specific files, material routes, gates, ordering steps, and readiness dropzone state.</x:v>
+      </x:c>
+      <x:c r="O59" t="str">
+        <x:v>SiteContent.GetService and GetServiceDetail resolve service slugs to current detail profiles or a default profile; QuoteDisabledAction supplies localized disabled quote action copy.</x:v>
+      </x:c>
+      <x:c r="P59" t="str">
+        <x:v>Mapped tests: ServicesUseRealRoutesAndDisabledQuoteActions and service quote-dropzone localization coverage.</x:v>
+      </x:c>
+      <x:c r="Q59" t="str">
+        <x:v>Maliev.Web Client and static SiteContent boundary</x:v>
+      </x:c>
+      <x:c r="R59" t="str">
+        <x:v>Service slug, localized ServicePageContent, ServiceDetailProfile, QuoteDisabledAction, customer-facing route state.</x:v>
+      </x:c>
+      <x:c r="S59" t="str">
+        <x:v>Needs browser retest for every service card route, missing slug fallback, localized detail copy, disabled dropzone state, and Make Studio CTA path.</x:v>
+      </x:c>
+      <x:c r="T59" t="str">
+        <x:v>Maliev.Web.Client/Pages/Services.razor:1,19,25; Maliev.Web.Client/Pages/ServicePage.razor:1,31,51,75,94,110,136,146,147,150; Maliev.Web.Client/Content/SiteContent.cs:16,1558,1628,1693,1734,1775,1816,1857,2258,2263,2280,3149; Maliev.Web.Tests/HeroLayoutSourceTests.cs:2238; Maliev.Web.Tests/LocalizationTests.cs:131</x:v>
+      </x:c>
+      <x:c r="U59" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>WEB-059</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>Static company, policy, account-quote, and contact routes</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>As a visitor or customer, I can open the public company, policy, support, and account-quote routes and see the correct page content and contact paths.</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>StaticPage declares current routes for about, contact, FAQ, shipping and returns, privacy, terms, cookie policy, refund policy, warranty policy, industries, account quotes, blog, and case-study paths. It renders page metadata, localized content, primary and secondary actions, logo-mark contact CTAs, contact business panels, maps, LINE/social channels, profile-aware contact forms, file-upload state, status messages, and map dialogs.</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>Mapped current static-page and contact-source tests; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>No workbook-pass behavior error documented; public route smoke testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L60" t="str">
+        <x:v>StaticPage.razor route switch -&gt; SiteContent static content -&gt; contact form/profile/upload helpers -&gt; ContactController boundary from existing contact rows</x:v>
+      </x:c>
+      <x:c r="M60" t="str">
+        <x:v>StaticPage.razor; SiteContent.cs; StaticPage.razor.css</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>StaticPage renders public information routes, policy routes, account quote placeholder route, contact business panels, map/dialog UI, profile-aware contact form, support file list, and status feedback.</x:v>
+      </x:c>
+      <x:c r="O60" t="str">
+        <x:v>The route declarations map one component to multiple public paths, while contact submission and support-file behavior reuse the Web BFF contact boundary tracked separately.</x:v>
+      </x:c>
+      <x:c r="P60" t="str">
+        <x:v>Mapped tests: StaticPagesCoverCustomerRoutesAndContactBoundary, StaticPageSecondaryContactCtaUsesLogoMark, ContactPageShowsBusinessChannelsMapAndHours, and contact autofill/boundary tests.</x:v>
+      </x:c>
+      <x:c r="Q60" t="str">
+        <x:v>Maliev.Web Client, Web BFF contact boundary, CustomerService profile lookup, static content assets</x:v>
+      </x:c>
+      <x:c r="R60" t="str">
+        <x:v>Route path, localized static content, contact form DTO, uploaded support file states, map dialog state, profile autofill state.</x:v>
+      </x:c>
+      <x:c r="S60" t="str">
+        <x:v>Needs browser route sweep for all declared static paths, contact map dialog, secondary logo CTA, contact profile autofill, support uploads, and policy navigation.</x:v>
+      </x:c>
+      <x:c r="T60" t="str">
+        <x:v>Maliev.Web.Client/Pages/StaticPage.razor:1,2,3,4,5,6,7,8,9,10,15,22,39,277,281,305,309,373,396,441,457,469,484,505,528,594,607; Maliev.Web.Tests/HeroLayoutSourceTests.cs:1421,2311,2425; Maliev.Web.Tests/ContactPageAutoFillTests.cs:19; Maliev.Web.Tests/ContactMessageBoundaryTests.cs:19</x:v>
+      </x:c>
+      <x:c r="U60" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>WEB-060</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>Journal and case-study discovery and detail pages</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>As a visitor researching manufacturing decisions, I can browse journal notes and case studies, filter or search them, and open detail pages with useful calls to action.</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>StaticPage renders the blog index with search, category filters, result count, pagination, image cards, and detail pages with sections, checklist styling, images, sidebar actions, practical-note PDF download, and Make Studio CTAs. The same component renders case-study index cards and case-study detail pages with localized sections, evidence images, results, and Start a similar quote action.</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>Mapped current journal/case-study source tests and SiteContent article structures; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>No workbook-pass behavior error documented; blog/case-study browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L61" t="str">
+        <x:v>StaticPage blog/case-study routes -&gt; SiteContent BlogPosts/CaseStudies -&gt; blog filtering/pagination/detail helpers -&gt; BlogController PDF endpoint for downloads</x:v>
+      </x:c>
+      <x:c r="M61" t="str">
+        <x:v>StaticPage.razor; SiteContent.cs; BlogController; BlogEbookPdfService</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>Blog index renders search, category filters, pagination, cards, and result counts; blog detail renders article sections, checklist styling, image content, sidebar CTAs, and PDF download; case-study pages render index/detail content and quote CTA.</x:v>
+      </x:c>
+      <x:c r="O61" t="str">
+        <x:v>SiteContent supplies BlogPostContent, CaseStudyContent, ArticleSectionContent, article images, category matching, and PDF filename/content data used by StaticPage and BlogController.</x:v>
+      </x:c>
+      <x:c r="P61" t="str">
+        <x:v>Mapped tests: JournalAndCaseStudyCardsHaveRealDetailPages, BlogPosts_HaveInformativeContentAndUniqueImages, BlogEbookPdfIsRenderedByPdfServiceNotWebBff, GET_BlogEbookPdf_ReturnsGeneratedPdfDownload.</x:v>
+      </x:c>
+      <x:c r="Q61" t="str">
+        <x:v>Maliev.Web Client, static SiteContent, Web BFF BlogController, PdfService</x:v>
+      </x:c>
+      <x:c r="R61" t="str">
+        <x:v>Blog query, category filters, page number, selected post slug, case-study slug, article sections/images, PDF request state.</x:v>
+      </x:c>
+      <x:c r="S61" t="str">
+        <x:v>Needs browser retest for blog search/filter/pagination, blog detail images and download, case-study index/detail routes, missing slugs, and Make Studio CTA links.</x:v>
+      </x:c>
+      <x:c r="T61" t="str">
+        <x:v>Maliev.Web.Client/Pages/StaticPage.razor:11,12,13,14,59,87,95,117,130,133,148,167,210,214,224,257,258,619,620,639,646,654; Maliev.Web.Client/Content/SiteContent.cs:1903,1934,2211,2219,2234,3167,3177,3186,3192; Maliev.Web.Bff/Controllers/BlogController.cs:31; Maliev.Web.Tests/HeroLayoutSourceTests.cs:2367; Maliev.Web.Tests/BlogContentQualityTests.cs:18; Maliev.Web.Tests/BlogEbookPdfSourceTests.cs:12; Maliev.Web.Tests/WebBffEndpointTests.cs:93</x:v>
+      </x:c>
+      <x:c r="U61" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" t="str">
+        <x:v>WEB-061</x:v>
+      </x:c>
+      <x:c r="B62" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C62" t="str">
+        <x:v>Material library search, detail guidance, and same-process comparison</x:v>
+      </x:c>
+      <x:c r="D62" t="str">
+        <x:v>As a buyer choosing a material, I can search the material library, open a material, download its datasheet, and compare it against similar options.</x:v>
+      </x:c>
+      <x:c r="E62" t="str">
+        <x:v>The materials overview groups visible materials by process category, searches by name, family, process, category, best-fit text, and standards, shows empty-state feedback, and links each material card to detail. The detail page handles missing materials, renders breadcrumb, standards, best-fit copy, datasheet download action, spec rows, selection guidance, pro/con insight blocks, same-process comparison chips, selected comparison matrix, and localized datasheet URLs and filenames.</x:v>
+      </x:c>
+      <x:c r="F62" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G62" t="str">
+        <x:v>Mapped current material source tests and material content helpers; not rerun in this workbook pass.</x:v>
+      </x:c>
+      <x:c r="H62" t="str">
+        <x:v>No workbook-pass behavior error documented; material browser testing loop pending.</x:v>
+      </x:c>
+      <x:c r="I62" t="str">
+        <x:v>No app fix applied; tracker row only.</x:v>
+      </x:c>
+      <x:c r="J62" t="str">
+        <x:v>Pending story-by-story test loop.</x:v>
+      </x:c>
+      <x:c r="K62" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L62" t="str">
+        <x:v>Materials.razor overview -&gt; MaterialDetail.razor -&gt; SiteContent material catalog -&gt; MaterialController/PdfService boundary for datasheet rows tracked separately</x:v>
+      </x:c>
+      <x:c r="M62" t="str">
+        <x:v>Materials.razor; MaterialDetail.razor; SiteContent.cs</x:v>
+      </x:c>
+      <x:c r="N62" t="str">
+        <x:v>Materials overview renders search, category sections, material cards, image alt text, specs, and empty state; MaterialDetail renders guidance, insight blocks, same-process comparison, datasheet download, and missing-material fallback.</x:v>
+      </x:c>
+      <x:c r="O62" t="str">
+        <x:v>SiteContent resolves materials, categories, same-category peers, localized datasheet hrefs, and datasheet filenames; material datasheet BFF/PDF behavior is tracked in the PDF boundary row.</x:v>
+      </x:c>
+      <x:c r="P62" t="str">
+        <x:v>Mapped tests: MaterialsDirectComparisonUsesSingleLabelColumnAndInsightIcons, Material search and datasheet source tests, and WebBffEndpoint material datasheet endpoint tests.</x:v>
+      </x:c>
+      <x:c r="Q62" t="str">
+        <x:v>Maliev.Web Client, static SiteContent, Web BFF material datasheet boundary</x:v>
+      </x:c>
+      <x:c r="R62" t="str">
+        <x:v>Search string, material slug, selected comparison slugs, material specs/guidance text, datasheet URL and filename.</x:v>
+      </x:c>
+      <x:c r="S62" t="str">
+        <x:v>Needs browser retest for search, empty state, material detail fallback, compare chip toggle, comparison matrix, datasheet download, and localized text.</x:v>
+      </x:c>
+      <x:c r="T62" t="str">
+        <x:v>Maliev.Web.Client/Pages/Materials.razor:1,17,22,27,35,45,60,70,94,99,104,106,109,117,119; Maliev.Web.Client/Pages/MaterialDetail.razor:1,13,23,39,48,51,60,80,91,110,119,132,152,160,167,174,181,188,221,228,262,264,275,276; Maliev.Web.Client/Content/SiteContent.cs:2319,2324,2329,2332,2338,2341,2347,2391,3104,3125; Maliev.Web.Tests/HeroLayoutSourceTests.cs:2272; Maliev.Web.Tests/MaterialDatasheetPdfSourceTests.cs:12; Maliev.Web.Tests/WebBffEndpointTests.cs:130</x:v>
+      </x:c>
+      <x:c r="U62" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fcfd078b6854a84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9cec153de4054bac"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11636,7 +11961,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb6ccc49362be435a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R28781e43658a4ae0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -16667,7 +16992,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Recd1a663fe9645b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a2937cde1b54f50"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add QuoteEngine drawing workspace stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rb7ecaa4f46974883"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4b69b6d1b8b24a00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Ra4ff4e7ce368496d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Raede19e6a5cc49f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc073e4ab36e44cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rbe04bf0c924c4f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rbf6d51e48499423e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rcb57f3dd383e46b6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -521,7 +521,7 @@
         <x:v>Maliev.QuoteEngine</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>55</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>194</x:v>
+        <x:v>196</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R865f272e0cfd46ee"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra09fed2ca29441e4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9777,7 +9777,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3563fef9059847df"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ad4794649274a08"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13450,10 +13450,140 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>QE-056</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>Part drawing attachments tab</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>As a customer, I can keep drawings and supporting files attached to the selected manufacturing part.</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>The selected part detail card exposes a Drawing tab that opens a two-column attachment surface. Customers can add up to ten drawing/support files at a time, see file type, size, and kind, select a file for preview, remove a file, and have drawing changes emitted through the same part-change callback used by estimates, drafts, formal quotes, and order snapshots. Previewable signed or relative storage paths render in an iframe; session-local files remain listed until they are submitted with the quote/project payload.</x:v>
+      </x:c>
+      <x:c r="F57" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G57" t="str">
+        <x:v>Mapped to current source and existing source/endpoint tests; focused test execution not run in this workbook slice.</x:v>
+      </x:c>
+      <x:c r="H57" t="str">
+        <x:v>No behavior error documented in this tracker slice; live browser upload/preview/remove retest remains pending.</x:v>
+      </x:c>
+      <x:c r="I57" t="str">
+        <x:v>No app fix applied; spreadsheet-only code-derived tracker update.</x:v>
+      </x:c>
+      <x:c r="J57" t="str">
+        <x:v>Pending story-level execution in the next testing loop.</x:v>
+      </x:c>
+      <x:c r="K57" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L57" t="str">
+        <x:v>QePartDetailCard Drawing tab -&gt; QeDrawingAttachmentsTab file list/preview/remove state -&gt; QuotePartViewModel.DrawingFiles -&gt; QuotePartDraftDto.DrawingFiles -&gt; QuoteController draft/quote/order payloads</x:v>
+      </x:c>
+      <x:c r="M57" t="str">
+        <x:v>QePartDetailCard.razor; QeDrawingAttachmentsTab.razor; QuoteWorkspace.razor; QuoteEngineDtos.cs; QuoteController.cs</x:v>
+      </x:c>
+      <x:c r="N57" t="str">
+        <x:v>QePartDetailCard switches CenterMode to drawing, shows the drawing count, and renders QeDrawingAttachmentsTab for the selected part. QeDrawingAttachmentsTab renders a compact dropzone, file rows, delete controls, empty state, iframe preview for usable storage paths, and file-selection placeholders.</x:v>
+      </x:c>
+      <x:c r="O57" t="str">
+        <x:v>QuotePartAttachmentDto and QuotePartDraftDto carry drawing files; QuoteController includes drawing notes in estimates, draft/formal quote data, order production configuration snapshots, and configured order requirement text.</x:v>
+      </x:c>
+      <x:c r="P57" t="str">
+        <x:v>Existing evidence: QuoteEngineSourceTests covers QeDrawingAttachmentsTab two-column surface and drawing file DTO serialization; QuoteEngineEndpointTests covers drawing persistence through draft/duplicate/order flows.</x:v>
+      </x:c>
+      <x:c r="Q57" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, quote DTOs, project/draft/formal quote/order boundaries</x:v>
+      </x:c>
+      <x:c r="R57" t="str">
+        <x:v>QuotePartAttachmentDto records, Part.DrawingFiles list, selected drawing preview state, draft/formal quote/order configuration snapshots and requirement summaries</x:v>
+      </x:c>
+      <x:c r="S57" t="str">
+        <x:v>Needs live browser retest for file selection, previewable URL rendering, removal, and persistence through draft/quote/order actions against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T57" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteEngine/QePartDetailCard.razor:33,71,73; Maliev.QuoteEngine.Client/Components/QuoteEngine/QeDrawingAttachmentsTab.razor:1,6,12,19,26,50,67,92,117,124,133,141; Maliev.QuoteEngine.Shared/Quotes/QuoteEngineDtos.cs:159,346; Maliev.QuoteEngine.Bff/Controllers/QuoteController.cs:489,844,893,1478,1529; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:450,486,2904,4037; Maliev.QuoteEngine.Tests/QuoteEngineEndpointTests.cs:2784,2914,3422,3504</x:v>
+      </x:c>
+      <x:c r="U57" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" t="str">
+        <x:v>QE-057</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>Supplemental drawing interpretation</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>As a customer, I can attach drawings or sketches and have the agent extract usable manufacturing requirements without pretending they replace CAD geometry.</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>When a customer sends drawings, PDFs, photos, or sketches as supplemental manufacturing context, the agent session records them as visible artifacts, marks them as not satisfying the geometry gate, summarizes quantity/process/material/finish/tolerance/lead-time assumptions where inferable, stores requirement facts, attaches supplemental files to the relevant part when CAD is also present, and includes drawing guidance in later agent prompts. The agent should summarize readable drawing context and only ask for measurements that are genuinely missing.</x:v>
+      </x:c>
+      <x:c r="F58" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G58" t="str">
+        <x:v>Mapped to existing QuoteAgent endpoint and source tests; focused test execution not run in this workbook slice.</x:v>
+      </x:c>
+      <x:c r="H58" t="str">
+        <x:v>No behavior error documented in this tracker slice; live chatbot drawing-interpretation retest remains pending.</x:v>
+      </x:c>
+      <x:c r="I58" t="str">
+        <x:v>No app fix applied; spreadsheet-only code-derived tracker update.</x:v>
+      </x:c>
+      <x:c r="J58" t="str">
+        <x:v>Pending story-level execution in the next testing loop.</x:v>
+      </x:c>
+      <x:c r="K58" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L58" t="str">
+        <x:v>QuoteAgentLaunchShell sent attachments -&gt; QuoteAgentMessageRequest attachments -&gt; AgentController message/stream endpoints -&gt; QuoteAgentService supplemental artifact creation, requirement facts, part attachment, prompt grounding -&gt; QuoteAgentStateResponse.RequirementFacts and artifacts</x:v>
+      </x:c>
+      <x:c r="M58" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; AgentController.cs; QuoteAgentService.cs; QuoteAgentDtos.cs; QuoteEngineDtos.cs</x:v>
+      </x:c>
+      <x:c r="N58" t="str">
+        <x:v>Customer drawing/sketch/photo/PDF attachments appear in the agent composer and sent-message attachment UI; when used with CAD they can be associated to the part drawing file list and reflected in the part workspace.</x:v>
+      </x:c>
+      <x:c r="O58" t="str">
+        <x:v>QuoteAgentService creates supplemental artifacts with file metadata and satisfiesGeometryGate=false, infers source types and manufacturing facts, attaches supplemental manufacturing files to part DrawingFiles, builds manufacturing notes such as technical drawing supplied, and instructs the agent to inspect PDF/technical drawing context before asking for missing facts.</x:v>
+      </x:c>
+      <x:c r="P58" t="str">
+        <x:v>Existing evidence: QuoteAgentEndpointTests covers supplemental drawing gate behavior, structured requirement extraction, CAD+drawing part attachment, resumed session drawing context, and session search metadata.</x:v>
+      </x:c>
+      <x:c r="Q58" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, QuoteAgentService, QuoteAgentSessionStore, ChatbotService request context, quote DTOs</x:v>
+      </x:c>
+      <x:c r="R58" t="str">
+        <x:v>QuoteAgentArtifactDto supplemental artifacts, artifact metadata, requirement facts, part DrawingFiles, session attachment state, chatbot prompt context</x:v>
+      </x:c>
+      <x:c r="S58" t="str">
+        <x:v>Needs live browser and agent retest for drawing/PDF/sketch uploads, requirement extraction, follow-up question quality, and part association in a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T58" t="str">
+        <x:v>Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:4937,4967,5008,5062,5101,5151,5201,5357,5377,5384,5726; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs:161,652; Maliev.QuoteEngine.Shared/Quotes/QuoteEngineDtos.cs:159,346; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:1743,1794,1880,1926,2077,2104,3701,3752,3985,4032,4966</x:v>
+      </x:c>
+      <x:c r="U58" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra05cbff06ad24343"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfc855fd4554965"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add QuoteEngine composer preview stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc073e4ab36e44cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rbe04bf0c924c4f60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rbf6d51e48499423e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rcb57f3dd383e46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7fecbb8f4957478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rae288499ffb94164"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R859a06f13c1e4b07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Ra1e4e098eb814dbf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -521,7 +521,7 @@
         <x:v>Maliev.QuoteEngine</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>57</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>196</x:v>
+        <x:v>198</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra09fed2ca29441e4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf93180b44ce040be"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9777,7 +9777,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ad4794649274a08"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96e6582c4c6a45e7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13580,10 +13580,140 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="59">
+      <x:c r="A59" t="str">
+        <x:v>QE-058</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>Voice dictation composer</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>As a customer, I can dictate quote instructions into the agent composer in English or Thai.</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
+        <x:v>Customers can use the composer microphone button or a hold-to-talk spacebar shortcut to capture speech, see active and processing states, watch a timer and volume meter, preview live dictated text in the composer, and have recognized speech cleaned before it is inserted back into the draft message. Browser microphone errors stay as dismissible composer notices, unsupported browsers disable the button, and the customer can continue typing without losing the draft.</x:v>
+      </x:c>
+      <x:c r="F59" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G59" t="str">
+        <x:v>Mapped to current source and existing source tests; focused test execution not run in this workbook slice.</x:v>
+      </x:c>
+      <x:c r="H59" t="str">
+        <x:v>No behavior error documented in this tracker slice; live microphone permission and speech-recognition retest remains pending.</x:v>
+      </x:c>
+      <x:c r="I59" t="str">
+        <x:v>No app fix applied; spreadsheet-only code-derived tracker update.</x:v>
+      </x:c>
+      <x:c r="J59" t="str">
+        <x:v>Pending story-level execution in the next testing loop.</x:v>
+      </x:c>
+      <x:c r="K59" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L59" t="str">
+        <x:v>QuoteAgentLaunchShell composer UI -&gt; quote-agent-composer.js Web Speech API session -&gt; JSInvokable dictation lifecycle callbacks -&gt; QuoteEngineApiClient CleanSpeechAsync -&gt; AgentController clean-speech endpoint -&gt; ChatbotService speech cleanup</x:v>
+      </x:c>
+      <x:c r="M59" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; quote-agent-composer.js; QuoteEngineApiClient.cs; AgentController.cs; QuoteAgentDtos.cs</x:v>
+      </x:c>
+      <x:c r="N59" t="str">
+        <x:v>The launch shell renders a microphone button, tooltip, disabled state, spinner, timer, meter, and dismissible microphone notice; the textarea declares culture-aware speech-recognition language attributes and the JS module initializes with the dictation button reference.</x:v>
+      </x:c>
+      <x:c r="O59" t="str">
+        <x:v>POST quote/v1/agent/clean-speech accepts QuoteAgentCleanSpeechRequest with required speech and optional en/th language, rate-limits the BFF endpoint, calls ChatbotService CleanSpeechAsync, and returns cleaned text or the original speech when cleanup returns empty.</x:v>
+      </x:c>
+      <x:c r="P59" t="str">
+        <x:v>Existing evidence: QuoteEngineSourceTests covers composer initialization with dictation button, speech support detection, language configuration, live/final preview spans, meter styling, hold-delay shortcut, non-blocking notices, and CleanSpeechAsync integration.</x:v>
+      </x:c>
+      <x:c r="Q59" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, ChatbotService speech cleanup, browser Web Speech API</x:v>
+      </x:c>
+      <x:c r="R59" t="str">
+        <x:v>Draft message text, dictation lifecycle flags, culture-specific speech language attributes, cleaned speech text, microphone notice state</x:v>
+      </x:c>
+      <x:c r="S59" t="str">
+        <x:v>Needs live browser retest for microphone permission flows, Thai/English recognition, hold-to-talk timing, cleanup fallback, and composer focus after completion against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T59" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:1098,1217,1221,1233,1238,2293,2301,2726,2727,3258,3295,3307,3345,3410; Maliev.QuoteEngine.Client/wwwroot/js/quote-agent-composer.js:3,8,54,76,97,115,198,699,750,802,990,1013,1198,1250; Maliev.QuoteEngine.Client/Services/QuoteEngineApiClient.cs:321; Maliev.QuoteEngine.Bff/Controllers/AgentController.cs:113; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs:876; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1088,1138,1372,1414,1512,1530,2104</x:v>
+      </x:c>
+      <x:c r="U59" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" t="str">
+        <x:v>QE-059</x:v>
+      </x:c>
+      <x:c r="B60" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C60" t="str">
+        <x:v>File preview modal navigation</x:v>
+      </x:c>
+      <x:c r="D60" t="str">
+        <x:v>As a customer, I can open uploaded files, sketches, and workflow artifacts in one preview modal and move between them.</x:v>
+      </x:c>
+      <x:c r="E60" t="str">
+        <x:v>Customers can open a focused file preview dialog from uploaded parts, sketches, or visible workflow artifacts. The dialog shows the file kind, title, and status, renders image and PDF previews inline, falls back to an attached-file state for other formats, closes from the backdrop or close button, and navigates previous/next across the combined preview list without leaving the agent workspace.</x:v>
+      </x:c>
+      <x:c r="F60" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G60" t="str">
+        <x:v>Mapped to current source and existing source tests; focused test execution not run in this workbook slice.</x:v>
+      </x:c>
+      <x:c r="H60" t="str">
+        <x:v>No behavior error documented in this tracker slice; live modal preview navigation retest remains pending.</x:v>
+      </x:c>
+      <x:c r="I60" t="str">
+        <x:v>No app fix applied; spreadsheet-only code-derived tracker update.</x:v>
+      </x:c>
+      <x:c r="J60" t="str">
+        <x:v>Pending story-level execution in the next testing loop.</x:v>
+      </x:c>
+      <x:c r="K60" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L60" t="str">
+        <x:v>QuoteAgentLaunchShell preview open handlers -&gt; BuildPreviewItems uploaded/artifact/sketch aggregation -&gt; PreviewItem URL and content-type resolution -&gt; preview dialog image/PDF/fallback rendering -&gt; artifact download URL routing for storage paths</x:v>
+      </x:c>
+      <x:c r="M60" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; QuoteAgentUiHelpers.cs; AgentController.cs; QuoteAgentService.cs; QuoteAgentDtos.cs</x:v>
+      </x:c>
+      <x:c r="N60" t="str">
+        <x:v>The launch shell renders qe-agent-preview-modal with a backdrop, dialog header, close action, previous/next buttons, image stage, PDF iframe, and fallback panel; OpenUploadedPreview, OpenArtifactPreview, OpenSketchPreview, MovePreview, and BuildPreviewItems coordinate the selected preview index.</x:v>
+      </x:c>
+      <x:c r="O60" t="str">
+        <x:v>ArtifactPreviewUrl accepts data, blob, absolute, and app-relative URLs directly and routes storage paths through /quote/v1/agent/sessions/{sessionId}/artifacts/download so session-owned artifacts still use the BFF download boundary.</x:v>
+      </x:c>
+      <x:c r="P60" t="str">
+        <x:v>Existing evidence: QuoteEngineSourceTests covers modal markup, preview navigation controls, selected artifact preview item, single selected artifact preview surface, and artifact preview item placement relative to feedback handling.</x:v>
+      </x:c>
+      <x:c r="Q60" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF artifact download endpoint, QuoteAgentService artifact/session state</x:v>
+      </x:c>
+      <x:c r="R60" t="str">
+        <x:v>Preview dialog open state, preview index, PreviewItem records, selected artifact state, storage-path download URLs</x:v>
+      </x:c>
+      <x:c r="S60" t="str">
+        <x:v>Needs live browser retest for uploaded-part preview, sketch preview, artifact preview, PDF iframe rendering, image preview rendering, keyboard/focus behavior, and previous/next navigation against a running QuoteEngine host.</x:v>
+      </x:c>
+      <x:c r="T60" t="str">
+        <x:v>Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:1581,1593,1604,1608,1821,1823,1838,1844,1863,2340,3956,4013,5117,5146; Maliev.QuoteEngine.Client/wwwroot/css/app.css:5382,5391,5403,5448,5457,5469,5488,5505,5509,5513; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:1575,1583,2143,5134</x:v>
+      </x:c>
+      <x:c r="U60" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7bfc855fd4554965"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R267d58ddf1dd4be0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet NDA workflow stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7fecbb8f4957478a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rae288499ffb94164"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R859a06f13c1e4b07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Ra1e4e098eb814dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra1f4cd5649984f0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Reb592620736b41c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R75db5d127bde4df0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R192271ccc226416f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>78</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>198</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf93180b44ce040be"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79c4f74c1a8d4de3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9774,10 +9774,140 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="80">
+      <x:c r="A80" t="str">
+        <x:v>INT-079</x:v>
+      </x:c>
+      <x:c r="B80" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C80" t="str">
+        <x:v>Customer NDA intake and signed-document upload</x:v>
+      </x:c>
+      <x:c r="D80" t="str">
+        <x:v>As a sales or support employee, I can upload signed NDA documents and capture NDA lifecycle details while creating or updating a customer.</x:v>
+      </x:c>
+      <x:c r="E80" t="str">
+        <x:v>The new-customer workflow keeps standard customer documents and NDA documents in separate upload groups, accepts up to ten NDA files, assigns the NDA document subtype during create, and builds a CreateNDARequest from the first uploaded NDA document. The sign-NDA dialog accepts a signed document, calls AI date extraction, asks for manual expiration review when no date is detected, uploads the file as an NDA document, links it to the customer, and returns expiration and file-reference details.</x:v>
+      </x:c>
+      <x:c r="F80" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G80" t="str">
+        <x:v>Existing source and client tests cover the customer NDA document tab, Draft-first lifecycle status, separate NDA upload group, NDA subtype mapping, and customer-service create-with-documents boundary. Focused tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H80" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I80" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J80" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K80" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L80" t="str">
+        <x:v>CustomerNew NDA document panel -&gt; UploadDocumentGroupAsync -&gt; CreateNDARequest/CreateNdaStepRequest -&gt; CustomersController.CreateNda -&gt; CustomerServiceClient.CreateNdaWithDocumentsAsync; SignNdaDialog -&gt; AiProcessingController extract/upload/link document endpoints -&gt; customer NDA payload</x:v>
+      </x:c>
+      <x:c r="M80" t="str">
+        <x:v>CustomerNew.razor; SignNdaDialog.razor; CustomersController.cs; CustomerServiceClient.cs; AiProcessingController.cs; CustomerDtos.cs; CommonDtos.cs</x:v>
+      </x:c>
+      <x:c r="N80" t="str">
+        <x:v>/customers/new and /sales/customers/new show separated customer/NDA document upload panels, an NDA lifecycle section, NDA file picker, upload list, and signed-NDA dialog expiration review state.</x:v>
+      </x:c>
+      <x:c r="O80" t="str">
+        <x:v>CustomersController creates customer-scoped NDA records with documents; CustomerServiceClient forwards CreateNDARequest and document lists; AiProcessingController exposes NDA date extraction, document upload, and document link endpoints.</x:v>
+      </x:c>
+      <x:c r="P80" t="str">
+        <x:v>ModuleRegressionSourceTests CustomerNew NDA assertions; CustomerServiceClient tests for customer onboarding/create NDA document payloads where present.</x:v>
+      </x:c>
+      <x:c r="Q80" t="str">
+        <x:v>Intranet Client, Intranet BFF, CustomerService, AiProcessing, document storage</x:v>
+      </x:c>
+      <x:c r="R80" t="str">
+        <x:v>NDA document uploads, CreateNDARequest, linked customer documents, extracted expiration/effective/signed dates, file reference metadata</x:v>
+      </x:c>
+      <x:c r="S80" t="str">
+        <x:v>Needs live browser retest for PDF/image upload, AI date detection, manual expiration fallback, document link, and customer-create submission.</x:v>
+      </x:c>
+      <x:c r="T80" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Customers/CustomerNew.razor:410,470,485,500,929,932,1110,1204,1214,1222,1803; Maliev.Intranet.Client/Components/SignNdaDialog.razor:9,27,60,106,109,151,162,164,171,177,178; Maliev.Intranet.Bff/Controllers/CustomersController.cs:177,179; Maliev.Intranet.Bff/Clients/CustomerServiceClient.cs:80,85,866; Maliev.Intranet.Bff/Controllers/AiProcessingController.cs:643,708,717,729,889,940; Maliev.Intranet.Shared/Dtos/CommonDtos.cs:450; Maliev.Intranet.Shared/Dtos/CustomerDtos.cs:923,968; Maliev.Intranet.Tests/Client/Pages/ModuleRegressionSourceTests.cs:1774,1776,1781,1782,1783</x:v>
+      </x:c>
+      <x:c r="U80" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" t="str">
+        <x:v>INT-080</x:v>
+      </x:c>
+      <x:c r="B81" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C81" t="str">
+        <x:v>Customer NDA lifecycle status, revocation, and audit history</x:v>
+      </x:c>
+      <x:c r="D81" t="str">
+        <x:v>As a sales or compliance employee, I can update NDA status, require revocation reasons, and review audit history for customer NDAs.</x:v>
+      </x:c>
+      <x:c r="E81" t="str">
+        <x:v>The NDA settings dialog loads the existing NDA expiration and status, supports Draft, Signed, Expired, and Revoked states, disables saving a revoked NDA until a reason is entered, and returns version, signed, revoked, and revoke-reason fields. The revoke dialog requires a reason before closing. The history dialog loads NDA audit records, shows action and status transitions, actor display, document creation or replacement, expiration changes, revoked dates, and an empty-history state.</x:v>
+      </x:c>
+      <x:c r="F81" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G81" t="str">
+        <x:v>Existing source and client tests cover NDA DTO construction and GetNdaHistoryAsync client behavior. Focused tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H81" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I81" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J81" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K81" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L81" t="str">
+        <x:v>Customer NDA dialogs -&gt; CustomersController UpdateNdaStatus/UpdateNda/DeleteNda/GetNdaHistory -&gt; CustomerServiceClient NDA APIs -&gt; CustomerService NDA and audit DTOs</x:v>
+      </x:c>
+      <x:c r="M81" t="str">
+        <x:v>AddNdaDialog.razor; RevokeNdaDialog.razor; NdaHistoryDialog.razor; CustomersController.cs; CustomerServiceClient.cs; CustomerDtos.cs</x:v>
+      </x:c>
+      <x:c r="N81" t="str">
+        <x:v>NDA settings and revoke dialogs enforce required revocation reason; audit dialog shows timeline status, actor, document, expiration, revoked-date, and no-history states.</x:v>
+      </x:c>
+      <x:c r="O81" t="str">
+        <x:v>CustomersController routes NDA delete, status update, detail update, and audit-history requests to CustomerServiceClient; CustomerServiceClient exposes matching NDA update/delete/history calls.</x:v>
+      </x:c>
+      <x:c r="P81" t="str">
+        <x:v>CustomerServiceClientTests.GetNdaHistoryAsync_ShouldReturnData; DtoTests NDAResponse construction.</x:v>
+      </x:c>
+      <x:c r="Q81" t="str">
+        <x:v>Intranet Client, Intranet BFF, CustomerService</x:v>
+      </x:c>
+      <x:c r="R81" t="str">
+        <x:v>NDA status, expiration, row-version token, signed/revoked metadata, revoke reason, audit log records</x:v>
+      </x:c>
+      <x:c r="S81" t="str">
+        <x:v>Needs live browser retest for edit, revoke, history timeline rendering, and actor resolution.</x:v>
+      </x:c>
+      <x:c r="T81" t="str">
+        <x:v>Maliev.Intranet.Client/Components/AddNdaDialog.razor:8,14,18,20,28,35,43,44,51,52,53,54,56,57; Maliev.Intranet.Client/Components/RevokeNdaDialog.razor:7,12; Maliev.Intranet.Client/Components/NdaHistoryDialog.razor:8,14,21,27,33,39,45,49,53,60,66,71,82,102,119,131,153,158; Maliev.Intranet.Bff/Controllers/CustomersController.cs:345,348,360,362,374,376,457,459; Maliev.Intranet.Bff/Clients/CustomerServiceClient.cs:757,766,801,811; Maliev.Intranet.Shared/Dtos/CustomerDtos.cs:281,313,345; Maliev.Intranet.Tests/Bff/Clients/CustomerServiceClientTests.cs:817,827; Maliev.Intranet.Tests/Shared/DtoTests.cs:59</x:v>
+      </x:c>
+      <x:c r="U81" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R96e6582c4c6a45e7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3a582d5426d47d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13713,7 +13843,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R267d58ddf1dd4be0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeb50075043641de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet invoice workflow stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Ra1f4cd5649984f0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Reb592620736b41c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R75db5d127bde4df0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R192271ccc226416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R80d805b7e6354537"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rabd9225fc4e940d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R38076ce902ad4384"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R996b856f5ae841c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>80</x:v>
+        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>200</x:v>
+        <x:v>202</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79c4f74c1a8d4de3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d5d3a5bdbdc4715"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9904,10 +9904,140 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="82">
+      <x:c r="A82" t="str">
+        <x:v>INT-081</x:v>
+      </x:c>
+      <x:c r="B82" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C82" t="str">
+        <x:v>Invoice creation, customer billing, and PO attachment</x:v>
+      </x:c>
+      <x:c r="D82" t="str">
+        <x:v>As a finance employee, I can create an invoice from a selected customer, validate billing details, and attach the customer PO document.</x:v>
+      </x:c>
+      <x:c r="E82" t="str">
+        <x:v>The new-invoice page opens at the accounting create route, searches/selects an existing customer, loads customer detail, applies company or customer billing name, tax ID, billing and shipping address data, sets issue date, due date, payment terms, PO number, and a manufacturing-services line item, and validates customer, billing, tax, address, line amount, and due-date requirements before posting. Optional customer PO files are capped at 25 MB and, after invoice creation succeeds, are uploaded to the invoice file endpoint as a CustomerPO attachment.</x:v>
+      </x:c>
+      <x:c r="F82" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G82" t="str">
+        <x:v>Existing InvoiceServiceClient tests cover create-invoice service contract mapping and invoice-file reference registration. Focused tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H82" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I82" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J82" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K82" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L82" t="str">
+        <x:v>InvoiceNew page -&gt; customer search/detail APIs -&gt; CreateInvoiceRequest/InvoiceItemDto -&gt; InvoicesController.Create -&gt; InvoiceServiceClient.CreateInvoiceAsync; PO file input -&gt; InvoicesController.UploadFile -&gt; UploadServiceClient -&gt; InvoiceServiceClient.RegisterFileAsync</x:v>
+      </x:c>
+      <x:c r="M82" t="str">
+        <x:v>InvoiceNew.razor; InvoicesController.cs; InvoiceServiceClient.cs; FinanceDtos.cs; InvoiceServiceClientTests.cs</x:v>
+      </x:c>
+      <x:c r="N82" t="str">
+        <x:v>/accounting/new renders customer picker, PO number/document fields, due date, tax rate, billing preview, validation messages, and Create Invoice action.</x:v>
+      </x:c>
+      <x:c r="O82" t="str">
+        <x:v>api/v1/invoices creates invoices through InvoiceService; api/v1/invoices/{id}/files uploads and registers customer PO attachments with storage metadata and invoice file reference data.</x:v>
+      </x:c>
+      <x:c r="P82" t="str">
+        <x:v>InvoiceServiceClientTests.CreateInvoiceAsync_PostsInvoiceServiceContract; InvoiceServiceClientTests.RegisterFileAsync_PostsInvoiceFileReferenceContract.</x:v>
+      </x:c>
+      <x:c r="Q82" t="str">
+        <x:v>Intranet Client, Intranet BFF, CustomerService, InvoiceService, UploadService</x:v>
+      </x:c>
+      <x:c r="R82" t="str">
+        <x:v>Invoice header, invoice line item, payment terms, customer billing snapshot, PO file storage path, invoice file reference</x:v>
+      </x:c>
+      <x:c r="S82" t="str">
+        <x:v>Needs live browser retest for customer search, billing data load, validation failures, invoice creation, oversized PO rejection, and PO attachment success/failure handling.</x:v>
+      </x:c>
+      <x:c r="T82" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Accounting/InvoiceNew.razor:1,11,23,36,37,49,80,82,86,90,135,187,201,225,227,234,239,251,258,264,282,322,341,350; Maliev.Intranet.Bff/Controllers/InvoicesController.cs:57,59,84,86,98,121,127; Maliev.Intranet.Bff/Clients/InvoiceServiceClient.cs:49,65,83,95,106; Maliev.Intranet.Shared/Dtos/FinanceDtos.cs:272,293,338,359; Maliev.Intranet.Tests/Bff/Clients/InvoiceServiceClientTests.cs:64,87,168,190,201</x:v>
+      </x:c>
+      <x:c r="U82" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="83">
+      <x:c r="A83" t="str">
+        <x:v>INT-082</x:v>
+      </x:c>
+      <x:c r="B83" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C83" t="str">
+        <x:v>Invoice detail payment, receipt, PDF, and lifecycle actions</x:v>
+      </x:c>
+      <x:c r="D83" t="str">
+        <x:v>As a finance employee, I can inspect invoice details, record payment, create receipts, and rely on invoice lifecycle/PDF actions behind the same BFF contract.</x:v>
+      </x:c>
+      <x:c r="E83" t="str">
+        <x:v>The invoice detail pages load by invoice ID from accounting or finance routes, show status, tax, total, due date, customer/tax information, line items, payment controls, and receipt history. Payment recording is disabled for closed invoice statuses, posts amount/date/method/reference to the invoice payment endpoint, updates the invoice response, and seeds receipt creation from the paid amount. Receipt creation posts to the receipts endpoint and refreshes the local receipt list. The BFF also exposes guarded invoice list/detail, update, finalize, cancel, split, and invoice-PDF generation routes for the same invoice service boundary.</x:v>
+      </x:c>
+      <x:c r="F83" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G83" t="str">
+        <x:v>Existing InvoiceServiceClient tests cover invoice list/detail mapping, finalize payload, and payment creation plus allocation to invoice. Focused tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H83" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I83" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J83" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K83" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L83" t="str">
+        <x:v>InvoiceDetail page -&gt; InvoicesController.GetById/RecordPayment -&gt; InvoiceServiceClient -&gt; InvoiceService payment allocation; InvoiceDetail receipt panel -&gt; Receipts API; lifecycle/PDF endpoints -&gt; InvoiceServiceClient/PdfServiceClient</x:v>
+      </x:c>
+      <x:c r="M83" t="str">
+        <x:v>InvoiceDetail.razor; InvoiceList.razor; InvoicesController.cs; InvoiceServiceClient.cs; FinanceDtos.cs; PdfDataDtos.cs; InvoiceServiceClientTests.cs</x:v>
+      </x:c>
+      <x:c r="N83" t="str">
+        <x:v>/accounting/{Id:guid} and /finance/invoices/{Id:guid} render invoice status/totals/customer/line items, payment form, receipt form, receipt history, and closed-status guards.</x:v>
+      </x:c>
+      <x:c r="O83" t="str">
+        <x:v>api/v1/invoices supports list, detail, update, finalize, payment, cancel, split, and generate-pdf operations; api/v1/receipts supports receipt creation/listing used by the detail page.</x:v>
+      </x:c>
+      <x:c r="P83" t="str">
+        <x:v>InvoiceServiceClientTests.GetInvoicesAsync_MapsInvoiceServicePaginationAndTotals; GetInvoiceByIdAsync_MapsInvoiceServiceLinesToDetailItems; FinalizeInvoiceAsync_PostsRequiredFinalizedByPayload; RecordInvoicePaymentAsync_PostsPaymentAndLinksAllocationToInvoice.</x:v>
+      </x:c>
+      <x:c r="Q83" t="str">
+        <x:v>Intranet Client, Intranet BFF, InvoiceService, ReceiptService, PdfService</x:v>
+      </x:c>
+      <x:c r="R83" t="str">
+        <x:v>Invoice status/detail response, payment allocation, receipt records, PDF generation request, lifecycle state changes</x:v>
+      </x:c>
+      <x:c r="S83" t="str">
+        <x:v>Needs live browser retest for invoice detail load, payment disabled states, payment recording, receipt creation, receipt history refresh, and lifecycle/PDF route smoke.</x:v>
+      </x:c>
+      <x:c r="T83" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Accounting/InvoiceDetail.razor:1,2,12,31,33,39,44,62,82,85,87,102,105,108,135,136,150,156,167,182,188,194,198,200,209,218,229,232,251,257,274,277,281,294,302; Maliev.Intranet.Client/Pages/Accounting/InvoiceList.razor:1,2,51,56,79,287,288,289,290,566; Maliev.Intranet.Bff/Controllers/InvoicesController.cs:32,34,46,48,149,151,160,162,171,173,191,193,202,204,216,218,223,235,236; Maliev.Intranet.Bff/Clients/InvoiceServiceClient.cs:22,33,118,131,143,154,167,185,192,213,222; Maliev.Intranet.Shared/Dtos/FinanceDtos.cs:8,44,489,536; Maliev.Intranet.Shared/Dtos/PdfDataDtos.cs:384,395; Maliev.Intranet.Tests/Bff/Clients/InvoiceServiceClientTests.cs:13,232,289,316,366,381,382</x:v>
+      </x:c>
+      <x:c r="U83" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3a582d5426d47d8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3326ec7529934892"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13843,7 +13973,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdeb50075043641de"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ebdccdd4d4a4230"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet accounting workflow stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R80d805b7e6354537"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rabd9225fc4e940d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R38076ce902ad4384"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R996b856f5ae841c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3ec2195332de4b92"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Ra76335bf9dea49f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5a42528812b7409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R080b16a0907e4849"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>82</x:v>
+        <x:v>84</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>202</x:v>
+        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9d5d3a5bdbdc4715"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfac5e84222894dde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10034,10 +10034,140 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="84">
+      <x:c r="A84" t="str">
+        <x:v>INT-083</x:v>
+      </x:c>
+      <x:c r="B84" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C84" t="str">
+        <x:v>Accounting quick journal entry, AI extraction, and evidence upload</x:v>
+      </x:c>
+      <x:c r="D84" t="str">
+        <x:v>As a finance employee, I can create income or expense journal entries from typed data, extracted document data, and uploaded evidence.</x:v>
+      </x:c>
+      <x:c r="E84" t="str">
+        <x:v>The accounting page exposes Income Entry and Expense Entry tabs with description, debit account, credit account, amount, currency, exchange rate, base-amount preview, and evidence-document inputs. The AI extraction panel accepts text or up to five files, rejects files above the accounting document limit, posts to the accounting extraction endpoint, applies extracted description, amount, currency, exchange rate, and account suggestions, then leaves the draft ready for review. Posting validates accounts, positive amount, and exchange rate, optionally uploads evidence as IncomeEvidence or ExpenseEvidence, creates balanced debit and credit journal lines with transaction and base amounts, and clears evidence/extraction state after success.</x:v>
+      </x:c>
+      <x:c r="F84" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G84" t="str">
+        <x:v>Existing AccountingServiceClient tests cover journal-entry pagination and real create-journal payload names. Focused tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H84" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I84" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J84" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K84" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L84" t="str">
+        <x:v>Accounting InvoiceList quick-entry tabs -&gt; AiProcessingController extract-accounting-entry -&gt; AccountingController.UploadDocument/CreateJournalEntry -&gt; AccountingServiceClient -&gt; AccountingService journal DTOs</x:v>
+      </x:c>
+      <x:c r="M84" t="str">
+        <x:v>InvoiceList.razor; AiProcessingController.cs; AccountingController.cs; AccountingServiceClient.cs; AccountingDtos.cs; AccountingServiceClientTests.cs</x:v>
+      </x:c>
+      <x:c r="N84" t="str">
+        <x:v>/accounting and /finance/invoices render Income Entry and Expense Entry tabs, extraction text/file controls, account selectors, currency/exchange-rate fields, evidence document picker, status/error messages, and Post Entry action.</x:v>
+      </x:c>
+      <x:c r="O84" t="str">
+        <x:v>api/v1/aiprocessing/extract-accounting-entry extracts accounting fields; api/v1/accounting/documents uploads evidence; api/v1/accounting/journal-entries creates journal entries with two balanced lines.</x:v>
+      </x:c>
+      <x:c r="P84" t="str">
+        <x:v>AccountingServiceClientTests.GetJournalEntriesAsync_TargetsJournalEntriesRouteWithPagination; AccountingServiceClientTests.CreateJournalEntryAsync_UsesRealJournalEntryPayloadNames.</x:v>
+      </x:c>
+      <x:c r="Q84" t="str">
+        <x:v>Intranet Client, Intranet BFF, AiProcessing, AccountingService, UploadService, CurrencyService</x:v>
+      </x:c>
+      <x:c r="R84" t="str">
+        <x:v>Quick journal draft fields, extracted accounting facts, evidence file reference, journal entry lines, transaction/base currency amounts</x:v>
+      </x:c>
+      <x:c r="S84" t="str">
+        <x:v>Needs live browser retest for extraction text/files, oversized-file rejection, currency-rate lookup, evidence upload failure, validation messages, and final journal creation.</x:v>
+      </x:c>
+      <x:c r="T84" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Accounting/InvoiceList.razor:16,125,174,382,413,414,428,452,467,490,653,656,671,681,689,708,715,724,736,743,746,754,781,785,790,794,798,805,811,818,821,822,828,831,835,838,841,842,854,856,858,872,885,901,908,916,924,925,929,938,1037,1040,1046,1213,1217,1221,1223,1225,1229,1233,1237,1245,1250; Maliev.Intranet.Bff/Controllers/AiProcessingController.cs:500,501,602,605,1001,1038,1077; Maliev.Intranet.Bff/Controllers/AccountingController.cs:59,61,63,188,190,205,207,224; Maliev.Intranet.Bff/Clients/AccountingServiceClient.cs:96,142,168; Maliev.Intranet.Shared/Dtos/AccountingDtos.cs:258,308; Maliev.Intranet.Tests/Bff/Clients/AccountingServiceClientTests.cs:42,82</x:v>
+      </x:c>
+      <x:c r="U84" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="85">
+      <x:c r="A85" t="str">
+        <x:v>INT-084</x:v>
+      </x:c>
+      <x:c r="B85" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C85" t="str">
+        <x:v>Accounting reports, periods, reconciliation, and payroll journal visibility</x:v>
+      </x:c>
+      <x:c r="D85" t="str">
+        <x:v>As a finance employee, I can review accounting reports, download report PDFs, manage accounting periods, run reconciliation, and see payroll-generated journal impact.</x:v>
+      </x:c>
+      <x:c r="E85" t="str">
+        <x:v>The accounting page exposes Reports, Periods, and Payroll Journals tabs. Reports render financial report sections, row amounts, totals, and a PDF download link. Periods list accounting periods, let finance open a period for a selected date, choose a reconciliation source with explanatory text, run reconciliation for a period, and display reconciliation status, difference count, and net difference. Payroll Journals shows journal entries produced by CompensationService payroll runs and explains when no payroll journal impact is present. The BFF guards report export, period, and reconciliation endpoints with accounting permissions and maps financial reports into the PdfService accounting-report contract.</x:v>
+      </x:c>
+      <x:c r="F85" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G85" t="str">
+        <x:v>Existing source/controller tests cover accounting module reports/periods/reconciliation/payroll UI markers, accounting endpoint permissions, and report-PDF PdfService contract mapping. Focused tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H85" t="str">
+        <x:v>No current tracker behavior error documented for this story.</x:v>
+      </x:c>
+      <x:c r="I85" t="str">
+        <x:v>No app fix applied in this spreadsheet slice.</x:v>
+      </x:c>
+      <x:c r="J85" t="str">
+        <x:v>Not yet retested in the current loop; existing automated tests mapped as secondary evidence.</x:v>
+      </x:c>
+      <x:c r="K85" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L85" t="str">
+        <x:v>Accounting InvoiceList reports/periods/payroll tabs -&gt; AccountingController report/period/reconciliation endpoints -&gt; AccountingServiceClient -&gt; PdfService report export</x:v>
+      </x:c>
+      <x:c r="M85" t="str">
+        <x:v>InvoiceList.razor; AccountingController.cs; AccountingServiceClient.cs; AccountingDtos.cs; AccountingControllerTests.cs; ModuleRegressionSourceTests.cs</x:v>
+      </x:c>
+      <x:c r="N85" t="str">
+        <x:v>/accounting and /finance/invoices render Reports with Download PDF, Periods and reconciliation controls, and Payroll Journals impact/empty-state messaging.</x:v>
+      </x:c>
+      <x:c r="O85" t="str">
+        <x:v>api/v1/accounting/reports/{type}, report PDF export, periods, open/close/reopen period, and reconciliation endpoints proxy AccountingService and PdfService boundaries with permission checks.</x:v>
+      </x:c>
+      <x:c r="P85" t="str">
+        <x:v>ModuleRegressionSourceTests accounting module report/period/reconciliation/payroll assertions; AccountingControllerTests.AccountingEndpoints_RequireActualAccountingServicePermissions; AccountingControllerTests.DownloadReportPdf_UsesPdfServiceReportContractAndReturnsPdfFile.</x:v>
+      </x:c>
+      <x:c r="Q85" t="str">
+        <x:v>Intranet Client, Intranet BFF, AccountingService, PdfService, CompensationService</x:v>
+      </x:c>
+      <x:c r="R85" t="str">
+        <x:v>Financial report sections/rows/totals, report PDF request, accounting periods, reconciliation result, payroll journal visibility</x:v>
+      </x:c>
+      <x:c r="S85" t="str">
+        <x:v>Needs live browser retest for report loading and PDF download, period open/reconcile actions, reconciliation source switching, and payroll-journal filtering/empty state.</x:v>
+      </x:c>
+      <x:c r="T85" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Accounting/InvoiceList.razor:81,111,223,259,263,265,288,290,326,328,343,346,361,374,384,385,401,549,582,975,995,1001,1005,1015,1017,1096,1098,1211; Maliev.Intranet.Bff/Controllers/AccountingController.cs:81,83,92,94,108,133,135,144,146,154,156,164,166,174,176,181,231,239,248,252,266,287; Maliev.Intranet.Bff/Clients/AccountingServiceClient.cs:44,49,54,59,64,69,175,195,199,206,213,220,234,271,277,295,310,341; Maliev.Intranet.Shared/Dtos/AccountingDtos.cs:406,421,427,451,475,485,496; Maliev.Intranet.Tests/Client/Pages/ModuleRegressionSourceTests.cs:588,594,613,614,620,624,627,634; Maliev.Intranet.Tests/Bff/Controllers/AccountingControllerTests.cs:19,20,21,22,23,24,25,26,27,28,29,42,106</x:v>
+      </x:c>
+      <x:c r="U85" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3326ec7529934892"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a8bcadea776426a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13973,7 +14103,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ebdccdd4d4a4230"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74f2e790866443ce"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet purchasing workflow stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3ec2195332de4b92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Ra76335bf9dea49f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5a42528812b7409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R080b16a0907e4849"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rba7030d0617647b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rf277f6ef88c34c8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Raff41aefb6784d73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R7541e67bc3084684"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>84</x:v>
+        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>204</x:v>
+        <x:v>207</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfac5e84222894dde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R057c7082a6224f70"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10164,10 +10164,205 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="86">
+      <x:c r="A86" t="str">
+        <x:v>INT-085</x:v>
+      </x:c>
+      <x:c r="B86" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C86" t="str">
+        <x:v>Supplier intake, registry-assisted creation, and profile lifecycle</x:v>
+      </x:c>
+      <x:c r="D86" t="str">
+        <x:v>As a purchasing employee, I can create supplier profiles from manual input, AI extraction, or Thai registry lookup and maintain supplier profile and status details.</x:v>
+      </x:c>
+      <x:c r="E86" t="str">
+        <x:v>Supplier Profiles opens the supplier list, supports showing the create panel from the New Supplier button or the create query parameter, loads paged suppliers with status, and validates required name, tax ID, email, address, city, and country fields before creating a supplier. The create panel can extract supplier fields from text or files, search the Thai company registry by name or 13-digit tax ID, apply official or extracted name, tax, contact, and address fields, trim and normalize country and capabilities, create the supplier through the BFF, and optionally return to the caller with the new supplier id. Supplier detail loads the profile, contact, capability, and status data, supports row-version guarded edits, and can send a status transition with a reason.</x:v>
+      </x:c>
+      <x:c r="F86" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G86" t="str">
+        <x:v>SupplierServiceClient tests cover create, detail mapping, update, and status-update contract mapping. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H86" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I86" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J86" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K86" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L86" t="str">
+        <x:v>SupplierList and SupplierDetail pages -&gt; AI supplier extraction and registry search -&gt; SuppliersController list/create/update/status/deactivate -&gt; SupplierServiceClient -&gt; SupplierService supplier/profile DTOs</x:v>
+      </x:c>
+      <x:c r="M86" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Purchasing/SupplierList.razor; Maliev.Intranet.Client/Pages/Purchasing/SupplierDetail.razor; Maliev.Intranet.Bff/Controllers/SuppliersController.cs; Maliev.Intranet.Bff/Clients/SupplierServiceClient.cs</x:v>
+      </x:c>
+      <x:c r="N86" t="str">
+        <x:v>/purchasing/suppliers and /purchasing/suppliers/{Id:guid} render supplier list, create panel, registry search, extracted-field review, supplier table/status, profile detail, edit/save, and status transition controls.</x:v>
+      </x:c>
+      <x:c r="O86" t="str">
+        <x:v>api/v1/suppliers lists, creates, updates, status-updates, deactivates, and loads supplier profiles; SupplierServiceClient maps Intranet create/update/status DTOs to SupplierService contacts, capabilities, status, row-version, and profile fields.</x:v>
+      </x:c>
+      <x:c r="P86" t="str">
+        <x:v>SupplierServiceClientTests.CreateSupplierAsync_MapsIntranetSupplierRequestToSupplierServiceContract; SupplierServiceClientTests.GetSupplierByIdAsync_MapsSupplierServiceDetailToIntranetSupplierDetail; SupplierServiceClientTests.UpdateSupplierAsync_MapsIntranetSupplierRequestToSupplierServiceConcurrencyContract; SupplierServiceClientTests.UpdateSupplierStatusAsync_MapsStatusAndRowVersionToSupplierServiceContract.</x:v>
+      </x:c>
+      <x:c r="Q86" t="str">
+        <x:v>Intranet Client, Intranet BFF, SupplierService, RegistryService, AiProcessing</x:v>
+      </x:c>
+      <x:c r="R86" t="str">
+        <x:v>Supplier profile fields, primary contact, capabilities, status, row-version, registry profile fields, extracted supplier fields</x:v>
+      </x:c>
+      <x:c r="S86" t="str">
+        <x:v>Live browser retest pending for create, extraction, registry search, edit, and status transition.</x:v>
+      </x:c>
+      <x:c r="T86" t="str">
+        <x:v>SupplierList.razor:1,12-13,24-136,213-224,254,379,438-464; SupplierDetail.razor:1,112-126,286,359,397-405; SuppliersController.cs:62-88,130-163; SupplierServiceClient.cs:127-175,367-400; SupplierServiceClientTests.cs:13,204.</x:v>
+      </x:c>
+      <x:c r="U86" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="87">
+      <x:c r="A87" t="str">
+        <x:v>INT-086</x:v>
+      </x:c>
+      <x:c r="B87" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C87" t="str">
+        <x:v>Supplier document upload, review, signed access, and deletion</x:v>
+      </x:c>
+      <x:c r="D87" t="str">
+        <x:v>As a purchasing employee, I can attach, review, open, and remove supplier documents with document type and date metadata.</x:v>
+      </x:c>
+      <x:c r="E87" t="str">
+        <x:v>Supplier detail exposes a Supplier Documents panel with document type, document name, issue date, expiration date, file input, upload action, and existing document list. It rejects missing type or name and files above 10 MB, uploads files to supplier document storage, records SupplierService document metadata, adds created documents to the profile, displays document type, status, and date labels, opens a signed download URL, and deletes documents from the profile when the BFF delete succeeds.</x:v>
+      </x:c>
+      <x:c r="F87" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G87" t="str">
+        <x:v>SupplierServiceClient tests cover supplier detail document mapping and add-document contract mapping. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H87" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I87" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J87" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K87" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L87" t="str">
+        <x:v>SupplierDetail document panel -&gt; SuppliersController AddDocument/DeleteDocument/GetDocumentDownloadUrl -&gt; UploadServiceClient signed storage path -&gt; SupplierServiceClient Add/Delete document metadata</x:v>
+      </x:c>
+      <x:c r="M87" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Purchasing/SupplierDetail.razor; Maliev.Intranet.Bff/Controllers/SuppliersController.cs; Maliev.Intranet.Bff/Clients/SupplierServiceClient.cs</x:v>
+      </x:c>
+      <x:c r="N87" t="str">
+        <x:v>/purchasing/suppliers/{Id:guid} renders the Supplier Documents panel, upload form, existing document table, open action, and delete action.</x:v>
+      </x:c>
+      <x:c r="O87" t="str">
+        <x:v>api/v1/suppliers/{id}/documents accepts multipart upload and document metadata, api/v1/suppliers/{id}/documents/{documentId} deletes metadata, and api/v1/suppliers/{id}/documents/download-url returns signed access for stored files.</x:v>
+      </x:c>
+      <x:c r="P87" t="str">
+        <x:v>SupplierServiceClientTests.GetSupplierByIdAsync_MapsSupplierServiceDetailToIntranetSupplierDetail; SupplierServiceClientTests.AddSupplierDocumentAsync_MapsIntranetDocumentToSupplierCertificationContract.</x:v>
+      </x:c>
+      <x:c r="Q87" t="str">
+        <x:v>Intranet Client, Intranet BFF, UploadService, SupplierService</x:v>
+      </x:c>
+      <x:c r="R87" t="str">
+        <x:v>Supplier document metadata, storage object reference, issue date, expiration date, document status, signed access URL</x:v>
+      </x:c>
+      <x:c r="S87" t="str">
+        <x:v>Live browser retest pending for upload, open/download, and delete flows.</x:v>
+      </x:c>
+      <x:c r="T87" t="str">
+        <x:v>SupplierDetail.razor:132-206,472,544,550-613,652; SuppliersController.cs:196-225,243-270; SupplierServiceClient.cs:203-221,400; SupplierServiceClientTests.cs:76-153,243-288.</x:v>
+      </x:c>
+      <x:c r="U87" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="88">
+      <x:c r="A88" t="str">
+        <x:v>INT-087</x:v>
+      </x:c>
+      <x:c r="B88" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C88" t="str">
+        <x:v>Purchase order list, creation, lifecycle actions, files, and export</x:v>
+      </x:c>
+      <x:c r="D88" t="str">
+        <x:v>As a purchasing employee, I can list purchase orders, create a supplier purchase order from a source order, progress its lifecycle, export it, and attach supporting files.</x:v>
+      </x:c>
+      <x:c r="E88" t="str">
+        <x:v>Purchasing opens at /purchasing and /mfg/procurement with status, type, order id, and supplier filters, supplier readiness state, and create action. New purchase order requires an available supplier, source order, and purchasable line item; it loads suppliers, source orders, and currencies, accepts supplier, source, line, quantity, currency, withholding tax, expected delivery, and notes, posts api/v1/procurement, and navigates to the created purchase order. Detail loads the purchase order, gates approve, send, receive, and cancel buttons by status, requires a cancel reason through the cancel panel, exports a PDF, and attaches files up to 25 MB by registering uploaded file metadata.</x:v>
+      </x:c>
+      <x:c r="F88" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G88" t="str">
+        <x:v>PurchaseOrderServiceClient tests cover list and filter routing, create DTO JSON names, lifecycle routes, and file-registration contract mapping. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H88" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I88" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J88" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K88" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L88" t="str">
+        <x:v>PoList/PoNew/PoDetail pages -&gt; ProcurementController -&gt; PurchaseOrderServiceClient -&gt; PurchaseOrderService DTOs and UploadService file registration</x:v>
+      </x:c>
+      <x:c r="M88" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Purchasing/PoList.razor; Maliev.Intranet.Client/Pages/Purchasing/PoNew.razor; Maliev.Intranet.Client/Pages/Purchasing/PoDetail.razor; Maliev.Intranet.Bff/Controllers/ProcurementController.cs; Maliev.Intranet.Bff/Clients/PurchaseOrderServiceClient.cs</x:v>
+      </x:c>
+      <x:c r="N88" t="str">
+        <x:v>/purchasing, /mfg/procurement, /purchasing/new, /purchasing/{Id:int}, and /mfg/procurement/{Id:int} render list filters, prerequisite guidance, purchase-order creation, lifecycle buttons, export, cancel, and file attachment.</x:v>
+      </x:c>
+      <x:c r="O88" t="str">
+        <x:v>api/v1/procurement lists, creates, loads detail, approves, sends to supplier, receives, cancels, uploads files, and exports; PurchaseOrderServiceClient maps to /purchase-order/v1/purchase-orders routes and JSON names including supplierID, orderID, sourceOrderId, customerPO, and file metadata.</x:v>
+      </x:c>
+      <x:c r="P88" t="str">
+        <x:v>PurchaseOrderServiceClientTests.GetPurchaseOrdersAsync_TargetsPurchaseOrdersEndpoint; PurchaseOrderServiceClientTests.GetPurchaseOrdersAsync_ForwardsFiltersToPurchaseOrderService; PurchaseOrderServiceClientTests.CreatePurchaseOrderAsync_UsesRealCreateDtoJsonNames; PurchaseOrderServiceClientTests.LifecycleMethods_TargetRealPurchaseOrderRoutes; PurchaseOrderServiceClientTests.RegisterFileAsync_TargetsPurchaseOrderFilesEndpoint.</x:v>
+      </x:c>
+      <x:c r="Q88" t="str">
+        <x:v>Intranet Client, Intranet BFF, PurchaseOrderService, SupplierService, OrderService, ReferenceDataService, UploadService</x:v>
+      </x:c>
+      <x:c r="R88" t="str">
+        <x:v>Purchase order fields, line items, lifecycle status, cancel reason, export response, uploaded file metadata, storage object reference</x:v>
+      </x:c>
+      <x:c r="S88" t="str">
+        <x:v>Live browser retest pending for list filters, prerequisites, create, lifecycle actions, export, and file attachment.</x:v>
+      </x:c>
+      <x:c r="T88" t="str">
+        <x:v>PoList.razor:1-2,13,57-135,276-284; PoNew.razor:1,25-34,50-106,143-196,254-294,353; PoDetail.razor:1-2,31-47,120-154,182-196,209-239,245-330; ProcurementController.cs:24-77,87-129,139-206; PurchaseOrderServiceClient.cs:83-201,500-565; PurchaseOrderServiceClientTests.cs:13-77,140-226,264-317.</x:v>
+      </x:c>
+      <x:c r="U88" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0a8bcadea776426a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31ef1e82accd4be9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14103,7 +14298,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R74f2e790866443ce"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a2efbb12bc04581"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet admin workflow stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rba7030d0617647b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rf277f6ef88c34c8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Raff41aefb6784d73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R7541e67bc3084684"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R12debab7a5314521"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R8ac07f7207ba4b85"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R18201182c5da407f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Ra5d51cf5e2084b59"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>87</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>207</x:v>
+        <x:v>210</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R057c7082a6224f70"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31b96d109fd14440"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10359,10 +10359,205 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="89">
+      <x:c r="A89" t="str">
+        <x:v>INT-088</x:v>
+      </x:c>
+      <x:c r="B89" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C89" t="str">
+        <x:v>Chatbot instruction profile management and AI draft refinement</x:v>
+      </x:c>
+      <x:c r="D89" t="str">
+        <x:v>As an administrator, I can search, edit, create, and AI-refine chatbot core persona and topic skill instructions used by customer-facing conversations.</x:v>
+      </x:c>
+      <x:c r="E89" t="str">
+        <x:v>The Chatbot Instructions page opens with read permission, loads instruction profiles from the BFF using category, topic key, and active-only filters, auto-selects the website core profile when present, and lets an admin select rows for editing. The editor captures name, category, topic key, priority, active state, persona definition, and business constraints, shows live character counters and near-limit or over-limit warnings, blocks save when instruction text is too long, clamps priority to the shared limits, posts create or update requests to the BFF, reloads the list after save, and can request an AI-improved draft without saving it.</x:v>
+      </x:c>
+      <x:c r="F89" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G89" t="str">
+        <x:v>ChatbotInstructions source tests cover version display, text limits, AI refinement UI, and priority validation; ChatController tests cover instruction list, update, and refinement proxy behavior. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H89" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I89" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J89" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K89" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L89" t="str">
+        <x:v>ChatbotInstructions.razor -&gt; ChatController instruction endpoints -&gt; ChatbotServiceClient admin instruction routes -&gt; Chat DTO validation limits and instruction/refinement DTOs</x:v>
+      </x:c>
+      <x:c r="M89" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Admin/ChatbotInstructions.razor; Maliev.Intranet.Bff/Controllers/ChatController.cs; Maliev.Intranet.Bff/Clients/ChatbotServiceClient.cs; Maliev.Intranet.Shared/Dtos/ChatDtos.cs</x:v>
+      </x:c>
+      <x:c r="N89" t="str">
+        <x:v>/admin/chatbot-instructions renders search and category filters, instruction table, selectable rows, editable prompt fields, active and priority controls, reset/save actions, and AI refinement action.</x:v>
+      </x:c>
+      <x:c r="O89" t="str">
+        <x:v>api/v1/chat/instructions lists, creates, and updates instruction profiles; api/v1/chat/instructions/refine returns an AI-improved draft; ChatbotServiceClient maps to /chatbot/v1/admin/instructions and /chatbot/v1/admin/instructions/refine using shared BffSystemInstruction DTOs.</x:v>
+      </x:c>
+      <x:c r="P89" t="str">
+        <x:v>ChatbotInstructionsSourceTests.InstructionTextFields_ShowCountsAndLengthWarnings; ChatbotInstructionsSourceTests.InstructionEditor_OffersAiRefinement; ChatControllerTests.GetInstructions_ShouldReturnInstructionProfiles; ChatControllerTests.UpdateInstruction_ShouldProxyWritablePromptMutation; ChatControllerTests.RefineInstruction_ShouldProxyWritablePromptDraft.</x:v>
+      </x:c>
+      <x:c r="Q89" t="str">
+        <x:v>Intranet Client, Intranet BFF, ChatbotService</x:v>
+      </x:c>
+      <x:c r="R89" t="str">
+        <x:v>Instruction profile name, category, topic key, priority, active state, persona definition, business constraints, refined draft content, version metadata</x:v>
+      </x:c>
+      <x:c r="S89" t="str">
+        <x:v>Live browser retest pending for filter, select, create, update, and refine behavior.</x:v>
+      </x:c>
+      <x:c r="T89" t="str">
+        <x:v>ChatbotInstructions.razor:1,12-23,38-59,76-90,120-230,327-344,357-390,405-454,547-575,601-654; ChatController.cs:106-164; ChatbotServiceClient.cs:258-402; ChatDtos.cs:8,107-261; ChatbotInstructionsSourceTests.cs:55-96; ChatControllerTests.cs:158-251.</x:v>
+      </x:c>
+      <x:c r="U89" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" t="str">
+        <x:v>INT-089</x:v>
+      </x:c>
+      <x:c r="B90" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C90" t="str">
+        <x:v>System health dashboard, live probes, and seven-day history</x:v>
+      </x:c>
+      <x:c r="D90" t="str">
+        <x:v>As an administrator, I can monitor service liveness/readiness, review seven-day health history, and refresh health checks from the Admin area.</x:v>
+      </x:c>
+      <x:c r="E90" t="str">
+        <x:v>The System Health page opens with system health read permission, loads live service health and seven-day history together, shows overall status, last-checked time, auto-refresh interval, service counts, healthy and issue totals, critical issue count, and a per-service history strip. It displays current live and ready probe statuses, auto-refreshes every 60 seconds, supports manual refresh with a loading skeleton, handles unavailable data with an empty state, and cancels the refresh timer on disposal. The BFF computes overall status from critical and non-critical service results, probes liveness and readiness paths with retry, timeout, and concurrency controls, persists health samples, and returns bucketed history.</x:v>
+      </x:c>
+      <x:c r="F90" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G90" t="str">
+        <x:v>SystemHealth controller/service tests cover permission, liveness/readiness routes, readiness failure handling, transient retry, timeout settings, concurrent probe throttling, response shape, history service output, and bucket aggregation. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H90" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I90" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J90" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K90" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L90" t="str">
+        <x:v>SystemHealth.razor -&gt; SystemHealthController -&gt; SystemHealthProbeService and SystemHealthHistoryService -&gt; persisted HealthCheckSamples and SystemHealth DTOs</x:v>
+      </x:c>
+      <x:c r="M90" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Admin/SystemHealth.razor; Maliev.Intranet.Bff/Controllers/SystemHealthController.cs; Maliev.Intranet.Bff/Services/SystemHealthProbeService.cs; Maliev.Intranet.Bff/Services/SystemHealthHistoryService.cs; Maliev.Intranet.Bff/Services/SystemHealthHistoryAggregator.cs</x:v>
+      </x:c>
+      <x:c r="N90" t="str">
+        <x:v>/admin/system-health renders overall status, last checked time, refresh control, auto-refresh interval, summary stat tiles, service history strips, and live/ready probe grid.</x:v>
+      </x:c>
+      <x:c r="O90" t="str">
+        <x:v>api/v1/system-health returns live probe status for registered services; api/v1/system-health/history?days=7 returns bucketed historical samples; the probe service checks configured service targets with service-specific timeout and concurrency settings.</x:v>
+      </x:c>
+      <x:c r="P90" t="str">
+        <x:v>SystemHealthControllerTests.Controller_RequiresSystemHealthReadPermission; SystemHealthControllerTests.GetSystemHealth_UsesServiceLivenessAndReadinessEndpoints; SystemHealthControllerTests.GetSystemHealth_WhenReadinessFails_MarksServiceUnhealthyNotUnreachable; SystemHealthControllerTests.GetSystemHealth_ThrottlesConcurrentServiceProbes; SystemHealthControllerTests.GetSystemHealth_UsesProbeServiceAndPreservesLiveResponseShape; SystemHealthControllerTests.GetSystemHealthHistory_ReturnsHistoryFromHistoryService; SystemHealthHistoryAggregatorTests.BuildHistory_ExcludesMissingBucketsFromUptimeAndPreservesChronologicalOrder; IntranetDbContextTests.SystemHealthHistoryService_ReturnsSevenDaysOfFiveMinuteBucketsAndDeletesExpiredSamples.</x:v>
+      </x:c>
+      <x:c r="Q90" t="str">
+        <x:v>Intranet Client, Intranet BFF, registered MALIEV HTTP services, Intranet database</x:v>
+      </x:c>
+      <x:c r="R90" t="str">
+        <x:v>Live health probe result, readiness/liveness status, response time, error message, health sample record, seven-day bucketed history</x:v>
+      </x:c>
+      <x:c r="S90" t="str">
+        <x:v>Live browser retest pending for refresh, auto-refresh, empty state, and status-strip behavior.</x:v>
+      </x:c>
+      <x:c r="T90" t="str">
+        <x:v>SystemHealth.razor:1,10-21,24-78,102-143,172-248; SystemHealthController.cs:15-57; SystemHealthProbeService.cs:21-85,152-153; SystemHealthHistoryService.cs:16-62; SystemHealthHistoryAggregator.cs:21-93; SystemHealthControllerTests.cs:15-223; IntranetDbContextTests.cs:73-129.</x:v>
+      </x:c>
+      <x:c r="U90" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="91">
+      <x:c r="A91" t="str">
+        <x:v>INT-090</x:v>
+      </x:c>
+      <x:c r="B91" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C91" t="str">
+        <x:v>Website content inventory and routed content-surface ownership</x:v>
+      </x:c>
+      <x:c r="D91" t="str">
+        <x:v>As an administrator, I can see which current systems own public website content surfaces and where to manage each surface.</x:v>
+      </x:c>
+      <x:c r="E91" t="str">
+        <x:v>The Website Content page opens with web content read permission and presents a code-backed content inventory for public site operations. It lists content surfaces for blog and article copy, homepage and marketing copy, product catalog content, and website chatbot instructions, showing the owner/source, current status, supporting description, and route used to manage or inspect the surface. The Admin page links to the website content surface, and navigation tests keep the route available from the client shell.</x:v>
+      </x:c>
+      <x:c r="F91" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G91" t="str">
+        <x:v>Navigation and layout source tests cover the web-content route and homepage/blog content-surface links. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H91" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I91" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J91" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K91" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L91" t="str">
+        <x:v>WebContent.razor static content-surface inventory -&gt; AdminPage navigation -&gt; MalievPermissions.WebContent -&gt; related source systems for public content ownership</x:v>
+      </x:c>
+      <x:c r="M91" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Admin/WebContent.razor; Maliev.Intranet.Client/Pages/Admin/AdminPage.razor; Maliev.Intranet.Shared/Dtos/MalievPermissions.cs</x:v>
+      </x:c>
+      <x:c r="N91" t="str">
+        <x:v>/admin/web-content renders the Website Content page; /admin links to it; rows point to blog/article, homepage/marketing, product catalog, and chatbot instruction management routes.</x:v>
+      </x:c>
+      <x:c r="O91" t="str">
+        <x:v>No mutation endpoint is used by this page; the current behavior is a permission-gated UI inventory that points administrators to code-backed public content and service-owned surfaces.</x:v>
+      </x:c>
+      <x:c r="P91" t="str">
+        <x:v>NavigationTests includes /admin/web-content; Phase2NavLayoutTests assert admin/web-content, blog section, and homepage section links; ModuleRegressionSourceTests assert Admin page routes to /admin/system-health and instruction management while preserving Admin navigation structure.</x:v>
+      </x:c>
+      <x:c r="Q91" t="str">
+        <x:v>Intranet Client, Maliev.Web content files, CommerceService, ChatbotService</x:v>
+      </x:c>
+      <x:c r="R91" t="str">
+        <x:v>No user data is mutated by this page; it exposes content-surface metadata and management route targets.</x:v>
+      </x:c>
+      <x:c r="S91" t="str">
+        <x:v>Live browser retest pending for route rendering and content-surface links.</x:v>
+      </x:c>
+      <x:c r="T91" t="str">
+        <x:v>WebContent.razor:1-14,51-63,74-116; AdminPage.razor:55-76; MalievPermissions.cs:417-422; NavigationTests.cs:19; Phase2NavLayoutTests.cs:152-169; ModuleRegressionSourceTests.cs:169-181.</x:v>
+      </x:c>
+      <x:c r="U91" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31ef1e82accd4be9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6b7c97c48ec4e36"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14298,7 +14493,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9a2efbb12bc04581"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0e9b8cc07eb44e8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet delivery workflow stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R12debab7a5314521"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R8ac07f7207ba4b85"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R18201182c5da407f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Ra5d51cf5e2084b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R822e98f43fcf4030"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R0995b2f59dd84f01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R52e0b266f7e94723"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Raecb4767364c4b7c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>90</x:v>
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>210</x:v>
+        <x:v>213</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31b96d109fd14440"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e8657689bd748d4"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10554,10 +10554,205 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="92">
+      <x:c r="A92" t="str">
+        <x:v>INT-091</x:v>
+      </x:c>
+      <x:c r="B92" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C92" t="str">
+        <x:v>Delivery note list, pagination, status summary, and detail navigation</x:v>
+      </x:c>
+      <x:c r="D92" t="str">
+        <x:v>As an operations or finance employee, I can review outbound delivery notes, see shipment status at a glance, page through records, and open the delivery detail.</x:v>
+      </x:c>
+      <x:c r="E92" t="str">
+        <x:v>Delivery Notes opens from /finance/delivery-notes or /delivery-notes, shows matching-note, pending, in-transit, and delivered stat tiles, renders loading and error states, and displays a table of delivery note number, source order, customer, status, carrier, tracking number, item count, and delivery date. It reads page and pageSize from the query string, normalizes page size to 10, 20, or 50, updates the route when pagination changes, reloads from api/v1/deliverynotes, navigates table rows to /finance/delivery-notes/{DeliveryNoteId}, and shows an empty state with a Create Delivery Note action.</x:v>
+      </x:c>
+      <x:c r="F92" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G92" t="str">
+        <x:v>DeliveryServiceClient tests cover delivery-note pagination mapping and the registered DeliveryService client. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H92" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I92" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J92" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K92" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L92" t="str">
+        <x:v>DeliveryNoteList.razor -&gt; DeliveryNotesController GET -&gt; DeliveryServiceClient.GetDeliveryNotesAsync -&gt; DeliveryService /delivery/v1/delivery-notes pagination DTOs</x:v>
+      </x:c>
+      <x:c r="M92" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Delivery/DeliveryNoteList.razor; Maliev.Intranet.Bff/Controllers/DeliveryNotesController.cs; Maliev.Intranet.Bff/Clients/DeliveryServiceClient.cs; Maliev.Intranet.Shared/Dtos/DeliveryDtos.cs</x:v>
+      </x:c>
+      <x:c r="N92" t="str">
+        <x:v>/finance/delivery-notes and /delivery-notes render status summary tiles, paged delivery-note table, empty state, refresh action, New Delivery Note action, and row navigation to the detail page.</x:v>
+      </x:c>
+      <x:c r="O92" t="str">
+        <x:v>api/v1/deliverynotes returns PagedResponse&lt;DeliveryNoteSummaryDto&gt;; DeliveryServiceClient maps DeliveryService pagination from /delivery/v1/delivery-notes?page={page}&amp;pageSize={pageSize}&amp;sortBy=delivery_date&amp;sortOrder=desc and normalizes delivery note identifiers.</x:v>
+      </x:c>
+      <x:c r="P92" t="str">
+        <x:v>DeliveryServiceClientTests.GetDeliveryNotesAsync_MapsDeliveryServicePagination; ProgramHttpClientConfigurationTests.DeliveryNotesController_ClientInterface_IsRegistered.</x:v>
+      </x:c>
+      <x:c r="Q92" t="str">
+        <x:v>Intranet Client, Intranet BFF, DeliveryService</x:v>
+      </x:c>
+      <x:c r="R92" t="str">
+        <x:v>No mutation from the list page; reads delivery note summaries, pagination metadata, carrier/tracking fields, status, and delivery dates.</x:v>
+      </x:c>
+      <x:c r="S92" t="str">
+        <x:v>Live browser retest pending for pagination, reload, empty state, and row navigation.</x:v>
+      </x:c>
+      <x:c r="T92" t="str">
+        <x:v>DeliveryNoteList.razor:1-72,91-136,161; DeliveryNotesController.cs:23-35; DeliveryServiceClient.cs:85-109,318-333; DeliveryDtos.cs:8-50; DeliveryServiceClientTests.cs:13-55.</x:v>
+      </x:c>
+      <x:c r="U92" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="93">
+      <x:c r="A93" t="str">
+        <x:v>INT-092</x:v>
+      </x:c>
+      <x:c r="B93" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C93" t="str">
+        <x:v>Delivery note creation with shipment identity, item validation, and live courier rates</x:v>
+      </x:c>
+      <x:c r="D93" t="str">
+        <x:v>As an operations or finance employee, I can create shipment documentation from an order or purchase-order context and use live courier rates to populate carrier and shipping cost.</x:v>
+      </x:c>
+      <x:c r="E93" t="str">
+        <x:v>New Delivery Note opens at /finance/delivery-notes/new, loads reference currencies, countries, and couriers, defaults delivery date to tomorrow, Thailand, and THB, and captures order or purchase-order ID, customer ID/name, shipping address, contact details, instructions, parcel dimensions, carrier/tracking, shipping cost, and a delivered item. Fetch Rates validates destination address, city, province, postal code, contact phone, and positive parcel dimensions, builds a ShippingRateRequestDto from MALIEV origin and customer destination data, and posts to the shipping rates endpoint. Selecting a rate copies courier/product name, total price, currency, and courier code. Create validates order/purchase-order context, customer GUID, customer name, product code/name, and positive delivered quantity not exceeding ordered or manufactured quantity, posts api/v1/deliverynotes, and navigates to the created delivery note.</x:v>
+      </x:c>
+      <x:c r="F93" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G93" t="str">
+        <x:v>DeliveryServiceClient tests cover create DTO mapping and shipping courier/rate/tracking contracts; ShippingService tests cover the client-side shipping rates payload. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H93" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I93" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J93" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K93" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L93" t="str">
+        <x:v>DeliveryNoteNew.razor and ShippingService -&gt; reference data endpoints, api/v1/shipping/couriers, api/v1/shipping/rates, api/v1/deliverynotes -&gt; DeliveryNotesController Create -&gt; DeliveryServiceClient create and shipping DTO mappings</x:v>
+      </x:c>
+      <x:c r="M93" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Delivery/DeliveryNoteNew.razor; Maliev.Intranet.Client/Services/ShippingService.cs; Maliev.Intranet.Bff/Controllers/DeliveryNotesController.cs; Maliev.Intranet.Bff/Clients/DeliveryServiceClient.cs</x:v>
+      </x:c>
+      <x:c r="N93" t="str">
+        <x:v>/finance/delivery-notes/new renders shipment identity, destination/contact form, courier-rate action and results, parcel dimensions, delivery item entry, cancel, and create actions.</x:v>
+      </x:c>
+      <x:c r="O93" t="str">
+        <x:v>api/v1/referenceData/currencies, api/v1/referenceData/countries, api/v1/shipping/couriers, api/v1/shipping/rates, and api/v1/deliverynotes support the create flow; DeliveryServiceClient posts /delivery/v1/delivery-notes and maps shipment/customer/item fields plus shipping cost and instructions.</x:v>
+      </x:c>
+      <x:c r="P93" t="str">
+        <x:v>DeliveryServiceClientTests.CreateDeliveryNoteAsync_PostsDeliveryServiceContract; DeliveryServiceClientTests.GetShippingCouriersAsync_TargetsDeliveryServiceShippingCouriersRoute; DeliveryServiceClientTests.GetShippingRatesAsync_PostsDeliveryServiceShippingRateContract; DeliveryServiceClientTests.GetShippingTrackingAsync_TargetsDeliveryServiceTrackingRoute; ShippingServiceTests.GetRatesAsync_PostsDeliveryServiceShippingPayload; IntranetOrderFlowTests.CreateDeliveryNote_ReturnsCreatedWithDetail_WhenSuccessful.</x:v>
+      </x:c>
+      <x:c r="Q93" t="str">
+        <x:v>Intranet Client, Intranet BFF, DeliveryService, ReferenceDataService</x:v>
+      </x:c>
+      <x:c r="R93" t="str">
+        <x:v>Delivery note header, customer/shipping/contact fields, courier selection, shipping cost/currency, parcel request fields, delivery item and quantity data</x:v>
+      </x:c>
+      <x:c r="S93" t="str">
+        <x:v>Live browser retest pending for rate lookup, rate selection, validation errors, create success, and create failure messaging.</x:v>
+      </x:c>
+      <x:c r="T93" t="str">
+        <x:v>DeliveryNoteNew.razor:1,11,38-62,106,113-128,150-184,204-282,294-345; ShippingService.cs:30-45; DeliveryNotesController.cs:43-50; DeliveryServiceClient.cs:127-135,222-274,280-310; DeliveryServiceClientTests.cs:61-149,337-527; ShippingServiceTests.cs:14-83; IntranetOrderFlowTests.cs:384-413.</x:v>
+      </x:c>
+      <x:c r="U93" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94">
+      <x:c r="A94" t="str">
+        <x:v>INT-093</x:v>
+      </x:c>
+      <x:c r="B94" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C94" t="str">
+        <x:v>Delivery note detail status, PDF request, proof-file upload, and document access</x:v>
+      </x:c>
+      <x:c r="D94" t="str">
+        <x:v>As an operations or finance employee, I can inspect a delivery note, update shipment status, request the PDF, and attach proof-of-delivery documents.</x:v>
+      </x:c>
+      <x:c r="E94" t="str">
+        <x:v>Delivery note detail opens at /finance/delivery-notes/{DeliveryNoteId}, loads the detail and file list, shows shipment status, carrier/tracking, delivery contact/address/instructions, signature proof ID, item quantities, and attached files. It enables Mark In Transit only from Pending and Mark Delivered from InTransit or PartiallyDelivered, requires a received-by name when marking delivered, sends actual delivery time and signature file ID only for Delivered status, updates the local detail from the BFF response, and shows actionable failure messages. Request PDF posts to the delivery note PDF endpoint, stores the PDF request response, and reloads files. Proof upload accepts document or signature types, description, and PDF/image files up to 5 MB, posts multipart content to the delivery note files endpoint, updates the signature file ID when a Signature file is uploaded, refreshes the file list, and previews stored file URLs when provided.</x:v>
+      </x:c>
+      <x:c r="F94" t="str">
+        <x:v>Implemented in current code</x:v>
+      </x:c>
+      <x:c r="G94" t="str">
+        <x:v>DeliveryServiceClient tests cover status update, PDF generation, file list, download route, and multipart upload contracts; controller flow tests cover create and delivered-status updates. Tests were mapped as secondary evidence in this tracker slice but not rerun.</x:v>
+      </x:c>
+      <x:c r="H94" t="str">
+        <x:v>No current tracker error recorded.</x:v>
+      </x:c>
+      <x:c r="I94" t="str">
+        <x:v>No code fix in this tracker row; documented current behavior.</x:v>
+      </x:c>
+      <x:c r="J94" t="str">
+        <x:v>Manual browser retest pending.</x:v>
+      </x:c>
+      <x:c r="K94" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L94" t="str">
+        <x:v>DeliveryNoteDetail.razor -&gt; DeliveryNotesController detail/status/pdf/files/download endpoints -&gt; DeliveryServiceClient -&gt; DeliveryService status, PDF, file, and proof DTO contracts</x:v>
+      </x:c>
+      <x:c r="M94" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Delivery/DeliveryNoteDetail.razor; Maliev.Intranet.Bff/Controllers/DeliveryNotesController.cs; Maliev.Intranet.Bff/Clients/DeliveryServiceClient.cs; Maliev.Intranet.Shared/Dtos/DeliveryDtos.cs</x:v>
+      </x:c>
+      <x:c r="N94" t="str">
+        <x:v>/finance/delivery-notes/{DeliveryNoteId} renders delivery status controls, received-by and actual-delivery inputs, item table, proof file upload, file table, preview links, PDF request, reload, and not-found/error states.</x:v>
+      </x:c>
+      <x:c r="O94" t="str">
+        <x:v>api/v1/deliverynotes/{id}, api/v1/deliverynotes/{id}/status, api/v1/deliverynotes/{id}/pdf, api/v1/deliverynotes/{id}/files, and api/v1/deliverynotes/{id}/files/{fileId}/download proxy DeliveryService detail, status, PDF, file-list, upload, and download routes.</x:v>
+      </x:c>
+      <x:c r="P94" t="str">
+        <x:v>DeliveryServiceClientTests.UpdateDeliveryStatusAsync_PostsDeliveryStatusContract; DeliveryServiceClientTests.GeneratePdfAsync_TargetsDeliveryServiceGenerateRoute; DeliveryServiceClientTests.GetFilesAsync_MapsDeliveryServiceFiles; DeliveryServiceClientTests.DownloadFileAsync_CallsDeliveryServiceDownloadRoute; DeliveryServiceClientTests.UploadFileAsync_PostsDeliveryServiceMultipartFileContract; IntranetOrderFlowTests.UpdateDeliveryStatus_ToDelivered_ReturnsOk_WhenSuccessful.</x:v>
+      </x:c>
+      <x:c r="Q94" t="str">
+        <x:v>Intranet Client, Intranet BFF, DeliveryService</x:v>
+      </x:c>
+      <x:c r="R94" t="str">
+        <x:v>Delivery status, received-by name, actual delivery time, signature file ID, PDF request metadata, proof-file metadata, stored file URLs</x:v>
+      </x:c>
+      <x:c r="S94" t="str">
+        <x:v>Live browser retest pending for status transitions, PDF request, proof upload, signature-file selection, and file preview/download.</x:v>
+      </x:c>
+      <x:c r="T94" t="str">
+        <x:v>DeliveryNoteDetail.razor:1,11,35-49,68,106-154,184-199,201-215,223-255,275-333,338; DeliveryNotesController.cs:34-35,56-69,78-93,111-136; DeliveryServiceClient.cs:109-186,193-215,310-333; DeliveryDtos.cs:56-161,212-248,358-380; DeliveryServiceClientTests.cs:149-322; IntranetOrderFlowTests.cs:423-471.</x:v>
+      </x:c>
+      <x:c r="U94" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf6b7c97c48ec4e36"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b1f99361bd24e9c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14493,7 +14688,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb0e9b8cc07eb44e8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R262d60450a3d463f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet contact request workflow stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R822e98f43fcf4030"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R0995b2f59dd84f01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R52e0b266f7e94723"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Raecb4767364c4b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3e96b4001b224b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re566e303d6f040ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R58938734cfb54538"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R42296d34d7ef44db"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>93</x:v>
+        <x:v>96</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>213</x:v>
+        <x:v>216</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e8657689bd748d4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R931067bac7ac4f7c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10749,10 +10749,205 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="95">
+      <x:c r="A95" t="str">
+        <x:v>INT-094</x:v>
+      </x:c>
+      <x:c r="B95" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C95" t="str">
+        <x:v>Contact request inbox</x:v>
+      </x:c>
+      <x:c r="D95" t="str">
+        <x:v>As an employee, I can review website contact requests in a filtered, paginated queue.</x:v>
+      </x:c>
+      <x:c r="E95" t="str">
+        <x:v>The contact request list opens from the sales contact-request route, requires contact-request read permission, shows matching/new/in-progress/resolved counters from the loaded page, lets employees filter by lifecycle status and email, persists page/pageSize/status/email into the URL, normalizes page size to 10/20/50 in the client, calls the BFF list endpoint with encoded query values, shows loading and warning states, and navigates a selected row to the request detail page.</x:v>
+      </x:c>
+      <x:c r="F95" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G95" t="str">
+        <x:v>Mapped to current UI/BFF/client/DTO code; focused controller permission tests cover the read endpoint permission. No browser execution in this slice.</x:v>
+      </x:c>
+      <x:c r="H95" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I95" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J95" t="str">
+        <x:v>Pending live browser retest of status/email filters, pagination, row navigation, and empty/error states.</x:v>
+      </x:c>
+      <x:c r="K95" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L95" t="str">
+        <x:v>ContactRequestList.razor route/query state -&gt; Intranet BFF ContactRequestsController GET api/v1/contactrequests -&gt; ContactRequestServiceClient GET /contact/v1/contacts -&gt; ContactService contact request list DTOs</x:v>
+      </x:c>
+      <x:c r="M95" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Contacts/ContactRequestList.razor; Maliev.Intranet.Bff/Controllers/ContactRequestsController.cs; Maliev.Intranet.Bff/Clients/ContactRequestServiceClient.cs; Maliev.Intranet.Shared/Dtos/ContactRequestDtos.cs</x:v>
+      </x:c>
+      <x:c r="N95" t="str">
+        <x:v>/sales/contact-requests and /contact-requests routes; RequirePermission ContactRequest.Read; ModuleHeader, StatBar, status/email filters, Clear/Apply actions, table rows, PaginationFooter, row click navigation to /sales/contact-requests/{id}</x:v>
+      </x:c>
+      <x:c r="O95" t="str">
+        <x:v>GET api/v1/contactrequests accepts page, pageSize, status, and email; ContactRequestServiceClient calls /contact/v1/contacts with normalized page size and encoded email, normalizes missing public references to MLV-C-{id}, and returns PagedResponse metadata.</x:v>
+      </x:c>
+      <x:c r="P95" t="str">
+        <x:v>ContactRequestsControllerTests.ContactRequestEndpoints_RequireContactPermissions verifies GetAsync requires ContactRequest.Read; ModuleRegressionSourceTests reads ContactRequestList source as page regression evidence.</x:v>
+      </x:c>
+      <x:c r="Q95" t="str">
+        <x:v>Intranet Client, Intranet BFF, ContactService</x:v>
+      </x:c>
+      <x:c r="R95" t="str">
+        <x:v>URL query state only; no contact request mutation from the list view.</x:v>
+      </x:c>
+      <x:c r="S95" t="str">
+        <x:v>Needs live browser retest and downstream ContactService pagination contract confirmation because the BFF currently wraps the returned list count into one-page PagedResponse metadata.</x:v>
+      </x:c>
+      <x:c r="T95" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Contacts/ContactRequestList.razor:1,3,11,17,28,36,63,76,103,143,175,198,206,215,232; Maliev.Intranet.Bff/Controllers/ContactRequestsController.cs:19,26,28,35; Maliev.Intranet.Bff/Clients/ContactRequestServiceClient.cs:14,47,56,65,71,148; Maliev.Intranet.Shared/Dtos/ContactRequestDtos.cs:6,21,36,49; Maliev.Intranet.Tests/Bff/Controllers/ContactRequestsControllerTests.cs:69</x:v>
+      </x:c>
+      <x:c r="U95" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="96">
+      <x:c r="A96" t="str">
+        <x:v>INT-095</x:v>
+      </x:c>
+      <x:c r="B96" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C96" t="str">
+        <x:v>Contact request detail lifecycle and attachments</x:v>
+      </x:c>
+      <x:c r="D96" t="str">
+        <x:v>As an employee, I can open a website contact request, inspect customer details and attachments, and update its lifecycle or priority.</x:v>
+      </x:c>
+      <x:c r="E96" t="str">
+        <x:v>The detail page loads a single contact request by id, requires contact-request read permission, shows loading/not-found/error states, displays status, priority, attachment count, received/updated timestamps, sender identity, subject, message, and contact type, supports Start work, Resolve, Close, and explicit status/priority save actions, PATCHes status and optional priority through the BFF, refreshes the returned request state, and exposes attachment download links that open the BFF download route in a new tab with file name, object name, content type, size, and upload time visible.</x:v>
+      </x:c>
+      <x:c r="F96" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G96" t="str">
+        <x:v>Mapped to current detail UI, BFF endpoints, downstream client, and DTOs; focused controller permission tests cover get/update/download permissions. No browser execution in this slice.</x:v>
+      </x:c>
+      <x:c r="H96" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I96" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J96" t="str">
+        <x:v>Pending live browser retest of detail load, lifecycle buttons, manual lifecycle save, attachment table, and file download route.</x:v>
+      </x:c>
+      <x:c r="K96" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L96" t="str">
+        <x:v>ContactRequestDetail.razor detail/lifecycle/attachment UI -&gt; Intranet BFF ContactRequestsController GET/PATCH/download -&gt; ContactRequestServiceClient GET/PUT/download -&gt; ContactService contact request/file endpoints</x:v>
+      </x:c>
+      <x:c r="M96" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Contacts/ContactRequestDetail.razor; Maliev.Intranet.Bff/Controllers/ContactRequestsController.cs; Maliev.Intranet.Bff/Clients/ContactRequestServiceClient.cs; Maliev.Intranet.Shared/Dtos/ContactRequestDtos.cs</x:v>
+      </x:c>
+      <x:c r="N96" t="str">
+        <x:v>/sales/contact-requests/{ContactRequestId:int}; RequirePermission ContactRequest.Read; lifecycle toolbar, status/priority selects, Save lifecycle, Customer request panel, Attachments table, Download link to api/v1/contactrequests/{id}/files/{fileId}/download</x:v>
+      </x:c>
+      <x:c r="O96" t="str">
+        <x:v>GET api/v1/contactrequests/{id} returns NotFound or ContactRequestDto; PATCH api/v1/contactrequests/{id}/status requires ContactRequest.Update and forwards status/priority; GET api/v1/contactrequests/{id}/files/{fileId}/download returns file content, content type, and resolved file name or NotFound.</x:v>
+      </x:c>
+      <x:c r="P96" t="str">
+        <x:v>ContactRequestsControllerTests.ContactRequestEndpoints_RequireContactPermissions verifies GetByIdAsync and DownloadFileAsync require ContactRequest.Read and UpdateStatusAsync requires ContactRequest.Update.</x:v>
+      </x:c>
+      <x:c r="Q96" t="str">
+        <x:v>Intranet Client, Intranet BFF, ContactService</x:v>
+      </x:c>
+      <x:c r="R96" t="str">
+        <x:v>Contact request lifecycle status and priority; attachment download response stream.</x:v>
+      </x:c>
+      <x:c r="S96" t="str">
+        <x:v>Needs live browser retest and downstream file authorization/scoping confirmation against ContactService.</x:v>
+      </x:c>
+      <x:c r="T96" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Contacts/ContactRequestDetail.razor:1,2,18,27,35,48,56,72,92,102,121,151,191,213,218,230,284; Maliev.Intranet.Bff/Controllers/ContactRequestsController.cs:42,44,53,55,112,114; Maliev.Intranet.Bff/Clients/ContactRequestServiceClient.cs:86,104,126,144,148,159; Maliev.Intranet.Shared/Dtos/ContactRequestDtos.cs:49,97,103,130; Maliev.Intranet.Tests/Bff/Controllers/ContactRequestsControllerTests.cs:69</x:v>
+      </x:c>
+      <x:c r="U96" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="97">
+      <x:c r="A97" t="str">
+        <x:v>INT-096</x:v>
+      </x:c>
+      <x:c r="B97" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C97" t="str">
+        <x:v>Contact request employee reply</x:v>
+      </x:c>
+      <x:c r="D97" t="str">
+        <x:v>As an employee, I can send a reply to a website contact requester and optionally mark the request resolved.</x:v>
+      </x:c>
+      <x:c r="E97" t="str">
+        <x:v>The detail page requires a non-empty reply message before enabling send, posts the reply text and mark-resolved choice to the BFF, shows warning feedback for failed sends, clears the reply box on success, updates the displayed status from the response, and uses the BFF to trim and dispatch a NotificationService direct-email event with contact recipient, subject/reference, contact id, and reply message parameters; when mark-resolved is selected, the BFF updates the contact request status to Resolved while preserving the contact priority.</x:v>
+      </x:c>
+      <x:c r="F97" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G97" t="str">
+        <x:v>Focused controller test covers valid reply dispatch, direct-email payload shape, template id, target user, and mark-resolved lifecycle update.</x:v>
+      </x:c>
+      <x:c r="H97" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I97" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J97" t="str">
+        <x:v>Pending live browser retest of disabled send state, successful reply snackbar, status update, and NotificationService delivery path in an integrated environment.</x:v>
+      </x:c>
+      <x:c r="K97" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L97" t="str">
+        <x:v>ContactRequestDetail.razor reply form -&gt; Intranet BFF ContactRequestsController POST reply -&gt; INotificationServiceClient NotificationEvent -&gt; ContactRequestServiceClient optional resolved status update -&gt; ContactService lifecycle state</x:v>
+      </x:c>
+      <x:c r="M97" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Contacts/ContactRequestDetail.razor; Maliev.Intranet.Bff/Controllers/ContactRequestsController.cs; Maliev.Intranet.Shared/Dtos/ContactRequestDtos.cs; Maliev.Intranet.Tests/Bff/Controllers/ContactRequestsControllerTests.cs</x:v>
+      </x:c>
+      <x:c r="N97" t="str">
+        <x:v>Reply from Intranet panel with textarea, Mark resolved after sending checkbox, disabled Send reply command until text is present, and success/warning snackbar feedback.</x:v>
+      </x:c>
+      <x:c r="O97" t="str">
+        <x:v>POST api/v1/contactrequests/{id}/reply requires ContactRequest.Update, rejects blank ReplyMessage, loads the contact, dispatches NotificationEvent type ContactMessageEmployeeReply with template contact-message-employee-reply and direct-email target, optionally PUTs resolved status through ContactService, then returns ContactRequestReplyResponse.</x:v>
+      </x:c>
+      <x:c r="P97" t="str">
+        <x:v>ContactRequestsControllerTests.SendReplyAsync_ValidRequest_DispatchesDirectEmailReplyAndMarksResolved; ContactRequestsControllerTests.ContactRequestEndpoints_RequireContactPermissions verifies SendReplyAsync requires ContactRequest.Update.</x:v>
+      </x:c>
+      <x:c r="Q97" t="str">
+        <x:v>Intranet Client, Intranet BFF, ContactService, NotificationService</x:v>
+      </x:c>
+      <x:c r="R97" t="str">
+        <x:v>NotificationEvent for customer reply; optional contact request status mutation to Resolved.</x:v>
+      </x:c>
+      <x:c r="S97" t="str">
+        <x:v>Needs integrated NotificationService delivery verification and browser retest; tracker currently documents the code path and focused controller coverage only.</x:v>
+      </x:c>
+      <x:c r="T97" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Contacts/ContactRequestDetail.razor:126,130,138,256,268,277; Maliev.Intranet.Bff/Controllers/ContactRequestsController.cs:67,69,75,79,84,88,92,101,122,143; Maliev.Intranet.Shared/Dtos/ContactRequestDtos.cs:142,154; Maliev.Intranet.Tests/Bff/Controllers/ContactRequestsControllerTests.cs:13,41,53,59,69</x:v>
+      </x:c>
+      <x:c r="U97" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8b1f99361bd24e9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc132b970f6bd4522"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14688,7 +14883,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R262d60450a3d463f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re621299c3a7c489b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet HR profile and leave stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R3e96b4001b224b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Re566e303d6f040ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R58938734cfb54538"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R42296d34d7ef44db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R749cc9003bad4452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R006a092a0b7b4b38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Ra280d321180643b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R554dd43226e14bd9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>96</x:v>
+        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>216</x:v>
+        <x:v>220</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R931067bac7ac4f7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R627682a97033414c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -10944,10 +10944,270 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="98">
+      <x:c r="A98" t="str">
+        <x:v>INT-097</x:v>
+      </x:c>
+      <x:c r="B98" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C98" t="str">
+        <x:v>Employee self-service profile overview and editable contact details</x:v>
+      </x:c>
+      <x:c r="D98" t="str">
+        <x:v>As an employee, I can view my employee profile and update my permitted self-service contact fields.</x:v>
+      </x:c>
+      <x:c r="E98" t="str">
+        <x:v>The HR profile route loads employee detail, self-service profile, and scoped preference data together; shows loading, warning, and missing-profile states; displays profile/preferences tabs, status, department, job title, manager, employee details, team assignments, and employee documents; and lets the employee edit preferred name, personal email, and mobile phone. Saving sends a PUT to the self-service profile endpoint, refreshes the returned self-profile values, exits edit mode on success, and shows failure feedback without mutating the visible state.</x:v>
+      </x:c>
+      <x:c r="F98" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G98" t="str">
+        <x:v>Mapped to current HR profile UI, Employees BFF controller, EmployeeServiceClient, DTOs, and focused client/BFF/client tests.</x:v>
+      </x:c>
+      <x:c r="H98" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I98" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J98" t="str">
+        <x:v>Pending live browser retest of profile load, edit/cancel/save states, validation messages, team/document empty states, and employee-service error handling.</x:v>
+      </x:c>
+      <x:c r="K98" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L98" t="str">
+        <x:v>Profile.razor profile tab -&gt; EmployeesController me/profile endpoints -&gt; EmployeeServiceClient self-service profile contract -&gt; EmployeeService profile storage and principal claim resolution</x:v>
+      </x:c>
+      <x:c r="M98" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Profile.razor; Maliev.Intranet.Bff/Controllers/EmployeesController.cs; Maliev.Intranet.Bff/Clients/EmployeeServiceClient.cs; Maliev.Intranet.Shared/Dtos/HRDtos.cs</x:v>
+      </x:c>
+      <x:c r="N98" t="str">
+        <x:v>/hr/profile route; profile/preference tab navigation; employee details card; edit profile command; preferred name, personal email, mobile phone fields; Save changes and Cancel actions; teams and documents panels.</x:v>
+      </x:c>
+      <x:c r="O98" t="str">
+        <x:v>GET api/v1/employees/me enriches current profile from principal claims and IAM created-at data; GET api/v1/employees/me/profile resolves the current employee and reads /employee/v1/profile/{employeeId}/profile; PUT api/v1/employees/me/profile forwards allowed self-profile fields and rereads the profile after update.</x:v>
+      </x:c>
+      <x:c r="P98" t="str">
+        <x:v>HrProfilePageTests.Profile_RendersSelfServiceEditFields; HrProfilePageTests.Profile_SaveProfile_PutsSelfServiceProfileRequest; EmployeesControllerProfileTests.GetMyProfile_UsesCookieNameIdentifierClaim; EmployeeServiceClientTests.GetSelfServiceProfileAsync_UsesEmployeeServiceProfileContract; EmployeeServiceClientTests.UpdateSelfServiceProfileAsync_UsesEmployeeServiceProfileContract.</x:v>
+      </x:c>
+      <x:c r="Q98" t="str">
+        <x:v>Intranet Client, Intranet BFF, EmployeeService, IAMService</x:v>
+      </x:c>
+      <x:c r="R98" t="str">
+        <x:v>Employee self-profile preferred name, personal email, mobile phone, and optional profile image URL; read-only employee detail/team/document display state.</x:v>
+      </x:c>
+      <x:c r="S98" t="str">
+        <x:v>Needs integrated authorization and browser verification against EmployeeService; current focused tests cover source behavior and request shape but not full host/browser execution.</x:v>
+      </x:c>
+      <x:c r="T98" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Profile.razor:1,34,190,209,213,435,436,463,496,501; Maliev.Intranet.Bff/Controllers/EmployeesController.cs:88,89,96,105,122,173,188; Maliev.Intranet.Bff/Clients/EmployeeServiceClient.cs:101,112,215; Maliev.Intranet.Shared/Dtos/HRDtos.cs:49,101,112; Maliev.Intranet.Tests/Client/Pages/HrProfilePageTests.cs:42,76; Maliev.Intranet.Tests/Bff/Controllers/EmployeesControllerProfileTests.cs:128; Maliev.Intranet.Tests/Bff/Clients/EmployeeServiceClientTests.cs:70,114</x:v>
+      </x:c>
+      <x:c r="U98" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" t="str">
+        <x:v>INT-098</x:v>
+      </x:c>
+      <x:c r="B99" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C99" t="str">
+        <x:v>Scoped profile workspace preferences and email signatures</x:v>
+      </x:c>
+      <x:c r="D99" t="str">
+        <x:v>As an employee, I can save personal workspace defaults and email signatures that follow my intranet login.</x:v>
+      </x:c>
+      <x:c r="E99" t="str">
+        <x:v>The preferences tab opens from /hr/profile?tab=preferences, shows the intranet-profile scope, configured-key count, last-saved label, and workspace-default fields for theme, start page, default currency, language, time zone, date format, compact workspace, operational digest, full email signature, and short email signature. It loads saved preferences or builds defaults from employee/profile data, validates signature length, saves a scoped preference payload, applies theme/date/time-zone/density defaults through LayoutService, applies the selected currency through CurrencyService, and returns an empty scoped preference instead of a 404 when no saved preference exists.</x:v>
+      </x:c>
+      <x:c r="F99" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G99" t="str">
+        <x:v>Mapped to current profile preferences UI, Preferences BFF controller, EmployeeService preference mapping, DTOs, and focused client/controller/client tests.</x:v>
+      </x:c>
+      <x:c r="H99" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I99" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J99" t="str">
+        <x:v>Pending live browser retest of preference reload/save, layout preference application, currency switching, and saved signature persistence in an integrated session.</x:v>
+      </x:c>
+      <x:c r="K99" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L99" t="str">
+        <x:v>Profile.razor preferences tab -&gt; PreferencesController scoped endpoints -&gt; EmployeeServiceClient preference JSON-string mapping -&gt; EmployeeService preference storage -&gt; LayoutService/CurrencyService local application</x:v>
+      </x:c>
+      <x:c r="M99" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Profile.razor; Maliev.Intranet.Bff/Controllers/PreferencesController.cs; Maliev.Intranet.Bff/Clients/EmployeeServiceClient.cs; Maliev.Intranet.Shared/Dtos/PreferenceDtos.cs; Maliev.Intranet.Client/Services/LayoutService.cs; Maliev.Intranet.Client/Services/CurrencyService.cs</x:v>
+      </x:c>
+      <x:c r="N99" t="str">
+        <x:v>/hr/profile?tab=preferences; Workspace defaults form; preference selects/toggles; full and short signature textareas with counters; Reload and Save preferences commands; profile summary link to Edit preferences.</x:v>
+      </x:c>
+      <x:c r="O99" t="str">
+        <x:v>GET api/v1/preferences/{scope} requires Employee.ProfileRead and returns an empty UserPreferenceDto when no scoped preference exists; PUT api/v1/preferences/{scope} requires Employee.ProfileUpdate and forwards PreferenceData as EmployeeService preferenceData JSON; Profile.razor builds and applies workspace preferences after save or reload.</x:v>
+      </x:c>
+      <x:c r="P99" t="str">
+        <x:v>HrProfilePageTests.Profile_PreferencesQueryTab_RendersPreferenceEditor; HrProfilePageTests.Profile_PreferencesQueryTab_DefaultsSignaturesFromEmployeeProfile; HrProfilePageTests.Profile_SavePreferences_PutsScopedPreferenceRequest; PreferencesControllerTests.PreferenceEndpoints_RequireEmployeeProfilePermissions; EmployeeServiceClientTests.GetPreferenceAsync_MapsEmployeeServiceJsonStringPayload; EmployeeServiceClientTests.UpsertPreferenceAsync_SendsEmployeeServiceJsonStringPayload.</x:v>
+      </x:c>
+      <x:c r="Q99" t="str">
+        <x:v>Intranet Client, Intranet BFF, EmployeeService, reference-data currency endpoint</x:v>
+      </x:c>
+      <x:c r="R99" t="str">
+        <x:v>UserPreferenceDto for intranet-profile scope; preference keys for themeMode, landingPage, defaultCurrency, language, timeZone, dateFormat, compactWorkspace, operationalDigest, emailSignature, and shortEmailSignature.</x:v>
+      </x:c>
+      <x:c r="S99" t="str">
+        <x:v>Needs live browser retest and end-to-end persistence verification across sign-out/sign-in; no app code changed in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="T99" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Profile.razor:45,58,66,82,190,256,403,437,533,539,551,561,564,596,611,627,636,783; Maliev.Intranet.Bff/Controllers/PreferencesController.cs:15,22,24,41,43,52,54; Maliev.Intranet.Bff/Clients/EmployeeServiceClient.cs:143,156,247,263,281; Maliev.Intranet.Shared/Dtos/PreferenceDtos.cs:8,26; Maliev.Intranet.Tests/Client/Pages/HrProfilePageTests.cs:99,117,138; Maliev.Intranet.Tests/Bff/Controllers/PreferencesControllerTests.cs:14; Maliev.Intranet.Tests/Bff/Clients/EmployeeServiceClientTests.cs:151,190</x:v>
+      </x:c>
+      <x:c r="U99" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="100">
+      <x:c r="A100" t="str">
+        <x:v>INT-099</x:v>
+      </x:c>
+      <x:c r="B100" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C100" t="str">
+        <x:v>Leave balances, request history, and leave submission</x:v>
+      </x:c>
+      <x:c r="D100" t="str">
+        <x:v>As an employee, I can review my leave balances and submit a new leave request from the HR leave page.</x:v>
+      </x:c>
+      <x:c r="E100" t="str">
+        <x:v>The Leave Management route loads balances, my requests, and pending approvals together; shows available, used, request, and approval totals; renders balance and request tables with empty states; and provides a request form for Annual, Sick, Personal, and Unpaid leave. The duration control supports full day, morning, and afternoon selections, half-day choices keep the end date equal to the start date, and the form posts leave type, start date, end date, half-day period, and reason. On success, the form resets to a planned annual leave seven days ahead, reloads the page data, and shows success feedback; on downstream rejection, the page displays the returned API message.</x:v>
+      </x:c>
+      <x:c r="F100" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G100" t="str">
+        <x:v>Mapped to current leave UI, TimeOff BFF controller, LeaveServiceClient mapping, leave DTOs, and focused client tests for LeaveService payload and error mapping.</x:v>
+      </x:c>
+      <x:c r="H100" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I100" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J100" t="str">
+        <x:v>Pending live browser retest of leave form validation, half-day behavior, submission success/reload, and downstream insufficient-balance error display.</x:v>
+      </x:c>
+      <x:c r="K100" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L100" t="str">
+        <x:v>Leave.razor balances/request UI -&gt; TimeOffController current-employee resolution -&gt; LeaveServiceClient LeaveService contracts -&gt; LeaveService balance/request storage</x:v>
+      </x:c>
+      <x:c r="M100" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Leave.razor; Maliev.Intranet.Bff/Controllers/TimeOffController.cs; Maliev.Intranet.Bff/Clients/LeaveServiceClient.cs; Maliev.Intranet.Shared/Dtos/LeaveDtos.cs; Maliev.Intranet.Shared/Dtos/HRDtos.cs</x:v>
+      </x:c>
+      <x:c r="N100" t="str">
+        <x:v>/hr/leave route; stat tiles for Available/Used/Requests/Approvals; Request leave card; duration radio group; start/end date fields; Reason textarea; Balances and My leave requests tables; loading/error/empty states.</x:v>
+      </x:c>
+      <x:c r="O100" t="str">
+        <x:v>GET api/v1/timeoff/balances requires Leave.BalanceRead; GET api/v1/timeoff/requests requires Leave.RequestsRead and uses the current UTC year; POST api/v1/timeoff/requests requires Leave.Write, resolves the employee and optional manager approver, posts numeric snake_case LeaveService payload fields, and converts downstream rejection into ApiErrorResponse.</x:v>
+      </x:c>
+      <x:c r="P100" t="str">
+        <x:v>LeaveServiceClientTests.GetMyRequestsAsync_MapsSnakeCaseEnumPayload; LeaveServiceClientTests.SubmitRequestAsync_SendsSnakeCaseNumericPayloadWithTrustedApprover; LeaveServiceClientTests.SubmitRequestAsync_WhenDownstreamRejects_PreservesErrorMessage; shared DTO serialization tests cover LeaveBalanceDto, SubmitLeaveRequestDto, and LeaveRequestSummaryDto.</x:v>
+      </x:c>
+      <x:c r="Q100" t="str">
+        <x:v>Intranet Client, Intranet BFF, EmployeeService, LeaveService</x:v>
+      </x:c>
+      <x:c r="R100" t="str">
+        <x:v>Leave request submission; leave balance and request list reads; API error message surfaced into page state.</x:v>
+      </x:c>
+      <x:c r="S100" t="str">
+        <x:v>Needs live browser retest and BFF controller-level coverage for current-employee resolution and permission branches.</x:v>
+      </x:c>
+      <x:c r="T100" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Leave.razor:1,10,26,34,35,49,52,83,109,165,183,184,204,210,213,219,270,285,295,320; Maliev.Intranet.Bff/Controllers/TimeOffController.cs:17,20,53,55,67,69,81,83,94; Maliev.Intranet.Bff/Clients/LeaveServiceClient.cs:46,71,113,122,134,138,141,150,249,265; Maliev.Intranet.Shared/Dtos/LeaveDtos.cs:10,31; Maliev.Intranet.Shared/Dtos/HRDtos.cs:443,456; Maliev.Intranet.Tests/Bff/Clients/LeaveServiceClientTests.cs:13,46,85</x:v>
+      </x:c>
+      <x:c r="U100" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="101">
+      <x:c r="A101" t="str">
+        <x:v>INT-100</x:v>
+      </x:c>
+      <x:c r="B101" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C101" t="str">
+        <x:v>Leave pending approvals and manager decision submission</x:v>
+      </x:c>
+      <x:c r="D101" t="str">
+        <x:v>As a manager, I can review pending leave requests assigned to me and approve a request from the leave page.</x:v>
+      </x:c>
+      <x:c r="E101" t="str">
+        <x:v>The Leave Management page loads pending approvals for the current employee, includes the approval count in the stat bar, shows an empty state when no approvals are assigned, and renders each pending approval with leave type, date range, reason, and an Approve request action. Approving posts a decision payload with Decision set to Approved and a standard Intranet comment, shows failure feedback when the BFF rejects the decision, shows success feedback on approval, and reloads balances, requests, and approvals afterward.</x:v>
+      </x:c>
+      <x:c r="F101" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G101" t="str">
+        <x:v>Mapped to current leave UI, TimeOff BFF decision endpoint, LeaveServiceClient decision contract, and route/source tests; no focused approval-decision unit test was found in this slice.</x:v>
+      </x:c>
+      <x:c r="H101" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I101" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J101" t="str">
+        <x:v>Pending focused automated coverage and live browser retest for manager approval permissions, decision failure messages, and post-approval reload.</x:v>
+      </x:c>
+      <x:c r="K101" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L101" t="str">
+        <x:v>Leave.razor pending approvals panel -&gt; TimeOffController approvals/decision endpoints -&gt; LeaveServiceClient manager approval contracts -&gt; LeaveService decision workflow</x:v>
+      </x:c>
+      <x:c r="M101" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Leave.razor; Maliev.Intranet.Bff/Controllers/TimeOffController.cs; Maliev.Intranet.Bff/Clients/LeaveServiceClient.cs; Maliev.Intranet.Shared/Dtos/LeaveDtos.cs</x:v>
+      </x:c>
+      <x:c r="N101" t="str">
+        <x:v>Pending approvals panel on /hr/leave; approval count stat tile; Approve request button per approval row; loading/error/empty state behavior reused from the leave page.</x:v>
+      </x:c>
+      <x:c r="O101" t="str">
+        <x:v>GET api/v1/timeoff/approvals requires Leave.RequestsRead and calls /leave/v1/LeaveRequests/pending/{managerId}; POST api/v1/timeoff/requests/{requestId}/decision requires Leave.Approve and calls /leave/v1/LeaveRequests/{requestId}/decision?approverId={employeeId} with numeric decision mapping for approve/reject.</x:v>
+      </x:c>
+      <x:c r="P101" t="str">
+        <x:v>ModuleRegressionSourceTests confirms the leave navigation and segmented duration source shape; ControllerRouteTests includes /api/v1/timeoff/balances. No focused approval-decision unit test was found during this slice.</x:v>
+      </x:c>
+      <x:c r="Q101" t="str">
+        <x:v>Intranet Client, Intranet BFF, EmployeeService, LeaveService</x:v>
+      </x:c>
+      <x:c r="R101" t="str">
+        <x:v>Leave approval decision mutation and pending approval reads.</x:v>
+      </x:c>
+      <x:c r="S101" t="str">
+        <x:v>Needs focused BFF/client test coverage for ProcessDecisionAsync and a live browser retest for approval action behavior.</x:v>
+      </x:c>
+      <x:c r="T101" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Hr/Leave.razor:1,26,29,135,150,183,185,234,241,250; Maliev.Intranet.Bff/Controllers/TimeOffController.cs:17,20,116,118,130,132,140; Maliev.Intranet.Bff/Clients/LeaveServiceClient.cs:30,35,176,189,193,273; Maliev.Intranet.Shared/Dtos/LeaveDtos.cs:54,75; Maliev.Intranet.Tests/Client/Pages/ModuleRegressionSourceTests.cs:322,337; Maliev.Intranet.Tests/Bff/ControllerRouteTests.cs:26</x:v>
+      </x:c>
+      <x:c r="U101" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc132b970f6bd4522"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18075dab11694cbe"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14883,7 +15143,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re621299c3a7c489b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd5d488a621a46cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet HR API surface stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R749cc9003bad4452"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R006a092a0b7b4b38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Ra280d321180643b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R554dd43226e14bd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9de72b969f924e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4b6177341b134650"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rfc0f259de56349be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R239002755bb643b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>100</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>220</x:v>
+        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4606,7 +4606,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R627682a97033414c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R331b3105df084e69"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11204,10 +11204,270 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="102">
+      <x:c r="A102" t="str">
+        <x:v>INT-101</x:v>
+      </x:c>
+      <x:c r="B102" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C102" t="str">
+        <x:v>Compliance records, alerts, statistics, and resolution</x:v>
+      </x:c>
+      <x:c r="D102" t="str">
+        <x:v>As a compliance or HR employee, I can review compliance alert-derived records, see compliance statistics, and resolve a record through the Intranet BFF.</x:v>
+      </x:c>
+      <x:c r="E102" t="str">
+        <x:v>The compliance API requires compliance read permission for stats, list, and detail reads, and compliance write permission for create and delete/resolve operations. Stats map ComplianceService report values into expiring-30-days, expiring-60-days, and total-active counts. The record list reads unresolved compliance alerts, maps alert id, employee id, alert type, created date, and severity/status into paged ComplianceRecordDto rows, and supports detail lookup by id. Delete resolves the downstream alert with an Intranet resolution note, while the current create path returns BadRequest unless the downstream client can create a record.</x:v>
+      </x:c>
+      <x:c r="F102" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G102" t="str">
+        <x:v>Focused compliance controller and client tests cover empty stats fallback, created-at route response, delete failure, permissions, unresolved alert mapping, report-to-stats mapping, and resolve request shape.</x:v>
+      </x:c>
+      <x:c r="H102" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I102" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J102" t="str">
+        <x:v>Pending live API/browser workflow retest; current client code does not expose a dedicated compliance Blazor page.</x:v>
+      </x:c>
+      <x:c r="K102" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L102" t="str">
+        <x:v>ComplianceController BFF endpoints -&gt; ComplianceServiceClient -&gt; ComplianceService compliance-alert and compliance-report contracts -&gt; Compliance DTOs</x:v>
+      </x:c>
+      <x:c r="M102" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/ComplianceController.cs; Maliev.Intranet.Bff/Clients/ComplianceServiceClient.cs; Maliev.Intranet.Shared/Dtos/ComplianceDtos.cs</x:v>
+      </x:c>
+      <x:c r="N102" t="str">
+        <x:v>No current dedicated Blazor page was found under Maliev.Intranet.Client/Pages for compliance; the current entry point is api/v1/compliance plus permissions.</x:v>
+      </x:c>
+      <x:c r="O102" t="str">
+        <x:v>GET api/v1/compliance/stats, GET api/v1/compliance, GET api/v1/compliance/{id}, POST api/v1/compliance, and DELETE api/v1/compliance/{id}; downstream calls /compliance/v1/compliance-alerts?isResolved=false, /compliance/v1/compliance-alerts, /compliance/v1/compliance-reports/compliance, and /compliance/v1/compliance-alerts/{id}/resolve.</x:v>
+      </x:c>
+      <x:c r="P102" t="str">
+        <x:v>ComplianceControllerTests.GetStats_WhenClientReturnsNull_ReturnsEmptyStats; Create_WhenClientCreatesRecord_ReturnsCreatedAtGetById; Delete_WhenClientReportsFailure_ReturnsNotFound; ComplianceEndpoints_RequireCompliancePermissions; ComplianceServiceClient_MapsUnresolvedAlertsToPagedRecords; ComplianceServiceClient_MapsComplianceReportToStats; ComplianceServiceClient_DeleteResolvesAlert.</x:v>
+      </x:c>
+      <x:c r="Q102" t="str">
+        <x:v>Intranet BFF, ComplianceService</x:v>
+      </x:c>
+      <x:c r="R102" t="str">
+        <x:v>Compliance alert resolution state; compliance record create request when supported by downstream service; compliance report/read models.</x:v>
+      </x:c>
+      <x:c r="S102" t="str">
+        <x:v>No dedicated current Blazor compliance page was found; create support is limited by the current ComplianceServiceClient returning null for CreateComplianceRecordAsync.</x:v>
+      </x:c>
+      <x:c r="T102" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/ComplianceController.cs:18,23,25,37,39,50,52,64,66,78,80; Maliev.Intranet.Bff/Clients/ComplianceServiceClient.cs:45,47,66,68,82,94,96; Maliev.Intranet.Shared/Dtos/ComplianceDtos.cs:8,44; Maliev.Intranet.Tests/Bff/Controllers/ComplianceControllerTests.cs:21,49,64,81,94,133,159</x:v>
+      </x:c>
+      <x:c r="U102" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>INT-102</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>Employee onboarding summaries, checklist, and task completion</x:v>
+      </x:c>
+      <x:c r="D103" t="str">
+        <x:v>As an HR employee, I can review onboarding progress, open an employee checklist, and mark completed onboarding tasks.</x:v>
+      </x:c>
+      <x:c r="E103" t="str">
+        <x:v>The onboarding API requires onboarding read permission for paged onboarding summaries and employee checklist reads, and onboarding write permission for checklist task updates. The list endpoint converts LifecycleService pending onboarding status into a paged summary with employee id, start date, status, and percent progress from completed and total items. The checklist endpoint reads the employee onboarding status and maps tasks with id, title, description, assignee, and completion state. Updating a task only proceeds when the request marks the task completed, then calls the downstream complete endpoint and returns NoContent when accepted.</x:v>
+      </x:c>
+      <x:c r="F103" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G103" t="str">
+        <x:v>Focused onboarding controller and lifecycle client tests cover empty list fallback, missing checklist NotFound, update success/failure, permissions, pending-summary mapping, checklist task mapping, and complete-only task update behavior.</x:v>
+      </x:c>
+      <x:c r="H103" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I103" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J103" t="str">
+        <x:v>Pending live API/browser workflow retest; current client code exposes onboarding navigation labels but no dedicated Blazor onboarding page was found.</x:v>
+      </x:c>
+      <x:c r="K103" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L103" t="str">
+        <x:v>OnboardingController BFF endpoints -&gt; LifecycleServiceClient -&gt; LifecycleService onboarding status/checklist/complete contracts -&gt; Onboarding DTOs</x:v>
+      </x:c>
+      <x:c r="M103" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/OnboardingController.cs; Maliev.Intranet.Bff/Clients/LifecycleServiceClient.cs; Maliev.Intranet.Shared/Dtos/OnboardingDtos.cs</x:v>
+      </x:c>
+      <x:c r="N103" t="str">
+        <x:v>No current dedicated Blazor page was found under Maliev.Intranet.Client/Pages/Hr for onboarding; ChatDrawer source contains an /hr/onboarding label, but the current BFF entry point is api/v1/onboarding.</x:v>
+      </x:c>
+      <x:c r="O103" t="str">
+        <x:v>GET api/v1/onboarding?page=&amp;pageSize=, GET api/v1/onboarding/{employeeId}/checklist, PATCH api/v1/onboarding/{employeeId}/tasks; downstream calls /lifecycle/v1/onboarding/pending, /lifecycle/v1/employees/{employeeId}/onboarding/status, and /lifecycle/v1/onboarding-items/{taskId}/complete.</x:v>
+      </x:c>
+      <x:c r="P103" t="str">
+        <x:v>OnboardingControllerTests.Get_WhenClientReturnsNull_ReturnsEmptyPagedResponse; GetChecklist_WhenChecklistMissing_ReturnsNotFound; UpdateTask_WhenClientUpdatesTask_ReturnsNoContent; OnboardingEndpoints_RequireOnboardingPermissions; LifecycleServiceClient_MapsPendingOnboardingToPagedSummaries; LifecycleServiceClient_MapsEmployeeChecklistTasks; LifecycleServiceClient_UpdateTask_CompletesOnlyCompletedRequests; ChatDrawer_ExposesOnboardingNavigationLabel.</x:v>
+      </x:c>
+      <x:c r="Q103" t="str">
+        <x:v>Intranet BFF, LifecycleService</x:v>
+      </x:c>
+      <x:c r="R103" t="str">
+        <x:v>Onboarding task completion state and checklist/progress read models.</x:v>
+      </x:c>
+      <x:c r="S103" t="str">
+        <x:v>No dedicated current Blazor onboarding page was found; update behavior cannot mark tasks incomplete because the current client returns false unless IsCompleted is true.</x:v>
+      </x:c>
+      <x:c r="T103" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/OnboardingController.cs:16,21,23,32,34,43,45; Maliev.Intranet.Bff/Clients/LifecycleServiceClient.cs:34,37,54,56,61,68; Maliev.Intranet.Shared/Dtos/OnboardingDtos.cs:8,54,85,106; Maliev.Intranet.Tests/Bff/Controllers/OnboardingControllerTests.cs:20,34,46,73,86,127,176</x:v>
+      </x:c>
+      <x:c r="U103" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>INT-103</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>Performance review and goal read models</x:v>
+      </x:c>
+      <x:c r="D104" t="str">
+        <x:v>As an HR or manager employee, I can read performance reviews and employee goals through the Intranet BFF.</x:v>
+      </x:c>
+      <x:c r="E104" t="str">
+        <x:v>The performance API requires performance read permission for review and goal reads. Reviews are returned from the PerformanceService reviews endpoint with review id, employee id, reviewer id, cycle, rating, comments, status, and reviewer name. Goals are returned from the PerformanceService goals endpoint with goal id, employee id, title, description, status, due date, and progress. The controller returns empty lists instead of null when the downstream client has no data.</x:v>
+      </x:c>
+      <x:c r="F104" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G104" t="str">
+        <x:v>Focused performance controller and client tests cover null-to-empty fallback, read permissions, review service path mapping, and goal service path mapping.</x:v>
+      </x:c>
+      <x:c r="H104" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I104" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J104" t="str">
+        <x:v>Pending live API/browser workflow retest; current client code exposes a performance navigation label but no dedicated Blazor performance page was found.</x:v>
+      </x:c>
+      <x:c r="K104" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L104" t="str">
+        <x:v>PerformanceController BFF endpoints -&gt; PerformanceServiceClient -&gt; PerformanceService reviews/goals contracts -&gt; Performance DTOs</x:v>
+      </x:c>
+      <x:c r="M104" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/PerformanceController.cs; Maliev.Intranet.Bff/Clients/PerformanceServiceClient.cs; Maliev.Intranet.Shared/Dtos/PerformanceDtos.cs</x:v>
+      </x:c>
+      <x:c r="N104" t="str">
+        <x:v>No current dedicated Blazor page was found under Maliev.Intranet.Client/Pages/Hr for performance; ChatDrawer source contains an /hr/performance label, but the current BFF entry point is api/v1/performance.</x:v>
+      </x:c>
+      <x:c r="O104" t="str">
+        <x:v>GET api/v1/performance/reviews and GET api/v1/performance/goals; downstream calls /performance/v1/reviews and /performance/v1/goals.</x:v>
+      </x:c>
+      <x:c r="P104" t="str">
+        <x:v>PerformanceControllerTests.GetReviews_WhenClientReturnsNull_ReturnsEmptyList; GetGoals_WhenClientReturnsNull_ReturnsEmptyList; PerformanceEndpoints_RequirePerformanceReadPermission; PerformanceServiceClient_ReadsReviewsFromPerformanceService; PerformanceServiceClient_ReadsGoalsFromPerformanceService; ChatDrawer_ExposesPerformanceNavigationLabel.</x:v>
+      </x:c>
+      <x:c r="Q104" t="str">
+        <x:v>Intranet BFF, PerformanceService</x:v>
+      </x:c>
+      <x:c r="R104" t="str">
+        <x:v>Read-only performance review and goal data in this current code path.</x:v>
+      </x:c>
+      <x:c r="S104" t="str">
+        <x:v>No dedicated current Blazor performance page or write workflow was found in this slice.</x:v>
+      </x:c>
+      <x:c r="T104" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/PerformanceController.cs:18,23,25,34,36; Maliev.Intranet.Bff/Clients/PerformanceServiceClient.cs:29,31,35,37; Maliev.Intranet.Shared/Dtos/PerformanceDtos.cs:8,33; Maliev.Intranet.Tests/Bff/Controllers/PerformanceControllerTests.cs:20,34,50,63,104</x:v>
+      </x:c>
+      <x:c r="U104" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="105">
+      <x:c r="A105" t="str">
+        <x:v>INT-104</x:v>
+      </x:c>
+      <x:c r="B105" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C105" t="str">
+        <x:v>Compensation summary and benefits read models</x:v>
+      </x:c>
+      <x:c r="D105" t="str">
+        <x:v>As an HR or finance employee, I can read compensation summary and benefits data through the Intranet BFF.</x:v>
+      </x:c>
+      <x:c r="E105" t="str">
+        <x:v>The compensation API requires compensation read permission for summary and benefits endpoints. The summary endpoint reads CompensationService compensation-analysis data and maps average salary into base salary, total annual budget into total compensation, and default zero values for annual bonus and percentage change. The benefits endpoint returns the current benefit list from CompensationService. The controller returns an empty CompensationSummaryDto or empty benefit list when the downstream client returns no data.</x:v>
+      </x:c>
+      <x:c r="F105" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G105" t="str">
+        <x:v>Mapped to current compensation controller, client, DTOs, and contract-inventory/shared DTO coverage; no focused compensation controller unit test was found in this slice.</x:v>
+      </x:c>
+      <x:c r="H105" t="str">
+        <x:v>No behavior error documented in this tracker slice.</x:v>
+      </x:c>
+      <x:c r="I105" t="str">
+        <x:v>No app fix applied; workbook tracking only.</x:v>
+      </x:c>
+      <x:c r="J105" t="str">
+        <x:v>Pending focused automated controller/client tests and live API/browser workflow retest; current client code does not expose a dedicated compensation Blazor page.</x:v>
+      </x:c>
+      <x:c r="K105" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L105" t="str">
+        <x:v>CompensationController BFF endpoints -&gt; CompensationServiceClient -&gt; CompensationService analysis/benefits contracts -&gt; HR DTOs</x:v>
+      </x:c>
+      <x:c r="M105" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/CompensationController.cs; Maliev.Intranet.Bff/Clients/CompensationServiceClient.cs; Maliev.Intranet.Shared/Dtos/HRDtos.cs</x:v>
+      </x:c>
+      <x:c r="N105" t="str">
+        <x:v>No current dedicated Blazor page was found under Maliev.Intranet.Client/Pages for compensation; the current entry point is api/v1/compensation plus permissions.</x:v>
+      </x:c>
+      <x:c r="O105" t="str">
+        <x:v>GET api/v1/compensation/summary and GET api/v1/compensation/benefits; downstream calls /compensation/v1/reports/compensation-analysis and /compensation/v1/benefits.</x:v>
+      </x:c>
+      <x:c r="P105" t="str">
+        <x:v>PlatformContractInventoryTests maps CompensationServiceClient to Maliev.CompensationService; shared DTO smoke tests instantiate CompensationSummaryDto. No focused compensation endpoint unit test was found during this slice.</x:v>
+      </x:c>
+      <x:c r="Q105" t="str">
+        <x:v>Intranet BFF, CompensationService</x:v>
+      </x:c>
+      <x:c r="R105" t="str">
+        <x:v>Read-only compensation summary and benefit list data in this current code path.</x:v>
+      </x:c>
+      <x:c r="S105" t="str">
+        <x:v>No dedicated current Blazor compensation page was found; no focused compensation controller/client tests were found in this slice.</x:v>
+      </x:c>
+      <x:c r="T105" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/CompensationController.cs:18,23,25,34,36; Maliev.Intranet.Bff/Clients/CompensationServiceClient.cs:29,31,44,46; Maliev.Intranet.Shared/Dtos/HRDtos.cs:316,374; Maliev.Intranet.Tests/Bff/PlatformContractInventoryTests.cs:42; Maliev.Intranet.Tests/Shared/DtoTests.cs:90</x:v>
+      </x:c>
+      <x:c r="U105" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R18075dab11694cbe"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72edcb39aa2e4c6d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15143,7 +15403,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcd5d488a621a46cc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref5e06851d8343c9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Web assistant handoff tracker story
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9de72b969f924e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R4b6177341b134650"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rfc0f259de56349be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R239002755bb643b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5191673fb8f841c7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R1b9247a440894f9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R44db3078102d43f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R4502945520d94a73"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -505,7 +505,7 @@
         <x:v>Maliev.Web</x:v>
       </x:c>
       <x:c r="B5" s="8" t="n">
-        <x:v>61</x:v>
+        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="6" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>224</x:v>
+        <x:v>225</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -2466,61 +2466,61 @@
         <x:v>Maliev.Web</x:v>
       </x:c>
       <x:c r="C30" s="8" t="str">
-        <x:v>SEO metadata</x:v>
+        <x:v>SEO crawler metadata</x:v>
       </x:c>
       <x:c r="D30" s="8" t="str">
-        <x:v>As a crawler or visitor, I can access robots and sitemap metadata.</x:v>
+        <x:v>As a crawler or visitor, I can access robots and sitemap metadata for public MALIEV pages.</x:v>
       </x:c>
       <x:c r="E30" s="8" t="str">
-        <x:v>SEO controller serves robots.txt and sitemap.xml.</x:v>
+        <x:v>The BFF serves /robots.txt as text/plain with User-agent *, Allow /, Disallow rules for account, cart, checkout, and /web/ endpoints, plus the production sitemap URL. The BFF also serves /sitemap.xml as application/xml from a fixed public route list that includes home, services, service detail routes, materials, industries, case studies, blog, shop, contact, FAQ, crawlable policy routes, terms, and quote; service routes can include lastmod values.</x:v>
       </x:c>
       <x:c r="F30" s="8" t="str">
         <x:v>Current code-derived</x:v>
       </x:c>
       <x:c r="G30" s="8" t="str">
-        <x:v>Automated Web suite passed 2026-06-23</x:v>
+        <x:v>Not yet tested in browser; source and controller evidence documented 2026-06-29.</x:v>
       </x:c>
       <x:c r="H30" s="8" t="str">
-        <x:v>No behavior error observed in current Web automated suite.</x:v>
+        <x:v>No behavior error observed from current source inspection.</x:v>
       </x:c>
       <x:c r="I30" s="8" t="str">
-        <x:v>No fix needed from current Web automated suite.</x:v>
+        <x:v>No app fix applied; tracker-only documentation slice.</x:v>
       </x:c>
       <x:c r="J30" s="8" t="str">
-        <x:v>Current automated suite passed.</x:v>
+        <x:v>Pending story-by-story behavior testing loop.</x:v>
       </x:c>
       <x:c r="K30" s="8" t="str">
-        <x:v>P2</x:v>
+        <x:v>P1</x:v>
       </x:c>
       <x:c r="L30" s="8" t="str">
-        <x:v>Public SEO endpoints -&gt; static generated metadata</x:v>
+        <x:v>GET /robots.txt and GET /sitemap.xml -&gt; SeoController fixed PublicRoutes -&gt; crawler text/XML responses using https://www.maliev.com canonical URLs</x:v>
       </x:c>
       <x:c r="M30" s="8" t="str">
-        <x:v>SeoController</x:v>
+        <x:v>SeoController.cs</x:v>
       </x:c>
       <x:c r="N30" s="8" t="str">
-        <x:v>/robots.txt, /sitemap.xml</x:v>
+        <x:v>SeoController declares anonymous /robots.txt and /sitemap.xml endpoints; robots emits Allow/Disallow lines and the canonical sitemap URL; sitemap maps PublicRoutes to URL XML entries and returns application/xml.</x:v>
       </x:c>
       <x:c r="O30" s="8" t="str">
-        <x:v>SeoController GET robots/sitemap</x:v>
+        <x:v>No downstream service call; SEO metadata is generated by the Web BFF from its in-process PublicRoutes array.</x:v>
       </x:c>
       <x:c r="P30" s="8" t="str">
-        <x:v>WebBffEndpointTests Seo | Current suite: dotnet test Maliev.Web.slnx --verbosity minimal passed 235/235 on 2026-06-23.</x:v>
+        <x:v>No focused SEO endpoint test was found in this slice; AGENTS/README document sitemap and policy route expectations.</x:v>
       </x:c>
       <x:c r="Q30" s="8" t="str">
-        <x:v>Web BFF</x:v>
+        <x:v>Web BFF SEO endpoint</x:v>
       </x:c>
       <x:c r="R30" s="8" t="str">
-        <x:v>Read-only SEO content</x:v>
+        <x:v>No mutation; generated robots text and sitemap XML only.</x:v>
       </x:c>
       <x:c r="S30" s="8" t="str">
-        <x:v>Needs deployment hostname review</x:v>
+        <x:v>Needs HTTP smoke test validating robots.txt and sitemap.xml status, content types, canonical production URLs, policy pages, and exclusion of private account/cart/checkout/API routes.</x:v>
       </x:c>
       <x:c r="T30" s="8" t="str">
-        <x:v>SeoController.cs:49,58</x:v>
+        <x:v>Maliev.Web.Bff/Controllers/SeoController.cs:11,13,37,42,50,52,59,61,69; Maliev.Web/AGENTS.md:9,13,16; README.md:128</x:v>
       </x:c>
       <x:c r="U30" s="8" t="str">
-        <x:v>2026-06-23</x:v>
+        <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
     <x:row r="31" s="6" customFormat="1" ht="73.44999694824219" customHeight="1">
@@ -4603,10 +4603,75 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="63">
+      <x:c r="A63" t="str">
+        <x:v>WEB-062</x:v>
+      </x:c>
+      <x:c r="B63" t="str">
+        <x:v>Maliev.Web</x:v>
+      </x:c>
+      <x:c r="C63" t="str">
+        <x:v>Customer assistant verified handoff</x:v>
+      </x:c>
+      <x:c r="D63" t="str">
+        <x:v>As a signed-in or anonymous visitor using the website assistant, I can continue an assistant session through a signed Web-to-Make-Studio handoff.</x:v>
+      </x:c>
+      <x:c r="E63" t="str">
+        <x:v>Starting an assistant session or sending an assistant message through the Web BFF appends a signed maliev_customer_assistant_handoff cookie whenever the assistant response includes a session id. The cookie carries session id, trimmed user key when available, normalized language, authentication flag, issued/expiry timestamps, a 30-day max age, root path, SameSite=Lax, HttpOnly, HTTPS-only Secure behavior, and a shared .maliev.com domain on MALIEV hosts. If the user must sign in from the assistant, the widget routes Google or email auth back to /auth/chatbot-complete, which notifies the opener that authentication completed.</x:v>
+      </x:c>
+      <x:c r="F63" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G63" t="str">
+        <x:v>Focused existing Web BFF endpoint tests cover Set-Cookie on chatbot message and session routes; source and UI return route inspected 2026-06-29.</x:v>
+      </x:c>
+      <x:c r="H63" t="str">
+        <x:v>No behavior error observed from current source inspection.</x:v>
+      </x:c>
+      <x:c r="I63" t="str">
+        <x:v>No app fix applied; tracker-only documentation slice.</x:v>
+      </x:c>
+      <x:c r="J63" t="str">
+        <x:v>Pending live browser retest of assistant sign-in popup, cookie sharing, and Make Studio continuation.</x:v>
+      </x:c>
+      <x:c r="K63" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L63" t="str">
+        <x:v>CustomerChatbot UI -&gt; /web/v1/chatbot/sessions or /web/v1/chatbot/messages -&gt; ChatbotController -&gt; CustomerChatbotService -&gt; CustomerAssistantHandoffCookie -&gt; browser Set-Cookie -&gt; /auth/chatbot-complete JS notification</x:v>
+      </x:c>
+      <x:c r="M63" t="str">
+        <x:v>CustomerChatbot.razor; ChatbotController; CustomerAssistantHandoffCookie; AuthChatbotComplete.razor; Program.cs</x:v>
+      </x:c>
+      <x:c r="N63" t="str">
+        <x:v>CustomerChatbot uses /auth/chatbot-complete as the assistant auth return URL for Google/email sign-in and shows a verified-session error when the assistant cannot open; AuthChatbotComplete calls malievChatbot.notifyAuthenticationComplete after first render.</x:v>
+      </x:c>
+      <x:c r="O63" t="str">
+        <x:v>ChatbotController appends the handoff cookie on successful session or message responses with a session id; CustomerAssistantHandoffCookie signs the payload with HMACSHA256 and sets HttpOnly, SameSite=Lax, root path, 30-day MaxAge, host-sensitive domain, and HTTPS-sensitive Secure options.</x:v>
+      </x:c>
+      <x:c r="P63" t="str">
+        <x:v>WebBffEndpointTests.POST_ChatbotMessage_RoutesThroughChatbotBoundary and POST_ChatbotSession_StartsChatbotBoundarySession assert Set-Cookie contains maliev_customer_assistant_handoff, path=/, and HttpOnly.</x:v>
+      </x:c>
+      <x:c r="Q63" t="str">
+        <x:v>Web Client, Web BFF, CustomerChatbotService, ChatbotService, browser cookie jar, Make Studio shared customer-assistant handoff</x:v>
+      </x:c>
+      <x:c r="R63" t="str">
+        <x:v>Signed customer assistant handoff cookie, assistant session id, language, user key, authentication flag, assistant UI auth-return state.</x:v>
+      </x:c>
+      <x:c r="S63" t="str">
+        <x:v>Needs live browser retest for popup auth completion, cross-subdomain cookie visibility, and Make Studio consumption of the signed handoff cookie.</x:v>
+      </x:c>
+      <x:c r="T63" t="str">
+        <x:v>Maliev.Web.Client/Components/CustomerChatbot.razor:185,794,1118,1119; Maliev.Web.Client/Pages/AuthChatbotComplete.razor:1,29; Maliev.Web.Bff/Controllers/ChatbotController.cs:25,38,39,63,77,98,105,116; Maliev.Web.Bff/Security/CustomerAssistantHandoffCookie.cs:14,21,30,45,48,50,52,53,59,68,83; Maliev.Web.Bff/Program.cs:149; Maliev.Web.Tests/WebBffEndpointTests.cs:487,503,514,529</x:v>
+      </x:c>
+      <x:c r="U63" t="str">
+        <x:v>2026-06-29</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R331b3105df084e69"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1bdbf447a504813"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11467,7 +11532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R72edcb39aa2e4c6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8270e8075b6245eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15403,7 +15468,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref5e06851d8343c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52aeee457d624df8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add QuoteEngine auth handoff tracker story
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R5191673fb8f841c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R1b9247a440894f9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R44db3078102d43f8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R4502945520d94a73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R73cead61a7b74eda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R6594fde1d9bf4512"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rdff3b9b537114a29"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R2c4bab6aae034c98"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -481,7 +481,7 @@
         <x:v>Expanded current-code rebuild</x:v>
       </x:c>
       <x:c r="B2" s="8" t="str">
-        <x:v>2026-06-29</x:v>
+        <x:v>2026-06-30</x:v>
       </x:c>
     </x:row>
     <x:row r="3" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -521,7 +521,7 @@
         <x:v>Maliev.QuoteEngine</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>59</x:v>
+        <x:v>60</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>225</x:v>
+        <x:v>226</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4671,7 +4671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1bdbf447a504813"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd584062f33c2440e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11532,7 +11532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8270e8075b6245eb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0214abd5e1b04860"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15465,10 +15465,75 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="61">
+      <x:c r="A61" t="str">
+        <x:v>QE-060</x:v>
+      </x:c>
+      <x:c r="B61" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C61" t="str">
+        <x:v>Agent trusted auth handoff methods</x:v>
+      </x:c>
+      <x:c r="D61" t="str">
+        <x:v>As an anonymous customer, I can use trusted sign-in options shown by the quote agent without the agent collecting credentials or exposing raw auth links.</x:v>
+      </x:c>
+      <x:c r="E61" t="str">
+        <x:v>The agent response state can include a QuoteAgentAuthHandoffResponse when authentication is required for formal quote, order, payment, connector, or account-protected actions. If the customer is already authenticated, the response reports already_authenticated. Otherwise it returns authentication_required, a normalized local return URL, the customer_authenticated gate code, and three customer-safe methods: Google as preferred, passkey as browser-supported with email-password fallback, and email/password through the shared MALIEV auth page. Assistant text that tries to include direct sign-in URLs while the auth gate is blocked is replaced with copy telling the customer to use the secure sign-in options in chat.</x:v>
+      </x:c>
+      <x:c r="F61" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G61" t="str">
+        <x:v>Existing focused auth-handoff and source tests mapped 2026-06-30; live browser auth popup retest still pending.</x:v>
+      </x:c>
+      <x:c r="H61" t="str">
+        <x:v>No behavior error observed from current source inspection.</x:v>
+      </x:c>
+      <x:c r="I61" t="str">
+        <x:v>No app fix applied; tracker-only documentation slice.</x:v>
+      </x:c>
+      <x:c r="J61" t="str">
+        <x:v>Pending story-by-story behavior testing loop.</x:v>
+      </x:c>
+      <x:c r="K61" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L61" t="str">
+        <x:v>QuoteAgentService gate/action state -&gt; QuoteAgentAuthHandoffResponse DTO -&gt; QuoteAgentLaunchShell auth handoff UI -&gt; /auth/sign-in or /auth/sign-up shared Web auth routes -&gt; AuthChatbotComplete return</x:v>
+      </x:c>
+      <x:c r="M61" t="str">
+        <x:v>QuoteAgentLaunchShell.razor; QuoteAgentService.cs; QuoteAgentDtos.cs; QuoteAgentEndpointTests.cs; QuoteEngineSourceTests.cs</x:v>
+      </x:c>
+      <x:c r="N61" t="str">
+        <x:v>QuoteAgentLaunchShell shows auth handoff cards when ShouldShowAuthHandoff is true, applies auth handoff from streamed/final agent responses, opens sign-in/sign-up dialogs, and uses /auth/chatbot-complete as the auth return path for assistant continuation.</x:v>
+      </x:c>
+      <x:c r="O61" t="str">
+        <x:v>QuoteAgentService.BuildAuthHandoff resolves customer state, intent, and safe return URL; returns already_authenticated when a customer id is available; otherwise returns authentication_required with Google, passkey, and email-password method metadata. GroundAuthHandoffText removes raw /auth/sign-in links from blocked assistant text and replaces them with secure in-chat handoff copy.</x:v>
+      </x:c>
+      <x:c r="P61" t="str">
+        <x:v>Mapped tests: QuoteAgentEndpointTests auth handoff tool returnUrl/method assertions, default /auth/chatbot-complete handoff, unauthenticated turn auth handoff method set, and auth-link grounding; QuoteEngineSourceTests auth handoff UI rendering and default chat auth path source checks.</x:v>
+      </x:c>
+      <x:c r="Q61" t="str">
+        <x:v>QuoteEngine Client, QuoteEngine BFF, QuoteAgentService, ChatbotService, Maliev.Web shared auth surface</x:v>
+      </x:c>
+      <x:c r="R61" t="str">
+        <x:v>QuoteAgentAuthHandoffResponse state, auth handoff method list, customer-auth gate state, normalized return URL; no persisted data mutation.</x:v>
+      </x:c>
+      <x:c r="S61" t="str">
+        <x:v>Needs live browser retest for Google, passkey-capable browser, email fallback, auth return popup/redirect, and continuation of the pending agent action after sign-in.</x:v>
+      </x:c>
+      <x:c r="T61" t="str">
+        <x:v>Maliev.QuoteEngine.Bff/Services/QuoteAgentService.cs:110,237,414,829,2451,2464,2481,2487,2502,2523,6453,6491; Maliev.QuoteEngine.Shared/Agent/QuoteAgentDtos.cs:210,776,794,797; Maliev.QuoteEngine.Client/Components/QuoteAgent/QuoteAgentLaunchShell.razor:1039,2042,2969,3903,3909,5249,5955; Maliev.QuoteEngine.Client/Pages/AuthChatbotComplete.razor:1; Maliev.QuoteEngine.Tests/QuoteAgentEndpointTests.cs:4691,4712,4719,4720,4721,4739,4778,4779,4780,4781,4782,4783,4784,4826,4827; Maliev.QuoteEngine.Tests/QuoteEngineSourceTests.cs:2150,2156,2157</x:v>
+      </x:c>
+      <x:c r="U61" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52aeee457d624df8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e370dadd4764267"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Intranet upload and search tracker stories
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R73cead61a7b74eda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R6594fde1d9bf4512"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rdff3b9b537114a29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R2c4bab6aae034c98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rc102b505a4ea4194"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R2e3604444a374ebf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rb89ca852c6164178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Ra0e5fbdecb8c4bfa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -513,7 +513,7 @@
         <x:v>Maliev.Intranet</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>104</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="7" s="6" customFormat="1" ht="16.649999618530273" customHeight="1">
@@ -529,7 +529,7 @@
         <x:v>Total</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>226</x:v>
+        <x:v>228</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="6" customFormat="1" ht="31.600000381469727" customHeight="1">
@@ -4671,7 +4671,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd584062f33c2440e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04730cd1fc6848dc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11529,10 +11529,140 @@
         <x:v>2026-06-29</x:v>
       </x:c>
     </x:row>
+    <x:row r="106">
+      <x:c r="A106" t="str">
+        <x:v>INT-105</x:v>
+      </x:c>
+      <x:c r="B106" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C106" t="str">
+        <x:v>Shared upload, signed file access, and project file migration</x:v>
+      </x:c>
+      <x:c r="D106" t="str">
+        <x:v>As an employee working with project files, drawings, previews, and documents, I can upload, retrieve, preview, and migrate files through a single Intranet BFF boundary.</x:v>
+      </x:c>
+      <x:c r="E106" t="str">
+        <x:v>The Intranet upload boundary accepts single, batch, resumable, and fallback streamed project uploads; builds project/customer-scoped storage paths; adds browser-primary metadata for supported CAD formats; completes UploadService sessions; exposes bounded analysis status, viewer URLs, preview URLs, attachment upload/delete, file-id download URLs, and by-path signed URLs; and can migrate temporary project artifacts to customer/project paths while reconciling cached analysis status and signed GLB/thumbnail URLs.</x:v>
+      </x:c>
+      <x:c r="F106" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G106" t="str">
+        <x:v>Existing BFF, DTO, and client tests mapped 2026-06-30; full live upload/migration retest still pending.</x:v>
+      </x:c>
+      <x:c r="H106" t="str">
+        <x:v>No behavior error observed from current source inspection.</x:v>
+      </x:c>
+      <x:c r="I106" t="str">
+        <x:v>No app fix applied; tracker-only documentation slice.</x:v>
+      </x:c>
+      <x:c r="J106" t="str">
+        <x:v>Pending story-by-story behavior testing loop.</x:v>
+      </x:c>
+      <x:c r="K106" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="L106" t="str">
+        <x:v>ProjectNew, drawing/part components, document dialogs, and other file consumers -&gt; /api/v1/uploads endpoints -&gt; UploadServiceClient -&gt; UploadService storage, signed URL, and migration APIs -&gt; FileAnalysisStatusService analysis cache and shared DTOs</x:v>
+      </x:c>
+      <x:c r="M106" t="str">
+        <x:v>UploadsController.cs; UploadServiceClient.cs; FileAnalysisStatusService.cs; ProjectNew.razor.cs; DrawingAttachmentsTab.razor; CommonDtos.cs; UploadMigrationDtos.cs; UploadsControllerResumableTests.cs; UploadAnalysisStatusTests.cs</x:v>
+      </x:c>
+      <x:c r="N106" t="str">
+        <x:v>ProjectNew starts resumable uploads through api/v1/uploads/resumable, proxies raw upload bytes when needed, completes sessions, resolves signed download/viewer URLs, polls analysis-status, deletes uploaded attachments, and calls api/v1/uploads/migrate-project when draft files need project-scoped storage. Drawing and part detail components call the attachment and preview-url endpoints for supporting files.</x:v>
+      </x:c>
+      <x:c r="O106" t="str">
+        <x:v>UploadsController exposes POST uploads, POST uploads/batch, POST uploads/resumable, PUT uploads/resumable/{uploadId}, POST uploads/resumable/{uploadId}/complete, GET uploads/analysis-status, GET uploads/viewer-url, GET uploads/preview-url, POST/DELETE uploads/attachments, GET uploads/{fileId}/download-url, POST uploads/by-path/signed-url, and POST uploads/migrate-project. The controller delegates storage and signed URL work to UploadServiceClient and reconciles migrated file-analysis status through FileAnalysisStatusService.</x:v>
+      </x:c>
+      <x:c r="P106" t="str">
+        <x:v>Mapped tests: UploadsControllerResumableTests for resumable session creation, browser-primary metadata, extension acceptance/rejection, raw-body proxying, completion, project migration, and migration wire shape; UploadAnalysisStatusTests for analysis-status/viewer-url signed URL behavior; DtoSerializationTests for BffUploadResponse and BffMigrateProjectResponseDto wire shape; DrawingAttachmentsTabTests and ProjectNewAutoSaveTests for client upload and migration calls.</x:v>
+      </x:c>
+      <x:c r="Q106" t="str">
+        <x:v>Intranet Client, Intranet BFF, UploadService, Geometry/FileAnalysis event cache, ProjectService consumers</x:v>
+      </x:c>
+      <x:c r="R106" t="str">
+        <x:v>BffUploadResponse, BffInitiateResumableUploadRequest, BffResumableUploadSessionResponse, DraftProjectAttachmentDto, signed URL responses, FileAnalysisStatusDto, BffMigrateProjectResponseDto, upload storage paths, migrated analysis-cache aliases</x:v>
+      </x:c>
+      <x:c r="S106" t="str">
+        <x:v>Needs browser retest for large CAD resumable upload, fallback proxy upload, attachment preview/delete, signed-url expiry refresh, and dry-run versus live project migration.</x:v>
+      </x:c>
+      <x:c r="T106" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/UploadsController.cs:60,95,139,143,165,166,190,193,208,212,244,245,294,295,446,447,473,474,541,542,563,564,579,582,617,621,633,637,674,819,832; Maliev.Intranet.Client/Pages/ProjectNew.razor.cs:662,684,697,979,1781,1843,1864,1876,2301,2725,4819,5017,5024; Maliev.Intranet.Client/Components/Project/DrawingAttachmentsTab.razor:154,197,216; Maliev.Intranet.Shared/Dtos/CommonDtos.cs:330,366,372,408; Maliev.Intranet.Shared/Dtos/UploadMigrationDtos.cs:6,39; Maliev.Intranet.Tests/Bff/Controllers/UploadsControllerResumableTests.cs:30,84,131,158,177,209,269,371,400; Maliev.Intranet.Tests/Bff/Controllers/UploadAnalysisStatusTests.cs:18,94,158,202,284,333; Maliev.Intranet.Tests/Shared/DtoSerializationTests.cs:183,210</x:v>
+      </x:c>
+      <x:c r="U106" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="107">
+      <x:c r="A107" t="str">
+        <x:v>INT-106</x:v>
+      </x:c>
+      <x:c r="B107" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C107" t="str">
+        <x:v>Global search enrichment and thumbnail navigation</x:v>
+      </x:c>
+      <x:c r="D107" t="str">
+        <x:v>As an employee searching the intranet, I can search across operational records and navigate to enriched results with statuses, grouped areas, and project-part thumbnails.</x:v>
+      </x:c>
+      <x:c r="E107" t="str">
+        <x:v>The Search page and global search box require at least two characters before querying, call api/v1/search with a bounded limit, show loading/empty states, group full-page results by area, navigate result rows to their resolved HREFs, show status badges, allow view-all and first-result keyboard navigation from the global search box, and render project-part thumbnails when the BFF enriches raw SearchService rows with signed thumbnail URLs.</x:v>
+      </x:c>
+      <x:c r="F107" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G107" t="str">
+        <x:v>Existing source/component/BFF tests mapped 2026-06-30; live search index retest still pending.</x:v>
+      </x:c>
+      <x:c r="H107" t="str">
+        <x:v>No behavior error observed from current source inspection.</x:v>
+      </x:c>
+      <x:c r="I107" t="str">
+        <x:v>No app fix applied; tracker-only documentation slice.</x:v>
+      </x:c>
+      <x:c r="J107" t="str">
+        <x:v>Pending story-by-story behavior testing loop.</x:v>
+      </x:c>
+      <x:c r="K107" t="str">
+        <x:v>P1</x:v>
+      </x:c>
+      <x:c r="L107" t="str">
+        <x:v>Search.razor and GlobalSearchBox UI -&gt; GET api/v1/search -&gt; SearchController validation and limit clamp -&gt; SearchServiceClient -&gt; SearchResultMapper HREF/status mapping -&gt; GlobalSearchResultEnricher -&gt; ProjectServiceClient and UploadServiceClient signed thumbnail URLs</x:v>
+      </x:c>
+      <x:c r="M107" t="str">
+        <x:v>Search.razor; GlobalSearchBox.razor; SearchController.cs; SearchResultMapper.cs; GlobalSearchResultEnricher.cs; GlobalSearchBoxTests.cs; SearchResultMapperTests.cs; GlobalSearchResultEnricherTests.cs; SearchControllerTests.cs</x:v>
+      </x:c>
+      <x:c r="N107" t="str">
+        <x:v>Search.razor displays a full search page, reads the query parameter, blocks queries shorter than two characters, requests up to 50 results, groups results by area, renders title/subtitle/status, and navigates to the selected result. GlobalSearchBox renders inline suggestions, thumbnails/avatars, a view-all action, click-away close behavior, and Enter navigation to the first result.</x:v>
+      </x:c>
+      <x:c r="O107" t="str">
+        <x:v>SearchController trims the query, rejects empty and over-120-character searches, clamps limit from 1 to 50, calls SearchServiceClient.SearchAsync, and returns GlobalSearchResultEnricher.ToGlobalSearchResponseAsync. The enricher maps SearchService rows to GlobalSearchResultDto and resolves project-part thumbnails from project details and UploadService signed by-path URLs.</x:v>
+      </x:c>
+      <x:c r="P107" t="str">
+        <x:v>Mapped tests: GlobalSearchBoxTests for query length guard, result rendering/navigation, project-part thumbnails, click-away, open-layer styling, and Enter navigation; SearchResultMapperTests for customer, project, project-part, purchase-order, and material HREF resolution; GlobalSearchResultEnricherTests for existing thumbnails and signed thumbnail resolution; SearchControllerTests and SearchServiceClientTests for BFF validation and wire shape.</x:v>
+      </x:c>
+      <x:c r="Q107" t="str">
+        <x:v>Intranet Client, Intranet BFF, SearchService, ProjectService, UploadService</x:v>
+      </x:c>
+      <x:c r="R107" t="str">
+        <x:v>GlobalSearchResponseDto, GlobalSearchResultDto, SearchServiceResponseDto, signed thumbnail URLs; no persistent data mutation from search.</x:v>
+      </x:c>
+      <x:c r="S107" t="str">
+        <x:v>Needs live search-index retest for each major resource type and thumbnail signing behavior against current seeded/project data.</x:v>
+      </x:c>
+      <x:c r="T107" t="str">
+        <x:v>Maliev.Intranet.Client/Pages/Search.razor:1,8,20,29,34,40,45,57,59,64,68,89; Maliev.Intranet.Client/Components/Shared/GlobalSearchBox.razor:43,61,63,97,141,177,186,190,200,219,224,232,235,248; Maliev.Intranet.Bff/Controllers/SearchController.cs:17,26,28,33,41,44,45,47; Maliev.Intranet.Bff/Services/SearchResultMapper.cs:18,37,39,94; Maliev.Intranet.Bff/Services/GlobalSearchResultEnricher.cs:24,31,38,47,55,74,92,101,125,144; Maliev.Intranet.Tests/Client/Components/GlobalSearchBoxTests.cs:48,66,96,124,152,169,181,191,219,246; Maliev.Intranet.Tests/Bff/Services/SearchResultMapperTests.cs:14,25,37,48,59,74,89,103; Maliev.Intranet.Tests/Bff/Services/GlobalSearchResultEnricherTests.cs:41,81; Maliev.Intranet.Tests/Bff/Controllers/SearchControllerTests.cs:13,30,66; Maliev.Intranet.Tests/Bff/Clients/SearchServiceClientTests.cs:11,31</x:v>
+      </x:c>
+      <x:c r="U107" t="str">
+        <x:v>2026-06-30</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0214abd5e1b04860"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ebff454643a4769"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -15533,7 +15663,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e370dadd4764267"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7147fb77424456a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh Intranet billing tracker row
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rab9555a566f44c01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="R576e7530b9a84aa6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R563d9c7b5be44ada"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R11e494dc3eef47df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9b7531848d9d47f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Raddc9b154b46411a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rc1ecf6c5dca94f38"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rd7ba2c03cc714bc2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7341,7 +7341,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b6656610583497f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7f48f1168d04246"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9729,110 +9729,68 @@
       </x:c>
     </x:row>
     <x:row r="23" s="6" customFormat="1" ht="65.25" customHeight="1">
-      <x:c r="A23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">INT-022</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Maliev.Intranet</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Billing notes and credit terms</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">As finance staff, I can manage billing notes and credit terms.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Billing notes support list/create/detail; credit terms expose available terms.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current code-derived</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Automated Intranet suite passed 2026-06-23 after UX fix</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No behavior error observed in current Intranet automated retest.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No fix needed for this story from current Intranet automated retest.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current automated suite passed.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P2</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Finance UI -&gt; billing-notes/credit-terms controllers -&gt; InvoiceService</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Finance/accounting pages</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Billing and credit controls</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BillingNotesController GET/POST/detail; CreditTermsController GET</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Finance tests where present | Current suite: dotnet test Maliev.Intranet.slnx --verbosity minimal passed 1143/1150 with 7 skipped on 2026-06-23 after fix. Initial full run failed 1/1150 on ModuleRegressionSourceTests.ClientTextInputs_UpdateOnInputInsteadOfBlur.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Intranet BFF, InvoiceService</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Billing notes, credit-term state</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs UI route mapping review</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">BillingNotesController.cs:15-44; CreditTermsController.cs:15-22</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="U23" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-06-23</x:t>
-        </x:is>
+      <x:c r="A23" s="8" t="str">
+        <x:v>INT-022</x:v>
+      </x:c>
+      <x:c r="B23" s="8" t="str">
+        <x:v>Maliev.Intranet</x:v>
+      </x:c>
+      <x:c r="C23" s="8" t="str">
+        <x:v>Billing note lifecycle and credit terms reference</x:v>
+      </x:c>
+      <x:c r="D23" s="8" t="str">
+        <x:v>As a finance employee, I can read and create billing notes tied to customer invoices and retrieve credit-term reference data for invoice and payment workflows.</x:v>
+      </x:c>
+      <x:c r="E23" s="8" t="str">
+        <x:v>The billing-notes BFF requires billing-note read/write permissions, returns a paged billing-note list with optional invoice filtering, creates a billing note from customer, invoice IDs, issue date, due date, and notes, returns detail by ID, and responds NotFound when a note does not exist. The credit-terms BFF requires invoice read permission, retrieves all active terms through InvoiceServiceClient, and returns an empty list when the downstream service has no terms.</x:v>
+      </x:c>
+      <x:c r="F23" s="8" t="str">
+        <x:v>Current code-derived</x:v>
+      </x:c>
+      <x:c r="G23" s="8" t="str">
+        <x:v>Existing route and DTO coverage mapped 2026-06-30; no focused billing-note or credit-term controller/client behavior test was found in the current source slice.</x:v>
+      </x:c>
+      <x:c r="H23" s="8" t="str">
+        <x:v>No behavior error observed from current source inspection; no dedicated billing-note or credit-term UI controls were found in the current Accounting page inventory.</x:v>
+      </x:c>
+      <x:c r="I23" s="8" t="str">
+        <x:v>No app fix applied; tracker row refreshed to the current BFF/InvoiceService boundary without unsupported UI claims.</x:v>
+      </x:c>
+      <x:c r="J23" s="8" t="str">
+        <x:v>Pending full story-by-story behavior testing loop.</x:v>
+      </x:c>
+      <x:c r="K23" s="8" t="str">
+        <x:v>P2</x:v>
+      </x:c>
+      <x:c r="L23" s="8" t="str">
+        <x:v>Finance/accounting consumers -&gt; api/v1/billing-notes and api/v1/credit-terms BFF endpoints -&gt; InvoiceServiceClient -&gt; InvoiceService billing-note and credit-term DTO contracts with permission checks</x:v>
+      </x:c>
+      <x:c r="M23" s="8" t="str">
+        <x:v>BillingNotesController.cs; CreditTermsController.cs; InvoiceServiceClient.cs; BillingNoteDtos.cs; BillingDtos.cs; ControllerRouteTests.cs; DtoTests.cs</x:v>
+      </x:c>
+      <x:c r="N23" s="8" t="str">
+        <x:v>Current inspected UI evidence did not find dedicated billing-note or credit-term controls in Maliev.Intranet.Client/Pages/Accounting. The verifiable current surfaces are GET api/v1/billing-notes, POST api/v1/billing-notes, GET api/v1/billing-notes/{id}, and GET api/v1/credit-terms.</x:v>
+      </x:c>
+      <x:c r="O23" s="8" t="str">
+        <x:v>BillingNotesController maps list/create/detail routes to InvoiceServiceClient.GetBillingNotesAsync, CreateBillingNoteAsync, and GetBillingNoteByIdAsync. InvoiceServiceClient calls /invoice/v1/billing-notes with page/pageSize and optional invoiceId, POSTs create payloads to /invoice/v1/billing-notes, reads detail from /invoice/v1/billing-notes/{id}, and retrieves credit terms from /invoice/v1/credit-terms.</x:v>
+      </x:c>
+      <x:c r="P23" s="8" t="str">
+        <x:v>Mapped tests: ControllerRouteTests includes /api/v1/billing-notes and /api/v1/credit-terms route coverage; DtoTests instantiates BillingNoteDto and CreditTermDto. No focused billing-note or credit-term controller/client behavior test was found in this slice.</x:v>
+      </x:c>
+      <x:c r="Q23" s="8" t="str">
+        <x:v>Intranet BFF, InvoiceService</x:v>
+      </x:c>
+      <x:c r="R23" s="8" t="str">
+        <x:v>Billing note records, associated invoice IDs, issue and due dates, billing-note notes, credit-term reference records</x:v>
+      </x:c>
+      <x:c r="S23" s="8" t="str">
+        <x:v>Needs focused controller/client tests for billing-note list/create/detail and credit-term fallback behavior, plus a live finance workflow decision or browser retest if these controls should be exposed in the UI.</x:v>
+      </x:c>
+      <x:c r="T23" s="8" t="str">
+        <x:v>Maliev.Intranet.Bff/Controllers/BillingNotesController.cs:15,21,22,23,25,32,33,34,36,43,44,45,47; Maliev.Intranet.Bff/Controllers/CreditTermsController.cs:15,21,22,23,25,26; Maliev.Intranet.Bff/Clients/InvoiceServiceClient.cs:232,234,242,244,247,253,255,261,263; Maliev.Intranet.Shared/Dtos/BillingNoteDtos.cs:8,18,23,28,33,38,43,48,53,59,64,71,77,83,88; Maliev.Intranet.Shared/Dtos/BillingDtos.cs:32,37,42,47,52,57; Maliev.Intranet.Tests/Bff/ControllerRouteTests.cs:42,43; Maliev.Intranet.Tests/Shared/DtoTests.cs:77,78</x:v>
+      </x:c>
+      <x:c r="U23" s="8" t="str">
+        <x:v>2026-06-30</x:v>
       </x:c>
     </x:row>
     <x:row r="24" s="6" customFormat="1" ht="65.25" customHeight="1">
@@ -18742,7 +18700,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc235005a55b4db1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3e5362b5edf410a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25305,7 +25263,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53b5e4280bdd40b7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rae1e97c0053b425d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh QuoteEngine action-flow tracker rows
</commit_message>
<xml_diff>
--- a/docs/maliev-feature-user-story-status.xlsx
+++ b/docs/maliev-feature-user-story-status.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R9b7531848d9d47f3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Raddc9b154b46411a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="Rc1ecf6c5dca94f38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="Rd7ba2c03cc714bc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R7e05c27e30014d8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Web" sheetId="2" r:id="Rfcc3ea26baed4b01"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.Intranet" sheetId="3" r:id="R5caeeb0b12054b73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Maliev.QuoteEngine" sheetId="4" r:id="R5bc6f73becd7446e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -7341,7 +7341,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra7f48f1168d04246"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e0ff109d5d14072"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18700,7 +18700,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3e5362b5edf410a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3a1574717ca14d87"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20874,538 +20874,328 @@
       </x:c>
     </x:row>
     <x:row r="21" s="6" customFormat="1" ht="79.25" customHeight="1">
-      <x:c r="A21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QE-020</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Maliev.QuoteEngine</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Estimate</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">As a customer, I can request a quote estimate for configured parts.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Estimate endpoint prices configured parts and returns lead-time/total data for the summary/actions.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current code-derived</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Automated QuoteEngine suite passed 2026-06-23 after workspace cleanup</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No behavior error observed in current QuoteEngine automated retest.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">No fix needed for this story from current QuoteEngine automated retest.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="J21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Current automated suite passed.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="K21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">P0</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="L21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Workspace/summary -&gt; QuoteController estimate -&gt; Pricing service</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="M21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QuoteWorkspace.razor; QeQuoteSummaryBar.razor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="N21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Estimate action</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="O21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QuoteController POST estimate</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="P21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Pricing/QuoteEngine tests | Current suite: dotnet test Maliev.QuoteEngine.slnx --verbosity minimal passed 539/539 on 2026-06-23 after workspace cleanup.</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="Q21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QuoteEngine BFF, PricingService</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="R21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Estimate request/response</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="S21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Needs current pricing acceptance checks</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="T21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">QuoteController.cs:301; QeQuoteSummaryBar.razor</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="U21" s="8" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">2026-06-23</x:t>
-        </x:is>
+      <x:c r="A21" s="8" t="str">
+        <x:v>QE-020</x:v>
+      </x:c>
+      <x:c r="B21" s="8" t="str">
+        <x:v>Maliev.QuoteEngine</x:v>
+      </x:c>
+      <x:c r="C21" s